<commit_message>
docs(REV-158): sync SA-26..SA-34 into QA checklist workbook and correct REV-157 hash
The QA checklist workbook stopped at SA-25; append SA-26 through SA-34
from the CSV and extend the Summary formulas, Status dropdown,
conditional formatting and filter range to row 160. Correct the REV-157
commit reference from the pre-amend hash 3e928c1 to d8a826b.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
+++ b/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
@@ -11,7 +11,7 @@
     <sheet name="QA Checklist" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$151</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$160</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'QA Checklist'!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -582,7 +582,7 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTA('QA Checklist'!$A$5:$A$151)</f>
+        <f>COUNTA('QA Checklist'!$A$5:$A$160)</f>
         <v/>
       </c>
     </row>
@@ -593,7 +593,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$151,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$151,"Pass")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$160,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$160,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -604,7 +604,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$151,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$151,"Fail")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$160,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$160,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -615,7 +615,7 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$151,"Pending")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$160,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -669,19 +669,19 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$151,$A12)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$160,$A12)</f>
         <v/>
       </c>
       <c r="C12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$151,$A12,'QA Checklist'!$H$5:$H$151,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$151,$A12,'QA Checklist'!$H$5:$H$151,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$160,$A12,'QA Checklist'!$H$5:$H$160,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$160,$A12,'QA Checklist'!$H$5:$H$160,"Pass")</f>
         <v/>
       </c>
       <c r="D12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$151,$A12,'QA Checklist'!$H$5:$H$151,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$151,$A12,'QA Checklist'!$H$5:$H$151,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$160,$A12,'QA Checklist'!$H$5:$H$160,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$160,$A12,'QA Checklist'!$H$5:$H$160,"Fail")</f>
         <v/>
       </c>
       <c r="E12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$151,$A12,'QA Checklist'!$H$5:$H$151,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$160,$A12,'QA Checklist'!$H$5:$H$160,"Pending")</f>
         <v/>
       </c>
       <c r="F12" s="8">
@@ -696,19 +696,19 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$151,$A13)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$160,$A13)</f>
         <v/>
       </c>
       <c r="C13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$151,$A13,'QA Checklist'!$H$5:$H$151,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$151,$A13,'QA Checklist'!$H$5:$H$151,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$160,$A13,'QA Checklist'!$H$5:$H$160,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$160,$A13,'QA Checklist'!$H$5:$H$160,"Pass")</f>
         <v/>
       </c>
       <c r="D13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$151,$A13,'QA Checklist'!$H$5:$H$151,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$151,$A13,'QA Checklist'!$H$5:$H$151,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$160,$A13,'QA Checklist'!$H$5:$H$160,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$160,$A13,'QA Checklist'!$H$5:$H$160,"Fail")</f>
         <v/>
       </c>
       <c r="E13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$151,$A13,'QA Checklist'!$H$5:$H$151,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$160,$A13,'QA Checklist'!$H$5:$H$160,"Pending")</f>
         <v/>
       </c>
       <c r="F13" s="8">
@@ -723,19 +723,19 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$151,$A14)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$160,$A14)</f>
         <v/>
       </c>
       <c r="C14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$151,$A14,'QA Checklist'!$H$5:$H$151,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$151,$A14,'QA Checklist'!$H$5:$H$151,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$160,$A14,'QA Checklist'!$H$5:$H$160,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$160,$A14,'QA Checklist'!$H$5:$H$160,"Pass")</f>
         <v/>
       </c>
       <c r="D14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$151,$A14,'QA Checklist'!$H$5:$H$151,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$151,$A14,'QA Checklist'!$H$5:$H$151,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$160,$A14,'QA Checklist'!$H$5:$H$160,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$160,$A14,'QA Checklist'!$H$5:$H$160,"Fail")</f>
         <v/>
       </c>
       <c r="E14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$151,$A14,'QA Checklist'!$H$5:$H$151,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$160,$A14,'QA Checklist'!$H$5:$H$160,"Pending")</f>
         <v/>
       </c>
       <c r="F14" s="8">
@@ -750,19 +750,19 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$151,$A15)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$160,$A15)</f>
         <v/>
       </c>
       <c r="C15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$151,$A15,'QA Checklist'!$H$5:$H$151,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$151,$A15,'QA Checklist'!$H$5:$H$151,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$160,$A15,'QA Checklist'!$H$5:$H$160,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$160,$A15,'QA Checklist'!$H$5:$H$160,"Pass")</f>
         <v/>
       </c>
       <c r="D15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$151,$A15,'QA Checklist'!$H$5:$H$151,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$151,$A15,'QA Checklist'!$H$5:$H$151,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$160,$A15,'QA Checklist'!$H$5:$H$160,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$160,$A15,'QA Checklist'!$H$5:$H$160,"Fail")</f>
         <v/>
       </c>
       <c r="E15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$151,$A15,'QA Checklist'!$H$5:$H$151,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$160,$A15,'QA Checklist'!$H$5:$H$160,"Pending")</f>
         <v/>
       </c>
       <c r="F15" s="8">
@@ -777,19 +777,19 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$151,$A16)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$160,$A16)</f>
         <v/>
       </c>
       <c r="C16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$151,$A16,'QA Checklist'!$H$5:$H$151,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$151,$A16,'QA Checklist'!$H$5:$H$151,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$160,$A16,'QA Checklist'!$H$5:$H$160,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$160,$A16,'QA Checklist'!$H$5:$H$160,"Pass")</f>
         <v/>
       </c>
       <c r="D16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$151,$A16,'QA Checklist'!$H$5:$H$151,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$151,$A16,'QA Checklist'!$H$5:$H$151,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$160,$A16,'QA Checklist'!$H$5:$H$160,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$160,$A16,'QA Checklist'!$H$5:$H$160,"Fail")</f>
         <v/>
       </c>
       <c r="E16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$151,$A16,'QA Checklist'!$H$5:$H$151,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$160,$A16,'QA Checklist'!$H$5:$H$160,"Pending")</f>
         <v/>
       </c>
       <c r="F16" s="8">
@@ -804,19 +804,19 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$151,$A17)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$160,$A17)</f>
         <v/>
       </c>
       <c r="C17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$151,$A17,'QA Checklist'!$H$5:$H$151,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$151,$A17,'QA Checklist'!$H$5:$H$151,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$160,$A17,'QA Checklist'!$H$5:$H$160,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$160,$A17,'QA Checklist'!$H$5:$H$160,"Pass")</f>
         <v/>
       </c>
       <c r="D17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$151,$A17,'QA Checklist'!$H$5:$H$151,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$151,$A17,'QA Checklist'!$H$5:$H$151,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$160,$A17,'QA Checklist'!$H$5:$H$160,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$160,$A17,'QA Checklist'!$H$5:$H$160,"Fail")</f>
         <v/>
       </c>
       <c r="E17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$151,$A17,'QA Checklist'!$H$5:$H$151,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$160,$A17,'QA Checklist'!$H$5:$H$160,"Pending")</f>
         <v/>
       </c>
       <c r="F17" s="8">
@@ -831,19 +831,19 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$151,$A18)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$160,$A18)</f>
         <v/>
       </c>
       <c r="C18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$151,$A18,'QA Checklist'!$H$5:$H$151,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$151,$A18,'QA Checklist'!$H$5:$H$151,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$160,$A18,'QA Checklist'!$H$5:$H$160,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$160,$A18,'QA Checklist'!$H$5:$H$160,"Pass")</f>
         <v/>
       </c>
       <c r="D18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$151,$A18,'QA Checklist'!$H$5:$H$151,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$151,$A18,'QA Checklist'!$H$5:$H$151,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$160,$A18,'QA Checklist'!$H$5:$H$160,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$160,$A18,'QA Checklist'!$H$5:$H$160,"Fail")</f>
         <v/>
       </c>
       <c r="E18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$151,$A18,'QA Checklist'!$H$5:$H$151,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$160,$A18,'QA Checklist'!$H$5:$H$160,"Pending")</f>
         <v/>
       </c>
       <c r="F18" s="8">
@@ -858,19 +858,19 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$151,$A19)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$160,$A19)</f>
         <v/>
       </c>
       <c r="C19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$151,$A19,'QA Checklist'!$H$5:$H$151,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$151,$A19,'QA Checklist'!$H$5:$H$151,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$160,$A19,'QA Checklist'!$H$5:$H$160,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$160,$A19,'QA Checklist'!$H$5:$H$160,"Pass")</f>
         <v/>
       </c>
       <c r="D19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$151,$A19,'QA Checklist'!$H$5:$H$151,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$151,$A19,'QA Checklist'!$H$5:$H$151,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$160,$A19,'QA Checklist'!$H$5:$H$160,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$160,$A19,'QA Checklist'!$H$5:$H$160,"Fail")</f>
         <v/>
       </c>
       <c r="E19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$151,$A19,'QA Checklist'!$H$5:$H$151,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$160,$A19,'QA Checklist'!$H$5:$H$160,"Pending")</f>
         <v/>
       </c>
       <c r="F19" s="8">
@@ -885,19 +885,19 @@
         </is>
       </c>
       <c r="B20" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$151,$A20)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$160,$A20)</f>
         <v/>
       </c>
       <c r="C20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$151,$A20,'QA Checklist'!$H$5:$H$151,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$151,$A20,'QA Checklist'!$H$5:$H$151,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$160,$A20,'QA Checklist'!$H$5:$H$160,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$160,$A20,'QA Checklist'!$H$5:$H$160,"Pass")</f>
         <v/>
       </c>
       <c r="D20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$151,$A20,'QA Checklist'!$H$5:$H$151,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$151,$A20,'QA Checklist'!$H$5:$H$151,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$160,$A20,'QA Checklist'!$H$5:$H$160,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$160,$A20,'QA Checklist'!$H$5:$H$160,"Fail")</f>
         <v/>
       </c>
       <c r="E20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$151,$A20,'QA Checklist'!$H$5:$H$151,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$160,$A20,'QA Checklist'!$H$5:$H$160,"Pending")</f>
         <v/>
       </c>
       <c r="F20" s="8">
@@ -912,19 +912,19 @@
         </is>
       </c>
       <c r="B21" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$151,$A21)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$160,$A21)</f>
         <v/>
       </c>
       <c r="C21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$151,$A21,'QA Checklist'!$H$5:$H$151,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$151,$A21,'QA Checklist'!$H$5:$H$151,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$160,$A21,'QA Checklist'!$H$5:$H$160,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$160,$A21,'QA Checklist'!$H$5:$H$160,"Pass")</f>
         <v/>
       </c>
       <c r="D21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$151,$A21,'QA Checklist'!$H$5:$H$151,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$151,$A21,'QA Checklist'!$H$5:$H$151,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$160,$A21,'QA Checklist'!$H$5:$H$160,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$160,$A21,'QA Checklist'!$H$5:$H$160,"Fail")</f>
         <v/>
       </c>
       <c r="E21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$151,$A21,'QA Checklist'!$H$5:$H$151,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$160,$A21,'QA Checklist'!$H$5:$H$160,"Pending")</f>
         <v/>
       </c>
       <c r="F21" s="8">
@@ -939,19 +939,19 @@
         </is>
       </c>
       <c r="B22" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$151,$A22)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$160,$A22)</f>
         <v/>
       </c>
       <c r="C22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$151,$A22,'QA Checklist'!$H$5:$H$151,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$151,$A22,'QA Checklist'!$H$5:$H$151,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$160,$A22,'QA Checklist'!$H$5:$H$160,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$160,$A22,'QA Checklist'!$H$5:$H$160,"Pass")</f>
         <v/>
       </c>
       <c r="D22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$151,$A22,'QA Checklist'!$H$5:$H$151,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$151,$A22,'QA Checklist'!$H$5:$H$151,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$160,$A22,'QA Checklist'!$H$5:$H$160,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$160,$A22,'QA Checklist'!$H$5:$H$160,"Fail")</f>
         <v/>
       </c>
       <c r="E22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$151,$A22,'QA Checklist'!$H$5:$H$151,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$160,$A22,'QA Checklist'!$H$5:$H$160,"Pending")</f>
         <v/>
       </c>
       <c r="F22" s="8">
@@ -1020,19 +1020,19 @@
         </is>
       </c>
       <c r="B26" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$151,$A26&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$160,$A26&amp;"*")</f>
         <v/>
       </c>
       <c r="C26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$151,$A26&amp;"*",'QA Checklist'!$H$5:$H$151,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$151,$A26&amp;"*",'QA Checklist'!$H$5:$H$151,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$160,$A26&amp;"*",'QA Checklist'!$H$5:$H$160,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$160,$A26&amp;"*",'QA Checklist'!$H$5:$H$160,"Pass")</f>
         <v/>
       </c>
       <c r="D26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$151,$A26&amp;"*",'QA Checklist'!$H$5:$H$151,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$151,$A26&amp;"*",'QA Checklist'!$H$5:$H$151,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$160,$A26&amp;"*",'QA Checklist'!$H$5:$H$160,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$160,$A26&amp;"*",'QA Checklist'!$H$5:$H$160,"Fail")</f>
         <v/>
       </c>
       <c r="E26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$151,$A26&amp;"*",'QA Checklist'!$H$5:$H$151,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$160,$A26&amp;"*",'QA Checklist'!$H$5:$H$160,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1043,19 +1043,19 @@
         </is>
       </c>
       <c r="B27" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$151,$A27&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$160,$A27&amp;"*")</f>
         <v/>
       </c>
       <c r="C27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$151,$A27&amp;"*",'QA Checklist'!$H$5:$H$151,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$151,$A27&amp;"*",'QA Checklist'!$H$5:$H$151,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$160,$A27&amp;"*",'QA Checklist'!$H$5:$H$160,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$160,$A27&amp;"*",'QA Checklist'!$H$5:$H$160,"Pass")</f>
         <v/>
       </c>
       <c r="D27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$151,$A27&amp;"*",'QA Checklist'!$H$5:$H$151,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$151,$A27&amp;"*",'QA Checklist'!$H$5:$H$151,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$160,$A27&amp;"*",'QA Checklist'!$H$5:$H$160,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$160,$A27&amp;"*",'QA Checklist'!$H$5:$H$160,"Fail")</f>
         <v/>
       </c>
       <c r="E27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$151,$A27&amp;"*",'QA Checklist'!$H$5:$H$151,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$160,$A27&amp;"*",'QA Checklist'!$H$5:$H$160,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1066,19 +1066,19 @@
         </is>
       </c>
       <c r="B28" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$151,$A28&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$160,$A28&amp;"*")</f>
         <v/>
       </c>
       <c r="C28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$151,$A28&amp;"*",'QA Checklist'!$H$5:$H$151,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$151,$A28&amp;"*",'QA Checklist'!$H$5:$H$151,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$160,$A28&amp;"*",'QA Checklist'!$H$5:$H$160,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$160,$A28&amp;"*",'QA Checklist'!$H$5:$H$160,"Pass")</f>
         <v/>
       </c>
       <c r="D28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$151,$A28&amp;"*",'QA Checklist'!$H$5:$H$151,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$151,$A28&amp;"*",'QA Checklist'!$H$5:$H$151,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$160,$A28&amp;"*",'QA Checklist'!$H$5:$H$160,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$160,$A28&amp;"*",'QA Checklist'!$H$5:$H$160,"Fail")</f>
         <v/>
       </c>
       <c r="E28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$151,$A28&amp;"*",'QA Checklist'!$H$5:$H$151,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$160,$A28&amp;"*",'QA Checklist'!$H$5:$H$160,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1093,7 +1093,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I151"/>
+  <dimension ref="A1:I160"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1121,6 +1121,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="11" t="inlineStr">
         <is>
@@ -7633,12 +7634,435 @@
         </is>
       </c>
     </row>
+    <row r="152">
+      <c r="A152" s="12" t="inlineStr">
+        <is>
+          <t>SA-26</t>
+        </is>
+      </c>
+      <c r="B152" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="C152" s="13" t="inlineStr">
+        <is>
+          <t>Tier 2 (Workflow &amp; Ergonomics)</t>
+        </is>
+      </c>
+      <c r="D152" s="13" t="inlineStr">
+        <is>
+          <t>Form 1/3 PDF Pixel-Perfect Visual Calibration for Concern, Interviewed By, Authorization &amp; Signatures</t>
+        </is>
+      </c>
+      <c r="E152" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="F152" s="13" t="inlineStr">
+        <is>
+          <t>Log in as Service Advisor, open 2025 RO Excel Studio, fill Customer and Vehicle details, type Customer Concern, set Service Advisor name, fill Authorization and Lower Signatures, and inspect Form 1/3 live PDF preview / download PDF</t>
+        </is>
+      </c>
+      <c r="G152" s="13" t="inlineStr">
+        <is>
+          <t>Customer Concern sits centered horizontally and vertically inside the white Concern Box without overlapping NOTE legal text; Interviewed by Service Advisor sits cleanly above the underline at Y=583.5 with masked underline area; Customer Name and Signature rests directly on the Authorization underline at Y=545.5 with template ghost '0' masked; Parts &amp; Materials table aligns with true visual coordinates at Y=495.5 with 7.32pt pitch and Amount ghost whiteouts; Lower signatures and Filipino Claim Stub baselines align with true template underlines</t>
+        </is>
+      </c>
+      <c r="H152" s="14" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="I152" s="13" t="inlineStr">
+        <is>
+          <t>Verified by Automated Unit Tests (tests/frontend/app.test.js AUT-FRONT-116 and tests/frontend/sla_and_logic.test.js) and headless Chrome visual verification</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="12" t="inlineStr">
+        <is>
+          <t>SA-27</t>
+        </is>
+      </c>
+      <c r="B153" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="C153" s="13" t="inlineStr">
+        <is>
+          <t>Tier 2 (Workflow &amp; Ergonomics)</t>
+        </is>
+      </c>
+      <c r="D153" s="13" t="inlineStr">
+        <is>
+          <t>Form 1/3 PDF Table Grid Integrity &amp; Lower Signatures Calibration</t>
+        </is>
+      </c>
+      <c r="E153" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="F153" s="13" t="inlineStr">
+        <is>
+          <t>Log in as Service Advisor, open 2025 RO Excel Studio, add Parts and Materials line items, view/download Form 1/3 PDF, and inspect table grid lines, totals boxes, and signatures</t>
+        </is>
+      </c>
+      <c r="G153" s="13" t="inlineStr">
+        <is>
+          <t>Parts &amp; Materials table row 0 starts cleanly inside the first row at Y=497.75 with 7.78pt row step; whiteout is applied only to populated rows strictly inside cell margins without erasing black horizontal grid lines; all 23 rows retain 100% intact grid borders with zero white stripe artifacts; Parts Subtotal, Materials Subtotal, and Grand Total boxes display numbers cleanly within box borders without erasing surrounding lines; Recommending Approval and Approved By rest at Y=220.5 above Y=219.0 underline; Conforme Customer and Concurred By Manager rest at Y=186.5 above Y=185.0 underline without horizontal line cutting through letters</t>
+        </is>
+      </c>
+      <c r="H153" s="14" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="I153" s="13" t="inlineStr">
+        <is>
+          <t>Verified by Automated Unit Tests (tests/frontend/app.test.js AUT-FRONT-116 and tests/frontend/sla_and_logic.test.js) and headless Chrome rendering inspection</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="12" t="inlineStr">
+        <is>
+          <t>SA-28</t>
+        </is>
+      </c>
+      <c r="B154" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="C154" s="13" t="inlineStr">
+        <is>
+          <t>Tier 2 (Workflow &amp; Ergonomics)</t>
+        </is>
+      </c>
+      <c r="D154" s="13" t="inlineStr">
+        <is>
+          <t>Current_2025 BLANK RO UPDATED_v3 Job_Order_Wide Official Template Migration &amp; Coordinate Calibration</t>
+        </is>
+      </c>
+      <c r="E154" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="F154" s="13" t="inlineStr">
+        <is>
+          <t>Log in as Service Advisor, open 2025 RO Excel Studio, inspect Job_Order (Form 1/3) live PDF viewer, type customer information, concern, parts/materials, and click Export Official PDF / Download PDF</t>
+        </is>
+      </c>
+      <c r="G154" s="13" t="inlineStr">
+        <is>
+          <t>New wide template 'Current_2025 BLANK RO UPDATED_v3.xlsx - Job_Order_Wide.pdf' is embedded in frontend/assets/ as form13_template.pdf with old version cleanly removed; Job Order No (Y=792.2) and Date (Y=767.0) align with template underlines; Customer details sit on 8.11pt spaced baselines (Y=723.5, 715.4, 707.3, 699.2); Concern box is centered horizontally at X=299.4 with max width 430pt without text truncation or ellipsis; Parts &amp; Materials table aligns with 8.11pt row step starting at Y=494.6; Subtotals and Grand Total boxes display cleanly with targeted whiteouts; Lower signatures and Filipino Claim Stub align with true vector baseline coordinates</t>
+        </is>
+      </c>
+      <c r="H154" s="14" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="I154" s="13" t="inlineStr">
+        <is>
+          <t>Verified by Automated Unit Tests (144/144 passing in tests/frontend/app.test.js &amp; sla_and_logic.test.js) and vector geometry extraction</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="12" t="inlineStr">
+        <is>
+          <t>SA-29</t>
+        </is>
+      </c>
+      <c r="B155" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="C155" s="13" t="inlineStr">
+        <is>
+          <t>Tier 2 (Workflow &amp; Ergonomics)</t>
+        </is>
+      </c>
+      <c r="D155" s="13" t="inlineStr">
+        <is>
+          <t>Form 1/3 Parts &amp; Materials Table Amount Alignment &amp; Ghost Crescent Removal</t>
+        </is>
+      </c>
+      <c r="E155" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="F155" s="13" t="inlineStr">
+        <is>
+          <t>Log in as Service Advisor, open 2025 RO Excel Studio, inspect Job_Order (Form 1/3) live PDF viewer, add parts (e.g. Engine Oil Filter 450.00, Brake Pads 1850.00) and materials, observe AMOUNT column in live preview and exported PDF</t>
+        </is>
+      </c>
+      <c r="G155" s="13" t="inlineStr">
+        <is>
+          <t>Whiteout width is calibrated to 64.2pt for parts (covering up to X=352.7) and 48.2pt for materials (covering up to X=522.7) completely masking pre-printed 0.00 template characters; eliminated right-edge phantom crescent ')' artifact; amount values right-align precisely at X=351.6 (parts) and X=521.4 (materials) exactly aligning with pre-printed 0.00 rows below</t>
+        </is>
+      </c>
+      <c r="H155" s="14" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="I155" s="13" t="inlineStr">
+        <is>
+          <t>Verified by Automated Unit Tests (144/144 passing in tests/frontend/app.test.js &amp; sla_and_logic.test.js) and vector geometry extraction</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="12" t="inlineStr">
+        <is>
+          <t>SA-30</t>
+        </is>
+      </c>
+      <c r="B156" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="C156" s="13" t="inlineStr">
+        <is>
+          <t>Tier 2 (Workflow &amp; Ergonomics)</t>
+        </is>
+      </c>
+      <c r="D156" s="13" t="inlineStr">
+        <is>
+          <t>Form 1/3 Customer Conforme Signature &amp; Filipino Claim Stub Data Alignment</t>
+        </is>
+      </c>
+      <c r="E156" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="F156" s="13" t="inlineStr">
+        <is>
+          <t>Log in as Service Advisor, open 2025 RO Excel Studio (Form 1/3), observe default customer dossier and bottom claim stub, or type customer details and inspect live PDF preview</t>
+        </is>
+      </c>
+      <c r="G156" s="13" t="inlineStr">
+        <is>
+          <t>Customer Name and Signature is populated above the CONFORME line (Y=169.0) with default demo fallback and reactive live typing; Bottom Filipino Claim Stub displays Name (X=140), Plate No (centered at X=378.1), Year/Model (X=424), Service Advisor (X=140), Contact (X=355), Intake Date (X=140), and bold Claim Stub ID (centered at X=438.45); Date awkward center offset eliminated and aligned vertically with Name and SA; all claim stub fields update reactively with zero lag</t>
+        </is>
+      </c>
+      <c r="H156" s="14" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="I156" s="13" t="inlineStr">
+        <is>
+          <t>Verified by Automated Unit Tests (144/144 passing in tests/frontend/app.test.js &amp; sla_and_logic.test.js) and manual PDF inspection</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="12" t="inlineStr">
+        <is>
+          <t>SA-31</t>
+        </is>
+      </c>
+      <c r="B157" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="C157" s="13" t="inlineStr">
+        <is>
+          <t>Tier 2 (Workflow &amp; Ergonomics)</t>
+        </is>
+      </c>
+      <c r="D157" s="13" t="inlineStr">
+        <is>
+          <t>Form 1/3 &amp; RO Excel Export Multi-Sheet Cross-Verification with Live PDF Data</t>
+        </is>
+      </c>
+      <c r="E157" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="F157" s="13" t="inlineStr">
+        <is>
+          <t>Log in as Service Advisor, open 2025 RO Excel Studio, type customer, vehicle, contact, parts, and materials data in Form 1/3, click Export .xlsx, and inspect all 7 sheets of the downloaded Excel workbook against the live PDF preview</t>
+        </is>
+      </c>
+      <c r="G157" s="13" t="inlineStr">
+        <is>
+          <t>Sheet 1 (Job_Order) injects identical customer details (C10 Name, C11 Address, C12 Contact, C13 Email, K10 Plate, H10 Model, K11 Date, K12 Promise, K13 Color, H11 KM, H12 Engine, H13 Chassis), Concern (B17), Diagnostic (B27..B52), Parts (D27..G52), Materials (H27..K52), Subtotals (G53, K53, K54), Signatures (C53, I53, C58, H58, C61, H61), and complete Claim Stub (C70 Name, H70 Plate, J70 Model, I70 Plate/Model, C71 SA, H71/I71 Contact, C72 Date, H72/I72 Claim Stub ID); Sheets 2-4 (Quotation), Sheets 5-6 (Billing), and Sheet 7 (Checklist) inject identical mirrored datasets matching PDF output 1:1</t>
+        </is>
+      </c>
+      <c r="H157" s="14" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="I157" s="13" t="inlineStr">
+        <is>
+          <t>Verified by Automated Unit Tests (144/144 passing in tests/frontend/app.test.js &amp; sla_and_logic.test.js) and OpenXML extraction</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="12" t="inlineStr">
+        <is>
+          <t>SA-32</t>
+        </is>
+      </c>
+      <c r="B158" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="C158" s="13" t="inlineStr">
+        <is>
+          <t>Tier 2 (Workflow &amp; Ergonomics)</t>
+        </is>
+      </c>
+      <c r="D158" s="13" t="inlineStr">
+        <is>
+          <t>Quotation Form 2/3 PDF Coordinate Calibration &amp; Overlap Elimination</t>
+        </is>
+      </c>
+      <c r="E158" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="F158" s="13" t="inlineStr">
+        <is>
+          <t>Log in as Service Advisor, open 2025 RO Excel Studio, switch to Quotation sheet (Form 2/3), fill customer dossier &amp; repair items, and click 'Full PDF' or inspect live preview</t>
+        </is>
+      </c>
+      <c r="G158" s="13" t="inlineStr">
+        <is>
+          <t>Quotation No (e.g. QT-2026-9749) centers cleanly on top underline (X=500.9, Y=726.5) with zero overlap into 'QUOTATION NO.' text; Date, Job Order No, and Promised Date sit on true header cell baselines (Y=699.34, 690.46, 681.58) with labels intact and zero label truncation; Customer Details box baselines sit at Y=654.94, 646.06, 637.18 with pre-printed '0' ghosts cleanly masked and borders 100% intact; 30-row parts/labor table starts below header card at Y=610.54 without overlapping customer details; Lower signatures and Conforme line align cleanly with authentic template underlines</t>
+        </is>
+      </c>
+      <c r="H158" s="14" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="I158" s="13" t="inlineStr">
+        <is>
+          <t>Verified by Automated Unit Tests (144/144 passing in tests/frontend/app.test.js &amp; sla_and_logic.test.js) and vector geometry extraction</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="12" t="inlineStr">
+        <is>
+          <t>SA-33</t>
+        </is>
+      </c>
+      <c r="B159" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="C159" s="13" t="inlineStr">
+        <is>
+          <t>Tier 2 (Workflow &amp; Ergonomics)</t>
+        </is>
+      </c>
+      <c r="D159" s="13" t="inlineStr">
+        <is>
+          <t>Quotation Form 2/3 Exact Visual Vector Calibration &amp; Border-Safe Masking</t>
+        </is>
+      </c>
+      <c r="E159" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="F159" s="13" t="inlineStr">
+        <is>
+          <t>Log in as Service Advisor, open 2025 RO Excel Studio, switch to Quotation tab (Form 2/3), fill customer &amp; repair items, and click 'Full PDF' or 'Download PDF'</t>
+        </is>
+      </c>
+      <c r="G159" s="13" t="inlineStr">
+        <is>
+          <t>Quotation No (e.g. QT-2026-5777) centers directly on the template underline at Y=772.0 above DATE box with zero vertical displacement; Right Meta Box correctly renders Date (Y=742.8), Job Order No (Y=733.2), and Promised Date (Y=723.8) strictly inside their boxes with ghost '0' masked; Customer Details align on exact baselines (Y=694.8, 685.4, 675.9) with all '0' ghost placeholders 100% eliminated without cutting through black underlines; 30 table rows align with exact cell geometry starting at Y=647.42 with 100% intact grid borders and zero ghost artifacts; Totals block right-aligns inside cell at X=516.5; Lower signatures (SA, Manager, Conforme) rest cleanly on authentic underlines</t>
+        </is>
+      </c>
+      <c r="H159" s="14" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="I159" s="13" t="inlineStr">
+        <is>
+          <t>Verified by Automated Unit Tests (145/145 passing in tests/frontend/sla_and_logic.test.js AUT-FRONT-111) and pypdfium2 visual rendering inspection</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="12" t="inlineStr">
+        <is>
+          <t>SA-34</t>
+        </is>
+      </c>
+      <c r="B160" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="C160" s="13" t="inlineStr">
+        <is>
+          <t>Tier 2 (Workflow &amp; Ergonomics)</t>
+        </is>
+      </c>
+      <c r="D160" s="13" t="inlineStr">
+        <is>
+          <t>Billing Form 3/3 Measured Vector Alignment &amp; Border-Safe Ghost Masking</t>
+        </is>
+      </c>
+      <c r="E160" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="F160" s="13" t="inlineStr">
+        <is>
+          <t>Log in as Service Advisor, open 2025 RO Excel Studio, switch to Billing tab (Form 3/3), fill customer details and billing line items, and click 'Full PDF' or 'Download PDF'</t>
+        </is>
+      </c>
+      <c r="G160" s="13" t="inlineStr">
+        <is>
+          <t>Billing No sits on the underline to the right of BILLING NO. without overlapping the title; Date, Job Order No and Quotation No sit inside their boxes with no caret (^) artifacts and intact box lines; Customer Details values rest on their underlines with no ghost 0 or caret marks and no broken underline segments; Km Reading value does not overlap its label; bill amount fits its underline without covering the word 'with'; item descriptions stay inside the table's left border, all 36 rows keep intact grid lines, and empty AMOUNT cells show no dash artifacts; LABOR, VAT 12%, MATERIALS, PARTS and TOTAL values sit centered inside their boxes</t>
+        </is>
+      </c>
+      <c r="H160" s="14" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="I160" s="13" t="inlineStr">
+        <is>
+          <t>Verified by Automated Unit Tests (146/146 passing in tests/frontend/sla_and_logic.test.js AUT-FRONT-117) and pdf-lib/pdfplumber rendered PDF inspection</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:I151"/>
+  <autoFilter ref="A4:I160"/>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="H5:H151">
+  <conditionalFormatting sqref="H5:H160">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$H5="Passed"</formula>
     </cfRule>
@@ -7655,13 +8079,13 @@
       <formula>$H5="Pending"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A5:A151">
+  <conditionalFormatting sqref="A5:A160">
     <cfRule type="expression" priority="6" dxfId="3">
-      <formula>COUNTIF($A$5:$A$151,$A5)&gt;1</formula>
+      <formula>COUNTIF($A$5:$A$160,$A5)&gt;1</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H5:H151" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H5:H160" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pending,Passed,Failed"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
fix(REV-159): center Billing Form 3/3 Service Advisor signature on signature line
Center the Service Advisor name at X=123.4 (midpoint of the x 28.6-218.1
signature line) on baseline Y=90.6, aligned with the "Service Advisor"
label and clear of "HONTECH MANGEMENT:", shrinking to fit long names.
Bump cache buster to v=3.12, add AUT-FRONT-118, and sync REV-159 / SA-35
into the revisions log, checklists and QA workbook.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
+++ b/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
@@ -11,7 +11,7 @@
     <sheet name="QA Checklist" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$160</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$161</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'QA Checklist'!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -563,6 +563,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -582,7 +583,7 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTA('QA Checklist'!$A$5:$A$160)</f>
+        <f>COUNTA('QA Checklist'!$A$5:$A$161)</f>
         <v/>
       </c>
     </row>
@@ -593,7 +594,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$160,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$160,"Pass")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$161,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$161,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -604,7 +605,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$160,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$160,"Fail")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$161,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$161,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -615,7 +616,7 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$160,"Pending")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$161,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -630,6 +631,7 @@
         <v/>
       </c>
     </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
@@ -669,19 +671,19 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$160,$A12)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$161,$A12)</f>
         <v/>
       </c>
       <c r="C12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$160,$A12,'QA Checklist'!$H$5:$H$160,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$160,$A12,'QA Checklist'!$H$5:$H$160,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$161,$A12,'QA Checklist'!$H$5:$H$161,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$161,$A12,'QA Checklist'!$H$5:$H$161,"Pass")</f>
         <v/>
       </c>
       <c r="D12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$160,$A12,'QA Checklist'!$H$5:$H$160,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$160,$A12,'QA Checklist'!$H$5:$H$160,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$161,$A12,'QA Checklist'!$H$5:$H$161,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$161,$A12,'QA Checklist'!$H$5:$H$161,"Fail")</f>
         <v/>
       </c>
       <c r="E12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$160,$A12,'QA Checklist'!$H$5:$H$160,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$161,$A12,'QA Checklist'!$H$5:$H$161,"Pending")</f>
         <v/>
       </c>
       <c r="F12" s="8">
@@ -696,19 +698,19 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$160,$A13)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$161,$A13)</f>
         <v/>
       </c>
       <c r="C13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$160,$A13,'QA Checklist'!$H$5:$H$160,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$160,$A13,'QA Checklist'!$H$5:$H$160,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$161,$A13,'QA Checklist'!$H$5:$H$161,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$161,$A13,'QA Checklist'!$H$5:$H$161,"Pass")</f>
         <v/>
       </c>
       <c r="D13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$160,$A13,'QA Checklist'!$H$5:$H$160,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$160,$A13,'QA Checklist'!$H$5:$H$160,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$161,$A13,'QA Checklist'!$H$5:$H$161,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$161,$A13,'QA Checklist'!$H$5:$H$161,"Fail")</f>
         <v/>
       </c>
       <c r="E13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$160,$A13,'QA Checklist'!$H$5:$H$160,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$161,$A13,'QA Checklist'!$H$5:$H$161,"Pending")</f>
         <v/>
       </c>
       <c r="F13" s="8">
@@ -723,19 +725,19 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$160,$A14)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$161,$A14)</f>
         <v/>
       </c>
       <c r="C14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$160,$A14,'QA Checklist'!$H$5:$H$160,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$160,$A14,'QA Checklist'!$H$5:$H$160,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$161,$A14,'QA Checklist'!$H$5:$H$161,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$161,$A14,'QA Checklist'!$H$5:$H$161,"Pass")</f>
         <v/>
       </c>
       <c r="D14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$160,$A14,'QA Checklist'!$H$5:$H$160,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$160,$A14,'QA Checklist'!$H$5:$H$160,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$161,$A14,'QA Checklist'!$H$5:$H$161,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$161,$A14,'QA Checklist'!$H$5:$H$161,"Fail")</f>
         <v/>
       </c>
       <c r="E14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$160,$A14,'QA Checklist'!$H$5:$H$160,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$161,$A14,'QA Checklist'!$H$5:$H$161,"Pending")</f>
         <v/>
       </c>
       <c r="F14" s="8">
@@ -750,19 +752,19 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$160,$A15)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$161,$A15)</f>
         <v/>
       </c>
       <c r="C15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$160,$A15,'QA Checklist'!$H$5:$H$160,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$160,$A15,'QA Checklist'!$H$5:$H$160,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$161,$A15,'QA Checklist'!$H$5:$H$161,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$161,$A15,'QA Checklist'!$H$5:$H$161,"Pass")</f>
         <v/>
       </c>
       <c r="D15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$160,$A15,'QA Checklist'!$H$5:$H$160,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$160,$A15,'QA Checklist'!$H$5:$H$160,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$161,$A15,'QA Checklist'!$H$5:$H$161,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$161,$A15,'QA Checklist'!$H$5:$H$161,"Fail")</f>
         <v/>
       </c>
       <c r="E15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$160,$A15,'QA Checklist'!$H$5:$H$160,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$161,$A15,'QA Checklist'!$H$5:$H$161,"Pending")</f>
         <v/>
       </c>
       <c r="F15" s="8">
@@ -777,19 +779,19 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$160,$A16)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$161,$A16)</f>
         <v/>
       </c>
       <c r="C16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$160,$A16,'QA Checklist'!$H$5:$H$160,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$160,$A16,'QA Checklist'!$H$5:$H$160,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$161,$A16,'QA Checklist'!$H$5:$H$161,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$161,$A16,'QA Checklist'!$H$5:$H$161,"Pass")</f>
         <v/>
       </c>
       <c r="D16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$160,$A16,'QA Checklist'!$H$5:$H$160,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$160,$A16,'QA Checklist'!$H$5:$H$160,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$161,$A16,'QA Checklist'!$H$5:$H$161,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$161,$A16,'QA Checklist'!$H$5:$H$161,"Fail")</f>
         <v/>
       </c>
       <c r="E16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$160,$A16,'QA Checklist'!$H$5:$H$160,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$161,$A16,'QA Checklist'!$H$5:$H$161,"Pending")</f>
         <v/>
       </c>
       <c r="F16" s="8">
@@ -804,19 +806,19 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$160,$A17)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$161,$A17)</f>
         <v/>
       </c>
       <c r="C17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$160,$A17,'QA Checklist'!$H$5:$H$160,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$160,$A17,'QA Checklist'!$H$5:$H$160,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$161,$A17,'QA Checklist'!$H$5:$H$161,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$161,$A17,'QA Checklist'!$H$5:$H$161,"Pass")</f>
         <v/>
       </c>
       <c r="D17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$160,$A17,'QA Checklist'!$H$5:$H$160,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$160,$A17,'QA Checklist'!$H$5:$H$160,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$161,$A17,'QA Checklist'!$H$5:$H$161,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$161,$A17,'QA Checklist'!$H$5:$H$161,"Fail")</f>
         <v/>
       </c>
       <c r="E17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$160,$A17,'QA Checklist'!$H$5:$H$160,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$161,$A17,'QA Checklist'!$H$5:$H$161,"Pending")</f>
         <v/>
       </c>
       <c r="F17" s="8">
@@ -831,19 +833,19 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$160,$A18)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$161,$A18)</f>
         <v/>
       </c>
       <c r="C18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$160,$A18,'QA Checklist'!$H$5:$H$160,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$160,$A18,'QA Checklist'!$H$5:$H$160,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$161,$A18,'QA Checklist'!$H$5:$H$161,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$161,$A18,'QA Checklist'!$H$5:$H$161,"Pass")</f>
         <v/>
       </c>
       <c r="D18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$160,$A18,'QA Checklist'!$H$5:$H$160,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$160,$A18,'QA Checklist'!$H$5:$H$160,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$161,$A18,'QA Checklist'!$H$5:$H$161,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$161,$A18,'QA Checklist'!$H$5:$H$161,"Fail")</f>
         <v/>
       </c>
       <c r="E18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$160,$A18,'QA Checklist'!$H$5:$H$160,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$161,$A18,'QA Checklist'!$H$5:$H$161,"Pending")</f>
         <v/>
       </c>
       <c r="F18" s="8">
@@ -858,19 +860,19 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$160,$A19)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$161,$A19)</f>
         <v/>
       </c>
       <c r="C19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$160,$A19,'QA Checklist'!$H$5:$H$160,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$160,$A19,'QA Checklist'!$H$5:$H$160,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$161,$A19,'QA Checklist'!$H$5:$H$161,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$161,$A19,'QA Checklist'!$H$5:$H$161,"Pass")</f>
         <v/>
       </c>
       <c r="D19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$160,$A19,'QA Checklist'!$H$5:$H$160,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$160,$A19,'QA Checklist'!$H$5:$H$160,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$161,$A19,'QA Checklist'!$H$5:$H$161,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$161,$A19,'QA Checklist'!$H$5:$H$161,"Fail")</f>
         <v/>
       </c>
       <c r="E19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$160,$A19,'QA Checklist'!$H$5:$H$160,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$161,$A19,'QA Checklist'!$H$5:$H$161,"Pending")</f>
         <v/>
       </c>
       <c r="F19" s="8">
@@ -885,19 +887,19 @@
         </is>
       </c>
       <c r="B20" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$160,$A20)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$161,$A20)</f>
         <v/>
       </c>
       <c r="C20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$160,$A20,'QA Checklist'!$H$5:$H$160,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$160,$A20,'QA Checklist'!$H$5:$H$160,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$161,$A20,'QA Checklist'!$H$5:$H$161,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$161,$A20,'QA Checklist'!$H$5:$H$161,"Pass")</f>
         <v/>
       </c>
       <c r="D20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$160,$A20,'QA Checklist'!$H$5:$H$160,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$160,$A20,'QA Checklist'!$H$5:$H$160,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$161,$A20,'QA Checklist'!$H$5:$H$161,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$161,$A20,'QA Checklist'!$H$5:$H$161,"Fail")</f>
         <v/>
       </c>
       <c r="E20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$160,$A20,'QA Checklist'!$H$5:$H$160,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$161,$A20,'QA Checklist'!$H$5:$H$161,"Pending")</f>
         <v/>
       </c>
       <c r="F20" s="8">
@@ -912,19 +914,19 @@
         </is>
       </c>
       <c r="B21" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$160,$A21)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$161,$A21)</f>
         <v/>
       </c>
       <c r="C21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$160,$A21,'QA Checklist'!$H$5:$H$160,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$160,$A21,'QA Checklist'!$H$5:$H$160,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$161,$A21,'QA Checklist'!$H$5:$H$161,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$161,$A21,'QA Checklist'!$H$5:$H$161,"Pass")</f>
         <v/>
       </c>
       <c r="D21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$160,$A21,'QA Checklist'!$H$5:$H$160,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$160,$A21,'QA Checklist'!$H$5:$H$160,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$161,$A21,'QA Checklist'!$H$5:$H$161,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$161,$A21,'QA Checklist'!$H$5:$H$161,"Fail")</f>
         <v/>
       </c>
       <c r="E21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$160,$A21,'QA Checklist'!$H$5:$H$160,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$161,$A21,'QA Checklist'!$H$5:$H$161,"Pending")</f>
         <v/>
       </c>
       <c r="F21" s="8">
@@ -939,19 +941,19 @@
         </is>
       </c>
       <c r="B22" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$160,$A22)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$161,$A22)</f>
         <v/>
       </c>
       <c r="C22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$160,$A22,'QA Checklist'!$H$5:$H$160,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$160,$A22,'QA Checklist'!$H$5:$H$160,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$161,$A22,'QA Checklist'!$H$5:$H$161,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$161,$A22,'QA Checklist'!$H$5:$H$161,"Pass")</f>
         <v/>
       </c>
       <c r="D22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$160,$A22,'QA Checklist'!$H$5:$H$160,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$160,$A22,'QA Checklist'!$H$5:$H$160,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$161,$A22,'QA Checklist'!$H$5:$H$161,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$161,$A22,'QA Checklist'!$H$5:$H$161,"Fail")</f>
         <v/>
       </c>
       <c r="E22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$160,$A22,'QA Checklist'!$H$5:$H$160,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$161,$A22,'QA Checklist'!$H$5:$H$161,"Pending")</f>
         <v/>
       </c>
       <c r="F22" s="8">
@@ -986,6 +988,7 @@
         <v/>
       </c>
     </row>
+    <row r="24"/>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
@@ -1020,19 +1023,19 @@
         </is>
       </c>
       <c r="B26" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$160,$A26&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$161,$A26&amp;"*")</f>
         <v/>
       </c>
       <c r="C26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$160,$A26&amp;"*",'QA Checklist'!$H$5:$H$160,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$160,$A26&amp;"*",'QA Checklist'!$H$5:$H$160,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$161,$A26&amp;"*",'QA Checklist'!$H$5:$H$161,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$161,$A26&amp;"*",'QA Checklist'!$H$5:$H$161,"Pass")</f>
         <v/>
       </c>
       <c r="D26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$160,$A26&amp;"*",'QA Checklist'!$H$5:$H$160,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$160,$A26&amp;"*",'QA Checklist'!$H$5:$H$160,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$161,$A26&amp;"*",'QA Checklist'!$H$5:$H$161,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$161,$A26&amp;"*",'QA Checklist'!$H$5:$H$161,"Fail")</f>
         <v/>
       </c>
       <c r="E26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$160,$A26&amp;"*",'QA Checklist'!$H$5:$H$160,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$161,$A26&amp;"*",'QA Checklist'!$H$5:$H$161,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1043,19 +1046,19 @@
         </is>
       </c>
       <c r="B27" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$160,$A27&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$161,$A27&amp;"*")</f>
         <v/>
       </c>
       <c r="C27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$160,$A27&amp;"*",'QA Checklist'!$H$5:$H$160,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$160,$A27&amp;"*",'QA Checklist'!$H$5:$H$160,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$161,$A27&amp;"*",'QA Checklist'!$H$5:$H$161,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$161,$A27&amp;"*",'QA Checklist'!$H$5:$H$161,"Pass")</f>
         <v/>
       </c>
       <c r="D27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$160,$A27&amp;"*",'QA Checklist'!$H$5:$H$160,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$160,$A27&amp;"*",'QA Checklist'!$H$5:$H$160,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$161,$A27&amp;"*",'QA Checklist'!$H$5:$H$161,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$161,$A27&amp;"*",'QA Checklist'!$H$5:$H$161,"Fail")</f>
         <v/>
       </c>
       <c r="E27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$160,$A27&amp;"*",'QA Checklist'!$H$5:$H$160,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$161,$A27&amp;"*",'QA Checklist'!$H$5:$H$161,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1066,19 +1069,19 @@
         </is>
       </c>
       <c r="B28" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$160,$A28&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$161,$A28&amp;"*")</f>
         <v/>
       </c>
       <c r="C28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$160,$A28&amp;"*",'QA Checklist'!$H$5:$H$160,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$160,$A28&amp;"*",'QA Checklist'!$H$5:$H$160,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$161,$A28&amp;"*",'QA Checklist'!$H$5:$H$161,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$161,$A28&amp;"*",'QA Checklist'!$H$5:$H$161,"Pass")</f>
         <v/>
       </c>
       <c r="D28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$160,$A28&amp;"*",'QA Checklist'!$H$5:$H$160,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$160,$A28&amp;"*",'QA Checklist'!$H$5:$H$160,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$161,$A28&amp;"*",'QA Checklist'!$H$5:$H$161,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$161,$A28&amp;"*",'QA Checklist'!$H$5:$H$161,"Fail")</f>
         <v/>
       </c>
       <c r="E28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$160,$A28&amp;"*",'QA Checklist'!$H$5:$H$160,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$161,$A28&amp;"*",'QA Checklist'!$H$5:$H$161,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1093,7 +1096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I160"/>
+  <dimension ref="A1:I161"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1121,7 +1124,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="11" t="inlineStr">
         <is>
@@ -8057,12 +8059,59 @@
         </is>
       </c>
     </row>
+    <row r="161">
+      <c r="A161" s="12" t="inlineStr">
+        <is>
+          <t>SA-35</t>
+        </is>
+      </c>
+      <c r="B161" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="C161" s="13" t="inlineStr">
+        <is>
+          <t>Tier 2 (Workflow &amp; Ergonomics)</t>
+        </is>
+      </c>
+      <c r="D161" s="13" t="inlineStr">
+        <is>
+          <t>Billing Form 3/3 Service Advisor Signature Alignment</t>
+        </is>
+      </c>
+      <c r="E161" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="F161" s="13" t="inlineStr">
+        <is>
+          <t>Log in as Service Advisor, open 2025 RO Excel Studio, switch to Billing tab (Form 3/3), set the Service Advisor name, and click 'Full PDF' or 'Download PDF'</t>
+        </is>
+      </c>
+      <c r="G161" s="13" t="inlineStr">
+        <is>
+          <t>The Service Advisor name sits horizontally centered on the signature line directly above it, vertically aligned with the 'Service Advisor' label below, without touching the line or the 'HONTECH MANGEMENT:' heading; long names shrink to stay within the line</t>
+        </is>
+      </c>
+      <c r="H161" s="14" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="I161" s="13" t="inlineStr">
+        <is>
+          <t>Verified by Automated Unit Tests (147/147 passing in tests/frontend/sla_and_logic.test.js AUT-FRONT-118) and 300 dpi rendered PDF inspection</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:I160"/>
+  <autoFilter ref="A4:I161"/>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="H5:H160">
+  <conditionalFormatting sqref="H5:H161">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$H5="Passed"</formula>
     </cfRule>
@@ -8079,13 +8128,13 @@
       <formula>$H5="Pending"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A5:A160">
+  <conditionalFormatting sqref="A5:A161">
     <cfRule type="expression" priority="6" dxfId="3">
-      <formula>COUNTIF($A$5:$A$160,$A5)&gt;1</formula>
+      <formula>COUNTIF($A$5:$A$161,$A5)&gt;1</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H5:H160" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H5:H161" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pending,Passed,Failed"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
fix(REV-160): calibrate Checklist Result status-box grid, header, comments and signatures
Recalibrate compileChecklistPDFBytes to geometry measured from the
CheckList_Result template: every inspection point is stamped as a dark
checkmark centered in the matching green/yellow/red box on its own row
(8 previously unmapped points included), battery and brake pads map to
their dedicated boxes, header placeholder ghosts are fully masked, the
date is centered, the fuel ring sits inside its cell, comments wrap onto
the ruled lines, and technician/customer names are centered on their
lines. Bump cache buster to v=3.13, add AUT-FRONT-119, and sync REV-160
and SA-36 into the revisions log, checklists and QA workbook.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
+++ b/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
@@ -11,7 +11,7 @@
     <sheet name="QA Checklist" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$161</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$162</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'QA Checklist'!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTA('QA Checklist'!$A$5:$A$161)</f>
+        <f>COUNTA('QA Checklist'!$A$5:$A$162)</f>
         <v/>
       </c>
     </row>
@@ -594,7 +594,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$161,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$161,"Pass")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$162,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$162,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$161,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$161,"Fail")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$162,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$162,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -616,7 +616,7 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$161,"Pending")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$162,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -671,19 +671,19 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$161,$A12)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$162,$A12)</f>
         <v/>
       </c>
       <c r="C12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$161,$A12,'QA Checklist'!$H$5:$H$161,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$161,$A12,'QA Checklist'!$H$5:$H$161,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$162,$A12,'QA Checklist'!$H$5:$H$162,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$162,$A12,'QA Checklist'!$H$5:$H$162,"Pass")</f>
         <v/>
       </c>
       <c r="D12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$161,$A12,'QA Checklist'!$H$5:$H$161,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$161,$A12,'QA Checklist'!$H$5:$H$161,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$162,$A12,'QA Checklist'!$H$5:$H$162,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$162,$A12,'QA Checklist'!$H$5:$H$162,"Fail")</f>
         <v/>
       </c>
       <c r="E12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$161,$A12,'QA Checklist'!$H$5:$H$161,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$162,$A12,'QA Checklist'!$H$5:$H$162,"Pending")</f>
         <v/>
       </c>
       <c r="F12" s="8">
@@ -698,19 +698,19 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$161,$A13)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$162,$A13)</f>
         <v/>
       </c>
       <c r="C13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$161,$A13,'QA Checklist'!$H$5:$H$161,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$161,$A13,'QA Checklist'!$H$5:$H$161,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$162,$A13,'QA Checklist'!$H$5:$H$162,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$162,$A13,'QA Checklist'!$H$5:$H$162,"Pass")</f>
         <v/>
       </c>
       <c r="D13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$161,$A13,'QA Checklist'!$H$5:$H$161,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$161,$A13,'QA Checklist'!$H$5:$H$161,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$162,$A13,'QA Checklist'!$H$5:$H$162,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$162,$A13,'QA Checklist'!$H$5:$H$162,"Fail")</f>
         <v/>
       </c>
       <c r="E13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$161,$A13,'QA Checklist'!$H$5:$H$161,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$162,$A13,'QA Checklist'!$H$5:$H$162,"Pending")</f>
         <v/>
       </c>
       <c r="F13" s="8">
@@ -725,19 +725,19 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$161,$A14)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$162,$A14)</f>
         <v/>
       </c>
       <c r="C14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$161,$A14,'QA Checklist'!$H$5:$H$161,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$161,$A14,'QA Checklist'!$H$5:$H$161,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$162,$A14,'QA Checklist'!$H$5:$H$162,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$162,$A14,'QA Checklist'!$H$5:$H$162,"Pass")</f>
         <v/>
       </c>
       <c r="D14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$161,$A14,'QA Checklist'!$H$5:$H$161,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$161,$A14,'QA Checklist'!$H$5:$H$161,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$162,$A14,'QA Checklist'!$H$5:$H$162,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$162,$A14,'QA Checklist'!$H$5:$H$162,"Fail")</f>
         <v/>
       </c>
       <c r="E14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$161,$A14,'QA Checklist'!$H$5:$H$161,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$162,$A14,'QA Checklist'!$H$5:$H$162,"Pending")</f>
         <v/>
       </c>
       <c r="F14" s="8">
@@ -752,19 +752,19 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$161,$A15)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$162,$A15)</f>
         <v/>
       </c>
       <c r="C15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$161,$A15,'QA Checklist'!$H$5:$H$161,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$161,$A15,'QA Checklist'!$H$5:$H$161,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$162,$A15,'QA Checklist'!$H$5:$H$162,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$162,$A15,'QA Checklist'!$H$5:$H$162,"Pass")</f>
         <v/>
       </c>
       <c r="D15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$161,$A15,'QA Checklist'!$H$5:$H$161,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$161,$A15,'QA Checklist'!$H$5:$H$161,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$162,$A15,'QA Checklist'!$H$5:$H$162,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$162,$A15,'QA Checklist'!$H$5:$H$162,"Fail")</f>
         <v/>
       </c>
       <c r="E15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$161,$A15,'QA Checklist'!$H$5:$H$161,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$162,$A15,'QA Checklist'!$H$5:$H$162,"Pending")</f>
         <v/>
       </c>
       <c r="F15" s="8">
@@ -779,19 +779,19 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$161,$A16)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$162,$A16)</f>
         <v/>
       </c>
       <c r="C16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$161,$A16,'QA Checklist'!$H$5:$H$161,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$161,$A16,'QA Checklist'!$H$5:$H$161,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$162,$A16,'QA Checklist'!$H$5:$H$162,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$162,$A16,'QA Checklist'!$H$5:$H$162,"Pass")</f>
         <v/>
       </c>
       <c r="D16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$161,$A16,'QA Checklist'!$H$5:$H$161,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$161,$A16,'QA Checklist'!$H$5:$H$161,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$162,$A16,'QA Checklist'!$H$5:$H$162,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$162,$A16,'QA Checklist'!$H$5:$H$162,"Fail")</f>
         <v/>
       </c>
       <c r="E16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$161,$A16,'QA Checklist'!$H$5:$H$161,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$162,$A16,'QA Checklist'!$H$5:$H$162,"Pending")</f>
         <v/>
       </c>
       <c r="F16" s="8">
@@ -806,19 +806,19 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$161,$A17)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$162,$A17)</f>
         <v/>
       </c>
       <c r="C17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$161,$A17,'QA Checklist'!$H$5:$H$161,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$161,$A17,'QA Checklist'!$H$5:$H$161,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$162,$A17,'QA Checklist'!$H$5:$H$162,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$162,$A17,'QA Checklist'!$H$5:$H$162,"Pass")</f>
         <v/>
       </c>
       <c r="D17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$161,$A17,'QA Checklist'!$H$5:$H$161,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$161,$A17,'QA Checklist'!$H$5:$H$161,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$162,$A17,'QA Checklist'!$H$5:$H$162,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$162,$A17,'QA Checklist'!$H$5:$H$162,"Fail")</f>
         <v/>
       </c>
       <c r="E17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$161,$A17,'QA Checklist'!$H$5:$H$161,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$162,$A17,'QA Checklist'!$H$5:$H$162,"Pending")</f>
         <v/>
       </c>
       <c r="F17" s="8">
@@ -833,19 +833,19 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$161,$A18)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$162,$A18)</f>
         <v/>
       </c>
       <c r="C18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$161,$A18,'QA Checklist'!$H$5:$H$161,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$161,$A18,'QA Checklist'!$H$5:$H$161,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$162,$A18,'QA Checklist'!$H$5:$H$162,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$162,$A18,'QA Checklist'!$H$5:$H$162,"Pass")</f>
         <v/>
       </c>
       <c r="D18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$161,$A18,'QA Checklist'!$H$5:$H$161,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$161,$A18,'QA Checklist'!$H$5:$H$161,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$162,$A18,'QA Checklist'!$H$5:$H$162,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$162,$A18,'QA Checklist'!$H$5:$H$162,"Fail")</f>
         <v/>
       </c>
       <c r="E18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$161,$A18,'QA Checklist'!$H$5:$H$161,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$162,$A18,'QA Checklist'!$H$5:$H$162,"Pending")</f>
         <v/>
       </c>
       <c r="F18" s="8">
@@ -860,19 +860,19 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$161,$A19)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$162,$A19)</f>
         <v/>
       </c>
       <c r="C19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$161,$A19,'QA Checklist'!$H$5:$H$161,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$161,$A19,'QA Checklist'!$H$5:$H$161,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$162,$A19,'QA Checklist'!$H$5:$H$162,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$162,$A19,'QA Checklist'!$H$5:$H$162,"Pass")</f>
         <v/>
       </c>
       <c r="D19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$161,$A19,'QA Checklist'!$H$5:$H$161,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$161,$A19,'QA Checklist'!$H$5:$H$161,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$162,$A19,'QA Checklist'!$H$5:$H$162,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$162,$A19,'QA Checklist'!$H$5:$H$162,"Fail")</f>
         <v/>
       </c>
       <c r="E19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$161,$A19,'QA Checklist'!$H$5:$H$161,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$162,$A19,'QA Checklist'!$H$5:$H$162,"Pending")</f>
         <v/>
       </c>
       <c r="F19" s="8">
@@ -887,19 +887,19 @@
         </is>
       </c>
       <c r="B20" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$161,$A20)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$162,$A20)</f>
         <v/>
       </c>
       <c r="C20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$161,$A20,'QA Checklist'!$H$5:$H$161,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$161,$A20,'QA Checklist'!$H$5:$H$161,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$162,$A20,'QA Checklist'!$H$5:$H$162,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$162,$A20,'QA Checklist'!$H$5:$H$162,"Pass")</f>
         <v/>
       </c>
       <c r="D20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$161,$A20,'QA Checklist'!$H$5:$H$161,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$161,$A20,'QA Checklist'!$H$5:$H$161,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$162,$A20,'QA Checklist'!$H$5:$H$162,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$162,$A20,'QA Checklist'!$H$5:$H$162,"Fail")</f>
         <v/>
       </c>
       <c r="E20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$161,$A20,'QA Checklist'!$H$5:$H$161,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$162,$A20,'QA Checklist'!$H$5:$H$162,"Pending")</f>
         <v/>
       </c>
       <c r="F20" s="8">
@@ -914,19 +914,19 @@
         </is>
       </c>
       <c r="B21" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$161,$A21)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$162,$A21)</f>
         <v/>
       </c>
       <c r="C21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$161,$A21,'QA Checklist'!$H$5:$H$161,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$161,$A21,'QA Checklist'!$H$5:$H$161,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$162,$A21,'QA Checklist'!$H$5:$H$162,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$162,$A21,'QA Checklist'!$H$5:$H$162,"Pass")</f>
         <v/>
       </c>
       <c r="D21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$161,$A21,'QA Checklist'!$H$5:$H$161,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$161,$A21,'QA Checklist'!$H$5:$H$161,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$162,$A21,'QA Checklist'!$H$5:$H$162,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$162,$A21,'QA Checklist'!$H$5:$H$162,"Fail")</f>
         <v/>
       </c>
       <c r="E21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$161,$A21,'QA Checklist'!$H$5:$H$161,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$162,$A21,'QA Checklist'!$H$5:$H$162,"Pending")</f>
         <v/>
       </c>
       <c r="F21" s="8">
@@ -941,19 +941,19 @@
         </is>
       </c>
       <c r="B22" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$161,$A22)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$162,$A22)</f>
         <v/>
       </c>
       <c r="C22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$161,$A22,'QA Checklist'!$H$5:$H$161,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$161,$A22,'QA Checklist'!$H$5:$H$161,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$162,$A22,'QA Checklist'!$H$5:$H$162,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$162,$A22,'QA Checklist'!$H$5:$H$162,"Pass")</f>
         <v/>
       </c>
       <c r="D22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$161,$A22,'QA Checklist'!$H$5:$H$161,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$161,$A22,'QA Checklist'!$H$5:$H$161,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$162,$A22,'QA Checklist'!$H$5:$H$162,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$162,$A22,'QA Checklist'!$H$5:$H$162,"Fail")</f>
         <v/>
       </c>
       <c r="E22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$161,$A22,'QA Checklist'!$H$5:$H$161,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$162,$A22,'QA Checklist'!$H$5:$H$162,"Pending")</f>
         <v/>
       </c>
       <c r="F22" s="8">
@@ -1023,19 +1023,19 @@
         </is>
       </c>
       <c r="B26" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$161,$A26&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$162,$A26&amp;"*")</f>
         <v/>
       </c>
       <c r="C26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$161,$A26&amp;"*",'QA Checklist'!$H$5:$H$161,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$161,$A26&amp;"*",'QA Checklist'!$H$5:$H$161,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$162,$A26&amp;"*",'QA Checklist'!$H$5:$H$162,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$162,$A26&amp;"*",'QA Checklist'!$H$5:$H$162,"Pass")</f>
         <v/>
       </c>
       <c r="D26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$161,$A26&amp;"*",'QA Checklist'!$H$5:$H$161,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$161,$A26&amp;"*",'QA Checklist'!$H$5:$H$161,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$162,$A26&amp;"*",'QA Checklist'!$H$5:$H$162,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$162,$A26&amp;"*",'QA Checklist'!$H$5:$H$162,"Fail")</f>
         <v/>
       </c>
       <c r="E26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$161,$A26&amp;"*",'QA Checklist'!$H$5:$H$161,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$162,$A26&amp;"*",'QA Checklist'!$H$5:$H$162,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1046,19 +1046,19 @@
         </is>
       </c>
       <c r="B27" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$161,$A27&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$162,$A27&amp;"*")</f>
         <v/>
       </c>
       <c r="C27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$161,$A27&amp;"*",'QA Checklist'!$H$5:$H$161,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$161,$A27&amp;"*",'QA Checklist'!$H$5:$H$161,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$162,$A27&amp;"*",'QA Checklist'!$H$5:$H$162,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$162,$A27&amp;"*",'QA Checklist'!$H$5:$H$162,"Pass")</f>
         <v/>
       </c>
       <c r="D27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$161,$A27&amp;"*",'QA Checklist'!$H$5:$H$161,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$161,$A27&amp;"*",'QA Checklist'!$H$5:$H$161,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$162,$A27&amp;"*",'QA Checklist'!$H$5:$H$162,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$162,$A27&amp;"*",'QA Checklist'!$H$5:$H$162,"Fail")</f>
         <v/>
       </c>
       <c r="E27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$161,$A27&amp;"*",'QA Checklist'!$H$5:$H$161,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$162,$A27&amp;"*",'QA Checklist'!$H$5:$H$162,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1069,19 +1069,19 @@
         </is>
       </c>
       <c r="B28" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$161,$A28&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$162,$A28&amp;"*")</f>
         <v/>
       </c>
       <c r="C28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$161,$A28&amp;"*",'QA Checklist'!$H$5:$H$161,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$161,$A28&amp;"*",'QA Checklist'!$H$5:$H$161,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$162,$A28&amp;"*",'QA Checklist'!$H$5:$H$162,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$162,$A28&amp;"*",'QA Checklist'!$H$5:$H$162,"Pass")</f>
         <v/>
       </c>
       <c r="D28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$161,$A28&amp;"*",'QA Checklist'!$H$5:$H$161,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$161,$A28&amp;"*",'QA Checklist'!$H$5:$H$161,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$162,$A28&amp;"*",'QA Checklist'!$H$5:$H$162,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$162,$A28&amp;"*",'QA Checklist'!$H$5:$H$162,"Fail")</f>
         <v/>
       </c>
       <c r="E28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$161,$A28&amp;"*",'QA Checklist'!$H$5:$H$161,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$162,$A28&amp;"*",'QA Checklist'!$H$5:$H$162,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1096,7 +1096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I161"/>
+  <dimension ref="A1:I162"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8106,12 +8106,59 @@
         </is>
       </c>
     </row>
+    <row r="162">
+      <c r="A162" s="12" t="inlineStr">
+        <is>
+          <t>SA-36</t>
+        </is>
+      </c>
+      <c r="B162" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="C162" s="13" t="inlineStr">
+        <is>
+          <t>Tier 2 (Workflow &amp; Ergonomics)</t>
+        </is>
+      </c>
+      <c r="D162" s="13" t="inlineStr">
+        <is>
+          <t>Checklist Result Measured Status-Box Grid, Header &amp; Signature Alignment</t>
+        </is>
+      </c>
+      <c r="E162" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="F162" s="13" t="inlineStr">
+        <is>
+          <t>Log in as Service Advisor, open 2025 RO Excel Studio, switch to Checklist tab, set a mix of Good / Attention / Defect / N/A statuses across all inspection points, choose a fuel level, optionally tick 'Brakes not inspected', enter comments, and click 'Full PDF' or 'Download PDF'</t>
+        </is>
+      </c>
+      <c r="G162" s="13" t="inlineStr">
+        <is>
+          <t>Each inspection point shows one dark checkmark centered inside the green (Good), yellow (Attention) or red (Defect) box on its own row, and N/A rows stay blank; Battery marks Good or Replace; Brake Pads mark all four wheel boxes or the 'Brakes not inspected' checkbox; Customer Name, Plate Number and Vehicle Year Model sit on their underlines with no caret or 0 artifacts; Date is centered on its underline; the selected fuel level is ringed inside its cell; comments wrap onto the ruled lines; Technician name and customer name are centered on their signature lines</t>
+        </is>
+      </c>
+      <c r="H162" s="14" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="I162" s="13" t="inlineStr">
+        <is>
+          <t>Verified by Automated Unit Tests (148/148 passing in tests/frontend/sla_and_logic.test.js AUT-FRONT-119) and 200 dpi rendered PDF inspection</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:I161"/>
+  <autoFilter ref="A4:I162"/>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="H5:H161">
+  <conditionalFormatting sqref="H5:H162">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$H5="Passed"</formula>
     </cfRule>
@@ -8128,13 +8175,13 @@
       <formula>$H5="Pending"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A5:A161">
+  <conditionalFormatting sqref="A5:A162">
     <cfRule type="expression" priority="6" dxfId="3">
-      <formula>COUNTIF($A$5:$A$161,$A5)&gt;1</formula>
+      <formula>COUNTIF($A$5:$A$162,$A5)&gt;1</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H5:H161" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H5:H162" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pending,Passed,Failed"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat(REV-161): unify checklist UI, PDF and Excel wording, colors and status symbols
Add CHECKLIST_STATUS_STYLES as the single source of truth for status
symbols and printed-form box colors (Good ✓ #2FB044, Attention ⚠ #FFED00,
Defect ✕ #EE1C25). The on-screen checklist now uses the printed form's
section and item wording (older drafts are migrated), paints selected
buttons with the form colors, and offers Good / Replace for the battery.
The PDF and Excel export stamp the same symbol per status; Excel maps
battery Attention to Replace, stops overwriting the printed M41/M59
text, and wraps comments across B53-B56. Bump cache buster to v=3.14,
add AUT-FRONT-120, and sync REV-161 / SA-37 into the revisions log,
checklists and QA workbook.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
+++ b/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
@@ -11,7 +11,7 @@
     <sheet name="QA Checklist" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$162</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$163</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'QA Checklist'!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTA('QA Checklist'!$A$5:$A$162)</f>
+        <f>COUNTA('QA Checklist'!$A$5:$A$163)</f>
         <v/>
       </c>
     </row>
@@ -594,7 +594,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$162,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$162,"Pass")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$163,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$163,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$162,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$162,"Fail")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$163,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$163,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -616,7 +616,7 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$162,"Pending")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$163,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -671,19 +671,19 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$162,$A12)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$163,$A12)</f>
         <v/>
       </c>
       <c r="C12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$162,$A12,'QA Checklist'!$H$5:$H$162,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$162,$A12,'QA Checklist'!$H$5:$H$162,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$163,$A12,'QA Checklist'!$H$5:$H$163,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$163,$A12,'QA Checklist'!$H$5:$H$163,"Pass")</f>
         <v/>
       </c>
       <c r="D12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$162,$A12,'QA Checklist'!$H$5:$H$162,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$162,$A12,'QA Checklist'!$H$5:$H$162,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$163,$A12,'QA Checklist'!$H$5:$H$163,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$163,$A12,'QA Checklist'!$H$5:$H$163,"Fail")</f>
         <v/>
       </c>
       <c r="E12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$162,$A12,'QA Checklist'!$H$5:$H$162,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$163,$A12,'QA Checklist'!$H$5:$H$163,"Pending")</f>
         <v/>
       </c>
       <c r="F12" s="8">
@@ -698,19 +698,19 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$162,$A13)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$163,$A13)</f>
         <v/>
       </c>
       <c r="C13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$162,$A13,'QA Checklist'!$H$5:$H$162,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$162,$A13,'QA Checklist'!$H$5:$H$162,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$163,$A13,'QA Checklist'!$H$5:$H$163,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$163,$A13,'QA Checklist'!$H$5:$H$163,"Pass")</f>
         <v/>
       </c>
       <c r="D13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$162,$A13,'QA Checklist'!$H$5:$H$162,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$162,$A13,'QA Checklist'!$H$5:$H$162,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$163,$A13,'QA Checklist'!$H$5:$H$163,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$163,$A13,'QA Checklist'!$H$5:$H$163,"Fail")</f>
         <v/>
       </c>
       <c r="E13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$162,$A13,'QA Checklist'!$H$5:$H$162,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$163,$A13,'QA Checklist'!$H$5:$H$163,"Pending")</f>
         <v/>
       </c>
       <c r="F13" s="8">
@@ -725,19 +725,19 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$162,$A14)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$163,$A14)</f>
         <v/>
       </c>
       <c r="C14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$162,$A14,'QA Checklist'!$H$5:$H$162,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$162,$A14,'QA Checklist'!$H$5:$H$162,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$163,$A14,'QA Checklist'!$H$5:$H$163,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$163,$A14,'QA Checklist'!$H$5:$H$163,"Pass")</f>
         <v/>
       </c>
       <c r="D14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$162,$A14,'QA Checklist'!$H$5:$H$162,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$162,$A14,'QA Checklist'!$H$5:$H$162,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$163,$A14,'QA Checklist'!$H$5:$H$163,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$163,$A14,'QA Checklist'!$H$5:$H$163,"Fail")</f>
         <v/>
       </c>
       <c r="E14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$162,$A14,'QA Checklist'!$H$5:$H$162,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$163,$A14,'QA Checklist'!$H$5:$H$163,"Pending")</f>
         <v/>
       </c>
       <c r="F14" s="8">
@@ -752,19 +752,19 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$162,$A15)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$163,$A15)</f>
         <v/>
       </c>
       <c r="C15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$162,$A15,'QA Checklist'!$H$5:$H$162,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$162,$A15,'QA Checklist'!$H$5:$H$162,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$163,$A15,'QA Checklist'!$H$5:$H$163,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$163,$A15,'QA Checklist'!$H$5:$H$163,"Pass")</f>
         <v/>
       </c>
       <c r="D15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$162,$A15,'QA Checklist'!$H$5:$H$162,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$162,$A15,'QA Checklist'!$H$5:$H$162,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$163,$A15,'QA Checklist'!$H$5:$H$163,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$163,$A15,'QA Checklist'!$H$5:$H$163,"Fail")</f>
         <v/>
       </c>
       <c r="E15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$162,$A15,'QA Checklist'!$H$5:$H$162,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$163,$A15,'QA Checklist'!$H$5:$H$163,"Pending")</f>
         <v/>
       </c>
       <c r="F15" s="8">
@@ -779,19 +779,19 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$162,$A16)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$163,$A16)</f>
         <v/>
       </c>
       <c r="C16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$162,$A16,'QA Checklist'!$H$5:$H$162,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$162,$A16,'QA Checklist'!$H$5:$H$162,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$163,$A16,'QA Checklist'!$H$5:$H$163,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$163,$A16,'QA Checklist'!$H$5:$H$163,"Pass")</f>
         <v/>
       </c>
       <c r="D16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$162,$A16,'QA Checklist'!$H$5:$H$162,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$162,$A16,'QA Checklist'!$H$5:$H$162,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$163,$A16,'QA Checklist'!$H$5:$H$163,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$163,$A16,'QA Checklist'!$H$5:$H$163,"Fail")</f>
         <v/>
       </c>
       <c r="E16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$162,$A16,'QA Checklist'!$H$5:$H$162,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$163,$A16,'QA Checklist'!$H$5:$H$163,"Pending")</f>
         <v/>
       </c>
       <c r="F16" s="8">
@@ -806,19 +806,19 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$162,$A17)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$163,$A17)</f>
         <v/>
       </c>
       <c r="C17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$162,$A17,'QA Checklist'!$H$5:$H$162,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$162,$A17,'QA Checklist'!$H$5:$H$162,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$163,$A17,'QA Checklist'!$H$5:$H$163,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$163,$A17,'QA Checklist'!$H$5:$H$163,"Pass")</f>
         <v/>
       </c>
       <c r="D17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$162,$A17,'QA Checklist'!$H$5:$H$162,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$162,$A17,'QA Checklist'!$H$5:$H$162,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$163,$A17,'QA Checklist'!$H$5:$H$163,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$163,$A17,'QA Checklist'!$H$5:$H$163,"Fail")</f>
         <v/>
       </c>
       <c r="E17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$162,$A17,'QA Checklist'!$H$5:$H$162,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$163,$A17,'QA Checklist'!$H$5:$H$163,"Pending")</f>
         <v/>
       </c>
       <c r="F17" s="8">
@@ -833,19 +833,19 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$162,$A18)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$163,$A18)</f>
         <v/>
       </c>
       <c r="C18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$162,$A18,'QA Checklist'!$H$5:$H$162,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$162,$A18,'QA Checklist'!$H$5:$H$162,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$163,$A18,'QA Checklist'!$H$5:$H$163,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$163,$A18,'QA Checklist'!$H$5:$H$163,"Pass")</f>
         <v/>
       </c>
       <c r="D18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$162,$A18,'QA Checklist'!$H$5:$H$162,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$162,$A18,'QA Checklist'!$H$5:$H$162,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$163,$A18,'QA Checklist'!$H$5:$H$163,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$163,$A18,'QA Checklist'!$H$5:$H$163,"Fail")</f>
         <v/>
       </c>
       <c r="E18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$162,$A18,'QA Checklist'!$H$5:$H$162,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$163,$A18,'QA Checklist'!$H$5:$H$163,"Pending")</f>
         <v/>
       </c>
       <c r="F18" s="8">
@@ -860,19 +860,19 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$162,$A19)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$163,$A19)</f>
         <v/>
       </c>
       <c r="C19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$162,$A19,'QA Checklist'!$H$5:$H$162,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$162,$A19,'QA Checklist'!$H$5:$H$162,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$163,$A19,'QA Checklist'!$H$5:$H$163,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$163,$A19,'QA Checklist'!$H$5:$H$163,"Pass")</f>
         <v/>
       </c>
       <c r="D19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$162,$A19,'QA Checklist'!$H$5:$H$162,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$162,$A19,'QA Checklist'!$H$5:$H$162,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$163,$A19,'QA Checklist'!$H$5:$H$163,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$163,$A19,'QA Checklist'!$H$5:$H$163,"Fail")</f>
         <v/>
       </c>
       <c r="E19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$162,$A19,'QA Checklist'!$H$5:$H$162,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$163,$A19,'QA Checklist'!$H$5:$H$163,"Pending")</f>
         <v/>
       </c>
       <c r="F19" s="8">
@@ -887,19 +887,19 @@
         </is>
       </c>
       <c r="B20" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$162,$A20)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$163,$A20)</f>
         <v/>
       </c>
       <c r="C20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$162,$A20,'QA Checklist'!$H$5:$H$162,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$162,$A20,'QA Checklist'!$H$5:$H$162,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$163,$A20,'QA Checklist'!$H$5:$H$163,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$163,$A20,'QA Checklist'!$H$5:$H$163,"Pass")</f>
         <v/>
       </c>
       <c r="D20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$162,$A20,'QA Checklist'!$H$5:$H$162,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$162,$A20,'QA Checklist'!$H$5:$H$162,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$163,$A20,'QA Checklist'!$H$5:$H$163,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$163,$A20,'QA Checklist'!$H$5:$H$163,"Fail")</f>
         <v/>
       </c>
       <c r="E20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$162,$A20,'QA Checklist'!$H$5:$H$162,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$163,$A20,'QA Checklist'!$H$5:$H$163,"Pending")</f>
         <v/>
       </c>
       <c r="F20" s="8">
@@ -914,19 +914,19 @@
         </is>
       </c>
       <c r="B21" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$162,$A21)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$163,$A21)</f>
         <v/>
       </c>
       <c r="C21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$162,$A21,'QA Checklist'!$H$5:$H$162,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$162,$A21,'QA Checklist'!$H$5:$H$162,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$163,$A21,'QA Checklist'!$H$5:$H$163,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$163,$A21,'QA Checklist'!$H$5:$H$163,"Pass")</f>
         <v/>
       </c>
       <c r="D21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$162,$A21,'QA Checklist'!$H$5:$H$162,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$162,$A21,'QA Checklist'!$H$5:$H$162,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$163,$A21,'QA Checklist'!$H$5:$H$163,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$163,$A21,'QA Checklist'!$H$5:$H$163,"Fail")</f>
         <v/>
       </c>
       <c r="E21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$162,$A21,'QA Checklist'!$H$5:$H$162,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$163,$A21,'QA Checklist'!$H$5:$H$163,"Pending")</f>
         <v/>
       </c>
       <c r="F21" s="8">
@@ -941,19 +941,19 @@
         </is>
       </c>
       <c r="B22" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$162,$A22)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$163,$A22)</f>
         <v/>
       </c>
       <c r="C22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$162,$A22,'QA Checklist'!$H$5:$H$162,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$162,$A22,'QA Checklist'!$H$5:$H$162,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$163,$A22,'QA Checklist'!$H$5:$H$163,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$163,$A22,'QA Checklist'!$H$5:$H$163,"Pass")</f>
         <v/>
       </c>
       <c r="D22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$162,$A22,'QA Checklist'!$H$5:$H$162,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$162,$A22,'QA Checklist'!$H$5:$H$162,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$163,$A22,'QA Checklist'!$H$5:$H$163,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$163,$A22,'QA Checklist'!$H$5:$H$163,"Fail")</f>
         <v/>
       </c>
       <c r="E22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$162,$A22,'QA Checklist'!$H$5:$H$162,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$163,$A22,'QA Checklist'!$H$5:$H$163,"Pending")</f>
         <v/>
       </c>
       <c r="F22" s="8">
@@ -1023,19 +1023,19 @@
         </is>
       </c>
       <c r="B26" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$162,$A26&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$163,$A26&amp;"*")</f>
         <v/>
       </c>
       <c r="C26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$162,$A26&amp;"*",'QA Checklist'!$H$5:$H$162,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$162,$A26&amp;"*",'QA Checklist'!$H$5:$H$162,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$163,$A26&amp;"*",'QA Checklist'!$H$5:$H$163,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$163,$A26&amp;"*",'QA Checklist'!$H$5:$H$163,"Pass")</f>
         <v/>
       </c>
       <c r="D26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$162,$A26&amp;"*",'QA Checklist'!$H$5:$H$162,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$162,$A26&amp;"*",'QA Checklist'!$H$5:$H$162,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$163,$A26&amp;"*",'QA Checklist'!$H$5:$H$163,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$163,$A26&amp;"*",'QA Checklist'!$H$5:$H$163,"Fail")</f>
         <v/>
       </c>
       <c r="E26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$162,$A26&amp;"*",'QA Checklist'!$H$5:$H$162,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$163,$A26&amp;"*",'QA Checklist'!$H$5:$H$163,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1046,19 +1046,19 @@
         </is>
       </c>
       <c r="B27" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$162,$A27&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$163,$A27&amp;"*")</f>
         <v/>
       </c>
       <c r="C27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$162,$A27&amp;"*",'QA Checklist'!$H$5:$H$162,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$162,$A27&amp;"*",'QA Checklist'!$H$5:$H$162,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$163,$A27&amp;"*",'QA Checklist'!$H$5:$H$163,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$163,$A27&amp;"*",'QA Checklist'!$H$5:$H$163,"Pass")</f>
         <v/>
       </c>
       <c r="D27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$162,$A27&amp;"*",'QA Checklist'!$H$5:$H$162,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$162,$A27&amp;"*",'QA Checklist'!$H$5:$H$162,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$163,$A27&amp;"*",'QA Checklist'!$H$5:$H$163,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$163,$A27&amp;"*",'QA Checklist'!$H$5:$H$163,"Fail")</f>
         <v/>
       </c>
       <c r="E27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$162,$A27&amp;"*",'QA Checklist'!$H$5:$H$162,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$163,$A27&amp;"*",'QA Checklist'!$H$5:$H$163,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1069,19 +1069,19 @@
         </is>
       </c>
       <c r="B28" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$162,$A28&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$163,$A28&amp;"*")</f>
         <v/>
       </c>
       <c r="C28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$162,$A28&amp;"*",'QA Checklist'!$H$5:$H$162,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$162,$A28&amp;"*",'QA Checklist'!$H$5:$H$162,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$163,$A28&amp;"*",'QA Checklist'!$H$5:$H$163,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$163,$A28&amp;"*",'QA Checklist'!$H$5:$H$163,"Pass")</f>
         <v/>
       </c>
       <c r="D28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$162,$A28&amp;"*",'QA Checklist'!$H$5:$H$162,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$162,$A28&amp;"*",'QA Checklist'!$H$5:$H$162,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$163,$A28&amp;"*",'QA Checklist'!$H$5:$H$163,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$163,$A28&amp;"*",'QA Checklist'!$H$5:$H$163,"Fail")</f>
         <v/>
       </c>
       <c r="E28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$162,$A28&amp;"*",'QA Checklist'!$H$5:$H$162,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$163,$A28&amp;"*",'QA Checklist'!$H$5:$H$163,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1096,7 +1096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I162"/>
+  <dimension ref="A1:I163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8153,12 +8153,59 @@
         </is>
       </c>
     </row>
+    <row r="163">
+      <c r="A163" s="12" t="inlineStr">
+        <is>
+          <t>SA-37</t>
+        </is>
+      </c>
+      <c r="B163" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="C163" s="13" t="inlineStr">
+        <is>
+          <t>Tier 2 (Workflow &amp; Ergonomics)</t>
+        </is>
+      </c>
+      <c r="D163" s="13" t="inlineStr">
+        <is>
+          <t>Checklist UI, PDF &amp; Excel Unified Wording, Colors &amp; Status Symbols</t>
+        </is>
+      </c>
+      <c r="E163" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="F163" s="13" t="inlineStr">
+        <is>
+          <t>Log in as Service Advisor, open 2025 RO Excel Studio, switch to Checklist tab, set a mix of Good / Attention / Defect / N/A statuses (battery Good or Replace), enter comments, then click 'Full PDF' and 'Export Excel' and compare all three</t>
+        </is>
+      </c>
+      <c r="G163" s="13" t="inlineStr">
+        <is>
+          <t>On-screen sections and items use the printed form wording (Interior/Exterior, Battery Performance, Under Hood, Under Vehicle, Tire Condition, Brake Condition); selected buttons use the form colors (green Good, yellow Attention, red Defect) with the form legend; the PDF and Excel show the same symbol as the button (✓ / ⚠ / ✕) in the matching green / yellow / red box, with N/A rows blank; battery shows Good or Replace consistently in all three; the Excel sheet keeps the printed 'Please Indicate Areas of External Damage or Wear' and brake fluid note text, and comments wrap across the Comments lines</t>
+        </is>
+      </c>
+      <c r="H163" s="14" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="I163" s="13" t="inlineStr">
+        <is>
+          <t>Verified by Automated Unit Tests (149/149 passing in tests/frontend/sla_and_logic.test.js AUT-FRONT-120) and headless Chrome UI render, PDF render and real Excel export read back with openpyxl</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:I162"/>
+  <autoFilter ref="A4:I163"/>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="H5:H162">
+  <conditionalFormatting sqref="H5:H163">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$H5="Passed"</formula>
     </cfRule>
@@ -8175,13 +8222,13 @@
       <formula>$H5="Pending"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A5:A162">
+  <conditionalFormatting sqref="A5:A163">
     <cfRule type="expression" priority="6" dxfId="3">
-      <formula>COUNTIF($A$5:$A$162,$A5)&gt;1</formula>
+      <formula>COUNTIF($A$5:$A$163,$A5)&gt;1</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H5:H162" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H5:H163" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pending,Passed,Failed"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat(REV-162): move brakes-not-inspected checkbox below checklist checkpoints
Move the "Brakes not inspected on this visit" toggle (Sheet 7: M37) from
the top of the Multi-Point Receiving Checkpoints card to the bottom,
directly before Inspector Remarks / Discovered Deficiencies, matching
its position below Brake Condition on the printed form. Bump cache
buster to v=3.15, add AUT-FRONT-121, and sync REV-162 / SA-38 into the
revisions log, checklists and QA workbook.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
+++ b/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
@@ -11,7 +11,7 @@
     <sheet name="QA Checklist" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$163</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$164</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'QA Checklist'!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTA('QA Checklist'!$A$5:$A$163)</f>
+        <f>COUNTA('QA Checklist'!$A$5:$A$164)</f>
         <v/>
       </c>
     </row>
@@ -594,7 +594,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$163,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$163,"Pass")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$164,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$164,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$163,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$163,"Fail")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$164,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$164,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -616,7 +616,7 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$163,"Pending")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$164,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -671,19 +671,19 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$163,$A12)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$164,$A12)</f>
         <v/>
       </c>
       <c r="C12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$163,$A12,'QA Checklist'!$H$5:$H$163,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$163,$A12,'QA Checklist'!$H$5:$H$163,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$164,$A12,'QA Checklist'!$H$5:$H$164,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$164,$A12,'QA Checklist'!$H$5:$H$164,"Pass")</f>
         <v/>
       </c>
       <c r="D12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$163,$A12,'QA Checklist'!$H$5:$H$163,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$163,$A12,'QA Checklist'!$H$5:$H$163,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$164,$A12,'QA Checklist'!$H$5:$H$164,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$164,$A12,'QA Checklist'!$H$5:$H$164,"Fail")</f>
         <v/>
       </c>
       <c r="E12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$163,$A12,'QA Checklist'!$H$5:$H$163,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$164,$A12,'QA Checklist'!$H$5:$H$164,"Pending")</f>
         <v/>
       </c>
       <c r="F12" s="8">
@@ -698,19 +698,19 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$163,$A13)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$164,$A13)</f>
         <v/>
       </c>
       <c r="C13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$163,$A13,'QA Checklist'!$H$5:$H$163,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$163,$A13,'QA Checklist'!$H$5:$H$163,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$164,$A13,'QA Checklist'!$H$5:$H$164,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$164,$A13,'QA Checklist'!$H$5:$H$164,"Pass")</f>
         <v/>
       </c>
       <c r="D13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$163,$A13,'QA Checklist'!$H$5:$H$163,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$163,$A13,'QA Checklist'!$H$5:$H$163,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$164,$A13,'QA Checklist'!$H$5:$H$164,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$164,$A13,'QA Checklist'!$H$5:$H$164,"Fail")</f>
         <v/>
       </c>
       <c r="E13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$163,$A13,'QA Checklist'!$H$5:$H$163,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$164,$A13,'QA Checklist'!$H$5:$H$164,"Pending")</f>
         <v/>
       </c>
       <c r="F13" s="8">
@@ -725,19 +725,19 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$163,$A14)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$164,$A14)</f>
         <v/>
       </c>
       <c r="C14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$163,$A14,'QA Checklist'!$H$5:$H$163,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$163,$A14,'QA Checklist'!$H$5:$H$163,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$164,$A14,'QA Checklist'!$H$5:$H$164,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$164,$A14,'QA Checklist'!$H$5:$H$164,"Pass")</f>
         <v/>
       </c>
       <c r="D14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$163,$A14,'QA Checklist'!$H$5:$H$163,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$163,$A14,'QA Checklist'!$H$5:$H$163,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$164,$A14,'QA Checklist'!$H$5:$H$164,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$164,$A14,'QA Checklist'!$H$5:$H$164,"Fail")</f>
         <v/>
       </c>
       <c r="E14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$163,$A14,'QA Checklist'!$H$5:$H$163,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$164,$A14,'QA Checklist'!$H$5:$H$164,"Pending")</f>
         <v/>
       </c>
       <c r="F14" s="8">
@@ -752,19 +752,19 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$163,$A15)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$164,$A15)</f>
         <v/>
       </c>
       <c r="C15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$163,$A15,'QA Checklist'!$H$5:$H$163,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$163,$A15,'QA Checklist'!$H$5:$H$163,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$164,$A15,'QA Checklist'!$H$5:$H$164,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$164,$A15,'QA Checklist'!$H$5:$H$164,"Pass")</f>
         <v/>
       </c>
       <c r="D15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$163,$A15,'QA Checklist'!$H$5:$H$163,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$163,$A15,'QA Checklist'!$H$5:$H$163,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$164,$A15,'QA Checklist'!$H$5:$H$164,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$164,$A15,'QA Checklist'!$H$5:$H$164,"Fail")</f>
         <v/>
       </c>
       <c r="E15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$163,$A15,'QA Checklist'!$H$5:$H$163,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$164,$A15,'QA Checklist'!$H$5:$H$164,"Pending")</f>
         <v/>
       </c>
       <c r="F15" s="8">
@@ -779,19 +779,19 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$163,$A16)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$164,$A16)</f>
         <v/>
       </c>
       <c r="C16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$163,$A16,'QA Checklist'!$H$5:$H$163,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$163,$A16,'QA Checklist'!$H$5:$H$163,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$164,$A16,'QA Checklist'!$H$5:$H$164,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$164,$A16,'QA Checklist'!$H$5:$H$164,"Pass")</f>
         <v/>
       </c>
       <c r="D16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$163,$A16,'QA Checklist'!$H$5:$H$163,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$163,$A16,'QA Checklist'!$H$5:$H$163,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$164,$A16,'QA Checklist'!$H$5:$H$164,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$164,$A16,'QA Checklist'!$H$5:$H$164,"Fail")</f>
         <v/>
       </c>
       <c r="E16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$163,$A16,'QA Checklist'!$H$5:$H$163,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$164,$A16,'QA Checklist'!$H$5:$H$164,"Pending")</f>
         <v/>
       </c>
       <c r="F16" s="8">
@@ -806,19 +806,19 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$163,$A17)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$164,$A17)</f>
         <v/>
       </c>
       <c r="C17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$163,$A17,'QA Checklist'!$H$5:$H$163,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$163,$A17,'QA Checklist'!$H$5:$H$163,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$164,$A17,'QA Checklist'!$H$5:$H$164,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$164,$A17,'QA Checklist'!$H$5:$H$164,"Pass")</f>
         <v/>
       </c>
       <c r="D17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$163,$A17,'QA Checklist'!$H$5:$H$163,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$163,$A17,'QA Checklist'!$H$5:$H$163,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$164,$A17,'QA Checklist'!$H$5:$H$164,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$164,$A17,'QA Checklist'!$H$5:$H$164,"Fail")</f>
         <v/>
       </c>
       <c r="E17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$163,$A17,'QA Checklist'!$H$5:$H$163,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$164,$A17,'QA Checklist'!$H$5:$H$164,"Pending")</f>
         <v/>
       </c>
       <c r="F17" s="8">
@@ -833,19 +833,19 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$163,$A18)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$164,$A18)</f>
         <v/>
       </c>
       <c r="C18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$163,$A18,'QA Checklist'!$H$5:$H$163,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$163,$A18,'QA Checklist'!$H$5:$H$163,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$164,$A18,'QA Checklist'!$H$5:$H$164,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$164,$A18,'QA Checklist'!$H$5:$H$164,"Pass")</f>
         <v/>
       </c>
       <c r="D18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$163,$A18,'QA Checklist'!$H$5:$H$163,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$163,$A18,'QA Checklist'!$H$5:$H$163,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$164,$A18,'QA Checklist'!$H$5:$H$164,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$164,$A18,'QA Checklist'!$H$5:$H$164,"Fail")</f>
         <v/>
       </c>
       <c r="E18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$163,$A18,'QA Checklist'!$H$5:$H$163,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$164,$A18,'QA Checklist'!$H$5:$H$164,"Pending")</f>
         <v/>
       </c>
       <c r="F18" s="8">
@@ -860,19 +860,19 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$163,$A19)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$164,$A19)</f>
         <v/>
       </c>
       <c r="C19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$163,$A19,'QA Checklist'!$H$5:$H$163,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$163,$A19,'QA Checklist'!$H$5:$H$163,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$164,$A19,'QA Checklist'!$H$5:$H$164,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$164,$A19,'QA Checklist'!$H$5:$H$164,"Pass")</f>
         <v/>
       </c>
       <c r="D19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$163,$A19,'QA Checklist'!$H$5:$H$163,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$163,$A19,'QA Checklist'!$H$5:$H$163,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$164,$A19,'QA Checklist'!$H$5:$H$164,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$164,$A19,'QA Checklist'!$H$5:$H$164,"Fail")</f>
         <v/>
       </c>
       <c r="E19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$163,$A19,'QA Checklist'!$H$5:$H$163,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$164,$A19,'QA Checklist'!$H$5:$H$164,"Pending")</f>
         <v/>
       </c>
       <c r="F19" s="8">
@@ -887,19 +887,19 @@
         </is>
       </c>
       <c r="B20" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$163,$A20)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$164,$A20)</f>
         <v/>
       </c>
       <c r="C20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$163,$A20,'QA Checklist'!$H$5:$H$163,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$163,$A20,'QA Checklist'!$H$5:$H$163,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$164,$A20,'QA Checklist'!$H$5:$H$164,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$164,$A20,'QA Checklist'!$H$5:$H$164,"Pass")</f>
         <v/>
       </c>
       <c r="D20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$163,$A20,'QA Checklist'!$H$5:$H$163,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$163,$A20,'QA Checklist'!$H$5:$H$163,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$164,$A20,'QA Checklist'!$H$5:$H$164,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$164,$A20,'QA Checklist'!$H$5:$H$164,"Fail")</f>
         <v/>
       </c>
       <c r="E20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$163,$A20,'QA Checklist'!$H$5:$H$163,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$164,$A20,'QA Checklist'!$H$5:$H$164,"Pending")</f>
         <v/>
       </c>
       <c r="F20" s="8">
@@ -914,19 +914,19 @@
         </is>
       </c>
       <c r="B21" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$163,$A21)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$164,$A21)</f>
         <v/>
       </c>
       <c r="C21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$163,$A21,'QA Checklist'!$H$5:$H$163,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$163,$A21,'QA Checklist'!$H$5:$H$163,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$164,$A21,'QA Checklist'!$H$5:$H$164,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$164,$A21,'QA Checklist'!$H$5:$H$164,"Pass")</f>
         <v/>
       </c>
       <c r="D21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$163,$A21,'QA Checklist'!$H$5:$H$163,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$163,$A21,'QA Checklist'!$H$5:$H$163,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$164,$A21,'QA Checklist'!$H$5:$H$164,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$164,$A21,'QA Checklist'!$H$5:$H$164,"Fail")</f>
         <v/>
       </c>
       <c r="E21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$163,$A21,'QA Checklist'!$H$5:$H$163,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$164,$A21,'QA Checklist'!$H$5:$H$164,"Pending")</f>
         <v/>
       </c>
       <c r="F21" s="8">
@@ -941,19 +941,19 @@
         </is>
       </c>
       <c r="B22" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$163,$A22)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$164,$A22)</f>
         <v/>
       </c>
       <c r="C22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$163,$A22,'QA Checklist'!$H$5:$H$163,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$163,$A22,'QA Checklist'!$H$5:$H$163,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$164,$A22,'QA Checklist'!$H$5:$H$164,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$164,$A22,'QA Checklist'!$H$5:$H$164,"Pass")</f>
         <v/>
       </c>
       <c r="D22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$163,$A22,'QA Checklist'!$H$5:$H$163,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$163,$A22,'QA Checklist'!$H$5:$H$163,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$164,$A22,'QA Checklist'!$H$5:$H$164,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$164,$A22,'QA Checklist'!$H$5:$H$164,"Fail")</f>
         <v/>
       </c>
       <c r="E22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$163,$A22,'QA Checklist'!$H$5:$H$163,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$164,$A22,'QA Checklist'!$H$5:$H$164,"Pending")</f>
         <v/>
       </c>
       <c r="F22" s="8">
@@ -1023,19 +1023,19 @@
         </is>
       </c>
       <c r="B26" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$163,$A26&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$164,$A26&amp;"*")</f>
         <v/>
       </c>
       <c r="C26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$163,$A26&amp;"*",'QA Checklist'!$H$5:$H$163,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$163,$A26&amp;"*",'QA Checklist'!$H$5:$H$163,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$164,$A26&amp;"*",'QA Checklist'!$H$5:$H$164,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$164,$A26&amp;"*",'QA Checklist'!$H$5:$H$164,"Pass")</f>
         <v/>
       </c>
       <c r="D26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$163,$A26&amp;"*",'QA Checklist'!$H$5:$H$163,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$163,$A26&amp;"*",'QA Checklist'!$H$5:$H$163,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$164,$A26&amp;"*",'QA Checklist'!$H$5:$H$164,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$164,$A26&amp;"*",'QA Checklist'!$H$5:$H$164,"Fail")</f>
         <v/>
       </c>
       <c r="E26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$163,$A26&amp;"*",'QA Checklist'!$H$5:$H$163,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$164,$A26&amp;"*",'QA Checklist'!$H$5:$H$164,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1046,19 +1046,19 @@
         </is>
       </c>
       <c r="B27" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$163,$A27&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$164,$A27&amp;"*")</f>
         <v/>
       </c>
       <c r="C27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$163,$A27&amp;"*",'QA Checklist'!$H$5:$H$163,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$163,$A27&amp;"*",'QA Checklist'!$H$5:$H$163,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$164,$A27&amp;"*",'QA Checklist'!$H$5:$H$164,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$164,$A27&amp;"*",'QA Checklist'!$H$5:$H$164,"Pass")</f>
         <v/>
       </c>
       <c r="D27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$163,$A27&amp;"*",'QA Checklist'!$H$5:$H$163,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$163,$A27&amp;"*",'QA Checklist'!$H$5:$H$163,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$164,$A27&amp;"*",'QA Checklist'!$H$5:$H$164,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$164,$A27&amp;"*",'QA Checklist'!$H$5:$H$164,"Fail")</f>
         <v/>
       </c>
       <c r="E27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$163,$A27&amp;"*",'QA Checklist'!$H$5:$H$163,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$164,$A27&amp;"*",'QA Checklist'!$H$5:$H$164,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1069,19 +1069,19 @@
         </is>
       </c>
       <c r="B28" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$163,$A28&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$164,$A28&amp;"*")</f>
         <v/>
       </c>
       <c r="C28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$163,$A28&amp;"*",'QA Checklist'!$H$5:$H$163,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$163,$A28&amp;"*",'QA Checklist'!$H$5:$H$163,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$164,$A28&amp;"*",'QA Checklist'!$H$5:$H$164,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$164,$A28&amp;"*",'QA Checklist'!$H$5:$H$164,"Pass")</f>
         <v/>
       </c>
       <c r="D28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$163,$A28&amp;"*",'QA Checklist'!$H$5:$H$163,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$163,$A28&amp;"*",'QA Checklist'!$H$5:$H$163,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$164,$A28&amp;"*",'QA Checklist'!$H$5:$H$164,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$164,$A28&amp;"*",'QA Checklist'!$H$5:$H$164,"Fail")</f>
         <v/>
       </c>
       <c r="E28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$163,$A28&amp;"*",'QA Checklist'!$H$5:$H$163,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$164,$A28&amp;"*",'QA Checklist'!$H$5:$H$164,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1096,7 +1096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I163"/>
+  <dimension ref="A1:I164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8200,12 +8200,59 @@
         </is>
       </c>
     </row>
+    <row r="164">
+      <c r="A164" s="12" t="inlineStr">
+        <is>
+          <t>SA-38</t>
+        </is>
+      </c>
+      <c r="B164" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="C164" s="13" t="inlineStr">
+        <is>
+          <t>Tier 2 (Workflow &amp; Ergonomics)</t>
+        </is>
+      </c>
+      <c r="D164" s="13" t="inlineStr">
+        <is>
+          <t>Checklist Brakes-Not-Inspected Checkbox Placement</t>
+        </is>
+      </c>
+      <c r="E164" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="F164" s="13" t="inlineStr">
+        <is>
+          <t>Log in as Service Advisor, open 2025 RO Excel Studio, switch to Checklist tab, scroll the Multi-Point Receiving Checkpoints card to the bottom, and tick / untick 'Brakes not inspected on this visit'</t>
+        </is>
+      </c>
+      <c r="G164" s="13" t="inlineStr">
+        <is>
+          <t>The 'Brakes not inspected on this visit' checkbox appears once, at the bottom of the Multi-Point Receiving Checkpoints card after the checkpoint list and directly above Inspector Remarks / Discovered Deficiencies; ticking it still marks the 'Brakes not inspected' box on the Checklist PDF and Excel (M37)</t>
+        </is>
+      </c>
+      <c r="H164" s="14" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="I164" s="13" t="inlineStr">
+        <is>
+          <t>Verified by Automated Unit Tests (150/150 passing in tests/frontend/sla_and_logic.test.js AUT-FRONT-121) and headless Chrome render inspection</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:I163"/>
+  <autoFilter ref="A4:I164"/>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="H5:H163">
+  <conditionalFormatting sqref="H5:H164">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$H5="Passed"</formula>
     </cfRule>
@@ -8222,13 +8269,13 @@
       <formula>$H5="Pending"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A5:A163">
+  <conditionalFormatting sqref="A5:A164">
     <cfRule type="expression" priority="6" dxfId="3">
-      <formula>COUNTIF($A$5:$A$163,$A5)&gt;1</formula>
+      <formula>COUNTIF($A$5:$A$164,$A5)&gt;1</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H5:H163" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H5:H164" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pending,Passed,Failed"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat(REV-163): professional neutral CheckList Studio redesign and fuel selector fix
Restyle the CheckList Studio editor in a neutral gray scale with Export
.xlsx as the single dark primary action: flat sections, outlined
secondary buttons, gray focus rings, a segmented fuel control and a
neutral segmented status control per checkpoint. The printed form's
green / yellow / red remain only as small swatches. Fix setChecklistFuel,
which looked buttons up by non-existent ids so the highlight never moved
and the fuel label never updated. PDF and Excel output are unchanged.
Bump cache buster to v=3.16, add AUT-FRONT-122, and sync REV-163 / SA-39
into the revisions log, checklists and QA workbook.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
+++ b/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
@@ -11,7 +11,7 @@
     <sheet name="QA Checklist" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$164</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$165</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'QA Checklist'!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTA('QA Checklist'!$A$5:$A$164)</f>
+        <f>COUNTA('QA Checklist'!$A$5:$A$165)</f>
         <v/>
       </c>
     </row>
@@ -594,7 +594,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$164,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$164,"Pass")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$165,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$165,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$164,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$164,"Fail")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$165,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$165,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -616,7 +616,7 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$164,"Pending")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$165,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -671,19 +671,19 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$164,$A12)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$165,$A12)</f>
         <v/>
       </c>
       <c r="C12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$164,$A12,'QA Checklist'!$H$5:$H$164,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$164,$A12,'QA Checklist'!$H$5:$H$164,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$165,$A12,'QA Checklist'!$H$5:$H$165,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$165,$A12,'QA Checklist'!$H$5:$H$165,"Pass")</f>
         <v/>
       </c>
       <c r="D12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$164,$A12,'QA Checklist'!$H$5:$H$164,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$164,$A12,'QA Checklist'!$H$5:$H$164,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$165,$A12,'QA Checklist'!$H$5:$H$165,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$165,$A12,'QA Checklist'!$H$5:$H$165,"Fail")</f>
         <v/>
       </c>
       <c r="E12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$164,$A12,'QA Checklist'!$H$5:$H$164,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$165,$A12,'QA Checklist'!$H$5:$H$165,"Pending")</f>
         <v/>
       </c>
       <c r="F12" s="8">
@@ -698,19 +698,19 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$164,$A13)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$165,$A13)</f>
         <v/>
       </c>
       <c r="C13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$164,$A13,'QA Checklist'!$H$5:$H$164,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$164,$A13,'QA Checklist'!$H$5:$H$164,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$165,$A13,'QA Checklist'!$H$5:$H$165,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$165,$A13,'QA Checklist'!$H$5:$H$165,"Pass")</f>
         <v/>
       </c>
       <c r="D13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$164,$A13,'QA Checklist'!$H$5:$H$164,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$164,$A13,'QA Checklist'!$H$5:$H$164,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$165,$A13,'QA Checklist'!$H$5:$H$165,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$165,$A13,'QA Checklist'!$H$5:$H$165,"Fail")</f>
         <v/>
       </c>
       <c r="E13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$164,$A13,'QA Checklist'!$H$5:$H$164,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$165,$A13,'QA Checklist'!$H$5:$H$165,"Pending")</f>
         <v/>
       </c>
       <c r="F13" s="8">
@@ -725,19 +725,19 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$164,$A14)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$165,$A14)</f>
         <v/>
       </c>
       <c r="C14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$164,$A14,'QA Checklist'!$H$5:$H$164,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$164,$A14,'QA Checklist'!$H$5:$H$164,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$165,$A14,'QA Checklist'!$H$5:$H$165,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$165,$A14,'QA Checklist'!$H$5:$H$165,"Pass")</f>
         <v/>
       </c>
       <c r="D14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$164,$A14,'QA Checklist'!$H$5:$H$164,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$164,$A14,'QA Checklist'!$H$5:$H$164,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$165,$A14,'QA Checklist'!$H$5:$H$165,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$165,$A14,'QA Checklist'!$H$5:$H$165,"Fail")</f>
         <v/>
       </c>
       <c r="E14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$164,$A14,'QA Checklist'!$H$5:$H$164,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$165,$A14,'QA Checklist'!$H$5:$H$165,"Pending")</f>
         <v/>
       </c>
       <c r="F14" s="8">
@@ -752,19 +752,19 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$164,$A15)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$165,$A15)</f>
         <v/>
       </c>
       <c r="C15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$164,$A15,'QA Checklist'!$H$5:$H$164,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$164,$A15,'QA Checklist'!$H$5:$H$164,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$165,$A15,'QA Checklist'!$H$5:$H$165,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$165,$A15,'QA Checklist'!$H$5:$H$165,"Pass")</f>
         <v/>
       </c>
       <c r="D15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$164,$A15,'QA Checklist'!$H$5:$H$164,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$164,$A15,'QA Checklist'!$H$5:$H$164,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$165,$A15,'QA Checklist'!$H$5:$H$165,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$165,$A15,'QA Checklist'!$H$5:$H$165,"Fail")</f>
         <v/>
       </c>
       <c r="E15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$164,$A15,'QA Checklist'!$H$5:$H$164,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$165,$A15,'QA Checklist'!$H$5:$H$165,"Pending")</f>
         <v/>
       </c>
       <c r="F15" s="8">
@@ -779,19 +779,19 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$164,$A16)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$165,$A16)</f>
         <v/>
       </c>
       <c r="C16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$164,$A16,'QA Checklist'!$H$5:$H$164,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$164,$A16,'QA Checklist'!$H$5:$H$164,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$165,$A16,'QA Checklist'!$H$5:$H$165,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$165,$A16,'QA Checklist'!$H$5:$H$165,"Pass")</f>
         <v/>
       </c>
       <c r="D16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$164,$A16,'QA Checklist'!$H$5:$H$164,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$164,$A16,'QA Checklist'!$H$5:$H$164,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$165,$A16,'QA Checklist'!$H$5:$H$165,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$165,$A16,'QA Checklist'!$H$5:$H$165,"Fail")</f>
         <v/>
       </c>
       <c r="E16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$164,$A16,'QA Checklist'!$H$5:$H$164,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$165,$A16,'QA Checklist'!$H$5:$H$165,"Pending")</f>
         <v/>
       </c>
       <c r="F16" s="8">
@@ -806,19 +806,19 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$164,$A17)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$165,$A17)</f>
         <v/>
       </c>
       <c r="C17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$164,$A17,'QA Checklist'!$H$5:$H$164,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$164,$A17,'QA Checklist'!$H$5:$H$164,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$165,$A17,'QA Checklist'!$H$5:$H$165,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$165,$A17,'QA Checklist'!$H$5:$H$165,"Pass")</f>
         <v/>
       </c>
       <c r="D17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$164,$A17,'QA Checklist'!$H$5:$H$164,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$164,$A17,'QA Checklist'!$H$5:$H$164,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$165,$A17,'QA Checklist'!$H$5:$H$165,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$165,$A17,'QA Checklist'!$H$5:$H$165,"Fail")</f>
         <v/>
       </c>
       <c r="E17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$164,$A17,'QA Checklist'!$H$5:$H$164,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$165,$A17,'QA Checklist'!$H$5:$H$165,"Pending")</f>
         <v/>
       </c>
       <c r="F17" s="8">
@@ -833,19 +833,19 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$164,$A18)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$165,$A18)</f>
         <v/>
       </c>
       <c r="C18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$164,$A18,'QA Checklist'!$H$5:$H$164,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$164,$A18,'QA Checklist'!$H$5:$H$164,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$165,$A18,'QA Checklist'!$H$5:$H$165,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$165,$A18,'QA Checklist'!$H$5:$H$165,"Pass")</f>
         <v/>
       </c>
       <c r="D18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$164,$A18,'QA Checklist'!$H$5:$H$164,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$164,$A18,'QA Checklist'!$H$5:$H$164,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$165,$A18,'QA Checklist'!$H$5:$H$165,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$165,$A18,'QA Checklist'!$H$5:$H$165,"Fail")</f>
         <v/>
       </c>
       <c r="E18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$164,$A18,'QA Checklist'!$H$5:$H$164,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$165,$A18,'QA Checklist'!$H$5:$H$165,"Pending")</f>
         <v/>
       </c>
       <c r="F18" s="8">
@@ -860,19 +860,19 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$164,$A19)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$165,$A19)</f>
         <v/>
       </c>
       <c r="C19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$164,$A19,'QA Checklist'!$H$5:$H$164,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$164,$A19,'QA Checklist'!$H$5:$H$164,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$165,$A19,'QA Checklist'!$H$5:$H$165,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$165,$A19,'QA Checklist'!$H$5:$H$165,"Pass")</f>
         <v/>
       </c>
       <c r="D19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$164,$A19,'QA Checklist'!$H$5:$H$164,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$164,$A19,'QA Checklist'!$H$5:$H$164,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$165,$A19,'QA Checklist'!$H$5:$H$165,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$165,$A19,'QA Checklist'!$H$5:$H$165,"Fail")</f>
         <v/>
       </c>
       <c r="E19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$164,$A19,'QA Checklist'!$H$5:$H$164,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$165,$A19,'QA Checklist'!$H$5:$H$165,"Pending")</f>
         <v/>
       </c>
       <c r="F19" s="8">
@@ -887,19 +887,19 @@
         </is>
       </c>
       <c r="B20" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$164,$A20)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$165,$A20)</f>
         <v/>
       </c>
       <c r="C20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$164,$A20,'QA Checklist'!$H$5:$H$164,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$164,$A20,'QA Checklist'!$H$5:$H$164,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$165,$A20,'QA Checklist'!$H$5:$H$165,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$165,$A20,'QA Checklist'!$H$5:$H$165,"Pass")</f>
         <v/>
       </c>
       <c r="D20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$164,$A20,'QA Checklist'!$H$5:$H$164,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$164,$A20,'QA Checklist'!$H$5:$H$164,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$165,$A20,'QA Checklist'!$H$5:$H$165,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$165,$A20,'QA Checklist'!$H$5:$H$165,"Fail")</f>
         <v/>
       </c>
       <c r="E20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$164,$A20,'QA Checklist'!$H$5:$H$164,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$165,$A20,'QA Checklist'!$H$5:$H$165,"Pending")</f>
         <v/>
       </c>
       <c r="F20" s="8">
@@ -914,19 +914,19 @@
         </is>
       </c>
       <c r="B21" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$164,$A21)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$165,$A21)</f>
         <v/>
       </c>
       <c r="C21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$164,$A21,'QA Checklist'!$H$5:$H$164,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$164,$A21,'QA Checklist'!$H$5:$H$164,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$165,$A21,'QA Checklist'!$H$5:$H$165,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$165,$A21,'QA Checklist'!$H$5:$H$165,"Pass")</f>
         <v/>
       </c>
       <c r="D21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$164,$A21,'QA Checklist'!$H$5:$H$164,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$164,$A21,'QA Checklist'!$H$5:$H$164,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$165,$A21,'QA Checklist'!$H$5:$H$165,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$165,$A21,'QA Checklist'!$H$5:$H$165,"Fail")</f>
         <v/>
       </c>
       <c r="E21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$164,$A21,'QA Checklist'!$H$5:$H$164,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$165,$A21,'QA Checklist'!$H$5:$H$165,"Pending")</f>
         <v/>
       </c>
       <c r="F21" s="8">
@@ -941,19 +941,19 @@
         </is>
       </c>
       <c r="B22" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$164,$A22)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$165,$A22)</f>
         <v/>
       </c>
       <c r="C22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$164,$A22,'QA Checklist'!$H$5:$H$164,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$164,$A22,'QA Checklist'!$H$5:$H$164,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$165,$A22,'QA Checklist'!$H$5:$H$165,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$165,$A22,'QA Checklist'!$H$5:$H$165,"Pass")</f>
         <v/>
       </c>
       <c r="D22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$164,$A22,'QA Checklist'!$H$5:$H$164,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$164,$A22,'QA Checklist'!$H$5:$H$164,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$165,$A22,'QA Checklist'!$H$5:$H$165,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$165,$A22,'QA Checklist'!$H$5:$H$165,"Fail")</f>
         <v/>
       </c>
       <c r="E22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$164,$A22,'QA Checklist'!$H$5:$H$164,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$165,$A22,'QA Checklist'!$H$5:$H$165,"Pending")</f>
         <v/>
       </c>
       <c r="F22" s="8">
@@ -1023,19 +1023,19 @@
         </is>
       </c>
       <c r="B26" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$164,$A26&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$165,$A26&amp;"*")</f>
         <v/>
       </c>
       <c r="C26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$164,$A26&amp;"*",'QA Checklist'!$H$5:$H$164,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$164,$A26&amp;"*",'QA Checklist'!$H$5:$H$164,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$165,$A26&amp;"*",'QA Checklist'!$H$5:$H$165,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$165,$A26&amp;"*",'QA Checklist'!$H$5:$H$165,"Pass")</f>
         <v/>
       </c>
       <c r="D26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$164,$A26&amp;"*",'QA Checklist'!$H$5:$H$164,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$164,$A26&amp;"*",'QA Checklist'!$H$5:$H$164,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$165,$A26&amp;"*",'QA Checklist'!$H$5:$H$165,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$165,$A26&amp;"*",'QA Checklist'!$H$5:$H$165,"Fail")</f>
         <v/>
       </c>
       <c r="E26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$164,$A26&amp;"*",'QA Checklist'!$H$5:$H$164,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$165,$A26&amp;"*",'QA Checklist'!$H$5:$H$165,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1046,19 +1046,19 @@
         </is>
       </c>
       <c r="B27" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$164,$A27&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$165,$A27&amp;"*")</f>
         <v/>
       </c>
       <c r="C27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$164,$A27&amp;"*",'QA Checklist'!$H$5:$H$164,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$164,$A27&amp;"*",'QA Checklist'!$H$5:$H$164,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$165,$A27&amp;"*",'QA Checklist'!$H$5:$H$165,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$165,$A27&amp;"*",'QA Checklist'!$H$5:$H$165,"Pass")</f>
         <v/>
       </c>
       <c r="D27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$164,$A27&amp;"*",'QA Checklist'!$H$5:$H$164,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$164,$A27&amp;"*",'QA Checklist'!$H$5:$H$164,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$165,$A27&amp;"*",'QA Checklist'!$H$5:$H$165,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$165,$A27&amp;"*",'QA Checklist'!$H$5:$H$165,"Fail")</f>
         <v/>
       </c>
       <c r="E27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$164,$A27&amp;"*",'QA Checklist'!$H$5:$H$164,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$165,$A27&amp;"*",'QA Checklist'!$H$5:$H$165,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1069,19 +1069,19 @@
         </is>
       </c>
       <c r="B28" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$164,$A28&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$165,$A28&amp;"*")</f>
         <v/>
       </c>
       <c r="C28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$164,$A28&amp;"*",'QA Checklist'!$H$5:$H$164,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$164,$A28&amp;"*",'QA Checklist'!$H$5:$H$164,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$165,$A28&amp;"*",'QA Checklist'!$H$5:$H$165,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$165,$A28&amp;"*",'QA Checklist'!$H$5:$H$165,"Pass")</f>
         <v/>
       </c>
       <c r="D28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$164,$A28&amp;"*",'QA Checklist'!$H$5:$H$164,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$164,$A28&amp;"*",'QA Checklist'!$H$5:$H$164,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$165,$A28&amp;"*",'QA Checklist'!$H$5:$H$165,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$165,$A28&amp;"*",'QA Checklist'!$H$5:$H$165,"Fail")</f>
         <v/>
       </c>
       <c r="E28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$164,$A28&amp;"*",'QA Checklist'!$H$5:$H$164,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$165,$A28&amp;"*",'QA Checklist'!$H$5:$H$165,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1096,7 +1096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I164"/>
+  <dimension ref="A1:I165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8247,12 +8247,59 @@
         </is>
       </c>
     </row>
+    <row r="165">
+      <c r="A165" s="12" t="inlineStr">
+        <is>
+          <t>SA-39</t>
+        </is>
+      </c>
+      <c r="B165" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="C165" s="13" t="inlineStr">
+        <is>
+          <t>Tier 2 (Workflow &amp; Ergonomics)</t>
+        </is>
+      </c>
+      <c r="D165" s="13" t="inlineStr">
+        <is>
+          <t>CheckList Studio Professional Neutral Redesign &amp; Fuel Selector</t>
+        </is>
+      </c>
+      <c r="E165" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="F165" s="13" t="inlineStr">
+        <is>
+          <t>Log in as Service Advisor, open 2025 RO Excel Studio, switch to Checklist tab, review the editor, pick each fuel level, set several checkpoint statuses, and view the page on a phone-sized screen</t>
+        </is>
+      </c>
+      <c r="G165" s="13" t="inlineStr">
+        <is>
+          <t>The editor uses a neutral gray design with Export .xlsx as the only dark primary button and no colored banners or pulsing badges; each checkpoint has a segmented Good / Attention / Defect / N/A control where the selected option turns dark and small green / yellow / red swatches match the printed form boxes; the selected fuel level is highlighted and the label shows the matching percentage; the layout stays readable on a phone-sized screen; the Checklist PDF and Excel output are unchanged</t>
+        </is>
+      </c>
+      <c r="H165" s="14" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="I165" s="13" t="inlineStr">
+        <is>
+          <t>Verified by Automated Unit Tests (151/151 passing in tests/frontend/sla_and_logic.test.js AUT-FRONT-122) and headless Chrome desktop / phone renders</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:I164"/>
+  <autoFilter ref="A4:I165"/>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="H5:H164">
+  <conditionalFormatting sqref="H5:H165">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$H5="Passed"</formula>
     </cfRule>
@@ -8269,13 +8316,13 @@
       <formula>$H5="Pending"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A5:A164">
+  <conditionalFormatting sqref="A5:A165">
     <cfRule type="expression" priority="6" dxfId="3">
-      <formula>COUNTIF($A$5:$A$164,$A5)&gt;1</formula>
+      <formula>COUNTIF($A$5:$A$165,$A5)&gt;1</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H5:H164" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H5:H165" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pending,Passed,Failed"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
fix(REV-164): restore original colors of CheckList Studio quick action buttons
Restore the original colors of the Save Draft and All Pass (light
emerald), Reset (gray with amber hover) and Export .xlsx (solid emerald)
buttons while keeping the REV-163 button shape and the rest of the
neutral design. Bump cache buster to v=3.17, add AUT-FRONT-123, scope
AUT-FRONT-122 to exclude the quick actions, and sync REV-164 / SA-40
into the revisions log, checklists and QA workbook.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
+++ b/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
@@ -11,7 +11,7 @@
     <sheet name="QA Checklist" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$166</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'QA Checklist'!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTA('QA Checklist'!$A$5:$A$165)</f>
+        <f>COUNTA('QA Checklist'!$A$5:$A$166)</f>
         <v/>
       </c>
     </row>
@@ -594,7 +594,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$165,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$165,"Pass")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$166,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$166,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$165,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$165,"Fail")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$166,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$166,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -616,7 +616,7 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$165,"Pending")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$166,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -671,19 +671,19 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$165,$A12)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$166,$A12)</f>
         <v/>
       </c>
       <c r="C12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$165,$A12,'QA Checklist'!$H$5:$H$165,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$165,$A12,'QA Checklist'!$H$5:$H$165,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$166,$A12,'QA Checklist'!$H$5:$H$166,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$166,$A12,'QA Checklist'!$H$5:$H$166,"Pass")</f>
         <v/>
       </c>
       <c r="D12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$165,$A12,'QA Checklist'!$H$5:$H$165,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$165,$A12,'QA Checklist'!$H$5:$H$165,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$166,$A12,'QA Checklist'!$H$5:$H$166,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$166,$A12,'QA Checklist'!$H$5:$H$166,"Fail")</f>
         <v/>
       </c>
       <c r="E12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$165,$A12,'QA Checklist'!$H$5:$H$165,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$166,$A12,'QA Checklist'!$H$5:$H$166,"Pending")</f>
         <v/>
       </c>
       <c r="F12" s="8">
@@ -698,19 +698,19 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$165,$A13)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$166,$A13)</f>
         <v/>
       </c>
       <c r="C13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$165,$A13,'QA Checklist'!$H$5:$H$165,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$165,$A13,'QA Checklist'!$H$5:$H$165,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$166,$A13,'QA Checklist'!$H$5:$H$166,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$166,$A13,'QA Checklist'!$H$5:$H$166,"Pass")</f>
         <v/>
       </c>
       <c r="D13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$165,$A13,'QA Checklist'!$H$5:$H$165,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$165,$A13,'QA Checklist'!$H$5:$H$165,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$166,$A13,'QA Checklist'!$H$5:$H$166,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$166,$A13,'QA Checklist'!$H$5:$H$166,"Fail")</f>
         <v/>
       </c>
       <c r="E13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$165,$A13,'QA Checklist'!$H$5:$H$165,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$166,$A13,'QA Checklist'!$H$5:$H$166,"Pending")</f>
         <v/>
       </c>
       <c r="F13" s="8">
@@ -725,19 +725,19 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$165,$A14)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$166,$A14)</f>
         <v/>
       </c>
       <c r="C14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$165,$A14,'QA Checklist'!$H$5:$H$165,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$165,$A14,'QA Checklist'!$H$5:$H$165,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$166,$A14,'QA Checklist'!$H$5:$H$166,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$166,$A14,'QA Checklist'!$H$5:$H$166,"Pass")</f>
         <v/>
       </c>
       <c r="D14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$165,$A14,'QA Checklist'!$H$5:$H$165,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$165,$A14,'QA Checklist'!$H$5:$H$165,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$166,$A14,'QA Checklist'!$H$5:$H$166,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$166,$A14,'QA Checklist'!$H$5:$H$166,"Fail")</f>
         <v/>
       </c>
       <c r="E14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$165,$A14,'QA Checklist'!$H$5:$H$165,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$166,$A14,'QA Checklist'!$H$5:$H$166,"Pending")</f>
         <v/>
       </c>
       <c r="F14" s="8">
@@ -752,19 +752,19 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$165,$A15)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$166,$A15)</f>
         <v/>
       </c>
       <c r="C15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$165,$A15,'QA Checklist'!$H$5:$H$165,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$165,$A15,'QA Checklist'!$H$5:$H$165,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$166,$A15,'QA Checklist'!$H$5:$H$166,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$166,$A15,'QA Checklist'!$H$5:$H$166,"Pass")</f>
         <v/>
       </c>
       <c r="D15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$165,$A15,'QA Checklist'!$H$5:$H$165,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$165,$A15,'QA Checklist'!$H$5:$H$165,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$166,$A15,'QA Checklist'!$H$5:$H$166,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$166,$A15,'QA Checklist'!$H$5:$H$166,"Fail")</f>
         <v/>
       </c>
       <c r="E15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$165,$A15,'QA Checklist'!$H$5:$H$165,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$166,$A15,'QA Checklist'!$H$5:$H$166,"Pending")</f>
         <v/>
       </c>
       <c r="F15" s="8">
@@ -779,19 +779,19 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$165,$A16)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$166,$A16)</f>
         <v/>
       </c>
       <c r="C16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$165,$A16,'QA Checklist'!$H$5:$H$165,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$165,$A16,'QA Checklist'!$H$5:$H$165,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$166,$A16,'QA Checklist'!$H$5:$H$166,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$166,$A16,'QA Checklist'!$H$5:$H$166,"Pass")</f>
         <v/>
       </c>
       <c r="D16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$165,$A16,'QA Checklist'!$H$5:$H$165,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$165,$A16,'QA Checklist'!$H$5:$H$165,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$166,$A16,'QA Checklist'!$H$5:$H$166,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$166,$A16,'QA Checklist'!$H$5:$H$166,"Fail")</f>
         <v/>
       </c>
       <c r="E16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$165,$A16,'QA Checklist'!$H$5:$H$165,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$166,$A16,'QA Checklist'!$H$5:$H$166,"Pending")</f>
         <v/>
       </c>
       <c r="F16" s="8">
@@ -806,19 +806,19 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$165,$A17)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$166,$A17)</f>
         <v/>
       </c>
       <c r="C17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$165,$A17,'QA Checklist'!$H$5:$H$165,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$165,$A17,'QA Checklist'!$H$5:$H$165,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$166,$A17,'QA Checklist'!$H$5:$H$166,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$166,$A17,'QA Checklist'!$H$5:$H$166,"Pass")</f>
         <v/>
       </c>
       <c r="D17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$165,$A17,'QA Checklist'!$H$5:$H$165,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$165,$A17,'QA Checklist'!$H$5:$H$165,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$166,$A17,'QA Checklist'!$H$5:$H$166,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$166,$A17,'QA Checklist'!$H$5:$H$166,"Fail")</f>
         <v/>
       </c>
       <c r="E17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$165,$A17,'QA Checklist'!$H$5:$H$165,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$166,$A17,'QA Checklist'!$H$5:$H$166,"Pending")</f>
         <v/>
       </c>
       <c r="F17" s="8">
@@ -833,19 +833,19 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$165,$A18)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$166,$A18)</f>
         <v/>
       </c>
       <c r="C18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$165,$A18,'QA Checklist'!$H$5:$H$165,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$165,$A18,'QA Checklist'!$H$5:$H$165,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$166,$A18,'QA Checklist'!$H$5:$H$166,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$166,$A18,'QA Checklist'!$H$5:$H$166,"Pass")</f>
         <v/>
       </c>
       <c r="D18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$165,$A18,'QA Checklist'!$H$5:$H$165,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$165,$A18,'QA Checklist'!$H$5:$H$165,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$166,$A18,'QA Checklist'!$H$5:$H$166,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$166,$A18,'QA Checklist'!$H$5:$H$166,"Fail")</f>
         <v/>
       </c>
       <c r="E18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$165,$A18,'QA Checklist'!$H$5:$H$165,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$166,$A18,'QA Checklist'!$H$5:$H$166,"Pending")</f>
         <v/>
       </c>
       <c r="F18" s="8">
@@ -860,19 +860,19 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$165,$A19)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$166,$A19)</f>
         <v/>
       </c>
       <c r="C19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$165,$A19,'QA Checklist'!$H$5:$H$165,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$165,$A19,'QA Checklist'!$H$5:$H$165,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$166,$A19,'QA Checklist'!$H$5:$H$166,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$166,$A19,'QA Checklist'!$H$5:$H$166,"Pass")</f>
         <v/>
       </c>
       <c r="D19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$165,$A19,'QA Checklist'!$H$5:$H$165,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$165,$A19,'QA Checklist'!$H$5:$H$165,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$166,$A19,'QA Checklist'!$H$5:$H$166,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$166,$A19,'QA Checklist'!$H$5:$H$166,"Fail")</f>
         <v/>
       </c>
       <c r="E19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$165,$A19,'QA Checklist'!$H$5:$H$165,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$166,$A19,'QA Checklist'!$H$5:$H$166,"Pending")</f>
         <v/>
       </c>
       <c r="F19" s="8">
@@ -887,19 +887,19 @@
         </is>
       </c>
       <c r="B20" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$165,$A20)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$166,$A20)</f>
         <v/>
       </c>
       <c r="C20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$165,$A20,'QA Checklist'!$H$5:$H$165,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$165,$A20,'QA Checklist'!$H$5:$H$165,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$166,$A20,'QA Checklist'!$H$5:$H$166,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$166,$A20,'QA Checklist'!$H$5:$H$166,"Pass")</f>
         <v/>
       </c>
       <c r="D20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$165,$A20,'QA Checklist'!$H$5:$H$165,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$165,$A20,'QA Checklist'!$H$5:$H$165,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$166,$A20,'QA Checklist'!$H$5:$H$166,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$166,$A20,'QA Checklist'!$H$5:$H$166,"Fail")</f>
         <v/>
       </c>
       <c r="E20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$165,$A20,'QA Checklist'!$H$5:$H$165,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$166,$A20,'QA Checklist'!$H$5:$H$166,"Pending")</f>
         <v/>
       </c>
       <c r="F20" s="8">
@@ -914,19 +914,19 @@
         </is>
       </c>
       <c r="B21" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$165,$A21)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$166,$A21)</f>
         <v/>
       </c>
       <c r="C21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$165,$A21,'QA Checklist'!$H$5:$H$165,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$165,$A21,'QA Checklist'!$H$5:$H$165,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$166,$A21,'QA Checklist'!$H$5:$H$166,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$166,$A21,'QA Checklist'!$H$5:$H$166,"Pass")</f>
         <v/>
       </c>
       <c r="D21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$165,$A21,'QA Checklist'!$H$5:$H$165,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$165,$A21,'QA Checklist'!$H$5:$H$165,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$166,$A21,'QA Checklist'!$H$5:$H$166,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$166,$A21,'QA Checklist'!$H$5:$H$166,"Fail")</f>
         <v/>
       </c>
       <c r="E21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$165,$A21,'QA Checklist'!$H$5:$H$165,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$166,$A21,'QA Checklist'!$H$5:$H$166,"Pending")</f>
         <v/>
       </c>
       <c r="F21" s="8">
@@ -941,19 +941,19 @@
         </is>
       </c>
       <c r="B22" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$165,$A22)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$166,$A22)</f>
         <v/>
       </c>
       <c r="C22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$165,$A22,'QA Checklist'!$H$5:$H$165,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$165,$A22,'QA Checklist'!$H$5:$H$165,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$166,$A22,'QA Checklist'!$H$5:$H$166,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$166,$A22,'QA Checklist'!$H$5:$H$166,"Pass")</f>
         <v/>
       </c>
       <c r="D22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$165,$A22,'QA Checklist'!$H$5:$H$165,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$165,$A22,'QA Checklist'!$H$5:$H$165,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$166,$A22,'QA Checklist'!$H$5:$H$166,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$166,$A22,'QA Checklist'!$H$5:$H$166,"Fail")</f>
         <v/>
       </c>
       <c r="E22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$165,$A22,'QA Checklist'!$H$5:$H$165,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$166,$A22,'QA Checklist'!$H$5:$H$166,"Pending")</f>
         <v/>
       </c>
       <c r="F22" s="8">
@@ -1023,19 +1023,19 @@
         </is>
       </c>
       <c r="B26" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$165,$A26&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$166,$A26&amp;"*")</f>
         <v/>
       </c>
       <c r="C26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$165,$A26&amp;"*",'QA Checklist'!$H$5:$H$165,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$165,$A26&amp;"*",'QA Checklist'!$H$5:$H$165,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$166,$A26&amp;"*",'QA Checklist'!$H$5:$H$166,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$166,$A26&amp;"*",'QA Checklist'!$H$5:$H$166,"Pass")</f>
         <v/>
       </c>
       <c r="D26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$165,$A26&amp;"*",'QA Checklist'!$H$5:$H$165,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$165,$A26&amp;"*",'QA Checklist'!$H$5:$H$165,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$166,$A26&amp;"*",'QA Checklist'!$H$5:$H$166,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$166,$A26&amp;"*",'QA Checklist'!$H$5:$H$166,"Fail")</f>
         <v/>
       </c>
       <c r="E26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$165,$A26&amp;"*",'QA Checklist'!$H$5:$H$165,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$166,$A26&amp;"*",'QA Checklist'!$H$5:$H$166,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1046,19 +1046,19 @@
         </is>
       </c>
       <c r="B27" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$165,$A27&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$166,$A27&amp;"*")</f>
         <v/>
       </c>
       <c r="C27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$165,$A27&amp;"*",'QA Checklist'!$H$5:$H$165,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$165,$A27&amp;"*",'QA Checklist'!$H$5:$H$165,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$166,$A27&amp;"*",'QA Checklist'!$H$5:$H$166,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$166,$A27&amp;"*",'QA Checklist'!$H$5:$H$166,"Pass")</f>
         <v/>
       </c>
       <c r="D27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$165,$A27&amp;"*",'QA Checklist'!$H$5:$H$165,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$165,$A27&amp;"*",'QA Checklist'!$H$5:$H$165,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$166,$A27&amp;"*",'QA Checklist'!$H$5:$H$166,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$166,$A27&amp;"*",'QA Checklist'!$H$5:$H$166,"Fail")</f>
         <v/>
       </c>
       <c r="E27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$165,$A27&amp;"*",'QA Checklist'!$H$5:$H$165,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$166,$A27&amp;"*",'QA Checklist'!$H$5:$H$166,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1069,19 +1069,19 @@
         </is>
       </c>
       <c r="B28" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$165,$A28&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$166,$A28&amp;"*")</f>
         <v/>
       </c>
       <c r="C28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$165,$A28&amp;"*",'QA Checklist'!$H$5:$H$165,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$165,$A28&amp;"*",'QA Checklist'!$H$5:$H$165,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$166,$A28&amp;"*",'QA Checklist'!$H$5:$H$166,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$166,$A28&amp;"*",'QA Checklist'!$H$5:$H$166,"Pass")</f>
         <v/>
       </c>
       <c r="D28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$165,$A28&amp;"*",'QA Checklist'!$H$5:$H$165,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$165,$A28&amp;"*",'QA Checklist'!$H$5:$H$165,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$166,$A28&amp;"*",'QA Checklist'!$H$5:$H$166,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$166,$A28&amp;"*",'QA Checklist'!$H$5:$H$166,"Fail")</f>
         <v/>
       </c>
       <c r="E28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$165,$A28&amp;"*",'QA Checklist'!$H$5:$H$165,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$166,$A28&amp;"*",'QA Checklist'!$H$5:$H$166,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1096,7 +1096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I165"/>
+  <dimension ref="A1:I166"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8294,12 +8294,59 @@
         </is>
       </c>
     </row>
+    <row r="166">
+      <c r="A166" s="12" t="inlineStr">
+        <is>
+          <t>SA-40</t>
+        </is>
+      </c>
+      <c r="B166" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="C166" s="13" t="inlineStr">
+        <is>
+          <t>Tier 2 (Workflow &amp; Ergonomics)</t>
+        </is>
+      </c>
+      <c r="D166" s="13" t="inlineStr">
+        <is>
+          <t>CheckList Studio Quick Actions Original Colors</t>
+        </is>
+      </c>
+      <c r="E166" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="F166" s="13" t="inlineStr">
+        <is>
+          <t>Log in as Service Advisor, open 2025 RO Excel Studio, switch to Checklist tab, and look at the Save Draft, All Pass, Reset and Export .xlsx buttons in the header; hover over each</t>
+        </is>
+      </c>
+      <c r="G166" s="13" t="inlineStr">
+        <is>
+          <t>Save Draft and All Pass show light green buttons with green text, Reset is light gray and turns amber on hover, and Export .xlsx is solid green with white text; all four keep the same size and rounded shape as the rest of the professional design, and the remainder of the editor stays neutral gray</t>
+        </is>
+      </c>
+      <c r="H166" s="14" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="I166" s="13" t="inlineStr">
+        <is>
+          <t>Verified by Automated Unit Tests (152/152 passing in tests/frontend/sla_and_logic.test.js AUT-FRONT-123) and headless Chrome render inspection</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:I165"/>
+  <autoFilter ref="A4:I166"/>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="H5:H165">
+  <conditionalFormatting sqref="H5:H166">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$H5="Passed"</formula>
     </cfRule>
@@ -8316,13 +8363,13 @@
       <formula>$H5="Pending"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A5:A165">
+  <conditionalFormatting sqref="A5:A166">
     <cfRule type="expression" priority="6" dxfId="3">
-      <formula>COUNTIF($A$5:$A$165,$A5)&gt;1</formula>
+      <formula>COUNTIF($A$5:$A$166,$A5)&gt;1</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H5:H165" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H5:H166" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pending,Passed,Failed"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
fix(REV-165): fill checklist status buttons with actual printed-form colors
Fill the selected checkpoint status option with the printed form's box
color (green Good, yellow Attention, red Defect / battery Replace, dark
gray N/A) instead of dark gray with small dot swatches, and show full
color blocks in the legend. Bump cache buster to v=3.18, add
AUT-FRONT-124, update AUT-FRONT-122, and sync REV-165 / SA-41 into the
revisions log, checklists and QA workbook.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
+++ b/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
@@ -11,7 +11,7 @@
     <sheet name="QA Checklist" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$166</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$167</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'QA Checklist'!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTA('QA Checklist'!$A$5:$A$166)</f>
+        <f>COUNTA('QA Checklist'!$A$5:$A$167)</f>
         <v/>
       </c>
     </row>
@@ -594,7 +594,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$166,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$166,"Pass")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$167,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$167,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$166,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$166,"Fail")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$167,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$167,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -616,7 +616,7 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$166,"Pending")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$167,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -671,19 +671,19 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$166,$A12)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$167,$A12)</f>
         <v/>
       </c>
       <c r="C12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$166,$A12,'QA Checklist'!$H$5:$H$166,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$166,$A12,'QA Checklist'!$H$5:$H$166,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$167,$A12,'QA Checklist'!$H$5:$H$167,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$167,$A12,'QA Checklist'!$H$5:$H$167,"Pass")</f>
         <v/>
       </c>
       <c r="D12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$166,$A12,'QA Checklist'!$H$5:$H$166,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$166,$A12,'QA Checklist'!$H$5:$H$166,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$167,$A12,'QA Checklist'!$H$5:$H$167,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$167,$A12,'QA Checklist'!$H$5:$H$167,"Fail")</f>
         <v/>
       </c>
       <c r="E12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$166,$A12,'QA Checklist'!$H$5:$H$166,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$167,$A12,'QA Checklist'!$H$5:$H$167,"Pending")</f>
         <v/>
       </c>
       <c r="F12" s="8">
@@ -698,19 +698,19 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$166,$A13)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$167,$A13)</f>
         <v/>
       </c>
       <c r="C13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$166,$A13,'QA Checklist'!$H$5:$H$166,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$166,$A13,'QA Checklist'!$H$5:$H$166,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$167,$A13,'QA Checklist'!$H$5:$H$167,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$167,$A13,'QA Checklist'!$H$5:$H$167,"Pass")</f>
         <v/>
       </c>
       <c r="D13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$166,$A13,'QA Checklist'!$H$5:$H$166,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$166,$A13,'QA Checklist'!$H$5:$H$166,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$167,$A13,'QA Checklist'!$H$5:$H$167,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$167,$A13,'QA Checklist'!$H$5:$H$167,"Fail")</f>
         <v/>
       </c>
       <c r="E13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$166,$A13,'QA Checklist'!$H$5:$H$166,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$167,$A13,'QA Checklist'!$H$5:$H$167,"Pending")</f>
         <v/>
       </c>
       <c r="F13" s="8">
@@ -725,19 +725,19 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$166,$A14)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$167,$A14)</f>
         <v/>
       </c>
       <c r="C14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$166,$A14,'QA Checklist'!$H$5:$H$166,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$166,$A14,'QA Checklist'!$H$5:$H$166,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$167,$A14,'QA Checklist'!$H$5:$H$167,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$167,$A14,'QA Checklist'!$H$5:$H$167,"Pass")</f>
         <v/>
       </c>
       <c r="D14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$166,$A14,'QA Checklist'!$H$5:$H$166,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$166,$A14,'QA Checklist'!$H$5:$H$166,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$167,$A14,'QA Checklist'!$H$5:$H$167,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$167,$A14,'QA Checklist'!$H$5:$H$167,"Fail")</f>
         <v/>
       </c>
       <c r="E14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$166,$A14,'QA Checklist'!$H$5:$H$166,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$167,$A14,'QA Checklist'!$H$5:$H$167,"Pending")</f>
         <v/>
       </c>
       <c r="F14" s="8">
@@ -752,19 +752,19 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$166,$A15)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$167,$A15)</f>
         <v/>
       </c>
       <c r="C15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$166,$A15,'QA Checklist'!$H$5:$H$166,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$166,$A15,'QA Checklist'!$H$5:$H$166,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$167,$A15,'QA Checklist'!$H$5:$H$167,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$167,$A15,'QA Checklist'!$H$5:$H$167,"Pass")</f>
         <v/>
       </c>
       <c r="D15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$166,$A15,'QA Checklist'!$H$5:$H$166,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$166,$A15,'QA Checklist'!$H$5:$H$166,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$167,$A15,'QA Checklist'!$H$5:$H$167,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$167,$A15,'QA Checklist'!$H$5:$H$167,"Fail")</f>
         <v/>
       </c>
       <c r="E15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$166,$A15,'QA Checklist'!$H$5:$H$166,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$167,$A15,'QA Checklist'!$H$5:$H$167,"Pending")</f>
         <v/>
       </c>
       <c r="F15" s="8">
@@ -779,19 +779,19 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$166,$A16)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$167,$A16)</f>
         <v/>
       </c>
       <c r="C16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$166,$A16,'QA Checklist'!$H$5:$H$166,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$166,$A16,'QA Checklist'!$H$5:$H$166,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$167,$A16,'QA Checklist'!$H$5:$H$167,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$167,$A16,'QA Checklist'!$H$5:$H$167,"Pass")</f>
         <v/>
       </c>
       <c r="D16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$166,$A16,'QA Checklist'!$H$5:$H$166,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$166,$A16,'QA Checklist'!$H$5:$H$166,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$167,$A16,'QA Checklist'!$H$5:$H$167,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$167,$A16,'QA Checklist'!$H$5:$H$167,"Fail")</f>
         <v/>
       </c>
       <c r="E16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$166,$A16,'QA Checklist'!$H$5:$H$166,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$167,$A16,'QA Checklist'!$H$5:$H$167,"Pending")</f>
         <v/>
       </c>
       <c r="F16" s="8">
@@ -806,19 +806,19 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$166,$A17)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$167,$A17)</f>
         <v/>
       </c>
       <c r="C17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$166,$A17,'QA Checklist'!$H$5:$H$166,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$166,$A17,'QA Checklist'!$H$5:$H$166,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$167,$A17,'QA Checklist'!$H$5:$H$167,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$167,$A17,'QA Checklist'!$H$5:$H$167,"Pass")</f>
         <v/>
       </c>
       <c r="D17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$166,$A17,'QA Checklist'!$H$5:$H$166,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$166,$A17,'QA Checklist'!$H$5:$H$166,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$167,$A17,'QA Checklist'!$H$5:$H$167,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$167,$A17,'QA Checklist'!$H$5:$H$167,"Fail")</f>
         <v/>
       </c>
       <c r="E17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$166,$A17,'QA Checklist'!$H$5:$H$166,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$167,$A17,'QA Checklist'!$H$5:$H$167,"Pending")</f>
         <v/>
       </c>
       <c r="F17" s="8">
@@ -833,19 +833,19 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$166,$A18)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$167,$A18)</f>
         <v/>
       </c>
       <c r="C18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$166,$A18,'QA Checklist'!$H$5:$H$166,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$166,$A18,'QA Checklist'!$H$5:$H$166,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$167,$A18,'QA Checklist'!$H$5:$H$167,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$167,$A18,'QA Checklist'!$H$5:$H$167,"Pass")</f>
         <v/>
       </c>
       <c r="D18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$166,$A18,'QA Checklist'!$H$5:$H$166,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$166,$A18,'QA Checklist'!$H$5:$H$166,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$167,$A18,'QA Checklist'!$H$5:$H$167,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$167,$A18,'QA Checklist'!$H$5:$H$167,"Fail")</f>
         <v/>
       </c>
       <c r="E18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$166,$A18,'QA Checklist'!$H$5:$H$166,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$167,$A18,'QA Checklist'!$H$5:$H$167,"Pending")</f>
         <v/>
       </c>
       <c r="F18" s="8">
@@ -860,19 +860,19 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$166,$A19)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$167,$A19)</f>
         <v/>
       </c>
       <c r="C19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$166,$A19,'QA Checklist'!$H$5:$H$166,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$166,$A19,'QA Checklist'!$H$5:$H$166,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$167,$A19,'QA Checklist'!$H$5:$H$167,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$167,$A19,'QA Checklist'!$H$5:$H$167,"Pass")</f>
         <v/>
       </c>
       <c r="D19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$166,$A19,'QA Checklist'!$H$5:$H$166,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$166,$A19,'QA Checklist'!$H$5:$H$166,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$167,$A19,'QA Checklist'!$H$5:$H$167,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$167,$A19,'QA Checklist'!$H$5:$H$167,"Fail")</f>
         <v/>
       </c>
       <c r="E19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$166,$A19,'QA Checklist'!$H$5:$H$166,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$167,$A19,'QA Checklist'!$H$5:$H$167,"Pending")</f>
         <v/>
       </c>
       <c r="F19" s="8">
@@ -887,19 +887,19 @@
         </is>
       </c>
       <c r="B20" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$166,$A20)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$167,$A20)</f>
         <v/>
       </c>
       <c r="C20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$166,$A20,'QA Checklist'!$H$5:$H$166,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$166,$A20,'QA Checklist'!$H$5:$H$166,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$167,$A20,'QA Checklist'!$H$5:$H$167,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$167,$A20,'QA Checklist'!$H$5:$H$167,"Pass")</f>
         <v/>
       </c>
       <c r="D20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$166,$A20,'QA Checklist'!$H$5:$H$166,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$166,$A20,'QA Checklist'!$H$5:$H$166,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$167,$A20,'QA Checklist'!$H$5:$H$167,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$167,$A20,'QA Checklist'!$H$5:$H$167,"Fail")</f>
         <v/>
       </c>
       <c r="E20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$166,$A20,'QA Checklist'!$H$5:$H$166,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$167,$A20,'QA Checklist'!$H$5:$H$167,"Pending")</f>
         <v/>
       </c>
       <c r="F20" s="8">
@@ -914,19 +914,19 @@
         </is>
       </c>
       <c r="B21" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$166,$A21)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$167,$A21)</f>
         <v/>
       </c>
       <c r="C21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$166,$A21,'QA Checklist'!$H$5:$H$166,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$166,$A21,'QA Checklist'!$H$5:$H$166,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$167,$A21,'QA Checklist'!$H$5:$H$167,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$167,$A21,'QA Checklist'!$H$5:$H$167,"Pass")</f>
         <v/>
       </c>
       <c r="D21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$166,$A21,'QA Checklist'!$H$5:$H$166,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$166,$A21,'QA Checklist'!$H$5:$H$166,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$167,$A21,'QA Checklist'!$H$5:$H$167,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$167,$A21,'QA Checklist'!$H$5:$H$167,"Fail")</f>
         <v/>
       </c>
       <c r="E21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$166,$A21,'QA Checklist'!$H$5:$H$166,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$167,$A21,'QA Checklist'!$H$5:$H$167,"Pending")</f>
         <v/>
       </c>
       <c r="F21" s="8">
@@ -941,19 +941,19 @@
         </is>
       </c>
       <c r="B22" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$166,$A22)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$167,$A22)</f>
         <v/>
       </c>
       <c r="C22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$166,$A22,'QA Checklist'!$H$5:$H$166,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$166,$A22,'QA Checklist'!$H$5:$H$166,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$167,$A22,'QA Checklist'!$H$5:$H$167,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$167,$A22,'QA Checklist'!$H$5:$H$167,"Pass")</f>
         <v/>
       </c>
       <c r="D22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$166,$A22,'QA Checklist'!$H$5:$H$166,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$166,$A22,'QA Checklist'!$H$5:$H$166,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$167,$A22,'QA Checklist'!$H$5:$H$167,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$167,$A22,'QA Checklist'!$H$5:$H$167,"Fail")</f>
         <v/>
       </c>
       <c r="E22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$166,$A22,'QA Checklist'!$H$5:$H$166,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$167,$A22,'QA Checklist'!$H$5:$H$167,"Pending")</f>
         <v/>
       </c>
       <c r="F22" s="8">
@@ -1023,19 +1023,19 @@
         </is>
       </c>
       <c r="B26" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$166,$A26&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$167,$A26&amp;"*")</f>
         <v/>
       </c>
       <c r="C26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$166,$A26&amp;"*",'QA Checklist'!$H$5:$H$166,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$166,$A26&amp;"*",'QA Checklist'!$H$5:$H$166,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$167,$A26&amp;"*",'QA Checklist'!$H$5:$H$167,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$167,$A26&amp;"*",'QA Checklist'!$H$5:$H$167,"Pass")</f>
         <v/>
       </c>
       <c r="D26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$166,$A26&amp;"*",'QA Checklist'!$H$5:$H$166,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$166,$A26&amp;"*",'QA Checklist'!$H$5:$H$166,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$167,$A26&amp;"*",'QA Checklist'!$H$5:$H$167,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$167,$A26&amp;"*",'QA Checklist'!$H$5:$H$167,"Fail")</f>
         <v/>
       </c>
       <c r="E26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$166,$A26&amp;"*",'QA Checklist'!$H$5:$H$166,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$167,$A26&amp;"*",'QA Checklist'!$H$5:$H$167,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1046,19 +1046,19 @@
         </is>
       </c>
       <c r="B27" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$166,$A27&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$167,$A27&amp;"*")</f>
         <v/>
       </c>
       <c r="C27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$166,$A27&amp;"*",'QA Checklist'!$H$5:$H$166,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$166,$A27&amp;"*",'QA Checklist'!$H$5:$H$166,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$167,$A27&amp;"*",'QA Checklist'!$H$5:$H$167,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$167,$A27&amp;"*",'QA Checklist'!$H$5:$H$167,"Pass")</f>
         <v/>
       </c>
       <c r="D27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$166,$A27&amp;"*",'QA Checklist'!$H$5:$H$166,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$166,$A27&amp;"*",'QA Checklist'!$H$5:$H$166,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$167,$A27&amp;"*",'QA Checklist'!$H$5:$H$167,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$167,$A27&amp;"*",'QA Checklist'!$H$5:$H$167,"Fail")</f>
         <v/>
       </c>
       <c r="E27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$166,$A27&amp;"*",'QA Checklist'!$H$5:$H$166,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$167,$A27&amp;"*",'QA Checklist'!$H$5:$H$167,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1069,19 +1069,19 @@
         </is>
       </c>
       <c r="B28" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$166,$A28&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$167,$A28&amp;"*")</f>
         <v/>
       </c>
       <c r="C28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$166,$A28&amp;"*",'QA Checklist'!$H$5:$H$166,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$166,$A28&amp;"*",'QA Checklist'!$H$5:$H$166,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$167,$A28&amp;"*",'QA Checklist'!$H$5:$H$167,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$167,$A28&amp;"*",'QA Checklist'!$H$5:$H$167,"Pass")</f>
         <v/>
       </c>
       <c r="D28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$166,$A28&amp;"*",'QA Checklist'!$H$5:$H$166,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$166,$A28&amp;"*",'QA Checklist'!$H$5:$H$166,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$167,$A28&amp;"*",'QA Checklist'!$H$5:$H$167,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$167,$A28&amp;"*",'QA Checklist'!$H$5:$H$167,"Fail")</f>
         <v/>
       </c>
       <c r="E28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$166,$A28&amp;"*",'QA Checklist'!$H$5:$H$166,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$167,$A28&amp;"*",'QA Checklist'!$H$5:$H$167,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1096,7 +1096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I166"/>
+  <dimension ref="A1:I167"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8341,12 +8341,59 @@
         </is>
       </c>
     </row>
+    <row r="167">
+      <c r="A167" s="12" t="inlineStr">
+        <is>
+          <t>SA-41</t>
+        </is>
+      </c>
+      <c r="B167" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="C167" s="13" t="inlineStr">
+        <is>
+          <t>Tier 2 (Workflow &amp; Ergonomics)</t>
+        </is>
+      </c>
+      <c r="D167" s="13" t="inlineStr">
+        <is>
+          <t>Checklist Status Buttons Filled With Actual Form Colors</t>
+        </is>
+      </c>
+      <c r="E167" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="F167" s="13" t="inlineStr">
+        <is>
+          <t>Log in as Service Advisor, open 2025 RO Excel Studio, switch to Checklist tab, and set checkpoints to Good, Attention, Defect and N/A (and the battery to Good / Replace)</t>
+        </is>
+      </c>
+      <c r="G167" s="13" t="inlineStr">
+        <is>
+          <t>The selected option of each checkpoint is fully filled with the printed form color: green for Good, yellow for Attention, red for Defect and battery Replace, dark gray for N/A, with readable text; unselected options are plain white; no small colored dots appear inside the buttons, and the legend shows full color blocks</t>
+        </is>
+      </c>
+      <c r="H167" s="14" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="I167" s="13" t="inlineStr">
+        <is>
+          <t>Verified by Automated Unit Tests (153/153 passing in tests/frontend/sla_and_logic.test.js AUT-FRONT-124) and headless Chrome render inspection</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:I166"/>
+  <autoFilter ref="A4:I167"/>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="H5:H166">
+  <conditionalFormatting sqref="H5:H167">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$H5="Passed"</formula>
     </cfRule>
@@ -8363,13 +8410,13 @@
       <formula>$H5="Pending"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A5:A166">
+  <conditionalFormatting sqref="A5:A167">
     <cfRule type="expression" priority="6" dxfId="3">
-      <formula>COUNTIF($A$5:$A$166,$A5)&gt;1</formula>
+      <formula>COUNTIF($A$5:$A$167,$A5)&gt;1</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H5:H166" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H5:H167" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pending,Passed,Failed"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat(REV-166): per-wheel brake condition status across checklist UI, PDF and Excel
Replace the single "Brake pads" status with independent Left Front,
Right Front, Left Rear and Right Rear statuses, matching the four brake
boxes on the printed form. Older drafts seed all four wheels from the
previous single status; "Brakes not inspected on this visit" sets every
wheel to N/A and restores each wheel's own status and notes when
unticked. The PDF and Excel export stamp each wheel in its own boxes.
Bump cache buster to v=3.19, add AUT-FRONT-125, and sync REV-166 / SA-42
into the revisions log, checklists and QA workbook.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
+++ b/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
@@ -11,7 +11,7 @@
     <sheet name="QA Checklist" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$167</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$168</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'QA Checklist'!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTA('QA Checklist'!$A$5:$A$167)</f>
+        <f>COUNTA('QA Checklist'!$A$5:$A$168)</f>
         <v/>
       </c>
     </row>
@@ -594,7 +594,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$167,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$167,"Pass")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$168,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$168,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$167,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$167,"Fail")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$168,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$168,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -616,7 +616,7 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$167,"Pending")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$168,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -671,19 +671,19 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$167,$A12)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$168,$A12)</f>
         <v/>
       </c>
       <c r="C12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$167,$A12,'QA Checklist'!$H$5:$H$167,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$167,$A12,'QA Checklist'!$H$5:$H$167,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$168,$A12,'QA Checklist'!$H$5:$H$168,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$168,$A12,'QA Checklist'!$H$5:$H$168,"Pass")</f>
         <v/>
       </c>
       <c r="D12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$167,$A12,'QA Checklist'!$H$5:$H$167,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$167,$A12,'QA Checklist'!$H$5:$H$167,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$168,$A12,'QA Checklist'!$H$5:$H$168,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$168,$A12,'QA Checklist'!$H$5:$H$168,"Fail")</f>
         <v/>
       </c>
       <c r="E12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$167,$A12,'QA Checklist'!$H$5:$H$167,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$168,$A12,'QA Checklist'!$H$5:$H$168,"Pending")</f>
         <v/>
       </c>
       <c r="F12" s="8">
@@ -698,19 +698,19 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$167,$A13)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$168,$A13)</f>
         <v/>
       </c>
       <c r="C13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$167,$A13,'QA Checklist'!$H$5:$H$167,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$167,$A13,'QA Checklist'!$H$5:$H$167,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$168,$A13,'QA Checklist'!$H$5:$H$168,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$168,$A13,'QA Checklist'!$H$5:$H$168,"Pass")</f>
         <v/>
       </c>
       <c r="D13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$167,$A13,'QA Checklist'!$H$5:$H$167,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$167,$A13,'QA Checklist'!$H$5:$H$167,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$168,$A13,'QA Checklist'!$H$5:$H$168,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$168,$A13,'QA Checklist'!$H$5:$H$168,"Fail")</f>
         <v/>
       </c>
       <c r="E13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$167,$A13,'QA Checklist'!$H$5:$H$167,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$168,$A13,'QA Checklist'!$H$5:$H$168,"Pending")</f>
         <v/>
       </c>
       <c r="F13" s="8">
@@ -725,19 +725,19 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$167,$A14)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$168,$A14)</f>
         <v/>
       </c>
       <c r="C14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$167,$A14,'QA Checklist'!$H$5:$H$167,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$167,$A14,'QA Checklist'!$H$5:$H$167,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$168,$A14,'QA Checklist'!$H$5:$H$168,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$168,$A14,'QA Checklist'!$H$5:$H$168,"Pass")</f>
         <v/>
       </c>
       <c r="D14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$167,$A14,'QA Checklist'!$H$5:$H$167,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$167,$A14,'QA Checklist'!$H$5:$H$167,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$168,$A14,'QA Checklist'!$H$5:$H$168,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$168,$A14,'QA Checklist'!$H$5:$H$168,"Fail")</f>
         <v/>
       </c>
       <c r="E14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$167,$A14,'QA Checklist'!$H$5:$H$167,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$168,$A14,'QA Checklist'!$H$5:$H$168,"Pending")</f>
         <v/>
       </c>
       <c r="F14" s="8">
@@ -752,19 +752,19 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$167,$A15)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$168,$A15)</f>
         <v/>
       </c>
       <c r="C15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$167,$A15,'QA Checklist'!$H$5:$H$167,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$167,$A15,'QA Checklist'!$H$5:$H$167,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$168,$A15,'QA Checklist'!$H$5:$H$168,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$168,$A15,'QA Checklist'!$H$5:$H$168,"Pass")</f>
         <v/>
       </c>
       <c r="D15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$167,$A15,'QA Checklist'!$H$5:$H$167,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$167,$A15,'QA Checklist'!$H$5:$H$167,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$168,$A15,'QA Checklist'!$H$5:$H$168,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$168,$A15,'QA Checklist'!$H$5:$H$168,"Fail")</f>
         <v/>
       </c>
       <c r="E15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$167,$A15,'QA Checklist'!$H$5:$H$167,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$168,$A15,'QA Checklist'!$H$5:$H$168,"Pending")</f>
         <v/>
       </c>
       <c r="F15" s="8">
@@ -779,19 +779,19 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$167,$A16)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$168,$A16)</f>
         <v/>
       </c>
       <c r="C16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$167,$A16,'QA Checklist'!$H$5:$H$167,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$167,$A16,'QA Checklist'!$H$5:$H$167,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$168,$A16,'QA Checklist'!$H$5:$H$168,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$168,$A16,'QA Checklist'!$H$5:$H$168,"Pass")</f>
         <v/>
       </c>
       <c r="D16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$167,$A16,'QA Checklist'!$H$5:$H$167,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$167,$A16,'QA Checklist'!$H$5:$H$167,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$168,$A16,'QA Checklist'!$H$5:$H$168,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$168,$A16,'QA Checklist'!$H$5:$H$168,"Fail")</f>
         <v/>
       </c>
       <c r="E16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$167,$A16,'QA Checklist'!$H$5:$H$167,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$168,$A16,'QA Checklist'!$H$5:$H$168,"Pending")</f>
         <v/>
       </c>
       <c r="F16" s="8">
@@ -806,19 +806,19 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$167,$A17)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$168,$A17)</f>
         <v/>
       </c>
       <c r="C17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$167,$A17,'QA Checklist'!$H$5:$H$167,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$167,$A17,'QA Checklist'!$H$5:$H$167,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$168,$A17,'QA Checklist'!$H$5:$H$168,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$168,$A17,'QA Checklist'!$H$5:$H$168,"Pass")</f>
         <v/>
       </c>
       <c r="D17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$167,$A17,'QA Checklist'!$H$5:$H$167,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$167,$A17,'QA Checklist'!$H$5:$H$167,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$168,$A17,'QA Checklist'!$H$5:$H$168,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$168,$A17,'QA Checklist'!$H$5:$H$168,"Fail")</f>
         <v/>
       </c>
       <c r="E17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$167,$A17,'QA Checklist'!$H$5:$H$167,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$168,$A17,'QA Checklist'!$H$5:$H$168,"Pending")</f>
         <v/>
       </c>
       <c r="F17" s="8">
@@ -833,19 +833,19 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$167,$A18)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$168,$A18)</f>
         <v/>
       </c>
       <c r="C18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$167,$A18,'QA Checklist'!$H$5:$H$167,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$167,$A18,'QA Checklist'!$H$5:$H$167,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$168,$A18,'QA Checklist'!$H$5:$H$168,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$168,$A18,'QA Checklist'!$H$5:$H$168,"Pass")</f>
         <v/>
       </c>
       <c r="D18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$167,$A18,'QA Checklist'!$H$5:$H$167,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$167,$A18,'QA Checklist'!$H$5:$H$167,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$168,$A18,'QA Checklist'!$H$5:$H$168,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$168,$A18,'QA Checklist'!$H$5:$H$168,"Fail")</f>
         <v/>
       </c>
       <c r="E18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$167,$A18,'QA Checklist'!$H$5:$H$167,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$168,$A18,'QA Checklist'!$H$5:$H$168,"Pending")</f>
         <v/>
       </c>
       <c r="F18" s="8">
@@ -860,19 +860,19 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$167,$A19)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$168,$A19)</f>
         <v/>
       </c>
       <c r="C19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$167,$A19,'QA Checklist'!$H$5:$H$167,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$167,$A19,'QA Checklist'!$H$5:$H$167,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$168,$A19,'QA Checklist'!$H$5:$H$168,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$168,$A19,'QA Checklist'!$H$5:$H$168,"Pass")</f>
         <v/>
       </c>
       <c r="D19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$167,$A19,'QA Checklist'!$H$5:$H$167,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$167,$A19,'QA Checklist'!$H$5:$H$167,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$168,$A19,'QA Checklist'!$H$5:$H$168,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$168,$A19,'QA Checklist'!$H$5:$H$168,"Fail")</f>
         <v/>
       </c>
       <c r="E19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$167,$A19,'QA Checklist'!$H$5:$H$167,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$168,$A19,'QA Checklist'!$H$5:$H$168,"Pending")</f>
         <v/>
       </c>
       <c r="F19" s="8">
@@ -887,19 +887,19 @@
         </is>
       </c>
       <c r="B20" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$167,$A20)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$168,$A20)</f>
         <v/>
       </c>
       <c r="C20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$167,$A20,'QA Checklist'!$H$5:$H$167,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$167,$A20,'QA Checklist'!$H$5:$H$167,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$168,$A20,'QA Checklist'!$H$5:$H$168,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$168,$A20,'QA Checklist'!$H$5:$H$168,"Pass")</f>
         <v/>
       </c>
       <c r="D20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$167,$A20,'QA Checklist'!$H$5:$H$167,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$167,$A20,'QA Checklist'!$H$5:$H$167,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$168,$A20,'QA Checklist'!$H$5:$H$168,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$168,$A20,'QA Checklist'!$H$5:$H$168,"Fail")</f>
         <v/>
       </c>
       <c r="E20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$167,$A20,'QA Checklist'!$H$5:$H$167,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$168,$A20,'QA Checklist'!$H$5:$H$168,"Pending")</f>
         <v/>
       </c>
       <c r="F20" s="8">
@@ -914,19 +914,19 @@
         </is>
       </c>
       <c r="B21" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$167,$A21)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$168,$A21)</f>
         <v/>
       </c>
       <c r="C21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$167,$A21,'QA Checklist'!$H$5:$H$167,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$167,$A21,'QA Checklist'!$H$5:$H$167,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$168,$A21,'QA Checklist'!$H$5:$H$168,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$168,$A21,'QA Checklist'!$H$5:$H$168,"Pass")</f>
         <v/>
       </c>
       <c r="D21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$167,$A21,'QA Checklist'!$H$5:$H$167,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$167,$A21,'QA Checklist'!$H$5:$H$167,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$168,$A21,'QA Checklist'!$H$5:$H$168,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$168,$A21,'QA Checklist'!$H$5:$H$168,"Fail")</f>
         <v/>
       </c>
       <c r="E21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$167,$A21,'QA Checklist'!$H$5:$H$167,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$168,$A21,'QA Checklist'!$H$5:$H$168,"Pending")</f>
         <v/>
       </c>
       <c r="F21" s="8">
@@ -941,19 +941,19 @@
         </is>
       </c>
       <c r="B22" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$167,$A22)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$168,$A22)</f>
         <v/>
       </c>
       <c r="C22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$167,$A22,'QA Checklist'!$H$5:$H$167,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$167,$A22,'QA Checklist'!$H$5:$H$167,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$168,$A22,'QA Checklist'!$H$5:$H$168,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$168,$A22,'QA Checklist'!$H$5:$H$168,"Pass")</f>
         <v/>
       </c>
       <c r="D22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$167,$A22,'QA Checklist'!$H$5:$H$167,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$167,$A22,'QA Checklist'!$H$5:$H$167,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$168,$A22,'QA Checklist'!$H$5:$H$168,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$168,$A22,'QA Checklist'!$H$5:$H$168,"Fail")</f>
         <v/>
       </c>
       <c r="E22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$167,$A22,'QA Checklist'!$H$5:$H$167,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$168,$A22,'QA Checklist'!$H$5:$H$168,"Pending")</f>
         <v/>
       </c>
       <c r="F22" s="8">
@@ -1023,19 +1023,19 @@
         </is>
       </c>
       <c r="B26" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$167,$A26&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$168,$A26&amp;"*")</f>
         <v/>
       </c>
       <c r="C26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$167,$A26&amp;"*",'QA Checklist'!$H$5:$H$167,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$167,$A26&amp;"*",'QA Checklist'!$H$5:$H$167,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$168,$A26&amp;"*",'QA Checklist'!$H$5:$H$168,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$168,$A26&amp;"*",'QA Checklist'!$H$5:$H$168,"Pass")</f>
         <v/>
       </c>
       <c r="D26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$167,$A26&amp;"*",'QA Checklist'!$H$5:$H$167,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$167,$A26&amp;"*",'QA Checklist'!$H$5:$H$167,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$168,$A26&amp;"*",'QA Checklist'!$H$5:$H$168,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$168,$A26&amp;"*",'QA Checklist'!$H$5:$H$168,"Fail")</f>
         <v/>
       </c>
       <c r="E26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$167,$A26&amp;"*",'QA Checklist'!$H$5:$H$167,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$168,$A26&amp;"*",'QA Checklist'!$H$5:$H$168,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1046,19 +1046,19 @@
         </is>
       </c>
       <c r="B27" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$167,$A27&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$168,$A27&amp;"*")</f>
         <v/>
       </c>
       <c r="C27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$167,$A27&amp;"*",'QA Checklist'!$H$5:$H$167,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$167,$A27&amp;"*",'QA Checklist'!$H$5:$H$167,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$168,$A27&amp;"*",'QA Checklist'!$H$5:$H$168,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$168,$A27&amp;"*",'QA Checklist'!$H$5:$H$168,"Pass")</f>
         <v/>
       </c>
       <c r="D27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$167,$A27&amp;"*",'QA Checklist'!$H$5:$H$167,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$167,$A27&amp;"*",'QA Checklist'!$H$5:$H$167,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$168,$A27&amp;"*",'QA Checklist'!$H$5:$H$168,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$168,$A27&amp;"*",'QA Checklist'!$H$5:$H$168,"Fail")</f>
         <v/>
       </c>
       <c r="E27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$167,$A27&amp;"*",'QA Checklist'!$H$5:$H$167,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$168,$A27&amp;"*",'QA Checklist'!$H$5:$H$168,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1069,19 +1069,19 @@
         </is>
       </c>
       <c r="B28" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$167,$A28&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$168,$A28&amp;"*")</f>
         <v/>
       </c>
       <c r="C28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$167,$A28&amp;"*",'QA Checklist'!$H$5:$H$167,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$167,$A28&amp;"*",'QA Checklist'!$H$5:$H$167,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$168,$A28&amp;"*",'QA Checklist'!$H$5:$H$168,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$168,$A28&amp;"*",'QA Checklist'!$H$5:$H$168,"Pass")</f>
         <v/>
       </c>
       <c r="D28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$167,$A28&amp;"*",'QA Checklist'!$H$5:$H$167,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$167,$A28&amp;"*",'QA Checklist'!$H$5:$H$167,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$168,$A28&amp;"*",'QA Checklist'!$H$5:$H$168,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$168,$A28&amp;"*",'QA Checklist'!$H$5:$H$168,"Fail")</f>
         <v/>
       </c>
       <c r="E28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$167,$A28&amp;"*",'QA Checklist'!$H$5:$H$167,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$168,$A28&amp;"*",'QA Checklist'!$H$5:$H$168,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1096,7 +1096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I167"/>
+  <dimension ref="A1:I168"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8388,12 +8388,59 @@
         </is>
       </c>
     </row>
+    <row r="168">
+      <c r="A168" s="12" t="inlineStr">
+        <is>
+          <t>SA-42</t>
+        </is>
+      </c>
+      <c r="B168" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="C168" s="13" t="inlineStr">
+        <is>
+          <t>Tier 2 (Workflow &amp; Ergonomics)</t>
+        </is>
+      </c>
+      <c r="D168" s="13" t="inlineStr">
+        <is>
+          <t>Checklist Brake Condition Per-Wheel Status</t>
+        </is>
+      </c>
+      <c r="E168" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="F168" s="13" t="inlineStr">
+        <is>
+          <t>Log in as Service Advisor, open 2025 RO Excel Studio, switch to Checklist tab, set a different status for Left Front, Right Front, Left Rear and Right Rear under Brake Condition, then view the Checklist PDF and export Excel; tick and untick 'Brakes not inspected on this visit'</t>
+        </is>
+      </c>
+      <c r="G168" s="13" t="inlineStr">
+        <is>
+          <t>Brake Condition shows four rows (Left Front, Right Front, Left Rear, Right Rear), each with its own status and notes; the PDF and Excel mark each wheel in its own green / yellow / red box with the matching symbol; ticking 'Brakes not inspected' sets all four wheels to N/A and marks the checkbox, and unticking restores each wheel's previous status and notes; older drafts open with all four wheels set to the previous single brake status</t>
+        </is>
+      </c>
+      <c r="H168" s="14" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="I168" s="13" t="inlineStr">
+        <is>
+          <t>Verified by Automated Unit Tests (154/154 passing in tests/frontend/sla_and_logic.test.js AUT-FRONT-125), Node logic run, headless Chrome UI render, PDF render and real Excel export read back with openpyxl</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:I167"/>
+  <autoFilter ref="A4:I168"/>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="H5:H167">
+  <conditionalFormatting sqref="H5:H168">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$H5="Passed"</formula>
     </cfRule>
@@ -8410,13 +8457,13 @@
       <formula>$H5="Pending"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A5:A167">
+  <conditionalFormatting sqref="A5:A168">
     <cfRule type="expression" priority="6" dxfId="3">
-      <formula>COUNTIF($A$5:$A$167,$A5)&gt;1</formula>
+      <formula>COUNTIF($A$5:$A$168,$A5)&gt;1</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H5:H167" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H5:H168" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pending,Passed,Failed"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat(REV-167): make checklist checkpoints selection-only
Remove the per-item notes text box from every checklist checkpoint so
the Service Advisor only selects a status; findings stay in Inspector
Remarks. PDF and Excel output are unchanged. Bump cache buster to
v=3.20, add AUT-FRONT-126, widen the AUT-FRONT-104/112 version pattern
to 3.00-3.99, and sync REV-167 / SA-43 into the revisions log,
checklists and QA workbook.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
+++ b/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
@@ -11,7 +11,7 @@
     <sheet name="QA Checklist" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$168</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$169</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'QA Checklist'!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTA('QA Checklist'!$A$5:$A$168)</f>
+        <f>COUNTA('QA Checklist'!$A$5:$A$169)</f>
         <v/>
       </c>
     </row>
@@ -594,7 +594,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$168,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$168,"Pass")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$169,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$169,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$168,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$168,"Fail")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$169,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$169,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -616,7 +616,7 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$168,"Pending")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$169,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -671,19 +671,19 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$168,$A12)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$169,$A12)</f>
         <v/>
       </c>
       <c r="C12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$168,$A12,'QA Checklist'!$H$5:$H$168,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$168,$A12,'QA Checklist'!$H$5:$H$168,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$169,$A12,'QA Checklist'!$H$5:$H$169,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$169,$A12,'QA Checklist'!$H$5:$H$169,"Pass")</f>
         <v/>
       </c>
       <c r="D12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$168,$A12,'QA Checklist'!$H$5:$H$168,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$168,$A12,'QA Checklist'!$H$5:$H$168,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$169,$A12,'QA Checklist'!$H$5:$H$169,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$169,$A12,'QA Checklist'!$H$5:$H$169,"Fail")</f>
         <v/>
       </c>
       <c r="E12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$168,$A12,'QA Checklist'!$H$5:$H$168,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$169,$A12,'QA Checklist'!$H$5:$H$169,"Pending")</f>
         <v/>
       </c>
       <c r="F12" s="8">
@@ -698,19 +698,19 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$168,$A13)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$169,$A13)</f>
         <v/>
       </c>
       <c r="C13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$168,$A13,'QA Checklist'!$H$5:$H$168,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$168,$A13,'QA Checklist'!$H$5:$H$168,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$169,$A13,'QA Checklist'!$H$5:$H$169,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$169,$A13,'QA Checklist'!$H$5:$H$169,"Pass")</f>
         <v/>
       </c>
       <c r="D13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$168,$A13,'QA Checklist'!$H$5:$H$168,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$168,$A13,'QA Checklist'!$H$5:$H$168,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$169,$A13,'QA Checklist'!$H$5:$H$169,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$169,$A13,'QA Checklist'!$H$5:$H$169,"Fail")</f>
         <v/>
       </c>
       <c r="E13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$168,$A13,'QA Checklist'!$H$5:$H$168,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$169,$A13,'QA Checklist'!$H$5:$H$169,"Pending")</f>
         <v/>
       </c>
       <c r="F13" s="8">
@@ -725,19 +725,19 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$168,$A14)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$169,$A14)</f>
         <v/>
       </c>
       <c r="C14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$168,$A14,'QA Checklist'!$H$5:$H$168,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$168,$A14,'QA Checklist'!$H$5:$H$168,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$169,$A14,'QA Checklist'!$H$5:$H$169,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$169,$A14,'QA Checklist'!$H$5:$H$169,"Pass")</f>
         <v/>
       </c>
       <c r="D14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$168,$A14,'QA Checklist'!$H$5:$H$168,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$168,$A14,'QA Checklist'!$H$5:$H$168,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$169,$A14,'QA Checklist'!$H$5:$H$169,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$169,$A14,'QA Checklist'!$H$5:$H$169,"Fail")</f>
         <v/>
       </c>
       <c r="E14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$168,$A14,'QA Checklist'!$H$5:$H$168,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$169,$A14,'QA Checklist'!$H$5:$H$169,"Pending")</f>
         <v/>
       </c>
       <c r="F14" s="8">
@@ -752,19 +752,19 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$168,$A15)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$169,$A15)</f>
         <v/>
       </c>
       <c r="C15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$168,$A15,'QA Checklist'!$H$5:$H$168,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$168,$A15,'QA Checklist'!$H$5:$H$168,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$169,$A15,'QA Checklist'!$H$5:$H$169,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$169,$A15,'QA Checklist'!$H$5:$H$169,"Pass")</f>
         <v/>
       </c>
       <c r="D15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$168,$A15,'QA Checklist'!$H$5:$H$168,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$168,$A15,'QA Checklist'!$H$5:$H$168,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$169,$A15,'QA Checklist'!$H$5:$H$169,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$169,$A15,'QA Checklist'!$H$5:$H$169,"Fail")</f>
         <v/>
       </c>
       <c r="E15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$168,$A15,'QA Checklist'!$H$5:$H$168,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$169,$A15,'QA Checklist'!$H$5:$H$169,"Pending")</f>
         <v/>
       </c>
       <c r="F15" s="8">
@@ -779,19 +779,19 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$168,$A16)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$169,$A16)</f>
         <v/>
       </c>
       <c r="C16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$168,$A16,'QA Checklist'!$H$5:$H$168,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$168,$A16,'QA Checklist'!$H$5:$H$168,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$169,$A16,'QA Checklist'!$H$5:$H$169,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$169,$A16,'QA Checklist'!$H$5:$H$169,"Pass")</f>
         <v/>
       </c>
       <c r="D16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$168,$A16,'QA Checklist'!$H$5:$H$168,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$168,$A16,'QA Checklist'!$H$5:$H$168,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$169,$A16,'QA Checklist'!$H$5:$H$169,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$169,$A16,'QA Checklist'!$H$5:$H$169,"Fail")</f>
         <v/>
       </c>
       <c r="E16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$168,$A16,'QA Checklist'!$H$5:$H$168,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$169,$A16,'QA Checklist'!$H$5:$H$169,"Pending")</f>
         <v/>
       </c>
       <c r="F16" s="8">
@@ -806,19 +806,19 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$168,$A17)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$169,$A17)</f>
         <v/>
       </c>
       <c r="C17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$168,$A17,'QA Checklist'!$H$5:$H$168,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$168,$A17,'QA Checklist'!$H$5:$H$168,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$169,$A17,'QA Checklist'!$H$5:$H$169,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$169,$A17,'QA Checklist'!$H$5:$H$169,"Pass")</f>
         <v/>
       </c>
       <c r="D17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$168,$A17,'QA Checklist'!$H$5:$H$168,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$168,$A17,'QA Checklist'!$H$5:$H$168,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$169,$A17,'QA Checklist'!$H$5:$H$169,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$169,$A17,'QA Checklist'!$H$5:$H$169,"Fail")</f>
         <v/>
       </c>
       <c r="E17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$168,$A17,'QA Checklist'!$H$5:$H$168,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$169,$A17,'QA Checklist'!$H$5:$H$169,"Pending")</f>
         <v/>
       </c>
       <c r="F17" s="8">
@@ -833,19 +833,19 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$168,$A18)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$169,$A18)</f>
         <v/>
       </c>
       <c r="C18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$168,$A18,'QA Checklist'!$H$5:$H$168,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$168,$A18,'QA Checklist'!$H$5:$H$168,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$169,$A18,'QA Checklist'!$H$5:$H$169,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$169,$A18,'QA Checklist'!$H$5:$H$169,"Pass")</f>
         <v/>
       </c>
       <c r="D18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$168,$A18,'QA Checklist'!$H$5:$H$168,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$168,$A18,'QA Checklist'!$H$5:$H$168,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$169,$A18,'QA Checklist'!$H$5:$H$169,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$169,$A18,'QA Checklist'!$H$5:$H$169,"Fail")</f>
         <v/>
       </c>
       <c r="E18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$168,$A18,'QA Checklist'!$H$5:$H$168,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$169,$A18,'QA Checklist'!$H$5:$H$169,"Pending")</f>
         <v/>
       </c>
       <c r="F18" s="8">
@@ -860,19 +860,19 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$168,$A19)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$169,$A19)</f>
         <v/>
       </c>
       <c r="C19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$168,$A19,'QA Checklist'!$H$5:$H$168,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$168,$A19,'QA Checklist'!$H$5:$H$168,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$169,$A19,'QA Checklist'!$H$5:$H$169,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$169,$A19,'QA Checklist'!$H$5:$H$169,"Pass")</f>
         <v/>
       </c>
       <c r="D19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$168,$A19,'QA Checklist'!$H$5:$H$168,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$168,$A19,'QA Checklist'!$H$5:$H$168,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$169,$A19,'QA Checklist'!$H$5:$H$169,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$169,$A19,'QA Checklist'!$H$5:$H$169,"Fail")</f>
         <v/>
       </c>
       <c r="E19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$168,$A19,'QA Checklist'!$H$5:$H$168,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$169,$A19,'QA Checklist'!$H$5:$H$169,"Pending")</f>
         <v/>
       </c>
       <c r="F19" s="8">
@@ -887,19 +887,19 @@
         </is>
       </c>
       <c r="B20" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$168,$A20)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$169,$A20)</f>
         <v/>
       </c>
       <c r="C20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$168,$A20,'QA Checklist'!$H$5:$H$168,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$168,$A20,'QA Checklist'!$H$5:$H$168,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$169,$A20,'QA Checklist'!$H$5:$H$169,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$169,$A20,'QA Checklist'!$H$5:$H$169,"Pass")</f>
         <v/>
       </c>
       <c r="D20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$168,$A20,'QA Checklist'!$H$5:$H$168,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$168,$A20,'QA Checklist'!$H$5:$H$168,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$169,$A20,'QA Checklist'!$H$5:$H$169,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$169,$A20,'QA Checklist'!$H$5:$H$169,"Fail")</f>
         <v/>
       </c>
       <c r="E20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$168,$A20,'QA Checklist'!$H$5:$H$168,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$169,$A20,'QA Checklist'!$H$5:$H$169,"Pending")</f>
         <v/>
       </c>
       <c r="F20" s="8">
@@ -914,19 +914,19 @@
         </is>
       </c>
       <c r="B21" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$168,$A21)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$169,$A21)</f>
         <v/>
       </c>
       <c r="C21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$168,$A21,'QA Checklist'!$H$5:$H$168,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$168,$A21,'QA Checklist'!$H$5:$H$168,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$169,$A21,'QA Checklist'!$H$5:$H$169,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$169,$A21,'QA Checklist'!$H$5:$H$169,"Pass")</f>
         <v/>
       </c>
       <c r="D21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$168,$A21,'QA Checklist'!$H$5:$H$168,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$168,$A21,'QA Checklist'!$H$5:$H$168,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$169,$A21,'QA Checklist'!$H$5:$H$169,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$169,$A21,'QA Checklist'!$H$5:$H$169,"Fail")</f>
         <v/>
       </c>
       <c r="E21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$168,$A21,'QA Checklist'!$H$5:$H$168,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$169,$A21,'QA Checklist'!$H$5:$H$169,"Pending")</f>
         <v/>
       </c>
       <c r="F21" s="8">
@@ -941,19 +941,19 @@
         </is>
       </c>
       <c r="B22" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$168,$A22)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$169,$A22)</f>
         <v/>
       </c>
       <c r="C22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$168,$A22,'QA Checklist'!$H$5:$H$168,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$168,$A22,'QA Checklist'!$H$5:$H$168,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$169,$A22,'QA Checklist'!$H$5:$H$169,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$169,$A22,'QA Checklist'!$H$5:$H$169,"Pass")</f>
         <v/>
       </c>
       <c r="D22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$168,$A22,'QA Checklist'!$H$5:$H$168,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$168,$A22,'QA Checklist'!$H$5:$H$168,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$169,$A22,'QA Checklist'!$H$5:$H$169,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$169,$A22,'QA Checklist'!$H$5:$H$169,"Fail")</f>
         <v/>
       </c>
       <c r="E22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$168,$A22,'QA Checklist'!$H$5:$H$168,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$169,$A22,'QA Checklist'!$H$5:$H$169,"Pending")</f>
         <v/>
       </c>
       <c r="F22" s="8">
@@ -1023,19 +1023,19 @@
         </is>
       </c>
       <c r="B26" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$168,$A26&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$169,$A26&amp;"*")</f>
         <v/>
       </c>
       <c r="C26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$168,$A26&amp;"*",'QA Checklist'!$H$5:$H$168,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$168,$A26&amp;"*",'QA Checklist'!$H$5:$H$168,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$169,$A26&amp;"*",'QA Checklist'!$H$5:$H$169,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$169,$A26&amp;"*",'QA Checklist'!$H$5:$H$169,"Pass")</f>
         <v/>
       </c>
       <c r="D26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$168,$A26&amp;"*",'QA Checklist'!$H$5:$H$168,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$168,$A26&amp;"*",'QA Checklist'!$H$5:$H$168,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$169,$A26&amp;"*",'QA Checklist'!$H$5:$H$169,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$169,$A26&amp;"*",'QA Checklist'!$H$5:$H$169,"Fail")</f>
         <v/>
       </c>
       <c r="E26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$168,$A26&amp;"*",'QA Checklist'!$H$5:$H$168,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$169,$A26&amp;"*",'QA Checklist'!$H$5:$H$169,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1046,19 +1046,19 @@
         </is>
       </c>
       <c r="B27" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$168,$A27&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$169,$A27&amp;"*")</f>
         <v/>
       </c>
       <c r="C27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$168,$A27&amp;"*",'QA Checklist'!$H$5:$H$168,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$168,$A27&amp;"*",'QA Checklist'!$H$5:$H$168,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$169,$A27&amp;"*",'QA Checklist'!$H$5:$H$169,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$169,$A27&amp;"*",'QA Checklist'!$H$5:$H$169,"Pass")</f>
         <v/>
       </c>
       <c r="D27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$168,$A27&amp;"*",'QA Checklist'!$H$5:$H$168,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$168,$A27&amp;"*",'QA Checklist'!$H$5:$H$168,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$169,$A27&amp;"*",'QA Checklist'!$H$5:$H$169,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$169,$A27&amp;"*",'QA Checklist'!$H$5:$H$169,"Fail")</f>
         <v/>
       </c>
       <c r="E27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$168,$A27&amp;"*",'QA Checklist'!$H$5:$H$168,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$169,$A27&amp;"*",'QA Checklist'!$H$5:$H$169,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1069,19 +1069,19 @@
         </is>
       </c>
       <c r="B28" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$168,$A28&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$169,$A28&amp;"*")</f>
         <v/>
       </c>
       <c r="C28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$168,$A28&amp;"*",'QA Checklist'!$H$5:$H$168,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$168,$A28&amp;"*",'QA Checklist'!$H$5:$H$168,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$169,$A28&amp;"*",'QA Checklist'!$H$5:$H$169,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$169,$A28&amp;"*",'QA Checklist'!$H$5:$H$169,"Pass")</f>
         <v/>
       </c>
       <c r="D28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$168,$A28&amp;"*",'QA Checklist'!$H$5:$H$168,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$168,$A28&amp;"*",'QA Checklist'!$H$5:$H$168,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$169,$A28&amp;"*",'QA Checklist'!$H$5:$H$169,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$169,$A28&amp;"*",'QA Checklist'!$H$5:$H$169,"Fail")</f>
         <v/>
       </c>
       <c r="E28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$168,$A28&amp;"*",'QA Checklist'!$H$5:$H$168,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$169,$A28&amp;"*",'QA Checklist'!$H$5:$H$169,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1096,7 +1096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I168"/>
+  <dimension ref="A1:I169"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8435,12 +8435,59 @@
         </is>
       </c>
     </row>
+    <row r="169">
+      <c r="A169" s="12" t="inlineStr">
+        <is>
+          <t>SA-43</t>
+        </is>
+      </c>
+      <c r="B169" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="C169" s="13" t="inlineStr">
+        <is>
+          <t>Tier 2 (Workflow &amp; Ergonomics)</t>
+        </is>
+      </c>
+      <c r="D169" s="13" t="inlineStr">
+        <is>
+          <t>Checklist Checkpoints Selection-Only</t>
+        </is>
+      </c>
+      <c r="E169" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="F169" s="13" t="inlineStr">
+        <is>
+          <t>Log in as Service Advisor, open 2025 RO Excel Studio, switch to Checklist tab, and review each checkpoint row</t>
+        </is>
+      </c>
+      <c r="G169" s="13" t="inlineStr">
+        <is>
+          <t>Each checkpoint shows only its name and the Good / Attention / Defect / N/A selector (battery Good / Replace / N/A) with no text box underneath; findings are typed only in Inspector Remarks / Discovered Deficiencies at the bottom; the Checklist PDF and Excel output are unchanged</t>
+        </is>
+      </c>
+      <c r="H169" s="14" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="I169" s="13" t="inlineStr">
+        <is>
+          <t>Verified by Automated Unit Tests (155/155 passing in tests/frontend/sla_and_logic.test.js AUT-FRONT-126) and headless Chrome render inspection</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:I168"/>
+  <autoFilter ref="A4:I169"/>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="H5:H168">
+  <conditionalFormatting sqref="H5:H169">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$H5="Passed"</formula>
     </cfRule>
@@ -8457,13 +8504,13 @@
       <formula>$H5="Pending"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A5:A168">
+  <conditionalFormatting sqref="A5:A169">
     <cfRule type="expression" priority="6" dxfId="3">
-      <formula>COUNTIF($A$5:$A$168,$A5)&gt;1</formula>
+      <formula>COUNTIF($A$5:$A$169,$A5)&gt;1</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H5:H168" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H5:H169" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pending,Passed,Failed"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat(REV-168): add gray header bands to checklist sections
Render each checklist section title (Interior/Exterior, Battery
Performance, Under Hood, Under Vehicle, Tire Condition, Brake Condition)
as a band in the printed form's header gray (#D0D1D3) with bold black
text, so each part is clearly separated. Bump cache buster to v=3.21,
add AUT-FRONT-127, and sync REV-168 / SA-44 into the revisions log,
checklists and QA workbook.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
+++ b/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
@@ -11,7 +11,7 @@
     <sheet name="QA Checklist" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$169</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$170</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'QA Checklist'!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTA('QA Checklist'!$A$5:$A$169)</f>
+        <f>COUNTA('QA Checklist'!$A$5:$A$170)</f>
         <v/>
       </c>
     </row>
@@ -594,7 +594,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$169,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$169,"Pass")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$170,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$170,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$169,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$169,"Fail")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$170,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$170,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -616,7 +616,7 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$169,"Pending")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$170,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -671,19 +671,19 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$169,$A12)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$170,$A12)</f>
         <v/>
       </c>
       <c r="C12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$169,$A12,'QA Checklist'!$H$5:$H$169,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$169,$A12,'QA Checklist'!$H$5:$H$169,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$170,$A12,'QA Checklist'!$H$5:$H$170,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$170,$A12,'QA Checklist'!$H$5:$H$170,"Pass")</f>
         <v/>
       </c>
       <c r="D12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$169,$A12,'QA Checklist'!$H$5:$H$169,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$169,$A12,'QA Checklist'!$H$5:$H$169,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$170,$A12,'QA Checklist'!$H$5:$H$170,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$170,$A12,'QA Checklist'!$H$5:$H$170,"Fail")</f>
         <v/>
       </c>
       <c r="E12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$169,$A12,'QA Checklist'!$H$5:$H$169,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$170,$A12,'QA Checklist'!$H$5:$H$170,"Pending")</f>
         <v/>
       </c>
       <c r="F12" s="8">
@@ -698,19 +698,19 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$169,$A13)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$170,$A13)</f>
         <v/>
       </c>
       <c r="C13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$169,$A13,'QA Checklist'!$H$5:$H$169,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$169,$A13,'QA Checklist'!$H$5:$H$169,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$170,$A13,'QA Checklist'!$H$5:$H$170,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$170,$A13,'QA Checklist'!$H$5:$H$170,"Pass")</f>
         <v/>
       </c>
       <c r="D13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$169,$A13,'QA Checklist'!$H$5:$H$169,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$169,$A13,'QA Checklist'!$H$5:$H$169,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$170,$A13,'QA Checklist'!$H$5:$H$170,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$170,$A13,'QA Checklist'!$H$5:$H$170,"Fail")</f>
         <v/>
       </c>
       <c r="E13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$169,$A13,'QA Checklist'!$H$5:$H$169,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$170,$A13,'QA Checklist'!$H$5:$H$170,"Pending")</f>
         <v/>
       </c>
       <c r="F13" s="8">
@@ -725,19 +725,19 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$169,$A14)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$170,$A14)</f>
         <v/>
       </c>
       <c r="C14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$169,$A14,'QA Checklist'!$H$5:$H$169,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$169,$A14,'QA Checklist'!$H$5:$H$169,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$170,$A14,'QA Checklist'!$H$5:$H$170,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$170,$A14,'QA Checklist'!$H$5:$H$170,"Pass")</f>
         <v/>
       </c>
       <c r="D14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$169,$A14,'QA Checklist'!$H$5:$H$169,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$169,$A14,'QA Checklist'!$H$5:$H$169,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$170,$A14,'QA Checklist'!$H$5:$H$170,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$170,$A14,'QA Checklist'!$H$5:$H$170,"Fail")</f>
         <v/>
       </c>
       <c r="E14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$169,$A14,'QA Checklist'!$H$5:$H$169,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$170,$A14,'QA Checklist'!$H$5:$H$170,"Pending")</f>
         <v/>
       </c>
       <c r="F14" s="8">
@@ -752,19 +752,19 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$169,$A15)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$170,$A15)</f>
         <v/>
       </c>
       <c r="C15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$169,$A15,'QA Checklist'!$H$5:$H$169,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$169,$A15,'QA Checklist'!$H$5:$H$169,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$170,$A15,'QA Checklist'!$H$5:$H$170,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$170,$A15,'QA Checklist'!$H$5:$H$170,"Pass")</f>
         <v/>
       </c>
       <c r="D15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$169,$A15,'QA Checklist'!$H$5:$H$169,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$169,$A15,'QA Checklist'!$H$5:$H$169,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$170,$A15,'QA Checklist'!$H$5:$H$170,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$170,$A15,'QA Checklist'!$H$5:$H$170,"Fail")</f>
         <v/>
       </c>
       <c r="E15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$169,$A15,'QA Checklist'!$H$5:$H$169,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$170,$A15,'QA Checklist'!$H$5:$H$170,"Pending")</f>
         <v/>
       </c>
       <c r="F15" s="8">
@@ -779,19 +779,19 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$169,$A16)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$170,$A16)</f>
         <v/>
       </c>
       <c r="C16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$169,$A16,'QA Checklist'!$H$5:$H$169,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$169,$A16,'QA Checklist'!$H$5:$H$169,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$170,$A16,'QA Checklist'!$H$5:$H$170,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$170,$A16,'QA Checklist'!$H$5:$H$170,"Pass")</f>
         <v/>
       </c>
       <c r="D16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$169,$A16,'QA Checklist'!$H$5:$H$169,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$169,$A16,'QA Checklist'!$H$5:$H$169,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$170,$A16,'QA Checklist'!$H$5:$H$170,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$170,$A16,'QA Checklist'!$H$5:$H$170,"Fail")</f>
         <v/>
       </c>
       <c r="E16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$169,$A16,'QA Checklist'!$H$5:$H$169,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$170,$A16,'QA Checklist'!$H$5:$H$170,"Pending")</f>
         <v/>
       </c>
       <c r="F16" s="8">
@@ -806,19 +806,19 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$169,$A17)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$170,$A17)</f>
         <v/>
       </c>
       <c r="C17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$169,$A17,'QA Checklist'!$H$5:$H$169,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$169,$A17,'QA Checklist'!$H$5:$H$169,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$170,$A17,'QA Checklist'!$H$5:$H$170,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$170,$A17,'QA Checklist'!$H$5:$H$170,"Pass")</f>
         <v/>
       </c>
       <c r="D17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$169,$A17,'QA Checklist'!$H$5:$H$169,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$169,$A17,'QA Checklist'!$H$5:$H$169,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$170,$A17,'QA Checklist'!$H$5:$H$170,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$170,$A17,'QA Checklist'!$H$5:$H$170,"Fail")</f>
         <v/>
       </c>
       <c r="E17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$169,$A17,'QA Checklist'!$H$5:$H$169,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$170,$A17,'QA Checklist'!$H$5:$H$170,"Pending")</f>
         <v/>
       </c>
       <c r="F17" s="8">
@@ -833,19 +833,19 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$169,$A18)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$170,$A18)</f>
         <v/>
       </c>
       <c r="C18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$169,$A18,'QA Checklist'!$H$5:$H$169,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$169,$A18,'QA Checklist'!$H$5:$H$169,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$170,$A18,'QA Checklist'!$H$5:$H$170,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$170,$A18,'QA Checklist'!$H$5:$H$170,"Pass")</f>
         <v/>
       </c>
       <c r="D18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$169,$A18,'QA Checklist'!$H$5:$H$169,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$169,$A18,'QA Checklist'!$H$5:$H$169,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$170,$A18,'QA Checklist'!$H$5:$H$170,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$170,$A18,'QA Checklist'!$H$5:$H$170,"Fail")</f>
         <v/>
       </c>
       <c r="E18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$169,$A18,'QA Checklist'!$H$5:$H$169,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$170,$A18,'QA Checklist'!$H$5:$H$170,"Pending")</f>
         <v/>
       </c>
       <c r="F18" s="8">
@@ -860,19 +860,19 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$169,$A19)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$170,$A19)</f>
         <v/>
       </c>
       <c r="C19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$169,$A19,'QA Checklist'!$H$5:$H$169,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$169,$A19,'QA Checklist'!$H$5:$H$169,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$170,$A19,'QA Checklist'!$H$5:$H$170,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$170,$A19,'QA Checklist'!$H$5:$H$170,"Pass")</f>
         <v/>
       </c>
       <c r="D19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$169,$A19,'QA Checklist'!$H$5:$H$169,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$169,$A19,'QA Checklist'!$H$5:$H$169,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$170,$A19,'QA Checklist'!$H$5:$H$170,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$170,$A19,'QA Checklist'!$H$5:$H$170,"Fail")</f>
         <v/>
       </c>
       <c r="E19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$169,$A19,'QA Checklist'!$H$5:$H$169,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$170,$A19,'QA Checklist'!$H$5:$H$170,"Pending")</f>
         <v/>
       </c>
       <c r="F19" s="8">
@@ -887,19 +887,19 @@
         </is>
       </c>
       <c r="B20" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$169,$A20)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$170,$A20)</f>
         <v/>
       </c>
       <c r="C20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$169,$A20,'QA Checklist'!$H$5:$H$169,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$169,$A20,'QA Checklist'!$H$5:$H$169,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$170,$A20,'QA Checklist'!$H$5:$H$170,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$170,$A20,'QA Checklist'!$H$5:$H$170,"Pass")</f>
         <v/>
       </c>
       <c r="D20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$169,$A20,'QA Checklist'!$H$5:$H$169,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$169,$A20,'QA Checklist'!$H$5:$H$169,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$170,$A20,'QA Checklist'!$H$5:$H$170,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$170,$A20,'QA Checklist'!$H$5:$H$170,"Fail")</f>
         <v/>
       </c>
       <c r="E20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$169,$A20,'QA Checklist'!$H$5:$H$169,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$170,$A20,'QA Checklist'!$H$5:$H$170,"Pending")</f>
         <v/>
       </c>
       <c r="F20" s="8">
@@ -914,19 +914,19 @@
         </is>
       </c>
       <c r="B21" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$169,$A21)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$170,$A21)</f>
         <v/>
       </c>
       <c r="C21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$169,$A21,'QA Checklist'!$H$5:$H$169,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$169,$A21,'QA Checklist'!$H$5:$H$169,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$170,$A21,'QA Checklist'!$H$5:$H$170,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$170,$A21,'QA Checklist'!$H$5:$H$170,"Pass")</f>
         <v/>
       </c>
       <c r="D21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$169,$A21,'QA Checklist'!$H$5:$H$169,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$169,$A21,'QA Checklist'!$H$5:$H$169,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$170,$A21,'QA Checklist'!$H$5:$H$170,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$170,$A21,'QA Checklist'!$H$5:$H$170,"Fail")</f>
         <v/>
       </c>
       <c r="E21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$169,$A21,'QA Checklist'!$H$5:$H$169,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$170,$A21,'QA Checklist'!$H$5:$H$170,"Pending")</f>
         <v/>
       </c>
       <c r="F21" s="8">
@@ -941,19 +941,19 @@
         </is>
       </c>
       <c r="B22" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$169,$A22)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$170,$A22)</f>
         <v/>
       </c>
       <c r="C22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$169,$A22,'QA Checklist'!$H$5:$H$169,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$169,$A22,'QA Checklist'!$H$5:$H$169,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$170,$A22,'QA Checklist'!$H$5:$H$170,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$170,$A22,'QA Checklist'!$H$5:$H$170,"Pass")</f>
         <v/>
       </c>
       <c r="D22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$169,$A22,'QA Checklist'!$H$5:$H$169,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$169,$A22,'QA Checklist'!$H$5:$H$169,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$170,$A22,'QA Checklist'!$H$5:$H$170,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$170,$A22,'QA Checklist'!$H$5:$H$170,"Fail")</f>
         <v/>
       </c>
       <c r="E22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$169,$A22,'QA Checklist'!$H$5:$H$169,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$170,$A22,'QA Checklist'!$H$5:$H$170,"Pending")</f>
         <v/>
       </c>
       <c r="F22" s="8">
@@ -1023,19 +1023,19 @@
         </is>
       </c>
       <c r="B26" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$169,$A26&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$170,$A26&amp;"*")</f>
         <v/>
       </c>
       <c r="C26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$169,$A26&amp;"*",'QA Checklist'!$H$5:$H$169,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$169,$A26&amp;"*",'QA Checklist'!$H$5:$H$169,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$170,$A26&amp;"*",'QA Checklist'!$H$5:$H$170,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$170,$A26&amp;"*",'QA Checklist'!$H$5:$H$170,"Pass")</f>
         <v/>
       </c>
       <c r="D26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$169,$A26&amp;"*",'QA Checklist'!$H$5:$H$169,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$169,$A26&amp;"*",'QA Checklist'!$H$5:$H$169,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$170,$A26&amp;"*",'QA Checklist'!$H$5:$H$170,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$170,$A26&amp;"*",'QA Checklist'!$H$5:$H$170,"Fail")</f>
         <v/>
       </c>
       <c r="E26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$169,$A26&amp;"*",'QA Checklist'!$H$5:$H$169,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$170,$A26&amp;"*",'QA Checklist'!$H$5:$H$170,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1046,19 +1046,19 @@
         </is>
       </c>
       <c r="B27" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$169,$A27&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$170,$A27&amp;"*")</f>
         <v/>
       </c>
       <c r="C27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$169,$A27&amp;"*",'QA Checklist'!$H$5:$H$169,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$169,$A27&amp;"*",'QA Checklist'!$H$5:$H$169,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$170,$A27&amp;"*",'QA Checklist'!$H$5:$H$170,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$170,$A27&amp;"*",'QA Checklist'!$H$5:$H$170,"Pass")</f>
         <v/>
       </c>
       <c r="D27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$169,$A27&amp;"*",'QA Checklist'!$H$5:$H$169,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$169,$A27&amp;"*",'QA Checklist'!$H$5:$H$169,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$170,$A27&amp;"*",'QA Checklist'!$H$5:$H$170,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$170,$A27&amp;"*",'QA Checklist'!$H$5:$H$170,"Fail")</f>
         <v/>
       </c>
       <c r="E27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$169,$A27&amp;"*",'QA Checklist'!$H$5:$H$169,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$170,$A27&amp;"*",'QA Checklist'!$H$5:$H$170,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1069,19 +1069,19 @@
         </is>
       </c>
       <c r="B28" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$169,$A28&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$170,$A28&amp;"*")</f>
         <v/>
       </c>
       <c r="C28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$169,$A28&amp;"*",'QA Checklist'!$H$5:$H$169,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$169,$A28&amp;"*",'QA Checklist'!$H$5:$H$169,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$170,$A28&amp;"*",'QA Checklist'!$H$5:$H$170,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$170,$A28&amp;"*",'QA Checklist'!$H$5:$H$170,"Pass")</f>
         <v/>
       </c>
       <c r="D28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$169,$A28&amp;"*",'QA Checklist'!$H$5:$H$169,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$169,$A28&amp;"*",'QA Checklist'!$H$5:$H$169,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$170,$A28&amp;"*",'QA Checklist'!$H$5:$H$170,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$170,$A28&amp;"*",'QA Checklist'!$H$5:$H$170,"Fail")</f>
         <v/>
       </c>
       <c r="E28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$169,$A28&amp;"*",'QA Checklist'!$H$5:$H$169,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$170,$A28&amp;"*",'QA Checklist'!$H$5:$H$170,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1096,7 +1096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I169"/>
+  <dimension ref="A1:I170"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8482,12 +8482,59 @@
         </is>
       </c>
     </row>
+    <row r="170">
+      <c r="A170" s="12" t="inlineStr">
+        <is>
+          <t>SA-44</t>
+        </is>
+      </c>
+      <c r="B170" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="C170" s="13" t="inlineStr">
+        <is>
+          <t>Tier 2 (Workflow &amp; Ergonomics)</t>
+        </is>
+      </c>
+      <c r="D170" s="13" t="inlineStr">
+        <is>
+          <t>Checklist Section Header Bands</t>
+        </is>
+      </c>
+      <c r="E170" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="F170" s="13" t="inlineStr">
+        <is>
+          <t>Log in as Service Advisor, open 2025 RO Excel Studio, switch to Checklist tab, and scroll through the Multi-Point Receiving Checkpoints</t>
+        </is>
+      </c>
+      <c r="G170" s="13" t="inlineStr">
+        <is>
+          <t>Each section title (Interior/Exterior, Battery Performance (see attached ED-18 printout), Under Hood, Under Vehicle, Tire Condition, Brake Condition) appears in bold black text on a gray band matching the printed form header, making it clear where each part starts</t>
+        </is>
+      </c>
+      <c r="H170" s="14" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="I170" s="13" t="inlineStr">
+        <is>
+          <t>Verified by Automated Unit Tests (156/156 passing in tests/frontend/sla_and_logic.test.js AUT-FRONT-127) and headless Chrome render inspection</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:I169"/>
+  <autoFilter ref="A4:I170"/>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="H5:H169">
+  <conditionalFormatting sqref="H5:H170">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$H5="Passed"</formula>
     </cfRule>
@@ -8504,13 +8551,13 @@
       <formula>$H5="Pending"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A5:A169">
+  <conditionalFormatting sqref="A5:A170">
     <cfRule type="expression" priority="6" dxfId="3">
-      <formula>COUNTIF($A$5:$A$169,$A5)&gt;1</formula>
+      <formula>COUNTIF($A$5:$A$170,$A5)&gt;1</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H5:H169" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H5:H170" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pending,Passed,Failed"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat(REV-169): shared PDF toolbar and CheckList design on all studio tabs
Give all four studio tabs one PDF view toolbar: title, subtitle and a
neutral Live synced tag, then Fit/185% zoom, outlined Maximize, Full PDF
and Download PDF buttons that no longer wrap, and the green Export
.xlsx. Apply the CheckList design to the Job Order, Quotation and
Billing editors (flat cards, gray labels and focus rings, neutral add
and preset buttons, original quick-action colors kept). Close the Job
Order Studio header card so later cards are no longer nested. Bump
cache buster to v=3.22, add AUT-FRONT-128, and sync REV-169 / SA-45 into
the revisions log, checklists and QA workbook.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
+++ b/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
@@ -11,7 +11,7 @@
     <sheet name="QA Checklist" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$170</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$171</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'QA Checklist'!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTA('QA Checklist'!$A$5:$A$170)</f>
+        <f>COUNTA('QA Checklist'!$A$5:$A$171)</f>
         <v/>
       </c>
     </row>
@@ -594,7 +594,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$170,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$170,"Pass")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$171,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$171,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$170,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$170,"Fail")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$171,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$171,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -616,7 +616,7 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$170,"Pending")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$171,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -671,19 +671,19 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$170,$A12)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$171,$A12)</f>
         <v/>
       </c>
       <c r="C12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$170,$A12,'QA Checklist'!$H$5:$H$170,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$170,$A12,'QA Checklist'!$H$5:$H$170,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$171,$A12,'QA Checklist'!$H$5:$H$171,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$171,$A12,'QA Checklist'!$H$5:$H$171,"Pass")</f>
         <v/>
       </c>
       <c r="D12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$170,$A12,'QA Checklist'!$H$5:$H$170,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$170,$A12,'QA Checklist'!$H$5:$H$170,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$171,$A12,'QA Checklist'!$H$5:$H$171,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$171,$A12,'QA Checklist'!$H$5:$H$171,"Fail")</f>
         <v/>
       </c>
       <c r="E12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$170,$A12,'QA Checklist'!$H$5:$H$170,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$171,$A12,'QA Checklist'!$H$5:$H$171,"Pending")</f>
         <v/>
       </c>
       <c r="F12" s="8">
@@ -698,19 +698,19 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$170,$A13)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$171,$A13)</f>
         <v/>
       </c>
       <c r="C13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$170,$A13,'QA Checklist'!$H$5:$H$170,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$170,$A13,'QA Checklist'!$H$5:$H$170,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$171,$A13,'QA Checklist'!$H$5:$H$171,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$171,$A13,'QA Checklist'!$H$5:$H$171,"Pass")</f>
         <v/>
       </c>
       <c r="D13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$170,$A13,'QA Checklist'!$H$5:$H$170,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$170,$A13,'QA Checklist'!$H$5:$H$170,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$171,$A13,'QA Checklist'!$H$5:$H$171,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$171,$A13,'QA Checklist'!$H$5:$H$171,"Fail")</f>
         <v/>
       </c>
       <c r="E13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$170,$A13,'QA Checklist'!$H$5:$H$170,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$171,$A13,'QA Checklist'!$H$5:$H$171,"Pending")</f>
         <v/>
       </c>
       <c r="F13" s="8">
@@ -725,19 +725,19 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$170,$A14)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$171,$A14)</f>
         <v/>
       </c>
       <c r="C14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$170,$A14,'QA Checklist'!$H$5:$H$170,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$170,$A14,'QA Checklist'!$H$5:$H$170,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$171,$A14,'QA Checklist'!$H$5:$H$171,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$171,$A14,'QA Checklist'!$H$5:$H$171,"Pass")</f>
         <v/>
       </c>
       <c r="D14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$170,$A14,'QA Checklist'!$H$5:$H$170,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$170,$A14,'QA Checklist'!$H$5:$H$170,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$171,$A14,'QA Checklist'!$H$5:$H$171,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$171,$A14,'QA Checklist'!$H$5:$H$171,"Fail")</f>
         <v/>
       </c>
       <c r="E14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$170,$A14,'QA Checklist'!$H$5:$H$170,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$171,$A14,'QA Checklist'!$H$5:$H$171,"Pending")</f>
         <v/>
       </c>
       <c r="F14" s="8">
@@ -752,19 +752,19 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$170,$A15)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$171,$A15)</f>
         <v/>
       </c>
       <c r="C15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$170,$A15,'QA Checklist'!$H$5:$H$170,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$170,$A15,'QA Checklist'!$H$5:$H$170,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$171,$A15,'QA Checklist'!$H$5:$H$171,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$171,$A15,'QA Checklist'!$H$5:$H$171,"Pass")</f>
         <v/>
       </c>
       <c r="D15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$170,$A15,'QA Checklist'!$H$5:$H$170,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$170,$A15,'QA Checklist'!$H$5:$H$170,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$171,$A15,'QA Checklist'!$H$5:$H$171,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$171,$A15,'QA Checklist'!$H$5:$H$171,"Fail")</f>
         <v/>
       </c>
       <c r="E15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$170,$A15,'QA Checklist'!$H$5:$H$170,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$171,$A15,'QA Checklist'!$H$5:$H$171,"Pending")</f>
         <v/>
       </c>
       <c r="F15" s="8">
@@ -779,19 +779,19 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$170,$A16)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$171,$A16)</f>
         <v/>
       </c>
       <c r="C16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$170,$A16,'QA Checklist'!$H$5:$H$170,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$170,$A16,'QA Checklist'!$H$5:$H$170,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$171,$A16,'QA Checklist'!$H$5:$H$171,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$171,$A16,'QA Checklist'!$H$5:$H$171,"Pass")</f>
         <v/>
       </c>
       <c r="D16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$170,$A16,'QA Checklist'!$H$5:$H$170,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$170,$A16,'QA Checklist'!$H$5:$H$170,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$171,$A16,'QA Checklist'!$H$5:$H$171,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$171,$A16,'QA Checklist'!$H$5:$H$171,"Fail")</f>
         <v/>
       </c>
       <c r="E16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$170,$A16,'QA Checklist'!$H$5:$H$170,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$171,$A16,'QA Checklist'!$H$5:$H$171,"Pending")</f>
         <v/>
       </c>
       <c r="F16" s="8">
@@ -806,19 +806,19 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$170,$A17)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$171,$A17)</f>
         <v/>
       </c>
       <c r="C17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$170,$A17,'QA Checklist'!$H$5:$H$170,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$170,$A17,'QA Checklist'!$H$5:$H$170,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$171,$A17,'QA Checklist'!$H$5:$H$171,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$171,$A17,'QA Checklist'!$H$5:$H$171,"Pass")</f>
         <v/>
       </c>
       <c r="D17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$170,$A17,'QA Checklist'!$H$5:$H$170,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$170,$A17,'QA Checklist'!$H$5:$H$170,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$171,$A17,'QA Checklist'!$H$5:$H$171,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$171,$A17,'QA Checklist'!$H$5:$H$171,"Fail")</f>
         <v/>
       </c>
       <c r="E17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$170,$A17,'QA Checklist'!$H$5:$H$170,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$171,$A17,'QA Checklist'!$H$5:$H$171,"Pending")</f>
         <v/>
       </c>
       <c r="F17" s="8">
@@ -833,19 +833,19 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$170,$A18)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$171,$A18)</f>
         <v/>
       </c>
       <c r="C18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$170,$A18,'QA Checklist'!$H$5:$H$170,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$170,$A18,'QA Checklist'!$H$5:$H$170,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$171,$A18,'QA Checklist'!$H$5:$H$171,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$171,$A18,'QA Checklist'!$H$5:$H$171,"Pass")</f>
         <v/>
       </c>
       <c r="D18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$170,$A18,'QA Checklist'!$H$5:$H$170,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$170,$A18,'QA Checklist'!$H$5:$H$170,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$171,$A18,'QA Checklist'!$H$5:$H$171,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$171,$A18,'QA Checklist'!$H$5:$H$171,"Fail")</f>
         <v/>
       </c>
       <c r="E18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$170,$A18,'QA Checklist'!$H$5:$H$170,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$171,$A18,'QA Checklist'!$H$5:$H$171,"Pending")</f>
         <v/>
       </c>
       <c r="F18" s="8">
@@ -860,19 +860,19 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$170,$A19)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$171,$A19)</f>
         <v/>
       </c>
       <c r="C19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$170,$A19,'QA Checklist'!$H$5:$H$170,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$170,$A19,'QA Checklist'!$H$5:$H$170,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$171,$A19,'QA Checklist'!$H$5:$H$171,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$171,$A19,'QA Checklist'!$H$5:$H$171,"Pass")</f>
         <v/>
       </c>
       <c r="D19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$170,$A19,'QA Checklist'!$H$5:$H$170,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$170,$A19,'QA Checklist'!$H$5:$H$170,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$171,$A19,'QA Checklist'!$H$5:$H$171,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$171,$A19,'QA Checklist'!$H$5:$H$171,"Fail")</f>
         <v/>
       </c>
       <c r="E19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$170,$A19,'QA Checklist'!$H$5:$H$170,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$171,$A19,'QA Checklist'!$H$5:$H$171,"Pending")</f>
         <v/>
       </c>
       <c r="F19" s="8">
@@ -887,19 +887,19 @@
         </is>
       </c>
       <c r="B20" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$170,$A20)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$171,$A20)</f>
         <v/>
       </c>
       <c r="C20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$170,$A20,'QA Checklist'!$H$5:$H$170,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$170,$A20,'QA Checklist'!$H$5:$H$170,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$171,$A20,'QA Checklist'!$H$5:$H$171,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$171,$A20,'QA Checklist'!$H$5:$H$171,"Pass")</f>
         <v/>
       </c>
       <c r="D20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$170,$A20,'QA Checklist'!$H$5:$H$170,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$170,$A20,'QA Checklist'!$H$5:$H$170,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$171,$A20,'QA Checklist'!$H$5:$H$171,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$171,$A20,'QA Checklist'!$H$5:$H$171,"Fail")</f>
         <v/>
       </c>
       <c r="E20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$170,$A20,'QA Checklist'!$H$5:$H$170,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$171,$A20,'QA Checklist'!$H$5:$H$171,"Pending")</f>
         <v/>
       </c>
       <c r="F20" s="8">
@@ -914,19 +914,19 @@
         </is>
       </c>
       <c r="B21" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$170,$A21)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$171,$A21)</f>
         <v/>
       </c>
       <c r="C21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$170,$A21,'QA Checklist'!$H$5:$H$170,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$170,$A21,'QA Checklist'!$H$5:$H$170,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$171,$A21,'QA Checklist'!$H$5:$H$171,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$171,$A21,'QA Checklist'!$H$5:$H$171,"Pass")</f>
         <v/>
       </c>
       <c r="D21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$170,$A21,'QA Checklist'!$H$5:$H$170,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$170,$A21,'QA Checklist'!$H$5:$H$170,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$171,$A21,'QA Checklist'!$H$5:$H$171,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$171,$A21,'QA Checklist'!$H$5:$H$171,"Fail")</f>
         <v/>
       </c>
       <c r="E21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$170,$A21,'QA Checklist'!$H$5:$H$170,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$171,$A21,'QA Checklist'!$H$5:$H$171,"Pending")</f>
         <v/>
       </c>
       <c r="F21" s="8">
@@ -941,19 +941,19 @@
         </is>
       </c>
       <c r="B22" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$170,$A22)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$171,$A22)</f>
         <v/>
       </c>
       <c r="C22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$170,$A22,'QA Checklist'!$H$5:$H$170,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$170,$A22,'QA Checklist'!$H$5:$H$170,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$171,$A22,'QA Checklist'!$H$5:$H$171,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$171,$A22,'QA Checklist'!$H$5:$H$171,"Pass")</f>
         <v/>
       </c>
       <c r="D22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$170,$A22,'QA Checklist'!$H$5:$H$170,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$170,$A22,'QA Checklist'!$H$5:$H$170,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$171,$A22,'QA Checklist'!$H$5:$H$171,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$171,$A22,'QA Checklist'!$H$5:$H$171,"Fail")</f>
         <v/>
       </c>
       <c r="E22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$170,$A22,'QA Checklist'!$H$5:$H$170,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$171,$A22,'QA Checklist'!$H$5:$H$171,"Pending")</f>
         <v/>
       </c>
       <c r="F22" s="8">
@@ -1023,19 +1023,19 @@
         </is>
       </c>
       <c r="B26" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$170,$A26&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$171,$A26&amp;"*")</f>
         <v/>
       </c>
       <c r="C26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$170,$A26&amp;"*",'QA Checklist'!$H$5:$H$170,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$170,$A26&amp;"*",'QA Checklist'!$H$5:$H$170,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$171,$A26&amp;"*",'QA Checklist'!$H$5:$H$171,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$171,$A26&amp;"*",'QA Checklist'!$H$5:$H$171,"Pass")</f>
         <v/>
       </c>
       <c r="D26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$170,$A26&amp;"*",'QA Checklist'!$H$5:$H$170,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$170,$A26&amp;"*",'QA Checklist'!$H$5:$H$170,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$171,$A26&amp;"*",'QA Checklist'!$H$5:$H$171,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$171,$A26&amp;"*",'QA Checklist'!$H$5:$H$171,"Fail")</f>
         <v/>
       </c>
       <c r="E26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$170,$A26&amp;"*",'QA Checklist'!$H$5:$H$170,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$171,$A26&amp;"*",'QA Checklist'!$H$5:$H$171,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1046,19 +1046,19 @@
         </is>
       </c>
       <c r="B27" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$170,$A27&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$171,$A27&amp;"*")</f>
         <v/>
       </c>
       <c r="C27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$170,$A27&amp;"*",'QA Checklist'!$H$5:$H$170,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$170,$A27&amp;"*",'QA Checklist'!$H$5:$H$170,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$171,$A27&amp;"*",'QA Checklist'!$H$5:$H$171,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$171,$A27&amp;"*",'QA Checklist'!$H$5:$H$171,"Pass")</f>
         <v/>
       </c>
       <c r="D27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$170,$A27&amp;"*",'QA Checklist'!$H$5:$H$170,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$170,$A27&amp;"*",'QA Checklist'!$H$5:$H$170,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$171,$A27&amp;"*",'QA Checklist'!$H$5:$H$171,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$171,$A27&amp;"*",'QA Checklist'!$H$5:$H$171,"Fail")</f>
         <v/>
       </c>
       <c r="E27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$170,$A27&amp;"*",'QA Checklist'!$H$5:$H$170,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$171,$A27&amp;"*",'QA Checklist'!$H$5:$H$171,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1069,19 +1069,19 @@
         </is>
       </c>
       <c r="B28" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$170,$A28&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$171,$A28&amp;"*")</f>
         <v/>
       </c>
       <c r="C28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$170,$A28&amp;"*",'QA Checklist'!$H$5:$H$170,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$170,$A28&amp;"*",'QA Checklist'!$H$5:$H$170,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$171,$A28&amp;"*",'QA Checklist'!$H$5:$H$171,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$171,$A28&amp;"*",'QA Checklist'!$H$5:$H$171,"Pass")</f>
         <v/>
       </c>
       <c r="D28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$170,$A28&amp;"*",'QA Checklist'!$H$5:$H$170,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$170,$A28&amp;"*",'QA Checklist'!$H$5:$H$170,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$171,$A28&amp;"*",'QA Checklist'!$H$5:$H$171,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$171,$A28&amp;"*",'QA Checklist'!$H$5:$H$171,"Fail")</f>
         <v/>
       </c>
       <c r="E28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$170,$A28&amp;"*",'QA Checklist'!$H$5:$H$170,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$171,$A28&amp;"*",'QA Checklist'!$H$5:$H$171,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1096,7 +1096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I170"/>
+  <dimension ref="A1:I171"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8529,12 +8529,59 @@
         </is>
       </c>
     </row>
+    <row r="171">
+      <c r="A171" s="12" t="inlineStr">
+        <is>
+          <t>SA-45</t>
+        </is>
+      </c>
+      <c r="B171" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="C171" s="13" t="inlineStr">
+        <is>
+          <t>Tier 2 (Workflow &amp; Ergonomics)</t>
+        </is>
+      </c>
+      <c r="D171" s="13" t="inlineStr">
+        <is>
+          <t>Studio-Wide CheckList Design &amp; Shared PDF Toolbar</t>
+        </is>
+      </c>
+      <c r="E171" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="F171" s="13" t="inlineStr">
+        <is>
+          <t>Log in as Service Advisor, open 2025 RO Excel Studio, and switch between Job_Order, Quotation_No, Billing_No and CheckList_Result; use Fit / 185%, Maximize, Full PDF, Download PDF and Export .xlsx on each tab</t>
+        </is>
+      </c>
+      <c r="G171" s="13" t="inlineStr">
+        <is>
+          <t>All four tabs show the same PDF toolbar: sheet title and subtitle with a Live synced tag, then Fit / 185%, Maximize, Full PDF and Download PDF on one line without wrapped labels, and the green Export .xlsx button; the Job Order, Quotation and Billing editors match the CheckList design (flat cards, small gray section titles and labels, gray input focus, neutral add and preset buttons) with Save Draft / Reset / Export keeping their original colors; on Job Order, Customer Dossier and the following cards appear as separate cards; Maximize turns dark while active</t>
+        </is>
+      </c>
+      <c r="H171" s="14" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="I171" s="13" t="inlineStr">
+        <is>
+          <t>Verified by Automated Unit Tests (157/157 passing in tests/frontend/sla_and_logic.test.js AUT-FRONT-128) and headless Chrome renders of all four tabs</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:I170"/>
+  <autoFilter ref="A4:I171"/>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="H5:H170">
+  <conditionalFormatting sqref="H5:H171">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$H5="Passed"</formula>
     </cfRule>
@@ -8551,13 +8598,13 @@
       <formula>$H5="Pending"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A5:A170">
+  <conditionalFormatting sqref="A5:A171">
     <cfRule type="expression" priority="6" dxfId="3">
-      <formula>COUNTIF($A$5:$A$170,$A5)&gt;1</formula>
+      <formula>COUNTIF($A$5:$A$171,$A5)&gt;1</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H5:H170" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H5:H171" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pending,Passed,Failed"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
fix(REV-170): make PDF and Excel show identical data and totals
Add shared header, line-item and totals rules used by the Quotation,
Billing and Checklist PDFs, the Excel export and the on-screen totals.
VAT 12% now follows the official workbook (labor only) and the billing
discount is subtracted in both the PDF and Excel. The export replaces
template formulas that showed different data: the Claim Stub (=K2),
labor cells (=D*550) and the =Job_Order header cells on the Quotation,
Billing and Checklist sheets. Billing sheets now list the Billing items,
and the Job Order TOTAL (K51) is filled. Verified end to end against a
LibreOffice-recalculated workbook. Bump cache buster to v=3.23, add
AUT-FRONT-129, and sync REV-170 / SA-46 into the revisions log,
checklists and QA workbook.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
+++ b/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
@@ -11,7 +11,7 @@
     <sheet name="QA Checklist" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$171</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$172</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'QA Checklist'!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTA('QA Checklist'!$A$5:$A$171)</f>
+        <f>COUNTA('QA Checklist'!$A$5:$A$172)</f>
         <v/>
       </c>
     </row>
@@ -594,7 +594,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$171,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$171,"Pass")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$172,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$172,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$171,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$171,"Fail")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$172,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$172,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -616,7 +616,7 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$171,"Pending")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$172,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -671,19 +671,19 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$171,$A12)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$172,$A12)</f>
         <v/>
       </c>
       <c r="C12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$171,$A12,'QA Checklist'!$H$5:$H$171,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$171,$A12,'QA Checklist'!$H$5:$H$171,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$172,$A12,'QA Checklist'!$H$5:$H$172,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$172,$A12,'QA Checklist'!$H$5:$H$172,"Pass")</f>
         <v/>
       </c>
       <c r="D12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$171,$A12,'QA Checklist'!$H$5:$H$171,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$171,$A12,'QA Checklist'!$H$5:$H$171,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$172,$A12,'QA Checklist'!$H$5:$H$172,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$172,$A12,'QA Checklist'!$H$5:$H$172,"Fail")</f>
         <v/>
       </c>
       <c r="E12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$171,$A12,'QA Checklist'!$H$5:$H$171,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$172,$A12,'QA Checklist'!$H$5:$H$172,"Pending")</f>
         <v/>
       </c>
       <c r="F12" s="8">
@@ -698,19 +698,19 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$171,$A13)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$172,$A13)</f>
         <v/>
       </c>
       <c r="C13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$171,$A13,'QA Checklist'!$H$5:$H$171,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$171,$A13,'QA Checklist'!$H$5:$H$171,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$172,$A13,'QA Checklist'!$H$5:$H$172,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$172,$A13,'QA Checklist'!$H$5:$H$172,"Pass")</f>
         <v/>
       </c>
       <c r="D13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$171,$A13,'QA Checklist'!$H$5:$H$171,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$171,$A13,'QA Checklist'!$H$5:$H$171,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$172,$A13,'QA Checklist'!$H$5:$H$172,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$172,$A13,'QA Checklist'!$H$5:$H$172,"Fail")</f>
         <v/>
       </c>
       <c r="E13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$171,$A13,'QA Checklist'!$H$5:$H$171,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$172,$A13,'QA Checklist'!$H$5:$H$172,"Pending")</f>
         <v/>
       </c>
       <c r="F13" s="8">
@@ -725,19 +725,19 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$171,$A14)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$172,$A14)</f>
         <v/>
       </c>
       <c r="C14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$171,$A14,'QA Checklist'!$H$5:$H$171,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$171,$A14,'QA Checklist'!$H$5:$H$171,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$172,$A14,'QA Checklist'!$H$5:$H$172,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$172,$A14,'QA Checklist'!$H$5:$H$172,"Pass")</f>
         <v/>
       </c>
       <c r="D14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$171,$A14,'QA Checklist'!$H$5:$H$171,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$171,$A14,'QA Checklist'!$H$5:$H$171,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$172,$A14,'QA Checklist'!$H$5:$H$172,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$172,$A14,'QA Checklist'!$H$5:$H$172,"Fail")</f>
         <v/>
       </c>
       <c r="E14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$171,$A14,'QA Checklist'!$H$5:$H$171,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$172,$A14,'QA Checklist'!$H$5:$H$172,"Pending")</f>
         <v/>
       </c>
       <c r="F14" s="8">
@@ -752,19 +752,19 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$171,$A15)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$172,$A15)</f>
         <v/>
       </c>
       <c r="C15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$171,$A15,'QA Checklist'!$H$5:$H$171,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$171,$A15,'QA Checklist'!$H$5:$H$171,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$172,$A15,'QA Checklist'!$H$5:$H$172,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$172,$A15,'QA Checklist'!$H$5:$H$172,"Pass")</f>
         <v/>
       </c>
       <c r="D15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$171,$A15,'QA Checklist'!$H$5:$H$171,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$171,$A15,'QA Checklist'!$H$5:$H$171,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$172,$A15,'QA Checklist'!$H$5:$H$172,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$172,$A15,'QA Checklist'!$H$5:$H$172,"Fail")</f>
         <v/>
       </c>
       <c r="E15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$171,$A15,'QA Checklist'!$H$5:$H$171,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$172,$A15,'QA Checklist'!$H$5:$H$172,"Pending")</f>
         <v/>
       </c>
       <c r="F15" s="8">
@@ -779,19 +779,19 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$171,$A16)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$172,$A16)</f>
         <v/>
       </c>
       <c r="C16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$171,$A16,'QA Checklist'!$H$5:$H$171,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$171,$A16,'QA Checklist'!$H$5:$H$171,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$172,$A16,'QA Checklist'!$H$5:$H$172,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$172,$A16,'QA Checklist'!$H$5:$H$172,"Pass")</f>
         <v/>
       </c>
       <c r="D16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$171,$A16,'QA Checklist'!$H$5:$H$171,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$171,$A16,'QA Checklist'!$H$5:$H$171,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$172,$A16,'QA Checklist'!$H$5:$H$172,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$172,$A16,'QA Checklist'!$H$5:$H$172,"Fail")</f>
         <v/>
       </c>
       <c r="E16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$171,$A16,'QA Checklist'!$H$5:$H$171,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$172,$A16,'QA Checklist'!$H$5:$H$172,"Pending")</f>
         <v/>
       </c>
       <c r="F16" s="8">
@@ -806,19 +806,19 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$171,$A17)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$172,$A17)</f>
         <v/>
       </c>
       <c r="C17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$171,$A17,'QA Checklist'!$H$5:$H$171,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$171,$A17,'QA Checklist'!$H$5:$H$171,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$172,$A17,'QA Checklist'!$H$5:$H$172,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$172,$A17,'QA Checklist'!$H$5:$H$172,"Pass")</f>
         <v/>
       </c>
       <c r="D17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$171,$A17,'QA Checklist'!$H$5:$H$171,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$171,$A17,'QA Checklist'!$H$5:$H$171,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$172,$A17,'QA Checklist'!$H$5:$H$172,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$172,$A17,'QA Checklist'!$H$5:$H$172,"Fail")</f>
         <v/>
       </c>
       <c r="E17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$171,$A17,'QA Checklist'!$H$5:$H$171,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$172,$A17,'QA Checklist'!$H$5:$H$172,"Pending")</f>
         <v/>
       </c>
       <c r="F17" s="8">
@@ -833,19 +833,19 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$171,$A18)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$172,$A18)</f>
         <v/>
       </c>
       <c r="C18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$171,$A18,'QA Checklist'!$H$5:$H$171,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$171,$A18,'QA Checklist'!$H$5:$H$171,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$172,$A18,'QA Checklist'!$H$5:$H$172,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$172,$A18,'QA Checklist'!$H$5:$H$172,"Pass")</f>
         <v/>
       </c>
       <c r="D18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$171,$A18,'QA Checklist'!$H$5:$H$171,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$171,$A18,'QA Checklist'!$H$5:$H$171,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$172,$A18,'QA Checklist'!$H$5:$H$172,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$172,$A18,'QA Checklist'!$H$5:$H$172,"Fail")</f>
         <v/>
       </c>
       <c r="E18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$171,$A18,'QA Checklist'!$H$5:$H$171,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$172,$A18,'QA Checklist'!$H$5:$H$172,"Pending")</f>
         <v/>
       </c>
       <c r="F18" s="8">
@@ -860,19 +860,19 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$171,$A19)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$172,$A19)</f>
         <v/>
       </c>
       <c r="C19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$171,$A19,'QA Checklist'!$H$5:$H$171,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$171,$A19,'QA Checklist'!$H$5:$H$171,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$172,$A19,'QA Checklist'!$H$5:$H$172,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$172,$A19,'QA Checklist'!$H$5:$H$172,"Pass")</f>
         <v/>
       </c>
       <c r="D19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$171,$A19,'QA Checklist'!$H$5:$H$171,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$171,$A19,'QA Checklist'!$H$5:$H$171,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$172,$A19,'QA Checklist'!$H$5:$H$172,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$172,$A19,'QA Checklist'!$H$5:$H$172,"Fail")</f>
         <v/>
       </c>
       <c r="E19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$171,$A19,'QA Checklist'!$H$5:$H$171,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$172,$A19,'QA Checklist'!$H$5:$H$172,"Pending")</f>
         <v/>
       </c>
       <c r="F19" s="8">
@@ -887,19 +887,19 @@
         </is>
       </c>
       <c r="B20" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$171,$A20)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$172,$A20)</f>
         <v/>
       </c>
       <c r="C20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$171,$A20,'QA Checklist'!$H$5:$H$171,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$171,$A20,'QA Checklist'!$H$5:$H$171,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$172,$A20,'QA Checklist'!$H$5:$H$172,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$172,$A20,'QA Checklist'!$H$5:$H$172,"Pass")</f>
         <v/>
       </c>
       <c r="D20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$171,$A20,'QA Checklist'!$H$5:$H$171,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$171,$A20,'QA Checklist'!$H$5:$H$171,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$172,$A20,'QA Checklist'!$H$5:$H$172,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$172,$A20,'QA Checklist'!$H$5:$H$172,"Fail")</f>
         <v/>
       </c>
       <c r="E20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$171,$A20,'QA Checklist'!$H$5:$H$171,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$172,$A20,'QA Checklist'!$H$5:$H$172,"Pending")</f>
         <v/>
       </c>
       <c r="F20" s="8">
@@ -914,19 +914,19 @@
         </is>
       </c>
       <c r="B21" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$171,$A21)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$172,$A21)</f>
         <v/>
       </c>
       <c r="C21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$171,$A21,'QA Checklist'!$H$5:$H$171,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$171,$A21,'QA Checklist'!$H$5:$H$171,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$172,$A21,'QA Checklist'!$H$5:$H$172,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$172,$A21,'QA Checklist'!$H$5:$H$172,"Pass")</f>
         <v/>
       </c>
       <c r="D21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$171,$A21,'QA Checklist'!$H$5:$H$171,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$171,$A21,'QA Checklist'!$H$5:$H$171,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$172,$A21,'QA Checklist'!$H$5:$H$172,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$172,$A21,'QA Checklist'!$H$5:$H$172,"Fail")</f>
         <v/>
       </c>
       <c r="E21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$171,$A21,'QA Checklist'!$H$5:$H$171,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$172,$A21,'QA Checklist'!$H$5:$H$172,"Pending")</f>
         <v/>
       </c>
       <c r="F21" s="8">
@@ -941,19 +941,19 @@
         </is>
       </c>
       <c r="B22" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$171,$A22)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$172,$A22)</f>
         <v/>
       </c>
       <c r="C22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$171,$A22,'QA Checklist'!$H$5:$H$171,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$171,$A22,'QA Checklist'!$H$5:$H$171,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$172,$A22,'QA Checklist'!$H$5:$H$172,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$172,$A22,'QA Checklist'!$H$5:$H$172,"Pass")</f>
         <v/>
       </c>
       <c r="D22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$171,$A22,'QA Checklist'!$H$5:$H$171,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$171,$A22,'QA Checklist'!$H$5:$H$171,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$172,$A22,'QA Checklist'!$H$5:$H$172,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$172,$A22,'QA Checklist'!$H$5:$H$172,"Fail")</f>
         <v/>
       </c>
       <c r="E22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$171,$A22,'QA Checklist'!$H$5:$H$171,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$172,$A22,'QA Checklist'!$H$5:$H$172,"Pending")</f>
         <v/>
       </c>
       <c r="F22" s="8">
@@ -1023,19 +1023,19 @@
         </is>
       </c>
       <c r="B26" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$171,$A26&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$172,$A26&amp;"*")</f>
         <v/>
       </c>
       <c r="C26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$171,$A26&amp;"*",'QA Checklist'!$H$5:$H$171,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$171,$A26&amp;"*",'QA Checklist'!$H$5:$H$171,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$172,$A26&amp;"*",'QA Checklist'!$H$5:$H$172,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$172,$A26&amp;"*",'QA Checklist'!$H$5:$H$172,"Pass")</f>
         <v/>
       </c>
       <c r="D26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$171,$A26&amp;"*",'QA Checklist'!$H$5:$H$171,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$171,$A26&amp;"*",'QA Checklist'!$H$5:$H$171,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$172,$A26&amp;"*",'QA Checklist'!$H$5:$H$172,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$172,$A26&amp;"*",'QA Checklist'!$H$5:$H$172,"Fail")</f>
         <v/>
       </c>
       <c r="E26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$171,$A26&amp;"*",'QA Checklist'!$H$5:$H$171,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$172,$A26&amp;"*",'QA Checklist'!$H$5:$H$172,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1046,19 +1046,19 @@
         </is>
       </c>
       <c r="B27" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$171,$A27&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$172,$A27&amp;"*")</f>
         <v/>
       </c>
       <c r="C27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$171,$A27&amp;"*",'QA Checklist'!$H$5:$H$171,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$171,$A27&amp;"*",'QA Checklist'!$H$5:$H$171,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$172,$A27&amp;"*",'QA Checklist'!$H$5:$H$172,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$172,$A27&amp;"*",'QA Checklist'!$H$5:$H$172,"Pass")</f>
         <v/>
       </c>
       <c r="D27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$171,$A27&amp;"*",'QA Checklist'!$H$5:$H$171,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$171,$A27&amp;"*",'QA Checklist'!$H$5:$H$171,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$172,$A27&amp;"*",'QA Checklist'!$H$5:$H$172,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$172,$A27&amp;"*",'QA Checklist'!$H$5:$H$172,"Fail")</f>
         <v/>
       </c>
       <c r="E27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$171,$A27&amp;"*",'QA Checklist'!$H$5:$H$171,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$172,$A27&amp;"*",'QA Checklist'!$H$5:$H$172,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1069,19 +1069,19 @@
         </is>
       </c>
       <c r="B28" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$171,$A28&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$172,$A28&amp;"*")</f>
         <v/>
       </c>
       <c r="C28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$171,$A28&amp;"*",'QA Checklist'!$H$5:$H$171,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$171,$A28&amp;"*",'QA Checklist'!$H$5:$H$171,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$172,$A28&amp;"*",'QA Checklist'!$H$5:$H$172,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$172,$A28&amp;"*",'QA Checklist'!$H$5:$H$172,"Pass")</f>
         <v/>
       </c>
       <c r="D28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$171,$A28&amp;"*",'QA Checklist'!$H$5:$H$171,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$171,$A28&amp;"*",'QA Checklist'!$H$5:$H$171,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$172,$A28&amp;"*",'QA Checklist'!$H$5:$H$172,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$172,$A28&amp;"*",'QA Checklist'!$H$5:$H$172,"Fail")</f>
         <v/>
       </c>
       <c r="E28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$171,$A28&amp;"*",'QA Checklist'!$H$5:$H$171,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$172,$A28&amp;"*",'QA Checklist'!$H$5:$H$172,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1096,7 +1096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I171"/>
+  <dimension ref="A1:I172"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8576,12 +8576,59 @@
         </is>
       </c>
     </row>
+    <row r="172">
+      <c r="A172" s="12" t="inlineStr">
+        <is>
+          <t>SA-46</t>
+        </is>
+      </c>
+      <c r="B172" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="C172" s="13" t="inlineStr">
+        <is>
+          <t>Tier 2 (Workflow &amp; Ergonomics)</t>
+        </is>
+      </c>
+      <c r="D172" s="13" t="inlineStr">
+        <is>
+          <t>PDF and Excel Data Parity</t>
+        </is>
+      </c>
+      <c r="E172" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="F172" s="13" t="inlineStr">
+        <is>
+          <t>Log in as Service Advisor, open 2025 RO Excel Studio, fill Job Order (with a Claim Stub ID), Quotation and Billing (including a labor item, a part, a material and a discount) and the Checklist; edit a customer field only on the Billing tab; download each PDF and export .xlsx; open the workbook and compare every value and total with the PDFs and the on-screen totals</t>
+        </is>
+      </c>
+      <c r="G172" s="13" t="inlineStr">
+        <is>
+          <t>Every header value, line item and amount on each PDF appears identically in its Excel sheet: Billing lists the Billing items; LABOR / PARTS / MATERIALS columns match; VAT 12% is charged on labor only in the PDF, Excel and on screen; Billing TOTAL and 'amount of' subtract the discount everywhere; the Claim Stub shows the Claim Stub ID; values edited on the Quotation, Billing or Checklist tab appear on both that PDF and its sheet; the Job Order TOTAL shows Parts + Materials</t>
+        </is>
+      </c>
+      <c r="H172" s="14" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="I172" s="13" t="inlineStr">
+        <is>
+          <t>Verified by Automated Unit Tests (158/158 passing in tests/frontend/sla_and_logic.test.js AUT-FRONT-129) and an end-to-end PDF vs LibreOffice-recalculated workbook comparison of every item row and total</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:I171"/>
+  <autoFilter ref="A4:I172"/>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="H5:H171">
+  <conditionalFormatting sqref="H5:H172">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$H5="Passed"</formula>
     </cfRule>
@@ -8598,13 +8645,13 @@
       <formula>$H5="Pending"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A5:A171">
+  <conditionalFormatting sqref="A5:A172">
     <cfRule type="expression" priority="6" dxfId="3">
-      <formula>COUNTIF($A$5:$A$171,$A5)&gt;1</formula>
+      <formula>COUNTIF($A$5:$A$172,$A5)&gt;1</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H5:H171" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H5:H172" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pending,Passed,Failed"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat(REV-171): colored section header bands on all RO Excel Studio tabs
Workshop Monitoring & Daily Intakes and every other section title on the
Job_Order, Quotation_No, Billing_No and CheckList_Result tabs now sit on a
light blue band with a blue left accent. Button colors unchanged.
Cache buster v=3.24, AUT-FRONT-130, SA-47.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
+++ b/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
@@ -11,7 +11,7 @@
     <sheet name="QA Checklist" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$172</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$173</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'QA Checklist'!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTA('QA Checklist'!$A$5:$A$172)</f>
+        <f>COUNTA('QA Checklist'!$A$5:$A$173)</f>
         <v/>
       </c>
     </row>
@@ -594,7 +594,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$172,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$172,"Pass")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$173,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$173,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$172,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$172,"Fail")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$173,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$173,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -616,7 +616,7 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$172,"Pending")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$173,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -671,19 +671,19 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$172,$A12)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$173,$A12)</f>
         <v/>
       </c>
       <c r="C12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$172,$A12,'QA Checklist'!$H$5:$H$172,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$172,$A12,'QA Checklist'!$H$5:$H$172,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$173,$A12,'QA Checklist'!$H$5:$H$173,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$173,$A12,'QA Checklist'!$H$5:$H$173,"Pass")</f>
         <v/>
       </c>
       <c r="D12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$172,$A12,'QA Checklist'!$H$5:$H$172,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$172,$A12,'QA Checklist'!$H$5:$H$172,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$173,$A12,'QA Checklist'!$H$5:$H$173,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$173,$A12,'QA Checklist'!$H$5:$H$173,"Fail")</f>
         <v/>
       </c>
       <c r="E12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$172,$A12,'QA Checklist'!$H$5:$H$172,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$173,$A12,'QA Checklist'!$H$5:$H$173,"Pending")</f>
         <v/>
       </c>
       <c r="F12" s="8">
@@ -698,19 +698,19 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$172,$A13)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$173,$A13)</f>
         <v/>
       </c>
       <c r="C13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$172,$A13,'QA Checklist'!$H$5:$H$172,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$172,$A13,'QA Checklist'!$H$5:$H$172,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$173,$A13,'QA Checklist'!$H$5:$H$173,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$173,$A13,'QA Checklist'!$H$5:$H$173,"Pass")</f>
         <v/>
       </c>
       <c r="D13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$172,$A13,'QA Checklist'!$H$5:$H$172,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$172,$A13,'QA Checklist'!$H$5:$H$172,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$173,$A13,'QA Checklist'!$H$5:$H$173,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$173,$A13,'QA Checklist'!$H$5:$H$173,"Fail")</f>
         <v/>
       </c>
       <c r="E13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$172,$A13,'QA Checklist'!$H$5:$H$172,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$173,$A13,'QA Checklist'!$H$5:$H$173,"Pending")</f>
         <v/>
       </c>
       <c r="F13" s="8">
@@ -725,19 +725,19 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$172,$A14)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$173,$A14)</f>
         <v/>
       </c>
       <c r="C14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$172,$A14,'QA Checklist'!$H$5:$H$172,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$172,$A14,'QA Checklist'!$H$5:$H$172,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$173,$A14,'QA Checklist'!$H$5:$H$173,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$173,$A14,'QA Checklist'!$H$5:$H$173,"Pass")</f>
         <v/>
       </c>
       <c r="D14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$172,$A14,'QA Checklist'!$H$5:$H$172,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$172,$A14,'QA Checklist'!$H$5:$H$172,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$173,$A14,'QA Checklist'!$H$5:$H$173,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$173,$A14,'QA Checklist'!$H$5:$H$173,"Fail")</f>
         <v/>
       </c>
       <c r="E14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$172,$A14,'QA Checklist'!$H$5:$H$172,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$173,$A14,'QA Checklist'!$H$5:$H$173,"Pending")</f>
         <v/>
       </c>
       <c r="F14" s="8">
@@ -752,19 +752,19 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$172,$A15)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$173,$A15)</f>
         <v/>
       </c>
       <c r="C15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$172,$A15,'QA Checklist'!$H$5:$H$172,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$172,$A15,'QA Checklist'!$H$5:$H$172,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$173,$A15,'QA Checklist'!$H$5:$H$173,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$173,$A15,'QA Checklist'!$H$5:$H$173,"Pass")</f>
         <v/>
       </c>
       <c r="D15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$172,$A15,'QA Checklist'!$H$5:$H$172,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$172,$A15,'QA Checklist'!$H$5:$H$172,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$173,$A15,'QA Checklist'!$H$5:$H$173,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$173,$A15,'QA Checklist'!$H$5:$H$173,"Fail")</f>
         <v/>
       </c>
       <c r="E15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$172,$A15,'QA Checklist'!$H$5:$H$172,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$173,$A15,'QA Checklist'!$H$5:$H$173,"Pending")</f>
         <v/>
       </c>
       <c r="F15" s="8">
@@ -779,19 +779,19 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$172,$A16)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$173,$A16)</f>
         <v/>
       </c>
       <c r="C16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$172,$A16,'QA Checklist'!$H$5:$H$172,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$172,$A16,'QA Checklist'!$H$5:$H$172,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$173,$A16,'QA Checklist'!$H$5:$H$173,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$173,$A16,'QA Checklist'!$H$5:$H$173,"Pass")</f>
         <v/>
       </c>
       <c r="D16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$172,$A16,'QA Checklist'!$H$5:$H$172,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$172,$A16,'QA Checklist'!$H$5:$H$172,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$173,$A16,'QA Checklist'!$H$5:$H$173,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$173,$A16,'QA Checklist'!$H$5:$H$173,"Fail")</f>
         <v/>
       </c>
       <c r="E16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$172,$A16,'QA Checklist'!$H$5:$H$172,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$173,$A16,'QA Checklist'!$H$5:$H$173,"Pending")</f>
         <v/>
       </c>
       <c r="F16" s="8">
@@ -806,19 +806,19 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$172,$A17)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$173,$A17)</f>
         <v/>
       </c>
       <c r="C17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$172,$A17,'QA Checklist'!$H$5:$H$172,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$172,$A17,'QA Checklist'!$H$5:$H$172,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$173,$A17,'QA Checklist'!$H$5:$H$173,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$173,$A17,'QA Checklist'!$H$5:$H$173,"Pass")</f>
         <v/>
       </c>
       <c r="D17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$172,$A17,'QA Checklist'!$H$5:$H$172,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$172,$A17,'QA Checklist'!$H$5:$H$172,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$173,$A17,'QA Checklist'!$H$5:$H$173,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$173,$A17,'QA Checklist'!$H$5:$H$173,"Fail")</f>
         <v/>
       </c>
       <c r="E17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$172,$A17,'QA Checklist'!$H$5:$H$172,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$173,$A17,'QA Checklist'!$H$5:$H$173,"Pending")</f>
         <v/>
       </c>
       <c r="F17" s="8">
@@ -833,19 +833,19 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$172,$A18)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$173,$A18)</f>
         <v/>
       </c>
       <c r="C18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$172,$A18,'QA Checklist'!$H$5:$H$172,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$172,$A18,'QA Checklist'!$H$5:$H$172,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$173,$A18,'QA Checklist'!$H$5:$H$173,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$173,$A18,'QA Checklist'!$H$5:$H$173,"Pass")</f>
         <v/>
       </c>
       <c r="D18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$172,$A18,'QA Checklist'!$H$5:$H$172,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$172,$A18,'QA Checklist'!$H$5:$H$172,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$173,$A18,'QA Checklist'!$H$5:$H$173,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$173,$A18,'QA Checklist'!$H$5:$H$173,"Fail")</f>
         <v/>
       </c>
       <c r="E18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$172,$A18,'QA Checklist'!$H$5:$H$172,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$173,$A18,'QA Checklist'!$H$5:$H$173,"Pending")</f>
         <v/>
       </c>
       <c r="F18" s="8">
@@ -860,19 +860,19 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$172,$A19)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$173,$A19)</f>
         <v/>
       </c>
       <c r="C19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$172,$A19,'QA Checklist'!$H$5:$H$172,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$172,$A19,'QA Checklist'!$H$5:$H$172,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$173,$A19,'QA Checklist'!$H$5:$H$173,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$173,$A19,'QA Checklist'!$H$5:$H$173,"Pass")</f>
         <v/>
       </c>
       <c r="D19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$172,$A19,'QA Checklist'!$H$5:$H$172,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$172,$A19,'QA Checklist'!$H$5:$H$172,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$173,$A19,'QA Checklist'!$H$5:$H$173,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$173,$A19,'QA Checklist'!$H$5:$H$173,"Fail")</f>
         <v/>
       </c>
       <c r="E19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$172,$A19,'QA Checklist'!$H$5:$H$172,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$173,$A19,'QA Checklist'!$H$5:$H$173,"Pending")</f>
         <v/>
       </c>
       <c r="F19" s="8">
@@ -887,19 +887,19 @@
         </is>
       </c>
       <c r="B20" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$172,$A20)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$173,$A20)</f>
         <v/>
       </c>
       <c r="C20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$172,$A20,'QA Checklist'!$H$5:$H$172,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$172,$A20,'QA Checklist'!$H$5:$H$172,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$173,$A20,'QA Checklist'!$H$5:$H$173,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$173,$A20,'QA Checklist'!$H$5:$H$173,"Pass")</f>
         <v/>
       </c>
       <c r="D20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$172,$A20,'QA Checklist'!$H$5:$H$172,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$172,$A20,'QA Checklist'!$H$5:$H$172,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$173,$A20,'QA Checklist'!$H$5:$H$173,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$173,$A20,'QA Checklist'!$H$5:$H$173,"Fail")</f>
         <v/>
       </c>
       <c r="E20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$172,$A20,'QA Checklist'!$H$5:$H$172,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$173,$A20,'QA Checklist'!$H$5:$H$173,"Pending")</f>
         <v/>
       </c>
       <c r="F20" s="8">
@@ -914,19 +914,19 @@
         </is>
       </c>
       <c r="B21" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$172,$A21)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$173,$A21)</f>
         <v/>
       </c>
       <c r="C21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$172,$A21,'QA Checklist'!$H$5:$H$172,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$172,$A21,'QA Checklist'!$H$5:$H$172,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$173,$A21,'QA Checklist'!$H$5:$H$173,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$173,$A21,'QA Checklist'!$H$5:$H$173,"Pass")</f>
         <v/>
       </c>
       <c r="D21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$172,$A21,'QA Checklist'!$H$5:$H$172,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$172,$A21,'QA Checklist'!$H$5:$H$172,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$173,$A21,'QA Checklist'!$H$5:$H$173,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$173,$A21,'QA Checklist'!$H$5:$H$173,"Fail")</f>
         <v/>
       </c>
       <c r="E21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$172,$A21,'QA Checklist'!$H$5:$H$172,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$173,$A21,'QA Checklist'!$H$5:$H$173,"Pending")</f>
         <v/>
       </c>
       <c r="F21" s="8">
@@ -941,19 +941,19 @@
         </is>
       </c>
       <c r="B22" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$172,$A22)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$173,$A22)</f>
         <v/>
       </c>
       <c r="C22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$172,$A22,'QA Checklist'!$H$5:$H$172,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$172,$A22,'QA Checklist'!$H$5:$H$172,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$173,$A22,'QA Checklist'!$H$5:$H$173,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$173,$A22,'QA Checklist'!$H$5:$H$173,"Pass")</f>
         <v/>
       </c>
       <c r="D22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$172,$A22,'QA Checklist'!$H$5:$H$172,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$172,$A22,'QA Checklist'!$H$5:$H$172,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$173,$A22,'QA Checklist'!$H$5:$H$173,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$173,$A22,'QA Checklist'!$H$5:$H$173,"Fail")</f>
         <v/>
       </c>
       <c r="E22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$172,$A22,'QA Checklist'!$H$5:$H$172,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$173,$A22,'QA Checklist'!$H$5:$H$173,"Pending")</f>
         <v/>
       </c>
       <c r="F22" s="8">
@@ -1023,19 +1023,19 @@
         </is>
       </c>
       <c r="B26" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$172,$A26&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$173,$A26&amp;"*")</f>
         <v/>
       </c>
       <c r="C26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$172,$A26&amp;"*",'QA Checklist'!$H$5:$H$172,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$172,$A26&amp;"*",'QA Checklist'!$H$5:$H$172,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$173,$A26&amp;"*",'QA Checklist'!$H$5:$H$173,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$173,$A26&amp;"*",'QA Checklist'!$H$5:$H$173,"Pass")</f>
         <v/>
       </c>
       <c r="D26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$172,$A26&amp;"*",'QA Checklist'!$H$5:$H$172,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$172,$A26&amp;"*",'QA Checklist'!$H$5:$H$172,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$173,$A26&amp;"*",'QA Checklist'!$H$5:$H$173,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$173,$A26&amp;"*",'QA Checklist'!$H$5:$H$173,"Fail")</f>
         <v/>
       </c>
       <c r="E26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$172,$A26&amp;"*",'QA Checklist'!$H$5:$H$172,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$173,$A26&amp;"*",'QA Checklist'!$H$5:$H$173,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1046,19 +1046,19 @@
         </is>
       </c>
       <c r="B27" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$172,$A27&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$173,$A27&amp;"*")</f>
         <v/>
       </c>
       <c r="C27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$172,$A27&amp;"*",'QA Checklist'!$H$5:$H$172,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$172,$A27&amp;"*",'QA Checklist'!$H$5:$H$172,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$173,$A27&amp;"*",'QA Checklist'!$H$5:$H$173,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$173,$A27&amp;"*",'QA Checklist'!$H$5:$H$173,"Pass")</f>
         <v/>
       </c>
       <c r="D27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$172,$A27&amp;"*",'QA Checklist'!$H$5:$H$172,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$172,$A27&amp;"*",'QA Checklist'!$H$5:$H$172,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$173,$A27&amp;"*",'QA Checklist'!$H$5:$H$173,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$173,$A27&amp;"*",'QA Checklist'!$H$5:$H$173,"Fail")</f>
         <v/>
       </c>
       <c r="E27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$172,$A27&amp;"*",'QA Checklist'!$H$5:$H$172,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$173,$A27&amp;"*",'QA Checklist'!$H$5:$H$173,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1069,19 +1069,19 @@
         </is>
       </c>
       <c r="B28" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$172,$A28&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$173,$A28&amp;"*")</f>
         <v/>
       </c>
       <c r="C28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$172,$A28&amp;"*",'QA Checklist'!$H$5:$H$172,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$172,$A28&amp;"*",'QA Checklist'!$H$5:$H$172,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$173,$A28&amp;"*",'QA Checklist'!$H$5:$H$173,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$173,$A28&amp;"*",'QA Checklist'!$H$5:$H$173,"Pass")</f>
         <v/>
       </c>
       <c r="D28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$172,$A28&amp;"*",'QA Checklist'!$H$5:$H$172,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$172,$A28&amp;"*",'QA Checklist'!$H$5:$H$172,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$173,$A28&amp;"*",'QA Checklist'!$H$5:$H$173,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$173,$A28&amp;"*",'QA Checklist'!$H$5:$H$173,"Fail")</f>
         <v/>
       </c>
       <c r="E28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$172,$A28&amp;"*",'QA Checklist'!$H$5:$H$172,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$173,$A28&amp;"*",'QA Checklist'!$H$5:$H$173,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1096,7 +1096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I172"/>
+  <dimension ref="A1:I173"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8623,12 +8623,59 @@
         </is>
       </c>
     </row>
+    <row r="173">
+      <c r="A173" s="12" t="inlineStr">
+        <is>
+          <t>SA-47</t>
+        </is>
+      </c>
+      <c r="B173" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="C173" s="13" t="inlineStr">
+        <is>
+          <t>Tier 2 (Workflow &amp; Ergonomics)</t>
+        </is>
+      </c>
+      <c r="D173" s="13" t="inlineStr">
+        <is>
+          <t>RO Excel Studio Section Header Bands</t>
+        </is>
+      </c>
+      <c r="E173" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="F173" s="13" t="inlineStr">
+        <is>
+          <t>Log in as Service Advisor, open 2025 RO Excel Studio and view the Job_Order, Quotation_No, Billing_No and CheckList_Result tabs</t>
+        </is>
+      </c>
+      <c r="G173" s="13" t="inlineStr">
+        <is>
+          <t>Workshop Monitoring &amp; Daily Intakes and every other section title on all four tabs sits on a light blue band with a blue left accent; titles and subtitles are clearly readable; Save Draft, All Pass, Reset, Export and Register buttons keep their original colors</t>
+        </is>
+      </c>
+      <c r="H173" s="14" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="I173" s="13" t="inlineStr">
+        <is>
+          <t>Verified by Automated Unit Tests (159 passing in tests/frontend/sla_and_logic.test.js AUT-FRONT-130) and headless Chrome renders of all four tabs</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:I172"/>
+  <autoFilter ref="A4:I173"/>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="H5:H172">
+  <conditionalFormatting sqref="H5:H173">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$H5="Passed"</formula>
     </cfRule>
@@ -8645,13 +8692,13 @@
       <formula>$H5="Pending"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A5:A172">
+  <conditionalFormatting sqref="A5:A173">
     <cfRule type="expression" priority="6" dxfId="3">
-      <formula>COUNTIF($A$5:$A$172,$A5)&gt;1</formula>
+      <formula>COUNTIF($A$5:$A$173,$A5)&gt;1</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H5:H172" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H5:H173" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pending,Passed,Failed"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat(REV-172): neutral CheckList-style section header bands on all studio tabs
Replace the blue header bands with the CheckList checkpoint group band
(#D0D1D3 gray, black bold titles, dark gray subtitles and icons).
Cache buster v=3.25, AUT-FRONT-131, SA-48.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
+++ b/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
@@ -11,7 +11,7 @@
     <sheet name="QA Checklist" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$173</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$174</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'QA Checklist'!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTA('QA Checklist'!$A$5:$A$173)</f>
+        <f>COUNTA('QA Checklist'!$A$5:$A$174)</f>
         <v/>
       </c>
     </row>
@@ -594,7 +594,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$173,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$173,"Pass")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$174,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$174,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$173,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$173,"Fail")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$174,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$174,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -616,7 +616,7 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$173,"Pending")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$174,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -671,19 +671,19 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$173,$A12)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$174,$A12)</f>
         <v/>
       </c>
       <c r="C12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$173,$A12,'QA Checklist'!$H$5:$H$173,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$173,$A12,'QA Checklist'!$H$5:$H$173,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$174,$A12,'QA Checklist'!$H$5:$H$174,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$174,$A12,'QA Checklist'!$H$5:$H$174,"Pass")</f>
         <v/>
       </c>
       <c r="D12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$173,$A12,'QA Checklist'!$H$5:$H$173,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$173,$A12,'QA Checklist'!$H$5:$H$173,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$174,$A12,'QA Checklist'!$H$5:$H$174,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$174,$A12,'QA Checklist'!$H$5:$H$174,"Fail")</f>
         <v/>
       </c>
       <c r="E12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$173,$A12,'QA Checklist'!$H$5:$H$173,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$174,$A12,'QA Checklist'!$H$5:$H$174,"Pending")</f>
         <v/>
       </c>
       <c r="F12" s="8">
@@ -698,19 +698,19 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$173,$A13)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$174,$A13)</f>
         <v/>
       </c>
       <c r="C13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$173,$A13,'QA Checklist'!$H$5:$H$173,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$173,$A13,'QA Checklist'!$H$5:$H$173,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$174,$A13,'QA Checklist'!$H$5:$H$174,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$174,$A13,'QA Checklist'!$H$5:$H$174,"Pass")</f>
         <v/>
       </c>
       <c r="D13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$173,$A13,'QA Checklist'!$H$5:$H$173,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$173,$A13,'QA Checklist'!$H$5:$H$173,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$174,$A13,'QA Checklist'!$H$5:$H$174,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$174,$A13,'QA Checklist'!$H$5:$H$174,"Fail")</f>
         <v/>
       </c>
       <c r="E13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$173,$A13,'QA Checklist'!$H$5:$H$173,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$174,$A13,'QA Checklist'!$H$5:$H$174,"Pending")</f>
         <v/>
       </c>
       <c r="F13" s="8">
@@ -725,19 +725,19 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$173,$A14)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$174,$A14)</f>
         <v/>
       </c>
       <c r="C14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$173,$A14,'QA Checklist'!$H$5:$H$173,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$173,$A14,'QA Checklist'!$H$5:$H$173,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$174,$A14,'QA Checklist'!$H$5:$H$174,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$174,$A14,'QA Checklist'!$H$5:$H$174,"Pass")</f>
         <v/>
       </c>
       <c r="D14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$173,$A14,'QA Checklist'!$H$5:$H$173,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$173,$A14,'QA Checklist'!$H$5:$H$173,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$174,$A14,'QA Checklist'!$H$5:$H$174,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$174,$A14,'QA Checklist'!$H$5:$H$174,"Fail")</f>
         <v/>
       </c>
       <c r="E14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$173,$A14,'QA Checklist'!$H$5:$H$173,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$174,$A14,'QA Checklist'!$H$5:$H$174,"Pending")</f>
         <v/>
       </c>
       <c r="F14" s="8">
@@ -752,19 +752,19 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$173,$A15)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$174,$A15)</f>
         <v/>
       </c>
       <c r="C15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$173,$A15,'QA Checklist'!$H$5:$H$173,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$173,$A15,'QA Checklist'!$H$5:$H$173,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$174,$A15,'QA Checklist'!$H$5:$H$174,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$174,$A15,'QA Checklist'!$H$5:$H$174,"Pass")</f>
         <v/>
       </c>
       <c r="D15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$173,$A15,'QA Checklist'!$H$5:$H$173,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$173,$A15,'QA Checklist'!$H$5:$H$173,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$174,$A15,'QA Checklist'!$H$5:$H$174,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$174,$A15,'QA Checklist'!$H$5:$H$174,"Fail")</f>
         <v/>
       </c>
       <c r="E15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$173,$A15,'QA Checklist'!$H$5:$H$173,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$174,$A15,'QA Checklist'!$H$5:$H$174,"Pending")</f>
         <v/>
       </c>
       <c r="F15" s="8">
@@ -779,19 +779,19 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$173,$A16)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$174,$A16)</f>
         <v/>
       </c>
       <c r="C16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$173,$A16,'QA Checklist'!$H$5:$H$173,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$173,$A16,'QA Checklist'!$H$5:$H$173,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$174,$A16,'QA Checklist'!$H$5:$H$174,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$174,$A16,'QA Checklist'!$H$5:$H$174,"Pass")</f>
         <v/>
       </c>
       <c r="D16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$173,$A16,'QA Checklist'!$H$5:$H$173,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$173,$A16,'QA Checklist'!$H$5:$H$173,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$174,$A16,'QA Checklist'!$H$5:$H$174,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$174,$A16,'QA Checklist'!$H$5:$H$174,"Fail")</f>
         <v/>
       </c>
       <c r="E16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$173,$A16,'QA Checklist'!$H$5:$H$173,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$174,$A16,'QA Checklist'!$H$5:$H$174,"Pending")</f>
         <v/>
       </c>
       <c r="F16" s="8">
@@ -806,19 +806,19 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$173,$A17)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$174,$A17)</f>
         <v/>
       </c>
       <c r="C17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$173,$A17,'QA Checklist'!$H$5:$H$173,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$173,$A17,'QA Checklist'!$H$5:$H$173,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$174,$A17,'QA Checklist'!$H$5:$H$174,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$174,$A17,'QA Checklist'!$H$5:$H$174,"Pass")</f>
         <v/>
       </c>
       <c r="D17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$173,$A17,'QA Checklist'!$H$5:$H$173,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$173,$A17,'QA Checklist'!$H$5:$H$173,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$174,$A17,'QA Checklist'!$H$5:$H$174,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$174,$A17,'QA Checklist'!$H$5:$H$174,"Fail")</f>
         <v/>
       </c>
       <c r="E17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$173,$A17,'QA Checklist'!$H$5:$H$173,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$174,$A17,'QA Checklist'!$H$5:$H$174,"Pending")</f>
         <v/>
       </c>
       <c r="F17" s="8">
@@ -833,19 +833,19 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$173,$A18)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$174,$A18)</f>
         <v/>
       </c>
       <c r="C18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$173,$A18,'QA Checklist'!$H$5:$H$173,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$173,$A18,'QA Checklist'!$H$5:$H$173,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$174,$A18,'QA Checklist'!$H$5:$H$174,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$174,$A18,'QA Checklist'!$H$5:$H$174,"Pass")</f>
         <v/>
       </c>
       <c r="D18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$173,$A18,'QA Checklist'!$H$5:$H$173,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$173,$A18,'QA Checklist'!$H$5:$H$173,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$174,$A18,'QA Checklist'!$H$5:$H$174,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$174,$A18,'QA Checklist'!$H$5:$H$174,"Fail")</f>
         <v/>
       </c>
       <c r="E18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$173,$A18,'QA Checklist'!$H$5:$H$173,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$174,$A18,'QA Checklist'!$H$5:$H$174,"Pending")</f>
         <v/>
       </c>
       <c r="F18" s="8">
@@ -860,19 +860,19 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$173,$A19)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$174,$A19)</f>
         <v/>
       </c>
       <c r="C19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$173,$A19,'QA Checklist'!$H$5:$H$173,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$173,$A19,'QA Checklist'!$H$5:$H$173,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$174,$A19,'QA Checklist'!$H$5:$H$174,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$174,$A19,'QA Checklist'!$H$5:$H$174,"Pass")</f>
         <v/>
       </c>
       <c r="D19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$173,$A19,'QA Checklist'!$H$5:$H$173,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$173,$A19,'QA Checklist'!$H$5:$H$173,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$174,$A19,'QA Checklist'!$H$5:$H$174,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$174,$A19,'QA Checklist'!$H$5:$H$174,"Fail")</f>
         <v/>
       </c>
       <c r="E19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$173,$A19,'QA Checklist'!$H$5:$H$173,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$174,$A19,'QA Checklist'!$H$5:$H$174,"Pending")</f>
         <v/>
       </c>
       <c r="F19" s="8">
@@ -887,19 +887,19 @@
         </is>
       </c>
       <c r="B20" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$173,$A20)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$174,$A20)</f>
         <v/>
       </c>
       <c r="C20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$173,$A20,'QA Checklist'!$H$5:$H$173,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$173,$A20,'QA Checklist'!$H$5:$H$173,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$174,$A20,'QA Checklist'!$H$5:$H$174,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$174,$A20,'QA Checklist'!$H$5:$H$174,"Pass")</f>
         <v/>
       </c>
       <c r="D20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$173,$A20,'QA Checklist'!$H$5:$H$173,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$173,$A20,'QA Checklist'!$H$5:$H$173,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$174,$A20,'QA Checklist'!$H$5:$H$174,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$174,$A20,'QA Checklist'!$H$5:$H$174,"Fail")</f>
         <v/>
       </c>
       <c r="E20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$173,$A20,'QA Checklist'!$H$5:$H$173,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$174,$A20,'QA Checklist'!$H$5:$H$174,"Pending")</f>
         <v/>
       </c>
       <c r="F20" s="8">
@@ -914,19 +914,19 @@
         </is>
       </c>
       <c r="B21" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$173,$A21)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$174,$A21)</f>
         <v/>
       </c>
       <c r="C21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$173,$A21,'QA Checklist'!$H$5:$H$173,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$173,$A21,'QA Checklist'!$H$5:$H$173,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$174,$A21,'QA Checklist'!$H$5:$H$174,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$174,$A21,'QA Checklist'!$H$5:$H$174,"Pass")</f>
         <v/>
       </c>
       <c r="D21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$173,$A21,'QA Checklist'!$H$5:$H$173,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$173,$A21,'QA Checklist'!$H$5:$H$173,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$174,$A21,'QA Checklist'!$H$5:$H$174,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$174,$A21,'QA Checklist'!$H$5:$H$174,"Fail")</f>
         <v/>
       </c>
       <c r="E21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$173,$A21,'QA Checklist'!$H$5:$H$173,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$174,$A21,'QA Checklist'!$H$5:$H$174,"Pending")</f>
         <v/>
       </c>
       <c r="F21" s="8">
@@ -941,19 +941,19 @@
         </is>
       </c>
       <c r="B22" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$173,$A22)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$174,$A22)</f>
         <v/>
       </c>
       <c r="C22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$173,$A22,'QA Checklist'!$H$5:$H$173,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$173,$A22,'QA Checklist'!$H$5:$H$173,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$174,$A22,'QA Checklist'!$H$5:$H$174,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$174,$A22,'QA Checklist'!$H$5:$H$174,"Pass")</f>
         <v/>
       </c>
       <c r="D22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$173,$A22,'QA Checklist'!$H$5:$H$173,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$173,$A22,'QA Checklist'!$H$5:$H$173,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$174,$A22,'QA Checklist'!$H$5:$H$174,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$174,$A22,'QA Checklist'!$H$5:$H$174,"Fail")</f>
         <v/>
       </c>
       <c r="E22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$173,$A22,'QA Checklist'!$H$5:$H$173,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$174,$A22,'QA Checklist'!$H$5:$H$174,"Pending")</f>
         <v/>
       </c>
       <c r="F22" s="8">
@@ -1023,19 +1023,19 @@
         </is>
       </c>
       <c r="B26" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$173,$A26&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$174,$A26&amp;"*")</f>
         <v/>
       </c>
       <c r="C26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$173,$A26&amp;"*",'QA Checklist'!$H$5:$H$173,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$173,$A26&amp;"*",'QA Checklist'!$H$5:$H$173,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$174,$A26&amp;"*",'QA Checklist'!$H$5:$H$174,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$174,$A26&amp;"*",'QA Checklist'!$H$5:$H$174,"Pass")</f>
         <v/>
       </c>
       <c r="D26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$173,$A26&amp;"*",'QA Checklist'!$H$5:$H$173,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$173,$A26&amp;"*",'QA Checklist'!$H$5:$H$173,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$174,$A26&amp;"*",'QA Checklist'!$H$5:$H$174,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$174,$A26&amp;"*",'QA Checklist'!$H$5:$H$174,"Fail")</f>
         <v/>
       </c>
       <c r="E26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$173,$A26&amp;"*",'QA Checklist'!$H$5:$H$173,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$174,$A26&amp;"*",'QA Checklist'!$H$5:$H$174,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1046,19 +1046,19 @@
         </is>
       </c>
       <c r="B27" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$173,$A27&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$174,$A27&amp;"*")</f>
         <v/>
       </c>
       <c r="C27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$173,$A27&amp;"*",'QA Checklist'!$H$5:$H$173,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$173,$A27&amp;"*",'QA Checklist'!$H$5:$H$173,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$174,$A27&amp;"*",'QA Checklist'!$H$5:$H$174,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$174,$A27&amp;"*",'QA Checklist'!$H$5:$H$174,"Pass")</f>
         <v/>
       </c>
       <c r="D27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$173,$A27&amp;"*",'QA Checklist'!$H$5:$H$173,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$173,$A27&amp;"*",'QA Checklist'!$H$5:$H$173,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$174,$A27&amp;"*",'QA Checklist'!$H$5:$H$174,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$174,$A27&amp;"*",'QA Checklist'!$H$5:$H$174,"Fail")</f>
         <v/>
       </c>
       <c r="E27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$173,$A27&amp;"*",'QA Checklist'!$H$5:$H$173,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$174,$A27&amp;"*",'QA Checklist'!$H$5:$H$174,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1069,19 +1069,19 @@
         </is>
       </c>
       <c r="B28" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$173,$A28&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$174,$A28&amp;"*")</f>
         <v/>
       </c>
       <c r="C28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$173,$A28&amp;"*",'QA Checklist'!$H$5:$H$173,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$173,$A28&amp;"*",'QA Checklist'!$H$5:$H$173,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$174,$A28&amp;"*",'QA Checklist'!$H$5:$H$174,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$174,$A28&amp;"*",'QA Checklist'!$H$5:$H$174,"Pass")</f>
         <v/>
       </c>
       <c r="D28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$173,$A28&amp;"*",'QA Checklist'!$H$5:$H$173,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$173,$A28&amp;"*",'QA Checklist'!$H$5:$H$173,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$174,$A28&amp;"*",'QA Checklist'!$H$5:$H$174,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$174,$A28&amp;"*",'QA Checklist'!$H$5:$H$174,"Fail")</f>
         <v/>
       </c>
       <c r="E28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$173,$A28&amp;"*",'QA Checklist'!$H$5:$H$173,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$174,$A28&amp;"*",'QA Checklist'!$H$5:$H$174,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1096,7 +1096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I173"/>
+  <dimension ref="A1:I174"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8670,12 +8670,59 @@
         </is>
       </c>
     </row>
+    <row r="174">
+      <c r="A174" s="12" t="inlineStr">
+        <is>
+          <t>SA-48</t>
+        </is>
+      </c>
+      <c r="B174" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="C174" s="13" t="inlineStr">
+        <is>
+          <t>Tier 2 (Workflow &amp; Ergonomics)</t>
+        </is>
+      </c>
+      <c r="D174" s="13" t="inlineStr">
+        <is>
+          <t>Neutral Studio Section Header Bands</t>
+        </is>
+      </c>
+      <c r="E174" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="F174" s="13" t="inlineStr">
+        <is>
+          <t>Log in as Service Advisor, open 2025 RO Excel Studio and view the Job_Order, Quotation_No, Billing_No and CheckList_Result tabs</t>
+        </is>
+      </c>
+      <c r="G174" s="13" t="inlineStr">
+        <is>
+          <t>Every section title (including Workshop Monitoring &amp; Daily Intakes) sits on the same light gray band as the CheckList checkpoint groups, with black titles; no blue bands or accents remain; button colors are unchanged</t>
+        </is>
+      </c>
+      <c r="H174" s="14" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="I174" s="13" t="inlineStr">
+        <is>
+          <t>Verified by Automated Unit Tests (160 passing in tests/frontend/sla_and_logic.test.js AUT-FRONT-131) and headless Chrome renders of all four tabs</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:I173"/>
+  <autoFilter ref="A4:I174"/>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="H5:H173">
+  <conditionalFormatting sqref="H5:H174">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$H5="Passed"</formula>
     </cfRule>
@@ -8692,13 +8739,13 @@
       <formula>$H5="Pending"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A5:A173">
+  <conditionalFormatting sqref="A5:A174">
     <cfRule type="expression" priority="6" dxfId="3">
-      <formula>COUNTIF($A$5:$A$173,$A5)&gt;1</formula>
+      <formula>COUNTIF($A$5:$A$174,$A5)&gt;1</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H5:H173" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H5:H174" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pending,Passed,Failed"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat(REV-173): Workshop_Monitoring studio tab for Daily Intakes entry
Add a fifth RO Excel Studio tab after CheckList_Result. The Workshop
Monitoring & Daily Intakes card moves there from Job_Order (field ids
unchanged) next to a live Daily Intakes entry preview.
Cache buster v=3.26, AUT-FRONT-132, SA-49.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
+++ b/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
@@ -11,7 +11,7 @@
     <sheet name="QA Checklist" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$174</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$175</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'QA Checklist'!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTA('QA Checklist'!$A$5:$A$174)</f>
+        <f>COUNTA('QA Checklist'!$A$5:$A$175)</f>
         <v/>
       </c>
     </row>
@@ -594,7 +594,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$174,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$174,"Pass")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$175,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$175,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$174,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$174,"Fail")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$175,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$175,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -616,7 +616,7 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$174,"Pending")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$175,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -671,19 +671,19 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$174,$A12)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$175,$A12)</f>
         <v/>
       </c>
       <c r="C12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$174,$A12,'QA Checklist'!$H$5:$H$174,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$174,$A12,'QA Checklist'!$H$5:$H$174,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$175,$A12,'QA Checklist'!$H$5:$H$175,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$175,$A12,'QA Checklist'!$H$5:$H$175,"Pass")</f>
         <v/>
       </c>
       <c r="D12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$174,$A12,'QA Checklist'!$H$5:$H$174,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$174,$A12,'QA Checklist'!$H$5:$H$174,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$175,$A12,'QA Checklist'!$H$5:$H$175,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$175,$A12,'QA Checklist'!$H$5:$H$175,"Fail")</f>
         <v/>
       </c>
       <c r="E12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$174,$A12,'QA Checklist'!$H$5:$H$174,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$175,$A12,'QA Checklist'!$H$5:$H$175,"Pending")</f>
         <v/>
       </c>
       <c r="F12" s="8">
@@ -698,19 +698,19 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$174,$A13)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$175,$A13)</f>
         <v/>
       </c>
       <c r="C13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$174,$A13,'QA Checklist'!$H$5:$H$174,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$174,$A13,'QA Checklist'!$H$5:$H$174,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$175,$A13,'QA Checklist'!$H$5:$H$175,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$175,$A13,'QA Checklist'!$H$5:$H$175,"Pass")</f>
         <v/>
       </c>
       <c r="D13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$174,$A13,'QA Checklist'!$H$5:$H$174,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$174,$A13,'QA Checklist'!$H$5:$H$174,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$175,$A13,'QA Checklist'!$H$5:$H$175,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$175,$A13,'QA Checklist'!$H$5:$H$175,"Fail")</f>
         <v/>
       </c>
       <c r="E13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$174,$A13,'QA Checklist'!$H$5:$H$174,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$175,$A13,'QA Checklist'!$H$5:$H$175,"Pending")</f>
         <v/>
       </c>
       <c r="F13" s="8">
@@ -725,19 +725,19 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$174,$A14)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$175,$A14)</f>
         <v/>
       </c>
       <c r="C14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$174,$A14,'QA Checklist'!$H$5:$H$174,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$174,$A14,'QA Checklist'!$H$5:$H$174,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$175,$A14,'QA Checklist'!$H$5:$H$175,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$175,$A14,'QA Checklist'!$H$5:$H$175,"Pass")</f>
         <v/>
       </c>
       <c r="D14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$174,$A14,'QA Checklist'!$H$5:$H$174,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$174,$A14,'QA Checklist'!$H$5:$H$174,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$175,$A14,'QA Checklist'!$H$5:$H$175,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$175,$A14,'QA Checklist'!$H$5:$H$175,"Fail")</f>
         <v/>
       </c>
       <c r="E14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$174,$A14,'QA Checklist'!$H$5:$H$174,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$175,$A14,'QA Checklist'!$H$5:$H$175,"Pending")</f>
         <v/>
       </c>
       <c r="F14" s="8">
@@ -752,19 +752,19 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$174,$A15)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$175,$A15)</f>
         <v/>
       </c>
       <c r="C15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$174,$A15,'QA Checklist'!$H$5:$H$174,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$174,$A15,'QA Checklist'!$H$5:$H$174,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$175,$A15,'QA Checklist'!$H$5:$H$175,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$175,$A15,'QA Checklist'!$H$5:$H$175,"Pass")</f>
         <v/>
       </c>
       <c r="D15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$174,$A15,'QA Checklist'!$H$5:$H$174,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$174,$A15,'QA Checklist'!$H$5:$H$174,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$175,$A15,'QA Checklist'!$H$5:$H$175,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$175,$A15,'QA Checklist'!$H$5:$H$175,"Fail")</f>
         <v/>
       </c>
       <c r="E15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$174,$A15,'QA Checklist'!$H$5:$H$174,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$175,$A15,'QA Checklist'!$H$5:$H$175,"Pending")</f>
         <v/>
       </c>
       <c r="F15" s="8">
@@ -779,19 +779,19 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$174,$A16)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$175,$A16)</f>
         <v/>
       </c>
       <c r="C16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$174,$A16,'QA Checklist'!$H$5:$H$174,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$174,$A16,'QA Checklist'!$H$5:$H$174,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$175,$A16,'QA Checklist'!$H$5:$H$175,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$175,$A16,'QA Checklist'!$H$5:$H$175,"Pass")</f>
         <v/>
       </c>
       <c r="D16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$174,$A16,'QA Checklist'!$H$5:$H$174,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$174,$A16,'QA Checklist'!$H$5:$H$174,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$175,$A16,'QA Checklist'!$H$5:$H$175,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$175,$A16,'QA Checklist'!$H$5:$H$175,"Fail")</f>
         <v/>
       </c>
       <c r="E16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$174,$A16,'QA Checklist'!$H$5:$H$174,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$175,$A16,'QA Checklist'!$H$5:$H$175,"Pending")</f>
         <v/>
       </c>
       <c r="F16" s="8">
@@ -806,19 +806,19 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$174,$A17)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$175,$A17)</f>
         <v/>
       </c>
       <c r="C17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$174,$A17,'QA Checklist'!$H$5:$H$174,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$174,$A17,'QA Checklist'!$H$5:$H$174,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$175,$A17,'QA Checklist'!$H$5:$H$175,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$175,$A17,'QA Checklist'!$H$5:$H$175,"Pass")</f>
         <v/>
       </c>
       <c r="D17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$174,$A17,'QA Checklist'!$H$5:$H$174,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$174,$A17,'QA Checklist'!$H$5:$H$174,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$175,$A17,'QA Checklist'!$H$5:$H$175,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$175,$A17,'QA Checklist'!$H$5:$H$175,"Fail")</f>
         <v/>
       </c>
       <c r="E17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$174,$A17,'QA Checklist'!$H$5:$H$174,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$175,$A17,'QA Checklist'!$H$5:$H$175,"Pending")</f>
         <v/>
       </c>
       <c r="F17" s="8">
@@ -833,19 +833,19 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$174,$A18)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$175,$A18)</f>
         <v/>
       </c>
       <c r="C18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$174,$A18,'QA Checklist'!$H$5:$H$174,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$174,$A18,'QA Checklist'!$H$5:$H$174,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$175,$A18,'QA Checklist'!$H$5:$H$175,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$175,$A18,'QA Checklist'!$H$5:$H$175,"Pass")</f>
         <v/>
       </c>
       <c r="D18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$174,$A18,'QA Checklist'!$H$5:$H$174,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$174,$A18,'QA Checklist'!$H$5:$H$174,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$175,$A18,'QA Checklist'!$H$5:$H$175,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$175,$A18,'QA Checklist'!$H$5:$H$175,"Fail")</f>
         <v/>
       </c>
       <c r="E18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$174,$A18,'QA Checklist'!$H$5:$H$174,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$175,$A18,'QA Checklist'!$H$5:$H$175,"Pending")</f>
         <v/>
       </c>
       <c r="F18" s="8">
@@ -860,19 +860,19 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$174,$A19)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$175,$A19)</f>
         <v/>
       </c>
       <c r="C19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$174,$A19,'QA Checklist'!$H$5:$H$174,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$174,$A19,'QA Checklist'!$H$5:$H$174,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$175,$A19,'QA Checklist'!$H$5:$H$175,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$175,$A19,'QA Checklist'!$H$5:$H$175,"Pass")</f>
         <v/>
       </c>
       <c r="D19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$174,$A19,'QA Checklist'!$H$5:$H$174,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$174,$A19,'QA Checklist'!$H$5:$H$174,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$175,$A19,'QA Checklist'!$H$5:$H$175,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$175,$A19,'QA Checklist'!$H$5:$H$175,"Fail")</f>
         <v/>
       </c>
       <c r="E19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$174,$A19,'QA Checklist'!$H$5:$H$174,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$175,$A19,'QA Checklist'!$H$5:$H$175,"Pending")</f>
         <v/>
       </c>
       <c r="F19" s="8">
@@ -887,19 +887,19 @@
         </is>
       </c>
       <c r="B20" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$174,$A20)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$175,$A20)</f>
         <v/>
       </c>
       <c r="C20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$174,$A20,'QA Checklist'!$H$5:$H$174,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$174,$A20,'QA Checklist'!$H$5:$H$174,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$175,$A20,'QA Checklist'!$H$5:$H$175,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$175,$A20,'QA Checklist'!$H$5:$H$175,"Pass")</f>
         <v/>
       </c>
       <c r="D20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$174,$A20,'QA Checklist'!$H$5:$H$174,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$174,$A20,'QA Checklist'!$H$5:$H$174,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$175,$A20,'QA Checklist'!$H$5:$H$175,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$175,$A20,'QA Checklist'!$H$5:$H$175,"Fail")</f>
         <v/>
       </c>
       <c r="E20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$174,$A20,'QA Checklist'!$H$5:$H$174,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$175,$A20,'QA Checklist'!$H$5:$H$175,"Pending")</f>
         <v/>
       </c>
       <c r="F20" s="8">
@@ -914,19 +914,19 @@
         </is>
       </c>
       <c r="B21" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$174,$A21)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$175,$A21)</f>
         <v/>
       </c>
       <c r="C21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$174,$A21,'QA Checklist'!$H$5:$H$174,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$174,$A21,'QA Checklist'!$H$5:$H$174,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$175,$A21,'QA Checklist'!$H$5:$H$175,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$175,$A21,'QA Checklist'!$H$5:$H$175,"Pass")</f>
         <v/>
       </c>
       <c r="D21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$174,$A21,'QA Checklist'!$H$5:$H$174,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$174,$A21,'QA Checklist'!$H$5:$H$174,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$175,$A21,'QA Checklist'!$H$5:$H$175,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$175,$A21,'QA Checklist'!$H$5:$H$175,"Fail")</f>
         <v/>
       </c>
       <c r="E21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$174,$A21,'QA Checklist'!$H$5:$H$174,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$175,$A21,'QA Checklist'!$H$5:$H$175,"Pending")</f>
         <v/>
       </c>
       <c r="F21" s="8">
@@ -941,19 +941,19 @@
         </is>
       </c>
       <c r="B22" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$174,$A22)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$175,$A22)</f>
         <v/>
       </c>
       <c r="C22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$174,$A22,'QA Checklist'!$H$5:$H$174,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$174,$A22,'QA Checklist'!$H$5:$H$174,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$175,$A22,'QA Checklist'!$H$5:$H$175,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$175,$A22,'QA Checklist'!$H$5:$H$175,"Pass")</f>
         <v/>
       </c>
       <c r="D22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$174,$A22,'QA Checklist'!$H$5:$H$174,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$174,$A22,'QA Checklist'!$H$5:$H$174,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$175,$A22,'QA Checklist'!$H$5:$H$175,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$175,$A22,'QA Checklist'!$H$5:$H$175,"Fail")</f>
         <v/>
       </c>
       <c r="E22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$174,$A22,'QA Checklist'!$H$5:$H$174,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$175,$A22,'QA Checklist'!$H$5:$H$175,"Pending")</f>
         <v/>
       </c>
       <c r="F22" s="8">
@@ -1023,19 +1023,19 @@
         </is>
       </c>
       <c r="B26" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$174,$A26&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$175,$A26&amp;"*")</f>
         <v/>
       </c>
       <c r="C26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$174,$A26&amp;"*",'QA Checklist'!$H$5:$H$174,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$174,$A26&amp;"*",'QA Checklist'!$H$5:$H$174,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$175,$A26&amp;"*",'QA Checklist'!$H$5:$H$175,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$175,$A26&amp;"*",'QA Checklist'!$H$5:$H$175,"Pass")</f>
         <v/>
       </c>
       <c r="D26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$174,$A26&amp;"*",'QA Checklist'!$H$5:$H$174,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$174,$A26&amp;"*",'QA Checklist'!$H$5:$H$174,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$175,$A26&amp;"*",'QA Checklist'!$H$5:$H$175,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$175,$A26&amp;"*",'QA Checklist'!$H$5:$H$175,"Fail")</f>
         <v/>
       </c>
       <c r="E26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$174,$A26&amp;"*",'QA Checklist'!$H$5:$H$174,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$175,$A26&amp;"*",'QA Checklist'!$H$5:$H$175,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1046,19 +1046,19 @@
         </is>
       </c>
       <c r="B27" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$174,$A27&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$175,$A27&amp;"*")</f>
         <v/>
       </c>
       <c r="C27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$174,$A27&amp;"*",'QA Checklist'!$H$5:$H$174,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$174,$A27&amp;"*",'QA Checklist'!$H$5:$H$174,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$175,$A27&amp;"*",'QA Checklist'!$H$5:$H$175,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$175,$A27&amp;"*",'QA Checklist'!$H$5:$H$175,"Pass")</f>
         <v/>
       </c>
       <c r="D27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$174,$A27&amp;"*",'QA Checklist'!$H$5:$H$174,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$174,$A27&amp;"*",'QA Checklist'!$H$5:$H$174,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$175,$A27&amp;"*",'QA Checklist'!$H$5:$H$175,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$175,$A27&amp;"*",'QA Checklist'!$H$5:$H$175,"Fail")</f>
         <v/>
       </c>
       <c r="E27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$174,$A27&amp;"*",'QA Checklist'!$H$5:$H$174,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$175,$A27&amp;"*",'QA Checklist'!$H$5:$H$175,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1069,19 +1069,19 @@
         </is>
       </c>
       <c r="B28" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$174,$A28&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$175,$A28&amp;"*")</f>
         <v/>
       </c>
       <c r="C28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$174,$A28&amp;"*",'QA Checklist'!$H$5:$H$174,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$174,$A28&amp;"*",'QA Checklist'!$H$5:$H$174,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$175,$A28&amp;"*",'QA Checklist'!$H$5:$H$175,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$175,$A28&amp;"*",'QA Checklist'!$H$5:$H$175,"Pass")</f>
         <v/>
       </c>
       <c r="D28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$174,$A28&amp;"*",'QA Checklist'!$H$5:$H$174,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$174,$A28&amp;"*",'QA Checklist'!$H$5:$H$174,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$175,$A28&amp;"*",'QA Checklist'!$H$5:$H$175,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$175,$A28&amp;"*",'QA Checklist'!$H$5:$H$175,"Fail")</f>
         <v/>
       </c>
       <c r="E28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$174,$A28&amp;"*",'QA Checklist'!$H$5:$H$174,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$175,$A28&amp;"*",'QA Checklist'!$H$5:$H$175,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1096,7 +1096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I174"/>
+  <dimension ref="A1:I175"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8717,12 +8717,59 @@
         </is>
       </c>
     </row>
+    <row r="175">
+      <c r="A175" s="12" t="inlineStr">
+        <is>
+          <t>SA-49</t>
+        </is>
+      </c>
+      <c r="B175" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="C175" s="13" t="inlineStr">
+        <is>
+          <t>Tier 2 (Workflow &amp; Ergonomics)</t>
+        </is>
+      </c>
+      <c r="D175" s="13" t="inlineStr">
+        <is>
+          <t>Workshop_Monitoring Studio Tab</t>
+        </is>
+      </c>
+      <c r="E175" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="F175" s="13" t="inlineStr">
+        <is>
+          <t>Log in as Service Advisor, open 2025 RO Excel Studio, fill Customer Name and Plate on Job_Order, open the Workshop_Monitoring tab, change the dispatch fields and press Register Repair Order to System</t>
+        </is>
+      </c>
+      <c r="G175" s="13" t="inlineStr">
+        <is>
+          <t>Workshop_Monitoring tab appears after CheckList_Result; it holds the Workshop Monitoring &amp; Daily Intakes fields (no longer on Job_Order); the preview shows the Job_Order and monitoring values live and turns Ready when Plate and Customer are filled; Register RO creates the Daily Intakes entry with these values</t>
+        </is>
+      </c>
+      <c r="H175" s="14" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="I175" s="13" t="inlineStr">
+        <is>
+          <t>Verified by Automated Unit Tests (161 passing in tests/frontend/sla_and_logic.test.js AUT-FRONT-132) and headless Chrome tab switch and screenshots</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:I174"/>
+  <autoFilter ref="A4:I175"/>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="H5:H174">
+  <conditionalFormatting sqref="H5:H175">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$H5="Passed"</formula>
     </cfRule>
@@ -8739,13 +8786,13 @@
       <formula>$H5="Pending"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A5:A174">
+  <conditionalFormatting sqref="A5:A175">
     <cfRule type="expression" priority="6" dxfId="3">
-      <formula>COUNTIF($A$5:$A$174,$A5)&gt;1</formula>
+      <formula>COUNTIF($A$5:$A$175,$A5)&gt;1</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H5:H174" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H5:H175" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pending,Passed,Failed"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat(REV-174): put Workshop_Monitoring first in the studio tab bar
Tab order is now Workshop_Monitoring, Job_Order, Quotation_No, Billing_No,
CheckList_Result. Cache buster v=3.27, AUT-FRONT-133, SA-50.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
+++ b/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
@@ -11,7 +11,7 @@
     <sheet name="QA Checklist" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$175</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$176</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'QA Checklist'!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTA('QA Checklist'!$A$5:$A$175)</f>
+        <f>COUNTA('QA Checklist'!$A$5:$A$176)</f>
         <v/>
       </c>
     </row>
@@ -594,7 +594,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$175,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$175,"Pass")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$176,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$176,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$175,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$175,"Fail")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$176,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$176,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -616,7 +616,7 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$175,"Pending")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$176,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -671,19 +671,19 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$175,$A12)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$176,$A12)</f>
         <v/>
       </c>
       <c r="C12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$175,$A12,'QA Checklist'!$H$5:$H$175,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$175,$A12,'QA Checklist'!$H$5:$H$175,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$176,$A12,'QA Checklist'!$H$5:$H$176,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$176,$A12,'QA Checklist'!$H$5:$H$176,"Pass")</f>
         <v/>
       </c>
       <c r="D12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$175,$A12,'QA Checklist'!$H$5:$H$175,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$175,$A12,'QA Checklist'!$H$5:$H$175,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$176,$A12,'QA Checklist'!$H$5:$H$176,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$176,$A12,'QA Checklist'!$H$5:$H$176,"Fail")</f>
         <v/>
       </c>
       <c r="E12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$175,$A12,'QA Checklist'!$H$5:$H$175,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$176,$A12,'QA Checklist'!$H$5:$H$176,"Pending")</f>
         <v/>
       </c>
       <c r="F12" s="8">
@@ -698,19 +698,19 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$175,$A13)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$176,$A13)</f>
         <v/>
       </c>
       <c r="C13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$175,$A13,'QA Checklist'!$H$5:$H$175,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$175,$A13,'QA Checklist'!$H$5:$H$175,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$176,$A13,'QA Checklist'!$H$5:$H$176,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$176,$A13,'QA Checklist'!$H$5:$H$176,"Pass")</f>
         <v/>
       </c>
       <c r="D13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$175,$A13,'QA Checklist'!$H$5:$H$175,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$175,$A13,'QA Checklist'!$H$5:$H$175,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$176,$A13,'QA Checklist'!$H$5:$H$176,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$176,$A13,'QA Checklist'!$H$5:$H$176,"Fail")</f>
         <v/>
       </c>
       <c r="E13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$175,$A13,'QA Checklist'!$H$5:$H$175,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$176,$A13,'QA Checklist'!$H$5:$H$176,"Pending")</f>
         <v/>
       </c>
       <c r="F13" s="8">
@@ -725,19 +725,19 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$175,$A14)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$176,$A14)</f>
         <v/>
       </c>
       <c r="C14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$175,$A14,'QA Checklist'!$H$5:$H$175,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$175,$A14,'QA Checklist'!$H$5:$H$175,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$176,$A14,'QA Checklist'!$H$5:$H$176,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$176,$A14,'QA Checklist'!$H$5:$H$176,"Pass")</f>
         <v/>
       </c>
       <c r="D14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$175,$A14,'QA Checklist'!$H$5:$H$175,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$175,$A14,'QA Checklist'!$H$5:$H$175,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$176,$A14,'QA Checklist'!$H$5:$H$176,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$176,$A14,'QA Checklist'!$H$5:$H$176,"Fail")</f>
         <v/>
       </c>
       <c r="E14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$175,$A14,'QA Checklist'!$H$5:$H$175,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$176,$A14,'QA Checklist'!$H$5:$H$176,"Pending")</f>
         <v/>
       </c>
       <c r="F14" s="8">
@@ -752,19 +752,19 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$175,$A15)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$176,$A15)</f>
         <v/>
       </c>
       <c r="C15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$175,$A15,'QA Checklist'!$H$5:$H$175,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$175,$A15,'QA Checklist'!$H$5:$H$175,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$176,$A15,'QA Checklist'!$H$5:$H$176,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$176,$A15,'QA Checklist'!$H$5:$H$176,"Pass")</f>
         <v/>
       </c>
       <c r="D15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$175,$A15,'QA Checklist'!$H$5:$H$175,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$175,$A15,'QA Checklist'!$H$5:$H$175,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$176,$A15,'QA Checklist'!$H$5:$H$176,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$176,$A15,'QA Checklist'!$H$5:$H$176,"Fail")</f>
         <v/>
       </c>
       <c r="E15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$175,$A15,'QA Checklist'!$H$5:$H$175,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$176,$A15,'QA Checklist'!$H$5:$H$176,"Pending")</f>
         <v/>
       </c>
       <c r="F15" s="8">
@@ -779,19 +779,19 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$175,$A16)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$176,$A16)</f>
         <v/>
       </c>
       <c r="C16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$175,$A16,'QA Checklist'!$H$5:$H$175,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$175,$A16,'QA Checklist'!$H$5:$H$175,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$176,$A16,'QA Checklist'!$H$5:$H$176,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$176,$A16,'QA Checklist'!$H$5:$H$176,"Pass")</f>
         <v/>
       </c>
       <c r="D16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$175,$A16,'QA Checklist'!$H$5:$H$175,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$175,$A16,'QA Checklist'!$H$5:$H$175,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$176,$A16,'QA Checklist'!$H$5:$H$176,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$176,$A16,'QA Checklist'!$H$5:$H$176,"Fail")</f>
         <v/>
       </c>
       <c r="E16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$175,$A16,'QA Checklist'!$H$5:$H$175,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$176,$A16,'QA Checklist'!$H$5:$H$176,"Pending")</f>
         <v/>
       </c>
       <c r="F16" s="8">
@@ -806,19 +806,19 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$175,$A17)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$176,$A17)</f>
         <v/>
       </c>
       <c r="C17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$175,$A17,'QA Checklist'!$H$5:$H$175,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$175,$A17,'QA Checklist'!$H$5:$H$175,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$176,$A17,'QA Checklist'!$H$5:$H$176,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$176,$A17,'QA Checklist'!$H$5:$H$176,"Pass")</f>
         <v/>
       </c>
       <c r="D17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$175,$A17,'QA Checklist'!$H$5:$H$175,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$175,$A17,'QA Checklist'!$H$5:$H$175,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$176,$A17,'QA Checklist'!$H$5:$H$176,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$176,$A17,'QA Checklist'!$H$5:$H$176,"Fail")</f>
         <v/>
       </c>
       <c r="E17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$175,$A17,'QA Checklist'!$H$5:$H$175,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$176,$A17,'QA Checklist'!$H$5:$H$176,"Pending")</f>
         <v/>
       </c>
       <c r="F17" s="8">
@@ -833,19 +833,19 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$175,$A18)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$176,$A18)</f>
         <v/>
       </c>
       <c r="C18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$175,$A18,'QA Checklist'!$H$5:$H$175,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$175,$A18,'QA Checklist'!$H$5:$H$175,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$176,$A18,'QA Checklist'!$H$5:$H$176,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$176,$A18,'QA Checklist'!$H$5:$H$176,"Pass")</f>
         <v/>
       </c>
       <c r="D18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$175,$A18,'QA Checklist'!$H$5:$H$175,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$175,$A18,'QA Checklist'!$H$5:$H$175,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$176,$A18,'QA Checklist'!$H$5:$H$176,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$176,$A18,'QA Checklist'!$H$5:$H$176,"Fail")</f>
         <v/>
       </c>
       <c r="E18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$175,$A18,'QA Checklist'!$H$5:$H$175,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$176,$A18,'QA Checklist'!$H$5:$H$176,"Pending")</f>
         <v/>
       </c>
       <c r="F18" s="8">
@@ -860,19 +860,19 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$175,$A19)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$176,$A19)</f>
         <v/>
       </c>
       <c r="C19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$175,$A19,'QA Checklist'!$H$5:$H$175,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$175,$A19,'QA Checklist'!$H$5:$H$175,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$176,$A19,'QA Checklist'!$H$5:$H$176,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$176,$A19,'QA Checklist'!$H$5:$H$176,"Pass")</f>
         <v/>
       </c>
       <c r="D19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$175,$A19,'QA Checklist'!$H$5:$H$175,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$175,$A19,'QA Checklist'!$H$5:$H$175,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$176,$A19,'QA Checklist'!$H$5:$H$176,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$176,$A19,'QA Checklist'!$H$5:$H$176,"Fail")</f>
         <v/>
       </c>
       <c r="E19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$175,$A19,'QA Checklist'!$H$5:$H$175,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$176,$A19,'QA Checklist'!$H$5:$H$176,"Pending")</f>
         <v/>
       </c>
       <c r="F19" s="8">
@@ -887,19 +887,19 @@
         </is>
       </c>
       <c r="B20" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$175,$A20)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$176,$A20)</f>
         <v/>
       </c>
       <c r="C20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$175,$A20,'QA Checklist'!$H$5:$H$175,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$175,$A20,'QA Checklist'!$H$5:$H$175,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$176,$A20,'QA Checklist'!$H$5:$H$176,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$176,$A20,'QA Checklist'!$H$5:$H$176,"Pass")</f>
         <v/>
       </c>
       <c r="D20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$175,$A20,'QA Checklist'!$H$5:$H$175,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$175,$A20,'QA Checklist'!$H$5:$H$175,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$176,$A20,'QA Checklist'!$H$5:$H$176,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$176,$A20,'QA Checklist'!$H$5:$H$176,"Fail")</f>
         <v/>
       </c>
       <c r="E20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$175,$A20,'QA Checklist'!$H$5:$H$175,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$176,$A20,'QA Checklist'!$H$5:$H$176,"Pending")</f>
         <v/>
       </c>
       <c r="F20" s="8">
@@ -914,19 +914,19 @@
         </is>
       </c>
       <c r="B21" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$175,$A21)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$176,$A21)</f>
         <v/>
       </c>
       <c r="C21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$175,$A21,'QA Checklist'!$H$5:$H$175,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$175,$A21,'QA Checklist'!$H$5:$H$175,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$176,$A21,'QA Checklist'!$H$5:$H$176,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$176,$A21,'QA Checklist'!$H$5:$H$176,"Pass")</f>
         <v/>
       </c>
       <c r="D21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$175,$A21,'QA Checklist'!$H$5:$H$175,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$175,$A21,'QA Checklist'!$H$5:$H$175,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$176,$A21,'QA Checklist'!$H$5:$H$176,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$176,$A21,'QA Checklist'!$H$5:$H$176,"Fail")</f>
         <v/>
       </c>
       <c r="E21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$175,$A21,'QA Checklist'!$H$5:$H$175,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$176,$A21,'QA Checklist'!$H$5:$H$176,"Pending")</f>
         <v/>
       </c>
       <c r="F21" s="8">
@@ -941,19 +941,19 @@
         </is>
       </c>
       <c r="B22" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$175,$A22)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$176,$A22)</f>
         <v/>
       </c>
       <c r="C22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$175,$A22,'QA Checklist'!$H$5:$H$175,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$175,$A22,'QA Checklist'!$H$5:$H$175,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$176,$A22,'QA Checklist'!$H$5:$H$176,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$176,$A22,'QA Checklist'!$H$5:$H$176,"Pass")</f>
         <v/>
       </c>
       <c r="D22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$175,$A22,'QA Checklist'!$H$5:$H$175,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$175,$A22,'QA Checklist'!$H$5:$H$175,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$176,$A22,'QA Checklist'!$H$5:$H$176,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$176,$A22,'QA Checklist'!$H$5:$H$176,"Fail")</f>
         <v/>
       </c>
       <c r="E22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$175,$A22,'QA Checklist'!$H$5:$H$175,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$176,$A22,'QA Checklist'!$H$5:$H$176,"Pending")</f>
         <v/>
       </c>
       <c r="F22" s="8">
@@ -1023,19 +1023,19 @@
         </is>
       </c>
       <c r="B26" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$175,$A26&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$176,$A26&amp;"*")</f>
         <v/>
       </c>
       <c r="C26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$175,$A26&amp;"*",'QA Checklist'!$H$5:$H$175,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$175,$A26&amp;"*",'QA Checklist'!$H$5:$H$175,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$176,$A26&amp;"*",'QA Checklist'!$H$5:$H$176,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$176,$A26&amp;"*",'QA Checklist'!$H$5:$H$176,"Pass")</f>
         <v/>
       </c>
       <c r="D26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$175,$A26&amp;"*",'QA Checklist'!$H$5:$H$175,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$175,$A26&amp;"*",'QA Checklist'!$H$5:$H$175,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$176,$A26&amp;"*",'QA Checklist'!$H$5:$H$176,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$176,$A26&amp;"*",'QA Checklist'!$H$5:$H$176,"Fail")</f>
         <v/>
       </c>
       <c r="E26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$175,$A26&amp;"*",'QA Checklist'!$H$5:$H$175,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$176,$A26&amp;"*",'QA Checklist'!$H$5:$H$176,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1046,19 +1046,19 @@
         </is>
       </c>
       <c r="B27" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$175,$A27&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$176,$A27&amp;"*")</f>
         <v/>
       </c>
       <c r="C27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$175,$A27&amp;"*",'QA Checklist'!$H$5:$H$175,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$175,$A27&amp;"*",'QA Checklist'!$H$5:$H$175,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$176,$A27&amp;"*",'QA Checklist'!$H$5:$H$176,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$176,$A27&amp;"*",'QA Checklist'!$H$5:$H$176,"Pass")</f>
         <v/>
       </c>
       <c r="D27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$175,$A27&amp;"*",'QA Checklist'!$H$5:$H$175,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$175,$A27&amp;"*",'QA Checklist'!$H$5:$H$175,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$176,$A27&amp;"*",'QA Checklist'!$H$5:$H$176,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$176,$A27&amp;"*",'QA Checklist'!$H$5:$H$176,"Fail")</f>
         <v/>
       </c>
       <c r="E27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$175,$A27&amp;"*",'QA Checklist'!$H$5:$H$175,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$176,$A27&amp;"*",'QA Checklist'!$H$5:$H$176,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1069,19 +1069,19 @@
         </is>
       </c>
       <c r="B28" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$175,$A28&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$176,$A28&amp;"*")</f>
         <v/>
       </c>
       <c r="C28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$175,$A28&amp;"*",'QA Checklist'!$H$5:$H$175,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$175,$A28&amp;"*",'QA Checklist'!$H$5:$H$175,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$176,$A28&amp;"*",'QA Checklist'!$H$5:$H$176,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$176,$A28&amp;"*",'QA Checklist'!$H$5:$H$176,"Pass")</f>
         <v/>
       </c>
       <c r="D28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$175,$A28&amp;"*",'QA Checklist'!$H$5:$H$175,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$175,$A28&amp;"*",'QA Checklist'!$H$5:$H$175,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$176,$A28&amp;"*",'QA Checklist'!$H$5:$H$176,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$176,$A28&amp;"*",'QA Checklist'!$H$5:$H$176,"Fail")</f>
         <v/>
       </c>
       <c r="E28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$175,$A28&amp;"*",'QA Checklist'!$H$5:$H$175,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$176,$A28&amp;"*",'QA Checklist'!$H$5:$H$176,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1096,7 +1096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I175"/>
+  <dimension ref="A1:I176"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8764,12 +8764,59 @@
         </is>
       </c>
     </row>
+    <row r="176">
+      <c r="A176" s="12" t="inlineStr">
+        <is>
+          <t>SA-50</t>
+        </is>
+      </c>
+      <c r="B176" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="C176" s="13" t="inlineStr">
+        <is>
+          <t>Tier 2 (Workflow &amp; Ergonomics)</t>
+        </is>
+      </c>
+      <c r="D176" s="13" t="inlineStr">
+        <is>
+          <t>Workshop_Monitoring First Tab</t>
+        </is>
+      </c>
+      <c r="E176" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="F176" s="13" t="inlineStr">
+        <is>
+          <t>Log in as Service Advisor, open 2025 RO Excel Studio and look at the tab bar, then click each tab</t>
+        </is>
+      </c>
+      <c r="G176" s="13" t="inlineStr">
+        <is>
+          <t>Tabs read Workshop_Monitoring, Job_Order, Quotation_No, Billing_No, CheckList_Result from left to right and each opens its own view</t>
+        </is>
+      </c>
+      <c r="H176" s="14" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="I176" s="13" t="inlineStr">
+        <is>
+          <t>Verified by Automated Unit Tests (162 passing in tests/frontend/sla_and_logic.test.js AUT-FRONT-133) and a headless Chrome tab bar render</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:I175"/>
+  <autoFilter ref="A4:I176"/>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="H5:H175">
+  <conditionalFormatting sqref="H5:H176">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$H5="Passed"</formula>
     </cfRule>
@@ -8786,13 +8833,13 @@
       <formula>$H5="Pending"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A5:A175">
+  <conditionalFormatting sqref="A5:A176">
     <cfRule type="expression" priority="6" dxfId="3">
-      <formula>COUNTIF($A$5:$A$175,$A5)&gt;1</formula>
+      <formula>COUNTIF($A$5:$A$176,$A5)&gt;1</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H5:H175" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H5:H176" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pending,Passed,Failed"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat(REV-175): automatic branch and arrival, Plate/Model on Workshop_Monitoring
Remove the Target Branch select and Arrival Time input: Register RO sends
the SA account's branch and stamps the clock time at submission. Add
Plate No. and Model (synced with Job_Order) and limit Intake Source to
Walk-in / Online Appointment. Cache buster v=3.28, AUT-FRONT-134, SA-51.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
+++ b/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
@@ -11,7 +11,7 @@
     <sheet name="QA Checklist" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$176</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$177</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'QA Checklist'!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTA('QA Checklist'!$A$5:$A$176)</f>
+        <f>COUNTA('QA Checklist'!$A$5:$A$177)</f>
         <v/>
       </c>
     </row>
@@ -594,7 +594,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$176,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$176,"Pass")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$177,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$177,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$176,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$176,"Fail")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$177,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$177,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -616,7 +616,7 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$176,"Pending")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$177,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -671,19 +671,19 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$176,$A12)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$177,$A12)</f>
         <v/>
       </c>
       <c r="C12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$176,$A12,'QA Checklist'!$H$5:$H$176,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$176,$A12,'QA Checklist'!$H$5:$H$176,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$177,$A12,'QA Checklist'!$H$5:$H$177,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$177,$A12,'QA Checklist'!$H$5:$H$177,"Pass")</f>
         <v/>
       </c>
       <c r="D12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$176,$A12,'QA Checklist'!$H$5:$H$176,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$176,$A12,'QA Checklist'!$H$5:$H$176,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$177,$A12,'QA Checklist'!$H$5:$H$177,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$177,$A12,'QA Checklist'!$H$5:$H$177,"Fail")</f>
         <v/>
       </c>
       <c r="E12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$176,$A12,'QA Checklist'!$H$5:$H$176,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$177,$A12,'QA Checklist'!$H$5:$H$177,"Pending")</f>
         <v/>
       </c>
       <c r="F12" s="8">
@@ -698,19 +698,19 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$176,$A13)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$177,$A13)</f>
         <v/>
       </c>
       <c r="C13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$176,$A13,'QA Checklist'!$H$5:$H$176,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$176,$A13,'QA Checklist'!$H$5:$H$176,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$177,$A13,'QA Checklist'!$H$5:$H$177,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$177,$A13,'QA Checklist'!$H$5:$H$177,"Pass")</f>
         <v/>
       </c>
       <c r="D13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$176,$A13,'QA Checklist'!$H$5:$H$176,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$176,$A13,'QA Checklist'!$H$5:$H$176,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$177,$A13,'QA Checklist'!$H$5:$H$177,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$177,$A13,'QA Checklist'!$H$5:$H$177,"Fail")</f>
         <v/>
       </c>
       <c r="E13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$176,$A13,'QA Checklist'!$H$5:$H$176,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$177,$A13,'QA Checklist'!$H$5:$H$177,"Pending")</f>
         <v/>
       </c>
       <c r="F13" s="8">
@@ -725,19 +725,19 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$176,$A14)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$177,$A14)</f>
         <v/>
       </c>
       <c r="C14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$176,$A14,'QA Checklist'!$H$5:$H$176,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$176,$A14,'QA Checklist'!$H$5:$H$176,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$177,$A14,'QA Checklist'!$H$5:$H$177,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$177,$A14,'QA Checklist'!$H$5:$H$177,"Pass")</f>
         <v/>
       </c>
       <c r="D14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$176,$A14,'QA Checklist'!$H$5:$H$176,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$176,$A14,'QA Checklist'!$H$5:$H$176,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$177,$A14,'QA Checklist'!$H$5:$H$177,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$177,$A14,'QA Checklist'!$H$5:$H$177,"Fail")</f>
         <v/>
       </c>
       <c r="E14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$176,$A14,'QA Checklist'!$H$5:$H$176,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$177,$A14,'QA Checklist'!$H$5:$H$177,"Pending")</f>
         <v/>
       </c>
       <c r="F14" s="8">
@@ -752,19 +752,19 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$176,$A15)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$177,$A15)</f>
         <v/>
       </c>
       <c r="C15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$176,$A15,'QA Checklist'!$H$5:$H$176,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$176,$A15,'QA Checklist'!$H$5:$H$176,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$177,$A15,'QA Checklist'!$H$5:$H$177,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$177,$A15,'QA Checklist'!$H$5:$H$177,"Pass")</f>
         <v/>
       </c>
       <c r="D15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$176,$A15,'QA Checklist'!$H$5:$H$176,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$176,$A15,'QA Checklist'!$H$5:$H$176,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$177,$A15,'QA Checklist'!$H$5:$H$177,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$177,$A15,'QA Checklist'!$H$5:$H$177,"Fail")</f>
         <v/>
       </c>
       <c r="E15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$176,$A15,'QA Checklist'!$H$5:$H$176,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$177,$A15,'QA Checklist'!$H$5:$H$177,"Pending")</f>
         <v/>
       </c>
       <c r="F15" s="8">
@@ -779,19 +779,19 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$176,$A16)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$177,$A16)</f>
         <v/>
       </c>
       <c r="C16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$176,$A16,'QA Checklist'!$H$5:$H$176,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$176,$A16,'QA Checklist'!$H$5:$H$176,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$177,$A16,'QA Checklist'!$H$5:$H$177,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$177,$A16,'QA Checklist'!$H$5:$H$177,"Pass")</f>
         <v/>
       </c>
       <c r="D16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$176,$A16,'QA Checklist'!$H$5:$H$176,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$176,$A16,'QA Checklist'!$H$5:$H$176,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$177,$A16,'QA Checklist'!$H$5:$H$177,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$177,$A16,'QA Checklist'!$H$5:$H$177,"Fail")</f>
         <v/>
       </c>
       <c r="E16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$176,$A16,'QA Checklist'!$H$5:$H$176,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$177,$A16,'QA Checklist'!$H$5:$H$177,"Pending")</f>
         <v/>
       </c>
       <c r="F16" s="8">
@@ -806,19 +806,19 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$176,$A17)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$177,$A17)</f>
         <v/>
       </c>
       <c r="C17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$176,$A17,'QA Checklist'!$H$5:$H$176,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$176,$A17,'QA Checklist'!$H$5:$H$176,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$177,$A17,'QA Checklist'!$H$5:$H$177,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$177,$A17,'QA Checklist'!$H$5:$H$177,"Pass")</f>
         <v/>
       </c>
       <c r="D17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$176,$A17,'QA Checklist'!$H$5:$H$176,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$176,$A17,'QA Checklist'!$H$5:$H$176,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$177,$A17,'QA Checklist'!$H$5:$H$177,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$177,$A17,'QA Checklist'!$H$5:$H$177,"Fail")</f>
         <v/>
       </c>
       <c r="E17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$176,$A17,'QA Checklist'!$H$5:$H$176,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$177,$A17,'QA Checklist'!$H$5:$H$177,"Pending")</f>
         <v/>
       </c>
       <c r="F17" s="8">
@@ -833,19 +833,19 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$176,$A18)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$177,$A18)</f>
         <v/>
       </c>
       <c r="C18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$176,$A18,'QA Checklist'!$H$5:$H$176,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$176,$A18,'QA Checklist'!$H$5:$H$176,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$177,$A18,'QA Checklist'!$H$5:$H$177,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$177,$A18,'QA Checklist'!$H$5:$H$177,"Pass")</f>
         <v/>
       </c>
       <c r="D18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$176,$A18,'QA Checklist'!$H$5:$H$176,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$176,$A18,'QA Checklist'!$H$5:$H$176,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$177,$A18,'QA Checklist'!$H$5:$H$177,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$177,$A18,'QA Checklist'!$H$5:$H$177,"Fail")</f>
         <v/>
       </c>
       <c r="E18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$176,$A18,'QA Checklist'!$H$5:$H$176,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$177,$A18,'QA Checklist'!$H$5:$H$177,"Pending")</f>
         <v/>
       </c>
       <c r="F18" s="8">
@@ -860,19 +860,19 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$176,$A19)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$177,$A19)</f>
         <v/>
       </c>
       <c r="C19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$176,$A19,'QA Checklist'!$H$5:$H$176,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$176,$A19,'QA Checklist'!$H$5:$H$176,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$177,$A19,'QA Checklist'!$H$5:$H$177,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$177,$A19,'QA Checklist'!$H$5:$H$177,"Pass")</f>
         <v/>
       </c>
       <c r="D19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$176,$A19,'QA Checklist'!$H$5:$H$176,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$176,$A19,'QA Checklist'!$H$5:$H$176,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$177,$A19,'QA Checklist'!$H$5:$H$177,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$177,$A19,'QA Checklist'!$H$5:$H$177,"Fail")</f>
         <v/>
       </c>
       <c r="E19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$176,$A19,'QA Checklist'!$H$5:$H$176,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$177,$A19,'QA Checklist'!$H$5:$H$177,"Pending")</f>
         <v/>
       </c>
       <c r="F19" s="8">
@@ -887,19 +887,19 @@
         </is>
       </c>
       <c r="B20" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$176,$A20)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$177,$A20)</f>
         <v/>
       </c>
       <c r="C20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$176,$A20,'QA Checklist'!$H$5:$H$176,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$176,$A20,'QA Checklist'!$H$5:$H$176,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$177,$A20,'QA Checklist'!$H$5:$H$177,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$177,$A20,'QA Checklist'!$H$5:$H$177,"Pass")</f>
         <v/>
       </c>
       <c r="D20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$176,$A20,'QA Checklist'!$H$5:$H$176,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$176,$A20,'QA Checklist'!$H$5:$H$176,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$177,$A20,'QA Checklist'!$H$5:$H$177,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$177,$A20,'QA Checklist'!$H$5:$H$177,"Fail")</f>
         <v/>
       </c>
       <c r="E20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$176,$A20,'QA Checklist'!$H$5:$H$176,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$177,$A20,'QA Checklist'!$H$5:$H$177,"Pending")</f>
         <v/>
       </c>
       <c r="F20" s="8">
@@ -914,19 +914,19 @@
         </is>
       </c>
       <c r="B21" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$176,$A21)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$177,$A21)</f>
         <v/>
       </c>
       <c r="C21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$176,$A21,'QA Checklist'!$H$5:$H$176,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$176,$A21,'QA Checklist'!$H$5:$H$176,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$177,$A21,'QA Checklist'!$H$5:$H$177,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$177,$A21,'QA Checklist'!$H$5:$H$177,"Pass")</f>
         <v/>
       </c>
       <c r="D21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$176,$A21,'QA Checklist'!$H$5:$H$176,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$176,$A21,'QA Checklist'!$H$5:$H$176,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$177,$A21,'QA Checklist'!$H$5:$H$177,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$177,$A21,'QA Checklist'!$H$5:$H$177,"Fail")</f>
         <v/>
       </c>
       <c r="E21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$176,$A21,'QA Checklist'!$H$5:$H$176,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$177,$A21,'QA Checklist'!$H$5:$H$177,"Pending")</f>
         <v/>
       </c>
       <c r="F21" s="8">
@@ -941,19 +941,19 @@
         </is>
       </c>
       <c r="B22" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$176,$A22)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$177,$A22)</f>
         <v/>
       </c>
       <c r="C22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$176,$A22,'QA Checklist'!$H$5:$H$176,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$176,$A22,'QA Checklist'!$H$5:$H$176,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$177,$A22,'QA Checklist'!$H$5:$H$177,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$177,$A22,'QA Checklist'!$H$5:$H$177,"Pass")</f>
         <v/>
       </c>
       <c r="D22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$176,$A22,'QA Checklist'!$H$5:$H$176,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$176,$A22,'QA Checklist'!$H$5:$H$176,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$177,$A22,'QA Checklist'!$H$5:$H$177,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$177,$A22,'QA Checklist'!$H$5:$H$177,"Fail")</f>
         <v/>
       </c>
       <c r="E22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$176,$A22,'QA Checklist'!$H$5:$H$176,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$177,$A22,'QA Checklist'!$H$5:$H$177,"Pending")</f>
         <v/>
       </c>
       <c r="F22" s="8">
@@ -1023,19 +1023,19 @@
         </is>
       </c>
       <c r="B26" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$176,$A26&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$177,$A26&amp;"*")</f>
         <v/>
       </c>
       <c r="C26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$176,$A26&amp;"*",'QA Checklist'!$H$5:$H$176,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$176,$A26&amp;"*",'QA Checklist'!$H$5:$H$176,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$177,$A26&amp;"*",'QA Checklist'!$H$5:$H$177,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$177,$A26&amp;"*",'QA Checklist'!$H$5:$H$177,"Pass")</f>
         <v/>
       </c>
       <c r="D26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$176,$A26&amp;"*",'QA Checklist'!$H$5:$H$176,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$176,$A26&amp;"*",'QA Checklist'!$H$5:$H$176,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$177,$A26&amp;"*",'QA Checklist'!$H$5:$H$177,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$177,$A26&amp;"*",'QA Checklist'!$H$5:$H$177,"Fail")</f>
         <v/>
       </c>
       <c r="E26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$176,$A26&amp;"*",'QA Checklist'!$H$5:$H$176,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$177,$A26&amp;"*",'QA Checklist'!$H$5:$H$177,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1046,19 +1046,19 @@
         </is>
       </c>
       <c r="B27" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$176,$A27&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$177,$A27&amp;"*")</f>
         <v/>
       </c>
       <c r="C27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$176,$A27&amp;"*",'QA Checklist'!$H$5:$H$176,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$176,$A27&amp;"*",'QA Checklist'!$H$5:$H$176,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$177,$A27&amp;"*",'QA Checklist'!$H$5:$H$177,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$177,$A27&amp;"*",'QA Checklist'!$H$5:$H$177,"Pass")</f>
         <v/>
       </c>
       <c r="D27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$176,$A27&amp;"*",'QA Checklist'!$H$5:$H$176,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$176,$A27&amp;"*",'QA Checklist'!$H$5:$H$176,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$177,$A27&amp;"*",'QA Checklist'!$H$5:$H$177,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$177,$A27&amp;"*",'QA Checklist'!$H$5:$H$177,"Fail")</f>
         <v/>
       </c>
       <c r="E27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$176,$A27&amp;"*",'QA Checklist'!$H$5:$H$176,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$177,$A27&amp;"*",'QA Checklist'!$H$5:$H$177,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1069,19 +1069,19 @@
         </is>
       </c>
       <c r="B28" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$176,$A28&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$177,$A28&amp;"*")</f>
         <v/>
       </c>
       <c r="C28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$176,$A28&amp;"*",'QA Checklist'!$H$5:$H$176,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$176,$A28&amp;"*",'QA Checklist'!$H$5:$H$176,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$177,$A28&amp;"*",'QA Checklist'!$H$5:$H$177,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$177,$A28&amp;"*",'QA Checklist'!$H$5:$H$177,"Pass")</f>
         <v/>
       </c>
       <c r="D28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$176,$A28&amp;"*",'QA Checklist'!$H$5:$H$176,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$176,$A28&amp;"*",'QA Checklist'!$H$5:$H$176,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$177,$A28&amp;"*",'QA Checklist'!$H$5:$H$177,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$177,$A28&amp;"*",'QA Checklist'!$H$5:$H$177,"Fail")</f>
         <v/>
       </c>
       <c r="E28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$176,$A28&amp;"*",'QA Checklist'!$H$5:$H$176,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$177,$A28&amp;"*",'QA Checklist'!$H$5:$H$177,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1096,7 +1096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I176"/>
+  <dimension ref="A1:I177"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8811,12 +8811,59 @@
         </is>
       </c>
     </row>
+    <row r="177">
+      <c r="A177" s="12" t="inlineStr">
+        <is>
+          <t>SA-51</t>
+        </is>
+      </c>
+      <c r="B177" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="C177" s="13" t="inlineStr">
+        <is>
+          <t>Tier 2 (Workflow &amp; Ergonomics)</t>
+        </is>
+      </c>
+      <c r="D177" s="13" t="inlineStr">
+        <is>
+          <t>Workshop_Monitoring Automatic Branch &amp; Arrival, Plate / Model</t>
+        </is>
+      </c>
+      <c r="E177" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="F177" s="13" t="inlineStr">
+        <is>
+          <t>Log in as a Marikina SA, open 2025 RO Excel Studio &gt; Workshop_Monitoring, type Plate No. and Model, choose Walk-in or Online Appointment, press Register Repair Order to System and open Daily Intakes; repeat as a Regalado SA</t>
+        </is>
+      </c>
+      <c r="G177" s="13" t="inlineStr">
+        <is>
+          <t>No Target Branch or Arrival Time fields on the card; Plate No. and Model appear on Job_Order as typed; the new Daily Intakes entry shows the SA branch and the arrival time of the moment Register was pressed, and the chosen source</t>
+        </is>
+      </c>
+      <c r="H177" s="14" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="I177" s="13" t="inlineStr">
+        <is>
+          <t>Verified by Automated Unit Tests (163 passing in tests/frontend/sla_and_logic.test.js AUT-FRONT-134) and a headless Chrome register payload check</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:I176"/>
+  <autoFilter ref="A4:I177"/>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="H5:H176">
+  <conditionalFormatting sqref="H5:H177">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$H5="Passed"</formula>
     </cfRule>
@@ -8833,13 +8880,13 @@
       <formula>$H5="Pending"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A5:A176">
+  <conditionalFormatting sqref="A5:A177">
     <cfRule type="expression" priority="6" dxfId="3">
-      <formula>COUNTIF($A$5:$A$176,$A5)&gt;1</formula>
+      <formula>COUNTIF($A$5:$A$177,$A5)&gt;1</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H5:H176" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H5:H177" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pending,Passed,Failed"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat(REV-176): intake paper / claim stub, monitoring clean-up, referral analytics
- jobs.referred_by (database.sql, migration.php, self-healing check);
  createJob saves the whitelisted referral, normalizeJob returns it
- Workshop_Monitoring: remove Parts / Bay / Floor Status; add Customer,
  Contact, Category, Concern, live Arrival Time (manual override) and
  Referred By; Print Claim Stub button
- Letter-size Customer Intake Paper with tear-off Claim Stub / Gate Pass
- Referral Sources & Acquisition Channels card in Owner / Admin Analytics
Cache buster v=3.29, AUT-FRONT-135, SA-52.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
+++ b/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
@@ -11,7 +11,7 @@
     <sheet name="QA Checklist" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$177</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$178</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'QA Checklist'!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTA('QA Checklist'!$A$5:$A$177)</f>
+        <f>COUNTA('QA Checklist'!$A$5:$A$178)</f>
         <v/>
       </c>
     </row>
@@ -594,7 +594,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$177,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$177,"Pass")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$178,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$178,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$177,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$177,"Fail")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$178,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$178,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -616,7 +616,7 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$177,"Pending")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$178,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -671,19 +671,19 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$177,$A12)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$178,$A12)</f>
         <v/>
       </c>
       <c r="C12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$177,$A12,'QA Checklist'!$H$5:$H$177,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$177,$A12,'QA Checklist'!$H$5:$H$177,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$178,$A12,'QA Checklist'!$H$5:$H$178,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$178,$A12,'QA Checklist'!$H$5:$H$178,"Pass")</f>
         <v/>
       </c>
       <c r="D12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$177,$A12,'QA Checklist'!$H$5:$H$177,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$177,$A12,'QA Checklist'!$H$5:$H$177,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$178,$A12,'QA Checklist'!$H$5:$H$178,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$178,$A12,'QA Checklist'!$H$5:$H$178,"Fail")</f>
         <v/>
       </c>
       <c r="E12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$177,$A12,'QA Checklist'!$H$5:$H$177,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$178,$A12,'QA Checklist'!$H$5:$H$178,"Pending")</f>
         <v/>
       </c>
       <c r="F12" s="8">
@@ -698,19 +698,19 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$177,$A13)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$178,$A13)</f>
         <v/>
       </c>
       <c r="C13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$177,$A13,'QA Checklist'!$H$5:$H$177,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$177,$A13,'QA Checklist'!$H$5:$H$177,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$178,$A13,'QA Checklist'!$H$5:$H$178,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$178,$A13,'QA Checklist'!$H$5:$H$178,"Pass")</f>
         <v/>
       </c>
       <c r="D13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$177,$A13,'QA Checklist'!$H$5:$H$177,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$177,$A13,'QA Checklist'!$H$5:$H$177,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$178,$A13,'QA Checklist'!$H$5:$H$178,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$178,$A13,'QA Checklist'!$H$5:$H$178,"Fail")</f>
         <v/>
       </c>
       <c r="E13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$177,$A13,'QA Checklist'!$H$5:$H$177,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$178,$A13,'QA Checklist'!$H$5:$H$178,"Pending")</f>
         <v/>
       </c>
       <c r="F13" s="8">
@@ -725,19 +725,19 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$177,$A14)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$178,$A14)</f>
         <v/>
       </c>
       <c r="C14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$177,$A14,'QA Checklist'!$H$5:$H$177,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$177,$A14,'QA Checklist'!$H$5:$H$177,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$178,$A14,'QA Checklist'!$H$5:$H$178,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$178,$A14,'QA Checklist'!$H$5:$H$178,"Pass")</f>
         <v/>
       </c>
       <c r="D14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$177,$A14,'QA Checklist'!$H$5:$H$177,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$177,$A14,'QA Checklist'!$H$5:$H$177,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$178,$A14,'QA Checklist'!$H$5:$H$178,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$178,$A14,'QA Checklist'!$H$5:$H$178,"Fail")</f>
         <v/>
       </c>
       <c r="E14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$177,$A14,'QA Checklist'!$H$5:$H$177,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$178,$A14,'QA Checklist'!$H$5:$H$178,"Pending")</f>
         <v/>
       </c>
       <c r="F14" s="8">
@@ -752,19 +752,19 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$177,$A15)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$178,$A15)</f>
         <v/>
       </c>
       <c r="C15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$177,$A15,'QA Checklist'!$H$5:$H$177,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$177,$A15,'QA Checklist'!$H$5:$H$177,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$178,$A15,'QA Checklist'!$H$5:$H$178,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$178,$A15,'QA Checklist'!$H$5:$H$178,"Pass")</f>
         <v/>
       </c>
       <c r="D15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$177,$A15,'QA Checklist'!$H$5:$H$177,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$177,$A15,'QA Checklist'!$H$5:$H$177,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$178,$A15,'QA Checklist'!$H$5:$H$178,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$178,$A15,'QA Checklist'!$H$5:$H$178,"Fail")</f>
         <v/>
       </c>
       <c r="E15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$177,$A15,'QA Checklist'!$H$5:$H$177,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$178,$A15,'QA Checklist'!$H$5:$H$178,"Pending")</f>
         <v/>
       </c>
       <c r="F15" s="8">
@@ -779,19 +779,19 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$177,$A16)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$178,$A16)</f>
         <v/>
       </c>
       <c r="C16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$177,$A16,'QA Checklist'!$H$5:$H$177,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$177,$A16,'QA Checklist'!$H$5:$H$177,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$178,$A16,'QA Checklist'!$H$5:$H$178,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$178,$A16,'QA Checklist'!$H$5:$H$178,"Pass")</f>
         <v/>
       </c>
       <c r="D16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$177,$A16,'QA Checklist'!$H$5:$H$177,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$177,$A16,'QA Checklist'!$H$5:$H$177,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$178,$A16,'QA Checklist'!$H$5:$H$178,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$178,$A16,'QA Checklist'!$H$5:$H$178,"Fail")</f>
         <v/>
       </c>
       <c r="E16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$177,$A16,'QA Checklist'!$H$5:$H$177,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$178,$A16,'QA Checklist'!$H$5:$H$178,"Pending")</f>
         <v/>
       </c>
       <c r="F16" s="8">
@@ -806,19 +806,19 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$177,$A17)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$178,$A17)</f>
         <v/>
       </c>
       <c r="C17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$177,$A17,'QA Checklist'!$H$5:$H$177,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$177,$A17,'QA Checklist'!$H$5:$H$177,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$178,$A17,'QA Checklist'!$H$5:$H$178,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$178,$A17,'QA Checklist'!$H$5:$H$178,"Pass")</f>
         <v/>
       </c>
       <c r="D17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$177,$A17,'QA Checklist'!$H$5:$H$177,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$177,$A17,'QA Checklist'!$H$5:$H$177,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$178,$A17,'QA Checklist'!$H$5:$H$178,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$178,$A17,'QA Checklist'!$H$5:$H$178,"Fail")</f>
         <v/>
       </c>
       <c r="E17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$177,$A17,'QA Checklist'!$H$5:$H$177,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$178,$A17,'QA Checklist'!$H$5:$H$178,"Pending")</f>
         <v/>
       </c>
       <c r="F17" s="8">
@@ -833,19 +833,19 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$177,$A18)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$178,$A18)</f>
         <v/>
       </c>
       <c r="C18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$177,$A18,'QA Checklist'!$H$5:$H$177,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$177,$A18,'QA Checklist'!$H$5:$H$177,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$178,$A18,'QA Checklist'!$H$5:$H$178,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$178,$A18,'QA Checklist'!$H$5:$H$178,"Pass")</f>
         <v/>
       </c>
       <c r="D18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$177,$A18,'QA Checklist'!$H$5:$H$177,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$177,$A18,'QA Checklist'!$H$5:$H$177,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$178,$A18,'QA Checklist'!$H$5:$H$178,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$178,$A18,'QA Checklist'!$H$5:$H$178,"Fail")</f>
         <v/>
       </c>
       <c r="E18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$177,$A18,'QA Checklist'!$H$5:$H$177,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$178,$A18,'QA Checklist'!$H$5:$H$178,"Pending")</f>
         <v/>
       </c>
       <c r="F18" s="8">
@@ -860,19 +860,19 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$177,$A19)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$178,$A19)</f>
         <v/>
       </c>
       <c r="C19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$177,$A19,'QA Checklist'!$H$5:$H$177,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$177,$A19,'QA Checklist'!$H$5:$H$177,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$178,$A19,'QA Checklist'!$H$5:$H$178,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$178,$A19,'QA Checklist'!$H$5:$H$178,"Pass")</f>
         <v/>
       </c>
       <c r="D19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$177,$A19,'QA Checklist'!$H$5:$H$177,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$177,$A19,'QA Checklist'!$H$5:$H$177,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$178,$A19,'QA Checklist'!$H$5:$H$178,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$178,$A19,'QA Checklist'!$H$5:$H$178,"Fail")</f>
         <v/>
       </c>
       <c r="E19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$177,$A19,'QA Checklist'!$H$5:$H$177,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$178,$A19,'QA Checklist'!$H$5:$H$178,"Pending")</f>
         <v/>
       </c>
       <c r="F19" s="8">
@@ -887,19 +887,19 @@
         </is>
       </c>
       <c r="B20" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$177,$A20)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$178,$A20)</f>
         <v/>
       </c>
       <c r="C20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$177,$A20,'QA Checklist'!$H$5:$H$177,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$177,$A20,'QA Checklist'!$H$5:$H$177,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$178,$A20,'QA Checklist'!$H$5:$H$178,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$178,$A20,'QA Checklist'!$H$5:$H$178,"Pass")</f>
         <v/>
       </c>
       <c r="D20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$177,$A20,'QA Checklist'!$H$5:$H$177,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$177,$A20,'QA Checklist'!$H$5:$H$177,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$178,$A20,'QA Checklist'!$H$5:$H$178,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$178,$A20,'QA Checklist'!$H$5:$H$178,"Fail")</f>
         <v/>
       </c>
       <c r="E20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$177,$A20,'QA Checklist'!$H$5:$H$177,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$178,$A20,'QA Checklist'!$H$5:$H$178,"Pending")</f>
         <v/>
       </c>
       <c r="F20" s="8">
@@ -914,19 +914,19 @@
         </is>
       </c>
       <c r="B21" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$177,$A21)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$178,$A21)</f>
         <v/>
       </c>
       <c r="C21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$177,$A21,'QA Checklist'!$H$5:$H$177,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$177,$A21,'QA Checklist'!$H$5:$H$177,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$178,$A21,'QA Checklist'!$H$5:$H$178,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$178,$A21,'QA Checklist'!$H$5:$H$178,"Pass")</f>
         <v/>
       </c>
       <c r="D21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$177,$A21,'QA Checklist'!$H$5:$H$177,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$177,$A21,'QA Checklist'!$H$5:$H$177,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$178,$A21,'QA Checklist'!$H$5:$H$178,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$178,$A21,'QA Checklist'!$H$5:$H$178,"Fail")</f>
         <v/>
       </c>
       <c r="E21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$177,$A21,'QA Checklist'!$H$5:$H$177,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$178,$A21,'QA Checklist'!$H$5:$H$178,"Pending")</f>
         <v/>
       </c>
       <c r="F21" s="8">
@@ -941,19 +941,19 @@
         </is>
       </c>
       <c r="B22" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$177,$A22)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$178,$A22)</f>
         <v/>
       </c>
       <c r="C22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$177,$A22,'QA Checklist'!$H$5:$H$177,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$177,$A22,'QA Checklist'!$H$5:$H$177,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$178,$A22,'QA Checklist'!$H$5:$H$178,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$178,$A22,'QA Checklist'!$H$5:$H$178,"Pass")</f>
         <v/>
       </c>
       <c r="D22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$177,$A22,'QA Checklist'!$H$5:$H$177,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$177,$A22,'QA Checklist'!$H$5:$H$177,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$178,$A22,'QA Checklist'!$H$5:$H$178,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$178,$A22,'QA Checklist'!$H$5:$H$178,"Fail")</f>
         <v/>
       </c>
       <c r="E22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$177,$A22,'QA Checklist'!$H$5:$H$177,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$178,$A22,'QA Checklist'!$H$5:$H$178,"Pending")</f>
         <v/>
       </c>
       <c r="F22" s="8">
@@ -1023,19 +1023,19 @@
         </is>
       </c>
       <c r="B26" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$177,$A26&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$178,$A26&amp;"*")</f>
         <v/>
       </c>
       <c r="C26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$177,$A26&amp;"*",'QA Checklist'!$H$5:$H$177,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$177,$A26&amp;"*",'QA Checklist'!$H$5:$H$177,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$178,$A26&amp;"*",'QA Checklist'!$H$5:$H$178,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$178,$A26&amp;"*",'QA Checklist'!$H$5:$H$178,"Pass")</f>
         <v/>
       </c>
       <c r="D26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$177,$A26&amp;"*",'QA Checklist'!$H$5:$H$177,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$177,$A26&amp;"*",'QA Checklist'!$H$5:$H$177,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$178,$A26&amp;"*",'QA Checklist'!$H$5:$H$178,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$178,$A26&amp;"*",'QA Checklist'!$H$5:$H$178,"Fail")</f>
         <v/>
       </c>
       <c r="E26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$177,$A26&amp;"*",'QA Checklist'!$H$5:$H$177,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$178,$A26&amp;"*",'QA Checklist'!$H$5:$H$178,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1046,19 +1046,19 @@
         </is>
       </c>
       <c r="B27" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$177,$A27&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$178,$A27&amp;"*")</f>
         <v/>
       </c>
       <c r="C27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$177,$A27&amp;"*",'QA Checklist'!$H$5:$H$177,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$177,$A27&amp;"*",'QA Checklist'!$H$5:$H$177,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$178,$A27&amp;"*",'QA Checklist'!$H$5:$H$178,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$178,$A27&amp;"*",'QA Checklist'!$H$5:$H$178,"Pass")</f>
         <v/>
       </c>
       <c r="D27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$177,$A27&amp;"*",'QA Checklist'!$H$5:$H$177,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$177,$A27&amp;"*",'QA Checklist'!$H$5:$H$177,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$178,$A27&amp;"*",'QA Checklist'!$H$5:$H$178,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$178,$A27&amp;"*",'QA Checklist'!$H$5:$H$178,"Fail")</f>
         <v/>
       </c>
       <c r="E27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$177,$A27&amp;"*",'QA Checklist'!$H$5:$H$177,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$178,$A27&amp;"*",'QA Checklist'!$H$5:$H$178,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1069,19 +1069,19 @@
         </is>
       </c>
       <c r="B28" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$177,$A28&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$178,$A28&amp;"*")</f>
         <v/>
       </c>
       <c r="C28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$177,$A28&amp;"*",'QA Checklist'!$H$5:$H$177,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$177,$A28&amp;"*",'QA Checklist'!$H$5:$H$177,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$178,$A28&amp;"*",'QA Checklist'!$H$5:$H$178,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$178,$A28&amp;"*",'QA Checklist'!$H$5:$H$178,"Pass")</f>
         <v/>
       </c>
       <c r="D28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$177,$A28&amp;"*",'QA Checklist'!$H$5:$H$177,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$177,$A28&amp;"*",'QA Checklist'!$H$5:$H$177,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$178,$A28&amp;"*",'QA Checklist'!$H$5:$H$178,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$178,$A28&amp;"*",'QA Checklist'!$H$5:$H$178,"Fail")</f>
         <v/>
       </c>
       <c r="E28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$177,$A28&amp;"*",'QA Checklist'!$H$5:$H$177,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$178,$A28&amp;"*",'QA Checklist'!$H$5:$H$178,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1096,7 +1096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I177"/>
+  <dimension ref="A1:I178"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8858,12 +8858,59 @@
         </is>
       </c>
     </row>
+    <row r="178">
+      <c r="A178" s="12" t="inlineStr">
+        <is>
+          <t>SA-52</t>
+        </is>
+      </c>
+      <c r="B178" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="C178" s="13" t="inlineStr">
+        <is>
+          <t>Tier 2 (Workflow &amp; Ergonomics)</t>
+        </is>
+      </c>
+      <c r="D178" s="13" t="inlineStr">
+        <is>
+          <t>Intake Paper / Claim Stub &amp; Referral Analytics</t>
+        </is>
+      </c>
+      <c r="E178" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="F178" s="13" t="inlineStr">
+        <is>
+          <t>Log in as SA, open 2025 RO Excel Studio &gt; Workshop_Monitoring, fill Customer, Contact, Plate, Model, Category, Concern and Referred By, leave Arrival on Auto (then set it manually), press Print Claim Stub and Register; log in as Owner / Admin and open Analytics</t>
+        </is>
+      </c>
+      <c r="G178" s="13" t="inlineStr">
+        <is>
+          <t>No Parts / Bay / Floor Status fields; Arrival follows the clock until edited; the printed paper shows all intake details, the 12-hour arrival, the referral source, reminders with RA 10173 consent, signatures and a tear-off gate pass; the Daily Intakes entry is Waiting with the arrival and referral; Analytics shows the referral channel counts and percentages for the selected period</t>
+        </is>
+      </c>
+      <c r="H178" s="14" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="I178" s="13" t="inlineStr">
+        <is>
+          <t>Verified by Automated Unit Tests (164 passing in tests/frontend/sla_and_logic.test.js AUT-FRONT-135), a backend end-to-end run on the local database and headless Chrome / PDF renders</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:I177"/>
+  <autoFilter ref="A4:I178"/>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="H5:H177">
+  <conditionalFormatting sqref="H5:H178">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$H5="Passed"</formula>
     </cfRule>
@@ -8880,13 +8927,13 @@
       <formula>$H5="Pending"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A5:A177">
+  <conditionalFormatting sqref="A5:A178">
     <cfRule type="expression" priority="6" dxfId="3">
-      <formula>COUNTIF($A$5:$A$177,$A5)&gt;1</formula>
+      <formula>COUNTIF($A$5:$A$178,$A5)&gt;1</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H5:H177" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H5:H178" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pending,Passed,Failed"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat(REV-177): remove Claim Stub printing from Workshop_Monitoring
Remove the Print Claim Stub button and printMonitoringClaimStub(); the
Register Repair Order button is full width again. Cache buster v=3.30,
AUT-FRONT-136, SA-53.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
+++ b/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
@@ -11,7 +11,7 @@
     <sheet name="QA Checklist" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$178</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$179</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'QA Checklist'!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTA('QA Checklist'!$A$5:$A$178)</f>
+        <f>COUNTA('QA Checklist'!$A$5:$A$179)</f>
         <v/>
       </c>
     </row>
@@ -594,7 +594,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$178,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$178,"Pass")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$179,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$179,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$178,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$178,"Fail")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$179,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$179,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -616,7 +616,7 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$178,"Pending")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$179,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -671,19 +671,19 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$178,$A12)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$179,$A12)</f>
         <v/>
       </c>
       <c r="C12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$178,$A12,'QA Checklist'!$H$5:$H$178,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$178,$A12,'QA Checklist'!$H$5:$H$178,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$179,$A12,'QA Checklist'!$H$5:$H$179,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$179,$A12,'QA Checklist'!$H$5:$H$179,"Pass")</f>
         <v/>
       </c>
       <c r="D12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$178,$A12,'QA Checklist'!$H$5:$H$178,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$178,$A12,'QA Checklist'!$H$5:$H$178,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$179,$A12,'QA Checklist'!$H$5:$H$179,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$179,$A12,'QA Checklist'!$H$5:$H$179,"Fail")</f>
         <v/>
       </c>
       <c r="E12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$178,$A12,'QA Checklist'!$H$5:$H$178,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$179,$A12,'QA Checklist'!$H$5:$H$179,"Pending")</f>
         <v/>
       </c>
       <c r="F12" s="8">
@@ -698,19 +698,19 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$178,$A13)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$179,$A13)</f>
         <v/>
       </c>
       <c r="C13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$178,$A13,'QA Checklist'!$H$5:$H$178,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$178,$A13,'QA Checklist'!$H$5:$H$178,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$179,$A13,'QA Checklist'!$H$5:$H$179,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$179,$A13,'QA Checklist'!$H$5:$H$179,"Pass")</f>
         <v/>
       </c>
       <c r="D13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$178,$A13,'QA Checklist'!$H$5:$H$178,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$178,$A13,'QA Checklist'!$H$5:$H$178,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$179,$A13,'QA Checklist'!$H$5:$H$179,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$179,$A13,'QA Checklist'!$H$5:$H$179,"Fail")</f>
         <v/>
       </c>
       <c r="E13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$178,$A13,'QA Checklist'!$H$5:$H$178,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$179,$A13,'QA Checklist'!$H$5:$H$179,"Pending")</f>
         <v/>
       </c>
       <c r="F13" s="8">
@@ -725,19 +725,19 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$178,$A14)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$179,$A14)</f>
         <v/>
       </c>
       <c r="C14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$178,$A14,'QA Checklist'!$H$5:$H$178,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$178,$A14,'QA Checklist'!$H$5:$H$178,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$179,$A14,'QA Checklist'!$H$5:$H$179,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$179,$A14,'QA Checklist'!$H$5:$H$179,"Pass")</f>
         <v/>
       </c>
       <c r="D14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$178,$A14,'QA Checklist'!$H$5:$H$178,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$178,$A14,'QA Checklist'!$H$5:$H$178,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$179,$A14,'QA Checklist'!$H$5:$H$179,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$179,$A14,'QA Checklist'!$H$5:$H$179,"Fail")</f>
         <v/>
       </c>
       <c r="E14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$178,$A14,'QA Checklist'!$H$5:$H$178,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$179,$A14,'QA Checklist'!$H$5:$H$179,"Pending")</f>
         <v/>
       </c>
       <c r="F14" s="8">
@@ -752,19 +752,19 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$178,$A15)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$179,$A15)</f>
         <v/>
       </c>
       <c r="C15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$178,$A15,'QA Checklist'!$H$5:$H$178,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$178,$A15,'QA Checklist'!$H$5:$H$178,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$179,$A15,'QA Checklist'!$H$5:$H$179,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$179,$A15,'QA Checklist'!$H$5:$H$179,"Pass")</f>
         <v/>
       </c>
       <c r="D15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$178,$A15,'QA Checklist'!$H$5:$H$178,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$178,$A15,'QA Checklist'!$H$5:$H$178,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$179,$A15,'QA Checklist'!$H$5:$H$179,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$179,$A15,'QA Checklist'!$H$5:$H$179,"Fail")</f>
         <v/>
       </c>
       <c r="E15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$178,$A15,'QA Checklist'!$H$5:$H$178,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$179,$A15,'QA Checklist'!$H$5:$H$179,"Pending")</f>
         <v/>
       </c>
       <c r="F15" s="8">
@@ -779,19 +779,19 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$178,$A16)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$179,$A16)</f>
         <v/>
       </c>
       <c r="C16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$178,$A16,'QA Checklist'!$H$5:$H$178,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$178,$A16,'QA Checklist'!$H$5:$H$178,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$179,$A16,'QA Checklist'!$H$5:$H$179,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$179,$A16,'QA Checklist'!$H$5:$H$179,"Pass")</f>
         <v/>
       </c>
       <c r="D16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$178,$A16,'QA Checklist'!$H$5:$H$178,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$178,$A16,'QA Checklist'!$H$5:$H$178,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$179,$A16,'QA Checklist'!$H$5:$H$179,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$179,$A16,'QA Checklist'!$H$5:$H$179,"Fail")</f>
         <v/>
       </c>
       <c r="E16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$178,$A16,'QA Checklist'!$H$5:$H$178,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$179,$A16,'QA Checklist'!$H$5:$H$179,"Pending")</f>
         <v/>
       </c>
       <c r="F16" s="8">
@@ -806,19 +806,19 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$178,$A17)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$179,$A17)</f>
         <v/>
       </c>
       <c r="C17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$178,$A17,'QA Checklist'!$H$5:$H$178,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$178,$A17,'QA Checklist'!$H$5:$H$178,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$179,$A17,'QA Checklist'!$H$5:$H$179,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$179,$A17,'QA Checklist'!$H$5:$H$179,"Pass")</f>
         <v/>
       </c>
       <c r="D17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$178,$A17,'QA Checklist'!$H$5:$H$178,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$178,$A17,'QA Checklist'!$H$5:$H$178,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$179,$A17,'QA Checklist'!$H$5:$H$179,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$179,$A17,'QA Checklist'!$H$5:$H$179,"Fail")</f>
         <v/>
       </c>
       <c r="E17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$178,$A17,'QA Checklist'!$H$5:$H$178,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$179,$A17,'QA Checklist'!$H$5:$H$179,"Pending")</f>
         <v/>
       </c>
       <c r="F17" s="8">
@@ -833,19 +833,19 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$178,$A18)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$179,$A18)</f>
         <v/>
       </c>
       <c r="C18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$178,$A18,'QA Checklist'!$H$5:$H$178,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$178,$A18,'QA Checklist'!$H$5:$H$178,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$179,$A18,'QA Checklist'!$H$5:$H$179,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$179,$A18,'QA Checklist'!$H$5:$H$179,"Pass")</f>
         <v/>
       </c>
       <c r="D18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$178,$A18,'QA Checklist'!$H$5:$H$178,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$178,$A18,'QA Checklist'!$H$5:$H$178,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$179,$A18,'QA Checklist'!$H$5:$H$179,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$179,$A18,'QA Checklist'!$H$5:$H$179,"Fail")</f>
         <v/>
       </c>
       <c r="E18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$178,$A18,'QA Checklist'!$H$5:$H$178,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$179,$A18,'QA Checklist'!$H$5:$H$179,"Pending")</f>
         <v/>
       </c>
       <c r="F18" s="8">
@@ -860,19 +860,19 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$178,$A19)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$179,$A19)</f>
         <v/>
       </c>
       <c r="C19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$178,$A19,'QA Checklist'!$H$5:$H$178,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$178,$A19,'QA Checklist'!$H$5:$H$178,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$179,$A19,'QA Checklist'!$H$5:$H$179,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$179,$A19,'QA Checklist'!$H$5:$H$179,"Pass")</f>
         <v/>
       </c>
       <c r="D19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$178,$A19,'QA Checklist'!$H$5:$H$178,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$178,$A19,'QA Checklist'!$H$5:$H$178,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$179,$A19,'QA Checklist'!$H$5:$H$179,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$179,$A19,'QA Checklist'!$H$5:$H$179,"Fail")</f>
         <v/>
       </c>
       <c r="E19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$178,$A19,'QA Checklist'!$H$5:$H$178,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$179,$A19,'QA Checklist'!$H$5:$H$179,"Pending")</f>
         <v/>
       </c>
       <c r="F19" s="8">
@@ -887,19 +887,19 @@
         </is>
       </c>
       <c r="B20" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$178,$A20)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$179,$A20)</f>
         <v/>
       </c>
       <c r="C20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$178,$A20,'QA Checklist'!$H$5:$H$178,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$178,$A20,'QA Checklist'!$H$5:$H$178,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$179,$A20,'QA Checklist'!$H$5:$H$179,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$179,$A20,'QA Checklist'!$H$5:$H$179,"Pass")</f>
         <v/>
       </c>
       <c r="D20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$178,$A20,'QA Checklist'!$H$5:$H$178,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$178,$A20,'QA Checklist'!$H$5:$H$178,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$179,$A20,'QA Checklist'!$H$5:$H$179,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$179,$A20,'QA Checklist'!$H$5:$H$179,"Fail")</f>
         <v/>
       </c>
       <c r="E20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$178,$A20,'QA Checklist'!$H$5:$H$178,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$179,$A20,'QA Checklist'!$H$5:$H$179,"Pending")</f>
         <v/>
       </c>
       <c r="F20" s="8">
@@ -914,19 +914,19 @@
         </is>
       </c>
       <c r="B21" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$178,$A21)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$179,$A21)</f>
         <v/>
       </c>
       <c r="C21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$178,$A21,'QA Checklist'!$H$5:$H$178,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$178,$A21,'QA Checklist'!$H$5:$H$178,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$179,$A21,'QA Checklist'!$H$5:$H$179,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$179,$A21,'QA Checklist'!$H$5:$H$179,"Pass")</f>
         <v/>
       </c>
       <c r="D21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$178,$A21,'QA Checklist'!$H$5:$H$178,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$178,$A21,'QA Checklist'!$H$5:$H$178,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$179,$A21,'QA Checklist'!$H$5:$H$179,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$179,$A21,'QA Checklist'!$H$5:$H$179,"Fail")</f>
         <v/>
       </c>
       <c r="E21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$178,$A21,'QA Checklist'!$H$5:$H$178,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$179,$A21,'QA Checklist'!$H$5:$H$179,"Pending")</f>
         <v/>
       </c>
       <c r="F21" s="8">
@@ -941,19 +941,19 @@
         </is>
       </c>
       <c r="B22" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$178,$A22)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$179,$A22)</f>
         <v/>
       </c>
       <c r="C22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$178,$A22,'QA Checklist'!$H$5:$H$178,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$178,$A22,'QA Checklist'!$H$5:$H$178,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$179,$A22,'QA Checklist'!$H$5:$H$179,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$179,$A22,'QA Checklist'!$H$5:$H$179,"Pass")</f>
         <v/>
       </c>
       <c r="D22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$178,$A22,'QA Checklist'!$H$5:$H$178,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$178,$A22,'QA Checklist'!$H$5:$H$178,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$179,$A22,'QA Checklist'!$H$5:$H$179,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$179,$A22,'QA Checklist'!$H$5:$H$179,"Fail")</f>
         <v/>
       </c>
       <c r="E22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$178,$A22,'QA Checklist'!$H$5:$H$178,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$179,$A22,'QA Checklist'!$H$5:$H$179,"Pending")</f>
         <v/>
       </c>
       <c r="F22" s="8">
@@ -1023,19 +1023,19 @@
         </is>
       </c>
       <c r="B26" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$178,$A26&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$179,$A26&amp;"*")</f>
         <v/>
       </c>
       <c r="C26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$178,$A26&amp;"*",'QA Checklist'!$H$5:$H$178,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$178,$A26&amp;"*",'QA Checklist'!$H$5:$H$178,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$179,$A26&amp;"*",'QA Checklist'!$H$5:$H$179,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$179,$A26&amp;"*",'QA Checklist'!$H$5:$H$179,"Pass")</f>
         <v/>
       </c>
       <c r="D26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$178,$A26&amp;"*",'QA Checklist'!$H$5:$H$178,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$178,$A26&amp;"*",'QA Checklist'!$H$5:$H$178,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$179,$A26&amp;"*",'QA Checklist'!$H$5:$H$179,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$179,$A26&amp;"*",'QA Checklist'!$H$5:$H$179,"Fail")</f>
         <v/>
       </c>
       <c r="E26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$178,$A26&amp;"*",'QA Checklist'!$H$5:$H$178,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$179,$A26&amp;"*",'QA Checklist'!$H$5:$H$179,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1046,19 +1046,19 @@
         </is>
       </c>
       <c r="B27" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$178,$A27&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$179,$A27&amp;"*")</f>
         <v/>
       </c>
       <c r="C27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$178,$A27&amp;"*",'QA Checklist'!$H$5:$H$178,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$178,$A27&amp;"*",'QA Checklist'!$H$5:$H$178,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$179,$A27&amp;"*",'QA Checklist'!$H$5:$H$179,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$179,$A27&amp;"*",'QA Checklist'!$H$5:$H$179,"Pass")</f>
         <v/>
       </c>
       <c r="D27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$178,$A27&amp;"*",'QA Checklist'!$H$5:$H$178,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$178,$A27&amp;"*",'QA Checklist'!$H$5:$H$178,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$179,$A27&amp;"*",'QA Checklist'!$H$5:$H$179,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$179,$A27&amp;"*",'QA Checklist'!$H$5:$H$179,"Fail")</f>
         <v/>
       </c>
       <c r="E27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$178,$A27&amp;"*",'QA Checklist'!$H$5:$H$178,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$179,$A27&amp;"*",'QA Checklist'!$H$5:$H$179,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1069,19 +1069,19 @@
         </is>
       </c>
       <c r="B28" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$178,$A28&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$179,$A28&amp;"*")</f>
         <v/>
       </c>
       <c r="C28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$178,$A28&amp;"*",'QA Checklist'!$H$5:$H$178,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$178,$A28&amp;"*",'QA Checklist'!$H$5:$H$178,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$179,$A28&amp;"*",'QA Checklist'!$H$5:$H$179,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$179,$A28&amp;"*",'QA Checklist'!$H$5:$H$179,"Pass")</f>
         <v/>
       </c>
       <c r="D28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$178,$A28&amp;"*",'QA Checklist'!$H$5:$H$178,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$178,$A28&amp;"*",'QA Checklist'!$H$5:$H$178,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$179,$A28&amp;"*",'QA Checklist'!$H$5:$H$179,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$179,$A28&amp;"*",'QA Checklist'!$H$5:$H$179,"Fail")</f>
         <v/>
       </c>
       <c r="E28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$178,$A28&amp;"*",'QA Checklist'!$H$5:$H$178,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$179,$A28&amp;"*",'QA Checklist'!$H$5:$H$179,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1096,7 +1096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I178"/>
+  <dimension ref="A1:I179"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8905,12 +8905,59 @@
         </is>
       </c>
     </row>
+    <row r="179">
+      <c r="A179" s="12" t="inlineStr">
+        <is>
+          <t>SA-53</t>
+        </is>
+      </c>
+      <c r="B179" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="C179" s="13" t="inlineStr">
+        <is>
+          <t>Tier 2 (Workflow &amp; Ergonomics)</t>
+        </is>
+      </c>
+      <c r="D179" s="13" t="inlineStr">
+        <is>
+          <t>Workshop_Monitoring Without Claim Stub Printing</t>
+        </is>
+      </c>
+      <c r="E179" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="F179" s="13" t="inlineStr">
+        <is>
+          <t>Log in as Service Advisor, open 2025 RO Excel Studio &gt; Workshop_Monitoring and look at the buttons at the bottom of the card</t>
+        </is>
+      </c>
+      <c r="G179" s="13" t="inlineStr">
+        <is>
+          <t>Only the full-width Register Repair Order to System button is shown; there is no Print Claim Stub button; the Claim Stub ID field is still auto-filled</t>
+        </is>
+      </c>
+      <c r="H179" s="14" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="I179" s="13" t="inlineStr">
+        <is>
+          <t>Verified by Automated Unit Tests (165 passing in tests/frontend/sla_and_logic.test.js AUT-FRONT-136) and a headless Chrome card render</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:I178"/>
+  <autoFilter ref="A4:I179"/>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="H5:H178">
+  <conditionalFormatting sqref="H5:H179">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$H5="Passed"</formula>
     </cfRule>
@@ -8927,13 +8974,13 @@
       <formula>$H5="Pending"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A5:A178">
+  <conditionalFormatting sqref="A5:A179">
     <cfRule type="expression" priority="6" dxfId="3">
-      <formula>COUNTIF($A$5:$A$178,$A5)&gt;1</formula>
+      <formula>COUNTIF($A$5:$A$179,$A5)&gt;1</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H5:H178" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H5:H179" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pending,Passed,Failed"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
fix(REV-178): center the studio PDF page in Maximize / Normal View
applyStudioAspectFit() now centers the fitted PDF iframe in its container,
so the maximized view shows the page in the middle instead of pinned to
the left. No new tab is opened. Cache buster v=3.31, AUT-FRONT-137, SA-54.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
+++ b/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
@@ -11,7 +11,7 @@
     <sheet name="QA Checklist" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$179</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$180</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'QA Checklist'!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTA('QA Checklist'!$A$5:$A$179)</f>
+        <f>COUNTA('QA Checklist'!$A$5:$A$180)</f>
         <v/>
       </c>
     </row>
@@ -594,7 +594,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$179,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$179,"Pass")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$180,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$180,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$179,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$179,"Fail")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$180,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$180,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -616,7 +616,7 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$179,"Pending")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$180,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -671,19 +671,19 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$179,$A12)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$180,$A12)</f>
         <v/>
       </c>
       <c r="C12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$179,$A12,'QA Checklist'!$H$5:$H$179,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$179,$A12,'QA Checklist'!$H$5:$H$179,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$180,$A12,'QA Checklist'!$H$5:$H$180,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$180,$A12,'QA Checklist'!$H$5:$H$180,"Pass")</f>
         <v/>
       </c>
       <c r="D12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$179,$A12,'QA Checklist'!$H$5:$H$179,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$179,$A12,'QA Checklist'!$H$5:$H$179,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$180,$A12,'QA Checklist'!$H$5:$H$180,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$180,$A12,'QA Checklist'!$H$5:$H$180,"Fail")</f>
         <v/>
       </c>
       <c r="E12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$179,$A12,'QA Checklist'!$H$5:$H$179,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$180,$A12,'QA Checklist'!$H$5:$H$180,"Pending")</f>
         <v/>
       </c>
       <c r="F12" s="8">
@@ -698,19 +698,19 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$179,$A13)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$180,$A13)</f>
         <v/>
       </c>
       <c r="C13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$179,$A13,'QA Checklist'!$H$5:$H$179,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$179,$A13,'QA Checklist'!$H$5:$H$179,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$180,$A13,'QA Checklist'!$H$5:$H$180,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$180,$A13,'QA Checklist'!$H$5:$H$180,"Pass")</f>
         <v/>
       </c>
       <c r="D13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$179,$A13,'QA Checklist'!$H$5:$H$179,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$179,$A13,'QA Checklist'!$H$5:$H$179,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$180,$A13,'QA Checklist'!$H$5:$H$180,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$180,$A13,'QA Checklist'!$H$5:$H$180,"Fail")</f>
         <v/>
       </c>
       <c r="E13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$179,$A13,'QA Checklist'!$H$5:$H$179,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$180,$A13,'QA Checklist'!$H$5:$H$180,"Pending")</f>
         <v/>
       </c>
       <c r="F13" s="8">
@@ -725,19 +725,19 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$179,$A14)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$180,$A14)</f>
         <v/>
       </c>
       <c r="C14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$179,$A14,'QA Checklist'!$H$5:$H$179,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$179,$A14,'QA Checklist'!$H$5:$H$179,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$180,$A14,'QA Checklist'!$H$5:$H$180,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$180,$A14,'QA Checklist'!$H$5:$H$180,"Pass")</f>
         <v/>
       </c>
       <c r="D14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$179,$A14,'QA Checklist'!$H$5:$H$179,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$179,$A14,'QA Checklist'!$H$5:$H$179,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$180,$A14,'QA Checklist'!$H$5:$H$180,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$180,$A14,'QA Checklist'!$H$5:$H$180,"Fail")</f>
         <v/>
       </c>
       <c r="E14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$179,$A14,'QA Checklist'!$H$5:$H$179,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$180,$A14,'QA Checklist'!$H$5:$H$180,"Pending")</f>
         <v/>
       </c>
       <c r="F14" s="8">
@@ -752,19 +752,19 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$179,$A15)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$180,$A15)</f>
         <v/>
       </c>
       <c r="C15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$179,$A15,'QA Checklist'!$H$5:$H$179,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$179,$A15,'QA Checklist'!$H$5:$H$179,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$180,$A15,'QA Checklist'!$H$5:$H$180,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$180,$A15,'QA Checklist'!$H$5:$H$180,"Pass")</f>
         <v/>
       </c>
       <c r="D15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$179,$A15,'QA Checklist'!$H$5:$H$179,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$179,$A15,'QA Checklist'!$H$5:$H$179,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$180,$A15,'QA Checklist'!$H$5:$H$180,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$180,$A15,'QA Checklist'!$H$5:$H$180,"Fail")</f>
         <v/>
       </c>
       <c r="E15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$179,$A15,'QA Checklist'!$H$5:$H$179,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$180,$A15,'QA Checklist'!$H$5:$H$180,"Pending")</f>
         <v/>
       </c>
       <c r="F15" s="8">
@@ -779,19 +779,19 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$179,$A16)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$180,$A16)</f>
         <v/>
       </c>
       <c r="C16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$179,$A16,'QA Checklist'!$H$5:$H$179,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$179,$A16,'QA Checklist'!$H$5:$H$179,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$180,$A16,'QA Checklist'!$H$5:$H$180,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$180,$A16,'QA Checklist'!$H$5:$H$180,"Pass")</f>
         <v/>
       </c>
       <c r="D16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$179,$A16,'QA Checklist'!$H$5:$H$179,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$179,$A16,'QA Checklist'!$H$5:$H$179,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$180,$A16,'QA Checklist'!$H$5:$H$180,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$180,$A16,'QA Checklist'!$H$5:$H$180,"Fail")</f>
         <v/>
       </c>
       <c r="E16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$179,$A16,'QA Checklist'!$H$5:$H$179,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$180,$A16,'QA Checklist'!$H$5:$H$180,"Pending")</f>
         <v/>
       </c>
       <c r="F16" s="8">
@@ -806,19 +806,19 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$179,$A17)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$180,$A17)</f>
         <v/>
       </c>
       <c r="C17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$179,$A17,'QA Checklist'!$H$5:$H$179,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$179,$A17,'QA Checklist'!$H$5:$H$179,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$180,$A17,'QA Checklist'!$H$5:$H$180,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$180,$A17,'QA Checklist'!$H$5:$H$180,"Pass")</f>
         <v/>
       </c>
       <c r="D17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$179,$A17,'QA Checklist'!$H$5:$H$179,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$179,$A17,'QA Checklist'!$H$5:$H$179,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$180,$A17,'QA Checklist'!$H$5:$H$180,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$180,$A17,'QA Checklist'!$H$5:$H$180,"Fail")</f>
         <v/>
       </c>
       <c r="E17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$179,$A17,'QA Checklist'!$H$5:$H$179,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$180,$A17,'QA Checklist'!$H$5:$H$180,"Pending")</f>
         <v/>
       </c>
       <c r="F17" s="8">
@@ -833,19 +833,19 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$179,$A18)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$180,$A18)</f>
         <v/>
       </c>
       <c r="C18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$179,$A18,'QA Checklist'!$H$5:$H$179,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$179,$A18,'QA Checklist'!$H$5:$H$179,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$180,$A18,'QA Checklist'!$H$5:$H$180,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$180,$A18,'QA Checklist'!$H$5:$H$180,"Pass")</f>
         <v/>
       </c>
       <c r="D18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$179,$A18,'QA Checklist'!$H$5:$H$179,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$179,$A18,'QA Checklist'!$H$5:$H$179,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$180,$A18,'QA Checklist'!$H$5:$H$180,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$180,$A18,'QA Checklist'!$H$5:$H$180,"Fail")</f>
         <v/>
       </c>
       <c r="E18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$179,$A18,'QA Checklist'!$H$5:$H$179,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$180,$A18,'QA Checklist'!$H$5:$H$180,"Pending")</f>
         <v/>
       </c>
       <c r="F18" s="8">
@@ -860,19 +860,19 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$179,$A19)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$180,$A19)</f>
         <v/>
       </c>
       <c r="C19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$179,$A19,'QA Checklist'!$H$5:$H$179,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$179,$A19,'QA Checklist'!$H$5:$H$179,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$180,$A19,'QA Checklist'!$H$5:$H$180,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$180,$A19,'QA Checklist'!$H$5:$H$180,"Pass")</f>
         <v/>
       </c>
       <c r="D19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$179,$A19,'QA Checklist'!$H$5:$H$179,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$179,$A19,'QA Checklist'!$H$5:$H$179,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$180,$A19,'QA Checklist'!$H$5:$H$180,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$180,$A19,'QA Checklist'!$H$5:$H$180,"Fail")</f>
         <v/>
       </c>
       <c r="E19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$179,$A19,'QA Checklist'!$H$5:$H$179,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$180,$A19,'QA Checklist'!$H$5:$H$180,"Pending")</f>
         <v/>
       </c>
       <c r="F19" s="8">
@@ -887,19 +887,19 @@
         </is>
       </c>
       <c r="B20" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$179,$A20)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$180,$A20)</f>
         <v/>
       </c>
       <c r="C20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$179,$A20,'QA Checklist'!$H$5:$H$179,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$179,$A20,'QA Checklist'!$H$5:$H$179,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$180,$A20,'QA Checklist'!$H$5:$H$180,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$180,$A20,'QA Checklist'!$H$5:$H$180,"Pass")</f>
         <v/>
       </c>
       <c r="D20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$179,$A20,'QA Checklist'!$H$5:$H$179,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$179,$A20,'QA Checklist'!$H$5:$H$179,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$180,$A20,'QA Checklist'!$H$5:$H$180,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$180,$A20,'QA Checklist'!$H$5:$H$180,"Fail")</f>
         <v/>
       </c>
       <c r="E20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$179,$A20,'QA Checklist'!$H$5:$H$179,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$180,$A20,'QA Checklist'!$H$5:$H$180,"Pending")</f>
         <v/>
       </c>
       <c r="F20" s="8">
@@ -914,19 +914,19 @@
         </is>
       </c>
       <c r="B21" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$179,$A21)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$180,$A21)</f>
         <v/>
       </c>
       <c r="C21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$179,$A21,'QA Checklist'!$H$5:$H$179,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$179,$A21,'QA Checklist'!$H$5:$H$179,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$180,$A21,'QA Checklist'!$H$5:$H$180,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$180,$A21,'QA Checklist'!$H$5:$H$180,"Pass")</f>
         <v/>
       </c>
       <c r="D21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$179,$A21,'QA Checklist'!$H$5:$H$179,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$179,$A21,'QA Checklist'!$H$5:$H$179,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$180,$A21,'QA Checklist'!$H$5:$H$180,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$180,$A21,'QA Checklist'!$H$5:$H$180,"Fail")</f>
         <v/>
       </c>
       <c r="E21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$179,$A21,'QA Checklist'!$H$5:$H$179,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$180,$A21,'QA Checklist'!$H$5:$H$180,"Pending")</f>
         <v/>
       </c>
       <c r="F21" s="8">
@@ -941,19 +941,19 @@
         </is>
       </c>
       <c r="B22" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$179,$A22)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$180,$A22)</f>
         <v/>
       </c>
       <c r="C22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$179,$A22,'QA Checklist'!$H$5:$H$179,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$179,$A22,'QA Checklist'!$H$5:$H$179,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$180,$A22,'QA Checklist'!$H$5:$H$180,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$180,$A22,'QA Checklist'!$H$5:$H$180,"Pass")</f>
         <v/>
       </c>
       <c r="D22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$179,$A22,'QA Checklist'!$H$5:$H$179,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$179,$A22,'QA Checklist'!$H$5:$H$179,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$180,$A22,'QA Checklist'!$H$5:$H$180,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$180,$A22,'QA Checklist'!$H$5:$H$180,"Fail")</f>
         <v/>
       </c>
       <c r="E22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$179,$A22,'QA Checklist'!$H$5:$H$179,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$180,$A22,'QA Checklist'!$H$5:$H$180,"Pending")</f>
         <v/>
       </c>
       <c r="F22" s="8">
@@ -1023,19 +1023,19 @@
         </is>
       </c>
       <c r="B26" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$179,$A26&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$180,$A26&amp;"*")</f>
         <v/>
       </c>
       <c r="C26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$179,$A26&amp;"*",'QA Checklist'!$H$5:$H$179,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$179,$A26&amp;"*",'QA Checklist'!$H$5:$H$179,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$180,$A26&amp;"*",'QA Checklist'!$H$5:$H$180,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$180,$A26&amp;"*",'QA Checklist'!$H$5:$H$180,"Pass")</f>
         <v/>
       </c>
       <c r="D26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$179,$A26&amp;"*",'QA Checklist'!$H$5:$H$179,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$179,$A26&amp;"*",'QA Checklist'!$H$5:$H$179,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$180,$A26&amp;"*",'QA Checklist'!$H$5:$H$180,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$180,$A26&amp;"*",'QA Checklist'!$H$5:$H$180,"Fail")</f>
         <v/>
       </c>
       <c r="E26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$179,$A26&amp;"*",'QA Checklist'!$H$5:$H$179,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$180,$A26&amp;"*",'QA Checklist'!$H$5:$H$180,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1046,19 +1046,19 @@
         </is>
       </c>
       <c r="B27" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$179,$A27&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$180,$A27&amp;"*")</f>
         <v/>
       </c>
       <c r="C27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$179,$A27&amp;"*",'QA Checklist'!$H$5:$H$179,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$179,$A27&amp;"*",'QA Checklist'!$H$5:$H$179,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$180,$A27&amp;"*",'QA Checklist'!$H$5:$H$180,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$180,$A27&amp;"*",'QA Checklist'!$H$5:$H$180,"Pass")</f>
         <v/>
       </c>
       <c r="D27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$179,$A27&amp;"*",'QA Checklist'!$H$5:$H$179,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$179,$A27&amp;"*",'QA Checklist'!$H$5:$H$179,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$180,$A27&amp;"*",'QA Checklist'!$H$5:$H$180,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$180,$A27&amp;"*",'QA Checklist'!$H$5:$H$180,"Fail")</f>
         <v/>
       </c>
       <c r="E27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$179,$A27&amp;"*",'QA Checklist'!$H$5:$H$179,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$180,$A27&amp;"*",'QA Checklist'!$H$5:$H$180,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1069,19 +1069,19 @@
         </is>
       </c>
       <c r="B28" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$179,$A28&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$180,$A28&amp;"*")</f>
         <v/>
       </c>
       <c r="C28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$179,$A28&amp;"*",'QA Checklist'!$H$5:$H$179,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$179,$A28&amp;"*",'QA Checklist'!$H$5:$H$179,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$180,$A28&amp;"*",'QA Checklist'!$H$5:$H$180,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$180,$A28&amp;"*",'QA Checklist'!$H$5:$H$180,"Pass")</f>
         <v/>
       </c>
       <c r="D28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$179,$A28&amp;"*",'QA Checklist'!$H$5:$H$179,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$179,$A28&amp;"*",'QA Checklist'!$H$5:$H$179,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$180,$A28&amp;"*",'QA Checklist'!$H$5:$H$180,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$180,$A28&amp;"*",'QA Checklist'!$H$5:$H$180,"Fail")</f>
         <v/>
       </c>
       <c r="E28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$179,$A28&amp;"*",'QA Checklist'!$H$5:$H$179,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$180,$A28&amp;"*",'QA Checklist'!$H$5:$H$180,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1096,7 +1096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I179"/>
+  <dimension ref="A1:I180"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8952,12 +8952,59 @@
         </is>
       </c>
     </row>
+    <row r="180">
+      <c r="A180" s="12" t="inlineStr">
+        <is>
+          <t>SA-54</t>
+        </is>
+      </c>
+      <c r="B180" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="C180" s="13" t="inlineStr">
+        <is>
+          <t>Tier 2 (Workflow &amp; Ergonomics)</t>
+        </is>
+      </c>
+      <c r="D180" s="13" t="inlineStr">
+        <is>
+          <t>Centered PDF in Maximized Studio View</t>
+        </is>
+      </c>
+      <c r="E180" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="F180" s="13" t="inlineStr">
+        <is>
+          <t>Log in as Service Advisor, open 2025 RO Excel Studio, press Maximize PDF on each tab (Job_Order, Quotation_No, Billing_No, CheckList_Result), then press Normal View</t>
+        </is>
+      </c>
+      <c r="G180" s="13" t="inlineStr">
+        <is>
+          <t>In the maximized view the PDF page is centered in the pane, no new browser tab opens, and Normal View returns to the side-by-side layout with the page still centered</t>
+        </is>
+      </c>
+      <c r="H180" s="14" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="I180" s="13" t="inlineStr">
+        <is>
+          <t>Verified by Automated Unit Tests (166 passing in tests/frontend/sla_and_logic.test.js AUT-FRONT-137) and a headless Chrome centering check</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:I179"/>
+  <autoFilter ref="A4:I180"/>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="H5:H179">
+  <conditionalFormatting sqref="H5:H180">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$H5="Passed"</formula>
     </cfRule>
@@ -8974,13 +9021,13 @@
       <formula>$H5="Pending"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A5:A179">
+  <conditionalFormatting sqref="A5:A180">
     <cfRule type="expression" priority="6" dxfId="3">
-      <formula>COUNTIF($A$5:$A$179,$A5)&gt;1</formula>
+      <formula>COUNTIF($A$5:$A$180,$A5)&gt;1</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H5:H179" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H5:H180" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pending,Passed,Failed"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
fix(REV-179): stop maximized studio PDF from shrinking to a thumbnail
The Maximize toggle measured the pane before the Tailwind CDN applied
xl:col-span-12 (one grid column, ~94px), fitting the PDF to that width.
Drop the immediate re-fit and redraw the visible sheet's PDF from a
ResizeObserver once the container has its real size.
Cache buster v=3.32, AUT-FRONT-138, SA-55.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
+++ b/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
@@ -11,7 +11,7 @@
     <sheet name="QA Checklist" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$180</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$181</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'QA Checklist'!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTA('QA Checklist'!$A$5:$A$180)</f>
+        <f>COUNTA('QA Checklist'!$A$5:$A$181)</f>
         <v/>
       </c>
     </row>
@@ -594,7 +594,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$180,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$180,"Pass")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$181,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$181,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$180,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$180,"Fail")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$181,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$181,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -616,7 +616,7 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$180,"Pending")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$181,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -671,19 +671,19 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$180,$A12)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$181,$A12)</f>
         <v/>
       </c>
       <c r="C12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$180,$A12,'QA Checklist'!$H$5:$H$180,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$180,$A12,'QA Checklist'!$H$5:$H$180,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$181,$A12,'QA Checklist'!$H$5:$H$181,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$181,$A12,'QA Checklist'!$H$5:$H$181,"Pass")</f>
         <v/>
       </c>
       <c r="D12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$180,$A12,'QA Checklist'!$H$5:$H$180,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$180,$A12,'QA Checklist'!$H$5:$H$180,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$181,$A12,'QA Checklist'!$H$5:$H$181,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$181,$A12,'QA Checklist'!$H$5:$H$181,"Fail")</f>
         <v/>
       </c>
       <c r="E12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$180,$A12,'QA Checklist'!$H$5:$H$180,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$181,$A12,'QA Checklist'!$H$5:$H$181,"Pending")</f>
         <v/>
       </c>
       <c r="F12" s="8">
@@ -698,19 +698,19 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$180,$A13)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$181,$A13)</f>
         <v/>
       </c>
       <c r="C13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$180,$A13,'QA Checklist'!$H$5:$H$180,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$180,$A13,'QA Checklist'!$H$5:$H$180,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$181,$A13,'QA Checklist'!$H$5:$H$181,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$181,$A13,'QA Checklist'!$H$5:$H$181,"Pass")</f>
         <v/>
       </c>
       <c r="D13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$180,$A13,'QA Checklist'!$H$5:$H$180,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$180,$A13,'QA Checklist'!$H$5:$H$180,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$181,$A13,'QA Checklist'!$H$5:$H$181,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$181,$A13,'QA Checklist'!$H$5:$H$181,"Fail")</f>
         <v/>
       </c>
       <c r="E13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$180,$A13,'QA Checklist'!$H$5:$H$180,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$181,$A13,'QA Checklist'!$H$5:$H$181,"Pending")</f>
         <v/>
       </c>
       <c r="F13" s="8">
@@ -725,19 +725,19 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$180,$A14)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$181,$A14)</f>
         <v/>
       </c>
       <c r="C14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$180,$A14,'QA Checklist'!$H$5:$H$180,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$180,$A14,'QA Checklist'!$H$5:$H$180,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$181,$A14,'QA Checklist'!$H$5:$H$181,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$181,$A14,'QA Checklist'!$H$5:$H$181,"Pass")</f>
         <v/>
       </c>
       <c r="D14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$180,$A14,'QA Checklist'!$H$5:$H$180,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$180,$A14,'QA Checklist'!$H$5:$H$180,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$181,$A14,'QA Checklist'!$H$5:$H$181,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$181,$A14,'QA Checklist'!$H$5:$H$181,"Fail")</f>
         <v/>
       </c>
       <c r="E14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$180,$A14,'QA Checklist'!$H$5:$H$180,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$181,$A14,'QA Checklist'!$H$5:$H$181,"Pending")</f>
         <v/>
       </c>
       <c r="F14" s="8">
@@ -752,19 +752,19 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$180,$A15)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$181,$A15)</f>
         <v/>
       </c>
       <c r="C15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$180,$A15,'QA Checklist'!$H$5:$H$180,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$180,$A15,'QA Checklist'!$H$5:$H$180,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$181,$A15,'QA Checklist'!$H$5:$H$181,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$181,$A15,'QA Checklist'!$H$5:$H$181,"Pass")</f>
         <v/>
       </c>
       <c r="D15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$180,$A15,'QA Checklist'!$H$5:$H$180,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$180,$A15,'QA Checklist'!$H$5:$H$180,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$181,$A15,'QA Checklist'!$H$5:$H$181,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$181,$A15,'QA Checklist'!$H$5:$H$181,"Fail")</f>
         <v/>
       </c>
       <c r="E15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$180,$A15,'QA Checklist'!$H$5:$H$180,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$181,$A15,'QA Checklist'!$H$5:$H$181,"Pending")</f>
         <v/>
       </c>
       <c r="F15" s="8">
@@ -779,19 +779,19 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$180,$A16)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$181,$A16)</f>
         <v/>
       </c>
       <c r="C16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$180,$A16,'QA Checklist'!$H$5:$H$180,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$180,$A16,'QA Checklist'!$H$5:$H$180,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$181,$A16,'QA Checklist'!$H$5:$H$181,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$181,$A16,'QA Checklist'!$H$5:$H$181,"Pass")</f>
         <v/>
       </c>
       <c r="D16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$180,$A16,'QA Checklist'!$H$5:$H$180,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$180,$A16,'QA Checklist'!$H$5:$H$180,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$181,$A16,'QA Checklist'!$H$5:$H$181,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$181,$A16,'QA Checklist'!$H$5:$H$181,"Fail")</f>
         <v/>
       </c>
       <c r="E16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$180,$A16,'QA Checklist'!$H$5:$H$180,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$181,$A16,'QA Checklist'!$H$5:$H$181,"Pending")</f>
         <v/>
       </c>
       <c r="F16" s="8">
@@ -806,19 +806,19 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$180,$A17)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$181,$A17)</f>
         <v/>
       </c>
       <c r="C17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$180,$A17,'QA Checklist'!$H$5:$H$180,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$180,$A17,'QA Checklist'!$H$5:$H$180,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$181,$A17,'QA Checklist'!$H$5:$H$181,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$181,$A17,'QA Checklist'!$H$5:$H$181,"Pass")</f>
         <v/>
       </c>
       <c r="D17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$180,$A17,'QA Checklist'!$H$5:$H$180,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$180,$A17,'QA Checklist'!$H$5:$H$180,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$181,$A17,'QA Checklist'!$H$5:$H$181,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$181,$A17,'QA Checklist'!$H$5:$H$181,"Fail")</f>
         <v/>
       </c>
       <c r="E17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$180,$A17,'QA Checklist'!$H$5:$H$180,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$181,$A17,'QA Checklist'!$H$5:$H$181,"Pending")</f>
         <v/>
       </c>
       <c r="F17" s="8">
@@ -833,19 +833,19 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$180,$A18)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$181,$A18)</f>
         <v/>
       </c>
       <c r="C18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$180,$A18,'QA Checklist'!$H$5:$H$180,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$180,$A18,'QA Checklist'!$H$5:$H$180,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$181,$A18,'QA Checklist'!$H$5:$H$181,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$181,$A18,'QA Checklist'!$H$5:$H$181,"Pass")</f>
         <v/>
       </c>
       <c r="D18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$180,$A18,'QA Checklist'!$H$5:$H$180,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$180,$A18,'QA Checklist'!$H$5:$H$180,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$181,$A18,'QA Checklist'!$H$5:$H$181,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$181,$A18,'QA Checklist'!$H$5:$H$181,"Fail")</f>
         <v/>
       </c>
       <c r="E18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$180,$A18,'QA Checklist'!$H$5:$H$180,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$181,$A18,'QA Checklist'!$H$5:$H$181,"Pending")</f>
         <v/>
       </c>
       <c r="F18" s="8">
@@ -860,19 +860,19 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$180,$A19)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$181,$A19)</f>
         <v/>
       </c>
       <c r="C19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$180,$A19,'QA Checklist'!$H$5:$H$180,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$180,$A19,'QA Checklist'!$H$5:$H$180,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$181,$A19,'QA Checklist'!$H$5:$H$181,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$181,$A19,'QA Checklist'!$H$5:$H$181,"Pass")</f>
         <v/>
       </c>
       <c r="D19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$180,$A19,'QA Checklist'!$H$5:$H$180,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$180,$A19,'QA Checklist'!$H$5:$H$180,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$181,$A19,'QA Checklist'!$H$5:$H$181,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$181,$A19,'QA Checklist'!$H$5:$H$181,"Fail")</f>
         <v/>
       </c>
       <c r="E19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$180,$A19,'QA Checklist'!$H$5:$H$180,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$181,$A19,'QA Checklist'!$H$5:$H$181,"Pending")</f>
         <v/>
       </c>
       <c r="F19" s="8">
@@ -887,19 +887,19 @@
         </is>
       </c>
       <c r="B20" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$180,$A20)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$181,$A20)</f>
         <v/>
       </c>
       <c r="C20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$180,$A20,'QA Checklist'!$H$5:$H$180,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$180,$A20,'QA Checklist'!$H$5:$H$180,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$181,$A20,'QA Checklist'!$H$5:$H$181,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$181,$A20,'QA Checklist'!$H$5:$H$181,"Pass")</f>
         <v/>
       </c>
       <c r="D20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$180,$A20,'QA Checklist'!$H$5:$H$180,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$180,$A20,'QA Checklist'!$H$5:$H$180,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$181,$A20,'QA Checklist'!$H$5:$H$181,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$181,$A20,'QA Checklist'!$H$5:$H$181,"Fail")</f>
         <v/>
       </c>
       <c r="E20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$180,$A20,'QA Checklist'!$H$5:$H$180,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$181,$A20,'QA Checklist'!$H$5:$H$181,"Pending")</f>
         <v/>
       </c>
       <c r="F20" s="8">
@@ -914,19 +914,19 @@
         </is>
       </c>
       <c r="B21" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$180,$A21)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$181,$A21)</f>
         <v/>
       </c>
       <c r="C21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$180,$A21,'QA Checklist'!$H$5:$H$180,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$180,$A21,'QA Checklist'!$H$5:$H$180,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$181,$A21,'QA Checklist'!$H$5:$H$181,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$181,$A21,'QA Checklist'!$H$5:$H$181,"Pass")</f>
         <v/>
       </c>
       <c r="D21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$180,$A21,'QA Checklist'!$H$5:$H$180,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$180,$A21,'QA Checklist'!$H$5:$H$180,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$181,$A21,'QA Checklist'!$H$5:$H$181,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$181,$A21,'QA Checklist'!$H$5:$H$181,"Fail")</f>
         <v/>
       </c>
       <c r="E21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$180,$A21,'QA Checklist'!$H$5:$H$180,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$181,$A21,'QA Checklist'!$H$5:$H$181,"Pending")</f>
         <v/>
       </c>
       <c r="F21" s="8">
@@ -941,19 +941,19 @@
         </is>
       </c>
       <c r="B22" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$180,$A22)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$181,$A22)</f>
         <v/>
       </c>
       <c r="C22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$180,$A22,'QA Checklist'!$H$5:$H$180,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$180,$A22,'QA Checklist'!$H$5:$H$180,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$181,$A22,'QA Checklist'!$H$5:$H$181,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$181,$A22,'QA Checklist'!$H$5:$H$181,"Pass")</f>
         <v/>
       </c>
       <c r="D22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$180,$A22,'QA Checklist'!$H$5:$H$180,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$180,$A22,'QA Checklist'!$H$5:$H$180,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$181,$A22,'QA Checklist'!$H$5:$H$181,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$181,$A22,'QA Checklist'!$H$5:$H$181,"Fail")</f>
         <v/>
       </c>
       <c r="E22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$180,$A22,'QA Checklist'!$H$5:$H$180,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$181,$A22,'QA Checklist'!$H$5:$H$181,"Pending")</f>
         <v/>
       </c>
       <c r="F22" s="8">
@@ -1023,19 +1023,19 @@
         </is>
       </c>
       <c r="B26" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$180,$A26&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$181,$A26&amp;"*")</f>
         <v/>
       </c>
       <c r="C26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$180,$A26&amp;"*",'QA Checklist'!$H$5:$H$180,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$180,$A26&amp;"*",'QA Checklist'!$H$5:$H$180,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$181,$A26&amp;"*",'QA Checklist'!$H$5:$H$181,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$181,$A26&amp;"*",'QA Checklist'!$H$5:$H$181,"Pass")</f>
         <v/>
       </c>
       <c r="D26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$180,$A26&amp;"*",'QA Checklist'!$H$5:$H$180,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$180,$A26&amp;"*",'QA Checklist'!$H$5:$H$180,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$181,$A26&amp;"*",'QA Checklist'!$H$5:$H$181,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$181,$A26&amp;"*",'QA Checklist'!$H$5:$H$181,"Fail")</f>
         <v/>
       </c>
       <c r="E26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$180,$A26&amp;"*",'QA Checklist'!$H$5:$H$180,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$181,$A26&amp;"*",'QA Checklist'!$H$5:$H$181,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1046,19 +1046,19 @@
         </is>
       </c>
       <c r="B27" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$180,$A27&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$181,$A27&amp;"*")</f>
         <v/>
       </c>
       <c r="C27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$180,$A27&amp;"*",'QA Checklist'!$H$5:$H$180,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$180,$A27&amp;"*",'QA Checklist'!$H$5:$H$180,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$181,$A27&amp;"*",'QA Checklist'!$H$5:$H$181,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$181,$A27&amp;"*",'QA Checklist'!$H$5:$H$181,"Pass")</f>
         <v/>
       </c>
       <c r="D27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$180,$A27&amp;"*",'QA Checklist'!$H$5:$H$180,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$180,$A27&amp;"*",'QA Checklist'!$H$5:$H$180,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$181,$A27&amp;"*",'QA Checklist'!$H$5:$H$181,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$181,$A27&amp;"*",'QA Checklist'!$H$5:$H$181,"Fail")</f>
         <v/>
       </c>
       <c r="E27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$180,$A27&amp;"*",'QA Checklist'!$H$5:$H$180,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$181,$A27&amp;"*",'QA Checklist'!$H$5:$H$181,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1069,19 +1069,19 @@
         </is>
       </c>
       <c r="B28" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$180,$A28&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$181,$A28&amp;"*")</f>
         <v/>
       </c>
       <c r="C28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$180,$A28&amp;"*",'QA Checklist'!$H$5:$H$180,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$180,$A28&amp;"*",'QA Checklist'!$H$5:$H$180,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$181,$A28&amp;"*",'QA Checklist'!$H$5:$H$181,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$181,$A28&amp;"*",'QA Checklist'!$H$5:$H$181,"Pass")</f>
         <v/>
       </c>
       <c r="D28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$180,$A28&amp;"*",'QA Checklist'!$H$5:$H$180,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$180,$A28&amp;"*",'QA Checklist'!$H$5:$H$180,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$181,$A28&amp;"*",'QA Checklist'!$H$5:$H$181,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$181,$A28&amp;"*",'QA Checklist'!$H$5:$H$181,"Fail")</f>
         <v/>
       </c>
       <c r="E28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$180,$A28&amp;"*",'QA Checklist'!$H$5:$H$180,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$181,$A28&amp;"*",'QA Checklist'!$H$5:$H$181,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1096,7 +1096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I180"/>
+  <dimension ref="A1:I181"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8999,12 +8999,59 @@
         </is>
       </c>
     </row>
+    <row r="181">
+      <c r="A181" s="12" t="inlineStr">
+        <is>
+          <t>SA-55</t>
+        </is>
+      </c>
+      <c r="B181" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="C181" s="13" t="inlineStr">
+        <is>
+          <t>Tier 2 (Workflow &amp; Ergonomics)</t>
+        </is>
+      </c>
+      <c r="D181" s="13" t="inlineStr">
+        <is>
+          <t>Maximized Studio PDF Size &amp; Centering</t>
+        </is>
+      </c>
+      <c r="E181" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="F181" s="13" t="inlineStr">
+        <is>
+          <t>Log in as Service Advisor, open 2025 RO Excel Studio, press Maximize PDF on Job_Order, Quotation_No, Billing_No and CheckList_Result, then Normal View; also press Hide Preview and resize the window</t>
+        </is>
+      </c>
+      <c r="G181" s="13" t="inlineStr">
+        <is>
+          <t>In the maximized view the PDF page shows at full height and centered (never as a small thumbnail); Normal View and Hide Preview redraw it to fit; no new browser tab opens</t>
+        </is>
+      </c>
+      <c r="H181" s="14" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="I181" s="13" t="inlineStr">
+        <is>
+          <t>Verified by Automated Unit Tests (167 passing in tests/frontend/sla_and_logic.test.js AUT-FRONT-138) and a real-time headless Chrome measurement</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:I180"/>
+  <autoFilter ref="A4:I181"/>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="H5:H180">
+  <conditionalFormatting sqref="H5:H181">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$H5="Passed"</formula>
     </cfRule>
@@ -9021,13 +9068,13 @@
       <formula>$H5="Pending"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A5:A180">
+  <conditionalFormatting sqref="A5:A181">
     <cfRule type="expression" priority="6" dxfId="3">
-      <formula>COUNTIF($A$5:$A$180,$A5)&gt;1</formula>
+      <formula>COUNTIF($A$5:$A$181,$A5)&gt;1</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H5:H180" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H5:H181" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pending,Passed,Failed"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat(REV-180): maximized studio PDF fills the pane width
While maximized, the studio PDF iframe uses the whole pane and loads with
view=FitH, so the page is shown at full pane width (scroll to read)
instead of a narrow whole-page fit. Normal View is unchanged.
Cache buster v=3.33, AUT-FRONT-139, SA-56.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
+++ b/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
@@ -11,7 +11,7 @@
     <sheet name="QA Checklist" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$181</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$182</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'QA Checklist'!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTA('QA Checklist'!$A$5:$A$181)</f>
+        <f>COUNTA('QA Checklist'!$A$5:$A$182)</f>
         <v/>
       </c>
     </row>
@@ -594,7 +594,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$181,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$181,"Pass")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$182,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$182,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$181,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$181,"Fail")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$182,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$182,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -616,7 +616,7 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$181,"Pending")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$182,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -671,19 +671,19 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$181,$A12)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$182,$A12)</f>
         <v/>
       </c>
       <c r="C12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$181,$A12,'QA Checklist'!$H$5:$H$181,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$181,$A12,'QA Checklist'!$H$5:$H$181,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$182,$A12,'QA Checklist'!$H$5:$H$182,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$182,$A12,'QA Checklist'!$H$5:$H$182,"Pass")</f>
         <v/>
       </c>
       <c r="D12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$181,$A12,'QA Checklist'!$H$5:$H$181,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$181,$A12,'QA Checklist'!$H$5:$H$181,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$182,$A12,'QA Checklist'!$H$5:$H$182,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$182,$A12,'QA Checklist'!$H$5:$H$182,"Fail")</f>
         <v/>
       </c>
       <c r="E12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$181,$A12,'QA Checklist'!$H$5:$H$181,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$182,$A12,'QA Checklist'!$H$5:$H$182,"Pending")</f>
         <v/>
       </c>
       <c r="F12" s="8">
@@ -698,19 +698,19 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$181,$A13)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$182,$A13)</f>
         <v/>
       </c>
       <c r="C13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$181,$A13,'QA Checklist'!$H$5:$H$181,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$181,$A13,'QA Checklist'!$H$5:$H$181,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$182,$A13,'QA Checklist'!$H$5:$H$182,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$182,$A13,'QA Checklist'!$H$5:$H$182,"Pass")</f>
         <v/>
       </c>
       <c r="D13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$181,$A13,'QA Checklist'!$H$5:$H$181,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$181,$A13,'QA Checklist'!$H$5:$H$181,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$182,$A13,'QA Checklist'!$H$5:$H$182,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$182,$A13,'QA Checklist'!$H$5:$H$182,"Fail")</f>
         <v/>
       </c>
       <c r="E13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$181,$A13,'QA Checklist'!$H$5:$H$181,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$182,$A13,'QA Checklist'!$H$5:$H$182,"Pending")</f>
         <v/>
       </c>
       <c r="F13" s="8">
@@ -725,19 +725,19 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$181,$A14)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$182,$A14)</f>
         <v/>
       </c>
       <c r="C14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$181,$A14,'QA Checklist'!$H$5:$H$181,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$181,$A14,'QA Checklist'!$H$5:$H$181,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$182,$A14,'QA Checklist'!$H$5:$H$182,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$182,$A14,'QA Checklist'!$H$5:$H$182,"Pass")</f>
         <v/>
       </c>
       <c r="D14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$181,$A14,'QA Checklist'!$H$5:$H$181,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$181,$A14,'QA Checklist'!$H$5:$H$181,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$182,$A14,'QA Checklist'!$H$5:$H$182,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$182,$A14,'QA Checklist'!$H$5:$H$182,"Fail")</f>
         <v/>
       </c>
       <c r="E14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$181,$A14,'QA Checklist'!$H$5:$H$181,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$182,$A14,'QA Checklist'!$H$5:$H$182,"Pending")</f>
         <v/>
       </c>
       <c r="F14" s="8">
@@ -752,19 +752,19 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$181,$A15)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$182,$A15)</f>
         <v/>
       </c>
       <c r="C15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$181,$A15,'QA Checklist'!$H$5:$H$181,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$181,$A15,'QA Checklist'!$H$5:$H$181,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$182,$A15,'QA Checklist'!$H$5:$H$182,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$182,$A15,'QA Checklist'!$H$5:$H$182,"Pass")</f>
         <v/>
       </c>
       <c r="D15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$181,$A15,'QA Checklist'!$H$5:$H$181,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$181,$A15,'QA Checklist'!$H$5:$H$181,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$182,$A15,'QA Checklist'!$H$5:$H$182,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$182,$A15,'QA Checklist'!$H$5:$H$182,"Fail")</f>
         <v/>
       </c>
       <c r="E15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$181,$A15,'QA Checklist'!$H$5:$H$181,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$182,$A15,'QA Checklist'!$H$5:$H$182,"Pending")</f>
         <v/>
       </c>
       <c r="F15" s="8">
@@ -779,19 +779,19 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$181,$A16)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$182,$A16)</f>
         <v/>
       </c>
       <c r="C16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$181,$A16,'QA Checklist'!$H$5:$H$181,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$181,$A16,'QA Checklist'!$H$5:$H$181,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$182,$A16,'QA Checklist'!$H$5:$H$182,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$182,$A16,'QA Checklist'!$H$5:$H$182,"Pass")</f>
         <v/>
       </c>
       <c r="D16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$181,$A16,'QA Checklist'!$H$5:$H$181,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$181,$A16,'QA Checklist'!$H$5:$H$181,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$182,$A16,'QA Checklist'!$H$5:$H$182,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$182,$A16,'QA Checklist'!$H$5:$H$182,"Fail")</f>
         <v/>
       </c>
       <c r="E16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$181,$A16,'QA Checklist'!$H$5:$H$181,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$182,$A16,'QA Checklist'!$H$5:$H$182,"Pending")</f>
         <v/>
       </c>
       <c r="F16" s="8">
@@ -806,19 +806,19 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$181,$A17)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$182,$A17)</f>
         <v/>
       </c>
       <c r="C17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$181,$A17,'QA Checklist'!$H$5:$H$181,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$181,$A17,'QA Checklist'!$H$5:$H$181,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$182,$A17,'QA Checklist'!$H$5:$H$182,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$182,$A17,'QA Checklist'!$H$5:$H$182,"Pass")</f>
         <v/>
       </c>
       <c r="D17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$181,$A17,'QA Checklist'!$H$5:$H$181,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$181,$A17,'QA Checklist'!$H$5:$H$181,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$182,$A17,'QA Checklist'!$H$5:$H$182,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$182,$A17,'QA Checklist'!$H$5:$H$182,"Fail")</f>
         <v/>
       </c>
       <c r="E17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$181,$A17,'QA Checklist'!$H$5:$H$181,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$182,$A17,'QA Checklist'!$H$5:$H$182,"Pending")</f>
         <v/>
       </c>
       <c r="F17" s="8">
@@ -833,19 +833,19 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$181,$A18)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$182,$A18)</f>
         <v/>
       </c>
       <c r="C18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$181,$A18,'QA Checklist'!$H$5:$H$181,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$181,$A18,'QA Checklist'!$H$5:$H$181,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$182,$A18,'QA Checklist'!$H$5:$H$182,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$182,$A18,'QA Checklist'!$H$5:$H$182,"Pass")</f>
         <v/>
       </c>
       <c r="D18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$181,$A18,'QA Checklist'!$H$5:$H$181,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$181,$A18,'QA Checklist'!$H$5:$H$181,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$182,$A18,'QA Checklist'!$H$5:$H$182,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$182,$A18,'QA Checklist'!$H$5:$H$182,"Fail")</f>
         <v/>
       </c>
       <c r="E18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$181,$A18,'QA Checklist'!$H$5:$H$181,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$182,$A18,'QA Checklist'!$H$5:$H$182,"Pending")</f>
         <v/>
       </c>
       <c r="F18" s="8">
@@ -860,19 +860,19 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$181,$A19)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$182,$A19)</f>
         <v/>
       </c>
       <c r="C19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$181,$A19,'QA Checklist'!$H$5:$H$181,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$181,$A19,'QA Checklist'!$H$5:$H$181,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$182,$A19,'QA Checklist'!$H$5:$H$182,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$182,$A19,'QA Checklist'!$H$5:$H$182,"Pass")</f>
         <v/>
       </c>
       <c r="D19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$181,$A19,'QA Checklist'!$H$5:$H$181,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$181,$A19,'QA Checklist'!$H$5:$H$181,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$182,$A19,'QA Checklist'!$H$5:$H$182,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$182,$A19,'QA Checklist'!$H$5:$H$182,"Fail")</f>
         <v/>
       </c>
       <c r="E19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$181,$A19,'QA Checklist'!$H$5:$H$181,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$182,$A19,'QA Checklist'!$H$5:$H$182,"Pending")</f>
         <v/>
       </c>
       <c r="F19" s="8">
@@ -887,19 +887,19 @@
         </is>
       </c>
       <c r="B20" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$181,$A20)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$182,$A20)</f>
         <v/>
       </c>
       <c r="C20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$181,$A20,'QA Checklist'!$H$5:$H$181,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$181,$A20,'QA Checklist'!$H$5:$H$181,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$182,$A20,'QA Checklist'!$H$5:$H$182,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$182,$A20,'QA Checklist'!$H$5:$H$182,"Pass")</f>
         <v/>
       </c>
       <c r="D20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$181,$A20,'QA Checklist'!$H$5:$H$181,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$181,$A20,'QA Checklist'!$H$5:$H$181,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$182,$A20,'QA Checklist'!$H$5:$H$182,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$182,$A20,'QA Checklist'!$H$5:$H$182,"Fail")</f>
         <v/>
       </c>
       <c r="E20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$181,$A20,'QA Checklist'!$H$5:$H$181,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$182,$A20,'QA Checklist'!$H$5:$H$182,"Pending")</f>
         <v/>
       </c>
       <c r="F20" s="8">
@@ -914,19 +914,19 @@
         </is>
       </c>
       <c r="B21" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$181,$A21)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$182,$A21)</f>
         <v/>
       </c>
       <c r="C21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$181,$A21,'QA Checklist'!$H$5:$H$181,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$181,$A21,'QA Checklist'!$H$5:$H$181,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$182,$A21,'QA Checklist'!$H$5:$H$182,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$182,$A21,'QA Checklist'!$H$5:$H$182,"Pass")</f>
         <v/>
       </c>
       <c r="D21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$181,$A21,'QA Checklist'!$H$5:$H$181,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$181,$A21,'QA Checklist'!$H$5:$H$181,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$182,$A21,'QA Checklist'!$H$5:$H$182,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$182,$A21,'QA Checklist'!$H$5:$H$182,"Fail")</f>
         <v/>
       </c>
       <c r="E21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$181,$A21,'QA Checklist'!$H$5:$H$181,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$182,$A21,'QA Checklist'!$H$5:$H$182,"Pending")</f>
         <v/>
       </c>
       <c r="F21" s="8">
@@ -941,19 +941,19 @@
         </is>
       </c>
       <c r="B22" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$181,$A22)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$182,$A22)</f>
         <v/>
       </c>
       <c r="C22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$181,$A22,'QA Checklist'!$H$5:$H$181,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$181,$A22,'QA Checklist'!$H$5:$H$181,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$182,$A22,'QA Checklist'!$H$5:$H$182,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$182,$A22,'QA Checklist'!$H$5:$H$182,"Pass")</f>
         <v/>
       </c>
       <c r="D22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$181,$A22,'QA Checklist'!$H$5:$H$181,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$181,$A22,'QA Checklist'!$H$5:$H$181,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$182,$A22,'QA Checklist'!$H$5:$H$182,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$182,$A22,'QA Checklist'!$H$5:$H$182,"Fail")</f>
         <v/>
       </c>
       <c r="E22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$181,$A22,'QA Checklist'!$H$5:$H$181,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$182,$A22,'QA Checklist'!$H$5:$H$182,"Pending")</f>
         <v/>
       </c>
       <c r="F22" s="8">
@@ -1023,19 +1023,19 @@
         </is>
       </c>
       <c r="B26" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$181,$A26&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$182,$A26&amp;"*")</f>
         <v/>
       </c>
       <c r="C26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$181,$A26&amp;"*",'QA Checklist'!$H$5:$H$181,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$181,$A26&amp;"*",'QA Checklist'!$H$5:$H$181,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$182,$A26&amp;"*",'QA Checklist'!$H$5:$H$182,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$182,$A26&amp;"*",'QA Checklist'!$H$5:$H$182,"Pass")</f>
         <v/>
       </c>
       <c r="D26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$181,$A26&amp;"*",'QA Checklist'!$H$5:$H$181,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$181,$A26&amp;"*",'QA Checklist'!$H$5:$H$181,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$182,$A26&amp;"*",'QA Checklist'!$H$5:$H$182,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$182,$A26&amp;"*",'QA Checklist'!$H$5:$H$182,"Fail")</f>
         <v/>
       </c>
       <c r="E26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$181,$A26&amp;"*",'QA Checklist'!$H$5:$H$181,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$182,$A26&amp;"*",'QA Checklist'!$H$5:$H$182,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1046,19 +1046,19 @@
         </is>
       </c>
       <c r="B27" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$181,$A27&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$182,$A27&amp;"*")</f>
         <v/>
       </c>
       <c r="C27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$181,$A27&amp;"*",'QA Checklist'!$H$5:$H$181,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$181,$A27&amp;"*",'QA Checklist'!$H$5:$H$181,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$182,$A27&amp;"*",'QA Checklist'!$H$5:$H$182,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$182,$A27&amp;"*",'QA Checklist'!$H$5:$H$182,"Pass")</f>
         <v/>
       </c>
       <c r="D27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$181,$A27&amp;"*",'QA Checklist'!$H$5:$H$181,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$181,$A27&amp;"*",'QA Checklist'!$H$5:$H$181,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$182,$A27&amp;"*",'QA Checklist'!$H$5:$H$182,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$182,$A27&amp;"*",'QA Checklist'!$H$5:$H$182,"Fail")</f>
         <v/>
       </c>
       <c r="E27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$181,$A27&amp;"*",'QA Checklist'!$H$5:$H$181,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$182,$A27&amp;"*",'QA Checklist'!$H$5:$H$182,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1069,19 +1069,19 @@
         </is>
       </c>
       <c r="B28" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$181,$A28&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$182,$A28&amp;"*")</f>
         <v/>
       </c>
       <c r="C28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$181,$A28&amp;"*",'QA Checklist'!$H$5:$H$181,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$181,$A28&amp;"*",'QA Checklist'!$H$5:$H$181,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$182,$A28&amp;"*",'QA Checklist'!$H$5:$H$182,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$182,$A28&amp;"*",'QA Checklist'!$H$5:$H$182,"Pass")</f>
         <v/>
       </c>
       <c r="D28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$181,$A28&amp;"*",'QA Checklist'!$H$5:$H$181,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$181,$A28&amp;"*",'QA Checklist'!$H$5:$H$181,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$182,$A28&amp;"*",'QA Checklist'!$H$5:$H$182,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$182,$A28&amp;"*",'QA Checklist'!$H$5:$H$182,"Fail")</f>
         <v/>
       </c>
       <c r="E28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$181,$A28&amp;"*",'QA Checklist'!$H$5:$H$181,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$182,$A28&amp;"*",'QA Checklist'!$H$5:$H$182,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1096,7 +1096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I181"/>
+  <dimension ref="A1:I182"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9046,12 +9046,59 @@
         </is>
       </c>
     </row>
+    <row r="182">
+      <c r="A182" s="12" t="inlineStr">
+        <is>
+          <t>SA-56</t>
+        </is>
+      </c>
+      <c r="B182" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="C182" s="13" t="inlineStr">
+        <is>
+          <t>Tier 2 (Workflow &amp; Ergonomics)</t>
+        </is>
+      </c>
+      <c r="D182" s="13" t="inlineStr">
+        <is>
+          <t>Bigger PDF in Maximized Studio View</t>
+        </is>
+      </c>
+      <c r="E182" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="F182" s="13" t="inlineStr">
+        <is>
+          <t>Log in as Service Advisor, open 2025 RO Excel Studio, press Maximize PDF on each tab, scroll the document, then press Normal View</t>
+        </is>
+      </c>
+      <c r="G182" s="13" t="inlineStr">
+        <is>
+          <t>Maximized: the PDF fills the pane width (large, readable) and scrolls vertically; Normal View: the whole page fits beside the form again; no new tab opens</t>
+        </is>
+      </c>
+      <c r="H182" s="14" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="I182" s="13" t="inlineStr">
+        <is>
+          <t>Verified by Automated Unit Tests (168 passing in tests/frontend/sla_and_logic.test.js AUT-FRONT-139) and a real-time headless Chrome screenshot</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:I181"/>
+  <autoFilter ref="A4:I182"/>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="H5:H181">
+  <conditionalFormatting sqref="H5:H182">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$H5="Passed"</formula>
     </cfRule>
@@ -9068,13 +9115,13 @@
       <formula>$H5="Pending"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A5:A181">
+  <conditionalFormatting sqref="A5:A182">
     <cfRule type="expression" priority="6" dxfId="3">
-      <formula>COUNTIF($A$5:$A$181,$A5)&gt;1</formula>
+      <formula>COUNTIF($A$5:$A$182,$A5)&gt;1</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H5:H181" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H5:H182" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pending,Passed,Failed"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat(REV-181): professional neutral headers for the Full PDF viewers
Replace the dark, colorful headers (colored icon tiles, pills, pulsing
"Full Scale High-Def" badge, colored print buttons) of the Job Order,
Quotation, Billing and Checklist Full PDF viewers with one neutral header
matching the studio PDF toolbar. Ids and button actions unchanged.
Cache buster v=3.34, AUT-FRONT-140, SA-57.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
+++ b/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
@@ -11,7 +11,7 @@
     <sheet name="QA Checklist" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$182</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$183</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'QA Checklist'!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTA('QA Checklist'!$A$5:$A$182)</f>
+        <f>COUNTA('QA Checklist'!$A$5:$A$183)</f>
         <v/>
       </c>
     </row>
@@ -594,7 +594,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$182,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$182,"Pass")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$183,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$183,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$182,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$182,"Fail")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$183,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$183,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -616,7 +616,7 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$182,"Pending")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$183,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -671,19 +671,19 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$182,$A12)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$183,$A12)</f>
         <v/>
       </c>
       <c r="C12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$182,$A12,'QA Checklist'!$H$5:$H$182,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$182,$A12,'QA Checklist'!$H$5:$H$182,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$183,$A12,'QA Checklist'!$H$5:$H$183,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$183,$A12,'QA Checklist'!$H$5:$H$183,"Pass")</f>
         <v/>
       </c>
       <c r="D12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$182,$A12,'QA Checklist'!$H$5:$H$182,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$182,$A12,'QA Checklist'!$H$5:$H$182,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$183,$A12,'QA Checklist'!$H$5:$H$183,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$183,$A12,'QA Checklist'!$H$5:$H$183,"Fail")</f>
         <v/>
       </c>
       <c r="E12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$182,$A12,'QA Checklist'!$H$5:$H$182,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$183,$A12,'QA Checklist'!$H$5:$H$183,"Pending")</f>
         <v/>
       </c>
       <c r="F12" s="8">
@@ -698,19 +698,19 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$182,$A13)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$183,$A13)</f>
         <v/>
       </c>
       <c r="C13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$182,$A13,'QA Checklist'!$H$5:$H$182,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$182,$A13,'QA Checklist'!$H$5:$H$182,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$183,$A13,'QA Checklist'!$H$5:$H$183,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$183,$A13,'QA Checklist'!$H$5:$H$183,"Pass")</f>
         <v/>
       </c>
       <c r="D13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$182,$A13,'QA Checklist'!$H$5:$H$182,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$182,$A13,'QA Checklist'!$H$5:$H$182,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$183,$A13,'QA Checklist'!$H$5:$H$183,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$183,$A13,'QA Checklist'!$H$5:$H$183,"Fail")</f>
         <v/>
       </c>
       <c r="E13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$182,$A13,'QA Checklist'!$H$5:$H$182,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$183,$A13,'QA Checklist'!$H$5:$H$183,"Pending")</f>
         <v/>
       </c>
       <c r="F13" s="8">
@@ -725,19 +725,19 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$182,$A14)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$183,$A14)</f>
         <v/>
       </c>
       <c r="C14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$182,$A14,'QA Checklist'!$H$5:$H$182,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$182,$A14,'QA Checklist'!$H$5:$H$182,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$183,$A14,'QA Checklist'!$H$5:$H$183,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$183,$A14,'QA Checklist'!$H$5:$H$183,"Pass")</f>
         <v/>
       </c>
       <c r="D14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$182,$A14,'QA Checklist'!$H$5:$H$182,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$182,$A14,'QA Checklist'!$H$5:$H$182,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$183,$A14,'QA Checklist'!$H$5:$H$183,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$183,$A14,'QA Checklist'!$H$5:$H$183,"Fail")</f>
         <v/>
       </c>
       <c r="E14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$182,$A14,'QA Checklist'!$H$5:$H$182,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$183,$A14,'QA Checklist'!$H$5:$H$183,"Pending")</f>
         <v/>
       </c>
       <c r="F14" s="8">
@@ -752,19 +752,19 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$182,$A15)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$183,$A15)</f>
         <v/>
       </c>
       <c r="C15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$182,$A15,'QA Checklist'!$H$5:$H$182,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$182,$A15,'QA Checklist'!$H$5:$H$182,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$183,$A15,'QA Checklist'!$H$5:$H$183,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$183,$A15,'QA Checklist'!$H$5:$H$183,"Pass")</f>
         <v/>
       </c>
       <c r="D15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$182,$A15,'QA Checklist'!$H$5:$H$182,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$182,$A15,'QA Checklist'!$H$5:$H$182,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$183,$A15,'QA Checklist'!$H$5:$H$183,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$183,$A15,'QA Checklist'!$H$5:$H$183,"Fail")</f>
         <v/>
       </c>
       <c r="E15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$182,$A15,'QA Checklist'!$H$5:$H$182,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$183,$A15,'QA Checklist'!$H$5:$H$183,"Pending")</f>
         <v/>
       </c>
       <c r="F15" s="8">
@@ -779,19 +779,19 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$182,$A16)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$183,$A16)</f>
         <v/>
       </c>
       <c r="C16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$182,$A16,'QA Checklist'!$H$5:$H$182,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$182,$A16,'QA Checklist'!$H$5:$H$182,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$183,$A16,'QA Checklist'!$H$5:$H$183,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$183,$A16,'QA Checklist'!$H$5:$H$183,"Pass")</f>
         <v/>
       </c>
       <c r="D16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$182,$A16,'QA Checklist'!$H$5:$H$182,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$182,$A16,'QA Checklist'!$H$5:$H$182,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$183,$A16,'QA Checklist'!$H$5:$H$183,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$183,$A16,'QA Checklist'!$H$5:$H$183,"Fail")</f>
         <v/>
       </c>
       <c r="E16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$182,$A16,'QA Checklist'!$H$5:$H$182,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$183,$A16,'QA Checklist'!$H$5:$H$183,"Pending")</f>
         <v/>
       </c>
       <c r="F16" s="8">
@@ -806,19 +806,19 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$182,$A17)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$183,$A17)</f>
         <v/>
       </c>
       <c r="C17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$182,$A17,'QA Checklist'!$H$5:$H$182,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$182,$A17,'QA Checklist'!$H$5:$H$182,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$183,$A17,'QA Checklist'!$H$5:$H$183,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$183,$A17,'QA Checklist'!$H$5:$H$183,"Pass")</f>
         <v/>
       </c>
       <c r="D17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$182,$A17,'QA Checklist'!$H$5:$H$182,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$182,$A17,'QA Checklist'!$H$5:$H$182,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$183,$A17,'QA Checklist'!$H$5:$H$183,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$183,$A17,'QA Checklist'!$H$5:$H$183,"Fail")</f>
         <v/>
       </c>
       <c r="E17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$182,$A17,'QA Checklist'!$H$5:$H$182,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$183,$A17,'QA Checklist'!$H$5:$H$183,"Pending")</f>
         <v/>
       </c>
       <c r="F17" s="8">
@@ -833,19 +833,19 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$182,$A18)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$183,$A18)</f>
         <v/>
       </c>
       <c r="C18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$182,$A18,'QA Checklist'!$H$5:$H$182,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$182,$A18,'QA Checklist'!$H$5:$H$182,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$183,$A18,'QA Checklist'!$H$5:$H$183,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$183,$A18,'QA Checklist'!$H$5:$H$183,"Pass")</f>
         <v/>
       </c>
       <c r="D18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$182,$A18,'QA Checklist'!$H$5:$H$182,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$182,$A18,'QA Checklist'!$H$5:$H$182,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$183,$A18,'QA Checklist'!$H$5:$H$183,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$183,$A18,'QA Checklist'!$H$5:$H$183,"Fail")</f>
         <v/>
       </c>
       <c r="E18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$182,$A18,'QA Checklist'!$H$5:$H$182,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$183,$A18,'QA Checklist'!$H$5:$H$183,"Pending")</f>
         <v/>
       </c>
       <c r="F18" s="8">
@@ -860,19 +860,19 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$182,$A19)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$183,$A19)</f>
         <v/>
       </c>
       <c r="C19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$182,$A19,'QA Checklist'!$H$5:$H$182,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$182,$A19,'QA Checklist'!$H$5:$H$182,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$183,$A19,'QA Checklist'!$H$5:$H$183,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$183,$A19,'QA Checklist'!$H$5:$H$183,"Pass")</f>
         <v/>
       </c>
       <c r="D19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$182,$A19,'QA Checklist'!$H$5:$H$182,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$182,$A19,'QA Checklist'!$H$5:$H$182,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$183,$A19,'QA Checklist'!$H$5:$H$183,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$183,$A19,'QA Checklist'!$H$5:$H$183,"Fail")</f>
         <v/>
       </c>
       <c r="E19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$182,$A19,'QA Checklist'!$H$5:$H$182,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$183,$A19,'QA Checklist'!$H$5:$H$183,"Pending")</f>
         <v/>
       </c>
       <c r="F19" s="8">
@@ -887,19 +887,19 @@
         </is>
       </c>
       <c r="B20" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$182,$A20)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$183,$A20)</f>
         <v/>
       </c>
       <c r="C20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$182,$A20,'QA Checklist'!$H$5:$H$182,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$182,$A20,'QA Checklist'!$H$5:$H$182,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$183,$A20,'QA Checklist'!$H$5:$H$183,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$183,$A20,'QA Checklist'!$H$5:$H$183,"Pass")</f>
         <v/>
       </c>
       <c r="D20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$182,$A20,'QA Checklist'!$H$5:$H$182,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$182,$A20,'QA Checklist'!$H$5:$H$182,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$183,$A20,'QA Checklist'!$H$5:$H$183,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$183,$A20,'QA Checklist'!$H$5:$H$183,"Fail")</f>
         <v/>
       </c>
       <c r="E20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$182,$A20,'QA Checklist'!$H$5:$H$182,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$183,$A20,'QA Checklist'!$H$5:$H$183,"Pending")</f>
         <v/>
       </c>
       <c r="F20" s="8">
@@ -914,19 +914,19 @@
         </is>
       </c>
       <c r="B21" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$182,$A21)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$183,$A21)</f>
         <v/>
       </c>
       <c r="C21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$182,$A21,'QA Checklist'!$H$5:$H$182,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$182,$A21,'QA Checklist'!$H$5:$H$182,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$183,$A21,'QA Checklist'!$H$5:$H$183,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$183,$A21,'QA Checklist'!$H$5:$H$183,"Pass")</f>
         <v/>
       </c>
       <c r="D21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$182,$A21,'QA Checklist'!$H$5:$H$182,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$182,$A21,'QA Checklist'!$H$5:$H$182,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$183,$A21,'QA Checklist'!$H$5:$H$183,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$183,$A21,'QA Checklist'!$H$5:$H$183,"Fail")</f>
         <v/>
       </c>
       <c r="E21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$182,$A21,'QA Checklist'!$H$5:$H$182,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$183,$A21,'QA Checklist'!$H$5:$H$183,"Pending")</f>
         <v/>
       </c>
       <c r="F21" s="8">
@@ -941,19 +941,19 @@
         </is>
       </c>
       <c r="B22" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$182,$A22)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$183,$A22)</f>
         <v/>
       </c>
       <c r="C22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$182,$A22,'QA Checklist'!$H$5:$H$182,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$182,$A22,'QA Checklist'!$H$5:$H$182,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$183,$A22,'QA Checklist'!$H$5:$H$183,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$183,$A22,'QA Checklist'!$H$5:$H$183,"Pass")</f>
         <v/>
       </c>
       <c r="D22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$182,$A22,'QA Checklist'!$H$5:$H$182,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$182,$A22,'QA Checklist'!$H$5:$H$182,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$183,$A22,'QA Checklist'!$H$5:$H$183,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$183,$A22,'QA Checklist'!$H$5:$H$183,"Fail")</f>
         <v/>
       </c>
       <c r="E22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$182,$A22,'QA Checklist'!$H$5:$H$182,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$183,$A22,'QA Checklist'!$H$5:$H$183,"Pending")</f>
         <v/>
       </c>
       <c r="F22" s="8">
@@ -1023,19 +1023,19 @@
         </is>
       </c>
       <c r="B26" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$182,$A26&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$183,$A26&amp;"*")</f>
         <v/>
       </c>
       <c r="C26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$182,$A26&amp;"*",'QA Checklist'!$H$5:$H$182,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$182,$A26&amp;"*",'QA Checklist'!$H$5:$H$182,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$183,$A26&amp;"*",'QA Checklist'!$H$5:$H$183,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$183,$A26&amp;"*",'QA Checklist'!$H$5:$H$183,"Pass")</f>
         <v/>
       </c>
       <c r="D26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$182,$A26&amp;"*",'QA Checklist'!$H$5:$H$182,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$182,$A26&amp;"*",'QA Checklist'!$H$5:$H$182,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$183,$A26&amp;"*",'QA Checklist'!$H$5:$H$183,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$183,$A26&amp;"*",'QA Checklist'!$H$5:$H$183,"Fail")</f>
         <v/>
       </c>
       <c r="E26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$182,$A26&amp;"*",'QA Checklist'!$H$5:$H$182,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$183,$A26&amp;"*",'QA Checklist'!$H$5:$H$183,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1046,19 +1046,19 @@
         </is>
       </c>
       <c r="B27" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$182,$A27&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$183,$A27&amp;"*")</f>
         <v/>
       </c>
       <c r="C27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$182,$A27&amp;"*",'QA Checklist'!$H$5:$H$182,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$182,$A27&amp;"*",'QA Checklist'!$H$5:$H$182,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$183,$A27&amp;"*",'QA Checklist'!$H$5:$H$183,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$183,$A27&amp;"*",'QA Checklist'!$H$5:$H$183,"Pass")</f>
         <v/>
       </c>
       <c r="D27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$182,$A27&amp;"*",'QA Checklist'!$H$5:$H$182,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$182,$A27&amp;"*",'QA Checklist'!$H$5:$H$182,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$183,$A27&amp;"*",'QA Checklist'!$H$5:$H$183,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$183,$A27&amp;"*",'QA Checklist'!$H$5:$H$183,"Fail")</f>
         <v/>
       </c>
       <c r="E27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$182,$A27&amp;"*",'QA Checklist'!$H$5:$H$182,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$183,$A27&amp;"*",'QA Checklist'!$H$5:$H$183,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1069,19 +1069,19 @@
         </is>
       </c>
       <c r="B28" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$182,$A28&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$183,$A28&amp;"*")</f>
         <v/>
       </c>
       <c r="C28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$182,$A28&amp;"*",'QA Checklist'!$H$5:$H$182,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$182,$A28&amp;"*",'QA Checklist'!$H$5:$H$182,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$183,$A28&amp;"*",'QA Checklist'!$H$5:$H$183,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$183,$A28&amp;"*",'QA Checklist'!$H$5:$H$183,"Pass")</f>
         <v/>
       </c>
       <c r="D28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$182,$A28&amp;"*",'QA Checklist'!$H$5:$H$182,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$182,$A28&amp;"*",'QA Checklist'!$H$5:$H$182,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$183,$A28&amp;"*",'QA Checklist'!$H$5:$H$183,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$183,$A28&amp;"*",'QA Checklist'!$H$5:$H$183,"Fail")</f>
         <v/>
       </c>
       <c r="E28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$182,$A28&amp;"*",'QA Checklist'!$H$5:$H$182,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$183,$A28&amp;"*",'QA Checklist'!$H$5:$H$183,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1096,7 +1096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I182"/>
+  <dimension ref="A1:I183"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9093,12 +9093,59 @@
         </is>
       </c>
     </row>
+    <row r="183">
+      <c r="A183" s="12" t="inlineStr">
+        <is>
+          <t>SA-57</t>
+        </is>
+      </c>
+      <c r="B183" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="C183" s="13" t="inlineStr">
+        <is>
+          <t>Tier 2 (Workflow &amp; Ergonomics)</t>
+        </is>
+      </c>
+      <c r="D183" s="13" t="inlineStr">
+        <is>
+          <t>Neutral Full PDF Viewer Headers</t>
+        </is>
+      </c>
+      <c r="E183" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="F183" s="13" t="inlineStr">
+        <is>
+          <t>Log in as Service Advisor, open 2025 RO Excel Studio and press Full PDF on Job_Order, Quotation_No, Billing_No and CheckList_Result; use New Tab, Download PDF, Print and Close</t>
+        </is>
+      </c>
+      <c r="G183" s="13" t="inlineStr">
+        <is>
+          <t>Each viewer shows the same white neutral header (title, document number, Official PDF view subtitle, white buttons) without colored tiles or pills; all buttons still work</t>
+        </is>
+      </c>
+      <c r="H183" s="14" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="I183" s="13" t="inlineStr">
+        <is>
+          <t>Verified by Automated Unit Tests (169 passing in tests/frontend/sla_and_logic.test.js AUT-FRONT-140) and a headless Chrome render of the headers</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:I182"/>
+  <autoFilter ref="A4:I183"/>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="H5:H182">
+  <conditionalFormatting sqref="H5:H183">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$H5="Passed"</formula>
     </cfRule>
@@ -9115,13 +9162,13 @@
       <formula>$H5="Pending"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A5:A182">
+  <conditionalFormatting sqref="A5:A183">
     <cfRule type="expression" priority="6" dxfId="3">
-      <formula>COUNTIF($A$5:$A$182,$A5)&gt;1</formula>
+      <formula>COUNTIF($A$5:$A$183,$A5)&gt;1</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H5:H182" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H5:H183" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pending,Passed,Failed"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat(REV-182): previous / next document arrows in the studio and Full PDF
Add a neutral "< n / 4 >" control to the four studio PDF toolbars and the
four Full PDF viewer headers to move Job_Order -> Quotation_No ->
Billing_No -> CheckList_Result (wrapping). In the Full PDF viewer the
arrows and Left / Right keys open the next document and the studio follows.
Cache buster v=3.35, AUT-FRONT-141, SA-58.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
+++ b/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
@@ -11,7 +11,7 @@
     <sheet name="QA Checklist" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$183</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$184</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'QA Checklist'!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTA('QA Checklist'!$A$5:$A$183)</f>
+        <f>COUNTA('QA Checklist'!$A$5:$A$184)</f>
         <v/>
       </c>
     </row>
@@ -594,7 +594,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$183,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$183,"Pass")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$184,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$184,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$183,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$183,"Fail")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$184,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$184,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -616,7 +616,7 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$183,"Pending")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$184,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -671,19 +671,19 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$183,$A12)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$184,$A12)</f>
         <v/>
       </c>
       <c r="C12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$183,$A12,'QA Checklist'!$H$5:$H$183,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$183,$A12,'QA Checklist'!$H$5:$H$183,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$184,$A12,'QA Checklist'!$H$5:$H$184,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$184,$A12,'QA Checklist'!$H$5:$H$184,"Pass")</f>
         <v/>
       </c>
       <c r="D12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$183,$A12,'QA Checklist'!$H$5:$H$183,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$183,$A12,'QA Checklist'!$H$5:$H$183,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$184,$A12,'QA Checklist'!$H$5:$H$184,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$184,$A12,'QA Checklist'!$H$5:$H$184,"Fail")</f>
         <v/>
       </c>
       <c r="E12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$183,$A12,'QA Checklist'!$H$5:$H$183,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$184,$A12,'QA Checklist'!$H$5:$H$184,"Pending")</f>
         <v/>
       </c>
       <c r="F12" s="8">
@@ -698,19 +698,19 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$183,$A13)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$184,$A13)</f>
         <v/>
       </c>
       <c r="C13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$183,$A13,'QA Checklist'!$H$5:$H$183,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$183,$A13,'QA Checklist'!$H$5:$H$183,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$184,$A13,'QA Checklist'!$H$5:$H$184,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$184,$A13,'QA Checklist'!$H$5:$H$184,"Pass")</f>
         <v/>
       </c>
       <c r="D13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$183,$A13,'QA Checklist'!$H$5:$H$183,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$183,$A13,'QA Checklist'!$H$5:$H$183,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$184,$A13,'QA Checklist'!$H$5:$H$184,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$184,$A13,'QA Checklist'!$H$5:$H$184,"Fail")</f>
         <v/>
       </c>
       <c r="E13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$183,$A13,'QA Checklist'!$H$5:$H$183,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$184,$A13,'QA Checklist'!$H$5:$H$184,"Pending")</f>
         <v/>
       </c>
       <c r="F13" s="8">
@@ -725,19 +725,19 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$183,$A14)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$184,$A14)</f>
         <v/>
       </c>
       <c r="C14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$183,$A14,'QA Checklist'!$H$5:$H$183,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$183,$A14,'QA Checklist'!$H$5:$H$183,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$184,$A14,'QA Checklist'!$H$5:$H$184,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$184,$A14,'QA Checklist'!$H$5:$H$184,"Pass")</f>
         <v/>
       </c>
       <c r="D14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$183,$A14,'QA Checklist'!$H$5:$H$183,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$183,$A14,'QA Checklist'!$H$5:$H$183,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$184,$A14,'QA Checklist'!$H$5:$H$184,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$184,$A14,'QA Checklist'!$H$5:$H$184,"Fail")</f>
         <v/>
       </c>
       <c r="E14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$183,$A14,'QA Checklist'!$H$5:$H$183,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$184,$A14,'QA Checklist'!$H$5:$H$184,"Pending")</f>
         <v/>
       </c>
       <c r="F14" s="8">
@@ -752,19 +752,19 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$183,$A15)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$184,$A15)</f>
         <v/>
       </c>
       <c r="C15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$183,$A15,'QA Checklist'!$H$5:$H$183,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$183,$A15,'QA Checklist'!$H$5:$H$183,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$184,$A15,'QA Checklist'!$H$5:$H$184,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$184,$A15,'QA Checklist'!$H$5:$H$184,"Pass")</f>
         <v/>
       </c>
       <c r="D15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$183,$A15,'QA Checklist'!$H$5:$H$183,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$183,$A15,'QA Checklist'!$H$5:$H$183,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$184,$A15,'QA Checklist'!$H$5:$H$184,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$184,$A15,'QA Checklist'!$H$5:$H$184,"Fail")</f>
         <v/>
       </c>
       <c r="E15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$183,$A15,'QA Checklist'!$H$5:$H$183,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$184,$A15,'QA Checklist'!$H$5:$H$184,"Pending")</f>
         <v/>
       </c>
       <c r="F15" s="8">
@@ -779,19 +779,19 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$183,$A16)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$184,$A16)</f>
         <v/>
       </c>
       <c r="C16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$183,$A16,'QA Checklist'!$H$5:$H$183,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$183,$A16,'QA Checklist'!$H$5:$H$183,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$184,$A16,'QA Checklist'!$H$5:$H$184,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$184,$A16,'QA Checklist'!$H$5:$H$184,"Pass")</f>
         <v/>
       </c>
       <c r="D16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$183,$A16,'QA Checklist'!$H$5:$H$183,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$183,$A16,'QA Checklist'!$H$5:$H$183,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$184,$A16,'QA Checklist'!$H$5:$H$184,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$184,$A16,'QA Checklist'!$H$5:$H$184,"Fail")</f>
         <v/>
       </c>
       <c r="E16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$183,$A16,'QA Checklist'!$H$5:$H$183,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$184,$A16,'QA Checklist'!$H$5:$H$184,"Pending")</f>
         <v/>
       </c>
       <c r="F16" s="8">
@@ -806,19 +806,19 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$183,$A17)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$184,$A17)</f>
         <v/>
       </c>
       <c r="C17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$183,$A17,'QA Checklist'!$H$5:$H$183,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$183,$A17,'QA Checklist'!$H$5:$H$183,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$184,$A17,'QA Checklist'!$H$5:$H$184,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$184,$A17,'QA Checklist'!$H$5:$H$184,"Pass")</f>
         <v/>
       </c>
       <c r="D17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$183,$A17,'QA Checklist'!$H$5:$H$183,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$183,$A17,'QA Checklist'!$H$5:$H$183,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$184,$A17,'QA Checklist'!$H$5:$H$184,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$184,$A17,'QA Checklist'!$H$5:$H$184,"Fail")</f>
         <v/>
       </c>
       <c r="E17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$183,$A17,'QA Checklist'!$H$5:$H$183,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$184,$A17,'QA Checklist'!$H$5:$H$184,"Pending")</f>
         <v/>
       </c>
       <c r="F17" s="8">
@@ -833,19 +833,19 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$183,$A18)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$184,$A18)</f>
         <v/>
       </c>
       <c r="C18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$183,$A18,'QA Checklist'!$H$5:$H$183,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$183,$A18,'QA Checklist'!$H$5:$H$183,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$184,$A18,'QA Checklist'!$H$5:$H$184,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$184,$A18,'QA Checklist'!$H$5:$H$184,"Pass")</f>
         <v/>
       </c>
       <c r="D18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$183,$A18,'QA Checklist'!$H$5:$H$183,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$183,$A18,'QA Checklist'!$H$5:$H$183,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$184,$A18,'QA Checklist'!$H$5:$H$184,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$184,$A18,'QA Checklist'!$H$5:$H$184,"Fail")</f>
         <v/>
       </c>
       <c r="E18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$183,$A18,'QA Checklist'!$H$5:$H$183,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$184,$A18,'QA Checklist'!$H$5:$H$184,"Pending")</f>
         <v/>
       </c>
       <c r="F18" s="8">
@@ -860,19 +860,19 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$183,$A19)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$184,$A19)</f>
         <v/>
       </c>
       <c r="C19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$183,$A19,'QA Checklist'!$H$5:$H$183,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$183,$A19,'QA Checklist'!$H$5:$H$183,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$184,$A19,'QA Checklist'!$H$5:$H$184,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$184,$A19,'QA Checklist'!$H$5:$H$184,"Pass")</f>
         <v/>
       </c>
       <c r="D19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$183,$A19,'QA Checklist'!$H$5:$H$183,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$183,$A19,'QA Checklist'!$H$5:$H$183,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$184,$A19,'QA Checklist'!$H$5:$H$184,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$184,$A19,'QA Checklist'!$H$5:$H$184,"Fail")</f>
         <v/>
       </c>
       <c r="E19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$183,$A19,'QA Checklist'!$H$5:$H$183,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$184,$A19,'QA Checklist'!$H$5:$H$184,"Pending")</f>
         <v/>
       </c>
       <c r="F19" s="8">
@@ -887,19 +887,19 @@
         </is>
       </c>
       <c r="B20" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$183,$A20)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$184,$A20)</f>
         <v/>
       </c>
       <c r="C20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$183,$A20,'QA Checklist'!$H$5:$H$183,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$183,$A20,'QA Checklist'!$H$5:$H$183,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$184,$A20,'QA Checklist'!$H$5:$H$184,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$184,$A20,'QA Checklist'!$H$5:$H$184,"Pass")</f>
         <v/>
       </c>
       <c r="D20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$183,$A20,'QA Checklist'!$H$5:$H$183,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$183,$A20,'QA Checklist'!$H$5:$H$183,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$184,$A20,'QA Checklist'!$H$5:$H$184,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$184,$A20,'QA Checklist'!$H$5:$H$184,"Fail")</f>
         <v/>
       </c>
       <c r="E20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$183,$A20,'QA Checklist'!$H$5:$H$183,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$184,$A20,'QA Checklist'!$H$5:$H$184,"Pending")</f>
         <v/>
       </c>
       <c r="F20" s="8">
@@ -914,19 +914,19 @@
         </is>
       </c>
       <c r="B21" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$183,$A21)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$184,$A21)</f>
         <v/>
       </c>
       <c r="C21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$183,$A21,'QA Checklist'!$H$5:$H$183,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$183,$A21,'QA Checklist'!$H$5:$H$183,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$184,$A21,'QA Checklist'!$H$5:$H$184,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$184,$A21,'QA Checklist'!$H$5:$H$184,"Pass")</f>
         <v/>
       </c>
       <c r="D21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$183,$A21,'QA Checklist'!$H$5:$H$183,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$183,$A21,'QA Checklist'!$H$5:$H$183,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$184,$A21,'QA Checklist'!$H$5:$H$184,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$184,$A21,'QA Checklist'!$H$5:$H$184,"Fail")</f>
         <v/>
       </c>
       <c r="E21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$183,$A21,'QA Checklist'!$H$5:$H$183,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$184,$A21,'QA Checklist'!$H$5:$H$184,"Pending")</f>
         <v/>
       </c>
       <c r="F21" s="8">
@@ -941,19 +941,19 @@
         </is>
       </c>
       <c r="B22" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$183,$A22)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$184,$A22)</f>
         <v/>
       </c>
       <c r="C22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$183,$A22,'QA Checklist'!$H$5:$H$183,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$183,$A22,'QA Checklist'!$H$5:$H$183,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$184,$A22,'QA Checklist'!$H$5:$H$184,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$184,$A22,'QA Checklist'!$H$5:$H$184,"Pass")</f>
         <v/>
       </c>
       <c r="D22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$183,$A22,'QA Checklist'!$H$5:$H$183,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$183,$A22,'QA Checklist'!$H$5:$H$183,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$184,$A22,'QA Checklist'!$H$5:$H$184,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$184,$A22,'QA Checklist'!$H$5:$H$184,"Fail")</f>
         <v/>
       </c>
       <c r="E22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$183,$A22,'QA Checklist'!$H$5:$H$183,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$184,$A22,'QA Checklist'!$H$5:$H$184,"Pending")</f>
         <v/>
       </c>
       <c r="F22" s="8">
@@ -1023,19 +1023,19 @@
         </is>
       </c>
       <c r="B26" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$183,$A26&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$184,$A26&amp;"*")</f>
         <v/>
       </c>
       <c r="C26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$183,$A26&amp;"*",'QA Checklist'!$H$5:$H$183,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$183,$A26&amp;"*",'QA Checklist'!$H$5:$H$183,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$184,$A26&amp;"*",'QA Checklist'!$H$5:$H$184,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$184,$A26&amp;"*",'QA Checklist'!$H$5:$H$184,"Pass")</f>
         <v/>
       </c>
       <c r="D26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$183,$A26&amp;"*",'QA Checklist'!$H$5:$H$183,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$183,$A26&amp;"*",'QA Checklist'!$H$5:$H$183,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$184,$A26&amp;"*",'QA Checklist'!$H$5:$H$184,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$184,$A26&amp;"*",'QA Checklist'!$H$5:$H$184,"Fail")</f>
         <v/>
       </c>
       <c r="E26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$183,$A26&amp;"*",'QA Checklist'!$H$5:$H$183,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$184,$A26&amp;"*",'QA Checklist'!$H$5:$H$184,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1046,19 +1046,19 @@
         </is>
       </c>
       <c r="B27" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$183,$A27&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$184,$A27&amp;"*")</f>
         <v/>
       </c>
       <c r="C27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$183,$A27&amp;"*",'QA Checklist'!$H$5:$H$183,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$183,$A27&amp;"*",'QA Checklist'!$H$5:$H$183,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$184,$A27&amp;"*",'QA Checklist'!$H$5:$H$184,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$184,$A27&amp;"*",'QA Checklist'!$H$5:$H$184,"Pass")</f>
         <v/>
       </c>
       <c r="D27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$183,$A27&amp;"*",'QA Checklist'!$H$5:$H$183,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$183,$A27&amp;"*",'QA Checklist'!$H$5:$H$183,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$184,$A27&amp;"*",'QA Checklist'!$H$5:$H$184,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$184,$A27&amp;"*",'QA Checklist'!$H$5:$H$184,"Fail")</f>
         <v/>
       </c>
       <c r="E27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$183,$A27&amp;"*",'QA Checklist'!$H$5:$H$183,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$184,$A27&amp;"*",'QA Checklist'!$H$5:$H$184,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1069,19 +1069,19 @@
         </is>
       </c>
       <c r="B28" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$183,$A28&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$184,$A28&amp;"*")</f>
         <v/>
       </c>
       <c r="C28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$183,$A28&amp;"*",'QA Checklist'!$H$5:$H$183,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$183,$A28&amp;"*",'QA Checklist'!$H$5:$H$183,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$184,$A28&amp;"*",'QA Checklist'!$H$5:$H$184,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$184,$A28&amp;"*",'QA Checklist'!$H$5:$H$184,"Pass")</f>
         <v/>
       </c>
       <c r="D28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$183,$A28&amp;"*",'QA Checklist'!$H$5:$H$183,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$183,$A28&amp;"*",'QA Checklist'!$H$5:$H$183,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$184,$A28&amp;"*",'QA Checklist'!$H$5:$H$184,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$184,$A28&amp;"*",'QA Checklist'!$H$5:$H$184,"Fail")</f>
         <v/>
       </c>
       <c r="E28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$183,$A28&amp;"*",'QA Checklist'!$H$5:$H$183,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$184,$A28&amp;"*",'QA Checklist'!$H$5:$H$184,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1096,7 +1096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I183"/>
+  <dimension ref="A1:I184"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9140,12 +9140,59 @@
         </is>
       </c>
     </row>
+    <row r="184">
+      <c r="A184" s="12" t="inlineStr">
+        <is>
+          <t>SA-58</t>
+        </is>
+      </c>
+      <c r="B184" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="C184" s="13" t="inlineStr">
+        <is>
+          <t>Tier 2 (Workflow &amp; Ergonomics)</t>
+        </is>
+      </c>
+      <c r="D184" s="13" t="inlineStr">
+        <is>
+          <t>Document Arrows in PDF Views</t>
+        </is>
+      </c>
+      <c r="E184" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="F184" s="13" t="inlineStr">
+        <is>
+          <t>Log in as Service Advisor, open 2025 RO Excel Studio, use the ‹ › arrows in the PDF toolbar (also with Maximize on), open Full PDF and use its arrows and the Left / Right keys, then close the viewer</t>
+        </is>
+      </c>
+      <c r="G184" s="13" t="inlineStr">
+        <is>
+          <t>Arrows move Job_Order -&gt; Quotation_No -&gt; Billing_No -&gt; CheckList_Result and wrap around; the n / 4 indicator matches; in Full PDF the next document opens in the viewer and closing it leaves the studio on that document</t>
+        </is>
+      </c>
+      <c r="H184" s="14" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="I184" s="13" t="inlineStr">
+        <is>
+          <t>Verified by Automated Unit Tests (170 passing in tests/frontend/sla_and_logic.test.js AUT-FRONT-141) and a real-time headless Chrome navigation check</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:I183"/>
+  <autoFilter ref="A4:I184"/>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="H5:H183">
+  <conditionalFormatting sqref="H5:H184">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$H5="Passed"</formula>
     </cfRule>
@@ -9162,13 +9209,13 @@
       <formula>$H5="Pending"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A5:A183">
+  <conditionalFormatting sqref="A5:A184">
     <cfRule type="expression" priority="6" dxfId="3">
-      <formula>COUNTIF($A$5:$A$183,$A5)&gt;1</formula>
+      <formula>COUNTIF($A$5:$A$184,$A5)&gt;1</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H5:H183" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H5:H184" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pending,Passed,Failed"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat(REV-183): remove Print buttons from the PDF toolbar and Full PDF viewers
Remove "Print Form 1/3" from the Job_Order studio PDF toolbar and the
Print buttons from the Job Order / Checklist Full PDF headers; the PDF
viewer has its own print button. Top tab bar print unchanged.
Cache buster v=3.36, AUT-FRONT-142, SA-59.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
+++ b/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
@@ -11,7 +11,7 @@
     <sheet name="QA Checklist" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$184</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$185</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'QA Checklist'!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTA('QA Checklist'!$A$5:$A$184)</f>
+        <f>COUNTA('QA Checklist'!$A$5:$A$185)</f>
         <v/>
       </c>
     </row>
@@ -594,7 +594,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$184,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$184,"Pass")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$185,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$185,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$184,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$184,"Fail")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$185,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$185,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -616,7 +616,7 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$184,"Pending")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$185,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -671,19 +671,19 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$184,$A12)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$185,$A12)</f>
         <v/>
       </c>
       <c r="C12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$184,$A12,'QA Checklist'!$H$5:$H$184,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$184,$A12,'QA Checklist'!$H$5:$H$184,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$185,$A12,'QA Checklist'!$H$5:$H$185,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$185,$A12,'QA Checklist'!$H$5:$H$185,"Pass")</f>
         <v/>
       </c>
       <c r="D12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$184,$A12,'QA Checklist'!$H$5:$H$184,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$184,$A12,'QA Checklist'!$H$5:$H$184,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$185,$A12,'QA Checklist'!$H$5:$H$185,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$185,$A12,'QA Checklist'!$H$5:$H$185,"Fail")</f>
         <v/>
       </c>
       <c r="E12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$184,$A12,'QA Checklist'!$H$5:$H$184,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$185,$A12,'QA Checklist'!$H$5:$H$185,"Pending")</f>
         <v/>
       </c>
       <c r="F12" s="8">
@@ -698,19 +698,19 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$184,$A13)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$185,$A13)</f>
         <v/>
       </c>
       <c r="C13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$184,$A13,'QA Checklist'!$H$5:$H$184,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$184,$A13,'QA Checklist'!$H$5:$H$184,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$185,$A13,'QA Checklist'!$H$5:$H$185,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$185,$A13,'QA Checklist'!$H$5:$H$185,"Pass")</f>
         <v/>
       </c>
       <c r="D13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$184,$A13,'QA Checklist'!$H$5:$H$184,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$184,$A13,'QA Checklist'!$H$5:$H$184,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$185,$A13,'QA Checklist'!$H$5:$H$185,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$185,$A13,'QA Checklist'!$H$5:$H$185,"Fail")</f>
         <v/>
       </c>
       <c r="E13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$184,$A13,'QA Checklist'!$H$5:$H$184,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$185,$A13,'QA Checklist'!$H$5:$H$185,"Pending")</f>
         <v/>
       </c>
       <c r="F13" s="8">
@@ -725,19 +725,19 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$184,$A14)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$185,$A14)</f>
         <v/>
       </c>
       <c r="C14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$184,$A14,'QA Checklist'!$H$5:$H$184,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$184,$A14,'QA Checklist'!$H$5:$H$184,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$185,$A14,'QA Checklist'!$H$5:$H$185,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$185,$A14,'QA Checklist'!$H$5:$H$185,"Pass")</f>
         <v/>
       </c>
       <c r="D14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$184,$A14,'QA Checklist'!$H$5:$H$184,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$184,$A14,'QA Checklist'!$H$5:$H$184,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$185,$A14,'QA Checklist'!$H$5:$H$185,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$185,$A14,'QA Checklist'!$H$5:$H$185,"Fail")</f>
         <v/>
       </c>
       <c r="E14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$184,$A14,'QA Checklist'!$H$5:$H$184,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$185,$A14,'QA Checklist'!$H$5:$H$185,"Pending")</f>
         <v/>
       </c>
       <c r="F14" s="8">
@@ -752,19 +752,19 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$184,$A15)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$185,$A15)</f>
         <v/>
       </c>
       <c r="C15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$184,$A15,'QA Checklist'!$H$5:$H$184,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$184,$A15,'QA Checklist'!$H$5:$H$184,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$185,$A15,'QA Checklist'!$H$5:$H$185,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$185,$A15,'QA Checklist'!$H$5:$H$185,"Pass")</f>
         <v/>
       </c>
       <c r="D15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$184,$A15,'QA Checklist'!$H$5:$H$184,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$184,$A15,'QA Checklist'!$H$5:$H$184,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$185,$A15,'QA Checklist'!$H$5:$H$185,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$185,$A15,'QA Checklist'!$H$5:$H$185,"Fail")</f>
         <v/>
       </c>
       <c r="E15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$184,$A15,'QA Checklist'!$H$5:$H$184,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$185,$A15,'QA Checklist'!$H$5:$H$185,"Pending")</f>
         <v/>
       </c>
       <c r="F15" s="8">
@@ -779,19 +779,19 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$184,$A16)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$185,$A16)</f>
         <v/>
       </c>
       <c r="C16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$184,$A16,'QA Checklist'!$H$5:$H$184,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$184,$A16,'QA Checklist'!$H$5:$H$184,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$185,$A16,'QA Checklist'!$H$5:$H$185,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$185,$A16,'QA Checklist'!$H$5:$H$185,"Pass")</f>
         <v/>
       </c>
       <c r="D16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$184,$A16,'QA Checklist'!$H$5:$H$184,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$184,$A16,'QA Checklist'!$H$5:$H$184,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$185,$A16,'QA Checklist'!$H$5:$H$185,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$185,$A16,'QA Checklist'!$H$5:$H$185,"Fail")</f>
         <v/>
       </c>
       <c r="E16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$184,$A16,'QA Checklist'!$H$5:$H$184,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$185,$A16,'QA Checklist'!$H$5:$H$185,"Pending")</f>
         <v/>
       </c>
       <c r="F16" s="8">
@@ -806,19 +806,19 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$184,$A17)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$185,$A17)</f>
         <v/>
       </c>
       <c r="C17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$184,$A17,'QA Checklist'!$H$5:$H$184,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$184,$A17,'QA Checklist'!$H$5:$H$184,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$185,$A17,'QA Checklist'!$H$5:$H$185,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$185,$A17,'QA Checklist'!$H$5:$H$185,"Pass")</f>
         <v/>
       </c>
       <c r="D17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$184,$A17,'QA Checklist'!$H$5:$H$184,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$184,$A17,'QA Checklist'!$H$5:$H$184,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$185,$A17,'QA Checklist'!$H$5:$H$185,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$185,$A17,'QA Checklist'!$H$5:$H$185,"Fail")</f>
         <v/>
       </c>
       <c r="E17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$184,$A17,'QA Checklist'!$H$5:$H$184,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$185,$A17,'QA Checklist'!$H$5:$H$185,"Pending")</f>
         <v/>
       </c>
       <c r="F17" s="8">
@@ -833,19 +833,19 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$184,$A18)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$185,$A18)</f>
         <v/>
       </c>
       <c r="C18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$184,$A18,'QA Checklist'!$H$5:$H$184,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$184,$A18,'QA Checklist'!$H$5:$H$184,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$185,$A18,'QA Checklist'!$H$5:$H$185,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$185,$A18,'QA Checklist'!$H$5:$H$185,"Pass")</f>
         <v/>
       </c>
       <c r="D18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$184,$A18,'QA Checklist'!$H$5:$H$184,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$184,$A18,'QA Checklist'!$H$5:$H$184,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$185,$A18,'QA Checklist'!$H$5:$H$185,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$185,$A18,'QA Checklist'!$H$5:$H$185,"Fail")</f>
         <v/>
       </c>
       <c r="E18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$184,$A18,'QA Checklist'!$H$5:$H$184,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$185,$A18,'QA Checklist'!$H$5:$H$185,"Pending")</f>
         <v/>
       </c>
       <c r="F18" s="8">
@@ -860,19 +860,19 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$184,$A19)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$185,$A19)</f>
         <v/>
       </c>
       <c r="C19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$184,$A19,'QA Checklist'!$H$5:$H$184,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$184,$A19,'QA Checklist'!$H$5:$H$184,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$185,$A19,'QA Checklist'!$H$5:$H$185,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$185,$A19,'QA Checklist'!$H$5:$H$185,"Pass")</f>
         <v/>
       </c>
       <c r="D19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$184,$A19,'QA Checklist'!$H$5:$H$184,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$184,$A19,'QA Checklist'!$H$5:$H$184,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$185,$A19,'QA Checklist'!$H$5:$H$185,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$185,$A19,'QA Checklist'!$H$5:$H$185,"Fail")</f>
         <v/>
       </c>
       <c r="E19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$184,$A19,'QA Checklist'!$H$5:$H$184,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$185,$A19,'QA Checklist'!$H$5:$H$185,"Pending")</f>
         <v/>
       </c>
       <c r="F19" s="8">
@@ -887,19 +887,19 @@
         </is>
       </c>
       <c r="B20" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$184,$A20)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$185,$A20)</f>
         <v/>
       </c>
       <c r="C20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$184,$A20,'QA Checklist'!$H$5:$H$184,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$184,$A20,'QA Checklist'!$H$5:$H$184,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$185,$A20,'QA Checklist'!$H$5:$H$185,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$185,$A20,'QA Checklist'!$H$5:$H$185,"Pass")</f>
         <v/>
       </c>
       <c r="D20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$184,$A20,'QA Checklist'!$H$5:$H$184,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$184,$A20,'QA Checklist'!$H$5:$H$184,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$185,$A20,'QA Checklist'!$H$5:$H$185,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$185,$A20,'QA Checklist'!$H$5:$H$185,"Fail")</f>
         <v/>
       </c>
       <c r="E20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$184,$A20,'QA Checklist'!$H$5:$H$184,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$185,$A20,'QA Checklist'!$H$5:$H$185,"Pending")</f>
         <v/>
       </c>
       <c r="F20" s="8">
@@ -914,19 +914,19 @@
         </is>
       </c>
       <c r="B21" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$184,$A21)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$185,$A21)</f>
         <v/>
       </c>
       <c r="C21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$184,$A21,'QA Checklist'!$H$5:$H$184,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$184,$A21,'QA Checklist'!$H$5:$H$184,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$185,$A21,'QA Checklist'!$H$5:$H$185,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$185,$A21,'QA Checklist'!$H$5:$H$185,"Pass")</f>
         <v/>
       </c>
       <c r="D21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$184,$A21,'QA Checklist'!$H$5:$H$184,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$184,$A21,'QA Checklist'!$H$5:$H$184,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$185,$A21,'QA Checklist'!$H$5:$H$185,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$185,$A21,'QA Checklist'!$H$5:$H$185,"Fail")</f>
         <v/>
       </c>
       <c r="E21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$184,$A21,'QA Checklist'!$H$5:$H$184,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$185,$A21,'QA Checklist'!$H$5:$H$185,"Pending")</f>
         <v/>
       </c>
       <c r="F21" s="8">
@@ -941,19 +941,19 @@
         </is>
       </c>
       <c r="B22" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$184,$A22)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$185,$A22)</f>
         <v/>
       </c>
       <c r="C22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$184,$A22,'QA Checklist'!$H$5:$H$184,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$184,$A22,'QA Checklist'!$H$5:$H$184,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$185,$A22,'QA Checklist'!$H$5:$H$185,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$185,$A22,'QA Checklist'!$H$5:$H$185,"Pass")</f>
         <v/>
       </c>
       <c r="D22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$184,$A22,'QA Checklist'!$H$5:$H$184,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$184,$A22,'QA Checklist'!$H$5:$H$184,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$185,$A22,'QA Checklist'!$H$5:$H$185,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$185,$A22,'QA Checklist'!$H$5:$H$185,"Fail")</f>
         <v/>
       </c>
       <c r="E22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$184,$A22,'QA Checklist'!$H$5:$H$184,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$185,$A22,'QA Checklist'!$H$5:$H$185,"Pending")</f>
         <v/>
       </c>
       <c r="F22" s="8">
@@ -1023,19 +1023,19 @@
         </is>
       </c>
       <c r="B26" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$184,$A26&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$185,$A26&amp;"*")</f>
         <v/>
       </c>
       <c r="C26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$184,$A26&amp;"*",'QA Checklist'!$H$5:$H$184,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$184,$A26&amp;"*",'QA Checklist'!$H$5:$H$184,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$185,$A26&amp;"*",'QA Checklist'!$H$5:$H$185,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$185,$A26&amp;"*",'QA Checklist'!$H$5:$H$185,"Pass")</f>
         <v/>
       </c>
       <c r="D26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$184,$A26&amp;"*",'QA Checklist'!$H$5:$H$184,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$184,$A26&amp;"*",'QA Checklist'!$H$5:$H$184,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$185,$A26&amp;"*",'QA Checklist'!$H$5:$H$185,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$185,$A26&amp;"*",'QA Checklist'!$H$5:$H$185,"Fail")</f>
         <v/>
       </c>
       <c r="E26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$184,$A26&amp;"*",'QA Checklist'!$H$5:$H$184,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$185,$A26&amp;"*",'QA Checklist'!$H$5:$H$185,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1046,19 +1046,19 @@
         </is>
       </c>
       <c r="B27" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$184,$A27&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$185,$A27&amp;"*")</f>
         <v/>
       </c>
       <c r="C27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$184,$A27&amp;"*",'QA Checklist'!$H$5:$H$184,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$184,$A27&amp;"*",'QA Checklist'!$H$5:$H$184,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$185,$A27&amp;"*",'QA Checklist'!$H$5:$H$185,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$185,$A27&amp;"*",'QA Checklist'!$H$5:$H$185,"Pass")</f>
         <v/>
       </c>
       <c r="D27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$184,$A27&amp;"*",'QA Checklist'!$H$5:$H$184,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$184,$A27&amp;"*",'QA Checklist'!$H$5:$H$184,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$185,$A27&amp;"*",'QA Checklist'!$H$5:$H$185,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$185,$A27&amp;"*",'QA Checklist'!$H$5:$H$185,"Fail")</f>
         <v/>
       </c>
       <c r="E27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$184,$A27&amp;"*",'QA Checklist'!$H$5:$H$184,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$185,$A27&amp;"*",'QA Checklist'!$H$5:$H$185,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1069,19 +1069,19 @@
         </is>
       </c>
       <c r="B28" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$184,$A28&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$185,$A28&amp;"*")</f>
         <v/>
       </c>
       <c r="C28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$184,$A28&amp;"*",'QA Checklist'!$H$5:$H$184,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$184,$A28&amp;"*",'QA Checklist'!$H$5:$H$184,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$185,$A28&amp;"*",'QA Checklist'!$H$5:$H$185,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$185,$A28&amp;"*",'QA Checklist'!$H$5:$H$185,"Pass")</f>
         <v/>
       </c>
       <c r="D28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$184,$A28&amp;"*",'QA Checklist'!$H$5:$H$184,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$184,$A28&amp;"*",'QA Checklist'!$H$5:$H$184,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$185,$A28&amp;"*",'QA Checklist'!$H$5:$H$185,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$185,$A28&amp;"*",'QA Checklist'!$H$5:$H$185,"Fail")</f>
         <v/>
       </c>
       <c r="E28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$184,$A28&amp;"*",'QA Checklist'!$H$5:$H$184,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$185,$A28&amp;"*",'QA Checklist'!$H$5:$H$185,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1096,7 +1096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I184"/>
+  <dimension ref="A1:I185"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9187,12 +9187,59 @@
         </is>
       </c>
     </row>
+    <row r="185">
+      <c r="A185" s="12" t="inlineStr">
+        <is>
+          <t>SA-59</t>
+        </is>
+      </c>
+      <c r="B185" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="C185" s="13" t="inlineStr">
+        <is>
+          <t>Tier 2 (Workflow &amp; Ergonomics)</t>
+        </is>
+      </c>
+      <c r="D185" s="13" t="inlineStr">
+        <is>
+          <t>No Print Buttons in PDF Views</t>
+        </is>
+      </c>
+      <c r="E185" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="F185" s="13" t="inlineStr">
+        <is>
+          <t>Log in as Service Advisor, open 2025 RO Excel Studio, look at the PDF toolbar on each tab (normal and Maximize) and open Full PDF for each document</t>
+        </is>
+      </c>
+      <c r="G185" s="13" t="inlineStr">
+        <is>
+          <t>No Print Form 1/3 / Print Checklist buttons in the PDF toolbars or Full PDF headers; printing is done from the PDF viewer print button</t>
+        </is>
+      </c>
+      <c r="H185" s="14" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="I185" s="13" t="inlineStr">
+        <is>
+          <t>Verified by Automated Unit Tests (171 passing in tests/frontend/sla_and_logic.test.js AUT-FRONT-142) and a headless Chrome render</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:I184"/>
+  <autoFilter ref="A4:I185"/>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="H5:H184">
+  <conditionalFormatting sqref="H5:H185">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$H5="Passed"</formula>
     </cfRule>
@@ -9209,13 +9256,13 @@
       <formula>$H5="Pending"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A5:A184">
+  <conditionalFormatting sqref="A5:A185">
     <cfRule type="expression" priority="6" dxfId="3">
-      <formula>COUNTIF($A$5:$A$184,$A5)&gt;1</formula>
+      <formula>COUNTIF($A$5:$A$185,$A5)&gt;1</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H5:H184" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H5:H185" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pending,Passed,Failed"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat(REV-184): remove the Import .xlsx button and logic
Remove the Import .xlsx button, importOfficialXLSX() and the SheetJS
script tag (used only by the import; vendor file kept for later).
Export .xlsx is unchanged. Cache buster v=3.37, AUT-FRONT-143, SA-60.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
+++ b/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
@@ -11,7 +11,7 @@
     <sheet name="QA Checklist" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$185</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$186</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'QA Checklist'!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTA('QA Checklist'!$A$5:$A$185)</f>
+        <f>COUNTA('QA Checklist'!$A$5:$A$186)</f>
         <v/>
       </c>
     </row>
@@ -594,7 +594,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$185,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$185,"Pass")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$186,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$186,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$185,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$185,"Fail")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$186,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$186,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -616,7 +616,7 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$185,"Pending")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$186,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -671,19 +671,19 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$185,$A12)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$186,$A12)</f>
         <v/>
       </c>
       <c r="C12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$185,$A12,'QA Checklist'!$H$5:$H$185,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$185,$A12,'QA Checklist'!$H$5:$H$185,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$186,$A12,'QA Checklist'!$H$5:$H$186,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$186,$A12,'QA Checklist'!$H$5:$H$186,"Pass")</f>
         <v/>
       </c>
       <c r="D12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$185,$A12,'QA Checklist'!$H$5:$H$185,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$185,$A12,'QA Checklist'!$H$5:$H$185,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$186,$A12,'QA Checklist'!$H$5:$H$186,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$186,$A12,'QA Checklist'!$H$5:$H$186,"Fail")</f>
         <v/>
       </c>
       <c r="E12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$185,$A12,'QA Checklist'!$H$5:$H$185,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$186,$A12,'QA Checklist'!$H$5:$H$186,"Pending")</f>
         <v/>
       </c>
       <c r="F12" s="8">
@@ -698,19 +698,19 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$185,$A13)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$186,$A13)</f>
         <v/>
       </c>
       <c r="C13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$185,$A13,'QA Checklist'!$H$5:$H$185,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$185,$A13,'QA Checklist'!$H$5:$H$185,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$186,$A13,'QA Checklist'!$H$5:$H$186,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$186,$A13,'QA Checklist'!$H$5:$H$186,"Pass")</f>
         <v/>
       </c>
       <c r="D13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$185,$A13,'QA Checklist'!$H$5:$H$185,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$185,$A13,'QA Checklist'!$H$5:$H$185,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$186,$A13,'QA Checklist'!$H$5:$H$186,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$186,$A13,'QA Checklist'!$H$5:$H$186,"Fail")</f>
         <v/>
       </c>
       <c r="E13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$185,$A13,'QA Checklist'!$H$5:$H$185,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$186,$A13,'QA Checklist'!$H$5:$H$186,"Pending")</f>
         <v/>
       </c>
       <c r="F13" s="8">
@@ -725,19 +725,19 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$185,$A14)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$186,$A14)</f>
         <v/>
       </c>
       <c r="C14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$185,$A14,'QA Checklist'!$H$5:$H$185,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$185,$A14,'QA Checklist'!$H$5:$H$185,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$186,$A14,'QA Checklist'!$H$5:$H$186,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$186,$A14,'QA Checklist'!$H$5:$H$186,"Pass")</f>
         <v/>
       </c>
       <c r="D14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$185,$A14,'QA Checklist'!$H$5:$H$185,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$185,$A14,'QA Checklist'!$H$5:$H$185,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$186,$A14,'QA Checklist'!$H$5:$H$186,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$186,$A14,'QA Checklist'!$H$5:$H$186,"Fail")</f>
         <v/>
       </c>
       <c r="E14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$185,$A14,'QA Checklist'!$H$5:$H$185,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$186,$A14,'QA Checklist'!$H$5:$H$186,"Pending")</f>
         <v/>
       </c>
       <c r="F14" s="8">
@@ -752,19 +752,19 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$185,$A15)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$186,$A15)</f>
         <v/>
       </c>
       <c r="C15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$185,$A15,'QA Checklist'!$H$5:$H$185,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$185,$A15,'QA Checklist'!$H$5:$H$185,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$186,$A15,'QA Checklist'!$H$5:$H$186,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$186,$A15,'QA Checklist'!$H$5:$H$186,"Pass")</f>
         <v/>
       </c>
       <c r="D15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$185,$A15,'QA Checklist'!$H$5:$H$185,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$185,$A15,'QA Checklist'!$H$5:$H$185,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$186,$A15,'QA Checklist'!$H$5:$H$186,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$186,$A15,'QA Checklist'!$H$5:$H$186,"Fail")</f>
         <v/>
       </c>
       <c r="E15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$185,$A15,'QA Checklist'!$H$5:$H$185,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$186,$A15,'QA Checklist'!$H$5:$H$186,"Pending")</f>
         <v/>
       </c>
       <c r="F15" s="8">
@@ -779,19 +779,19 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$185,$A16)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$186,$A16)</f>
         <v/>
       </c>
       <c r="C16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$185,$A16,'QA Checklist'!$H$5:$H$185,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$185,$A16,'QA Checklist'!$H$5:$H$185,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$186,$A16,'QA Checklist'!$H$5:$H$186,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$186,$A16,'QA Checklist'!$H$5:$H$186,"Pass")</f>
         <v/>
       </c>
       <c r="D16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$185,$A16,'QA Checklist'!$H$5:$H$185,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$185,$A16,'QA Checklist'!$H$5:$H$185,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$186,$A16,'QA Checklist'!$H$5:$H$186,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$186,$A16,'QA Checklist'!$H$5:$H$186,"Fail")</f>
         <v/>
       </c>
       <c r="E16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$185,$A16,'QA Checklist'!$H$5:$H$185,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$186,$A16,'QA Checklist'!$H$5:$H$186,"Pending")</f>
         <v/>
       </c>
       <c r="F16" s="8">
@@ -806,19 +806,19 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$185,$A17)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$186,$A17)</f>
         <v/>
       </c>
       <c r="C17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$185,$A17,'QA Checklist'!$H$5:$H$185,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$185,$A17,'QA Checklist'!$H$5:$H$185,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$186,$A17,'QA Checklist'!$H$5:$H$186,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$186,$A17,'QA Checklist'!$H$5:$H$186,"Pass")</f>
         <v/>
       </c>
       <c r="D17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$185,$A17,'QA Checklist'!$H$5:$H$185,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$185,$A17,'QA Checklist'!$H$5:$H$185,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$186,$A17,'QA Checklist'!$H$5:$H$186,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$186,$A17,'QA Checklist'!$H$5:$H$186,"Fail")</f>
         <v/>
       </c>
       <c r="E17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$185,$A17,'QA Checklist'!$H$5:$H$185,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$186,$A17,'QA Checklist'!$H$5:$H$186,"Pending")</f>
         <v/>
       </c>
       <c r="F17" s="8">
@@ -833,19 +833,19 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$185,$A18)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$186,$A18)</f>
         <v/>
       </c>
       <c r="C18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$185,$A18,'QA Checklist'!$H$5:$H$185,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$185,$A18,'QA Checklist'!$H$5:$H$185,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$186,$A18,'QA Checklist'!$H$5:$H$186,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$186,$A18,'QA Checklist'!$H$5:$H$186,"Pass")</f>
         <v/>
       </c>
       <c r="D18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$185,$A18,'QA Checklist'!$H$5:$H$185,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$185,$A18,'QA Checklist'!$H$5:$H$185,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$186,$A18,'QA Checklist'!$H$5:$H$186,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$186,$A18,'QA Checklist'!$H$5:$H$186,"Fail")</f>
         <v/>
       </c>
       <c r="E18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$185,$A18,'QA Checklist'!$H$5:$H$185,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$186,$A18,'QA Checklist'!$H$5:$H$186,"Pending")</f>
         <v/>
       </c>
       <c r="F18" s="8">
@@ -860,19 +860,19 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$185,$A19)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$186,$A19)</f>
         <v/>
       </c>
       <c r="C19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$185,$A19,'QA Checklist'!$H$5:$H$185,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$185,$A19,'QA Checklist'!$H$5:$H$185,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$186,$A19,'QA Checklist'!$H$5:$H$186,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$186,$A19,'QA Checklist'!$H$5:$H$186,"Pass")</f>
         <v/>
       </c>
       <c r="D19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$185,$A19,'QA Checklist'!$H$5:$H$185,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$185,$A19,'QA Checklist'!$H$5:$H$185,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$186,$A19,'QA Checklist'!$H$5:$H$186,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$186,$A19,'QA Checklist'!$H$5:$H$186,"Fail")</f>
         <v/>
       </c>
       <c r="E19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$185,$A19,'QA Checklist'!$H$5:$H$185,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$186,$A19,'QA Checklist'!$H$5:$H$186,"Pending")</f>
         <v/>
       </c>
       <c r="F19" s="8">
@@ -887,19 +887,19 @@
         </is>
       </c>
       <c r="B20" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$185,$A20)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$186,$A20)</f>
         <v/>
       </c>
       <c r="C20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$185,$A20,'QA Checklist'!$H$5:$H$185,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$185,$A20,'QA Checklist'!$H$5:$H$185,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$186,$A20,'QA Checklist'!$H$5:$H$186,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$186,$A20,'QA Checklist'!$H$5:$H$186,"Pass")</f>
         <v/>
       </c>
       <c r="D20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$185,$A20,'QA Checklist'!$H$5:$H$185,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$185,$A20,'QA Checklist'!$H$5:$H$185,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$186,$A20,'QA Checklist'!$H$5:$H$186,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$186,$A20,'QA Checklist'!$H$5:$H$186,"Fail")</f>
         <v/>
       </c>
       <c r="E20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$185,$A20,'QA Checklist'!$H$5:$H$185,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$186,$A20,'QA Checklist'!$H$5:$H$186,"Pending")</f>
         <v/>
       </c>
       <c r="F20" s="8">
@@ -914,19 +914,19 @@
         </is>
       </c>
       <c r="B21" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$185,$A21)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$186,$A21)</f>
         <v/>
       </c>
       <c r="C21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$185,$A21,'QA Checklist'!$H$5:$H$185,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$185,$A21,'QA Checklist'!$H$5:$H$185,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$186,$A21,'QA Checklist'!$H$5:$H$186,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$186,$A21,'QA Checklist'!$H$5:$H$186,"Pass")</f>
         <v/>
       </c>
       <c r="D21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$185,$A21,'QA Checklist'!$H$5:$H$185,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$185,$A21,'QA Checklist'!$H$5:$H$185,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$186,$A21,'QA Checklist'!$H$5:$H$186,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$186,$A21,'QA Checklist'!$H$5:$H$186,"Fail")</f>
         <v/>
       </c>
       <c r="E21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$185,$A21,'QA Checklist'!$H$5:$H$185,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$186,$A21,'QA Checklist'!$H$5:$H$186,"Pending")</f>
         <v/>
       </c>
       <c r="F21" s="8">
@@ -941,19 +941,19 @@
         </is>
       </c>
       <c r="B22" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$185,$A22)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$186,$A22)</f>
         <v/>
       </c>
       <c r="C22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$185,$A22,'QA Checklist'!$H$5:$H$185,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$185,$A22,'QA Checklist'!$H$5:$H$185,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$186,$A22,'QA Checklist'!$H$5:$H$186,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$186,$A22,'QA Checklist'!$H$5:$H$186,"Pass")</f>
         <v/>
       </c>
       <c r="D22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$185,$A22,'QA Checklist'!$H$5:$H$185,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$185,$A22,'QA Checklist'!$H$5:$H$185,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$186,$A22,'QA Checklist'!$H$5:$H$186,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$186,$A22,'QA Checklist'!$H$5:$H$186,"Fail")</f>
         <v/>
       </c>
       <c r="E22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$185,$A22,'QA Checklist'!$H$5:$H$185,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$186,$A22,'QA Checklist'!$H$5:$H$186,"Pending")</f>
         <v/>
       </c>
       <c r="F22" s="8">
@@ -1023,19 +1023,19 @@
         </is>
       </c>
       <c r="B26" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$185,$A26&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$186,$A26&amp;"*")</f>
         <v/>
       </c>
       <c r="C26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$185,$A26&amp;"*",'QA Checklist'!$H$5:$H$185,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$185,$A26&amp;"*",'QA Checklist'!$H$5:$H$185,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$186,$A26&amp;"*",'QA Checklist'!$H$5:$H$186,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$186,$A26&amp;"*",'QA Checklist'!$H$5:$H$186,"Pass")</f>
         <v/>
       </c>
       <c r="D26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$185,$A26&amp;"*",'QA Checklist'!$H$5:$H$185,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$185,$A26&amp;"*",'QA Checklist'!$H$5:$H$185,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$186,$A26&amp;"*",'QA Checklist'!$H$5:$H$186,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$186,$A26&amp;"*",'QA Checklist'!$H$5:$H$186,"Fail")</f>
         <v/>
       </c>
       <c r="E26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$185,$A26&amp;"*",'QA Checklist'!$H$5:$H$185,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$186,$A26&amp;"*",'QA Checklist'!$H$5:$H$186,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1046,19 +1046,19 @@
         </is>
       </c>
       <c r="B27" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$185,$A27&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$186,$A27&amp;"*")</f>
         <v/>
       </c>
       <c r="C27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$185,$A27&amp;"*",'QA Checklist'!$H$5:$H$185,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$185,$A27&amp;"*",'QA Checklist'!$H$5:$H$185,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$186,$A27&amp;"*",'QA Checklist'!$H$5:$H$186,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$186,$A27&amp;"*",'QA Checklist'!$H$5:$H$186,"Pass")</f>
         <v/>
       </c>
       <c r="D27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$185,$A27&amp;"*",'QA Checklist'!$H$5:$H$185,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$185,$A27&amp;"*",'QA Checklist'!$H$5:$H$185,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$186,$A27&amp;"*",'QA Checklist'!$H$5:$H$186,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$186,$A27&amp;"*",'QA Checklist'!$H$5:$H$186,"Fail")</f>
         <v/>
       </c>
       <c r="E27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$185,$A27&amp;"*",'QA Checklist'!$H$5:$H$185,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$186,$A27&amp;"*",'QA Checklist'!$H$5:$H$186,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1069,19 +1069,19 @@
         </is>
       </c>
       <c r="B28" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$185,$A28&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$186,$A28&amp;"*")</f>
         <v/>
       </c>
       <c r="C28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$185,$A28&amp;"*",'QA Checklist'!$H$5:$H$185,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$185,$A28&amp;"*",'QA Checklist'!$H$5:$H$185,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$186,$A28&amp;"*",'QA Checklist'!$H$5:$H$186,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$186,$A28&amp;"*",'QA Checklist'!$H$5:$H$186,"Pass")</f>
         <v/>
       </c>
       <c r="D28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$185,$A28&amp;"*",'QA Checklist'!$H$5:$H$185,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$185,$A28&amp;"*",'QA Checklist'!$H$5:$H$185,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$186,$A28&amp;"*",'QA Checklist'!$H$5:$H$186,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$186,$A28&amp;"*",'QA Checklist'!$H$5:$H$186,"Fail")</f>
         <v/>
       </c>
       <c r="E28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$185,$A28&amp;"*",'QA Checklist'!$H$5:$H$185,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$186,$A28&amp;"*",'QA Checklist'!$H$5:$H$186,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1096,7 +1096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I185"/>
+  <dimension ref="A1:I186"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9234,12 +9234,59 @@
         </is>
       </c>
     </row>
+    <row r="186">
+      <c r="A186" s="12" t="inlineStr">
+        <is>
+          <t>SA-60</t>
+        </is>
+      </c>
+      <c r="B186" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="C186" s="13" t="inlineStr">
+        <is>
+          <t>Tier 2 (Workflow &amp; Ergonomics)</t>
+        </is>
+      </c>
+      <c r="D186" s="13" t="inlineStr">
+        <is>
+          <t>Excel Import Removed</t>
+        </is>
+      </c>
+      <c r="E186" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="F186" s="13" t="inlineStr">
+        <is>
+          <t>Log in as Service Advisor, open 2025 RO Excel Studio &gt; Job_Order and look at the studio header buttons, then press Export .xlsx</t>
+        </is>
+      </c>
+      <c r="G186" s="13" t="inlineStr">
+        <is>
+          <t>No Import .xlsx button; Save Draft, Reset Form, Export .xlsx and Register RO still shown and Export .xlsx still downloads the workbook</t>
+        </is>
+      </c>
+      <c r="H186" s="14" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="I186" s="13" t="inlineStr">
+        <is>
+          <t>Verified by Automated Unit Tests (172 passing in tests/frontend/sla_and_logic.test.js AUT-FRONT-143) and a headless Chrome render</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:I185"/>
+  <autoFilter ref="A4:I186"/>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="H5:H185">
+  <conditionalFormatting sqref="H5:H186">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$H5="Passed"</formula>
     </cfRule>
@@ -9256,13 +9303,13 @@
       <formula>$H5="Pending"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A5:A185">
+  <conditionalFormatting sqref="A5:A186">
     <cfRule type="expression" priority="6" dxfId="3">
-      <formula>COUNTIF($A$5:$A$185,$A5)&gt;1</formula>
+      <formula>COUNTIF($A$5:$A$186,$A5)&gt;1</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H5:H185" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H5:H186" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pending,Passed,Failed"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
fix(REV-185): TV Monitor phase 1 - Smart TV page loads on XAMPP and offline
tv.html resolves the API like the main app (project folder safe), loads Tailwind / Lucide locally, and the TV Broadcast Hub link points at frontend/tv.html. Cache buster v=3.38, AUT-FRONT-144, SA-61.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
+++ b/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
@@ -11,7 +11,7 @@
     <sheet name="QA Checklist" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$186</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$187</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'QA Checklist'!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTA('QA Checklist'!$A$5:$A$186)</f>
+        <f>COUNTA('QA Checklist'!$A$5:$A$187)</f>
         <v/>
       </c>
     </row>
@@ -594,7 +594,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$186,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$186,"Pass")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$187,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$187,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$186,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$186,"Fail")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$187,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$187,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -616,7 +616,7 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$186,"Pending")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$187,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -671,19 +671,19 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$186,$A12)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$187,$A12)</f>
         <v/>
       </c>
       <c r="C12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$186,$A12,'QA Checklist'!$H$5:$H$186,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$186,$A12,'QA Checklist'!$H$5:$H$186,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$187,$A12,'QA Checklist'!$H$5:$H$187,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$187,$A12,'QA Checklist'!$H$5:$H$187,"Pass")</f>
         <v/>
       </c>
       <c r="D12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$186,$A12,'QA Checklist'!$H$5:$H$186,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$186,$A12,'QA Checklist'!$H$5:$H$186,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$187,$A12,'QA Checklist'!$H$5:$H$187,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$187,$A12,'QA Checklist'!$H$5:$H$187,"Fail")</f>
         <v/>
       </c>
       <c r="E12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$186,$A12,'QA Checklist'!$H$5:$H$186,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$187,$A12,'QA Checklist'!$H$5:$H$187,"Pending")</f>
         <v/>
       </c>
       <c r="F12" s="8">
@@ -698,19 +698,19 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$186,$A13)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$187,$A13)</f>
         <v/>
       </c>
       <c r="C13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$186,$A13,'QA Checklist'!$H$5:$H$186,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$186,$A13,'QA Checklist'!$H$5:$H$186,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$187,$A13,'QA Checklist'!$H$5:$H$187,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$187,$A13,'QA Checklist'!$H$5:$H$187,"Pass")</f>
         <v/>
       </c>
       <c r="D13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$186,$A13,'QA Checklist'!$H$5:$H$186,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$186,$A13,'QA Checklist'!$H$5:$H$186,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$187,$A13,'QA Checklist'!$H$5:$H$187,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$187,$A13,'QA Checklist'!$H$5:$H$187,"Fail")</f>
         <v/>
       </c>
       <c r="E13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$186,$A13,'QA Checklist'!$H$5:$H$186,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$187,$A13,'QA Checklist'!$H$5:$H$187,"Pending")</f>
         <v/>
       </c>
       <c r="F13" s="8">
@@ -725,19 +725,19 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$186,$A14)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$187,$A14)</f>
         <v/>
       </c>
       <c r="C14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$186,$A14,'QA Checklist'!$H$5:$H$186,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$186,$A14,'QA Checklist'!$H$5:$H$186,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$187,$A14,'QA Checklist'!$H$5:$H$187,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$187,$A14,'QA Checklist'!$H$5:$H$187,"Pass")</f>
         <v/>
       </c>
       <c r="D14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$186,$A14,'QA Checklist'!$H$5:$H$186,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$186,$A14,'QA Checklist'!$H$5:$H$186,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$187,$A14,'QA Checklist'!$H$5:$H$187,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$187,$A14,'QA Checklist'!$H$5:$H$187,"Fail")</f>
         <v/>
       </c>
       <c r="E14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$186,$A14,'QA Checklist'!$H$5:$H$186,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$187,$A14,'QA Checklist'!$H$5:$H$187,"Pending")</f>
         <v/>
       </c>
       <c r="F14" s="8">
@@ -752,19 +752,19 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$186,$A15)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$187,$A15)</f>
         <v/>
       </c>
       <c r="C15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$186,$A15,'QA Checklist'!$H$5:$H$186,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$186,$A15,'QA Checklist'!$H$5:$H$186,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$187,$A15,'QA Checklist'!$H$5:$H$187,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$187,$A15,'QA Checklist'!$H$5:$H$187,"Pass")</f>
         <v/>
       </c>
       <c r="D15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$186,$A15,'QA Checklist'!$H$5:$H$186,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$186,$A15,'QA Checklist'!$H$5:$H$186,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$187,$A15,'QA Checklist'!$H$5:$H$187,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$187,$A15,'QA Checklist'!$H$5:$H$187,"Fail")</f>
         <v/>
       </c>
       <c r="E15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$186,$A15,'QA Checklist'!$H$5:$H$186,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$187,$A15,'QA Checklist'!$H$5:$H$187,"Pending")</f>
         <v/>
       </c>
       <c r="F15" s="8">
@@ -779,19 +779,19 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$186,$A16)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$187,$A16)</f>
         <v/>
       </c>
       <c r="C16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$186,$A16,'QA Checklist'!$H$5:$H$186,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$186,$A16,'QA Checklist'!$H$5:$H$186,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$187,$A16,'QA Checklist'!$H$5:$H$187,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$187,$A16,'QA Checklist'!$H$5:$H$187,"Pass")</f>
         <v/>
       </c>
       <c r="D16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$186,$A16,'QA Checklist'!$H$5:$H$186,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$186,$A16,'QA Checklist'!$H$5:$H$186,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$187,$A16,'QA Checklist'!$H$5:$H$187,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$187,$A16,'QA Checklist'!$H$5:$H$187,"Fail")</f>
         <v/>
       </c>
       <c r="E16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$186,$A16,'QA Checklist'!$H$5:$H$186,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$187,$A16,'QA Checklist'!$H$5:$H$187,"Pending")</f>
         <v/>
       </c>
       <c r="F16" s="8">
@@ -806,19 +806,19 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$186,$A17)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$187,$A17)</f>
         <v/>
       </c>
       <c r="C17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$186,$A17,'QA Checklist'!$H$5:$H$186,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$186,$A17,'QA Checklist'!$H$5:$H$186,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$187,$A17,'QA Checklist'!$H$5:$H$187,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$187,$A17,'QA Checklist'!$H$5:$H$187,"Pass")</f>
         <v/>
       </c>
       <c r="D17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$186,$A17,'QA Checklist'!$H$5:$H$186,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$186,$A17,'QA Checklist'!$H$5:$H$186,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$187,$A17,'QA Checklist'!$H$5:$H$187,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$187,$A17,'QA Checklist'!$H$5:$H$187,"Fail")</f>
         <v/>
       </c>
       <c r="E17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$186,$A17,'QA Checklist'!$H$5:$H$186,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$187,$A17,'QA Checklist'!$H$5:$H$187,"Pending")</f>
         <v/>
       </c>
       <c r="F17" s="8">
@@ -833,19 +833,19 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$186,$A18)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$187,$A18)</f>
         <v/>
       </c>
       <c r="C18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$186,$A18,'QA Checklist'!$H$5:$H$186,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$186,$A18,'QA Checklist'!$H$5:$H$186,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$187,$A18,'QA Checklist'!$H$5:$H$187,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$187,$A18,'QA Checklist'!$H$5:$H$187,"Pass")</f>
         <v/>
       </c>
       <c r="D18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$186,$A18,'QA Checklist'!$H$5:$H$186,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$186,$A18,'QA Checklist'!$H$5:$H$186,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$187,$A18,'QA Checklist'!$H$5:$H$187,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$187,$A18,'QA Checklist'!$H$5:$H$187,"Fail")</f>
         <v/>
       </c>
       <c r="E18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$186,$A18,'QA Checklist'!$H$5:$H$186,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$187,$A18,'QA Checklist'!$H$5:$H$187,"Pending")</f>
         <v/>
       </c>
       <c r="F18" s="8">
@@ -860,19 +860,19 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$186,$A19)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$187,$A19)</f>
         <v/>
       </c>
       <c r="C19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$186,$A19,'QA Checklist'!$H$5:$H$186,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$186,$A19,'QA Checklist'!$H$5:$H$186,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$187,$A19,'QA Checklist'!$H$5:$H$187,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$187,$A19,'QA Checklist'!$H$5:$H$187,"Pass")</f>
         <v/>
       </c>
       <c r="D19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$186,$A19,'QA Checklist'!$H$5:$H$186,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$186,$A19,'QA Checklist'!$H$5:$H$186,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$187,$A19,'QA Checklist'!$H$5:$H$187,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$187,$A19,'QA Checklist'!$H$5:$H$187,"Fail")</f>
         <v/>
       </c>
       <c r="E19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$186,$A19,'QA Checklist'!$H$5:$H$186,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$187,$A19,'QA Checklist'!$H$5:$H$187,"Pending")</f>
         <v/>
       </c>
       <c r="F19" s="8">
@@ -887,19 +887,19 @@
         </is>
       </c>
       <c r="B20" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$186,$A20)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$187,$A20)</f>
         <v/>
       </c>
       <c r="C20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$186,$A20,'QA Checklist'!$H$5:$H$186,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$186,$A20,'QA Checklist'!$H$5:$H$186,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$187,$A20,'QA Checklist'!$H$5:$H$187,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$187,$A20,'QA Checklist'!$H$5:$H$187,"Pass")</f>
         <v/>
       </c>
       <c r="D20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$186,$A20,'QA Checklist'!$H$5:$H$186,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$186,$A20,'QA Checklist'!$H$5:$H$186,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$187,$A20,'QA Checklist'!$H$5:$H$187,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$187,$A20,'QA Checklist'!$H$5:$H$187,"Fail")</f>
         <v/>
       </c>
       <c r="E20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$186,$A20,'QA Checklist'!$H$5:$H$186,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$187,$A20,'QA Checklist'!$H$5:$H$187,"Pending")</f>
         <v/>
       </c>
       <c r="F20" s="8">
@@ -914,19 +914,19 @@
         </is>
       </c>
       <c r="B21" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$186,$A21)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$187,$A21)</f>
         <v/>
       </c>
       <c r="C21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$186,$A21,'QA Checklist'!$H$5:$H$186,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$186,$A21,'QA Checklist'!$H$5:$H$186,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$187,$A21,'QA Checklist'!$H$5:$H$187,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$187,$A21,'QA Checklist'!$H$5:$H$187,"Pass")</f>
         <v/>
       </c>
       <c r="D21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$186,$A21,'QA Checklist'!$H$5:$H$186,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$186,$A21,'QA Checklist'!$H$5:$H$186,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$187,$A21,'QA Checklist'!$H$5:$H$187,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$187,$A21,'QA Checklist'!$H$5:$H$187,"Fail")</f>
         <v/>
       </c>
       <c r="E21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$186,$A21,'QA Checklist'!$H$5:$H$186,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$187,$A21,'QA Checklist'!$H$5:$H$187,"Pending")</f>
         <v/>
       </c>
       <c r="F21" s="8">
@@ -941,19 +941,19 @@
         </is>
       </c>
       <c r="B22" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$186,$A22)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$187,$A22)</f>
         <v/>
       </c>
       <c r="C22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$186,$A22,'QA Checklist'!$H$5:$H$186,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$186,$A22,'QA Checklist'!$H$5:$H$186,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$187,$A22,'QA Checklist'!$H$5:$H$187,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$187,$A22,'QA Checklist'!$H$5:$H$187,"Pass")</f>
         <v/>
       </c>
       <c r="D22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$186,$A22,'QA Checklist'!$H$5:$H$186,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$186,$A22,'QA Checklist'!$H$5:$H$186,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$187,$A22,'QA Checklist'!$H$5:$H$187,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$187,$A22,'QA Checklist'!$H$5:$H$187,"Fail")</f>
         <v/>
       </c>
       <c r="E22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$186,$A22,'QA Checklist'!$H$5:$H$186,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$187,$A22,'QA Checklist'!$H$5:$H$187,"Pending")</f>
         <v/>
       </c>
       <c r="F22" s="8">
@@ -1023,19 +1023,19 @@
         </is>
       </c>
       <c r="B26" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$186,$A26&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$187,$A26&amp;"*")</f>
         <v/>
       </c>
       <c r="C26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$186,$A26&amp;"*",'QA Checklist'!$H$5:$H$186,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$186,$A26&amp;"*",'QA Checklist'!$H$5:$H$186,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$187,$A26&amp;"*",'QA Checklist'!$H$5:$H$187,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$187,$A26&amp;"*",'QA Checklist'!$H$5:$H$187,"Pass")</f>
         <v/>
       </c>
       <c r="D26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$186,$A26&amp;"*",'QA Checklist'!$H$5:$H$186,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$186,$A26&amp;"*",'QA Checklist'!$H$5:$H$186,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$187,$A26&amp;"*",'QA Checklist'!$H$5:$H$187,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$187,$A26&amp;"*",'QA Checklist'!$H$5:$H$187,"Fail")</f>
         <v/>
       </c>
       <c r="E26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$186,$A26&amp;"*",'QA Checklist'!$H$5:$H$186,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$187,$A26&amp;"*",'QA Checklist'!$H$5:$H$187,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1046,19 +1046,19 @@
         </is>
       </c>
       <c r="B27" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$186,$A27&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$187,$A27&amp;"*")</f>
         <v/>
       </c>
       <c r="C27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$186,$A27&amp;"*",'QA Checklist'!$H$5:$H$186,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$186,$A27&amp;"*",'QA Checklist'!$H$5:$H$186,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$187,$A27&amp;"*",'QA Checklist'!$H$5:$H$187,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$187,$A27&amp;"*",'QA Checklist'!$H$5:$H$187,"Pass")</f>
         <v/>
       </c>
       <c r="D27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$186,$A27&amp;"*",'QA Checklist'!$H$5:$H$186,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$186,$A27&amp;"*",'QA Checklist'!$H$5:$H$186,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$187,$A27&amp;"*",'QA Checklist'!$H$5:$H$187,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$187,$A27&amp;"*",'QA Checklist'!$H$5:$H$187,"Fail")</f>
         <v/>
       </c>
       <c r="E27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$186,$A27&amp;"*",'QA Checklist'!$H$5:$H$186,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$187,$A27&amp;"*",'QA Checklist'!$H$5:$H$187,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1069,19 +1069,19 @@
         </is>
       </c>
       <c r="B28" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$186,$A28&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$187,$A28&amp;"*")</f>
         <v/>
       </c>
       <c r="C28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$186,$A28&amp;"*",'QA Checklist'!$H$5:$H$186,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$186,$A28&amp;"*",'QA Checklist'!$H$5:$H$186,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$187,$A28&amp;"*",'QA Checklist'!$H$5:$H$187,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$187,$A28&amp;"*",'QA Checklist'!$H$5:$H$187,"Pass")</f>
         <v/>
       </c>
       <c r="D28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$186,$A28&amp;"*",'QA Checklist'!$H$5:$H$186,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$186,$A28&amp;"*",'QA Checklist'!$H$5:$H$186,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$187,$A28&amp;"*",'QA Checklist'!$H$5:$H$187,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$187,$A28&amp;"*",'QA Checklist'!$H$5:$H$187,"Fail")</f>
         <v/>
       </c>
       <c r="E28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$186,$A28&amp;"*",'QA Checklist'!$H$5:$H$186,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$187,$A28&amp;"*",'QA Checklist'!$H$5:$H$187,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1096,7 +1096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I186"/>
+  <dimension ref="A1:I187"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9281,12 +9281,59 @@
         </is>
       </c>
     </row>
+    <row r="187">
+      <c r="A187" s="12" t="inlineStr">
+        <is>
+          <t>SA-61</t>
+        </is>
+      </c>
+      <c r="B187" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="C187" s="13" t="inlineStr">
+        <is>
+          <t>Tier 2 (Workflow &amp; Ergonomics)</t>
+        </is>
+      </c>
+      <c r="D187" s="13" t="inlineStr">
+        <is>
+          <t>TV Monitor Phase 1: TV Page Loads</t>
+        </is>
+      </c>
+      <c r="E187" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="F187" s="13" t="inlineStr">
+        <is>
+          <t>Log in as SA, open TV Monitor (Broadcast Hub), start the broadcast, open the shown link on another device or tab and enter the PIN; repeat with the internet disconnected</t>
+        </is>
+      </c>
+      <c r="G187" s="13" t="inlineStr">
+        <is>
+          <t>The link opens the TV page (no 404), the PIN unlocks it, live jobs appear and the page is fully styled even without internet</t>
+        </is>
+      </c>
+      <c r="H187" s="14" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="I187" s="13" t="inlineStr">
+        <is>
+          <t>Verified by Automated Unit Tests (173 passing in tests/frontend/sla_and_logic.test.js AUT-FRONT-144) and a live XAMPP headless Chrome check</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:I186"/>
+  <autoFilter ref="A4:I187"/>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="H5:H186">
+  <conditionalFormatting sqref="H5:H187">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$H5="Passed"</formula>
     </cfRule>
@@ -9303,13 +9350,13 @@
       <formula>$H5="Pending"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A5:A186">
+  <conditionalFormatting sqref="A5:A187">
     <cfRule type="expression" priority="6" dxfId="3">
-      <formula>COUNTIF($A$5:$A$186,$A5)&gt;1</formula>
+      <formula>COUNTIF($A$5:$A$187,$A5)&gt;1</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H5:H186" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H5:H187" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pending,Passed,Failed"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat(REV-186): TV Monitor phases 2-3 - secure per-branch broadcast, masked names
New TvController: per-branch tv_sessions, PIN -> branch-scoped HMAC token,
5-attempt PIN throttling, token-protected feed with only arrived vehicles,
masked names and no contact data. Session control is SA / Assistant only;
the public job list, public session routes and tracked tv_session.json are
gone. tv.html uses the token (no PIN in URLs), escapes output and takes
branch name / bay count from the feed; the Hub has no PIN links and opens a
staff kiosk. Cache buster v=3.39, AUT-FRONT-145, SA-62.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
+++ b/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
@@ -11,7 +11,7 @@
     <sheet name="QA Checklist" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$187</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$188</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'QA Checklist'!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTA('QA Checklist'!$A$5:$A$187)</f>
+        <f>COUNTA('QA Checklist'!$A$5:$A$188)</f>
         <v/>
       </c>
     </row>
@@ -594,7 +594,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$187,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$187,"Pass")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$188,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$188,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$187,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$187,"Fail")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$188,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$188,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -616,7 +616,7 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$187,"Pending")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$188,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -671,19 +671,19 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$187,$A12)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$188,$A12)</f>
         <v/>
       </c>
       <c r="C12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$187,$A12,'QA Checklist'!$H$5:$H$187,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$187,$A12,'QA Checklist'!$H$5:$H$187,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$188,$A12,'QA Checklist'!$H$5:$H$188,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$188,$A12,'QA Checklist'!$H$5:$H$188,"Pass")</f>
         <v/>
       </c>
       <c r="D12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$187,$A12,'QA Checklist'!$H$5:$H$187,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$187,$A12,'QA Checklist'!$H$5:$H$187,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$188,$A12,'QA Checklist'!$H$5:$H$188,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$188,$A12,'QA Checklist'!$H$5:$H$188,"Fail")</f>
         <v/>
       </c>
       <c r="E12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$187,$A12,'QA Checklist'!$H$5:$H$187,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$188,$A12,'QA Checklist'!$H$5:$H$188,"Pending")</f>
         <v/>
       </c>
       <c r="F12" s="8">
@@ -698,19 +698,19 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$187,$A13)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$188,$A13)</f>
         <v/>
       </c>
       <c r="C13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$187,$A13,'QA Checklist'!$H$5:$H$187,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$187,$A13,'QA Checklist'!$H$5:$H$187,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$188,$A13,'QA Checklist'!$H$5:$H$188,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$188,$A13,'QA Checklist'!$H$5:$H$188,"Pass")</f>
         <v/>
       </c>
       <c r="D13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$187,$A13,'QA Checklist'!$H$5:$H$187,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$187,$A13,'QA Checklist'!$H$5:$H$187,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$188,$A13,'QA Checklist'!$H$5:$H$188,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$188,$A13,'QA Checklist'!$H$5:$H$188,"Fail")</f>
         <v/>
       </c>
       <c r="E13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$187,$A13,'QA Checklist'!$H$5:$H$187,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$188,$A13,'QA Checklist'!$H$5:$H$188,"Pending")</f>
         <v/>
       </c>
       <c r="F13" s="8">
@@ -725,19 +725,19 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$187,$A14)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$188,$A14)</f>
         <v/>
       </c>
       <c r="C14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$187,$A14,'QA Checklist'!$H$5:$H$187,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$187,$A14,'QA Checklist'!$H$5:$H$187,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$188,$A14,'QA Checklist'!$H$5:$H$188,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$188,$A14,'QA Checklist'!$H$5:$H$188,"Pass")</f>
         <v/>
       </c>
       <c r="D14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$187,$A14,'QA Checklist'!$H$5:$H$187,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$187,$A14,'QA Checklist'!$H$5:$H$187,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$188,$A14,'QA Checklist'!$H$5:$H$188,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$188,$A14,'QA Checklist'!$H$5:$H$188,"Fail")</f>
         <v/>
       </c>
       <c r="E14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$187,$A14,'QA Checklist'!$H$5:$H$187,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$188,$A14,'QA Checklist'!$H$5:$H$188,"Pending")</f>
         <v/>
       </c>
       <c r="F14" s="8">
@@ -752,19 +752,19 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$187,$A15)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$188,$A15)</f>
         <v/>
       </c>
       <c r="C15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$187,$A15,'QA Checklist'!$H$5:$H$187,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$187,$A15,'QA Checklist'!$H$5:$H$187,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$188,$A15,'QA Checklist'!$H$5:$H$188,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$188,$A15,'QA Checklist'!$H$5:$H$188,"Pass")</f>
         <v/>
       </c>
       <c r="D15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$187,$A15,'QA Checklist'!$H$5:$H$187,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$187,$A15,'QA Checklist'!$H$5:$H$187,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$188,$A15,'QA Checklist'!$H$5:$H$188,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$188,$A15,'QA Checklist'!$H$5:$H$188,"Fail")</f>
         <v/>
       </c>
       <c r="E15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$187,$A15,'QA Checklist'!$H$5:$H$187,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$188,$A15,'QA Checklist'!$H$5:$H$188,"Pending")</f>
         <v/>
       </c>
       <c r="F15" s="8">
@@ -779,19 +779,19 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$187,$A16)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$188,$A16)</f>
         <v/>
       </c>
       <c r="C16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$187,$A16,'QA Checklist'!$H$5:$H$187,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$187,$A16,'QA Checklist'!$H$5:$H$187,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$188,$A16,'QA Checklist'!$H$5:$H$188,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$188,$A16,'QA Checklist'!$H$5:$H$188,"Pass")</f>
         <v/>
       </c>
       <c r="D16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$187,$A16,'QA Checklist'!$H$5:$H$187,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$187,$A16,'QA Checklist'!$H$5:$H$187,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$188,$A16,'QA Checklist'!$H$5:$H$188,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$188,$A16,'QA Checklist'!$H$5:$H$188,"Fail")</f>
         <v/>
       </c>
       <c r="E16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$187,$A16,'QA Checklist'!$H$5:$H$187,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$188,$A16,'QA Checklist'!$H$5:$H$188,"Pending")</f>
         <v/>
       </c>
       <c r="F16" s="8">
@@ -806,19 +806,19 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$187,$A17)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$188,$A17)</f>
         <v/>
       </c>
       <c r="C17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$187,$A17,'QA Checklist'!$H$5:$H$187,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$187,$A17,'QA Checklist'!$H$5:$H$187,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$188,$A17,'QA Checklist'!$H$5:$H$188,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$188,$A17,'QA Checklist'!$H$5:$H$188,"Pass")</f>
         <v/>
       </c>
       <c r="D17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$187,$A17,'QA Checklist'!$H$5:$H$187,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$187,$A17,'QA Checklist'!$H$5:$H$187,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$188,$A17,'QA Checklist'!$H$5:$H$188,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$188,$A17,'QA Checklist'!$H$5:$H$188,"Fail")</f>
         <v/>
       </c>
       <c r="E17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$187,$A17,'QA Checklist'!$H$5:$H$187,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$188,$A17,'QA Checklist'!$H$5:$H$188,"Pending")</f>
         <v/>
       </c>
       <c r="F17" s="8">
@@ -833,19 +833,19 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$187,$A18)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$188,$A18)</f>
         <v/>
       </c>
       <c r="C18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$187,$A18,'QA Checklist'!$H$5:$H$187,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$187,$A18,'QA Checklist'!$H$5:$H$187,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$188,$A18,'QA Checklist'!$H$5:$H$188,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$188,$A18,'QA Checklist'!$H$5:$H$188,"Pass")</f>
         <v/>
       </c>
       <c r="D18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$187,$A18,'QA Checklist'!$H$5:$H$187,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$187,$A18,'QA Checklist'!$H$5:$H$187,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$188,$A18,'QA Checklist'!$H$5:$H$188,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$188,$A18,'QA Checklist'!$H$5:$H$188,"Fail")</f>
         <v/>
       </c>
       <c r="E18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$187,$A18,'QA Checklist'!$H$5:$H$187,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$188,$A18,'QA Checklist'!$H$5:$H$188,"Pending")</f>
         <v/>
       </c>
       <c r="F18" s="8">
@@ -860,19 +860,19 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$187,$A19)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$188,$A19)</f>
         <v/>
       </c>
       <c r="C19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$187,$A19,'QA Checklist'!$H$5:$H$187,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$187,$A19,'QA Checklist'!$H$5:$H$187,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$188,$A19,'QA Checklist'!$H$5:$H$188,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$188,$A19,'QA Checklist'!$H$5:$H$188,"Pass")</f>
         <v/>
       </c>
       <c r="D19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$187,$A19,'QA Checklist'!$H$5:$H$187,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$187,$A19,'QA Checklist'!$H$5:$H$187,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$188,$A19,'QA Checklist'!$H$5:$H$188,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$188,$A19,'QA Checklist'!$H$5:$H$188,"Fail")</f>
         <v/>
       </c>
       <c r="E19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$187,$A19,'QA Checklist'!$H$5:$H$187,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$188,$A19,'QA Checklist'!$H$5:$H$188,"Pending")</f>
         <v/>
       </c>
       <c r="F19" s="8">
@@ -887,19 +887,19 @@
         </is>
       </c>
       <c r="B20" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$187,$A20)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$188,$A20)</f>
         <v/>
       </c>
       <c r="C20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$187,$A20,'QA Checklist'!$H$5:$H$187,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$187,$A20,'QA Checklist'!$H$5:$H$187,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$188,$A20,'QA Checklist'!$H$5:$H$188,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$188,$A20,'QA Checklist'!$H$5:$H$188,"Pass")</f>
         <v/>
       </c>
       <c r="D20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$187,$A20,'QA Checklist'!$H$5:$H$187,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$187,$A20,'QA Checklist'!$H$5:$H$187,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$188,$A20,'QA Checklist'!$H$5:$H$188,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$188,$A20,'QA Checklist'!$H$5:$H$188,"Fail")</f>
         <v/>
       </c>
       <c r="E20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$187,$A20,'QA Checklist'!$H$5:$H$187,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$188,$A20,'QA Checklist'!$H$5:$H$188,"Pending")</f>
         <v/>
       </c>
       <c r="F20" s="8">
@@ -914,19 +914,19 @@
         </is>
       </c>
       <c r="B21" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$187,$A21)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$188,$A21)</f>
         <v/>
       </c>
       <c r="C21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$187,$A21,'QA Checklist'!$H$5:$H$187,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$187,$A21,'QA Checklist'!$H$5:$H$187,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$188,$A21,'QA Checklist'!$H$5:$H$188,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$188,$A21,'QA Checklist'!$H$5:$H$188,"Pass")</f>
         <v/>
       </c>
       <c r="D21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$187,$A21,'QA Checklist'!$H$5:$H$187,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$187,$A21,'QA Checklist'!$H$5:$H$187,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$188,$A21,'QA Checklist'!$H$5:$H$188,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$188,$A21,'QA Checklist'!$H$5:$H$188,"Fail")</f>
         <v/>
       </c>
       <c r="E21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$187,$A21,'QA Checklist'!$H$5:$H$187,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$188,$A21,'QA Checklist'!$H$5:$H$188,"Pending")</f>
         <v/>
       </c>
       <c r="F21" s="8">
@@ -941,19 +941,19 @@
         </is>
       </c>
       <c r="B22" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$187,$A22)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$188,$A22)</f>
         <v/>
       </c>
       <c r="C22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$187,$A22,'QA Checklist'!$H$5:$H$187,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$187,$A22,'QA Checklist'!$H$5:$H$187,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$188,$A22,'QA Checklist'!$H$5:$H$188,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$188,$A22,'QA Checklist'!$H$5:$H$188,"Pass")</f>
         <v/>
       </c>
       <c r="D22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$187,$A22,'QA Checklist'!$H$5:$H$187,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$187,$A22,'QA Checklist'!$H$5:$H$187,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$188,$A22,'QA Checklist'!$H$5:$H$188,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$188,$A22,'QA Checklist'!$H$5:$H$188,"Fail")</f>
         <v/>
       </c>
       <c r="E22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$187,$A22,'QA Checklist'!$H$5:$H$187,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$188,$A22,'QA Checklist'!$H$5:$H$188,"Pending")</f>
         <v/>
       </c>
       <c r="F22" s="8">
@@ -1023,19 +1023,19 @@
         </is>
       </c>
       <c r="B26" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$187,$A26&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$188,$A26&amp;"*")</f>
         <v/>
       </c>
       <c r="C26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$187,$A26&amp;"*",'QA Checklist'!$H$5:$H$187,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$187,$A26&amp;"*",'QA Checklist'!$H$5:$H$187,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$188,$A26&amp;"*",'QA Checklist'!$H$5:$H$188,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$188,$A26&amp;"*",'QA Checklist'!$H$5:$H$188,"Pass")</f>
         <v/>
       </c>
       <c r="D26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$187,$A26&amp;"*",'QA Checklist'!$H$5:$H$187,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$187,$A26&amp;"*",'QA Checklist'!$H$5:$H$187,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$188,$A26&amp;"*",'QA Checklist'!$H$5:$H$188,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$188,$A26&amp;"*",'QA Checklist'!$H$5:$H$188,"Fail")</f>
         <v/>
       </c>
       <c r="E26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$187,$A26&amp;"*",'QA Checklist'!$H$5:$H$187,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$188,$A26&amp;"*",'QA Checklist'!$H$5:$H$188,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1046,19 +1046,19 @@
         </is>
       </c>
       <c r="B27" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$187,$A27&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$188,$A27&amp;"*")</f>
         <v/>
       </c>
       <c r="C27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$187,$A27&amp;"*",'QA Checklist'!$H$5:$H$187,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$187,$A27&amp;"*",'QA Checklist'!$H$5:$H$187,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$188,$A27&amp;"*",'QA Checklist'!$H$5:$H$188,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$188,$A27&amp;"*",'QA Checklist'!$H$5:$H$188,"Pass")</f>
         <v/>
       </c>
       <c r="D27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$187,$A27&amp;"*",'QA Checklist'!$H$5:$H$187,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$187,$A27&amp;"*",'QA Checklist'!$H$5:$H$187,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$188,$A27&amp;"*",'QA Checklist'!$H$5:$H$188,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$188,$A27&amp;"*",'QA Checklist'!$H$5:$H$188,"Fail")</f>
         <v/>
       </c>
       <c r="E27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$187,$A27&amp;"*",'QA Checklist'!$H$5:$H$187,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$188,$A27&amp;"*",'QA Checklist'!$H$5:$H$188,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1069,19 +1069,19 @@
         </is>
       </c>
       <c r="B28" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$187,$A28&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$188,$A28&amp;"*")</f>
         <v/>
       </c>
       <c r="C28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$187,$A28&amp;"*",'QA Checklist'!$H$5:$H$187,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$187,$A28&amp;"*",'QA Checklist'!$H$5:$H$187,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$188,$A28&amp;"*",'QA Checklist'!$H$5:$H$188,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$188,$A28&amp;"*",'QA Checklist'!$H$5:$H$188,"Pass")</f>
         <v/>
       </c>
       <c r="D28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$187,$A28&amp;"*",'QA Checklist'!$H$5:$H$187,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$187,$A28&amp;"*",'QA Checklist'!$H$5:$H$187,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$188,$A28&amp;"*",'QA Checklist'!$H$5:$H$188,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$188,$A28&amp;"*",'QA Checklist'!$H$5:$H$188,"Fail")</f>
         <v/>
       </c>
       <c r="E28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$187,$A28&amp;"*",'QA Checklist'!$H$5:$H$187,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$188,$A28&amp;"*",'QA Checklist'!$H$5:$H$188,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1096,7 +1096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I187"/>
+  <dimension ref="A1:I188"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9328,12 +9328,59 @@
         </is>
       </c>
     </row>
+    <row r="188">
+      <c r="A188" s="12" t="inlineStr">
+        <is>
+          <t>SA-62</t>
+        </is>
+      </c>
+      <c r="B188" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="C188" s="13" t="inlineStr">
+        <is>
+          <t>Tier 2 (Workflow &amp; Ergonomics)</t>
+        </is>
+      </c>
+      <c r="D188" s="13" t="inlineStr">
+        <is>
+          <t>TV Monitor Phases 2-3: Security &amp; Branches</t>
+        </is>
+      </c>
+      <c r="E188" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="F188" s="13" t="inlineStr">
+        <is>
+          <t>As a Marikina SA start the broadcast in the TV Broadcast Hub and enter the PIN on a TV; do the same as a Regalado SA on a second TV; pause / resume; generate a new PIN; try the TV link without a PIN and the API without logging in; open the HDMI kiosk</t>
+        </is>
+      </c>
+      <c r="G188" s="13" t="inlineStr">
+        <is>
+          <t>Each TV shows only its branch with masked names and the branch bay count; paused TVs show standby and resume by themselves; a new PIN signs the TVs out; without a PIN or login no data or PIN is returned; Owner / Admin cannot control the broadcast; the HDMI kiosk opens without a PIN</t>
+        </is>
+      </c>
+      <c r="H188" s="14" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="I188" s="13" t="inlineStr">
+        <is>
+          <t>Verified by Automated Unit Tests (174 passing in tests/frontend/sla_and_logic.test.js AUT-FRONT-145), live API checks 26/26 and headless Chrome end-to-end 9/9 on XAMPP</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:I187"/>
+  <autoFilter ref="A4:I188"/>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="H5:H187">
+  <conditionalFormatting sqref="H5:H188">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$H5="Passed"</formula>
     </cfRule>
@@ -9350,13 +9397,13 @@
       <formula>$H5="Pending"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A5:A187">
+  <conditionalFormatting sqref="A5:A188">
     <cfRule type="expression" priority="6" dxfId="3">
-      <formula>COUNTIF($A$5:$A$187,$A5)&gt;1</formula>
+      <formula>COUNTIF($A$5:$A$188,$A5)&gt;1</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H5:H187" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H5:H188" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pending,Passed,Failed"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat(REV-187): TV Monitor phase 4 - one group per vehicle, connection badge, sound prompt
Vehicles are grouped strictly by status (In Service / In Queue / Ready / Carry Over) with separate In Service and In Queue lists; a Connection lost badge shows the last update time; a Tap to enable sound prompt appears when the TV opened by itself; the simulation drawer only shows with ?dev=1. Cache buster v=3.40, AUT-FRONT-146, SA-63.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
+++ b/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
@@ -11,7 +11,7 @@
     <sheet name="QA Checklist" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$188</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$189</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'QA Checklist'!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTA('QA Checklist'!$A$5:$A$188)</f>
+        <f>COUNTA('QA Checklist'!$A$5:$A$189)</f>
         <v/>
       </c>
     </row>
@@ -594,7 +594,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$188,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$188,"Pass")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$189,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$189,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$188,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$188,"Fail")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$189,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$189,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -616,7 +616,7 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$188,"Pending")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$189,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -671,19 +671,19 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$188,$A12)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$189,$A12)</f>
         <v/>
       </c>
       <c r="C12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$188,$A12,'QA Checklist'!$H$5:$H$188,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$188,$A12,'QA Checklist'!$H$5:$H$188,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$189,$A12,'QA Checklist'!$H$5:$H$189,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$189,$A12,'QA Checklist'!$H$5:$H$189,"Pass")</f>
         <v/>
       </c>
       <c r="D12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$188,$A12,'QA Checklist'!$H$5:$H$188,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$188,$A12,'QA Checklist'!$H$5:$H$188,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$189,$A12,'QA Checklist'!$H$5:$H$189,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$189,$A12,'QA Checklist'!$H$5:$H$189,"Fail")</f>
         <v/>
       </c>
       <c r="E12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$188,$A12,'QA Checklist'!$H$5:$H$188,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$189,$A12,'QA Checklist'!$H$5:$H$189,"Pending")</f>
         <v/>
       </c>
       <c r="F12" s="8">
@@ -698,19 +698,19 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$188,$A13)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$189,$A13)</f>
         <v/>
       </c>
       <c r="C13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$188,$A13,'QA Checklist'!$H$5:$H$188,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$188,$A13,'QA Checklist'!$H$5:$H$188,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$189,$A13,'QA Checklist'!$H$5:$H$189,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$189,$A13,'QA Checklist'!$H$5:$H$189,"Pass")</f>
         <v/>
       </c>
       <c r="D13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$188,$A13,'QA Checklist'!$H$5:$H$188,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$188,$A13,'QA Checklist'!$H$5:$H$188,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$189,$A13,'QA Checklist'!$H$5:$H$189,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$189,$A13,'QA Checklist'!$H$5:$H$189,"Fail")</f>
         <v/>
       </c>
       <c r="E13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$188,$A13,'QA Checklist'!$H$5:$H$188,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$189,$A13,'QA Checklist'!$H$5:$H$189,"Pending")</f>
         <v/>
       </c>
       <c r="F13" s="8">
@@ -725,19 +725,19 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$188,$A14)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$189,$A14)</f>
         <v/>
       </c>
       <c r="C14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$188,$A14,'QA Checklist'!$H$5:$H$188,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$188,$A14,'QA Checklist'!$H$5:$H$188,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$189,$A14,'QA Checklist'!$H$5:$H$189,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$189,$A14,'QA Checklist'!$H$5:$H$189,"Pass")</f>
         <v/>
       </c>
       <c r="D14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$188,$A14,'QA Checklist'!$H$5:$H$188,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$188,$A14,'QA Checklist'!$H$5:$H$188,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$189,$A14,'QA Checklist'!$H$5:$H$189,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$189,$A14,'QA Checklist'!$H$5:$H$189,"Fail")</f>
         <v/>
       </c>
       <c r="E14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$188,$A14,'QA Checklist'!$H$5:$H$188,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$189,$A14,'QA Checklist'!$H$5:$H$189,"Pending")</f>
         <v/>
       </c>
       <c r="F14" s="8">
@@ -752,19 +752,19 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$188,$A15)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$189,$A15)</f>
         <v/>
       </c>
       <c r="C15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$188,$A15,'QA Checklist'!$H$5:$H$188,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$188,$A15,'QA Checklist'!$H$5:$H$188,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$189,$A15,'QA Checklist'!$H$5:$H$189,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$189,$A15,'QA Checklist'!$H$5:$H$189,"Pass")</f>
         <v/>
       </c>
       <c r="D15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$188,$A15,'QA Checklist'!$H$5:$H$188,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$188,$A15,'QA Checklist'!$H$5:$H$188,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$189,$A15,'QA Checklist'!$H$5:$H$189,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$189,$A15,'QA Checklist'!$H$5:$H$189,"Fail")</f>
         <v/>
       </c>
       <c r="E15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$188,$A15,'QA Checklist'!$H$5:$H$188,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$189,$A15,'QA Checklist'!$H$5:$H$189,"Pending")</f>
         <v/>
       </c>
       <c r="F15" s="8">
@@ -779,19 +779,19 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$188,$A16)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$189,$A16)</f>
         <v/>
       </c>
       <c r="C16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$188,$A16,'QA Checklist'!$H$5:$H$188,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$188,$A16,'QA Checklist'!$H$5:$H$188,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$189,$A16,'QA Checklist'!$H$5:$H$189,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$189,$A16,'QA Checklist'!$H$5:$H$189,"Pass")</f>
         <v/>
       </c>
       <c r="D16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$188,$A16,'QA Checklist'!$H$5:$H$188,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$188,$A16,'QA Checklist'!$H$5:$H$188,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$189,$A16,'QA Checklist'!$H$5:$H$189,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$189,$A16,'QA Checklist'!$H$5:$H$189,"Fail")</f>
         <v/>
       </c>
       <c r="E16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$188,$A16,'QA Checklist'!$H$5:$H$188,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$189,$A16,'QA Checklist'!$H$5:$H$189,"Pending")</f>
         <v/>
       </c>
       <c r="F16" s="8">
@@ -806,19 +806,19 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$188,$A17)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$189,$A17)</f>
         <v/>
       </c>
       <c r="C17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$188,$A17,'QA Checklist'!$H$5:$H$188,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$188,$A17,'QA Checklist'!$H$5:$H$188,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$189,$A17,'QA Checklist'!$H$5:$H$189,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$189,$A17,'QA Checklist'!$H$5:$H$189,"Pass")</f>
         <v/>
       </c>
       <c r="D17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$188,$A17,'QA Checklist'!$H$5:$H$188,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$188,$A17,'QA Checklist'!$H$5:$H$188,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$189,$A17,'QA Checklist'!$H$5:$H$189,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$189,$A17,'QA Checklist'!$H$5:$H$189,"Fail")</f>
         <v/>
       </c>
       <c r="E17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$188,$A17,'QA Checklist'!$H$5:$H$188,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$189,$A17,'QA Checklist'!$H$5:$H$189,"Pending")</f>
         <v/>
       </c>
       <c r="F17" s="8">
@@ -833,19 +833,19 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$188,$A18)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$189,$A18)</f>
         <v/>
       </c>
       <c r="C18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$188,$A18,'QA Checklist'!$H$5:$H$188,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$188,$A18,'QA Checklist'!$H$5:$H$188,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$189,$A18,'QA Checklist'!$H$5:$H$189,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$189,$A18,'QA Checklist'!$H$5:$H$189,"Pass")</f>
         <v/>
       </c>
       <c r="D18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$188,$A18,'QA Checklist'!$H$5:$H$188,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$188,$A18,'QA Checklist'!$H$5:$H$188,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$189,$A18,'QA Checklist'!$H$5:$H$189,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$189,$A18,'QA Checklist'!$H$5:$H$189,"Fail")</f>
         <v/>
       </c>
       <c r="E18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$188,$A18,'QA Checklist'!$H$5:$H$188,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$189,$A18,'QA Checklist'!$H$5:$H$189,"Pending")</f>
         <v/>
       </c>
       <c r="F18" s="8">
@@ -860,19 +860,19 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$188,$A19)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$189,$A19)</f>
         <v/>
       </c>
       <c r="C19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$188,$A19,'QA Checklist'!$H$5:$H$188,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$188,$A19,'QA Checklist'!$H$5:$H$188,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$189,$A19,'QA Checklist'!$H$5:$H$189,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$189,$A19,'QA Checklist'!$H$5:$H$189,"Pass")</f>
         <v/>
       </c>
       <c r="D19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$188,$A19,'QA Checklist'!$H$5:$H$188,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$188,$A19,'QA Checklist'!$H$5:$H$188,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$189,$A19,'QA Checklist'!$H$5:$H$189,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$189,$A19,'QA Checklist'!$H$5:$H$189,"Fail")</f>
         <v/>
       </c>
       <c r="E19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$188,$A19,'QA Checklist'!$H$5:$H$188,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$189,$A19,'QA Checklist'!$H$5:$H$189,"Pending")</f>
         <v/>
       </c>
       <c r="F19" s="8">
@@ -887,19 +887,19 @@
         </is>
       </c>
       <c r="B20" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$188,$A20)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$189,$A20)</f>
         <v/>
       </c>
       <c r="C20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$188,$A20,'QA Checklist'!$H$5:$H$188,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$188,$A20,'QA Checklist'!$H$5:$H$188,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$189,$A20,'QA Checklist'!$H$5:$H$189,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$189,$A20,'QA Checklist'!$H$5:$H$189,"Pass")</f>
         <v/>
       </c>
       <c r="D20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$188,$A20,'QA Checklist'!$H$5:$H$188,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$188,$A20,'QA Checklist'!$H$5:$H$188,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$189,$A20,'QA Checklist'!$H$5:$H$189,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$189,$A20,'QA Checklist'!$H$5:$H$189,"Fail")</f>
         <v/>
       </c>
       <c r="E20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$188,$A20,'QA Checklist'!$H$5:$H$188,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$189,$A20,'QA Checklist'!$H$5:$H$189,"Pending")</f>
         <v/>
       </c>
       <c r="F20" s="8">
@@ -914,19 +914,19 @@
         </is>
       </c>
       <c r="B21" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$188,$A21)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$189,$A21)</f>
         <v/>
       </c>
       <c r="C21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$188,$A21,'QA Checklist'!$H$5:$H$188,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$188,$A21,'QA Checklist'!$H$5:$H$188,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$189,$A21,'QA Checklist'!$H$5:$H$189,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$189,$A21,'QA Checklist'!$H$5:$H$189,"Pass")</f>
         <v/>
       </c>
       <c r="D21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$188,$A21,'QA Checklist'!$H$5:$H$188,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$188,$A21,'QA Checklist'!$H$5:$H$188,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$189,$A21,'QA Checklist'!$H$5:$H$189,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$189,$A21,'QA Checklist'!$H$5:$H$189,"Fail")</f>
         <v/>
       </c>
       <c r="E21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$188,$A21,'QA Checklist'!$H$5:$H$188,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$189,$A21,'QA Checklist'!$H$5:$H$189,"Pending")</f>
         <v/>
       </c>
       <c r="F21" s="8">
@@ -941,19 +941,19 @@
         </is>
       </c>
       <c r="B22" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$188,$A22)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$189,$A22)</f>
         <v/>
       </c>
       <c r="C22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$188,$A22,'QA Checklist'!$H$5:$H$188,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$188,$A22,'QA Checklist'!$H$5:$H$188,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$189,$A22,'QA Checklist'!$H$5:$H$189,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$189,$A22,'QA Checklist'!$H$5:$H$189,"Pass")</f>
         <v/>
       </c>
       <c r="D22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$188,$A22,'QA Checklist'!$H$5:$H$188,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$188,$A22,'QA Checklist'!$H$5:$H$188,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$189,$A22,'QA Checklist'!$H$5:$H$189,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$189,$A22,'QA Checklist'!$H$5:$H$189,"Fail")</f>
         <v/>
       </c>
       <c r="E22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$188,$A22,'QA Checklist'!$H$5:$H$188,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$189,$A22,'QA Checklist'!$H$5:$H$189,"Pending")</f>
         <v/>
       </c>
       <c r="F22" s="8">
@@ -1023,19 +1023,19 @@
         </is>
       </c>
       <c r="B26" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$188,$A26&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$189,$A26&amp;"*")</f>
         <v/>
       </c>
       <c r="C26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$188,$A26&amp;"*",'QA Checklist'!$H$5:$H$188,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$188,$A26&amp;"*",'QA Checklist'!$H$5:$H$188,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$189,$A26&amp;"*",'QA Checklist'!$H$5:$H$189,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$189,$A26&amp;"*",'QA Checklist'!$H$5:$H$189,"Pass")</f>
         <v/>
       </c>
       <c r="D26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$188,$A26&amp;"*",'QA Checklist'!$H$5:$H$188,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$188,$A26&amp;"*",'QA Checklist'!$H$5:$H$188,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$189,$A26&amp;"*",'QA Checklist'!$H$5:$H$189,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$189,$A26&amp;"*",'QA Checklist'!$H$5:$H$189,"Fail")</f>
         <v/>
       </c>
       <c r="E26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$188,$A26&amp;"*",'QA Checklist'!$H$5:$H$188,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$189,$A26&amp;"*",'QA Checklist'!$H$5:$H$189,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1046,19 +1046,19 @@
         </is>
       </c>
       <c r="B27" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$188,$A27&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$189,$A27&amp;"*")</f>
         <v/>
       </c>
       <c r="C27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$188,$A27&amp;"*",'QA Checklist'!$H$5:$H$188,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$188,$A27&amp;"*",'QA Checklist'!$H$5:$H$188,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$189,$A27&amp;"*",'QA Checklist'!$H$5:$H$189,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$189,$A27&amp;"*",'QA Checklist'!$H$5:$H$189,"Pass")</f>
         <v/>
       </c>
       <c r="D27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$188,$A27&amp;"*",'QA Checklist'!$H$5:$H$188,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$188,$A27&amp;"*",'QA Checklist'!$H$5:$H$188,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$189,$A27&amp;"*",'QA Checklist'!$H$5:$H$189,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$189,$A27&amp;"*",'QA Checklist'!$H$5:$H$189,"Fail")</f>
         <v/>
       </c>
       <c r="E27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$188,$A27&amp;"*",'QA Checklist'!$H$5:$H$188,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$189,$A27&amp;"*",'QA Checklist'!$H$5:$H$189,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1069,19 +1069,19 @@
         </is>
       </c>
       <c r="B28" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$188,$A28&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$189,$A28&amp;"*")</f>
         <v/>
       </c>
       <c r="C28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$188,$A28&amp;"*",'QA Checklist'!$H$5:$H$188,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$188,$A28&amp;"*",'QA Checklist'!$H$5:$H$188,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$189,$A28&amp;"*",'QA Checklist'!$H$5:$H$189,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$189,$A28&amp;"*",'QA Checklist'!$H$5:$H$189,"Pass")</f>
         <v/>
       </c>
       <c r="D28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$188,$A28&amp;"*",'QA Checklist'!$H$5:$H$188,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$188,$A28&amp;"*",'QA Checklist'!$H$5:$H$188,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$189,$A28&amp;"*",'QA Checklist'!$H$5:$H$189,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$189,$A28&amp;"*",'QA Checklist'!$H$5:$H$189,"Fail")</f>
         <v/>
       </c>
       <c r="E28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$188,$A28&amp;"*",'QA Checklist'!$H$5:$H$188,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$189,$A28&amp;"*",'QA Checklist'!$H$5:$H$189,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1096,7 +1096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I188"/>
+  <dimension ref="A1:I189"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9375,12 +9375,59 @@
         </is>
       </c>
     </row>
+    <row r="189">
+      <c r="A189" s="12" t="inlineStr">
+        <is>
+          <t>SA-63</t>
+        </is>
+      </c>
+      <c r="B189" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="C189" s="13" t="inlineStr">
+        <is>
+          <t>Tier 2 (Workflow &amp; Ergonomics)</t>
+        </is>
+      </c>
+      <c r="D189" s="13" t="inlineStr">
+        <is>
+          <t>TV Monitor Phase 4: Display Integrity</t>
+        </is>
+      </c>
+      <c r="E189" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="F189" s="13" t="inlineStr">
+        <is>
+          <t>Open the TV, check Slide 2 lists, unplug the network briefly, reload the TV page without touching it, then open tv.html?dev=1</t>
+        </is>
+      </c>
+      <c r="G189" s="13" t="inlineStr">
+        <is>
+          <t>Each vehicle appears once (In Service, In Queue, Ready, Carry Over); a Connection lost badge with the last update time shows while offline and clears when back; a Tap to enable sound prompt appears after a reload and disappears after one tap; the dev drawer only shows with ?dev=1</t>
+        </is>
+      </c>
+      <c r="H189" s="14" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="I189" s="13" t="inlineStr">
+        <is>
+          <t>Verified by Automated Unit Tests (175 passing in tests/frontend/sla_and_logic.test.js AUT-FRONT-146) and live XAMPP headless Chrome checks 12/12</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:I188"/>
+  <autoFilter ref="A4:I189"/>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="H5:H188">
+  <conditionalFormatting sqref="H5:H189">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$H5="Passed"</formula>
     </cfRule>
@@ -9397,13 +9444,13 @@
       <formula>$H5="Pending"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A5:A188">
+  <conditionalFormatting sqref="A5:A189">
     <cfRule type="expression" priority="6" dxfId="3">
-      <formula>COUNTIF($A$5:$A$188,$A5)&gt;1</formula>
+      <formula>COUNTIF($A$5:$A$189,$A5)&gt;1</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H5:H188" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H5:H189" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pending,Passed,Failed"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat(REV-188): TV Monitor phase 5 - in-app TV Monitor embeds the Smart TV page
The in-app TV Monitor shows tv.html?embedded=1 (same screen as the lounge TV, signed in as the staff member) and is loaded only while open. The separate in-app renderer, slide helpers and the dead ?mode=tv code are removed; renderTV stays as a no-op for existing callers. Cache buster v=3.41, AUT-FRONT-147, SA-64.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
+++ b/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
@@ -11,7 +11,7 @@
     <sheet name="QA Checklist" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$189</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$190</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'QA Checklist'!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTA('QA Checklist'!$A$5:$A$189)</f>
+        <f>COUNTA('QA Checklist'!$A$5:$A$190)</f>
         <v/>
       </c>
     </row>
@@ -594,7 +594,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$189,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$189,"Pass")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$190,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$190,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$189,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$189,"Fail")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$190,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$190,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -616,7 +616,7 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$189,"Pending")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$190,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -671,19 +671,19 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$189,$A12)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$190,$A12)</f>
         <v/>
       </c>
       <c r="C12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$189,$A12,'QA Checklist'!$H$5:$H$189,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$189,$A12,'QA Checklist'!$H$5:$H$189,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$190,$A12,'QA Checklist'!$H$5:$H$190,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$190,$A12,'QA Checklist'!$H$5:$H$190,"Pass")</f>
         <v/>
       </c>
       <c r="D12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$189,$A12,'QA Checklist'!$H$5:$H$189,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$189,$A12,'QA Checklist'!$H$5:$H$189,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$190,$A12,'QA Checklist'!$H$5:$H$190,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$190,$A12,'QA Checklist'!$H$5:$H$190,"Fail")</f>
         <v/>
       </c>
       <c r="E12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$189,$A12,'QA Checklist'!$H$5:$H$189,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$190,$A12,'QA Checklist'!$H$5:$H$190,"Pending")</f>
         <v/>
       </c>
       <c r="F12" s="8">
@@ -698,19 +698,19 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$189,$A13)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$190,$A13)</f>
         <v/>
       </c>
       <c r="C13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$189,$A13,'QA Checklist'!$H$5:$H$189,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$189,$A13,'QA Checklist'!$H$5:$H$189,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$190,$A13,'QA Checklist'!$H$5:$H$190,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$190,$A13,'QA Checklist'!$H$5:$H$190,"Pass")</f>
         <v/>
       </c>
       <c r="D13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$189,$A13,'QA Checklist'!$H$5:$H$189,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$189,$A13,'QA Checklist'!$H$5:$H$189,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$190,$A13,'QA Checklist'!$H$5:$H$190,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$190,$A13,'QA Checklist'!$H$5:$H$190,"Fail")</f>
         <v/>
       </c>
       <c r="E13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$189,$A13,'QA Checklist'!$H$5:$H$189,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$190,$A13,'QA Checklist'!$H$5:$H$190,"Pending")</f>
         <v/>
       </c>
       <c r="F13" s="8">
@@ -725,19 +725,19 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$189,$A14)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$190,$A14)</f>
         <v/>
       </c>
       <c r="C14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$189,$A14,'QA Checklist'!$H$5:$H$189,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$189,$A14,'QA Checklist'!$H$5:$H$189,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$190,$A14,'QA Checklist'!$H$5:$H$190,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$190,$A14,'QA Checklist'!$H$5:$H$190,"Pass")</f>
         <v/>
       </c>
       <c r="D14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$189,$A14,'QA Checklist'!$H$5:$H$189,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$189,$A14,'QA Checklist'!$H$5:$H$189,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$190,$A14,'QA Checklist'!$H$5:$H$190,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$190,$A14,'QA Checklist'!$H$5:$H$190,"Fail")</f>
         <v/>
       </c>
       <c r="E14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$189,$A14,'QA Checklist'!$H$5:$H$189,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$190,$A14,'QA Checklist'!$H$5:$H$190,"Pending")</f>
         <v/>
       </c>
       <c r="F14" s="8">
@@ -752,19 +752,19 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$189,$A15)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$190,$A15)</f>
         <v/>
       </c>
       <c r="C15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$189,$A15,'QA Checklist'!$H$5:$H$189,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$189,$A15,'QA Checklist'!$H$5:$H$189,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$190,$A15,'QA Checklist'!$H$5:$H$190,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$190,$A15,'QA Checklist'!$H$5:$H$190,"Pass")</f>
         <v/>
       </c>
       <c r="D15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$189,$A15,'QA Checklist'!$H$5:$H$189,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$189,$A15,'QA Checklist'!$H$5:$H$189,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$190,$A15,'QA Checklist'!$H$5:$H$190,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$190,$A15,'QA Checklist'!$H$5:$H$190,"Fail")</f>
         <v/>
       </c>
       <c r="E15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$189,$A15,'QA Checklist'!$H$5:$H$189,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$190,$A15,'QA Checklist'!$H$5:$H$190,"Pending")</f>
         <v/>
       </c>
       <c r="F15" s="8">
@@ -779,19 +779,19 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$189,$A16)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$190,$A16)</f>
         <v/>
       </c>
       <c r="C16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$189,$A16,'QA Checklist'!$H$5:$H$189,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$189,$A16,'QA Checklist'!$H$5:$H$189,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$190,$A16,'QA Checklist'!$H$5:$H$190,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$190,$A16,'QA Checklist'!$H$5:$H$190,"Pass")</f>
         <v/>
       </c>
       <c r="D16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$189,$A16,'QA Checklist'!$H$5:$H$189,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$189,$A16,'QA Checklist'!$H$5:$H$189,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$190,$A16,'QA Checklist'!$H$5:$H$190,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$190,$A16,'QA Checklist'!$H$5:$H$190,"Fail")</f>
         <v/>
       </c>
       <c r="E16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$189,$A16,'QA Checklist'!$H$5:$H$189,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$190,$A16,'QA Checklist'!$H$5:$H$190,"Pending")</f>
         <v/>
       </c>
       <c r="F16" s="8">
@@ -806,19 +806,19 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$189,$A17)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$190,$A17)</f>
         <v/>
       </c>
       <c r="C17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$189,$A17,'QA Checklist'!$H$5:$H$189,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$189,$A17,'QA Checklist'!$H$5:$H$189,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$190,$A17,'QA Checklist'!$H$5:$H$190,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$190,$A17,'QA Checklist'!$H$5:$H$190,"Pass")</f>
         <v/>
       </c>
       <c r="D17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$189,$A17,'QA Checklist'!$H$5:$H$189,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$189,$A17,'QA Checklist'!$H$5:$H$189,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$190,$A17,'QA Checklist'!$H$5:$H$190,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$190,$A17,'QA Checklist'!$H$5:$H$190,"Fail")</f>
         <v/>
       </c>
       <c r="E17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$189,$A17,'QA Checklist'!$H$5:$H$189,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$190,$A17,'QA Checklist'!$H$5:$H$190,"Pending")</f>
         <v/>
       </c>
       <c r="F17" s="8">
@@ -833,19 +833,19 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$189,$A18)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$190,$A18)</f>
         <v/>
       </c>
       <c r="C18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$189,$A18,'QA Checklist'!$H$5:$H$189,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$189,$A18,'QA Checklist'!$H$5:$H$189,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$190,$A18,'QA Checklist'!$H$5:$H$190,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$190,$A18,'QA Checklist'!$H$5:$H$190,"Pass")</f>
         <v/>
       </c>
       <c r="D18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$189,$A18,'QA Checklist'!$H$5:$H$189,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$189,$A18,'QA Checklist'!$H$5:$H$189,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$190,$A18,'QA Checklist'!$H$5:$H$190,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$190,$A18,'QA Checklist'!$H$5:$H$190,"Fail")</f>
         <v/>
       </c>
       <c r="E18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$189,$A18,'QA Checklist'!$H$5:$H$189,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$190,$A18,'QA Checklist'!$H$5:$H$190,"Pending")</f>
         <v/>
       </c>
       <c r="F18" s="8">
@@ -860,19 +860,19 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$189,$A19)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$190,$A19)</f>
         <v/>
       </c>
       <c r="C19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$189,$A19,'QA Checklist'!$H$5:$H$189,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$189,$A19,'QA Checklist'!$H$5:$H$189,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$190,$A19,'QA Checklist'!$H$5:$H$190,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$190,$A19,'QA Checklist'!$H$5:$H$190,"Pass")</f>
         <v/>
       </c>
       <c r="D19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$189,$A19,'QA Checklist'!$H$5:$H$189,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$189,$A19,'QA Checklist'!$H$5:$H$189,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$190,$A19,'QA Checklist'!$H$5:$H$190,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$190,$A19,'QA Checklist'!$H$5:$H$190,"Fail")</f>
         <v/>
       </c>
       <c r="E19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$189,$A19,'QA Checklist'!$H$5:$H$189,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$190,$A19,'QA Checklist'!$H$5:$H$190,"Pending")</f>
         <v/>
       </c>
       <c r="F19" s="8">
@@ -887,19 +887,19 @@
         </is>
       </c>
       <c r="B20" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$189,$A20)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$190,$A20)</f>
         <v/>
       </c>
       <c r="C20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$189,$A20,'QA Checklist'!$H$5:$H$189,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$189,$A20,'QA Checklist'!$H$5:$H$189,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$190,$A20,'QA Checklist'!$H$5:$H$190,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$190,$A20,'QA Checklist'!$H$5:$H$190,"Pass")</f>
         <v/>
       </c>
       <c r="D20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$189,$A20,'QA Checklist'!$H$5:$H$189,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$189,$A20,'QA Checklist'!$H$5:$H$189,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$190,$A20,'QA Checklist'!$H$5:$H$190,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$190,$A20,'QA Checklist'!$H$5:$H$190,"Fail")</f>
         <v/>
       </c>
       <c r="E20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$189,$A20,'QA Checklist'!$H$5:$H$189,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$190,$A20,'QA Checklist'!$H$5:$H$190,"Pending")</f>
         <v/>
       </c>
       <c r="F20" s="8">
@@ -914,19 +914,19 @@
         </is>
       </c>
       <c r="B21" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$189,$A21)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$190,$A21)</f>
         <v/>
       </c>
       <c r="C21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$189,$A21,'QA Checklist'!$H$5:$H$189,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$189,$A21,'QA Checklist'!$H$5:$H$189,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$190,$A21,'QA Checklist'!$H$5:$H$190,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$190,$A21,'QA Checklist'!$H$5:$H$190,"Pass")</f>
         <v/>
       </c>
       <c r="D21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$189,$A21,'QA Checklist'!$H$5:$H$189,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$189,$A21,'QA Checklist'!$H$5:$H$189,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$190,$A21,'QA Checklist'!$H$5:$H$190,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$190,$A21,'QA Checklist'!$H$5:$H$190,"Fail")</f>
         <v/>
       </c>
       <c r="E21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$189,$A21,'QA Checklist'!$H$5:$H$189,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$190,$A21,'QA Checklist'!$H$5:$H$190,"Pending")</f>
         <v/>
       </c>
       <c r="F21" s="8">
@@ -941,19 +941,19 @@
         </is>
       </c>
       <c r="B22" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$189,$A22)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$190,$A22)</f>
         <v/>
       </c>
       <c r="C22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$189,$A22,'QA Checklist'!$H$5:$H$189,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$189,$A22,'QA Checklist'!$H$5:$H$189,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$190,$A22,'QA Checklist'!$H$5:$H$190,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$190,$A22,'QA Checklist'!$H$5:$H$190,"Pass")</f>
         <v/>
       </c>
       <c r="D22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$189,$A22,'QA Checklist'!$H$5:$H$189,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$189,$A22,'QA Checklist'!$H$5:$H$189,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$190,$A22,'QA Checklist'!$H$5:$H$190,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$190,$A22,'QA Checklist'!$H$5:$H$190,"Fail")</f>
         <v/>
       </c>
       <c r="E22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$189,$A22,'QA Checklist'!$H$5:$H$189,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$190,$A22,'QA Checklist'!$H$5:$H$190,"Pending")</f>
         <v/>
       </c>
       <c r="F22" s="8">
@@ -1023,19 +1023,19 @@
         </is>
       </c>
       <c r="B26" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$189,$A26&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$190,$A26&amp;"*")</f>
         <v/>
       </c>
       <c r="C26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$189,$A26&amp;"*",'QA Checklist'!$H$5:$H$189,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$189,$A26&amp;"*",'QA Checklist'!$H$5:$H$189,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$190,$A26&amp;"*",'QA Checklist'!$H$5:$H$190,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$190,$A26&amp;"*",'QA Checklist'!$H$5:$H$190,"Pass")</f>
         <v/>
       </c>
       <c r="D26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$189,$A26&amp;"*",'QA Checklist'!$H$5:$H$189,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$189,$A26&amp;"*",'QA Checklist'!$H$5:$H$189,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$190,$A26&amp;"*",'QA Checklist'!$H$5:$H$190,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$190,$A26&amp;"*",'QA Checklist'!$H$5:$H$190,"Fail")</f>
         <v/>
       </c>
       <c r="E26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$189,$A26&amp;"*",'QA Checklist'!$H$5:$H$189,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$190,$A26&amp;"*",'QA Checklist'!$H$5:$H$190,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1046,19 +1046,19 @@
         </is>
       </c>
       <c r="B27" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$189,$A27&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$190,$A27&amp;"*")</f>
         <v/>
       </c>
       <c r="C27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$189,$A27&amp;"*",'QA Checklist'!$H$5:$H$189,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$189,$A27&amp;"*",'QA Checklist'!$H$5:$H$189,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$190,$A27&amp;"*",'QA Checklist'!$H$5:$H$190,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$190,$A27&amp;"*",'QA Checklist'!$H$5:$H$190,"Pass")</f>
         <v/>
       </c>
       <c r="D27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$189,$A27&amp;"*",'QA Checklist'!$H$5:$H$189,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$189,$A27&amp;"*",'QA Checklist'!$H$5:$H$189,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$190,$A27&amp;"*",'QA Checklist'!$H$5:$H$190,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$190,$A27&amp;"*",'QA Checklist'!$H$5:$H$190,"Fail")</f>
         <v/>
       </c>
       <c r="E27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$189,$A27&amp;"*",'QA Checklist'!$H$5:$H$189,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$190,$A27&amp;"*",'QA Checklist'!$H$5:$H$190,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1069,19 +1069,19 @@
         </is>
       </c>
       <c r="B28" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$189,$A28&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$190,$A28&amp;"*")</f>
         <v/>
       </c>
       <c r="C28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$189,$A28&amp;"*",'QA Checklist'!$H$5:$H$189,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$189,$A28&amp;"*",'QA Checklist'!$H$5:$H$189,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$190,$A28&amp;"*",'QA Checklist'!$H$5:$H$190,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$190,$A28&amp;"*",'QA Checklist'!$H$5:$H$190,"Pass")</f>
         <v/>
       </c>
       <c r="D28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$189,$A28&amp;"*",'QA Checklist'!$H$5:$H$189,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$189,$A28&amp;"*",'QA Checklist'!$H$5:$H$189,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$190,$A28&amp;"*",'QA Checklist'!$H$5:$H$190,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$190,$A28&amp;"*",'QA Checklist'!$H$5:$H$190,"Fail")</f>
         <v/>
       </c>
       <c r="E28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$189,$A28&amp;"*",'QA Checklist'!$H$5:$H$189,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$190,$A28&amp;"*",'QA Checklist'!$H$5:$H$190,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1096,7 +1096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I189"/>
+  <dimension ref="A1:I190"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9422,12 +9422,59 @@
         </is>
       </c>
     </row>
+    <row r="190">
+      <c r="A190" s="12" t="inlineStr">
+        <is>
+          <t>SA-64</t>
+        </is>
+      </c>
+      <c r="B190" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="C190" s="13" t="inlineStr">
+        <is>
+          <t>Tier 2 (Workflow &amp; Ergonomics)</t>
+        </is>
+      </c>
+      <c r="D190" s="13" t="inlineStr">
+        <is>
+          <t>TV Monitor Phase 5: In-App Preview</t>
+        </is>
+      </c>
+      <c r="E190" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="F190" s="13" t="inlineStr">
+        <is>
+          <t>Log in as SA, open TV Monitor &gt; Open In-App Slides, compare with the lounge TV, pause the broadcast, then switch to another module</t>
+        </is>
+      </c>
+      <c r="G190" s="13" t="inlineStr">
+        <is>
+          <t>The in-app preview is the same screen as the lounge TV for the SA branch (no PIN), shows standby while paused, and stops when leaving the module</t>
+        </is>
+      </c>
+      <c r="H190" s="14" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="I190" s="13" t="inlineStr">
+        <is>
+          <t>Verified by Automated Unit Tests (176 passing in tests/frontend/sla_and_logic.test.js AUT-FRONT-147) and live XAMPP headless Chrome 6/6</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:I189"/>
+  <autoFilter ref="A4:I190"/>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="H5:H189">
+  <conditionalFormatting sqref="H5:H190">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$H5="Passed"</formula>
     </cfRule>
@@ -9444,13 +9491,13 @@
       <formula>$H5="Pending"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A5:A189">
+  <conditionalFormatting sqref="A5:A190">
     <cfRule type="expression" priority="6" dxfId="3">
-      <formula>COUNTIF($A$5:$A$189,$A5)&gt;1</formula>
+      <formula>COUNTIF($A$5:$A$190,$A5)&gt;1</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H5:H189" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H5:H190" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pending,Passed,Failed"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat(REV-189): TV Monitor phase 6 - Daily Intakes announcements on the TV, Call Customer Again
The server records tv_announcements when an SA assigns a bay or changes a status (processing, ready, carry-over, returned, released); the lounge TV plays each once, in order (banner, chime, voice with plate and model), from GET /tv/announcements. Call Customer Again (Ready rows, 15 s throttle) and a TV sound check replace the app-side voice; the SA computer only chimes after a saved Ready / Released. Cache buster v=3.42, AUT-FRONT-148, SA-65.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
+++ b/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
@@ -11,7 +11,7 @@
     <sheet name="QA Checklist" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$190</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$191</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'QA Checklist'!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTA('QA Checklist'!$A$5:$A$190)</f>
+        <f>COUNTA('QA Checklist'!$A$5:$A$191)</f>
         <v/>
       </c>
     </row>
@@ -594,7 +594,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$190,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$190,"Pass")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$191,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$191,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$190,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$190,"Fail")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$191,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$191,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -616,7 +616,7 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$190,"Pending")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$191,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -671,19 +671,19 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$190,$A12)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$191,$A12)</f>
         <v/>
       </c>
       <c r="C12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$190,$A12,'QA Checklist'!$H$5:$H$190,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$190,$A12,'QA Checklist'!$H$5:$H$190,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$191,$A12,'QA Checklist'!$H$5:$H$191,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$191,$A12,'QA Checklist'!$H$5:$H$191,"Pass")</f>
         <v/>
       </c>
       <c r="D12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$190,$A12,'QA Checklist'!$H$5:$H$190,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$190,$A12,'QA Checklist'!$H$5:$H$190,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$191,$A12,'QA Checklist'!$H$5:$H$191,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$191,$A12,'QA Checklist'!$H$5:$H$191,"Fail")</f>
         <v/>
       </c>
       <c r="E12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$190,$A12,'QA Checklist'!$H$5:$H$190,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$191,$A12,'QA Checklist'!$H$5:$H$191,"Pending")</f>
         <v/>
       </c>
       <c r="F12" s="8">
@@ -698,19 +698,19 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$190,$A13)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$191,$A13)</f>
         <v/>
       </c>
       <c r="C13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$190,$A13,'QA Checklist'!$H$5:$H$190,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$190,$A13,'QA Checklist'!$H$5:$H$190,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$191,$A13,'QA Checklist'!$H$5:$H$191,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$191,$A13,'QA Checklist'!$H$5:$H$191,"Pass")</f>
         <v/>
       </c>
       <c r="D13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$190,$A13,'QA Checklist'!$H$5:$H$190,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$190,$A13,'QA Checklist'!$H$5:$H$190,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$191,$A13,'QA Checklist'!$H$5:$H$191,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$191,$A13,'QA Checklist'!$H$5:$H$191,"Fail")</f>
         <v/>
       </c>
       <c r="E13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$190,$A13,'QA Checklist'!$H$5:$H$190,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$191,$A13,'QA Checklist'!$H$5:$H$191,"Pending")</f>
         <v/>
       </c>
       <c r="F13" s="8">
@@ -725,19 +725,19 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$190,$A14)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$191,$A14)</f>
         <v/>
       </c>
       <c r="C14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$190,$A14,'QA Checklist'!$H$5:$H$190,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$190,$A14,'QA Checklist'!$H$5:$H$190,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$191,$A14,'QA Checklist'!$H$5:$H$191,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$191,$A14,'QA Checklist'!$H$5:$H$191,"Pass")</f>
         <v/>
       </c>
       <c r="D14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$190,$A14,'QA Checklist'!$H$5:$H$190,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$190,$A14,'QA Checklist'!$H$5:$H$190,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$191,$A14,'QA Checklist'!$H$5:$H$191,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$191,$A14,'QA Checklist'!$H$5:$H$191,"Fail")</f>
         <v/>
       </c>
       <c r="E14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$190,$A14,'QA Checklist'!$H$5:$H$190,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$191,$A14,'QA Checklist'!$H$5:$H$191,"Pending")</f>
         <v/>
       </c>
       <c r="F14" s="8">
@@ -752,19 +752,19 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$190,$A15)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$191,$A15)</f>
         <v/>
       </c>
       <c r="C15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$190,$A15,'QA Checklist'!$H$5:$H$190,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$190,$A15,'QA Checklist'!$H$5:$H$190,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$191,$A15,'QA Checklist'!$H$5:$H$191,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$191,$A15,'QA Checklist'!$H$5:$H$191,"Pass")</f>
         <v/>
       </c>
       <c r="D15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$190,$A15,'QA Checklist'!$H$5:$H$190,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$190,$A15,'QA Checklist'!$H$5:$H$190,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$191,$A15,'QA Checklist'!$H$5:$H$191,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$191,$A15,'QA Checklist'!$H$5:$H$191,"Fail")</f>
         <v/>
       </c>
       <c r="E15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$190,$A15,'QA Checklist'!$H$5:$H$190,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$191,$A15,'QA Checklist'!$H$5:$H$191,"Pending")</f>
         <v/>
       </c>
       <c r="F15" s="8">
@@ -779,19 +779,19 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$190,$A16)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$191,$A16)</f>
         <v/>
       </c>
       <c r="C16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$190,$A16,'QA Checklist'!$H$5:$H$190,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$190,$A16,'QA Checklist'!$H$5:$H$190,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$191,$A16,'QA Checklist'!$H$5:$H$191,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$191,$A16,'QA Checklist'!$H$5:$H$191,"Pass")</f>
         <v/>
       </c>
       <c r="D16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$190,$A16,'QA Checklist'!$H$5:$H$190,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$190,$A16,'QA Checklist'!$H$5:$H$190,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$191,$A16,'QA Checklist'!$H$5:$H$191,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$191,$A16,'QA Checklist'!$H$5:$H$191,"Fail")</f>
         <v/>
       </c>
       <c r="E16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$190,$A16,'QA Checklist'!$H$5:$H$190,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$191,$A16,'QA Checklist'!$H$5:$H$191,"Pending")</f>
         <v/>
       </c>
       <c r="F16" s="8">
@@ -806,19 +806,19 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$190,$A17)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$191,$A17)</f>
         <v/>
       </c>
       <c r="C17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$190,$A17,'QA Checklist'!$H$5:$H$190,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$190,$A17,'QA Checklist'!$H$5:$H$190,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$191,$A17,'QA Checklist'!$H$5:$H$191,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$191,$A17,'QA Checklist'!$H$5:$H$191,"Pass")</f>
         <v/>
       </c>
       <c r="D17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$190,$A17,'QA Checklist'!$H$5:$H$190,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$190,$A17,'QA Checklist'!$H$5:$H$190,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$191,$A17,'QA Checklist'!$H$5:$H$191,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$191,$A17,'QA Checklist'!$H$5:$H$191,"Fail")</f>
         <v/>
       </c>
       <c r="E17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$190,$A17,'QA Checklist'!$H$5:$H$190,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$191,$A17,'QA Checklist'!$H$5:$H$191,"Pending")</f>
         <v/>
       </c>
       <c r="F17" s="8">
@@ -833,19 +833,19 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$190,$A18)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$191,$A18)</f>
         <v/>
       </c>
       <c r="C18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$190,$A18,'QA Checklist'!$H$5:$H$190,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$190,$A18,'QA Checklist'!$H$5:$H$190,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$191,$A18,'QA Checklist'!$H$5:$H$191,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$191,$A18,'QA Checklist'!$H$5:$H$191,"Pass")</f>
         <v/>
       </c>
       <c r="D18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$190,$A18,'QA Checklist'!$H$5:$H$190,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$190,$A18,'QA Checklist'!$H$5:$H$190,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$191,$A18,'QA Checklist'!$H$5:$H$191,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$191,$A18,'QA Checklist'!$H$5:$H$191,"Fail")</f>
         <v/>
       </c>
       <c r="E18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$190,$A18,'QA Checklist'!$H$5:$H$190,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$191,$A18,'QA Checklist'!$H$5:$H$191,"Pending")</f>
         <v/>
       </c>
       <c r="F18" s="8">
@@ -860,19 +860,19 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$190,$A19)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$191,$A19)</f>
         <v/>
       </c>
       <c r="C19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$190,$A19,'QA Checklist'!$H$5:$H$190,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$190,$A19,'QA Checklist'!$H$5:$H$190,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$191,$A19,'QA Checklist'!$H$5:$H$191,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$191,$A19,'QA Checklist'!$H$5:$H$191,"Pass")</f>
         <v/>
       </c>
       <c r="D19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$190,$A19,'QA Checklist'!$H$5:$H$190,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$190,$A19,'QA Checklist'!$H$5:$H$190,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$191,$A19,'QA Checklist'!$H$5:$H$191,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$191,$A19,'QA Checklist'!$H$5:$H$191,"Fail")</f>
         <v/>
       </c>
       <c r="E19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$190,$A19,'QA Checklist'!$H$5:$H$190,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$191,$A19,'QA Checklist'!$H$5:$H$191,"Pending")</f>
         <v/>
       </c>
       <c r="F19" s="8">
@@ -887,19 +887,19 @@
         </is>
       </c>
       <c r="B20" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$190,$A20)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$191,$A20)</f>
         <v/>
       </c>
       <c r="C20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$190,$A20,'QA Checklist'!$H$5:$H$190,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$190,$A20,'QA Checklist'!$H$5:$H$190,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$191,$A20,'QA Checklist'!$H$5:$H$191,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$191,$A20,'QA Checklist'!$H$5:$H$191,"Pass")</f>
         <v/>
       </c>
       <c r="D20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$190,$A20,'QA Checklist'!$H$5:$H$190,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$190,$A20,'QA Checklist'!$H$5:$H$190,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$191,$A20,'QA Checklist'!$H$5:$H$191,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$191,$A20,'QA Checklist'!$H$5:$H$191,"Fail")</f>
         <v/>
       </c>
       <c r="E20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$190,$A20,'QA Checklist'!$H$5:$H$190,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$191,$A20,'QA Checklist'!$H$5:$H$191,"Pending")</f>
         <v/>
       </c>
       <c r="F20" s="8">
@@ -914,19 +914,19 @@
         </is>
       </c>
       <c r="B21" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$190,$A21)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$191,$A21)</f>
         <v/>
       </c>
       <c r="C21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$190,$A21,'QA Checklist'!$H$5:$H$190,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$190,$A21,'QA Checklist'!$H$5:$H$190,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$191,$A21,'QA Checklist'!$H$5:$H$191,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$191,$A21,'QA Checklist'!$H$5:$H$191,"Pass")</f>
         <v/>
       </c>
       <c r="D21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$190,$A21,'QA Checklist'!$H$5:$H$190,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$190,$A21,'QA Checklist'!$H$5:$H$190,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$191,$A21,'QA Checklist'!$H$5:$H$191,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$191,$A21,'QA Checklist'!$H$5:$H$191,"Fail")</f>
         <v/>
       </c>
       <c r="E21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$190,$A21,'QA Checklist'!$H$5:$H$190,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$191,$A21,'QA Checklist'!$H$5:$H$191,"Pending")</f>
         <v/>
       </c>
       <c r="F21" s="8">
@@ -941,19 +941,19 @@
         </is>
       </c>
       <c r="B22" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$190,$A22)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$191,$A22)</f>
         <v/>
       </c>
       <c r="C22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$190,$A22,'QA Checklist'!$H$5:$H$190,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$190,$A22,'QA Checklist'!$H$5:$H$190,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$191,$A22,'QA Checklist'!$H$5:$H$191,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$191,$A22,'QA Checklist'!$H$5:$H$191,"Pass")</f>
         <v/>
       </c>
       <c r="D22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$190,$A22,'QA Checklist'!$H$5:$H$190,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$190,$A22,'QA Checklist'!$H$5:$H$190,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$191,$A22,'QA Checklist'!$H$5:$H$191,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$191,$A22,'QA Checklist'!$H$5:$H$191,"Fail")</f>
         <v/>
       </c>
       <c r="E22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$190,$A22,'QA Checklist'!$H$5:$H$190,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$191,$A22,'QA Checklist'!$H$5:$H$191,"Pending")</f>
         <v/>
       </c>
       <c r="F22" s="8">
@@ -1023,19 +1023,19 @@
         </is>
       </c>
       <c r="B26" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$190,$A26&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$191,$A26&amp;"*")</f>
         <v/>
       </c>
       <c r="C26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$190,$A26&amp;"*",'QA Checklist'!$H$5:$H$190,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$190,$A26&amp;"*",'QA Checklist'!$H$5:$H$190,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$191,$A26&amp;"*",'QA Checklist'!$H$5:$H$191,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$191,$A26&amp;"*",'QA Checklist'!$H$5:$H$191,"Pass")</f>
         <v/>
       </c>
       <c r="D26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$190,$A26&amp;"*",'QA Checklist'!$H$5:$H$190,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$190,$A26&amp;"*",'QA Checklist'!$H$5:$H$190,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$191,$A26&amp;"*",'QA Checklist'!$H$5:$H$191,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$191,$A26&amp;"*",'QA Checklist'!$H$5:$H$191,"Fail")</f>
         <v/>
       </c>
       <c r="E26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$190,$A26&amp;"*",'QA Checklist'!$H$5:$H$190,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$191,$A26&amp;"*",'QA Checklist'!$H$5:$H$191,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1046,19 +1046,19 @@
         </is>
       </c>
       <c r="B27" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$190,$A27&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$191,$A27&amp;"*")</f>
         <v/>
       </c>
       <c r="C27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$190,$A27&amp;"*",'QA Checklist'!$H$5:$H$190,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$190,$A27&amp;"*",'QA Checklist'!$H$5:$H$190,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$191,$A27&amp;"*",'QA Checklist'!$H$5:$H$191,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$191,$A27&amp;"*",'QA Checklist'!$H$5:$H$191,"Pass")</f>
         <v/>
       </c>
       <c r="D27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$190,$A27&amp;"*",'QA Checklist'!$H$5:$H$190,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$190,$A27&amp;"*",'QA Checklist'!$H$5:$H$190,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$191,$A27&amp;"*",'QA Checklist'!$H$5:$H$191,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$191,$A27&amp;"*",'QA Checklist'!$H$5:$H$191,"Fail")</f>
         <v/>
       </c>
       <c r="E27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$190,$A27&amp;"*",'QA Checklist'!$H$5:$H$190,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$191,$A27&amp;"*",'QA Checklist'!$H$5:$H$191,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1069,19 +1069,19 @@
         </is>
       </c>
       <c r="B28" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$190,$A28&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$191,$A28&amp;"*")</f>
         <v/>
       </c>
       <c r="C28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$190,$A28&amp;"*",'QA Checklist'!$H$5:$H$190,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$190,$A28&amp;"*",'QA Checklist'!$H$5:$H$190,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$191,$A28&amp;"*",'QA Checklist'!$H$5:$H$191,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$191,$A28&amp;"*",'QA Checklist'!$H$5:$H$191,"Pass")</f>
         <v/>
       </c>
       <c r="D28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$190,$A28&amp;"*",'QA Checklist'!$H$5:$H$190,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$190,$A28&amp;"*",'QA Checklist'!$H$5:$H$190,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$191,$A28&amp;"*",'QA Checklist'!$H$5:$H$191,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$191,$A28&amp;"*",'QA Checklist'!$H$5:$H$191,"Fail")</f>
         <v/>
       </c>
       <c r="E28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$190,$A28&amp;"*",'QA Checklist'!$H$5:$H$190,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$191,$A28&amp;"*",'QA Checklist'!$H$5:$H$191,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1096,7 +1096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I190"/>
+  <dimension ref="A1:I191"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9469,12 +9469,59 @@
         </is>
       </c>
     </row>
+    <row r="191">
+      <c r="A191" s="12" t="inlineStr">
+        <is>
+          <t>SA-65</t>
+        </is>
+      </c>
+      <c r="B191" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="C191" s="13" t="inlineStr">
+        <is>
+          <t>Tier 2 (Workflow &amp; Ergonomics)</t>
+        </is>
+      </c>
+      <c r="D191" s="13" t="inlineStr">
+        <is>
+          <t>TV Monitor Phase 6: Announcements</t>
+        </is>
+      </c>
+      <c r="E191" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="F191" s="13" t="inlineStr">
+        <is>
+          <t>With the lounge TV live, in Daily Intakes assign a bay, set Ready to Release, press Call Again, then Release; in Settings press Test TV Announcement; watch a second branch TV and a TV opened afterwards</t>
+        </is>
+      </c>
+      <c r="G191" s="13" t="inlineStr">
+        <is>
+          <t>The lounge TV shows a banner, chimes and speaks each change once, in order, with plate and model (release thanks the customer); Call Again repeats the ready call (a second press within 15 s is refused); the SA computer only chimes after saving Ready / Released; other branch TVs and newly opened TVs do not play it</t>
+        </is>
+      </c>
+      <c r="H191" s="14" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="I191" s="13" t="inlineStr">
+        <is>
+          <t>Verified by Automated Unit Tests (177 passing in tests/frontend/sla_and_logic.test.js AUT-FRONT-148) and an XAMPP end-to-end run 8/8</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:I190"/>
+  <autoFilter ref="A4:I191"/>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="H5:H190">
+  <conditionalFormatting sqref="H5:H191">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$H5="Passed"</formula>
     </cfRule>
@@ -9491,13 +9538,13 @@
       <formula>$H5="Pending"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A5:A190">
+  <conditionalFormatting sqref="A5:A191">
     <cfRule type="expression" priority="6" dxfId="3">
-      <formula>COUNTIF($A$5:$A$190,$A5)&gt;1</formula>
+      <formula>COUNTIF($A$5:$A$191,$A5)&gt;1</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H5:H190" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H5:H191" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pending,Passed,Failed"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat(REV-190): real per-branch weather box on the TV
The TV weather box shows a real Open-Meteo reading for each branch pin (temperature, condition, feels like, humidity, rain chance), cached per branch for 15 minutes by the server (tv_weather_cache, GET /tv/weather). Offline it shows the last reading with its time or 'Weather unavailable' instead of invented values. Removed the unused app weather code. Cache buster v=3.43, AUT-FRONT-149, SA-66.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
+++ b/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
@@ -11,7 +11,7 @@
     <sheet name="QA Checklist" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$191</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$192</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'QA Checklist'!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTA('QA Checklist'!$A$5:$A$191)</f>
+        <f>COUNTA('QA Checklist'!$A$5:$A$192)</f>
         <v/>
       </c>
     </row>
@@ -594,7 +594,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$191,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$191,"Pass")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$192,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$192,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$191,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$191,"Fail")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$192,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$192,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -616,7 +616,7 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$191,"Pending")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$192,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -671,19 +671,19 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$191,$A12)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$192,$A12)</f>
         <v/>
       </c>
       <c r="C12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$191,$A12,'QA Checklist'!$H$5:$H$191,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$191,$A12,'QA Checklist'!$H$5:$H$191,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$192,$A12,'QA Checklist'!$H$5:$H$192,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$192,$A12,'QA Checklist'!$H$5:$H$192,"Pass")</f>
         <v/>
       </c>
       <c r="D12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$191,$A12,'QA Checklist'!$H$5:$H$191,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$191,$A12,'QA Checklist'!$H$5:$H$191,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$192,$A12,'QA Checklist'!$H$5:$H$192,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$192,$A12,'QA Checklist'!$H$5:$H$192,"Fail")</f>
         <v/>
       </c>
       <c r="E12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$191,$A12,'QA Checklist'!$H$5:$H$191,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$192,$A12,'QA Checklist'!$H$5:$H$192,"Pending")</f>
         <v/>
       </c>
       <c r="F12" s="8">
@@ -698,19 +698,19 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$191,$A13)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$192,$A13)</f>
         <v/>
       </c>
       <c r="C13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$191,$A13,'QA Checklist'!$H$5:$H$191,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$191,$A13,'QA Checklist'!$H$5:$H$191,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$192,$A13,'QA Checklist'!$H$5:$H$192,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$192,$A13,'QA Checklist'!$H$5:$H$192,"Pass")</f>
         <v/>
       </c>
       <c r="D13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$191,$A13,'QA Checklist'!$H$5:$H$191,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$191,$A13,'QA Checklist'!$H$5:$H$191,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$192,$A13,'QA Checklist'!$H$5:$H$192,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$192,$A13,'QA Checklist'!$H$5:$H$192,"Fail")</f>
         <v/>
       </c>
       <c r="E13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$191,$A13,'QA Checklist'!$H$5:$H$191,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$192,$A13,'QA Checklist'!$H$5:$H$192,"Pending")</f>
         <v/>
       </c>
       <c r="F13" s="8">
@@ -725,19 +725,19 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$191,$A14)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$192,$A14)</f>
         <v/>
       </c>
       <c r="C14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$191,$A14,'QA Checklist'!$H$5:$H$191,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$191,$A14,'QA Checklist'!$H$5:$H$191,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$192,$A14,'QA Checklist'!$H$5:$H$192,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$192,$A14,'QA Checklist'!$H$5:$H$192,"Pass")</f>
         <v/>
       </c>
       <c r="D14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$191,$A14,'QA Checklist'!$H$5:$H$191,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$191,$A14,'QA Checklist'!$H$5:$H$191,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$192,$A14,'QA Checklist'!$H$5:$H$192,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$192,$A14,'QA Checklist'!$H$5:$H$192,"Fail")</f>
         <v/>
       </c>
       <c r="E14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$191,$A14,'QA Checklist'!$H$5:$H$191,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$192,$A14,'QA Checklist'!$H$5:$H$192,"Pending")</f>
         <v/>
       </c>
       <c r="F14" s="8">
@@ -752,19 +752,19 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$191,$A15)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$192,$A15)</f>
         <v/>
       </c>
       <c r="C15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$191,$A15,'QA Checklist'!$H$5:$H$191,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$191,$A15,'QA Checklist'!$H$5:$H$191,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$192,$A15,'QA Checklist'!$H$5:$H$192,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$192,$A15,'QA Checklist'!$H$5:$H$192,"Pass")</f>
         <v/>
       </c>
       <c r="D15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$191,$A15,'QA Checklist'!$H$5:$H$191,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$191,$A15,'QA Checklist'!$H$5:$H$191,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$192,$A15,'QA Checklist'!$H$5:$H$192,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$192,$A15,'QA Checklist'!$H$5:$H$192,"Fail")</f>
         <v/>
       </c>
       <c r="E15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$191,$A15,'QA Checklist'!$H$5:$H$191,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$192,$A15,'QA Checklist'!$H$5:$H$192,"Pending")</f>
         <v/>
       </c>
       <c r="F15" s="8">
@@ -779,19 +779,19 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$191,$A16)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$192,$A16)</f>
         <v/>
       </c>
       <c r="C16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$191,$A16,'QA Checklist'!$H$5:$H$191,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$191,$A16,'QA Checklist'!$H$5:$H$191,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$192,$A16,'QA Checklist'!$H$5:$H$192,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$192,$A16,'QA Checklist'!$H$5:$H$192,"Pass")</f>
         <v/>
       </c>
       <c r="D16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$191,$A16,'QA Checklist'!$H$5:$H$191,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$191,$A16,'QA Checklist'!$H$5:$H$191,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$192,$A16,'QA Checklist'!$H$5:$H$192,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$192,$A16,'QA Checklist'!$H$5:$H$192,"Fail")</f>
         <v/>
       </c>
       <c r="E16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$191,$A16,'QA Checklist'!$H$5:$H$191,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$192,$A16,'QA Checklist'!$H$5:$H$192,"Pending")</f>
         <v/>
       </c>
       <c r="F16" s="8">
@@ -806,19 +806,19 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$191,$A17)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$192,$A17)</f>
         <v/>
       </c>
       <c r="C17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$191,$A17,'QA Checklist'!$H$5:$H$191,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$191,$A17,'QA Checklist'!$H$5:$H$191,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$192,$A17,'QA Checklist'!$H$5:$H$192,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$192,$A17,'QA Checklist'!$H$5:$H$192,"Pass")</f>
         <v/>
       </c>
       <c r="D17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$191,$A17,'QA Checklist'!$H$5:$H$191,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$191,$A17,'QA Checklist'!$H$5:$H$191,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$192,$A17,'QA Checklist'!$H$5:$H$192,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$192,$A17,'QA Checklist'!$H$5:$H$192,"Fail")</f>
         <v/>
       </c>
       <c r="E17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$191,$A17,'QA Checklist'!$H$5:$H$191,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$192,$A17,'QA Checklist'!$H$5:$H$192,"Pending")</f>
         <v/>
       </c>
       <c r="F17" s="8">
@@ -833,19 +833,19 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$191,$A18)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$192,$A18)</f>
         <v/>
       </c>
       <c r="C18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$191,$A18,'QA Checklist'!$H$5:$H$191,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$191,$A18,'QA Checklist'!$H$5:$H$191,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$192,$A18,'QA Checklist'!$H$5:$H$192,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$192,$A18,'QA Checklist'!$H$5:$H$192,"Pass")</f>
         <v/>
       </c>
       <c r="D18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$191,$A18,'QA Checklist'!$H$5:$H$191,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$191,$A18,'QA Checklist'!$H$5:$H$191,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$192,$A18,'QA Checklist'!$H$5:$H$192,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$192,$A18,'QA Checklist'!$H$5:$H$192,"Fail")</f>
         <v/>
       </c>
       <c r="E18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$191,$A18,'QA Checklist'!$H$5:$H$191,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$192,$A18,'QA Checklist'!$H$5:$H$192,"Pending")</f>
         <v/>
       </c>
       <c r="F18" s="8">
@@ -860,19 +860,19 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$191,$A19)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$192,$A19)</f>
         <v/>
       </c>
       <c r="C19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$191,$A19,'QA Checklist'!$H$5:$H$191,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$191,$A19,'QA Checklist'!$H$5:$H$191,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$192,$A19,'QA Checklist'!$H$5:$H$192,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$192,$A19,'QA Checklist'!$H$5:$H$192,"Pass")</f>
         <v/>
       </c>
       <c r="D19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$191,$A19,'QA Checklist'!$H$5:$H$191,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$191,$A19,'QA Checklist'!$H$5:$H$191,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$192,$A19,'QA Checklist'!$H$5:$H$192,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$192,$A19,'QA Checklist'!$H$5:$H$192,"Fail")</f>
         <v/>
       </c>
       <c r="E19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$191,$A19,'QA Checklist'!$H$5:$H$191,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$192,$A19,'QA Checklist'!$H$5:$H$192,"Pending")</f>
         <v/>
       </c>
       <c r="F19" s="8">
@@ -887,19 +887,19 @@
         </is>
       </c>
       <c r="B20" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$191,$A20)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$192,$A20)</f>
         <v/>
       </c>
       <c r="C20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$191,$A20,'QA Checklist'!$H$5:$H$191,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$191,$A20,'QA Checklist'!$H$5:$H$191,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$192,$A20,'QA Checklist'!$H$5:$H$192,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$192,$A20,'QA Checklist'!$H$5:$H$192,"Pass")</f>
         <v/>
       </c>
       <c r="D20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$191,$A20,'QA Checklist'!$H$5:$H$191,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$191,$A20,'QA Checklist'!$H$5:$H$191,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$192,$A20,'QA Checklist'!$H$5:$H$192,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$192,$A20,'QA Checklist'!$H$5:$H$192,"Fail")</f>
         <v/>
       </c>
       <c r="E20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$191,$A20,'QA Checklist'!$H$5:$H$191,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$192,$A20,'QA Checklist'!$H$5:$H$192,"Pending")</f>
         <v/>
       </c>
       <c r="F20" s="8">
@@ -914,19 +914,19 @@
         </is>
       </c>
       <c r="B21" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$191,$A21)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$192,$A21)</f>
         <v/>
       </c>
       <c r="C21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$191,$A21,'QA Checklist'!$H$5:$H$191,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$191,$A21,'QA Checklist'!$H$5:$H$191,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$192,$A21,'QA Checklist'!$H$5:$H$192,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$192,$A21,'QA Checklist'!$H$5:$H$192,"Pass")</f>
         <v/>
       </c>
       <c r="D21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$191,$A21,'QA Checklist'!$H$5:$H$191,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$191,$A21,'QA Checklist'!$H$5:$H$191,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$192,$A21,'QA Checklist'!$H$5:$H$192,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$192,$A21,'QA Checklist'!$H$5:$H$192,"Fail")</f>
         <v/>
       </c>
       <c r="E21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$191,$A21,'QA Checklist'!$H$5:$H$191,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$192,$A21,'QA Checklist'!$H$5:$H$192,"Pending")</f>
         <v/>
       </c>
       <c r="F21" s="8">
@@ -941,19 +941,19 @@
         </is>
       </c>
       <c r="B22" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$191,$A22)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$192,$A22)</f>
         <v/>
       </c>
       <c r="C22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$191,$A22,'QA Checklist'!$H$5:$H$191,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$191,$A22,'QA Checklist'!$H$5:$H$191,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$192,$A22,'QA Checklist'!$H$5:$H$192,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$192,$A22,'QA Checklist'!$H$5:$H$192,"Pass")</f>
         <v/>
       </c>
       <c r="D22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$191,$A22,'QA Checklist'!$H$5:$H$191,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$191,$A22,'QA Checklist'!$H$5:$H$191,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$192,$A22,'QA Checklist'!$H$5:$H$192,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$192,$A22,'QA Checklist'!$H$5:$H$192,"Fail")</f>
         <v/>
       </c>
       <c r="E22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$191,$A22,'QA Checklist'!$H$5:$H$191,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$192,$A22,'QA Checklist'!$H$5:$H$192,"Pending")</f>
         <v/>
       </c>
       <c r="F22" s="8">
@@ -1023,19 +1023,19 @@
         </is>
       </c>
       <c r="B26" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$191,$A26&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$192,$A26&amp;"*")</f>
         <v/>
       </c>
       <c r="C26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$191,$A26&amp;"*",'QA Checklist'!$H$5:$H$191,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$191,$A26&amp;"*",'QA Checklist'!$H$5:$H$191,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$192,$A26&amp;"*",'QA Checklist'!$H$5:$H$192,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$192,$A26&amp;"*",'QA Checklist'!$H$5:$H$192,"Pass")</f>
         <v/>
       </c>
       <c r="D26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$191,$A26&amp;"*",'QA Checklist'!$H$5:$H$191,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$191,$A26&amp;"*",'QA Checklist'!$H$5:$H$191,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$192,$A26&amp;"*",'QA Checklist'!$H$5:$H$192,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$192,$A26&amp;"*",'QA Checklist'!$H$5:$H$192,"Fail")</f>
         <v/>
       </c>
       <c r="E26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$191,$A26&amp;"*",'QA Checklist'!$H$5:$H$191,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$192,$A26&amp;"*",'QA Checklist'!$H$5:$H$192,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1046,19 +1046,19 @@
         </is>
       </c>
       <c r="B27" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$191,$A27&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$192,$A27&amp;"*")</f>
         <v/>
       </c>
       <c r="C27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$191,$A27&amp;"*",'QA Checklist'!$H$5:$H$191,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$191,$A27&amp;"*",'QA Checklist'!$H$5:$H$191,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$192,$A27&amp;"*",'QA Checklist'!$H$5:$H$192,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$192,$A27&amp;"*",'QA Checklist'!$H$5:$H$192,"Pass")</f>
         <v/>
       </c>
       <c r="D27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$191,$A27&amp;"*",'QA Checklist'!$H$5:$H$191,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$191,$A27&amp;"*",'QA Checklist'!$H$5:$H$191,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$192,$A27&amp;"*",'QA Checklist'!$H$5:$H$192,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$192,$A27&amp;"*",'QA Checklist'!$H$5:$H$192,"Fail")</f>
         <v/>
       </c>
       <c r="E27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$191,$A27&amp;"*",'QA Checklist'!$H$5:$H$191,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$192,$A27&amp;"*",'QA Checklist'!$H$5:$H$192,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1069,19 +1069,19 @@
         </is>
       </c>
       <c r="B28" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$191,$A28&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$192,$A28&amp;"*")</f>
         <v/>
       </c>
       <c r="C28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$191,$A28&amp;"*",'QA Checklist'!$H$5:$H$191,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$191,$A28&amp;"*",'QA Checklist'!$H$5:$H$191,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$192,$A28&amp;"*",'QA Checklist'!$H$5:$H$192,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$192,$A28&amp;"*",'QA Checklist'!$H$5:$H$192,"Pass")</f>
         <v/>
       </c>
       <c r="D28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$191,$A28&amp;"*",'QA Checklist'!$H$5:$H$191,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$191,$A28&amp;"*",'QA Checklist'!$H$5:$H$191,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$192,$A28&amp;"*",'QA Checklist'!$H$5:$H$192,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$192,$A28&amp;"*",'QA Checklist'!$H$5:$H$192,"Fail")</f>
         <v/>
       </c>
       <c r="E28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$191,$A28&amp;"*",'QA Checklist'!$H$5:$H$191,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$192,$A28&amp;"*",'QA Checklist'!$H$5:$H$192,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1096,7 +1096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I191"/>
+  <dimension ref="A1:I192"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9516,12 +9516,59 @@
         </is>
       </c>
     </row>
+    <row r="192">
+      <c r="A192" s="12" t="inlineStr">
+        <is>
+          <t>SA-66</t>
+        </is>
+      </c>
+      <c r="B192" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="C192" s="13" t="inlineStr">
+        <is>
+          <t>Tier 2 (Workflow &amp; Ergonomics)</t>
+        </is>
+      </c>
+      <c r="D192" s="13" t="inlineStr">
+        <is>
+          <t>TV Weather Box</t>
+        </is>
+      </c>
+      <c r="E192" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="F192" s="13" t="inlineStr">
+        <is>
+          <t>Open the Marikina and Regalado TVs, compare the weather box with a weather app for each area, then disconnect the server PC from the internet for 20 minutes</t>
+        </is>
+      </c>
+      <c r="G192" s="13" t="inlineStr">
+        <is>
+          <t>Each TV shows its branch temperature, condition, feels like and humidity (rain line only when rain is expected); offline it keeps the last reading with "As of hh:mm", or shows "Weather unavailable" - never made-up numbers</t>
+        </is>
+      </c>
+      <c r="H192" s="14" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="I192" s="13" t="inlineStr">
+        <is>
+          <t>Verified by Automated Unit Tests (178 passing in tests/frontend/sla_and_logic.test.js AUT-FRONT-149), server checks 6/6 and headless Chrome 7/7 on XAMPP</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:I191"/>
+  <autoFilter ref="A4:I192"/>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="H5:H191">
+  <conditionalFormatting sqref="H5:H192">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$H5="Passed"</formula>
     </cfRule>
@@ -9538,13 +9585,13 @@
       <formula>$H5="Pending"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A5:A191">
+  <conditionalFormatting sqref="A5:A192">
     <cfRule type="expression" priority="6" dxfId="3">
-      <formula>COUNTIF($A$5:$A$191,$A5)&gt;1</formula>
+      <formula>COUNTIF($A$5:$A$192,$A5)&gt;1</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H5:H191" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H5:H192" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pending,Passed,Failed"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat(REV-191): developer TV simulation in the Ctrl+D toolbox, locked to development
The lounge TV no longer has a developer drawer. The Ctrl+D toolbox opens only for a logged-in user when the server runs with APP_ENV=development, and its TV simulator (7 events) records real announcements for the user's branch TV via /auth/developer/tv-simulate. Old app-only simulation code removed. Cache buster v=3.44, AUT-FRONT-150, SA-67.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
+++ b/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
@@ -11,7 +11,7 @@
     <sheet name="QA Checklist" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$192</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$193</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'QA Checklist'!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTA('QA Checklist'!$A$5:$A$192)</f>
+        <f>COUNTA('QA Checklist'!$A$5:$A$193)</f>
         <v/>
       </c>
     </row>
@@ -594,7 +594,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$192,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$192,"Pass")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$193,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$193,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$192,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$192,"Fail")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$193,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$193,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -616,7 +616,7 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$192,"Pending")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$193,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -671,19 +671,19 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$192,$A12)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$193,$A12)</f>
         <v/>
       </c>
       <c r="C12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$192,$A12,'QA Checklist'!$H$5:$H$192,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$192,$A12,'QA Checklist'!$H$5:$H$192,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$193,$A12,'QA Checklist'!$H$5:$H$193,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$193,$A12,'QA Checklist'!$H$5:$H$193,"Pass")</f>
         <v/>
       </c>
       <c r="D12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$192,$A12,'QA Checklist'!$H$5:$H$192,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$192,$A12,'QA Checklist'!$H$5:$H$192,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$193,$A12,'QA Checklist'!$H$5:$H$193,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$193,$A12,'QA Checklist'!$H$5:$H$193,"Fail")</f>
         <v/>
       </c>
       <c r="E12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$192,$A12,'QA Checklist'!$H$5:$H$192,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$193,$A12,'QA Checklist'!$H$5:$H$193,"Pending")</f>
         <v/>
       </c>
       <c r="F12" s="8">
@@ -698,19 +698,19 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$192,$A13)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$193,$A13)</f>
         <v/>
       </c>
       <c r="C13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$192,$A13,'QA Checklist'!$H$5:$H$192,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$192,$A13,'QA Checklist'!$H$5:$H$192,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$193,$A13,'QA Checklist'!$H$5:$H$193,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$193,$A13,'QA Checklist'!$H$5:$H$193,"Pass")</f>
         <v/>
       </c>
       <c r="D13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$192,$A13,'QA Checklist'!$H$5:$H$192,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$192,$A13,'QA Checklist'!$H$5:$H$192,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$193,$A13,'QA Checklist'!$H$5:$H$193,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$193,$A13,'QA Checklist'!$H$5:$H$193,"Fail")</f>
         <v/>
       </c>
       <c r="E13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$192,$A13,'QA Checklist'!$H$5:$H$192,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$193,$A13,'QA Checklist'!$H$5:$H$193,"Pending")</f>
         <v/>
       </c>
       <c r="F13" s="8">
@@ -725,19 +725,19 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$192,$A14)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$193,$A14)</f>
         <v/>
       </c>
       <c r="C14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$192,$A14,'QA Checklist'!$H$5:$H$192,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$192,$A14,'QA Checklist'!$H$5:$H$192,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$193,$A14,'QA Checklist'!$H$5:$H$193,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$193,$A14,'QA Checklist'!$H$5:$H$193,"Pass")</f>
         <v/>
       </c>
       <c r="D14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$192,$A14,'QA Checklist'!$H$5:$H$192,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$192,$A14,'QA Checklist'!$H$5:$H$192,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$193,$A14,'QA Checklist'!$H$5:$H$193,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$193,$A14,'QA Checklist'!$H$5:$H$193,"Fail")</f>
         <v/>
       </c>
       <c r="E14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$192,$A14,'QA Checklist'!$H$5:$H$192,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$193,$A14,'QA Checklist'!$H$5:$H$193,"Pending")</f>
         <v/>
       </c>
       <c r="F14" s="8">
@@ -752,19 +752,19 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$192,$A15)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$193,$A15)</f>
         <v/>
       </c>
       <c r="C15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$192,$A15,'QA Checklist'!$H$5:$H$192,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$192,$A15,'QA Checklist'!$H$5:$H$192,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$193,$A15,'QA Checklist'!$H$5:$H$193,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$193,$A15,'QA Checklist'!$H$5:$H$193,"Pass")</f>
         <v/>
       </c>
       <c r="D15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$192,$A15,'QA Checklist'!$H$5:$H$192,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$192,$A15,'QA Checklist'!$H$5:$H$192,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$193,$A15,'QA Checklist'!$H$5:$H$193,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$193,$A15,'QA Checklist'!$H$5:$H$193,"Fail")</f>
         <v/>
       </c>
       <c r="E15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$192,$A15,'QA Checklist'!$H$5:$H$192,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$193,$A15,'QA Checklist'!$H$5:$H$193,"Pending")</f>
         <v/>
       </c>
       <c r="F15" s="8">
@@ -779,19 +779,19 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$192,$A16)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$193,$A16)</f>
         <v/>
       </c>
       <c r="C16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$192,$A16,'QA Checklist'!$H$5:$H$192,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$192,$A16,'QA Checklist'!$H$5:$H$192,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$193,$A16,'QA Checklist'!$H$5:$H$193,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$193,$A16,'QA Checklist'!$H$5:$H$193,"Pass")</f>
         <v/>
       </c>
       <c r="D16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$192,$A16,'QA Checklist'!$H$5:$H$192,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$192,$A16,'QA Checklist'!$H$5:$H$192,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$193,$A16,'QA Checklist'!$H$5:$H$193,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$193,$A16,'QA Checklist'!$H$5:$H$193,"Fail")</f>
         <v/>
       </c>
       <c r="E16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$192,$A16,'QA Checklist'!$H$5:$H$192,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$193,$A16,'QA Checklist'!$H$5:$H$193,"Pending")</f>
         <v/>
       </c>
       <c r="F16" s="8">
@@ -806,19 +806,19 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$192,$A17)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$193,$A17)</f>
         <v/>
       </c>
       <c r="C17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$192,$A17,'QA Checklist'!$H$5:$H$192,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$192,$A17,'QA Checklist'!$H$5:$H$192,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$193,$A17,'QA Checklist'!$H$5:$H$193,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$193,$A17,'QA Checklist'!$H$5:$H$193,"Pass")</f>
         <v/>
       </c>
       <c r="D17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$192,$A17,'QA Checklist'!$H$5:$H$192,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$192,$A17,'QA Checklist'!$H$5:$H$192,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$193,$A17,'QA Checklist'!$H$5:$H$193,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$193,$A17,'QA Checklist'!$H$5:$H$193,"Fail")</f>
         <v/>
       </c>
       <c r="E17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$192,$A17,'QA Checklist'!$H$5:$H$192,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$193,$A17,'QA Checklist'!$H$5:$H$193,"Pending")</f>
         <v/>
       </c>
       <c r="F17" s="8">
@@ -833,19 +833,19 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$192,$A18)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$193,$A18)</f>
         <v/>
       </c>
       <c r="C18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$192,$A18,'QA Checklist'!$H$5:$H$192,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$192,$A18,'QA Checklist'!$H$5:$H$192,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$193,$A18,'QA Checklist'!$H$5:$H$193,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$193,$A18,'QA Checklist'!$H$5:$H$193,"Pass")</f>
         <v/>
       </c>
       <c r="D18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$192,$A18,'QA Checklist'!$H$5:$H$192,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$192,$A18,'QA Checklist'!$H$5:$H$192,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$193,$A18,'QA Checklist'!$H$5:$H$193,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$193,$A18,'QA Checklist'!$H$5:$H$193,"Fail")</f>
         <v/>
       </c>
       <c r="E18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$192,$A18,'QA Checklist'!$H$5:$H$192,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$193,$A18,'QA Checklist'!$H$5:$H$193,"Pending")</f>
         <v/>
       </c>
       <c r="F18" s="8">
@@ -860,19 +860,19 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$192,$A19)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$193,$A19)</f>
         <v/>
       </c>
       <c r="C19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$192,$A19,'QA Checklist'!$H$5:$H$192,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$192,$A19,'QA Checklist'!$H$5:$H$192,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$193,$A19,'QA Checklist'!$H$5:$H$193,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$193,$A19,'QA Checklist'!$H$5:$H$193,"Pass")</f>
         <v/>
       </c>
       <c r="D19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$192,$A19,'QA Checklist'!$H$5:$H$192,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$192,$A19,'QA Checklist'!$H$5:$H$192,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$193,$A19,'QA Checklist'!$H$5:$H$193,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$193,$A19,'QA Checklist'!$H$5:$H$193,"Fail")</f>
         <v/>
       </c>
       <c r="E19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$192,$A19,'QA Checklist'!$H$5:$H$192,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$193,$A19,'QA Checklist'!$H$5:$H$193,"Pending")</f>
         <v/>
       </c>
       <c r="F19" s="8">
@@ -887,19 +887,19 @@
         </is>
       </c>
       <c r="B20" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$192,$A20)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$193,$A20)</f>
         <v/>
       </c>
       <c r="C20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$192,$A20,'QA Checklist'!$H$5:$H$192,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$192,$A20,'QA Checklist'!$H$5:$H$192,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$193,$A20,'QA Checklist'!$H$5:$H$193,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$193,$A20,'QA Checklist'!$H$5:$H$193,"Pass")</f>
         <v/>
       </c>
       <c r="D20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$192,$A20,'QA Checklist'!$H$5:$H$192,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$192,$A20,'QA Checklist'!$H$5:$H$192,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$193,$A20,'QA Checklist'!$H$5:$H$193,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$193,$A20,'QA Checklist'!$H$5:$H$193,"Fail")</f>
         <v/>
       </c>
       <c r="E20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$192,$A20,'QA Checklist'!$H$5:$H$192,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$193,$A20,'QA Checklist'!$H$5:$H$193,"Pending")</f>
         <v/>
       </c>
       <c r="F20" s="8">
@@ -914,19 +914,19 @@
         </is>
       </c>
       <c r="B21" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$192,$A21)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$193,$A21)</f>
         <v/>
       </c>
       <c r="C21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$192,$A21,'QA Checklist'!$H$5:$H$192,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$192,$A21,'QA Checklist'!$H$5:$H$192,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$193,$A21,'QA Checklist'!$H$5:$H$193,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$193,$A21,'QA Checklist'!$H$5:$H$193,"Pass")</f>
         <v/>
       </c>
       <c r="D21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$192,$A21,'QA Checklist'!$H$5:$H$192,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$192,$A21,'QA Checklist'!$H$5:$H$192,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$193,$A21,'QA Checklist'!$H$5:$H$193,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$193,$A21,'QA Checklist'!$H$5:$H$193,"Fail")</f>
         <v/>
       </c>
       <c r="E21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$192,$A21,'QA Checklist'!$H$5:$H$192,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$193,$A21,'QA Checklist'!$H$5:$H$193,"Pending")</f>
         <v/>
       </c>
       <c r="F21" s="8">
@@ -941,19 +941,19 @@
         </is>
       </c>
       <c r="B22" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$192,$A22)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$193,$A22)</f>
         <v/>
       </c>
       <c r="C22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$192,$A22,'QA Checklist'!$H$5:$H$192,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$192,$A22,'QA Checklist'!$H$5:$H$192,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$193,$A22,'QA Checklist'!$H$5:$H$193,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$193,$A22,'QA Checklist'!$H$5:$H$193,"Pass")</f>
         <v/>
       </c>
       <c r="D22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$192,$A22,'QA Checklist'!$H$5:$H$192,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$192,$A22,'QA Checklist'!$H$5:$H$192,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$193,$A22,'QA Checklist'!$H$5:$H$193,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$193,$A22,'QA Checklist'!$H$5:$H$193,"Fail")</f>
         <v/>
       </c>
       <c r="E22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$192,$A22,'QA Checklist'!$H$5:$H$192,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$193,$A22,'QA Checklist'!$H$5:$H$193,"Pending")</f>
         <v/>
       </c>
       <c r="F22" s="8">
@@ -1023,19 +1023,19 @@
         </is>
       </c>
       <c r="B26" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$192,$A26&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$193,$A26&amp;"*")</f>
         <v/>
       </c>
       <c r="C26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$192,$A26&amp;"*",'QA Checklist'!$H$5:$H$192,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$192,$A26&amp;"*",'QA Checklist'!$H$5:$H$192,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$193,$A26&amp;"*",'QA Checklist'!$H$5:$H$193,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$193,$A26&amp;"*",'QA Checklist'!$H$5:$H$193,"Pass")</f>
         <v/>
       </c>
       <c r="D26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$192,$A26&amp;"*",'QA Checklist'!$H$5:$H$192,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$192,$A26&amp;"*",'QA Checklist'!$H$5:$H$192,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$193,$A26&amp;"*",'QA Checklist'!$H$5:$H$193,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$193,$A26&amp;"*",'QA Checklist'!$H$5:$H$193,"Fail")</f>
         <v/>
       </c>
       <c r="E26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$192,$A26&amp;"*",'QA Checklist'!$H$5:$H$192,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$193,$A26&amp;"*",'QA Checklist'!$H$5:$H$193,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1046,19 +1046,19 @@
         </is>
       </c>
       <c r="B27" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$192,$A27&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$193,$A27&amp;"*")</f>
         <v/>
       </c>
       <c r="C27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$192,$A27&amp;"*",'QA Checklist'!$H$5:$H$192,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$192,$A27&amp;"*",'QA Checklist'!$H$5:$H$192,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$193,$A27&amp;"*",'QA Checklist'!$H$5:$H$193,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$193,$A27&amp;"*",'QA Checklist'!$H$5:$H$193,"Pass")</f>
         <v/>
       </c>
       <c r="D27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$192,$A27&amp;"*",'QA Checklist'!$H$5:$H$192,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$192,$A27&amp;"*",'QA Checklist'!$H$5:$H$192,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$193,$A27&amp;"*",'QA Checklist'!$H$5:$H$193,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$193,$A27&amp;"*",'QA Checklist'!$H$5:$H$193,"Fail")</f>
         <v/>
       </c>
       <c r="E27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$192,$A27&amp;"*",'QA Checklist'!$H$5:$H$192,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$193,$A27&amp;"*",'QA Checklist'!$H$5:$H$193,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1069,19 +1069,19 @@
         </is>
       </c>
       <c r="B28" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$192,$A28&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$193,$A28&amp;"*")</f>
         <v/>
       </c>
       <c r="C28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$192,$A28&amp;"*",'QA Checklist'!$H$5:$H$192,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$192,$A28&amp;"*",'QA Checklist'!$H$5:$H$192,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$193,$A28&amp;"*",'QA Checklist'!$H$5:$H$193,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$193,$A28&amp;"*",'QA Checklist'!$H$5:$H$193,"Pass")</f>
         <v/>
       </c>
       <c r="D28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$192,$A28&amp;"*",'QA Checklist'!$H$5:$H$192,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$192,$A28&amp;"*",'QA Checklist'!$H$5:$H$192,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$193,$A28&amp;"*",'QA Checklist'!$H$5:$H$193,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$193,$A28&amp;"*",'QA Checklist'!$H$5:$H$193,"Fail")</f>
         <v/>
       </c>
       <c r="E28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$192,$A28&amp;"*",'QA Checklist'!$H$5:$H$192,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$193,$A28&amp;"*",'QA Checklist'!$H$5:$H$193,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1096,7 +1096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I192"/>
+  <dimension ref="A1:I193"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9563,12 +9563,59 @@
         </is>
       </c>
     </row>
+    <row r="193">
+      <c r="A193" s="12" t="inlineStr">
+        <is>
+          <t>SA-67</t>
+        </is>
+      </c>
+      <c r="B193" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="C193" s="13" t="inlineStr">
+        <is>
+          <t>Tier 2 (Workflow &amp; Ergonomics)</t>
+        </is>
+      </c>
+      <c r="D193" s="13" t="inlineStr">
+        <is>
+          <t>Developer Toolbox (Ctrl+D) &amp; TV Simulation</t>
+        </is>
+      </c>
+      <c r="E193" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="F193" s="13" t="inlineStr">
+        <is>
+          <t>On the login screen press Ctrl+D; log in as SA and press Ctrl+D; with the branch TV live press Released and Call Customer Again in the toolbox; open the TV page and look for developer controls; repeat Ctrl+D on a server with APP_ENV=production</t>
+        </is>
+      </c>
+      <c r="G193" s="13" t="inlineStr">
+        <is>
+          <t>Ctrl+D does nothing when logged out or in production; for a logged-in user in development it opens the toolbox and the TV plays the simulated announcements; the TV page has no developer controls</t>
+        </is>
+      </c>
+      <c r="H193" s="14" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="I193" s="13" t="inlineStr">
+        <is>
+          <t>Verified by Automated Unit Tests (179 passing in tests/frontend/sla_and_logic.test.js AUT-FRONT-150) and headless Chrome 8/8 (development and production-mode servers)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:I192"/>
+  <autoFilter ref="A4:I193"/>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="H5:H192">
+  <conditionalFormatting sqref="H5:H193">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$H5="Passed"</formula>
     </cfRule>
@@ -9585,13 +9632,13 @@
       <formula>$H5="Pending"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A5:A192">
+  <conditionalFormatting sqref="A5:A193">
     <cfRule type="expression" priority="6" dxfId="3">
-      <formula>COUNTIF($A$5:$A$192,$A5)&gt;1</formula>
+      <formula>COUNTIF($A$5:$A$193,$A5)&gt;1</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H5:H192" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H5:H193" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pending,Passed,Failed"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat(REV-192): simple TV weather box with the real branch reading
Restore the old two-line weather box (icon, temperature, condition); drop the feels-like, rain, as-of and credit lines. Data is still the server-cached Open-Meteo reading per branch.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
+++ b/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
@@ -11,7 +11,7 @@
     <sheet name="QA Checklist" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$193</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$194</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'QA Checklist'!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTA('QA Checklist'!$A$5:$A$193)</f>
+        <f>COUNTA('QA Checklist'!$A$5:$A$194)</f>
         <v/>
       </c>
     </row>
@@ -594,7 +594,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$193,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$193,"Pass")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$194,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$194,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$193,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$193,"Fail")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$194,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$194,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -616,7 +616,7 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$193,"Pending")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$194,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -671,19 +671,19 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$193,$A12)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$194,$A12)</f>
         <v/>
       </c>
       <c r="C12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$193,$A12,'QA Checklist'!$H$5:$H$193,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$193,$A12,'QA Checklist'!$H$5:$H$193,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$194,$A12,'QA Checklist'!$H$5:$H$194,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$194,$A12,'QA Checklist'!$H$5:$H$194,"Pass")</f>
         <v/>
       </c>
       <c r="D12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$193,$A12,'QA Checklist'!$H$5:$H$193,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$193,$A12,'QA Checklist'!$H$5:$H$193,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$194,$A12,'QA Checklist'!$H$5:$H$194,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$194,$A12,'QA Checklist'!$H$5:$H$194,"Fail")</f>
         <v/>
       </c>
       <c r="E12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$193,$A12,'QA Checklist'!$H$5:$H$193,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$194,$A12,'QA Checklist'!$H$5:$H$194,"Pending")</f>
         <v/>
       </c>
       <c r="F12" s="8">
@@ -698,19 +698,19 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$193,$A13)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$194,$A13)</f>
         <v/>
       </c>
       <c r="C13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$193,$A13,'QA Checklist'!$H$5:$H$193,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$193,$A13,'QA Checklist'!$H$5:$H$193,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$194,$A13,'QA Checklist'!$H$5:$H$194,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$194,$A13,'QA Checklist'!$H$5:$H$194,"Pass")</f>
         <v/>
       </c>
       <c r="D13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$193,$A13,'QA Checklist'!$H$5:$H$193,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$193,$A13,'QA Checklist'!$H$5:$H$193,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$194,$A13,'QA Checklist'!$H$5:$H$194,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$194,$A13,'QA Checklist'!$H$5:$H$194,"Fail")</f>
         <v/>
       </c>
       <c r="E13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$193,$A13,'QA Checklist'!$H$5:$H$193,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$194,$A13,'QA Checklist'!$H$5:$H$194,"Pending")</f>
         <v/>
       </c>
       <c r="F13" s="8">
@@ -725,19 +725,19 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$193,$A14)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$194,$A14)</f>
         <v/>
       </c>
       <c r="C14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$193,$A14,'QA Checklist'!$H$5:$H$193,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$193,$A14,'QA Checklist'!$H$5:$H$193,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$194,$A14,'QA Checklist'!$H$5:$H$194,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$194,$A14,'QA Checklist'!$H$5:$H$194,"Pass")</f>
         <v/>
       </c>
       <c r="D14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$193,$A14,'QA Checklist'!$H$5:$H$193,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$193,$A14,'QA Checklist'!$H$5:$H$193,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$194,$A14,'QA Checklist'!$H$5:$H$194,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$194,$A14,'QA Checklist'!$H$5:$H$194,"Fail")</f>
         <v/>
       </c>
       <c r="E14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$193,$A14,'QA Checklist'!$H$5:$H$193,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$194,$A14,'QA Checklist'!$H$5:$H$194,"Pending")</f>
         <v/>
       </c>
       <c r="F14" s="8">
@@ -752,19 +752,19 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$193,$A15)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$194,$A15)</f>
         <v/>
       </c>
       <c r="C15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$193,$A15,'QA Checklist'!$H$5:$H$193,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$193,$A15,'QA Checklist'!$H$5:$H$193,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$194,$A15,'QA Checklist'!$H$5:$H$194,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$194,$A15,'QA Checklist'!$H$5:$H$194,"Pass")</f>
         <v/>
       </c>
       <c r="D15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$193,$A15,'QA Checklist'!$H$5:$H$193,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$193,$A15,'QA Checklist'!$H$5:$H$193,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$194,$A15,'QA Checklist'!$H$5:$H$194,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$194,$A15,'QA Checklist'!$H$5:$H$194,"Fail")</f>
         <v/>
       </c>
       <c r="E15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$193,$A15,'QA Checklist'!$H$5:$H$193,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$194,$A15,'QA Checklist'!$H$5:$H$194,"Pending")</f>
         <v/>
       </c>
       <c r="F15" s="8">
@@ -779,19 +779,19 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$193,$A16)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$194,$A16)</f>
         <v/>
       </c>
       <c r="C16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$193,$A16,'QA Checklist'!$H$5:$H$193,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$193,$A16,'QA Checklist'!$H$5:$H$193,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$194,$A16,'QA Checklist'!$H$5:$H$194,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$194,$A16,'QA Checklist'!$H$5:$H$194,"Pass")</f>
         <v/>
       </c>
       <c r="D16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$193,$A16,'QA Checklist'!$H$5:$H$193,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$193,$A16,'QA Checklist'!$H$5:$H$193,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$194,$A16,'QA Checklist'!$H$5:$H$194,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$194,$A16,'QA Checklist'!$H$5:$H$194,"Fail")</f>
         <v/>
       </c>
       <c r="E16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$193,$A16,'QA Checklist'!$H$5:$H$193,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$194,$A16,'QA Checklist'!$H$5:$H$194,"Pending")</f>
         <v/>
       </c>
       <c r="F16" s="8">
@@ -806,19 +806,19 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$193,$A17)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$194,$A17)</f>
         <v/>
       </c>
       <c r="C17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$193,$A17,'QA Checklist'!$H$5:$H$193,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$193,$A17,'QA Checklist'!$H$5:$H$193,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$194,$A17,'QA Checklist'!$H$5:$H$194,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$194,$A17,'QA Checklist'!$H$5:$H$194,"Pass")</f>
         <v/>
       </c>
       <c r="D17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$193,$A17,'QA Checklist'!$H$5:$H$193,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$193,$A17,'QA Checklist'!$H$5:$H$193,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$194,$A17,'QA Checklist'!$H$5:$H$194,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$194,$A17,'QA Checklist'!$H$5:$H$194,"Fail")</f>
         <v/>
       </c>
       <c r="E17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$193,$A17,'QA Checklist'!$H$5:$H$193,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$194,$A17,'QA Checklist'!$H$5:$H$194,"Pending")</f>
         <v/>
       </c>
       <c r="F17" s="8">
@@ -833,19 +833,19 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$193,$A18)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$194,$A18)</f>
         <v/>
       </c>
       <c r="C18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$193,$A18,'QA Checklist'!$H$5:$H$193,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$193,$A18,'QA Checklist'!$H$5:$H$193,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$194,$A18,'QA Checklist'!$H$5:$H$194,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$194,$A18,'QA Checklist'!$H$5:$H$194,"Pass")</f>
         <v/>
       </c>
       <c r="D18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$193,$A18,'QA Checklist'!$H$5:$H$193,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$193,$A18,'QA Checklist'!$H$5:$H$193,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$194,$A18,'QA Checklist'!$H$5:$H$194,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$194,$A18,'QA Checklist'!$H$5:$H$194,"Fail")</f>
         <v/>
       </c>
       <c r="E18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$193,$A18,'QA Checklist'!$H$5:$H$193,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$194,$A18,'QA Checklist'!$H$5:$H$194,"Pending")</f>
         <v/>
       </c>
       <c r="F18" s="8">
@@ -860,19 +860,19 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$193,$A19)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$194,$A19)</f>
         <v/>
       </c>
       <c r="C19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$193,$A19,'QA Checklist'!$H$5:$H$193,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$193,$A19,'QA Checklist'!$H$5:$H$193,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$194,$A19,'QA Checklist'!$H$5:$H$194,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$194,$A19,'QA Checklist'!$H$5:$H$194,"Pass")</f>
         <v/>
       </c>
       <c r="D19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$193,$A19,'QA Checklist'!$H$5:$H$193,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$193,$A19,'QA Checklist'!$H$5:$H$193,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$194,$A19,'QA Checklist'!$H$5:$H$194,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$194,$A19,'QA Checklist'!$H$5:$H$194,"Fail")</f>
         <v/>
       </c>
       <c r="E19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$193,$A19,'QA Checklist'!$H$5:$H$193,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$194,$A19,'QA Checklist'!$H$5:$H$194,"Pending")</f>
         <v/>
       </c>
       <c r="F19" s="8">
@@ -887,19 +887,19 @@
         </is>
       </c>
       <c r="B20" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$193,$A20)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$194,$A20)</f>
         <v/>
       </c>
       <c r="C20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$193,$A20,'QA Checklist'!$H$5:$H$193,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$193,$A20,'QA Checklist'!$H$5:$H$193,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$194,$A20,'QA Checklist'!$H$5:$H$194,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$194,$A20,'QA Checklist'!$H$5:$H$194,"Pass")</f>
         <v/>
       </c>
       <c r="D20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$193,$A20,'QA Checklist'!$H$5:$H$193,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$193,$A20,'QA Checklist'!$H$5:$H$193,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$194,$A20,'QA Checklist'!$H$5:$H$194,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$194,$A20,'QA Checklist'!$H$5:$H$194,"Fail")</f>
         <v/>
       </c>
       <c r="E20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$193,$A20,'QA Checklist'!$H$5:$H$193,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$194,$A20,'QA Checklist'!$H$5:$H$194,"Pending")</f>
         <v/>
       </c>
       <c r="F20" s="8">
@@ -914,19 +914,19 @@
         </is>
       </c>
       <c r="B21" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$193,$A21)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$194,$A21)</f>
         <v/>
       </c>
       <c r="C21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$193,$A21,'QA Checklist'!$H$5:$H$193,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$193,$A21,'QA Checklist'!$H$5:$H$193,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$194,$A21,'QA Checklist'!$H$5:$H$194,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$194,$A21,'QA Checklist'!$H$5:$H$194,"Pass")</f>
         <v/>
       </c>
       <c r="D21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$193,$A21,'QA Checklist'!$H$5:$H$193,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$193,$A21,'QA Checklist'!$H$5:$H$193,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$194,$A21,'QA Checklist'!$H$5:$H$194,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$194,$A21,'QA Checklist'!$H$5:$H$194,"Fail")</f>
         <v/>
       </c>
       <c r="E21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$193,$A21,'QA Checklist'!$H$5:$H$193,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$194,$A21,'QA Checklist'!$H$5:$H$194,"Pending")</f>
         <v/>
       </c>
       <c r="F21" s="8">
@@ -941,19 +941,19 @@
         </is>
       </c>
       <c r="B22" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$193,$A22)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$194,$A22)</f>
         <v/>
       </c>
       <c r="C22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$193,$A22,'QA Checklist'!$H$5:$H$193,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$193,$A22,'QA Checklist'!$H$5:$H$193,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$194,$A22,'QA Checklist'!$H$5:$H$194,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$194,$A22,'QA Checklist'!$H$5:$H$194,"Pass")</f>
         <v/>
       </c>
       <c r="D22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$193,$A22,'QA Checklist'!$H$5:$H$193,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$193,$A22,'QA Checklist'!$H$5:$H$193,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$194,$A22,'QA Checklist'!$H$5:$H$194,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$194,$A22,'QA Checklist'!$H$5:$H$194,"Fail")</f>
         <v/>
       </c>
       <c r="E22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$193,$A22,'QA Checklist'!$H$5:$H$193,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$194,$A22,'QA Checklist'!$H$5:$H$194,"Pending")</f>
         <v/>
       </c>
       <c r="F22" s="8">
@@ -1023,19 +1023,19 @@
         </is>
       </c>
       <c r="B26" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$193,$A26&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$194,$A26&amp;"*")</f>
         <v/>
       </c>
       <c r="C26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$193,$A26&amp;"*",'QA Checklist'!$H$5:$H$193,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$193,$A26&amp;"*",'QA Checklist'!$H$5:$H$193,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$194,$A26&amp;"*",'QA Checklist'!$H$5:$H$194,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$194,$A26&amp;"*",'QA Checklist'!$H$5:$H$194,"Pass")</f>
         <v/>
       </c>
       <c r="D26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$193,$A26&amp;"*",'QA Checklist'!$H$5:$H$193,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$193,$A26&amp;"*",'QA Checklist'!$H$5:$H$193,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$194,$A26&amp;"*",'QA Checklist'!$H$5:$H$194,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$194,$A26&amp;"*",'QA Checklist'!$H$5:$H$194,"Fail")</f>
         <v/>
       </c>
       <c r="E26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$193,$A26&amp;"*",'QA Checklist'!$H$5:$H$193,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$194,$A26&amp;"*",'QA Checklist'!$H$5:$H$194,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1046,19 +1046,19 @@
         </is>
       </c>
       <c r="B27" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$193,$A27&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$194,$A27&amp;"*")</f>
         <v/>
       </c>
       <c r="C27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$193,$A27&amp;"*",'QA Checklist'!$H$5:$H$193,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$193,$A27&amp;"*",'QA Checklist'!$H$5:$H$193,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$194,$A27&amp;"*",'QA Checklist'!$H$5:$H$194,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$194,$A27&amp;"*",'QA Checklist'!$H$5:$H$194,"Pass")</f>
         <v/>
       </c>
       <c r="D27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$193,$A27&amp;"*",'QA Checklist'!$H$5:$H$193,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$193,$A27&amp;"*",'QA Checklist'!$H$5:$H$193,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$194,$A27&amp;"*",'QA Checklist'!$H$5:$H$194,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$194,$A27&amp;"*",'QA Checklist'!$H$5:$H$194,"Fail")</f>
         <v/>
       </c>
       <c r="E27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$193,$A27&amp;"*",'QA Checklist'!$H$5:$H$193,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$194,$A27&amp;"*",'QA Checklist'!$H$5:$H$194,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1069,19 +1069,19 @@
         </is>
       </c>
       <c r="B28" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$193,$A28&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$194,$A28&amp;"*")</f>
         <v/>
       </c>
       <c r="C28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$193,$A28&amp;"*",'QA Checklist'!$H$5:$H$193,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$193,$A28&amp;"*",'QA Checklist'!$H$5:$H$193,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$194,$A28&amp;"*",'QA Checklist'!$H$5:$H$194,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$194,$A28&amp;"*",'QA Checklist'!$H$5:$H$194,"Pass")</f>
         <v/>
       </c>
       <c r="D28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$193,$A28&amp;"*",'QA Checklist'!$H$5:$H$193,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$193,$A28&amp;"*",'QA Checklist'!$H$5:$H$193,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$194,$A28&amp;"*",'QA Checklist'!$H$5:$H$194,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$194,$A28&amp;"*",'QA Checklist'!$H$5:$H$194,"Fail")</f>
         <v/>
       </c>
       <c r="E28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$193,$A28&amp;"*",'QA Checklist'!$H$5:$H$193,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$194,$A28&amp;"*",'QA Checklist'!$H$5:$H$194,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1096,7 +1096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I193"/>
+  <dimension ref="A1:I194"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9610,12 +9610,59 @@
         </is>
       </c>
     </row>
+    <row r="194">
+      <c r="A194" s="12" t="inlineStr">
+        <is>
+          <t>SA-68</t>
+        </is>
+      </c>
+      <c r="B194" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="C194" s="13" t="inlineStr">
+        <is>
+          <t>Tier 2 (Workflow &amp; Ergonomics)</t>
+        </is>
+      </c>
+      <c r="D194" s="13" t="inlineStr">
+        <is>
+          <t>TV Weather Box (Simple)</t>
+        </is>
+      </c>
+      <c r="E194" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="F194" s="13" t="inlineStr">
+        <is>
+          <t>Start the branch broadcast, open the TV page and enter the PIN; compare the weather box with the current weather for the branch; repeat on the other branch</t>
+        </is>
+      </c>
+      <c r="G194" s="13" t="inlineStr">
+        <is>
+          <t>The box shows only an icon, the real temperature and the condition for that branch; with no reading it shows --°C / Unavailable</t>
+        </is>
+      </c>
+      <c r="H194" s="14" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="I194" s="13" t="inlineStr">
+        <is>
+          <t>Verified by Automated Unit Tests (180 passing in tests/frontend/sla_and_logic.test.js AUT-FRONT-151) and headless Chrome 5/5 (both branch TVs)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:I193"/>
+  <autoFilter ref="A4:I194"/>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="H5:H193">
+  <conditionalFormatting sqref="H5:H194">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$H5="Passed"</formula>
     </cfRule>
@@ -9632,13 +9679,13 @@
       <formula>$H5="Pending"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A5:A193">
+  <conditionalFormatting sqref="A5:A194">
     <cfRule type="expression" priority="6" dxfId="3">
-      <formula>COUNTIF($A$5:$A$193,$A5)&gt;1</formula>
+      <formula>COUNTIF($A$5:$A$194,$A5)&gt;1</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H5:H193" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H5:H194" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pending,Passed,Failed"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat(REV-193): Customer Lookup with the RO Excel Studio sheet-tab design
Sheets-style filter tabs, studio search card and gray section heads; dossier split into Customer_Details and Service_History tabs; studio buttons and flat cards. Filtering, search and actions unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
+++ b/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
@@ -11,7 +11,7 @@
     <sheet name="QA Checklist" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$194</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$195</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'QA Checklist'!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTA('QA Checklist'!$A$5:$A$194)</f>
+        <f>COUNTA('QA Checklist'!$A$5:$A$195)</f>
         <v/>
       </c>
     </row>
@@ -594,7 +594,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$194,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$194,"Pass")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$195,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$195,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$194,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$194,"Fail")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$195,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$195,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -616,7 +616,7 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$194,"Pending")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$195,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -671,19 +671,19 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$194,$A12)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$195,$A12)</f>
         <v/>
       </c>
       <c r="C12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$194,$A12,'QA Checklist'!$H$5:$H$194,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$194,$A12,'QA Checklist'!$H$5:$H$194,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$195,$A12,'QA Checklist'!$H$5:$H$195,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$195,$A12,'QA Checklist'!$H$5:$H$195,"Pass")</f>
         <v/>
       </c>
       <c r="D12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$194,$A12,'QA Checklist'!$H$5:$H$194,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$194,$A12,'QA Checklist'!$H$5:$H$194,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$195,$A12,'QA Checklist'!$H$5:$H$195,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$195,$A12,'QA Checklist'!$H$5:$H$195,"Fail")</f>
         <v/>
       </c>
       <c r="E12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$194,$A12,'QA Checklist'!$H$5:$H$194,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$195,$A12,'QA Checklist'!$H$5:$H$195,"Pending")</f>
         <v/>
       </c>
       <c r="F12" s="8">
@@ -698,19 +698,19 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$194,$A13)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$195,$A13)</f>
         <v/>
       </c>
       <c r="C13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$194,$A13,'QA Checklist'!$H$5:$H$194,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$194,$A13,'QA Checklist'!$H$5:$H$194,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$195,$A13,'QA Checklist'!$H$5:$H$195,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$195,$A13,'QA Checklist'!$H$5:$H$195,"Pass")</f>
         <v/>
       </c>
       <c r="D13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$194,$A13,'QA Checklist'!$H$5:$H$194,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$194,$A13,'QA Checklist'!$H$5:$H$194,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$195,$A13,'QA Checklist'!$H$5:$H$195,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$195,$A13,'QA Checklist'!$H$5:$H$195,"Fail")</f>
         <v/>
       </c>
       <c r="E13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$194,$A13,'QA Checklist'!$H$5:$H$194,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$195,$A13,'QA Checklist'!$H$5:$H$195,"Pending")</f>
         <v/>
       </c>
       <c r="F13" s="8">
@@ -725,19 +725,19 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$194,$A14)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$195,$A14)</f>
         <v/>
       </c>
       <c r="C14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$194,$A14,'QA Checklist'!$H$5:$H$194,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$194,$A14,'QA Checklist'!$H$5:$H$194,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$195,$A14,'QA Checklist'!$H$5:$H$195,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$195,$A14,'QA Checklist'!$H$5:$H$195,"Pass")</f>
         <v/>
       </c>
       <c r="D14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$194,$A14,'QA Checklist'!$H$5:$H$194,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$194,$A14,'QA Checklist'!$H$5:$H$194,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$195,$A14,'QA Checklist'!$H$5:$H$195,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$195,$A14,'QA Checklist'!$H$5:$H$195,"Fail")</f>
         <v/>
       </c>
       <c r="E14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$194,$A14,'QA Checklist'!$H$5:$H$194,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$195,$A14,'QA Checklist'!$H$5:$H$195,"Pending")</f>
         <v/>
       </c>
       <c r="F14" s="8">
@@ -752,19 +752,19 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$194,$A15)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$195,$A15)</f>
         <v/>
       </c>
       <c r="C15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$194,$A15,'QA Checklist'!$H$5:$H$194,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$194,$A15,'QA Checklist'!$H$5:$H$194,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$195,$A15,'QA Checklist'!$H$5:$H$195,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$195,$A15,'QA Checklist'!$H$5:$H$195,"Pass")</f>
         <v/>
       </c>
       <c r="D15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$194,$A15,'QA Checklist'!$H$5:$H$194,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$194,$A15,'QA Checklist'!$H$5:$H$194,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$195,$A15,'QA Checklist'!$H$5:$H$195,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$195,$A15,'QA Checklist'!$H$5:$H$195,"Fail")</f>
         <v/>
       </c>
       <c r="E15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$194,$A15,'QA Checklist'!$H$5:$H$194,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$195,$A15,'QA Checklist'!$H$5:$H$195,"Pending")</f>
         <v/>
       </c>
       <c r="F15" s="8">
@@ -779,19 +779,19 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$194,$A16)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$195,$A16)</f>
         <v/>
       </c>
       <c r="C16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$194,$A16,'QA Checklist'!$H$5:$H$194,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$194,$A16,'QA Checklist'!$H$5:$H$194,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$195,$A16,'QA Checklist'!$H$5:$H$195,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$195,$A16,'QA Checklist'!$H$5:$H$195,"Pass")</f>
         <v/>
       </c>
       <c r="D16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$194,$A16,'QA Checklist'!$H$5:$H$194,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$194,$A16,'QA Checklist'!$H$5:$H$194,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$195,$A16,'QA Checklist'!$H$5:$H$195,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$195,$A16,'QA Checklist'!$H$5:$H$195,"Fail")</f>
         <v/>
       </c>
       <c r="E16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$194,$A16,'QA Checklist'!$H$5:$H$194,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$195,$A16,'QA Checklist'!$H$5:$H$195,"Pending")</f>
         <v/>
       </c>
       <c r="F16" s="8">
@@ -806,19 +806,19 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$194,$A17)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$195,$A17)</f>
         <v/>
       </c>
       <c r="C17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$194,$A17,'QA Checklist'!$H$5:$H$194,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$194,$A17,'QA Checklist'!$H$5:$H$194,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$195,$A17,'QA Checklist'!$H$5:$H$195,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$195,$A17,'QA Checklist'!$H$5:$H$195,"Pass")</f>
         <v/>
       </c>
       <c r="D17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$194,$A17,'QA Checklist'!$H$5:$H$194,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$194,$A17,'QA Checklist'!$H$5:$H$194,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$195,$A17,'QA Checklist'!$H$5:$H$195,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$195,$A17,'QA Checklist'!$H$5:$H$195,"Fail")</f>
         <v/>
       </c>
       <c r="E17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$194,$A17,'QA Checklist'!$H$5:$H$194,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$195,$A17,'QA Checklist'!$H$5:$H$195,"Pending")</f>
         <v/>
       </c>
       <c r="F17" s="8">
@@ -833,19 +833,19 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$194,$A18)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$195,$A18)</f>
         <v/>
       </c>
       <c r="C18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$194,$A18,'QA Checklist'!$H$5:$H$194,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$194,$A18,'QA Checklist'!$H$5:$H$194,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$195,$A18,'QA Checklist'!$H$5:$H$195,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$195,$A18,'QA Checklist'!$H$5:$H$195,"Pass")</f>
         <v/>
       </c>
       <c r="D18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$194,$A18,'QA Checklist'!$H$5:$H$194,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$194,$A18,'QA Checklist'!$H$5:$H$194,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$195,$A18,'QA Checklist'!$H$5:$H$195,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$195,$A18,'QA Checklist'!$H$5:$H$195,"Fail")</f>
         <v/>
       </c>
       <c r="E18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$194,$A18,'QA Checklist'!$H$5:$H$194,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$195,$A18,'QA Checklist'!$H$5:$H$195,"Pending")</f>
         <v/>
       </c>
       <c r="F18" s="8">
@@ -860,19 +860,19 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$194,$A19)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$195,$A19)</f>
         <v/>
       </c>
       <c r="C19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$194,$A19,'QA Checklist'!$H$5:$H$194,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$194,$A19,'QA Checklist'!$H$5:$H$194,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$195,$A19,'QA Checklist'!$H$5:$H$195,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$195,$A19,'QA Checklist'!$H$5:$H$195,"Pass")</f>
         <v/>
       </c>
       <c r="D19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$194,$A19,'QA Checklist'!$H$5:$H$194,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$194,$A19,'QA Checklist'!$H$5:$H$194,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$195,$A19,'QA Checklist'!$H$5:$H$195,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$195,$A19,'QA Checklist'!$H$5:$H$195,"Fail")</f>
         <v/>
       </c>
       <c r="E19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$194,$A19,'QA Checklist'!$H$5:$H$194,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$195,$A19,'QA Checklist'!$H$5:$H$195,"Pending")</f>
         <v/>
       </c>
       <c r="F19" s="8">
@@ -887,19 +887,19 @@
         </is>
       </c>
       <c r="B20" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$194,$A20)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$195,$A20)</f>
         <v/>
       </c>
       <c r="C20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$194,$A20,'QA Checklist'!$H$5:$H$194,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$194,$A20,'QA Checklist'!$H$5:$H$194,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$195,$A20,'QA Checklist'!$H$5:$H$195,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$195,$A20,'QA Checklist'!$H$5:$H$195,"Pass")</f>
         <v/>
       </c>
       <c r="D20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$194,$A20,'QA Checklist'!$H$5:$H$194,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$194,$A20,'QA Checklist'!$H$5:$H$194,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$195,$A20,'QA Checklist'!$H$5:$H$195,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$195,$A20,'QA Checklist'!$H$5:$H$195,"Fail")</f>
         <v/>
       </c>
       <c r="E20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$194,$A20,'QA Checklist'!$H$5:$H$194,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$195,$A20,'QA Checklist'!$H$5:$H$195,"Pending")</f>
         <v/>
       </c>
       <c r="F20" s="8">
@@ -914,19 +914,19 @@
         </is>
       </c>
       <c r="B21" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$194,$A21)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$195,$A21)</f>
         <v/>
       </c>
       <c r="C21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$194,$A21,'QA Checklist'!$H$5:$H$194,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$194,$A21,'QA Checklist'!$H$5:$H$194,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$195,$A21,'QA Checklist'!$H$5:$H$195,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$195,$A21,'QA Checklist'!$H$5:$H$195,"Pass")</f>
         <v/>
       </c>
       <c r="D21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$194,$A21,'QA Checklist'!$H$5:$H$194,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$194,$A21,'QA Checklist'!$H$5:$H$194,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$195,$A21,'QA Checklist'!$H$5:$H$195,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$195,$A21,'QA Checklist'!$H$5:$H$195,"Fail")</f>
         <v/>
       </c>
       <c r="E21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$194,$A21,'QA Checklist'!$H$5:$H$194,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$195,$A21,'QA Checklist'!$H$5:$H$195,"Pending")</f>
         <v/>
       </c>
       <c r="F21" s="8">
@@ -941,19 +941,19 @@
         </is>
       </c>
       <c r="B22" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$194,$A22)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$195,$A22)</f>
         <v/>
       </c>
       <c r="C22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$194,$A22,'QA Checklist'!$H$5:$H$194,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$194,$A22,'QA Checklist'!$H$5:$H$194,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$195,$A22,'QA Checklist'!$H$5:$H$195,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$195,$A22,'QA Checklist'!$H$5:$H$195,"Pass")</f>
         <v/>
       </c>
       <c r="D22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$194,$A22,'QA Checklist'!$H$5:$H$194,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$194,$A22,'QA Checklist'!$H$5:$H$194,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$195,$A22,'QA Checklist'!$H$5:$H$195,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$195,$A22,'QA Checklist'!$H$5:$H$195,"Fail")</f>
         <v/>
       </c>
       <c r="E22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$194,$A22,'QA Checklist'!$H$5:$H$194,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$195,$A22,'QA Checklist'!$H$5:$H$195,"Pending")</f>
         <v/>
       </c>
       <c r="F22" s="8">
@@ -1023,19 +1023,19 @@
         </is>
       </c>
       <c r="B26" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$194,$A26&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$195,$A26&amp;"*")</f>
         <v/>
       </c>
       <c r="C26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$194,$A26&amp;"*",'QA Checklist'!$H$5:$H$194,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$194,$A26&amp;"*",'QA Checklist'!$H$5:$H$194,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$195,$A26&amp;"*",'QA Checklist'!$H$5:$H$195,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$195,$A26&amp;"*",'QA Checklist'!$H$5:$H$195,"Pass")</f>
         <v/>
       </c>
       <c r="D26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$194,$A26&amp;"*",'QA Checklist'!$H$5:$H$194,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$194,$A26&amp;"*",'QA Checklist'!$H$5:$H$194,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$195,$A26&amp;"*",'QA Checklist'!$H$5:$H$195,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$195,$A26&amp;"*",'QA Checklist'!$H$5:$H$195,"Fail")</f>
         <v/>
       </c>
       <c r="E26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$194,$A26&amp;"*",'QA Checklist'!$H$5:$H$194,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$195,$A26&amp;"*",'QA Checklist'!$H$5:$H$195,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1046,19 +1046,19 @@
         </is>
       </c>
       <c r="B27" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$194,$A27&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$195,$A27&amp;"*")</f>
         <v/>
       </c>
       <c r="C27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$194,$A27&amp;"*",'QA Checklist'!$H$5:$H$194,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$194,$A27&amp;"*",'QA Checklist'!$H$5:$H$194,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$195,$A27&amp;"*",'QA Checklist'!$H$5:$H$195,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$195,$A27&amp;"*",'QA Checklist'!$H$5:$H$195,"Pass")</f>
         <v/>
       </c>
       <c r="D27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$194,$A27&amp;"*",'QA Checklist'!$H$5:$H$194,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$194,$A27&amp;"*",'QA Checklist'!$H$5:$H$194,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$195,$A27&amp;"*",'QA Checklist'!$H$5:$H$195,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$195,$A27&amp;"*",'QA Checklist'!$H$5:$H$195,"Fail")</f>
         <v/>
       </c>
       <c r="E27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$194,$A27&amp;"*",'QA Checklist'!$H$5:$H$194,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$195,$A27&amp;"*",'QA Checklist'!$H$5:$H$195,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1069,19 +1069,19 @@
         </is>
       </c>
       <c r="B28" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$194,$A28&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$195,$A28&amp;"*")</f>
         <v/>
       </c>
       <c r="C28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$194,$A28&amp;"*",'QA Checklist'!$H$5:$H$194,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$194,$A28&amp;"*",'QA Checklist'!$H$5:$H$194,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$195,$A28&amp;"*",'QA Checklist'!$H$5:$H$195,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$195,$A28&amp;"*",'QA Checklist'!$H$5:$H$195,"Pass")</f>
         <v/>
       </c>
       <c r="D28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$194,$A28&amp;"*",'QA Checklist'!$H$5:$H$194,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$194,$A28&amp;"*",'QA Checklist'!$H$5:$H$194,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$195,$A28&amp;"*",'QA Checklist'!$H$5:$H$195,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$195,$A28&amp;"*",'QA Checklist'!$H$5:$H$195,"Fail")</f>
         <v/>
       </c>
       <c r="E28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$194,$A28&amp;"*",'QA Checklist'!$H$5:$H$194,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$195,$A28&amp;"*",'QA Checklist'!$H$5:$H$195,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1096,7 +1096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I194"/>
+  <dimension ref="A1:I195"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9657,12 +9657,59 @@
         </is>
       </c>
     </row>
+    <row r="195">
+      <c r="A195" s="12" t="inlineStr">
+        <is>
+          <t>SA-69</t>
+        </is>
+      </c>
+      <c r="B195" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="C195" s="13" t="inlineStr">
+        <is>
+          <t>Tier 2 (Workflow &amp; Ergonomics)</t>
+        </is>
+      </c>
+      <c r="D195" s="13" t="inlineStr">
+        <is>
+          <t>Customer Lookup Sheet Tabs</t>
+        </is>
+      </c>
+      <c r="E195" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="F195" s="13" t="inlineStr">
+        <is>
+          <t>Open Customer Lookup as SA; click Regulars, Back_Jobs, Due_for_PMS and All_Customers; select a customer; switch between Customer_Details and Service_History; search and press Clear</t>
+        </is>
+      </c>
+      <c r="G195" s="13" t="inlineStr">
+        <is>
+          <t>Tabs look and behave like the RO Excel Studio tabs and filter the list; Customer_Details shows the RO details box, actions and metrics; Service_History shows the history logs with the count in the tab; Clear returns to All_Customers</t>
+        </is>
+      </c>
+      <c r="H195" s="14" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="I195" s="13" t="inlineStr">
+        <is>
+          <t>Verified by Automated Unit Tests (181 passing in tests/frontend/sla_and_logic.test.js AUT-FRONT-152) and headless Chrome 5/5</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:I194"/>
+  <autoFilter ref="A4:I195"/>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="H5:H194">
+  <conditionalFormatting sqref="H5:H195">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$H5="Passed"</formula>
     </cfRule>
@@ -9679,13 +9726,13 @@
       <formula>$H5="Pending"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A5:A194">
+  <conditionalFormatting sqref="A5:A195">
     <cfRule type="expression" priority="6" dxfId="3">
-      <formula>COUNTIF($A$5:$A$194,$A5)&gt;1</formula>
+      <formula>COUNTIF($A$5:$A$195,$A5)&gt;1</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H5:H194" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H5:H195" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pending,Passed,Failed"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat(REV-194): useful Service_History records in Customer Lookup
Real RO fields instead of placeholders (the old card read snake_case fields the API never returns), concern and findings, back-job link, 30-day back-job warranty status, Claim Stub and Issue Back-Job (released visits only). Last Service, Primary Advisor, Due for PMS and history order now use the real fields.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
+++ b/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
@@ -11,7 +11,7 @@
     <sheet name="QA Checklist" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$195</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$196</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'QA Checklist'!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTA('QA Checklist'!$A$5:$A$195)</f>
+        <f>COUNTA('QA Checklist'!$A$5:$A$196)</f>
         <v/>
       </c>
     </row>
@@ -594,7 +594,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$195,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$195,"Pass")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$196,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$196,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$195,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$195,"Fail")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$196,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$196,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -616,7 +616,7 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$195,"Pending")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$196,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -671,19 +671,19 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$195,$A12)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$196,$A12)</f>
         <v/>
       </c>
       <c r="C12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$195,$A12,'QA Checklist'!$H$5:$H$195,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$195,$A12,'QA Checklist'!$H$5:$H$195,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$196,$A12,'QA Checklist'!$H$5:$H$196,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$196,$A12,'QA Checklist'!$H$5:$H$196,"Pass")</f>
         <v/>
       </c>
       <c r="D12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$195,$A12,'QA Checklist'!$H$5:$H$195,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$195,$A12,'QA Checklist'!$H$5:$H$195,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$196,$A12,'QA Checklist'!$H$5:$H$196,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$196,$A12,'QA Checklist'!$H$5:$H$196,"Fail")</f>
         <v/>
       </c>
       <c r="E12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$195,$A12,'QA Checklist'!$H$5:$H$195,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$196,$A12,'QA Checklist'!$H$5:$H$196,"Pending")</f>
         <v/>
       </c>
       <c r="F12" s="8">
@@ -698,19 +698,19 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$195,$A13)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$196,$A13)</f>
         <v/>
       </c>
       <c r="C13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$195,$A13,'QA Checklist'!$H$5:$H$195,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$195,$A13,'QA Checklist'!$H$5:$H$195,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$196,$A13,'QA Checklist'!$H$5:$H$196,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$196,$A13,'QA Checklist'!$H$5:$H$196,"Pass")</f>
         <v/>
       </c>
       <c r="D13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$195,$A13,'QA Checklist'!$H$5:$H$195,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$195,$A13,'QA Checklist'!$H$5:$H$195,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$196,$A13,'QA Checklist'!$H$5:$H$196,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$196,$A13,'QA Checklist'!$H$5:$H$196,"Fail")</f>
         <v/>
       </c>
       <c r="E13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$195,$A13,'QA Checklist'!$H$5:$H$195,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$196,$A13,'QA Checklist'!$H$5:$H$196,"Pending")</f>
         <v/>
       </c>
       <c r="F13" s="8">
@@ -725,19 +725,19 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$195,$A14)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$196,$A14)</f>
         <v/>
       </c>
       <c r="C14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$195,$A14,'QA Checklist'!$H$5:$H$195,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$195,$A14,'QA Checklist'!$H$5:$H$195,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$196,$A14,'QA Checklist'!$H$5:$H$196,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$196,$A14,'QA Checklist'!$H$5:$H$196,"Pass")</f>
         <v/>
       </c>
       <c r="D14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$195,$A14,'QA Checklist'!$H$5:$H$195,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$195,$A14,'QA Checklist'!$H$5:$H$195,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$196,$A14,'QA Checklist'!$H$5:$H$196,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$196,$A14,'QA Checklist'!$H$5:$H$196,"Fail")</f>
         <v/>
       </c>
       <c r="E14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$195,$A14,'QA Checklist'!$H$5:$H$195,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$196,$A14,'QA Checklist'!$H$5:$H$196,"Pending")</f>
         <v/>
       </c>
       <c r="F14" s="8">
@@ -752,19 +752,19 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$195,$A15)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$196,$A15)</f>
         <v/>
       </c>
       <c r="C15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$195,$A15,'QA Checklist'!$H$5:$H$195,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$195,$A15,'QA Checklist'!$H$5:$H$195,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$196,$A15,'QA Checklist'!$H$5:$H$196,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$196,$A15,'QA Checklist'!$H$5:$H$196,"Pass")</f>
         <v/>
       </c>
       <c r="D15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$195,$A15,'QA Checklist'!$H$5:$H$195,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$195,$A15,'QA Checklist'!$H$5:$H$195,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$196,$A15,'QA Checklist'!$H$5:$H$196,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$196,$A15,'QA Checklist'!$H$5:$H$196,"Fail")</f>
         <v/>
       </c>
       <c r="E15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$195,$A15,'QA Checklist'!$H$5:$H$195,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$196,$A15,'QA Checklist'!$H$5:$H$196,"Pending")</f>
         <v/>
       </c>
       <c r="F15" s="8">
@@ -779,19 +779,19 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$195,$A16)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$196,$A16)</f>
         <v/>
       </c>
       <c r="C16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$195,$A16,'QA Checklist'!$H$5:$H$195,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$195,$A16,'QA Checklist'!$H$5:$H$195,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$196,$A16,'QA Checklist'!$H$5:$H$196,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$196,$A16,'QA Checklist'!$H$5:$H$196,"Pass")</f>
         <v/>
       </c>
       <c r="D16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$195,$A16,'QA Checklist'!$H$5:$H$195,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$195,$A16,'QA Checklist'!$H$5:$H$195,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$196,$A16,'QA Checklist'!$H$5:$H$196,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$196,$A16,'QA Checklist'!$H$5:$H$196,"Fail")</f>
         <v/>
       </c>
       <c r="E16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$195,$A16,'QA Checklist'!$H$5:$H$195,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$196,$A16,'QA Checklist'!$H$5:$H$196,"Pending")</f>
         <v/>
       </c>
       <c r="F16" s="8">
@@ -806,19 +806,19 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$195,$A17)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$196,$A17)</f>
         <v/>
       </c>
       <c r="C17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$195,$A17,'QA Checklist'!$H$5:$H$195,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$195,$A17,'QA Checklist'!$H$5:$H$195,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$196,$A17,'QA Checklist'!$H$5:$H$196,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$196,$A17,'QA Checklist'!$H$5:$H$196,"Pass")</f>
         <v/>
       </c>
       <c r="D17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$195,$A17,'QA Checklist'!$H$5:$H$195,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$195,$A17,'QA Checklist'!$H$5:$H$195,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$196,$A17,'QA Checklist'!$H$5:$H$196,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$196,$A17,'QA Checklist'!$H$5:$H$196,"Fail")</f>
         <v/>
       </c>
       <c r="E17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$195,$A17,'QA Checklist'!$H$5:$H$195,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$196,$A17,'QA Checklist'!$H$5:$H$196,"Pending")</f>
         <v/>
       </c>
       <c r="F17" s="8">
@@ -833,19 +833,19 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$195,$A18)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$196,$A18)</f>
         <v/>
       </c>
       <c r="C18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$195,$A18,'QA Checklist'!$H$5:$H$195,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$195,$A18,'QA Checklist'!$H$5:$H$195,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$196,$A18,'QA Checklist'!$H$5:$H$196,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$196,$A18,'QA Checklist'!$H$5:$H$196,"Pass")</f>
         <v/>
       </c>
       <c r="D18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$195,$A18,'QA Checklist'!$H$5:$H$195,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$195,$A18,'QA Checklist'!$H$5:$H$195,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$196,$A18,'QA Checklist'!$H$5:$H$196,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$196,$A18,'QA Checklist'!$H$5:$H$196,"Fail")</f>
         <v/>
       </c>
       <c r="E18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$195,$A18,'QA Checklist'!$H$5:$H$195,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$196,$A18,'QA Checklist'!$H$5:$H$196,"Pending")</f>
         <v/>
       </c>
       <c r="F18" s="8">
@@ -860,19 +860,19 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$195,$A19)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$196,$A19)</f>
         <v/>
       </c>
       <c r="C19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$195,$A19,'QA Checklist'!$H$5:$H$195,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$195,$A19,'QA Checklist'!$H$5:$H$195,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$196,$A19,'QA Checklist'!$H$5:$H$196,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$196,$A19,'QA Checklist'!$H$5:$H$196,"Pass")</f>
         <v/>
       </c>
       <c r="D19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$195,$A19,'QA Checklist'!$H$5:$H$195,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$195,$A19,'QA Checklist'!$H$5:$H$195,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$196,$A19,'QA Checklist'!$H$5:$H$196,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$196,$A19,'QA Checklist'!$H$5:$H$196,"Fail")</f>
         <v/>
       </c>
       <c r="E19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$195,$A19,'QA Checklist'!$H$5:$H$195,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$196,$A19,'QA Checklist'!$H$5:$H$196,"Pending")</f>
         <v/>
       </c>
       <c r="F19" s="8">
@@ -887,19 +887,19 @@
         </is>
       </c>
       <c r="B20" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$195,$A20)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$196,$A20)</f>
         <v/>
       </c>
       <c r="C20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$195,$A20,'QA Checklist'!$H$5:$H$195,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$195,$A20,'QA Checklist'!$H$5:$H$195,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$196,$A20,'QA Checklist'!$H$5:$H$196,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$196,$A20,'QA Checklist'!$H$5:$H$196,"Pass")</f>
         <v/>
       </c>
       <c r="D20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$195,$A20,'QA Checklist'!$H$5:$H$195,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$195,$A20,'QA Checklist'!$H$5:$H$195,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$196,$A20,'QA Checklist'!$H$5:$H$196,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$196,$A20,'QA Checklist'!$H$5:$H$196,"Fail")</f>
         <v/>
       </c>
       <c r="E20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$195,$A20,'QA Checklist'!$H$5:$H$195,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$196,$A20,'QA Checklist'!$H$5:$H$196,"Pending")</f>
         <v/>
       </c>
       <c r="F20" s="8">
@@ -914,19 +914,19 @@
         </is>
       </c>
       <c r="B21" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$195,$A21)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$196,$A21)</f>
         <v/>
       </c>
       <c r="C21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$195,$A21,'QA Checklist'!$H$5:$H$195,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$195,$A21,'QA Checklist'!$H$5:$H$195,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$196,$A21,'QA Checklist'!$H$5:$H$196,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$196,$A21,'QA Checklist'!$H$5:$H$196,"Pass")</f>
         <v/>
       </c>
       <c r="D21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$195,$A21,'QA Checklist'!$H$5:$H$195,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$195,$A21,'QA Checklist'!$H$5:$H$195,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$196,$A21,'QA Checklist'!$H$5:$H$196,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$196,$A21,'QA Checklist'!$H$5:$H$196,"Fail")</f>
         <v/>
       </c>
       <c r="E21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$195,$A21,'QA Checklist'!$H$5:$H$195,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$196,$A21,'QA Checklist'!$H$5:$H$196,"Pending")</f>
         <v/>
       </c>
       <c r="F21" s="8">
@@ -941,19 +941,19 @@
         </is>
       </c>
       <c r="B22" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$195,$A22)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$196,$A22)</f>
         <v/>
       </c>
       <c r="C22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$195,$A22,'QA Checklist'!$H$5:$H$195,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$195,$A22,'QA Checklist'!$H$5:$H$195,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$196,$A22,'QA Checklist'!$H$5:$H$196,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$196,$A22,'QA Checklist'!$H$5:$H$196,"Pass")</f>
         <v/>
       </c>
       <c r="D22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$195,$A22,'QA Checklist'!$H$5:$H$195,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$195,$A22,'QA Checklist'!$H$5:$H$195,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$196,$A22,'QA Checklist'!$H$5:$H$196,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$196,$A22,'QA Checklist'!$H$5:$H$196,"Fail")</f>
         <v/>
       </c>
       <c r="E22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$195,$A22,'QA Checklist'!$H$5:$H$195,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$196,$A22,'QA Checklist'!$H$5:$H$196,"Pending")</f>
         <v/>
       </c>
       <c r="F22" s="8">
@@ -1023,19 +1023,19 @@
         </is>
       </c>
       <c r="B26" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$195,$A26&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$196,$A26&amp;"*")</f>
         <v/>
       </c>
       <c r="C26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$195,$A26&amp;"*",'QA Checklist'!$H$5:$H$195,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$195,$A26&amp;"*",'QA Checklist'!$H$5:$H$195,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$196,$A26&amp;"*",'QA Checklist'!$H$5:$H$196,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$196,$A26&amp;"*",'QA Checklist'!$H$5:$H$196,"Pass")</f>
         <v/>
       </c>
       <c r="D26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$195,$A26&amp;"*",'QA Checklist'!$H$5:$H$195,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$195,$A26&amp;"*",'QA Checklist'!$H$5:$H$195,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$196,$A26&amp;"*",'QA Checklist'!$H$5:$H$196,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$196,$A26&amp;"*",'QA Checklist'!$H$5:$H$196,"Fail")</f>
         <v/>
       </c>
       <c r="E26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$195,$A26&amp;"*",'QA Checklist'!$H$5:$H$195,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$196,$A26&amp;"*",'QA Checklist'!$H$5:$H$196,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1046,19 +1046,19 @@
         </is>
       </c>
       <c r="B27" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$195,$A27&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$196,$A27&amp;"*")</f>
         <v/>
       </c>
       <c r="C27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$195,$A27&amp;"*",'QA Checklist'!$H$5:$H$195,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$195,$A27&amp;"*",'QA Checklist'!$H$5:$H$195,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$196,$A27&amp;"*",'QA Checklist'!$H$5:$H$196,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$196,$A27&amp;"*",'QA Checklist'!$H$5:$H$196,"Pass")</f>
         <v/>
       </c>
       <c r="D27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$195,$A27&amp;"*",'QA Checklist'!$H$5:$H$195,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$195,$A27&amp;"*",'QA Checklist'!$H$5:$H$195,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$196,$A27&amp;"*",'QA Checklist'!$H$5:$H$196,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$196,$A27&amp;"*",'QA Checklist'!$H$5:$H$196,"Fail")</f>
         <v/>
       </c>
       <c r="E27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$195,$A27&amp;"*",'QA Checklist'!$H$5:$H$195,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$196,$A27&amp;"*",'QA Checklist'!$H$5:$H$196,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1069,19 +1069,19 @@
         </is>
       </c>
       <c r="B28" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$195,$A28&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$196,$A28&amp;"*")</f>
         <v/>
       </c>
       <c r="C28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$195,$A28&amp;"*",'QA Checklist'!$H$5:$H$195,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$195,$A28&amp;"*",'QA Checklist'!$H$5:$H$195,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$196,$A28&amp;"*",'QA Checklist'!$H$5:$H$196,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$196,$A28&amp;"*",'QA Checklist'!$H$5:$H$196,"Pass")</f>
         <v/>
       </c>
       <c r="D28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$195,$A28&amp;"*",'QA Checklist'!$H$5:$H$195,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$195,$A28&amp;"*",'QA Checklist'!$H$5:$H$195,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$196,$A28&amp;"*",'QA Checklist'!$H$5:$H$196,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$196,$A28&amp;"*",'QA Checklist'!$H$5:$H$196,"Fail")</f>
         <v/>
       </c>
       <c r="E28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$195,$A28&amp;"*",'QA Checklist'!$H$5:$H$195,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$196,$A28&amp;"*",'QA Checklist'!$H$5:$H$196,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1096,7 +1096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I195"/>
+  <dimension ref="A1:I196"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9704,12 +9704,59 @@
         </is>
       </c>
     </row>
+    <row r="196">
+      <c r="A196" s="12" t="inlineStr">
+        <is>
+          <t>SA-70</t>
+        </is>
+      </c>
+      <c r="B196" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="C196" s="13" t="inlineStr">
+        <is>
+          <t>Tier 2 (Workflow &amp; Ergonomics)</t>
+        </is>
+      </c>
+      <c r="D196" s="13" t="inlineStr">
+        <is>
+          <t>Customer Lookup Service_History Records</t>
+        </is>
+      </c>
+      <c r="E196" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="F196" s="13" t="inlineStr">
+        <is>
+          <t>Open Customer Lookup as SA, select a customer and open Service_History; check a job still in the shop and a released job; for a released job press Issue Back-Job and Claim Stub</t>
+        </is>
+      </c>
+      <c r="G196" s="13" t="inlineStr">
+        <is>
+          <t>Each visit shows the real date, time, job order no., claim stub, advisor, bay, source, parts, promise date, concern and findings (blank fields show —); released visits show the 30-day back-job warranty status and Issue Back-Job; in-shop visits say the warranty starts on release</t>
+        </is>
+      </c>
+      <c r="H196" s="14" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="I196" s="13" t="inlineStr">
+        <is>
+          <t>Verified by Automated Unit Tests (182 passing in tests/frontend/sla_and_logic.test.js AUT-FRONT-153) and headless Chrome 10/10</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:I195"/>
+  <autoFilter ref="A4:I196"/>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="H5:H195">
+  <conditionalFormatting sqref="H5:H196">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$H5="Passed"</formula>
     </cfRule>
@@ -9726,13 +9773,13 @@
       <formula>$H5="Pending"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A5:A195">
+  <conditionalFormatting sqref="A5:A196">
     <cfRule type="expression" priority="6" dxfId="3">
-      <formula>COUNTIF($A$5:$A$195,$A5)&gt;1</formula>
+      <formula>COUNTIF($A$5:$A$196,$A5)&gt;1</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H5:H195" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H5:H196" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pending,Passed,Failed"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat(REV-195): responsive, scrollable TV slides 1-3
Slides fill the space in normal flow; responsive grids (bays 1/2/3 columns, queue panels stack, lanes 1/2/4); every list and slide area scrolls; bay text no longer overlaps; header wraps; page never scrolls sideways; auto-rotation holds 20 seconds after a scroll or touch.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
+++ b/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
@@ -11,7 +11,7 @@
     <sheet name="QA Checklist" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$196</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$197</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'QA Checklist'!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTA('QA Checklist'!$A$5:$A$196)</f>
+        <f>COUNTA('QA Checklist'!$A$5:$A$197)</f>
         <v/>
       </c>
     </row>
@@ -594,7 +594,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$196,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$196,"Pass")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$197,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$197,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$196,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$196,"Fail")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$197,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$197,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -616,7 +616,7 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$196,"Pending")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$197,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -671,19 +671,19 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$196,$A12)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$197,$A12)</f>
         <v/>
       </c>
       <c r="C12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$196,$A12,'QA Checklist'!$H$5:$H$196,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$196,$A12,'QA Checklist'!$H$5:$H$196,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$197,$A12,'QA Checklist'!$H$5:$H$197,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$197,$A12,'QA Checklist'!$H$5:$H$197,"Pass")</f>
         <v/>
       </c>
       <c r="D12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$196,$A12,'QA Checklist'!$H$5:$H$196,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$196,$A12,'QA Checklist'!$H$5:$H$196,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$197,$A12,'QA Checklist'!$H$5:$H$197,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$197,$A12,'QA Checklist'!$H$5:$H$197,"Fail")</f>
         <v/>
       </c>
       <c r="E12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$196,$A12,'QA Checklist'!$H$5:$H$196,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$197,$A12,'QA Checklist'!$H$5:$H$197,"Pending")</f>
         <v/>
       </c>
       <c r="F12" s="8">
@@ -698,19 +698,19 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$196,$A13)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$197,$A13)</f>
         <v/>
       </c>
       <c r="C13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$196,$A13,'QA Checklist'!$H$5:$H$196,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$196,$A13,'QA Checklist'!$H$5:$H$196,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$197,$A13,'QA Checklist'!$H$5:$H$197,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$197,$A13,'QA Checklist'!$H$5:$H$197,"Pass")</f>
         <v/>
       </c>
       <c r="D13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$196,$A13,'QA Checklist'!$H$5:$H$196,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$196,$A13,'QA Checklist'!$H$5:$H$196,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$197,$A13,'QA Checklist'!$H$5:$H$197,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$197,$A13,'QA Checklist'!$H$5:$H$197,"Fail")</f>
         <v/>
       </c>
       <c r="E13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$196,$A13,'QA Checklist'!$H$5:$H$196,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$197,$A13,'QA Checklist'!$H$5:$H$197,"Pending")</f>
         <v/>
       </c>
       <c r="F13" s="8">
@@ -725,19 +725,19 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$196,$A14)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$197,$A14)</f>
         <v/>
       </c>
       <c r="C14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$196,$A14,'QA Checklist'!$H$5:$H$196,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$196,$A14,'QA Checklist'!$H$5:$H$196,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$197,$A14,'QA Checklist'!$H$5:$H$197,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$197,$A14,'QA Checklist'!$H$5:$H$197,"Pass")</f>
         <v/>
       </c>
       <c r="D14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$196,$A14,'QA Checklist'!$H$5:$H$196,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$196,$A14,'QA Checklist'!$H$5:$H$196,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$197,$A14,'QA Checklist'!$H$5:$H$197,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$197,$A14,'QA Checklist'!$H$5:$H$197,"Fail")</f>
         <v/>
       </c>
       <c r="E14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$196,$A14,'QA Checklist'!$H$5:$H$196,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$197,$A14,'QA Checklist'!$H$5:$H$197,"Pending")</f>
         <v/>
       </c>
       <c r="F14" s="8">
@@ -752,19 +752,19 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$196,$A15)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$197,$A15)</f>
         <v/>
       </c>
       <c r="C15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$196,$A15,'QA Checklist'!$H$5:$H$196,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$196,$A15,'QA Checklist'!$H$5:$H$196,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$197,$A15,'QA Checklist'!$H$5:$H$197,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$197,$A15,'QA Checklist'!$H$5:$H$197,"Pass")</f>
         <v/>
       </c>
       <c r="D15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$196,$A15,'QA Checklist'!$H$5:$H$196,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$196,$A15,'QA Checklist'!$H$5:$H$196,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$197,$A15,'QA Checklist'!$H$5:$H$197,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$197,$A15,'QA Checklist'!$H$5:$H$197,"Fail")</f>
         <v/>
       </c>
       <c r="E15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$196,$A15,'QA Checklist'!$H$5:$H$196,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$197,$A15,'QA Checklist'!$H$5:$H$197,"Pending")</f>
         <v/>
       </c>
       <c r="F15" s="8">
@@ -779,19 +779,19 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$196,$A16)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$197,$A16)</f>
         <v/>
       </c>
       <c r="C16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$196,$A16,'QA Checklist'!$H$5:$H$196,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$196,$A16,'QA Checklist'!$H$5:$H$196,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$197,$A16,'QA Checklist'!$H$5:$H$197,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$197,$A16,'QA Checklist'!$H$5:$H$197,"Pass")</f>
         <v/>
       </c>
       <c r="D16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$196,$A16,'QA Checklist'!$H$5:$H$196,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$196,$A16,'QA Checklist'!$H$5:$H$196,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$197,$A16,'QA Checklist'!$H$5:$H$197,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$197,$A16,'QA Checklist'!$H$5:$H$197,"Fail")</f>
         <v/>
       </c>
       <c r="E16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$196,$A16,'QA Checklist'!$H$5:$H$196,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$197,$A16,'QA Checklist'!$H$5:$H$197,"Pending")</f>
         <v/>
       </c>
       <c r="F16" s="8">
@@ -806,19 +806,19 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$196,$A17)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$197,$A17)</f>
         <v/>
       </c>
       <c r="C17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$196,$A17,'QA Checklist'!$H$5:$H$196,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$196,$A17,'QA Checklist'!$H$5:$H$196,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$197,$A17,'QA Checklist'!$H$5:$H$197,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$197,$A17,'QA Checklist'!$H$5:$H$197,"Pass")</f>
         <v/>
       </c>
       <c r="D17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$196,$A17,'QA Checklist'!$H$5:$H$196,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$196,$A17,'QA Checklist'!$H$5:$H$196,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$197,$A17,'QA Checklist'!$H$5:$H$197,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$197,$A17,'QA Checklist'!$H$5:$H$197,"Fail")</f>
         <v/>
       </c>
       <c r="E17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$196,$A17,'QA Checklist'!$H$5:$H$196,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$197,$A17,'QA Checklist'!$H$5:$H$197,"Pending")</f>
         <v/>
       </c>
       <c r="F17" s="8">
@@ -833,19 +833,19 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$196,$A18)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$197,$A18)</f>
         <v/>
       </c>
       <c r="C18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$196,$A18,'QA Checklist'!$H$5:$H$196,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$196,$A18,'QA Checklist'!$H$5:$H$196,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$197,$A18,'QA Checklist'!$H$5:$H$197,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$197,$A18,'QA Checklist'!$H$5:$H$197,"Pass")</f>
         <v/>
       </c>
       <c r="D18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$196,$A18,'QA Checklist'!$H$5:$H$196,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$196,$A18,'QA Checklist'!$H$5:$H$196,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$197,$A18,'QA Checklist'!$H$5:$H$197,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$197,$A18,'QA Checklist'!$H$5:$H$197,"Fail")</f>
         <v/>
       </c>
       <c r="E18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$196,$A18,'QA Checklist'!$H$5:$H$196,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$197,$A18,'QA Checklist'!$H$5:$H$197,"Pending")</f>
         <v/>
       </c>
       <c r="F18" s="8">
@@ -860,19 +860,19 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$196,$A19)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$197,$A19)</f>
         <v/>
       </c>
       <c r="C19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$196,$A19,'QA Checklist'!$H$5:$H$196,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$196,$A19,'QA Checklist'!$H$5:$H$196,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$197,$A19,'QA Checklist'!$H$5:$H$197,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$197,$A19,'QA Checklist'!$H$5:$H$197,"Pass")</f>
         <v/>
       </c>
       <c r="D19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$196,$A19,'QA Checklist'!$H$5:$H$196,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$196,$A19,'QA Checklist'!$H$5:$H$196,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$197,$A19,'QA Checklist'!$H$5:$H$197,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$197,$A19,'QA Checklist'!$H$5:$H$197,"Fail")</f>
         <v/>
       </c>
       <c r="E19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$196,$A19,'QA Checklist'!$H$5:$H$196,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$197,$A19,'QA Checklist'!$H$5:$H$197,"Pending")</f>
         <v/>
       </c>
       <c r="F19" s="8">
@@ -887,19 +887,19 @@
         </is>
       </c>
       <c r="B20" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$196,$A20)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$197,$A20)</f>
         <v/>
       </c>
       <c r="C20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$196,$A20,'QA Checklist'!$H$5:$H$196,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$196,$A20,'QA Checklist'!$H$5:$H$196,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$197,$A20,'QA Checklist'!$H$5:$H$197,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$197,$A20,'QA Checklist'!$H$5:$H$197,"Pass")</f>
         <v/>
       </c>
       <c r="D20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$196,$A20,'QA Checklist'!$H$5:$H$196,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$196,$A20,'QA Checklist'!$H$5:$H$196,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$197,$A20,'QA Checklist'!$H$5:$H$197,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$197,$A20,'QA Checklist'!$H$5:$H$197,"Fail")</f>
         <v/>
       </c>
       <c r="E20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$196,$A20,'QA Checklist'!$H$5:$H$196,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$197,$A20,'QA Checklist'!$H$5:$H$197,"Pending")</f>
         <v/>
       </c>
       <c r="F20" s="8">
@@ -914,19 +914,19 @@
         </is>
       </c>
       <c r="B21" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$196,$A21)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$197,$A21)</f>
         <v/>
       </c>
       <c r="C21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$196,$A21,'QA Checklist'!$H$5:$H$196,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$196,$A21,'QA Checklist'!$H$5:$H$196,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$197,$A21,'QA Checklist'!$H$5:$H$197,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$197,$A21,'QA Checklist'!$H$5:$H$197,"Pass")</f>
         <v/>
       </c>
       <c r="D21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$196,$A21,'QA Checklist'!$H$5:$H$196,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$196,$A21,'QA Checklist'!$H$5:$H$196,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$197,$A21,'QA Checklist'!$H$5:$H$197,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$197,$A21,'QA Checklist'!$H$5:$H$197,"Fail")</f>
         <v/>
       </c>
       <c r="E21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$196,$A21,'QA Checklist'!$H$5:$H$196,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$197,$A21,'QA Checklist'!$H$5:$H$197,"Pending")</f>
         <v/>
       </c>
       <c r="F21" s="8">
@@ -941,19 +941,19 @@
         </is>
       </c>
       <c r="B22" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$196,$A22)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$197,$A22)</f>
         <v/>
       </c>
       <c r="C22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$196,$A22,'QA Checklist'!$H$5:$H$196,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$196,$A22,'QA Checklist'!$H$5:$H$196,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$197,$A22,'QA Checklist'!$H$5:$H$197,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$197,$A22,'QA Checklist'!$H$5:$H$197,"Pass")</f>
         <v/>
       </c>
       <c r="D22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$196,$A22,'QA Checklist'!$H$5:$H$196,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$196,$A22,'QA Checklist'!$H$5:$H$196,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$197,$A22,'QA Checklist'!$H$5:$H$197,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$197,$A22,'QA Checklist'!$H$5:$H$197,"Fail")</f>
         <v/>
       </c>
       <c r="E22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$196,$A22,'QA Checklist'!$H$5:$H$196,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$197,$A22,'QA Checklist'!$H$5:$H$197,"Pending")</f>
         <v/>
       </c>
       <c r="F22" s="8">
@@ -1023,19 +1023,19 @@
         </is>
       </c>
       <c r="B26" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$196,$A26&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$197,$A26&amp;"*")</f>
         <v/>
       </c>
       <c r="C26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$196,$A26&amp;"*",'QA Checklist'!$H$5:$H$196,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$196,$A26&amp;"*",'QA Checklist'!$H$5:$H$196,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$197,$A26&amp;"*",'QA Checklist'!$H$5:$H$197,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$197,$A26&amp;"*",'QA Checklist'!$H$5:$H$197,"Pass")</f>
         <v/>
       </c>
       <c r="D26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$196,$A26&amp;"*",'QA Checklist'!$H$5:$H$196,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$196,$A26&amp;"*",'QA Checklist'!$H$5:$H$196,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$197,$A26&amp;"*",'QA Checklist'!$H$5:$H$197,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$197,$A26&amp;"*",'QA Checklist'!$H$5:$H$197,"Fail")</f>
         <v/>
       </c>
       <c r="E26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$196,$A26&amp;"*",'QA Checklist'!$H$5:$H$196,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$197,$A26&amp;"*",'QA Checklist'!$H$5:$H$197,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1046,19 +1046,19 @@
         </is>
       </c>
       <c r="B27" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$196,$A27&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$197,$A27&amp;"*")</f>
         <v/>
       </c>
       <c r="C27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$196,$A27&amp;"*",'QA Checklist'!$H$5:$H$196,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$196,$A27&amp;"*",'QA Checklist'!$H$5:$H$196,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$197,$A27&amp;"*",'QA Checklist'!$H$5:$H$197,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$197,$A27&amp;"*",'QA Checklist'!$H$5:$H$197,"Pass")</f>
         <v/>
       </c>
       <c r="D27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$196,$A27&amp;"*",'QA Checklist'!$H$5:$H$196,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$196,$A27&amp;"*",'QA Checklist'!$H$5:$H$196,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$197,$A27&amp;"*",'QA Checklist'!$H$5:$H$197,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$197,$A27&amp;"*",'QA Checklist'!$H$5:$H$197,"Fail")</f>
         <v/>
       </c>
       <c r="E27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$196,$A27&amp;"*",'QA Checklist'!$H$5:$H$196,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$197,$A27&amp;"*",'QA Checklist'!$H$5:$H$197,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1069,19 +1069,19 @@
         </is>
       </c>
       <c r="B28" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$196,$A28&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$197,$A28&amp;"*")</f>
         <v/>
       </c>
       <c r="C28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$196,$A28&amp;"*",'QA Checklist'!$H$5:$H$196,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$196,$A28&amp;"*",'QA Checklist'!$H$5:$H$196,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$197,$A28&amp;"*",'QA Checklist'!$H$5:$H$197,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$197,$A28&amp;"*",'QA Checklist'!$H$5:$H$197,"Pass")</f>
         <v/>
       </c>
       <c r="D28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$196,$A28&amp;"*",'QA Checklist'!$H$5:$H$196,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$196,$A28&amp;"*",'QA Checklist'!$H$5:$H$196,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$197,$A28&amp;"*",'QA Checklist'!$H$5:$H$197,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$197,$A28&amp;"*",'QA Checklist'!$H$5:$H$197,"Fail")</f>
         <v/>
       </c>
       <c r="E28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$196,$A28&amp;"*",'QA Checklist'!$H$5:$H$196,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$197,$A28&amp;"*",'QA Checklist'!$H$5:$H$197,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1096,7 +1096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I196"/>
+  <dimension ref="A1:I197"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9751,12 +9751,59 @@
         </is>
       </c>
     </row>
+    <row r="197">
+      <c r="A197" s="12" t="inlineStr">
+        <is>
+          <t>SA-71</t>
+        </is>
+      </c>
+      <c r="B197" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="C197" s="13" t="inlineStr">
+        <is>
+          <t>Tier 2 (Workflow &amp; Ergonomics)</t>
+        </is>
+      </c>
+      <c r="D197" s="13" t="inlineStr">
+        <is>
+          <t>TV Slides Responsive &amp; Scrollable</t>
+        </is>
+      </c>
+      <c r="E197" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="F197" s="13" t="inlineStr">
+        <is>
+          <t>Open the TV on a large TV, a laptop, a tablet and a phone; go through slides 1-3; with many vehicles scroll the bay grid, the queue/ready/carry-over lists and each lane; watch that the slide does not change while scrolling</t>
+        </is>
+      </c>
+      <c r="G197" s="13" t="inlineStr">
+        <is>
+          <t>Layouts adapt to the screen with no overlapping text or sideways scrolling; every area scrolls when full; auto-rotation waits 20 seconds after the last scroll or touch</t>
+        </is>
+      </c>
+      <c r="H197" s="14" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="I197" s="13" t="inlineStr">
+        <is>
+          <t>Verified by Automated Unit Tests (183 passing in tests/frontend/sla_and_logic.test.js AUT-FRONT-154) and headless Chrome 22/22 at 1920x1080, 1366x768, 1024x768 and 390x844</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:I196"/>
+  <autoFilter ref="A4:I197"/>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="H5:H196">
+  <conditionalFormatting sqref="H5:H197">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$H5="Passed"</formula>
     </cfRule>
@@ -9773,13 +9820,13 @@
       <formula>$H5="Pending"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A5:A196">
+  <conditionalFormatting sqref="A5:A197">
     <cfRule type="expression" priority="6" dxfId="3">
-      <formula>COUNTIF($A$5:$A$196,$A5)&gt;1</formula>
+      <formula>COUNTIF($A$5:$A$197,$A5)&gt;1</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H5:H196" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H5:H197" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pending,Passed,Failed"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat(REV-196): TV auto-scroll and daily reset like Daily Intakes
Long TV lists scroll to the bottom and back by themselves (pause 3 s, 40 px/s); slides wait for them and interaction pauses them. The TV feed now shows today's intakes (Asia/Manila) plus carry-over vehicles only, so it resets each day like Daily Intakes while carry-overs stay.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
+++ b/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
@@ -11,7 +11,7 @@
     <sheet name="QA Checklist" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$197</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$198</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'QA Checklist'!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTA('QA Checklist'!$A$5:$A$197)</f>
+        <f>COUNTA('QA Checklist'!$A$5:$A$198)</f>
         <v/>
       </c>
     </row>
@@ -594,7 +594,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$197,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$197,"Pass")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$198,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$198,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$197,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$197,"Fail")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$198,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$198,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -616,7 +616,7 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$197,"Pending")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$198,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -671,19 +671,19 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$197,$A12)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$198,$A12)</f>
         <v/>
       </c>
       <c r="C12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$197,$A12,'QA Checklist'!$H$5:$H$197,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$197,$A12,'QA Checklist'!$H$5:$H$197,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$198,$A12,'QA Checklist'!$H$5:$H$198,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$198,$A12,'QA Checklist'!$H$5:$H$198,"Pass")</f>
         <v/>
       </c>
       <c r="D12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$197,$A12,'QA Checklist'!$H$5:$H$197,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$197,$A12,'QA Checklist'!$H$5:$H$197,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$198,$A12,'QA Checklist'!$H$5:$H$198,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$198,$A12,'QA Checklist'!$H$5:$H$198,"Fail")</f>
         <v/>
       </c>
       <c r="E12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$197,$A12,'QA Checklist'!$H$5:$H$197,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$198,$A12,'QA Checklist'!$H$5:$H$198,"Pending")</f>
         <v/>
       </c>
       <c r="F12" s="8">
@@ -698,19 +698,19 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$197,$A13)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$198,$A13)</f>
         <v/>
       </c>
       <c r="C13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$197,$A13,'QA Checklist'!$H$5:$H$197,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$197,$A13,'QA Checklist'!$H$5:$H$197,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$198,$A13,'QA Checklist'!$H$5:$H$198,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$198,$A13,'QA Checklist'!$H$5:$H$198,"Pass")</f>
         <v/>
       </c>
       <c r="D13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$197,$A13,'QA Checklist'!$H$5:$H$197,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$197,$A13,'QA Checklist'!$H$5:$H$197,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$198,$A13,'QA Checklist'!$H$5:$H$198,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$198,$A13,'QA Checklist'!$H$5:$H$198,"Fail")</f>
         <v/>
       </c>
       <c r="E13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$197,$A13,'QA Checklist'!$H$5:$H$197,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$198,$A13,'QA Checklist'!$H$5:$H$198,"Pending")</f>
         <v/>
       </c>
       <c r="F13" s="8">
@@ -725,19 +725,19 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$197,$A14)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$198,$A14)</f>
         <v/>
       </c>
       <c r="C14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$197,$A14,'QA Checklist'!$H$5:$H$197,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$197,$A14,'QA Checklist'!$H$5:$H$197,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$198,$A14,'QA Checklist'!$H$5:$H$198,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$198,$A14,'QA Checklist'!$H$5:$H$198,"Pass")</f>
         <v/>
       </c>
       <c r="D14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$197,$A14,'QA Checklist'!$H$5:$H$197,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$197,$A14,'QA Checklist'!$H$5:$H$197,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$198,$A14,'QA Checklist'!$H$5:$H$198,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$198,$A14,'QA Checklist'!$H$5:$H$198,"Fail")</f>
         <v/>
       </c>
       <c r="E14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$197,$A14,'QA Checklist'!$H$5:$H$197,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$198,$A14,'QA Checklist'!$H$5:$H$198,"Pending")</f>
         <v/>
       </c>
       <c r="F14" s="8">
@@ -752,19 +752,19 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$197,$A15)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$198,$A15)</f>
         <v/>
       </c>
       <c r="C15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$197,$A15,'QA Checklist'!$H$5:$H$197,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$197,$A15,'QA Checklist'!$H$5:$H$197,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$198,$A15,'QA Checklist'!$H$5:$H$198,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$198,$A15,'QA Checklist'!$H$5:$H$198,"Pass")</f>
         <v/>
       </c>
       <c r="D15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$197,$A15,'QA Checklist'!$H$5:$H$197,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$197,$A15,'QA Checklist'!$H$5:$H$197,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$198,$A15,'QA Checklist'!$H$5:$H$198,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$198,$A15,'QA Checklist'!$H$5:$H$198,"Fail")</f>
         <v/>
       </c>
       <c r="E15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$197,$A15,'QA Checklist'!$H$5:$H$197,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$198,$A15,'QA Checklist'!$H$5:$H$198,"Pending")</f>
         <v/>
       </c>
       <c r="F15" s="8">
@@ -779,19 +779,19 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$197,$A16)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$198,$A16)</f>
         <v/>
       </c>
       <c r="C16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$197,$A16,'QA Checklist'!$H$5:$H$197,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$197,$A16,'QA Checklist'!$H$5:$H$197,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$198,$A16,'QA Checklist'!$H$5:$H$198,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$198,$A16,'QA Checklist'!$H$5:$H$198,"Pass")</f>
         <v/>
       </c>
       <c r="D16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$197,$A16,'QA Checklist'!$H$5:$H$197,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$197,$A16,'QA Checklist'!$H$5:$H$197,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$198,$A16,'QA Checklist'!$H$5:$H$198,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$198,$A16,'QA Checklist'!$H$5:$H$198,"Fail")</f>
         <v/>
       </c>
       <c r="E16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$197,$A16,'QA Checklist'!$H$5:$H$197,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$198,$A16,'QA Checklist'!$H$5:$H$198,"Pending")</f>
         <v/>
       </c>
       <c r="F16" s="8">
@@ -806,19 +806,19 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$197,$A17)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$198,$A17)</f>
         <v/>
       </c>
       <c r="C17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$197,$A17,'QA Checklist'!$H$5:$H$197,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$197,$A17,'QA Checklist'!$H$5:$H$197,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$198,$A17,'QA Checklist'!$H$5:$H$198,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$198,$A17,'QA Checklist'!$H$5:$H$198,"Pass")</f>
         <v/>
       </c>
       <c r="D17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$197,$A17,'QA Checklist'!$H$5:$H$197,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$197,$A17,'QA Checklist'!$H$5:$H$197,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$198,$A17,'QA Checklist'!$H$5:$H$198,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$198,$A17,'QA Checklist'!$H$5:$H$198,"Fail")</f>
         <v/>
       </c>
       <c r="E17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$197,$A17,'QA Checklist'!$H$5:$H$197,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$198,$A17,'QA Checklist'!$H$5:$H$198,"Pending")</f>
         <v/>
       </c>
       <c r="F17" s="8">
@@ -833,19 +833,19 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$197,$A18)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$198,$A18)</f>
         <v/>
       </c>
       <c r="C18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$197,$A18,'QA Checklist'!$H$5:$H$197,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$197,$A18,'QA Checklist'!$H$5:$H$197,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$198,$A18,'QA Checklist'!$H$5:$H$198,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$198,$A18,'QA Checklist'!$H$5:$H$198,"Pass")</f>
         <v/>
       </c>
       <c r="D18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$197,$A18,'QA Checklist'!$H$5:$H$197,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$197,$A18,'QA Checklist'!$H$5:$H$197,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$198,$A18,'QA Checklist'!$H$5:$H$198,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$198,$A18,'QA Checklist'!$H$5:$H$198,"Fail")</f>
         <v/>
       </c>
       <c r="E18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$197,$A18,'QA Checklist'!$H$5:$H$197,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$198,$A18,'QA Checklist'!$H$5:$H$198,"Pending")</f>
         <v/>
       </c>
       <c r="F18" s="8">
@@ -860,19 +860,19 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$197,$A19)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$198,$A19)</f>
         <v/>
       </c>
       <c r="C19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$197,$A19,'QA Checklist'!$H$5:$H$197,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$197,$A19,'QA Checklist'!$H$5:$H$197,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$198,$A19,'QA Checklist'!$H$5:$H$198,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$198,$A19,'QA Checklist'!$H$5:$H$198,"Pass")</f>
         <v/>
       </c>
       <c r="D19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$197,$A19,'QA Checklist'!$H$5:$H$197,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$197,$A19,'QA Checklist'!$H$5:$H$197,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$198,$A19,'QA Checklist'!$H$5:$H$198,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$198,$A19,'QA Checklist'!$H$5:$H$198,"Fail")</f>
         <v/>
       </c>
       <c r="E19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$197,$A19,'QA Checklist'!$H$5:$H$197,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$198,$A19,'QA Checklist'!$H$5:$H$198,"Pending")</f>
         <v/>
       </c>
       <c r="F19" s="8">
@@ -887,19 +887,19 @@
         </is>
       </c>
       <c r="B20" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$197,$A20)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$198,$A20)</f>
         <v/>
       </c>
       <c r="C20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$197,$A20,'QA Checklist'!$H$5:$H$197,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$197,$A20,'QA Checklist'!$H$5:$H$197,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$198,$A20,'QA Checklist'!$H$5:$H$198,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$198,$A20,'QA Checklist'!$H$5:$H$198,"Pass")</f>
         <v/>
       </c>
       <c r="D20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$197,$A20,'QA Checklist'!$H$5:$H$197,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$197,$A20,'QA Checklist'!$H$5:$H$197,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$198,$A20,'QA Checklist'!$H$5:$H$198,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$198,$A20,'QA Checklist'!$H$5:$H$198,"Fail")</f>
         <v/>
       </c>
       <c r="E20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$197,$A20,'QA Checklist'!$H$5:$H$197,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$198,$A20,'QA Checklist'!$H$5:$H$198,"Pending")</f>
         <v/>
       </c>
       <c r="F20" s="8">
@@ -914,19 +914,19 @@
         </is>
       </c>
       <c r="B21" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$197,$A21)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$198,$A21)</f>
         <v/>
       </c>
       <c r="C21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$197,$A21,'QA Checklist'!$H$5:$H$197,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$197,$A21,'QA Checklist'!$H$5:$H$197,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$198,$A21,'QA Checklist'!$H$5:$H$198,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$198,$A21,'QA Checklist'!$H$5:$H$198,"Pass")</f>
         <v/>
       </c>
       <c r="D21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$197,$A21,'QA Checklist'!$H$5:$H$197,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$197,$A21,'QA Checklist'!$H$5:$H$197,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$198,$A21,'QA Checklist'!$H$5:$H$198,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$198,$A21,'QA Checklist'!$H$5:$H$198,"Fail")</f>
         <v/>
       </c>
       <c r="E21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$197,$A21,'QA Checklist'!$H$5:$H$197,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$198,$A21,'QA Checklist'!$H$5:$H$198,"Pending")</f>
         <v/>
       </c>
       <c r="F21" s="8">
@@ -941,19 +941,19 @@
         </is>
       </c>
       <c r="B22" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$197,$A22)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$198,$A22)</f>
         <v/>
       </c>
       <c r="C22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$197,$A22,'QA Checklist'!$H$5:$H$197,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$197,$A22,'QA Checklist'!$H$5:$H$197,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$198,$A22,'QA Checklist'!$H$5:$H$198,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$198,$A22,'QA Checklist'!$H$5:$H$198,"Pass")</f>
         <v/>
       </c>
       <c r="D22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$197,$A22,'QA Checklist'!$H$5:$H$197,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$197,$A22,'QA Checklist'!$H$5:$H$197,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$198,$A22,'QA Checklist'!$H$5:$H$198,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$198,$A22,'QA Checklist'!$H$5:$H$198,"Fail")</f>
         <v/>
       </c>
       <c r="E22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$197,$A22,'QA Checklist'!$H$5:$H$197,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$198,$A22,'QA Checklist'!$H$5:$H$198,"Pending")</f>
         <v/>
       </c>
       <c r="F22" s="8">
@@ -1023,19 +1023,19 @@
         </is>
       </c>
       <c r="B26" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$197,$A26&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$198,$A26&amp;"*")</f>
         <v/>
       </c>
       <c r="C26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$197,$A26&amp;"*",'QA Checklist'!$H$5:$H$197,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$197,$A26&amp;"*",'QA Checklist'!$H$5:$H$197,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$198,$A26&amp;"*",'QA Checklist'!$H$5:$H$198,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$198,$A26&amp;"*",'QA Checklist'!$H$5:$H$198,"Pass")</f>
         <v/>
       </c>
       <c r="D26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$197,$A26&amp;"*",'QA Checklist'!$H$5:$H$197,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$197,$A26&amp;"*",'QA Checklist'!$H$5:$H$197,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$198,$A26&amp;"*",'QA Checklist'!$H$5:$H$198,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$198,$A26&amp;"*",'QA Checklist'!$H$5:$H$198,"Fail")</f>
         <v/>
       </c>
       <c r="E26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$197,$A26&amp;"*",'QA Checklist'!$H$5:$H$197,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$198,$A26&amp;"*",'QA Checklist'!$H$5:$H$198,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1046,19 +1046,19 @@
         </is>
       </c>
       <c r="B27" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$197,$A27&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$198,$A27&amp;"*")</f>
         <v/>
       </c>
       <c r="C27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$197,$A27&amp;"*",'QA Checklist'!$H$5:$H$197,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$197,$A27&amp;"*",'QA Checklist'!$H$5:$H$197,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$198,$A27&amp;"*",'QA Checklist'!$H$5:$H$198,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$198,$A27&amp;"*",'QA Checklist'!$H$5:$H$198,"Pass")</f>
         <v/>
       </c>
       <c r="D27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$197,$A27&amp;"*",'QA Checklist'!$H$5:$H$197,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$197,$A27&amp;"*",'QA Checklist'!$H$5:$H$197,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$198,$A27&amp;"*",'QA Checklist'!$H$5:$H$198,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$198,$A27&amp;"*",'QA Checklist'!$H$5:$H$198,"Fail")</f>
         <v/>
       </c>
       <c r="E27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$197,$A27&amp;"*",'QA Checklist'!$H$5:$H$197,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$198,$A27&amp;"*",'QA Checklist'!$H$5:$H$198,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1069,19 +1069,19 @@
         </is>
       </c>
       <c r="B28" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$197,$A28&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$198,$A28&amp;"*")</f>
         <v/>
       </c>
       <c r="C28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$197,$A28&amp;"*",'QA Checklist'!$H$5:$H$197,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$197,$A28&amp;"*",'QA Checklist'!$H$5:$H$197,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$198,$A28&amp;"*",'QA Checklist'!$H$5:$H$198,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$198,$A28&amp;"*",'QA Checklist'!$H$5:$H$198,"Pass")</f>
         <v/>
       </c>
       <c r="D28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$197,$A28&amp;"*",'QA Checklist'!$H$5:$H$197,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$197,$A28&amp;"*",'QA Checklist'!$H$5:$H$197,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$198,$A28&amp;"*",'QA Checklist'!$H$5:$H$198,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$198,$A28&amp;"*",'QA Checklist'!$H$5:$H$198,"Fail")</f>
         <v/>
       </c>
       <c r="E28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$197,$A28&amp;"*",'QA Checklist'!$H$5:$H$197,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$198,$A28&amp;"*",'QA Checklist'!$H$5:$H$198,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1096,7 +1096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I197"/>
+  <dimension ref="A1:I198"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9798,12 +9798,59 @@
         </is>
       </c>
     </row>
+    <row r="198">
+      <c r="A198" s="12" t="inlineStr">
+        <is>
+          <t>SA-72</t>
+        </is>
+      </c>
+      <c r="B198" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="C198" s="13" t="inlineStr">
+        <is>
+          <t>Tier 2 (Workflow &amp; Ergonomics)</t>
+        </is>
+      </c>
+      <c r="D198" s="13" t="inlineStr">
+        <is>
+          <t>TV Auto-Scroll &amp; Daily Reset</t>
+        </is>
+      </c>
+      <c r="E198" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="F198" s="13" t="inlineStr">
+        <is>
+          <t>Fill a lane with more vehicles than fit and watch the TV; touch the screen while it scrolls; the next day, check that yesterday's vehicles are gone from the TV and carry-over vehicles are still shown</t>
+        </is>
+      </c>
+      <c r="G198" s="13" t="inlineStr">
+        <is>
+          <t>Long lists scroll to the bottom and back by themselves and the slide waits for them; touching pauses it; the TV shows only today's intakes plus all carry-over vehicles, matching Daily Intakes</t>
+        </is>
+      </c>
+      <c r="H198" s="14" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="I198" s="13" t="inlineStr">
+        <is>
+          <t>Verified by Automated Unit Tests (184 passing in tests/frontend/sla_and_logic.test.js AUT-FRONT-155), live feed check with temporary rows and headless Chrome 13/13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:I197"/>
+  <autoFilter ref="A4:I198"/>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="H5:H197">
+  <conditionalFormatting sqref="H5:H198">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$H5="Passed"</formula>
     </cfRule>
@@ -9820,13 +9867,13 @@
       <formula>$H5="Pending"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A5:A197">
+  <conditionalFormatting sqref="A5:A198">
     <cfRule type="expression" priority="6" dxfId="3">
-      <formula>COUNTIF($A$5:$A$197,$A5)&gt;1</formula>
+      <formula>COUNTIF($A$5:$A$198,$A5)&gt;1</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H5:H197" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H5:H198" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pending,Passed,Failed"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat(REV-197): open TVs update themselves; returned carry-overs tagged
The feed reports the TV page version and an open TV reloads itself once when a new version is published (an open page only downloads data, so TVs opened before an update kept the old page). In Service / In Queue cards of returned carry-over vehicles show a Carry-Over tag.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
+++ b/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
@@ -11,7 +11,7 @@
     <sheet name="QA Checklist" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$198</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$199</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'QA Checklist'!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTA('QA Checklist'!$A$5:$A$198)</f>
+        <f>COUNTA('QA Checklist'!$A$5:$A$199)</f>
         <v/>
       </c>
     </row>
@@ -594,7 +594,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$198,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$198,"Pass")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$199,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$199,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$198,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$198,"Fail")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$199,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$199,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -616,7 +616,7 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$198,"Pending")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$199,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -671,19 +671,19 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$198,$A12)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$199,$A12)</f>
         <v/>
       </c>
       <c r="C12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$198,$A12,'QA Checklist'!$H$5:$H$198,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$198,$A12,'QA Checklist'!$H$5:$H$198,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$199,$A12,'QA Checklist'!$H$5:$H$199,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$199,$A12,'QA Checklist'!$H$5:$H$199,"Pass")</f>
         <v/>
       </c>
       <c r="D12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$198,$A12,'QA Checklist'!$H$5:$H$198,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$198,$A12,'QA Checklist'!$H$5:$H$198,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$199,$A12,'QA Checklist'!$H$5:$H$199,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$199,$A12,'QA Checklist'!$H$5:$H$199,"Fail")</f>
         <v/>
       </c>
       <c r="E12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$198,$A12,'QA Checklist'!$H$5:$H$198,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$199,$A12,'QA Checklist'!$H$5:$H$199,"Pending")</f>
         <v/>
       </c>
       <c r="F12" s="8">
@@ -698,19 +698,19 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$198,$A13)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$199,$A13)</f>
         <v/>
       </c>
       <c r="C13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$198,$A13,'QA Checklist'!$H$5:$H$198,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$198,$A13,'QA Checklist'!$H$5:$H$198,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$199,$A13,'QA Checklist'!$H$5:$H$199,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$199,$A13,'QA Checklist'!$H$5:$H$199,"Pass")</f>
         <v/>
       </c>
       <c r="D13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$198,$A13,'QA Checklist'!$H$5:$H$198,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$198,$A13,'QA Checklist'!$H$5:$H$198,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$199,$A13,'QA Checklist'!$H$5:$H$199,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$199,$A13,'QA Checklist'!$H$5:$H$199,"Fail")</f>
         <v/>
       </c>
       <c r="E13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$198,$A13,'QA Checklist'!$H$5:$H$198,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$199,$A13,'QA Checklist'!$H$5:$H$199,"Pending")</f>
         <v/>
       </c>
       <c r="F13" s="8">
@@ -725,19 +725,19 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$198,$A14)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$199,$A14)</f>
         <v/>
       </c>
       <c r="C14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$198,$A14,'QA Checklist'!$H$5:$H$198,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$198,$A14,'QA Checklist'!$H$5:$H$198,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$199,$A14,'QA Checklist'!$H$5:$H$199,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$199,$A14,'QA Checklist'!$H$5:$H$199,"Pass")</f>
         <v/>
       </c>
       <c r="D14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$198,$A14,'QA Checklist'!$H$5:$H$198,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$198,$A14,'QA Checklist'!$H$5:$H$198,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$199,$A14,'QA Checklist'!$H$5:$H$199,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$199,$A14,'QA Checklist'!$H$5:$H$199,"Fail")</f>
         <v/>
       </c>
       <c r="E14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$198,$A14,'QA Checklist'!$H$5:$H$198,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$199,$A14,'QA Checklist'!$H$5:$H$199,"Pending")</f>
         <v/>
       </c>
       <c r="F14" s="8">
@@ -752,19 +752,19 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$198,$A15)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$199,$A15)</f>
         <v/>
       </c>
       <c r="C15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$198,$A15,'QA Checklist'!$H$5:$H$198,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$198,$A15,'QA Checklist'!$H$5:$H$198,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$199,$A15,'QA Checklist'!$H$5:$H$199,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$199,$A15,'QA Checklist'!$H$5:$H$199,"Pass")</f>
         <v/>
       </c>
       <c r="D15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$198,$A15,'QA Checklist'!$H$5:$H$198,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$198,$A15,'QA Checklist'!$H$5:$H$198,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$199,$A15,'QA Checklist'!$H$5:$H$199,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$199,$A15,'QA Checklist'!$H$5:$H$199,"Fail")</f>
         <v/>
       </c>
       <c r="E15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$198,$A15,'QA Checklist'!$H$5:$H$198,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$199,$A15,'QA Checklist'!$H$5:$H$199,"Pending")</f>
         <v/>
       </c>
       <c r="F15" s="8">
@@ -779,19 +779,19 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$198,$A16)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$199,$A16)</f>
         <v/>
       </c>
       <c r="C16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$198,$A16,'QA Checklist'!$H$5:$H$198,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$198,$A16,'QA Checklist'!$H$5:$H$198,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$199,$A16,'QA Checklist'!$H$5:$H$199,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$199,$A16,'QA Checklist'!$H$5:$H$199,"Pass")</f>
         <v/>
       </c>
       <c r="D16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$198,$A16,'QA Checklist'!$H$5:$H$198,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$198,$A16,'QA Checklist'!$H$5:$H$198,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$199,$A16,'QA Checklist'!$H$5:$H$199,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$199,$A16,'QA Checklist'!$H$5:$H$199,"Fail")</f>
         <v/>
       </c>
       <c r="E16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$198,$A16,'QA Checklist'!$H$5:$H$198,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$199,$A16,'QA Checklist'!$H$5:$H$199,"Pending")</f>
         <v/>
       </c>
       <c r="F16" s="8">
@@ -806,19 +806,19 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$198,$A17)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$199,$A17)</f>
         <v/>
       </c>
       <c r="C17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$198,$A17,'QA Checklist'!$H$5:$H$198,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$198,$A17,'QA Checklist'!$H$5:$H$198,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$199,$A17,'QA Checklist'!$H$5:$H$199,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$199,$A17,'QA Checklist'!$H$5:$H$199,"Pass")</f>
         <v/>
       </c>
       <c r="D17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$198,$A17,'QA Checklist'!$H$5:$H$198,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$198,$A17,'QA Checklist'!$H$5:$H$198,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$199,$A17,'QA Checklist'!$H$5:$H$199,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$199,$A17,'QA Checklist'!$H$5:$H$199,"Fail")</f>
         <v/>
       </c>
       <c r="E17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$198,$A17,'QA Checklist'!$H$5:$H$198,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$199,$A17,'QA Checklist'!$H$5:$H$199,"Pending")</f>
         <v/>
       </c>
       <c r="F17" s="8">
@@ -833,19 +833,19 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$198,$A18)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$199,$A18)</f>
         <v/>
       </c>
       <c r="C18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$198,$A18,'QA Checklist'!$H$5:$H$198,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$198,$A18,'QA Checklist'!$H$5:$H$198,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$199,$A18,'QA Checklist'!$H$5:$H$199,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$199,$A18,'QA Checklist'!$H$5:$H$199,"Pass")</f>
         <v/>
       </c>
       <c r="D18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$198,$A18,'QA Checklist'!$H$5:$H$198,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$198,$A18,'QA Checklist'!$H$5:$H$198,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$199,$A18,'QA Checklist'!$H$5:$H$199,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$199,$A18,'QA Checklist'!$H$5:$H$199,"Fail")</f>
         <v/>
       </c>
       <c r="E18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$198,$A18,'QA Checklist'!$H$5:$H$198,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$199,$A18,'QA Checklist'!$H$5:$H$199,"Pending")</f>
         <v/>
       </c>
       <c r="F18" s="8">
@@ -860,19 +860,19 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$198,$A19)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$199,$A19)</f>
         <v/>
       </c>
       <c r="C19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$198,$A19,'QA Checklist'!$H$5:$H$198,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$198,$A19,'QA Checklist'!$H$5:$H$198,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$199,$A19,'QA Checklist'!$H$5:$H$199,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$199,$A19,'QA Checklist'!$H$5:$H$199,"Pass")</f>
         <v/>
       </c>
       <c r="D19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$198,$A19,'QA Checklist'!$H$5:$H$198,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$198,$A19,'QA Checklist'!$H$5:$H$198,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$199,$A19,'QA Checklist'!$H$5:$H$199,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$199,$A19,'QA Checklist'!$H$5:$H$199,"Fail")</f>
         <v/>
       </c>
       <c r="E19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$198,$A19,'QA Checklist'!$H$5:$H$198,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$199,$A19,'QA Checklist'!$H$5:$H$199,"Pending")</f>
         <v/>
       </c>
       <c r="F19" s="8">
@@ -887,19 +887,19 @@
         </is>
       </c>
       <c r="B20" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$198,$A20)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$199,$A20)</f>
         <v/>
       </c>
       <c r="C20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$198,$A20,'QA Checklist'!$H$5:$H$198,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$198,$A20,'QA Checklist'!$H$5:$H$198,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$199,$A20,'QA Checklist'!$H$5:$H$199,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$199,$A20,'QA Checklist'!$H$5:$H$199,"Pass")</f>
         <v/>
       </c>
       <c r="D20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$198,$A20,'QA Checklist'!$H$5:$H$198,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$198,$A20,'QA Checklist'!$H$5:$H$198,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$199,$A20,'QA Checklist'!$H$5:$H$199,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$199,$A20,'QA Checklist'!$H$5:$H$199,"Fail")</f>
         <v/>
       </c>
       <c r="E20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$198,$A20,'QA Checklist'!$H$5:$H$198,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$199,$A20,'QA Checklist'!$H$5:$H$199,"Pending")</f>
         <v/>
       </c>
       <c r="F20" s="8">
@@ -914,19 +914,19 @@
         </is>
       </c>
       <c r="B21" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$198,$A21)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$199,$A21)</f>
         <v/>
       </c>
       <c r="C21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$198,$A21,'QA Checklist'!$H$5:$H$198,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$198,$A21,'QA Checklist'!$H$5:$H$198,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$199,$A21,'QA Checklist'!$H$5:$H$199,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$199,$A21,'QA Checklist'!$H$5:$H$199,"Pass")</f>
         <v/>
       </c>
       <c r="D21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$198,$A21,'QA Checklist'!$H$5:$H$198,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$198,$A21,'QA Checklist'!$H$5:$H$198,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$199,$A21,'QA Checklist'!$H$5:$H$199,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$199,$A21,'QA Checklist'!$H$5:$H$199,"Fail")</f>
         <v/>
       </c>
       <c r="E21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$198,$A21,'QA Checklist'!$H$5:$H$198,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$199,$A21,'QA Checklist'!$H$5:$H$199,"Pending")</f>
         <v/>
       </c>
       <c r="F21" s="8">
@@ -941,19 +941,19 @@
         </is>
       </c>
       <c r="B22" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$198,$A22)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$199,$A22)</f>
         <v/>
       </c>
       <c r="C22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$198,$A22,'QA Checklist'!$H$5:$H$198,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$198,$A22,'QA Checklist'!$H$5:$H$198,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$199,$A22,'QA Checklist'!$H$5:$H$199,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$199,$A22,'QA Checklist'!$H$5:$H$199,"Pass")</f>
         <v/>
       </c>
       <c r="D22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$198,$A22,'QA Checklist'!$H$5:$H$198,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$198,$A22,'QA Checklist'!$H$5:$H$198,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$199,$A22,'QA Checklist'!$H$5:$H$199,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$199,$A22,'QA Checklist'!$H$5:$H$199,"Fail")</f>
         <v/>
       </c>
       <c r="E22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$198,$A22,'QA Checklist'!$H$5:$H$198,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$199,$A22,'QA Checklist'!$H$5:$H$199,"Pending")</f>
         <v/>
       </c>
       <c r="F22" s="8">
@@ -1023,19 +1023,19 @@
         </is>
       </c>
       <c r="B26" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$198,$A26&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$199,$A26&amp;"*")</f>
         <v/>
       </c>
       <c r="C26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$198,$A26&amp;"*",'QA Checklist'!$H$5:$H$198,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$198,$A26&amp;"*",'QA Checklist'!$H$5:$H$198,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$199,$A26&amp;"*",'QA Checklist'!$H$5:$H$199,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$199,$A26&amp;"*",'QA Checklist'!$H$5:$H$199,"Pass")</f>
         <v/>
       </c>
       <c r="D26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$198,$A26&amp;"*",'QA Checklist'!$H$5:$H$198,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$198,$A26&amp;"*",'QA Checklist'!$H$5:$H$198,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$199,$A26&amp;"*",'QA Checklist'!$H$5:$H$199,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$199,$A26&amp;"*",'QA Checklist'!$H$5:$H$199,"Fail")</f>
         <v/>
       </c>
       <c r="E26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$198,$A26&amp;"*",'QA Checklist'!$H$5:$H$198,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$199,$A26&amp;"*",'QA Checklist'!$H$5:$H$199,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1046,19 +1046,19 @@
         </is>
       </c>
       <c r="B27" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$198,$A27&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$199,$A27&amp;"*")</f>
         <v/>
       </c>
       <c r="C27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$198,$A27&amp;"*",'QA Checklist'!$H$5:$H$198,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$198,$A27&amp;"*",'QA Checklist'!$H$5:$H$198,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$199,$A27&amp;"*",'QA Checklist'!$H$5:$H$199,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$199,$A27&amp;"*",'QA Checklist'!$H$5:$H$199,"Pass")</f>
         <v/>
       </c>
       <c r="D27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$198,$A27&amp;"*",'QA Checklist'!$H$5:$H$198,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$198,$A27&amp;"*",'QA Checklist'!$H$5:$H$198,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$199,$A27&amp;"*",'QA Checklist'!$H$5:$H$199,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$199,$A27&amp;"*",'QA Checklist'!$H$5:$H$199,"Fail")</f>
         <v/>
       </c>
       <c r="E27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$198,$A27&amp;"*",'QA Checklist'!$H$5:$H$198,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$199,$A27&amp;"*",'QA Checklist'!$H$5:$H$199,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1069,19 +1069,19 @@
         </is>
       </c>
       <c r="B28" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$198,$A28&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$199,$A28&amp;"*")</f>
         <v/>
       </c>
       <c r="C28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$198,$A28&amp;"*",'QA Checklist'!$H$5:$H$198,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$198,$A28&amp;"*",'QA Checklist'!$H$5:$H$198,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$199,$A28&amp;"*",'QA Checklist'!$H$5:$H$199,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$199,$A28&amp;"*",'QA Checklist'!$H$5:$H$199,"Pass")</f>
         <v/>
       </c>
       <c r="D28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$198,$A28&amp;"*",'QA Checklist'!$H$5:$H$198,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$198,$A28&amp;"*",'QA Checklist'!$H$5:$H$198,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$199,$A28&amp;"*",'QA Checklist'!$H$5:$H$199,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$199,$A28&amp;"*",'QA Checklist'!$H$5:$H$199,"Fail")</f>
         <v/>
       </c>
       <c r="E28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$198,$A28&amp;"*",'QA Checklist'!$H$5:$H$198,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$199,$A28&amp;"*",'QA Checklist'!$H$5:$H$199,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1096,7 +1096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I198"/>
+  <dimension ref="A1:I199"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9845,12 +9845,59 @@
         </is>
       </c>
     </row>
+    <row r="199">
+      <c r="A199" s="12" t="inlineStr">
+        <is>
+          <t>SA-73</t>
+        </is>
+      </c>
+      <c r="B199" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="C199" s="13" t="inlineStr">
+        <is>
+          <t>Tier 2 (Workflow &amp; Ergonomics)</t>
+        </is>
+      </c>
+      <c r="D199" s="13" t="inlineStr">
+        <is>
+          <t>TV Self-Update &amp; Carry-Over Tag</t>
+        </is>
+      </c>
+      <c r="E199" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="F199" s="13" t="inlineStr">
+        <is>
+          <t>Leave the TV open, publish a new TV page version, and watch the TV; send a carry-over vehicle back to work and look at In Service / In Queue on slide 2</t>
+        </is>
+      </c>
+      <c r="G199" s="13" t="inlineStr">
+        <is>
+          <t>The TV reloads by itself within seconds and returns to the live screen without a PIN; returned carry-over vehicles show a Carry-Over tag</t>
+        </is>
+      </c>
+      <c r="H199" s="14" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="I199" s="13" t="inlineStr">
+        <is>
+          <t>Verified by Automated Unit Tests (185 passing in tests/frontend/sla_and_logic.test.js AUT-FRONT-156) and headless Chrome 6/6</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:I198"/>
+  <autoFilter ref="A4:I199"/>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="H5:H198">
+  <conditionalFormatting sqref="H5:H199">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$H5="Passed"</formula>
     </cfRule>
@@ -9867,13 +9914,13 @@
       <formula>$H5="Pending"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A5:A198">
+  <conditionalFormatting sqref="A5:A199">
     <cfRule type="expression" priority="6" dxfId="3">
-      <formula>COUNTIF($A$5:$A$198,$A5)&gt;1</formula>
+      <formula>COUNTIF($A$5:$A$199,$A5)&gt;1</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H5:H198" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H5:H199" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pending,Passed,Failed"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
fix(REV-198): never serve HTML pages from a stale browser cache
Apache sent tv.html without Cache-Control, so browsers kept running an old TV page (without auto-scroll) for hours. HTML pages now get Cache-Control: no-cache and the in-app TV frame uses a versioned link.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
+++ b/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
@@ -11,7 +11,7 @@
     <sheet name="QA Checklist" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$199</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$200</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'QA Checklist'!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTA('QA Checklist'!$A$5:$A$199)</f>
+        <f>COUNTA('QA Checklist'!$A$5:$A$200)</f>
         <v/>
       </c>
     </row>
@@ -594,7 +594,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$199,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$199,"Pass")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$200,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$200,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$199,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$199,"Fail")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$200,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$200,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -616,7 +616,7 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$199,"Pending")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$200,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -671,19 +671,19 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$199,$A12)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$200,$A12)</f>
         <v/>
       </c>
       <c r="C12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$199,$A12,'QA Checklist'!$H$5:$H$199,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$199,$A12,'QA Checklist'!$H$5:$H$199,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$200,$A12,'QA Checklist'!$H$5:$H$200,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$200,$A12,'QA Checklist'!$H$5:$H$200,"Pass")</f>
         <v/>
       </c>
       <c r="D12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$199,$A12,'QA Checklist'!$H$5:$H$199,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$199,$A12,'QA Checklist'!$H$5:$H$199,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$200,$A12,'QA Checklist'!$H$5:$H$200,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$200,$A12,'QA Checklist'!$H$5:$H$200,"Fail")</f>
         <v/>
       </c>
       <c r="E12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$199,$A12,'QA Checklist'!$H$5:$H$199,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$200,$A12,'QA Checklist'!$H$5:$H$200,"Pending")</f>
         <v/>
       </c>
       <c r="F12" s="8">
@@ -698,19 +698,19 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$199,$A13)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$200,$A13)</f>
         <v/>
       </c>
       <c r="C13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$199,$A13,'QA Checklist'!$H$5:$H$199,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$199,$A13,'QA Checklist'!$H$5:$H$199,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$200,$A13,'QA Checklist'!$H$5:$H$200,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$200,$A13,'QA Checklist'!$H$5:$H$200,"Pass")</f>
         <v/>
       </c>
       <c r="D13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$199,$A13,'QA Checklist'!$H$5:$H$199,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$199,$A13,'QA Checklist'!$H$5:$H$199,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$200,$A13,'QA Checklist'!$H$5:$H$200,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$200,$A13,'QA Checklist'!$H$5:$H$200,"Fail")</f>
         <v/>
       </c>
       <c r="E13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$199,$A13,'QA Checklist'!$H$5:$H$199,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$200,$A13,'QA Checklist'!$H$5:$H$200,"Pending")</f>
         <v/>
       </c>
       <c r="F13" s="8">
@@ -725,19 +725,19 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$199,$A14)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$200,$A14)</f>
         <v/>
       </c>
       <c r="C14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$199,$A14,'QA Checklist'!$H$5:$H$199,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$199,$A14,'QA Checklist'!$H$5:$H$199,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$200,$A14,'QA Checklist'!$H$5:$H$200,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$200,$A14,'QA Checklist'!$H$5:$H$200,"Pass")</f>
         <v/>
       </c>
       <c r="D14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$199,$A14,'QA Checklist'!$H$5:$H$199,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$199,$A14,'QA Checklist'!$H$5:$H$199,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$200,$A14,'QA Checklist'!$H$5:$H$200,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$200,$A14,'QA Checklist'!$H$5:$H$200,"Fail")</f>
         <v/>
       </c>
       <c r="E14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$199,$A14,'QA Checklist'!$H$5:$H$199,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$200,$A14,'QA Checklist'!$H$5:$H$200,"Pending")</f>
         <v/>
       </c>
       <c r="F14" s="8">
@@ -752,19 +752,19 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$199,$A15)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$200,$A15)</f>
         <v/>
       </c>
       <c r="C15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$199,$A15,'QA Checklist'!$H$5:$H$199,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$199,$A15,'QA Checklist'!$H$5:$H$199,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$200,$A15,'QA Checklist'!$H$5:$H$200,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$200,$A15,'QA Checklist'!$H$5:$H$200,"Pass")</f>
         <v/>
       </c>
       <c r="D15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$199,$A15,'QA Checklist'!$H$5:$H$199,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$199,$A15,'QA Checklist'!$H$5:$H$199,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$200,$A15,'QA Checklist'!$H$5:$H$200,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$200,$A15,'QA Checklist'!$H$5:$H$200,"Fail")</f>
         <v/>
       </c>
       <c r="E15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$199,$A15,'QA Checklist'!$H$5:$H$199,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$200,$A15,'QA Checklist'!$H$5:$H$200,"Pending")</f>
         <v/>
       </c>
       <c r="F15" s="8">
@@ -779,19 +779,19 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$199,$A16)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$200,$A16)</f>
         <v/>
       </c>
       <c r="C16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$199,$A16,'QA Checklist'!$H$5:$H$199,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$199,$A16,'QA Checklist'!$H$5:$H$199,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$200,$A16,'QA Checklist'!$H$5:$H$200,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$200,$A16,'QA Checklist'!$H$5:$H$200,"Pass")</f>
         <v/>
       </c>
       <c r="D16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$199,$A16,'QA Checklist'!$H$5:$H$199,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$199,$A16,'QA Checklist'!$H$5:$H$199,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$200,$A16,'QA Checklist'!$H$5:$H$200,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$200,$A16,'QA Checklist'!$H$5:$H$200,"Fail")</f>
         <v/>
       </c>
       <c r="E16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$199,$A16,'QA Checklist'!$H$5:$H$199,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$200,$A16,'QA Checklist'!$H$5:$H$200,"Pending")</f>
         <v/>
       </c>
       <c r="F16" s="8">
@@ -806,19 +806,19 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$199,$A17)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$200,$A17)</f>
         <v/>
       </c>
       <c r="C17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$199,$A17,'QA Checklist'!$H$5:$H$199,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$199,$A17,'QA Checklist'!$H$5:$H$199,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$200,$A17,'QA Checklist'!$H$5:$H$200,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$200,$A17,'QA Checklist'!$H$5:$H$200,"Pass")</f>
         <v/>
       </c>
       <c r="D17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$199,$A17,'QA Checklist'!$H$5:$H$199,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$199,$A17,'QA Checklist'!$H$5:$H$199,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$200,$A17,'QA Checklist'!$H$5:$H$200,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$200,$A17,'QA Checklist'!$H$5:$H$200,"Fail")</f>
         <v/>
       </c>
       <c r="E17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$199,$A17,'QA Checklist'!$H$5:$H$199,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$200,$A17,'QA Checklist'!$H$5:$H$200,"Pending")</f>
         <v/>
       </c>
       <c r="F17" s="8">
@@ -833,19 +833,19 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$199,$A18)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$200,$A18)</f>
         <v/>
       </c>
       <c r="C18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$199,$A18,'QA Checklist'!$H$5:$H$199,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$199,$A18,'QA Checklist'!$H$5:$H$199,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$200,$A18,'QA Checklist'!$H$5:$H$200,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$200,$A18,'QA Checklist'!$H$5:$H$200,"Pass")</f>
         <v/>
       </c>
       <c r="D18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$199,$A18,'QA Checklist'!$H$5:$H$199,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$199,$A18,'QA Checklist'!$H$5:$H$199,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$200,$A18,'QA Checklist'!$H$5:$H$200,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$200,$A18,'QA Checklist'!$H$5:$H$200,"Fail")</f>
         <v/>
       </c>
       <c r="E18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$199,$A18,'QA Checklist'!$H$5:$H$199,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$200,$A18,'QA Checklist'!$H$5:$H$200,"Pending")</f>
         <v/>
       </c>
       <c r="F18" s="8">
@@ -860,19 +860,19 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$199,$A19)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$200,$A19)</f>
         <v/>
       </c>
       <c r="C19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$199,$A19,'QA Checklist'!$H$5:$H$199,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$199,$A19,'QA Checklist'!$H$5:$H$199,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$200,$A19,'QA Checklist'!$H$5:$H$200,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$200,$A19,'QA Checklist'!$H$5:$H$200,"Pass")</f>
         <v/>
       </c>
       <c r="D19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$199,$A19,'QA Checklist'!$H$5:$H$199,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$199,$A19,'QA Checklist'!$H$5:$H$199,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$200,$A19,'QA Checklist'!$H$5:$H$200,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$200,$A19,'QA Checklist'!$H$5:$H$200,"Fail")</f>
         <v/>
       </c>
       <c r="E19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$199,$A19,'QA Checklist'!$H$5:$H$199,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$200,$A19,'QA Checklist'!$H$5:$H$200,"Pending")</f>
         <v/>
       </c>
       <c r="F19" s="8">
@@ -887,19 +887,19 @@
         </is>
       </c>
       <c r="B20" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$199,$A20)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$200,$A20)</f>
         <v/>
       </c>
       <c r="C20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$199,$A20,'QA Checklist'!$H$5:$H$199,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$199,$A20,'QA Checklist'!$H$5:$H$199,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$200,$A20,'QA Checklist'!$H$5:$H$200,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$200,$A20,'QA Checklist'!$H$5:$H$200,"Pass")</f>
         <v/>
       </c>
       <c r="D20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$199,$A20,'QA Checklist'!$H$5:$H$199,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$199,$A20,'QA Checklist'!$H$5:$H$199,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$200,$A20,'QA Checklist'!$H$5:$H$200,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$200,$A20,'QA Checklist'!$H$5:$H$200,"Fail")</f>
         <v/>
       </c>
       <c r="E20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$199,$A20,'QA Checklist'!$H$5:$H$199,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$200,$A20,'QA Checklist'!$H$5:$H$200,"Pending")</f>
         <v/>
       </c>
       <c r="F20" s="8">
@@ -914,19 +914,19 @@
         </is>
       </c>
       <c r="B21" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$199,$A21)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$200,$A21)</f>
         <v/>
       </c>
       <c r="C21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$199,$A21,'QA Checklist'!$H$5:$H$199,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$199,$A21,'QA Checklist'!$H$5:$H$199,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$200,$A21,'QA Checklist'!$H$5:$H$200,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$200,$A21,'QA Checklist'!$H$5:$H$200,"Pass")</f>
         <v/>
       </c>
       <c r="D21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$199,$A21,'QA Checklist'!$H$5:$H$199,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$199,$A21,'QA Checklist'!$H$5:$H$199,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$200,$A21,'QA Checklist'!$H$5:$H$200,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$200,$A21,'QA Checklist'!$H$5:$H$200,"Fail")</f>
         <v/>
       </c>
       <c r="E21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$199,$A21,'QA Checklist'!$H$5:$H$199,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$200,$A21,'QA Checklist'!$H$5:$H$200,"Pending")</f>
         <v/>
       </c>
       <c r="F21" s="8">
@@ -941,19 +941,19 @@
         </is>
       </c>
       <c r="B22" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$199,$A22)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$200,$A22)</f>
         <v/>
       </c>
       <c r="C22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$199,$A22,'QA Checklist'!$H$5:$H$199,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$199,$A22,'QA Checklist'!$H$5:$H$199,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$200,$A22,'QA Checklist'!$H$5:$H$200,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$200,$A22,'QA Checklist'!$H$5:$H$200,"Pass")</f>
         <v/>
       </c>
       <c r="D22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$199,$A22,'QA Checklist'!$H$5:$H$199,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$199,$A22,'QA Checklist'!$H$5:$H$199,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$200,$A22,'QA Checklist'!$H$5:$H$200,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$200,$A22,'QA Checklist'!$H$5:$H$200,"Fail")</f>
         <v/>
       </c>
       <c r="E22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$199,$A22,'QA Checklist'!$H$5:$H$199,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$200,$A22,'QA Checklist'!$H$5:$H$200,"Pending")</f>
         <v/>
       </c>
       <c r="F22" s="8">
@@ -1023,19 +1023,19 @@
         </is>
       </c>
       <c r="B26" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$199,$A26&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$200,$A26&amp;"*")</f>
         <v/>
       </c>
       <c r="C26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$199,$A26&amp;"*",'QA Checklist'!$H$5:$H$199,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$199,$A26&amp;"*",'QA Checklist'!$H$5:$H$199,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$200,$A26&amp;"*",'QA Checklist'!$H$5:$H$200,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$200,$A26&amp;"*",'QA Checklist'!$H$5:$H$200,"Pass")</f>
         <v/>
       </c>
       <c r="D26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$199,$A26&amp;"*",'QA Checklist'!$H$5:$H$199,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$199,$A26&amp;"*",'QA Checklist'!$H$5:$H$199,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$200,$A26&amp;"*",'QA Checklist'!$H$5:$H$200,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$200,$A26&amp;"*",'QA Checklist'!$H$5:$H$200,"Fail")</f>
         <v/>
       </c>
       <c r="E26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$199,$A26&amp;"*",'QA Checklist'!$H$5:$H$199,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$200,$A26&amp;"*",'QA Checklist'!$H$5:$H$200,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1046,19 +1046,19 @@
         </is>
       </c>
       <c r="B27" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$199,$A27&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$200,$A27&amp;"*")</f>
         <v/>
       </c>
       <c r="C27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$199,$A27&amp;"*",'QA Checklist'!$H$5:$H$199,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$199,$A27&amp;"*",'QA Checklist'!$H$5:$H$199,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$200,$A27&amp;"*",'QA Checklist'!$H$5:$H$200,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$200,$A27&amp;"*",'QA Checklist'!$H$5:$H$200,"Pass")</f>
         <v/>
       </c>
       <c r="D27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$199,$A27&amp;"*",'QA Checklist'!$H$5:$H$199,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$199,$A27&amp;"*",'QA Checklist'!$H$5:$H$199,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$200,$A27&amp;"*",'QA Checklist'!$H$5:$H$200,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$200,$A27&amp;"*",'QA Checklist'!$H$5:$H$200,"Fail")</f>
         <v/>
       </c>
       <c r="E27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$199,$A27&amp;"*",'QA Checklist'!$H$5:$H$199,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$200,$A27&amp;"*",'QA Checklist'!$H$5:$H$200,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1069,19 +1069,19 @@
         </is>
       </c>
       <c r="B28" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$199,$A28&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$200,$A28&amp;"*")</f>
         <v/>
       </c>
       <c r="C28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$199,$A28&amp;"*",'QA Checklist'!$H$5:$H$199,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$199,$A28&amp;"*",'QA Checklist'!$H$5:$H$199,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$200,$A28&amp;"*",'QA Checklist'!$H$5:$H$200,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$200,$A28&amp;"*",'QA Checklist'!$H$5:$H$200,"Pass")</f>
         <v/>
       </c>
       <c r="D28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$199,$A28&amp;"*",'QA Checklist'!$H$5:$H$199,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$199,$A28&amp;"*",'QA Checklist'!$H$5:$H$199,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$200,$A28&amp;"*",'QA Checklist'!$H$5:$H$200,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$200,$A28&amp;"*",'QA Checklist'!$H$5:$H$200,"Fail")</f>
         <v/>
       </c>
       <c r="E28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$199,$A28&amp;"*",'QA Checklist'!$H$5:$H$199,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$200,$A28&amp;"*",'QA Checklist'!$H$5:$H$200,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1096,7 +1096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I199"/>
+  <dimension ref="A1:I200"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9892,12 +9892,59 @@
         </is>
       </c>
     </row>
+    <row r="200">
+      <c r="A200" s="12" t="inlineStr">
+        <is>
+          <t>SA-74</t>
+        </is>
+      </c>
+      <c r="B200" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="C200" s="13" t="inlineStr">
+        <is>
+          <t>Tier 2 (Workflow &amp; Ergonomics)</t>
+        </is>
+      </c>
+      <c r="D200" s="13" t="inlineStr">
+        <is>
+          <t>TV Page Always Up to Date</t>
+        </is>
+      </c>
+      <c r="E200" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="F200" s="13" t="inlineStr">
+        <is>
+          <t>Open the TV Monitor in the app and the stand-alone TV page; after an update reload them normally (F5) and check that slide 2 carry-over list scrolls by itself</t>
+        </is>
+      </c>
+      <c r="G200" s="13" t="inlineStr">
+        <is>
+          <t>Both load the newest TV page on a normal reload; tv.html and index.html are served with Cache-Control: no-cache; long lists auto-scroll</t>
+        </is>
+      </c>
+      <c r="H200" s="14" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="I200" s="13" t="inlineStr">
+        <is>
+          <t>Verified by Automated Unit Tests (186 passing in tests/frontend/sla_and_logic.test.js AUT-FRONT-157), XAMPP header check and headless Chrome</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:I199"/>
+  <autoFilter ref="A4:I200"/>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="H5:H199">
+  <conditionalFormatting sqref="H5:H200">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$H5="Passed"</formula>
     </cfRule>
@@ -9914,13 +9961,13 @@
       <formula>$H5="Pending"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A5:A199">
+  <conditionalFormatting sqref="A5:A200">
     <cfRule type="expression" priority="6" dxfId="3">
-      <formula>COUNTIF($A$5:$A$199,$A5)&gt;1</formula>
+      <formula>COUNTIF($A$5:$A$200,$A5)&gt;1</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H5:H199" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H5:H200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pending,Passed,Failed"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
fix(REV-199): Excel claim stub plate/model and contact match the PDF
The export also wrote 'plate / model' into the template's empty gap cell I70 (Excel cut it off at J70, showing 'ABC-') and the contact again into I71. Those two writes are removed; H70 plate, J70 model, H71 contact and H72 claim stub are unchanged. AUT-FRONT-89 updated accordingly.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
+++ b/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
@@ -11,7 +11,7 @@
     <sheet name="QA Checklist" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$200</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$201</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'QA Checklist'!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTA('QA Checklist'!$A$5:$A$200)</f>
+        <f>COUNTA('QA Checklist'!$A$5:$A$201)</f>
         <v/>
       </c>
     </row>
@@ -594,7 +594,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$200,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$200,"Pass")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$201,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$201,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$200,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$200,"Fail")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$201,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$201,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -616,7 +616,7 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$200,"Pending")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$201,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -671,19 +671,19 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$200,$A12)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$201,$A12)</f>
         <v/>
       </c>
       <c r="C12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$200,$A12,'QA Checklist'!$H$5:$H$200,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$200,$A12,'QA Checklist'!$H$5:$H$200,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$201,$A12,'QA Checklist'!$H$5:$H$201,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$201,$A12,'QA Checklist'!$H$5:$H$201,"Pass")</f>
         <v/>
       </c>
       <c r="D12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$200,$A12,'QA Checklist'!$H$5:$H$200,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$200,$A12,'QA Checklist'!$H$5:$H$200,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$201,$A12,'QA Checklist'!$H$5:$H$201,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$201,$A12,'QA Checklist'!$H$5:$H$201,"Fail")</f>
         <v/>
       </c>
       <c r="E12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$200,$A12,'QA Checklist'!$H$5:$H$200,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$201,$A12,'QA Checklist'!$H$5:$H$201,"Pending")</f>
         <v/>
       </c>
       <c r="F12" s="8">
@@ -698,19 +698,19 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$200,$A13)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$201,$A13)</f>
         <v/>
       </c>
       <c r="C13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$200,$A13,'QA Checklist'!$H$5:$H$200,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$200,$A13,'QA Checklist'!$H$5:$H$200,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$201,$A13,'QA Checklist'!$H$5:$H$201,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$201,$A13,'QA Checklist'!$H$5:$H$201,"Pass")</f>
         <v/>
       </c>
       <c r="D13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$200,$A13,'QA Checklist'!$H$5:$H$200,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$200,$A13,'QA Checklist'!$H$5:$H$200,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$201,$A13,'QA Checklist'!$H$5:$H$201,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$201,$A13,'QA Checklist'!$H$5:$H$201,"Fail")</f>
         <v/>
       </c>
       <c r="E13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$200,$A13,'QA Checklist'!$H$5:$H$200,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$201,$A13,'QA Checklist'!$H$5:$H$201,"Pending")</f>
         <v/>
       </c>
       <c r="F13" s="8">
@@ -725,19 +725,19 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$200,$A14)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$201,$A14)</f>
         <v/>
       </c>
       <c r="C14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$200,$A14,'QA Checklist'!$H$5:$H$200,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$200,$A14,'QA Checklist'!$H$5:$H$200,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$201,$A14,'QA Checklist'!$H$5:$H$201,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$201,$A14,'QA Checklist'!$H$5:$H$201,"Pass")</f>
         <v/>
       </c>
       <c r="D14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$200,$A14,'QA Checklist'!$H$5:$H$200,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$200,$A14,'QA Checklist'!$H$5:$H$200,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$201,$A14,'QA Checklist'!$H$5:$H$201,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$201,$A14,'QA Checklist'!$H$5:$H$201,"Fail")</f>
         <v/>
       </c>
       <c r="E14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$200,$A14,'QA Checklist'!$H$5:$H$200,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$201,$A14,'QA Checklist'!$H$5:$H$201,"Pending")</f>
         <v/>
       </c>
       <c r="F14" s="8">
@@ -752,19 +752,19 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$200,$A15)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$201,$A15)</f>
         <v/>
       </c>
       <c r="C15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$200,$A15,'QA Checklist'!$H$5:$H$200,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$200,$A15,'QA Checklist'!$H$5:$H$200,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$201,$A15,'QA Checklist'!$H$5:$H$201,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$201,$A15,'QA Checklist'!$H$5:$H$201,"Pass")</f>
         <v/>
       </c>
       <c r="D15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$200,$A15,'QA Checklist'!$H$5:$H$200,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$200,$A15,'QA Checklist'!$H$5:$H$200,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$201,$A15,'QA Checklist'!$H$5:$H$201,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$201,$A15,'QA Checklist'!$H$5:$H$201,"Fail")</f>
         <v/>
       </c>
       <c r="E15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$200,$A15,'QA Checklist'!$H$5:$H$200,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$201,$A15,'QA Checklist'!$H$5:$H$201,"Pending")</f>
         <v/>
       </c>
       <c r="F15" s="8">
@@ -779,19 +779,19 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$200,$A16)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$201,$A16)</f>
         <v/>
       </c>
       <c r="C16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$200,$A16,'QA Checklist'!$H$5:$H$200,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$200,$A16,'QA Checklist'!$H$5:$H$200,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$201,$A16,'QA Checklist'!$H$5:$H$201,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$201,$A16,'QA Checklist'!$H$5:$H$201,"Pass")</f>
         <v/>
       </c>
       <c r="D16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$200,$A16,'QA Checklist'!$H$5:$H$200,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$200,$A16,'QA Checklist'!$H$5:$H$200,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$201,$A16,'QA Checklist'!$H$5:$H$201,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$201,$A16,'QA Checklist'!$H$5:$H$201,"Fail")</f>
         <v/>
       </c>
       <c r="E16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$200,$A16,'QA Checklist'!$H$5:$H$200,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$201,$A16,'QA Checklist'!$H$5:$H$201,"Pending")</f>
         <v/>
       </c>
       <c r="F16" s="8">
@@ -806,19 +806,19 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$200,$A17)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$201,$A17)</f>
         <v/>
       </c>
       <c r="C17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$200,$A17,'QA Checklist'!$H$5:$H$200,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$200,$A17,'QA Checklist'!$H$5:$H$200,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$201,$A17,'QA Checklist'!$H$5:$H$201,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$201,$A17,'QA Checklist'!$H$5:$H$201,"Pass")</f>
         <v/>
       </c>
       <c r="D17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$200,$A17,'QA Checklist'!$H$5:$H$200,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$200,$A17,'QA Checklist'!$H$5:$H$200,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$201,$A17,'QA Checklist'!$H$5:$H$201,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$201,$A17,'QA Checklist'!$H$5:$H$201,"Fail")</f>
         <v/>
       </c>
       <c r="E17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$200,$A17,'QA Checklist'!$H$5:$H$200,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$201,$A17,'QA Checklist'!$H$5:$H$201,"Pending")</f>
         <v/>
       </c>
       <c r="F17" s="8">
@@ -833,19 +833,19 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$200,$A18)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$201,$A18)</f>
         <v/>
       </c>
       <c r="C18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$200,$A18,'QA Checklist'!$H$5:$H$200,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$200,$A18,'QA Checklist'!$H$5:$H$200,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$201,$A18,'QA Checklist'!$H$5:$H$201,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$201,$A18,'QA Checklist'!$H$5:$H$201,"Pass")</f>
         <v/>
       </c>
       <c r="D18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$200,$A18,'QA Checklist'!$H$5:$H$200,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$200,$A18,'QA Checklist'!$H$5:$H$200,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$201,$A18,'QA Checklist'!$H$5:$H$201,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$201,$A18,'QA Checklist'!$H$5:$H$201,"Fail")</f>
         <v/>
       </c>
       <c r="E18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$200,$A18,'QA Checklist'!$H$5:$H$200,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$201,$A18,'QA Checklist'!$H$5:$H$201,"Pending")</f>
         <v/>
       </c>
       <c r="F18" s="8">
@@ -860,19 +860,19 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$200,$A19)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$201,$A19)</f>
         <v/>
       </c>
       <c r="C19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$200,$A19,'QA Checklist'!$H$5:$H$200,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$200,$A19,'QA Checklist'!$H$5:$H$200,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$201,$A19,'QA Checklist'!$H$5:$H$201,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$201,$A19,'QA Checklist'!$H$5:$H$201,"Pass")</f>
         <v/>
       </c>
       <c r="D19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$200,$A19,'QA Checklist'!$H$5:$H$200,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$200,$A19,'QA Checklist'!$H$5:$H$200,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$201,$A19,'QA Checklist'!$H$5:$H$201,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$201,$A19,'QA Checklist'!$H$5:$H$201,"Fail")</f>
         <v/>
       </c>
       <c r="E19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$200,$A19,'QA Checklist'!$H$5:$H$200,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$201,$A19,'QA Checklist'!$H$5:$H$201,"Pending")</f>
         <v/>
       </c>
       <c r="F19" s="8">
@@ -887,19 +887,19 @@
         </is>
       </c>
       <c r="B20" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$200,$A20)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$201,$A20)</f>
         <v/>
       </c>
       <c r="C20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$200,$A20,'QA Checklist'!$H$5:$H$200,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$200,$A20,'QA Checklist'!$H$5:$H$200,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$201,$A20,'QA Checklist'!$H$5:$H$201,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$201,$A20,'QA Checklist'!$H$5:$H$201,"Pass")</f>
         <v/>
       </c>
       <c r="D20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$200,$A20,'QA Checklist'!$H$5:$H$200,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$200,$A20,'QA Checklist'!$H$5:$H$200,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$201,$A20,'QA Checklist'!$H$5:$H$201,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$201,$A20,'QA Checklist'!$H$5:$H$201,"Fail")</f>
         <v/>
       </c>
       <c r="E20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$200,$A20,'QA Checklist'!$H$5:$H$200,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$201,$A20,'QA Checklist'!$H$5:$H$201,"Pending")</f>
         <v/>
       </c>
       <c r="F20" s="8">
@@ -914,19 +914,19 @@
         </is>
       </c>
       <c r="B21" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$200,$A21)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$201,$A21)</f>
         <v/>
       </c>
       <c r="C21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$200,$A21,'QA Checklist'!$H$5:$H$200,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$200,$A21,'QA Checklist'!$H$5:$H$200,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$201,$A21,'QA Checklist'!$H$5:$H$201,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$201,$A21,'QA Checklist'!$H$5:$H$201,"Pass")</f>
         <v/>
       </c>
       <c r="D21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$200,$A21,'QA Checklist'!$H$5:$H$200,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$200,$A21,'QA Checklist'!$H$5:$H$200,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$201,$A21,'QA Checklist'!$H$5:$H$201,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$201,$A21,'QA Checklist'!$H$5:$H$201,"Fail")</f>
         <v/>
       </c>
       <c r="E21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$200,$A21,'QA Checklist'!$H$5:$H$200,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$201,$A21,'QA Checklist'!$H$5:$H$201,"Pending")</f>
         <v/>
       </c>
       <c r="F21" s="8">
@@ -941,19 +941,19 @@
         </is>
       </c>
       <c r="B22" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$200,$A22)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$201,$A22)</f>
         <v/>
       </c>
       <c r="C22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$200,$A22,'QA Checklist'!$H$5:$H$200,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$200,$A22,'QA Checklist'!$H$5:$H$200,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$201,$A22,'QA Checklist'!$H$5:$H$201,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$201,$A22,'QA Checklist'!$H$5:$H$201,"Pass")</f>
         <v/>
       </c>
       <c r="D22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$200,$A22,'QA Checklist'!$H$5:$H$200,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$200,$A22,'QA Checklist'!$H$5:$H$200,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$201,$A22,'QA Checklist'!$H$5:$H$201,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$201,$A22,'QA Checklist'!$H$5:$H$201,"Fail")</f>
         <v/>
       </c>
       <c r="E22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$200,$A22,'QA Checklist'!$H$5:$H$200,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$201,$A22,'QA Checklist'!$H$5:$H$201,"Pending")</f>
         <v/>
       </c>
       <c r="F22" s="8">
@@ -1023,19 +1023,19 @@
         </is>
       </c>
       <c r="B26" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$200,$A26&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$201,$A26&amp;"*")</f>
         <v/>
       </c>
       <c r="C26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$200,$A26&amp;"*",'QA Checklist'!$H$5:$H$200,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$200,$A26&amp;"*",'QA Checklist'!$H$5:$H$200,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$201,$A26&amp;"*",'QA Checklist'!$H$5:$H$201,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$201,$A26&amp;"*",'QA Checklist'!$H$5:$H$201,"Pass")</f>
         <v/>
       </c>
       <c r="D26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$200,$A26&amp;"*",'QA Checklist'!$H$5:$H$200,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$200,$A26&amp;"*",'QA Checklist'!$H$5:$H$200,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$201,$A26&amp;"*",'QA Checklist'!$H$5:$H$201,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$201,$A26&amp;"*",'QA Checklist'!$H$5:$H$201,"Fail")</f>
         <v/>
       </c>
       <c r="E26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$200,$A26&amp;"*",'QA Checklist'!$H$5:$H$200,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$201,$A26&amp;"*",'QA Checklist'!$H$5:$H$201,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1046,19 +1046,19 @@
         </is>
       </c>
       <c r="B27" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$200,$A27&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$201,$A27&amp;"*")</f>
         <v/>
       </c>
       <c r="C27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$200,$A27&amp;"*",'QA Checklist'!$H$5:$H$200,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$200,$A27&amp;"*",'QA Checklist'!$H$5:$H$200,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$201,$A27&amp;"*",'QA Checklist'!$H$5:$H$201,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$201,$A27&amp;"*",'QA Checklist'!$H$5:$H$201,"Pass")</f>
         <v/>
       </c>
       <c r="D27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$200,$A27&amp;"*",'QA Checklist'!$H$5:$H$200,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$200,$A27&amp;"*",'QA Checklist'!$H$5:$H$200,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$201,$A27&amp;"*",'QA Checklist'!$H$5:$H$201,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$201,$A27&amp;"*",'QA Checklist'!$H$5:$H$201,"Fail")</f>
         <v/>
       </c>
       <c r="E27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$200,$A27&amp;"*",'QA Checklist'!$H$5:$H$200,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$201,$A27&amp;"*",'QA Checklist'!$H$5:$H$201,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1069,19 +1069,19 @@
         </is>
       </c>
       <c r="B28" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$200,$A28&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$201,$A28&amp;"*")</f>
         <v/>
       </c>
       <c r="C28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$200,$A28&amp;"*",'QA Checklist'!$H$5:$H$200,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$200,$A28&amp;"*",'QA Checklist'!$H$5:$H$200,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$201,$A28&amp;"*",'QA Checklist'!$H$5:$H$201,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$201,$A28&amp;"*",'QA Checklist'!$H$5:$H$201,"Pass")</f>
         <v/>
       </c>
       <c r="D28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$200,$A28&amp;"*",'QA Checklist'!$H$5:$H$200,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$200,$A28&amp;"*",'QA Checklist'!$H$5:$H$200,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$201,$A28&amp;"*",'QA Checklist'!$H$5:$H$201,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$201,$A28&amp;"*",'QA Checklist'!$H$5:$H$201,"Fail")</f>
         <v/>
       </c>
       <c r="E28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$200,$A28&amp;"*",'QA Checklist'!$H$5:$H$200,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$201,$A28&amp;"*",'QA Checklist'!$H$5:$H$201,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1096,7 +1096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I200"/>
+  <dimension ref="A1:I201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9939,12 +9939,59 @@
         </is>
       </c>
     </row>
+    <row r="201">
+      <c r="A201" s="12" t="inlineStr">
+        <is>
+          <t>SA-75</t>
+        </is>
+      </c>
+      <c r="B201" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="C201" s="13" t="inlineStr">
+        <is>
+          <t>Tier 2 (Workflow &amp; Ergonomics)</t>
+        </is>
+      </c>
+      <c r="D201" s="13" t="inlineStr">
+        <is>
+          <t>Excel Claim Stub Rows</t>
+        </is>
+      </c>
+      <c r="E201" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="F201" s="13" t="inlineStr">
+        <is>
+          <t>Fill plate, model and contact in the Studio, press Export Official .xlsx and open the Job_Order sheet at the claim stub (rows 70-72); compare with the PDF</t>
+        </is>
+      </c>
+      <c r="G201" s="13" t="inlineStr">
+        <is>
+          <t>Plate No./Year/Model shows the plate and the model once each; Contact shows the number once; the Claim Stub is filled; same as the PDF</t>
+        </is>
+      </c>
+      <c r="H201" s="14" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="I201" s="13" t="inlineStr">
+        <is>
+          <t>Verified by Automated Unit Tests (187 passing in tests/frontend/sla_and_logic.test.js AUT-FRONT-158) and headless Chrome 3/3 on a real exported file</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:I200"/>
+  <autoFilter ref="A4:I201"/>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="H5:H200">
+  <conditionalFormatting sqref="H5:H201">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$H5="Passed"</formula>
     </cfRule>
@@ -9961,13 +10008,13 @@
       <formula>$H5="Pending"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A5:A200">
+  <conditionalFormatting sqref="A5:A201">
     <cfRule type="expression" priority="6" dxfId="3">
-      <formula>COUNTIF($A$5:$A$200,$A5)&gt;1</formula>
+      <formula>COUNTIF($A$5:$A$201,$A5)&gt;1</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H5:H200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H5:H201" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pending,Passed,Failed"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat(REV-200): remove the parts & materials editor from the Job Order tab
The SA has no authority over parts and materials. Removed the Parts / Materials repeater cards, presets and total banner, the sample and preset parts, and the Job Order -> Quotation/Billing item overwrite (Quotation and Billing now keep their own items; header fields still copy). Old draft parts are ignored; the Job Order PDF and Excel keep the parts area blank.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
+++ b/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
@@ -11,7 +11,7 @@
     <sheet name="QA Checklist" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$201</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$202</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'QA Checklist'!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTA('QA Checklist'!$A$5:$A$201)</f>
+        <f>COUNTA('QA Checklist'!$A$5:$A$202)</f>
         <v/>
       </c>
     </row>
@@ -594,7 +594,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$201,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$201,"Pass")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$202,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$202,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$201,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$201,"Fail")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$202,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$202,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -616,7 +616,7 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$201,"Pending")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$202,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -671,19 +671,19 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$201,$A12)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$202,$A12)</f>
         <v/>
       </c>
       <c r="C12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$201,$A12,'QA Checklist'!$H$5:$H$201,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$201,$A12,'QA Checklist'!$H$5:$H$201,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$202,$A12,'QA Checklist'!$H$5:$H$202,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$202,$A12,'QA Checklist'!$H$5:$H$202,"Pass")</f>
         <v/>
       </c>
       <c r="D12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$201,$A12,'QA Checklist'!$H$5:$H$201,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$201,$A12,'QA Checklist'!$H$5:$H$201,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$202,$A12,'QA Checklist'!$H$5:$H$202,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$202,$A12,'QA Checklist'!$H$5:$H$202,"Fail")</f>
         <v/>
       </c>
       <c r="E12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$201,$A12,'QA Checklist'!$H$5:$H$201,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$202,$A12,'QA Checklist'!$H$5:$H$202,"Pending")</f>
         <v/>
       </c>
       <c r="F12" s="8">
@@ -698,19 +698,19 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$201,$A13)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$202,$A13)</f>
         <v/>
       </c>
       <c r="C13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$201,$A13,'QA Checklist'!$H$5:$H$201,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$201,$A13,'QA Checklist'!$H$5:$H$201,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$202,$A13,'QA Checklist'!$H$5:$H$202,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$202,$A13,'QA Checklist'!$H$5:$H$202,"Pass")</f>
         <v/>
       </c>
       <c r="D13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$201,$A13,'QA Checklist'!$H$5:$H$201,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$201,$A13,'QA Checklist'!$H$5:$H$201,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$202,$A13,'QA Checklist'!$H$5:$H$202,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$202,$A13,'QA Checklist'!$H$5:$H$202,"Fail")</f>
         <v/>
       </c>
       <c r="E13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$201,$A13,'QA Checklist'!$H$5:$H$201,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$202,$A13,'QA Checklist'!$H$5:$H$202,"Pending")</f>
         <v/>
       </c>
       <c r="F13" s="8">
@@ -725,19 +725,19 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$201,$A14)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$202,$A14)</f>
         <v/>
       </c>
       <c r="C14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$201,$A14,'QA Checklist'!$H$5:$H$201,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$201,$A14,'QA Checklist'!$H$5:$H$201,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$202,$A14,'QA Checklist'!$H$5:$H$202,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$202,$A14,'QA Checklist'!$H$5:$H$202,"Pass")</f>
         <v/>
       </c>
       <c r="D14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$201,$A14,'QA Checklist'!$H$5:$H$201,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$201,$A14,'QA Checklist'!$H$5:$H$201,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$202,$A14,'QA Checklist'!$H$5:$H$202,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$202,$A14,'QA Checklist'!$H$5:$H$202,"Fail")</f>
         <v/>
       </c>
       <c r="E14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$201,$A14,'QA Checklist'!$H$5:$H$201,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$202,$A14,'QA Checklist'!$H$5:$H$202,"Pending")</f>
         <v/>
       </c>
       <c r="F14" s="8">
@@ -752,19 +752,19 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$201,$A15)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$202,$A15)</f>
         <v/>
       </c>
       <c r="C15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$201,$A15,'QA Checklist'!$H$5:$H$201,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$201,$A15,'QA Checklist'!$H$5:$H$201,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$202,$A15,'QA Checklist'!$H$5:$H$202,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$202,$A15,'QA Checklist'!$H$5:$H$202,"Pass")</f>
         <v/>
       </c>
       <c r="D15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$201,$A15,'QA Checklist'!$H$5:$H$201,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$201,$A15,'QA Checklist'!$H$5:$H$201,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$202,$A15,'QA Checklist'!$H$5:$H$202,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$202,$A15,'QA Checklist'!$H$5:$H$202,"Fail")</f>
         <v/>
       </c>
       <c r="E15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$201,$A15,'QA Checklist'!$H$5:$H$201,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$202,$A15,'QA Checklist'!$H$5:$H$202,"Pending")</f>
         <v/>
       </c>
       <c r="F15" s="8">
@@ -779,19 +779,19 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$201,$A16)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$202,$A16)</f>
         <v/>
       </c>
       <c r="C16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$201,$A16,'QA Checklist'!$H$5:$H$201,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$201,$A16,'QA Checklist'!$H$5:$H$201,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$202,$A16,'QA Checklist'!$H$5:$H$202,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$202,$A16,'QA Checklist'!$H$5:$H$202,"Pass")</f>
         <v/>
       </c>
       <c r="D16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$201,$A16,'QA Checklist'!$H$5:$H$201,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$201,$A16,'QA Checklist'!$H$5:$H$201,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$202,$A16,'QA Checklist'!$H$5:$H$202,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$202,$A16,'QA Checklist'!$H$5:$H$202,"Fail")</f>
         <v/>
       </c>
       <c r="E16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$201,$A16,'QA Checklist'!$H$5:$H$201,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$202,$A16,'QA Checklist'!$H$5:$H$202,"Pending")</f>
         <v/>
       </c>
       <c r="F16" s="8">
@@ -806,19 +806,19 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$201,$A17)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$202,$A17)</f>
         <v/>
       </c>
       <c r="C17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$201,$A17,'QA Checklist'!$H$5:$H$201,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$201,$A17,'QA Checklist'!$H$5:$H$201,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$202,$A17,'QA Checklist'!$H$5:$H$202,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$202,$A17,'QA Checklist'!$H$5:$H$202,"Pass")</f>
         <v/>
       </c>
       <c r="D17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$201,$A17,'QA Checklist'!$H$5:$H$201,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$201,$A17,'QA Checklist'!$H$5:$H$201,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$202,$A17,'QA Checklist'!$H$5:$H$202,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$202,$A17,'QA Checklist'!$H$5:$H$202,"Fail")</f>
         <v/>
       </c>
       <c r="E17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$201,$A17,'QA Checklist'!$H$5:$H$201,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$202,$A17,'QA Checklist'!$H$5:$H$202,"Pending")</f>
         <v/>
       </c>
       <c r="F17" s="8">
@@ -833,19 +833,19 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$201,$A18)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$202,$A18)</f>
         <v/>
       </c>
       <c r="C18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$201,$A18,'QA Checklist'!$H$5:$H$201,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$201,$A18,'QA Checklist'!$H$5:$H$201,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$202,$A18,'QA Checklist'!$H$5:$H$202,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$202,$A18,'QA Checklist'!$H$5:$H$202,"Pass")</f>
         <v/>
       </c>
       <c r="D18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$201,$A18,'QA Checklist'!$H$5:$H$201,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$201,$A18,'QA Checklist'!$H$5:$H$201,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$202,$A18,'QA Checklist'!$H$5:$H$202,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$202,$A18,'QA Checklist'!$H$5:$H$202,"Fail")</f>
         <v/>
       </c>
       <c r="E18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$201,$A18,'QA Checklist'!$H$5:$H$201,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$202,$A18,'QA Checklist'!$H$5:$H$202,"Pending")</f>
         <v/>
       </c>
       <c r="F18" s="8">
@@ -860,19 +860,19 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$201,$A19)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$202,$A19)</f>
         <v/>
       </c>
       <c r="C19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$201,$A19,'QA Checklist'!$H$5:$H$201,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$201,$A19,'QA Checklist'!$H$5:$H$201,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$202,$A19,'QA Checklist'!$H$5:$H$202,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$202,$A19,'QA Checklist'!$H$5:$H$202,"Pass")</f>
         <v/>
       </c>
       <c r="D19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$201,$A19,'QA Checklist'!$H$5:$H$201,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$201,$A19,'QA Checklist'!$H$5:$H$201,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$202,$A19,'QA Checklist'!$H$5:$H$202,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$202,$A19,'QA Checklist'!$H$5:$H$202,"Fail")</f>
         <v/>
       </c>
       <c r="E19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$201,$A19,'QA Checklist'!$H$5:$H$201,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$202,$A19,'QA Checklist'!$H$5:$H$202,"Pending")</f>
         <v/>
       </c>
       <c r="F19" s="8">
@@ -887,19 +887,19 @@
         </is>
       </c>
       <c r="B20" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$201,$A20)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$202,$A20)</f>
         <v/>
       </c>
       <c r="C20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$201,$A20,'QA Checklist'!$H$5:$H$201,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$201,$A20,'QA Checklist'!$H$5:$H$201,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$202,$A20,'QA Checklist'!$H$5:$H$202,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$202,$A20,'QA Checklist'!$H$5:$H$202,"Pass")</f>
         <v/>
       </c>
       <c r="D20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$201,$A20,'QA Checklist'!$H$5:$H$201,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$201,$A20,'QA Checklist'!$H$5:$H$201,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$202,$A20,'QA Checklist'!$H$5:$H$202,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$202,$A20,'QA Checklist'!$H$5:$H$202,"Fail")</f>
         <v/>
       </c>
       <c r="E20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$201,$A20,'QA Checklist'!$H$5:$H$201,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$202,$A20,'QA Checklist'!$H$5:$H$202,"Pending")</f>
         <v/>
       </c>
       <c r="F20" s="8">
@@ -914,19 +914,19 @@
         </is>
       </c>
       <c r="B21" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$201,$A21)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$202,$A21)</f>
         <v/>
       </c>
       <c r="C21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$201,$A21,'QA Checklist'!$H$5:$H$201,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$201,$A21,'QA Checklist'!$H$5:$H$201,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$202,$A21,'QA Checklist'!$H$5:$H$202,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$202,$A21,'QA Checklist'!$H$5:$H$202,"Pass")</f>
         <v/>
       </c>
       <c r="D21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$201,$A21,'QA Checklist'!$H$5:$H$201,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$201,$A21,'QA Checklist'!$H$5:$H$201,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$202,$A21,'QA Checklist'!$H$5:$H$202,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$202,$A21,'QA Checklist'!$H$5:$H$202,"Fail")</f>
         <v/>
       </c>
       <c r="E21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$201,$A21,'QA Checklist'!$H$5:$H$201,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$202,$A21,'QA Checklist'!$H$5:$H$202,"Pending")</f>
         <v/>
       </c>
       <c r="F21" s="8">
@@ -941,19 +941,19 @@
         </is>
       </c>
       <c r="B22" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$201,$A22)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$202,$A22)</f>
         <v/>
       </c>
       <c r="C22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$201,$A22,'QA Checklist'!$H$5:$H$201,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$201,$A22,'QA Checklist'!$H$5:$H$201,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$202,$A22,'QA Checklist'!$H$5:$H$202,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$202,$A22,'QA Checklist'!$H$5:$H$202,"Pass")</f>
         <v/>
       </c>
       <c r="D22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$201,$A22,'QA Checklist'!$H$5:$H$201,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$201,$A22,'QA Checklist'!$H$5:$H$201,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$202,$A22,'QA Checklist'!$H$5:$H$202,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$202,$A22,'QA Checklist'!$H$5:$H$202,"Fail")</f>
         <v/>
       </c>
       <c r="E22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$201,$A22,'QA Checklist'!$H$5:$H$201,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$202,$A22,'QA Checklist'!$H$5:$H$202,"Pending")</f>
         <v/>
       </c>
       <c r="F22" s="8">
@@ -1023,19 +1023,19 @@
         </is>
       </c>
       <c r="B26" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$201,$A26&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$202,$A26&amp;"*")</f>
         <v/>
       </c>
       <c r="C26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$201,$A26&amp;"*",'QA Checklist'!$H$5:$H$201,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$201,$A26&amp;"*",'QA Checklist'!$H$5:$H$201,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$202,$A26&amp;"*",'QA Checklist'!$H$5:$H$202,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$202,$A26&amp;"*",'QA Checklist'!$H$5:$H$202,"Pass")</f>
         <v/>
       </c>
       <c r="D26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$201,$A26&amp;"*",'QA Checklist'!$H$5:$H$201,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$201,$A26&amp;"*",'QA Checklist'!$H$5:$H$201,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$202,$A26&amp;"*",'QA Checklist'!$H$5:$H$202,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$202,$A26&amp;"*",'QA Checklist'!$H$5:$H$202,"Fail")</f>
         <v/>
       </c>
       <c r="E26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$201,$A26&amp;"*",'QA Checklist'!$H$5:$H$201,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$202,$A26&amp;"*",'QA Checklist'!$H$5:$H$202,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1046,19 +1046,19 @@
         </is>
       </c>
       <c r="B27" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$201,$A27&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$202,$A27&amp;"*")</f>
         <v/>
       </c>
       <c r="C27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$201,$A27&amp;"*",'QA Checklist'!$H$5:$H$201,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$201,$A27&amp;"*",'QA Checklist'!$H$5:$H$201,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$202,$A27&amp;"*",'QA Checklist'!$H$5:$H$202,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$202,$A27&amp;"*",'QA Checklist'!$H$5:$H$202,"Pass")</f>
         <v/>
       </c>
       <c r="D27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$201,$A27&amp;"*",'QA Checklist'!$H$5:$H$201,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$201,$A27&amp;"*",'QA Checklist'!$H$5:$H$201,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$202,$A27&amp;"*",'QA Checklist'!$H$5:$H$202,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$202,$A27&amp;"*",'QA Checklist'!$H$5:$H$202,"Fail")</f>
         <v/>
       </c>
       <c r="E27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$201,$A27&amp;"*",'QA Checklist'!$H$5:$H$201,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$202,$A27&amp;"*",'QA Checklist'!$H$5:$H$202,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1069,19 +1069,19 @@
         </is>
       </c>
       <c r="B28" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$201,$A28&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$202,$A28&amp;"*")</f>
         <v/>
       </c>
       <c r="C28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$201,$A28&amp;"*",'QA Checklist'!$H$5:$H$201,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$201,$A28&amp;"*",'QA Checklist'!$H$5:$H$201,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$202,$A28&amp;"*",'QA Checklist'!$H$5:$H$202,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$202,$A28&amp;"*",'QA Checklist'!$H$5:$H$202,"Pass")</f>
         <v/>
       </c>
       <c r="D28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$201,$A28&amp;"*",'QA Checklist'!$H$5:$H$201,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$201,$A28&amp;"*",'QA Checklist'!$H$5:$H$201,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$202,$A28&amp;"*",'QA Checklist'!$H$5:$H$202,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$202,$A28&amp;"*",'QA Checklist'!$H$5:$H$202,"Fail")</f>
         <v/>
       </c>
       <c r="E28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$201,$A28&amp;"*",'QA Checklist'!$H$5:$H$201,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$202,$A28&amp;"*",'QA Checklist'!$H$5:$H$202,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1096,7 +1096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I201"/>
+  <dimension ref="A1:I202"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9986,12 +9986,59 @@
         </is>
       </c>
     </row>
+    <row r="202">
+      <c r="A202" s="12" t="inlineStr">
+        <is>
+          <t>SA-76</t>
+        </is>
+      </c>
+      <c r="B202" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="C202" s="13" t="inlineStr">
+        <is>
+          <t>Tier 2 (Workflow &amp; Ergonomics)</t>
+        </is>
+      </c>
+      <c r="D202" s="13" t="inlineStr">
+        <is>
+          <t>Job Order Without Parts &amp; Materials Editor</t>
+        </is>
+      </c>
+      <c r="E202" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="F202" s="13" t="inlineStr">
+        <is>
+          <t>Open the Job Order tab; add an item on Quotation and on Billing; type in the Job Order and switch between the tabs; view the Job Order PDF and export the Excel</t>
+        </is>
+      </c>
+      <c r="G202" s="13" t="inlineStr">
+        <is>
+          <t>No parts/materials tables or totals on the Job Order; Quotation and Billing items stay; the customer name still copies; the Job Order PDF and Excel have a blank parts/materials area</t>
+        </is>
+      </c>
+      <c r="H202" s="14" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="I202" s="13" t="inlineStr">
+        <is>
+          <t>Verified by Automated Unit Tests (188 passing in tests/frontend/sla_and_logic.test.js AUT-FRONT-159) and headless Chrome 8/8</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:I201"/>
+  <autoFilter ref="A4:I202"/>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="H5:H201">
+  <conditionalFormatting sqref="H5:H202">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$H5="Passed"</formula>
     </cfRule>
@@ -10008,13 +10055,13 @@
       <formula>$H5="Pending"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A5:A201">
+  <conditionalFormatting sqref="A5:A202">
     <cfRule type="expression" priority="6" dxfId="3">
-      <formula>COUNTIF($A$5:$A$201,$A5)&gt;1</formula>
+      <formula>COUNTIF($A$5:$A$202,$A5)&gt;1</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H5:H201" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H5:H202" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pending,Passed,Failed"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat(REV-201): four lanes and a 2-hour Express limit
Lane lists now offer Flexible, Express Lane (2 Hours), PMS & GRS Lane and Priority Lane everywhere. PMS & GRS is kept as its own lane (both normalizers used to turn it into Flexible); retired Special / Regular lanes read as Flexible. The Express SLA is 120 minutes in the goal status, SLA badge and delay report, and all Express text says 2 hours. TV slide 3 shows Express, Flexible, PMS & GRS and Priority columns.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
+++ b/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
@@ -11,7 +11,7 @@
     <sheet name="QA Checklist" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$202</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$203</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'QA Checklist'!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTA('QA Checklist'!$A$5:$A$202)</f>
+        <f>COUNTA('QA Checklist'!$A$5:$A$203)</f>
         <v/>
       </c>
     </row>
@@ -594,7 +594,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$202,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$202,"Pass")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$203,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$203,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$202,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$202,"Fail")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$203,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$203,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -616,7 +616,7 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$202,"Pending")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$203,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -671,19 +671,19 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$202,$A12)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$203,$A12)</f>
         <v/>
       </c>
       <c r="C12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$202,$A12,'QA Checklist'!$H$5:$H$202,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$202,$A12,'QA Checklist'!$H$5:$H$202,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$203,$A12,'QA Checklist'!$H$5:$H$203,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$203,$A12,'QA Checklist'!$H$5:$H$203,"Pass")</f>
         <v/>
       </c>
       <c r="D12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$202,$A12,'QA Checklist'!$H$5:$H$202,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$202,$A12,'QA Checklist'!$H$5:$H$202,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$203,$A12,'QA Checklist'!$H$5:$H$203,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$203,$A12,'QA Checklist'!$H$5:$H$203,"Fail")</f>
         <v/>
       </c>
       <c r="E12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$202,$A12,'QA Checklist'!$H$5:$H$202,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$203,$A12,'QA Checklist'!$H$5:$H$203,"Pending")</f>
         <v/>
       </c>
       <c r="F12" s="8">
@@ -698,19 +698,19 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$202,$A13)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$203,$A13)</f>
         <v/>
       </c>
       <c r="C13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$202,$A13,'QA Checklist'!$H$5:$H$202,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$202,$A13,'QA Checklist'!$H$5:$H$202,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$203,$A13,'QA Checklist'!$H$5:$H$203,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$203,$A13,'QA Checklist'!$H$5:$H$203,"Pass")</f>
         <v/>
       </c>
       <c r="D13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$202,$A13,'QA Checklist'!$H$5:$H$202,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$202,$A13,'QA Checklist'!$H$5:$H$202,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$203,$A13,'QA Checklist'!$H$5:$H$203,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$203,$A13,'QA Checklist'!$H$5:$H$203,"Fail")</f>
         <v/>
       </c>
       <c r="E13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$202,$A13,'QA Checklist'!$H$5:$H$202,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$203,$A13,'QA Checklist'!$H$5:$H$203,"Pending")</f>
         <v/>
       </c>
       <c r="F13" s="8">
@@ -725,19 +725,19 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$202,$A14)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$203,$A14)</f>
         <v/>
       </c>
       <c r="C14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$202,$A14,'QA Checklist'!$H$5:$H$202,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$202,$A14,'QA Checklist'!$H$5:$H$202,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$203,$A14,'QA Checklist'!$H$5:$H$203,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$203,$A14,'QA Checklist'!$H$5:$H$203,"Pass")</f>
         <v/>
       </c>
       <c r="D14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$202,$A14,'QA Checklist'!$H$5:$H$202,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$202,$A14,'QA Checklist'!$H$5:$H$202,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$203,$A14,'QA Checklist'!$H$5:$H$203,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$203,$A14,'QA Checklist'!$H$5:$H$203,"Fail")</f>
         <v/>
       </c>
       <c r="E14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$202,$A14,'QA Checklist'!$H$5:$H$202,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$203,$A14,'QA Checklist'!$H$5:$H$203,"Pending")</f>
         <v/>
       </c>
       <c r="F14" s="8">
@@ -752,19 +752,19 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$202,$A15)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$203,$A15)</f>
         <v/>
       </c>
       <c r="C15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$202,$A15,'QA Checklist'!$H$5:$H$202,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$202,$A15,'QA Checklist'!$H$5:$H$202,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$203,$A15,'QA Checklist'!$H$5:$H$203,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$203,$A15,'QA Checklist'!$H$5:$H$203,"Pass")</f>
         <v/>
       </c>
       <c r="D15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$202,$A15,'QA Checklist'!$H$5:$H$202,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$202,$A15,'QA Checklist'!$H$5:$H$202,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$203,$A15,'QA Checklist'!$H$5:$H$203,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$203,$A15,'QA Checklist'!$H$5:$H$203,"Fail")</f>
         <v/>
       </c>
       <c r="E15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$202,$A15,'QA Checklist'!$H$5:$H$202,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$203,$A15,'QA Checklist'!$H$5:$H$203,"Pending")</f>
         <v/>
       </c>
       <c r="F15" s="8">
@@ -779,19 +779,19 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$202,$A16)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$203,$A16)</f>
         <v/>
       </c>
       <c r="C16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$202,$A16,'QA Checklist'!$H$5:$H$202,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$202,$A16,'QA Checklist'!$H$5:$H$202,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$203,$A16,'QA Checklist'!$H$5:$H$203,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$203,$A16,'QA Checklist'!$H$5:$H$203,"Pass")</f>
         <v/>
       </c>
       <c r="D16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$202,$A16,'QA Checklist'!$H$5:$H$202,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$202,$A16,'QA Checklist'!$H$5:$H$202,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$203,$A16,'QA Checklist'!$H$5:$H$203,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$203,$A16,'QA Checklist'!$H$5:$H$203,"Fail")</f>
         <v/>
       </c>
       <c r="E16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$202,$A16,'QA Checklist'!$H$5:$H$202,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$203,$A16,'QA Checklist'!$H$5:$H$203,"Pending")</f>
         <v/>
       </c>
       <c r="F16" s="8">
@@ -806,19 +806,19 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$202,$A17)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$203,$A17)</f>
         <v/>
       </c>
       <c r="C17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$202,$A17,'QA Checklist'!$H$5:$H$202,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$202,$A17,'QA Checklist'!$H$5:$H$202,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$203,$A17,'QA Checklist'!$H$5:$H$203,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$203,$A17,'QA Checklist'!$H$5:$H$203,"Pass")</f>
         <v/>
       </c>
       <c r="D17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$202,$A17,'QA Checklist'!$H$5:$H$202,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$202,$A17,'QA Checklist'!$H$5:$H$202,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$203,$A17,'QA Checklist'!$H$5:$H$203,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$203,$A17,'QA Checklist'!$H$5:$H$203,"Fail")</f>
         <v/>
       </c>
       <c r="E17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$202,$A17,'QA Checklist'!$H$5:$H$202,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$203,$A17,'QA Checklist'!$H$5:$H$203,"Pending")</f>
         <v/>
       </c>
       <c r="F17" s="8">
@@ -833,19 +833,19 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$202,$A18)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$203,$A18)</f>
         <v/>
       </c>
       <c r="C18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$202,$A18,'QA Checklist'!$H$5:$H$202,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$202,$A18,'QA Checklist'!$H$5:$H$202,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$203,$A18,'QA Checklist'!$H$5:$H$203,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$203,$A18,'QA Checklist'!$H$5:$H$203,"Pass")</f>
         <v/>
       </c>
       <c r="D18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$202,$A18,'QA Checklist'!$H$5:$H$202,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$202,$A18,'QA Checklist'!$H$5:$H$202,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$203,$A18,'QA Checklist'!$H$5:$H$203,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$203,$A18,'QA Checklist'!$H$5:$H$203,"Fail")</f>
         <v/>
       </c>
       <c r="E18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$202,$A18,'QA Checklist'!$H$5:$H$202,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$203,$A18,'QA Checklist'!$H$5:$H$203,"Pending")</f>
         <v/>
       </c>
       <c r="F18" s="8">
@@ -860,19 +860,19 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$202,$A19)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$203,$A19)</f>
         <v/>
       </c>
       <c r="C19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$202,$A19,'QA Checklist'!$H$5:$H$202,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$202,$A19,'QA Checklist'!$H$5:$H$202,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$203,$A19,'QA Checklist'!$H$5:$H$203,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$203,$A19,'QA Checklist'!$H$5:$H$203,"Pass")</f>
         <v/>
       </c>
       <c r="D19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$202,$A19,'QA Checklist'!$H$5:$H$202,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$202,$A19,'QA Checklist'!$H$5:$H$202,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$203,$A19,'QA Checklist'!$H$5:$H$203,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$203,$A19,'QA Checklist'!$H$5:$H$203,"Fail")</f>
         <v/>
       </c>
       <c r="E19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$202,$A19,'QA Checklist'!$H$5:$H$202,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$203,$A19,'QA Checklist'!$H$5:$H$203,"Pending")</f>
         <v/>
       </c>
       <c r="F19" s="8">
@@ -887,19 +887,19 @@
         </is>
       </c>
       <c r="B20" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$202,$A20)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$203,$A20)</f>
         <v/>
       </c>
       <c r="C20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$202,$A20,'QA Checklist'!$H$5:$H$202,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$202,$A20,'QA Checklist'!$H$5:$H$202,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$203,$A20,'QA Checklist'!$H$5:$H$203,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$203,$A20,'QA Checklist'!$H$5:$H$203,"Pass")</f>
         <v/>
       </c>
       <c r="D20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$202,$A20,'QA Checklist'!$H$5:$H$202,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$202,$A20,'QA Checklist'!$H$5:$H$202,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$203,$A20,'QA Checklist'!$H$5:$H$203,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$203,$A20,'QA Checklist'!$H$5:$H$203,"Fail")</f>
         <v/>
       </c>
       <c r="E20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$202,$A20,'QA Checklist'!$H$5:$H$202,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$203,$A20,'QA Checklist'!$H$5:$H$203,"Pending")</f>
         <v/>
       </c>
       <c r="F20" s="8">
@@ -914,19 +914,19 @@
         </is>
       </c>
       <c r="B21" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$202,$A21)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$203,$A21)</f>
         <v/>
       </c>
       <c r="C21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$202,$A21,'QA Checklist'!$H$5:$H$202,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$202,$A21,'QA Checklist'!$H$5:$H$202,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$203,$A21,'QA Checklist'!$H$5:$H$203,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$203,$A21,'QA Checklist'!$H$5:$H$203,"Pass")</f>
         <v/>
       </c>
       <c r="D21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$202,$A21,'QA Checklist'!$H$5:$H$202,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$202,$A21,'QA Checklist'!$H$5:$H$202,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$203,$A21,'QA Checklist'!$H$5:$H$203,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$203,$A21,'QA Checklist'!$H$5:$H$203,"Fail")</f>
         <v/>
       </c>
       <c r="E21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$202,$A21,'QA Checklist'!$H$5:$H$202,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$203,$A21,'QA Checklist'!$H$5:$H$203,"Pending")</f>
         <v/>
       </c>
       <c r="F21" s="8">
@@ -941,19 +941,19 @@
         </is>
       </c>
       <c r="B22" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$202,$A22)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$203,$A22)</f>
         <v/>
       </c>
       <c r="C22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$202,$A22,'QA Checklist'!$H$5:$H$202,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$202,$A22,'QA Checklist'!$H$5:$H$202,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$203,$A22,'QA Checklist'!$H$5:$H$203,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$203,$A22,'QA Checklist'!$H$5:$H$203,"Pass")</f>
         <v/>
       </c>
       <c r="D22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$202,$A22,'QA Checklist'!$H$5:$H$202,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$202,$A22,'QA Checklist'!$H$5:$H$202,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$203,$A22,'QA Checklist'!$H$5:$H$203,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$203,$A22,'QA Checklist'!$H$5:$H$203,"Fail")</f>
         <v/>
       </c>
       <c r="E22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$202,$A22,'QA Checklist'!$H$5:$H$202,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$203,$A22,'QA Checklist'!$H$5:$H$203,"Pending")</f>
         <v/>
       </c>
       <c r="F22" s="8">
@@ -1023,19 +1023,19 @@
         </is>
       </c>
       <c r="B26" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$202,$A26&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$203,$A26&amp;"*")</f>
         <v/>
       </c>
       <c r="C26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$202,$A26&amp;"*",'QA Checklist'!$H$5:$H$202,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$202,$A26&amp;"*",'QA Checklist'!$H$5:$H$202,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$203,$A26&amp;"*",'QA Checklist'!$H$5:$H$203,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$203,$A26&amp;"*",'QA Checklist'!$H$5:$H$203,"Pass")</f>
         <v/>
       </c>
       <c r="D26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$202,$A26&amp;"*",'QA Checklist'!$H$5:$H$202,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$202,$A26&amp;"*",'QA Checklist'!$H$5:$H$202,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$203,$A26&amp;"*",'QA Checklist'!$H$5:$H$203,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$203,$A26&amp;"*",'QA Checklist'!$H$5:$H$203,"Fail")</f>
         <v/>
       </c>
       <c r="E26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$202,$A26&amp;"*",'QA Checklist'!$H$5:$H$202,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$203,$A26&amp;"*",'QA Checklist'!$H$5:$H$203,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1046,19 +1046,19 @@
         </is>
       </c>
       <c r="B27" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$202,$A27&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$203,$A27&amp;"*")</f>
         <v/>
       </c>
       <c r="C27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$202,$A27&amp;"*",'QA Checklist'!$H$5:$H$202,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$202,$A27&amp;"*",'QA Checklist'!$H$5:$H$202,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$203,$A27&amp;"*",'QA Checklist'!$H$5:$H$203,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$203,$A27&amp;"*",'QA Checklist'!$H$5:$H$203,"Pass")</f>
         <v/>
       </c>
       <c r="D27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$202,$A27&amp;"*",'QA Checklist'!$H$5:$H$202,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$202,$A27&amp;"*",'QA Checklist'!$H$5:$H$202,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$203,$A27&amp;"*",'QA Checklist'!$H$5:$H$203,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$203,$A27&amp;"*",'QA Checklist'!$H$5:$H$203,"Fail")</f>
         <v/>
       </c>
       <c r="E27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$202,$A27&amp;"*",'QA Checklist'!$H$5:$H$202,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$203,$A27&amp;"*",'QA Checklist'!$H$5:$H$203,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1069,19 +1069,19 @@
         </is>
       </c>
       <c r="B28" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$202,$A28&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$203,$A28&amp;"*")</f>
         <v/>
       </c>
       <c r="C28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$202,$A28&amp;"*",'QA Checklist'!$H$5:$H$202,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$202,$A28&amp;"*",'QA Checklist'!$H$5:$H$202,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$203,$A28&amp;"*",'QA Checklist'!$H$5:$H$203,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$203,$A28&amp;"*",'QA Checklist'!$H$5:$H$203,"Pass")</f>
         <v/>
       </c>
       <c r="D28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$202,$A28&amp;"*",'QA Checklist'!$H$5:$H$202,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$202,$A28&amp;"*",'QA Checklist'!$H$5:$H$202,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$203,$A28&amp;"*",'QA Checklist'!$H$5:$H$203,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$203,$A28&amp;"*",'QA Checklist'!$H$5:$H$203,"Fail")</f>
         <v/>
       </c>
       <c r="E28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$202,$A28&amp;"*",'QA Checklist'!$H$5:$H$202,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$203,$A28&amp;"*",'QA Checklist'!$H$5:$H$203,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1096,7 +1096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I202"/>
+  <dimension ref="A1:I203"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10033,12 +10033,59 @@
         </is>
       </c>
     </row>
+    <row r="203">
+      <c r="A203" s="12" t="inlineStr">
+        <is>
+          <t>SA-77</t>
+        </is>
+      </c>
+      <c r="B203" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="C203" s="13" t="inlineStr">
+        <is>
+          <t>Tier 2 (Workflow &amp; Ergonomics)</t>
+        </is>
+      </c>
+      <c r="D203" s="13" t="inlineStr">
+        <is>
+          <t>Four Lanes &amp; 2-Hour Express</t>
+        </is>
+      </c>
+      <c r="E203" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="F203" s="13" t="inlineStr">
+        <is>
+          <t>Open the lane lists in the Studio, the intake form and the Daily Intakes table; save a vehicle on PMS &amp; GRS Lane; complete an Express vehicle in 1h45 and another in 2h15; check analytics text and TV slide 3</t>
+        </is>
+      </c>
+      <c r="G203" s="13" t="inlineStr">
+        <is>
+          <t>Only Flexible, Express Lane (2 Hours), PMS &amp; GRS Lane and Priority Lane are offered; PMS &amp; GRS stays PMS &amp; GRS; 1h45 is on time and 2h15 is late; all Express text says 2 hours; the TV shows Express (≤ 2 Hours), Flexible, PMS &amp; GRS and Priority columns</t>
+        </is>
+      </c>
+      <c r="H203" s="14" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="I203" s="13" t="inlineStr">
+        <is>
+          <t>Verified by Automated Unit Tests (189 passing in tests/frontend/sla_and_logic.test.js AUT-FRONT-160) and a live 11/11 check</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:I202"/>
+  <autoFilter ref="A4:I203"/>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="H5:H202">
+  <conditionalFormatting sqref="H5:H203">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$H5="Passed"</formula>
     </cfRule>
@@ -10055,13 +10102,13 @@
       <formula>$H5="Pending"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A5:A202">
+  <conditionalFormatting sqref="A5:A203">
     <cfRule type="expression" priority="6" dxfId="3">
-      <formula>COUNTIF($A$5:$A$202,$A5)&gt;1</formula>
+      <formula>COUNTIF($A$5:$A$203,$A5)&gt;1</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H5:H202" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H5:H203" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pending,Passed,Failed"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
fix(REV-202): registered ROs are same-day jobs; C.O. field and Job Order category removed
Daily Intakes marked any job with a promise date as carry-over, and the Studio always fills the promise date, so every registered RO looked like a carry-over. Carry-over now means status Carry Over or a carry-over record (tag, counts and the Return Carry Over label). The unused Carry-Over (C.O.) field is removed and the duplicate Service Category on Job_Order is hidden (chosen on Workshop_Monitoring).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
+++ b/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
@@ -11,7 +11,7 @@
     <sheet name="QA Checklist" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$203</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$204</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'QA Checklist'!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTA('QA Checklist'!$A$5:$A$203)</f>
+        <f>COUNTA('QA Checklist'!$A$5:$A$204)</f>
         <v/>
       </c>
     </row>
@@ -594,7 +594,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$203,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$203,"Pass")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$204,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$204,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$203,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$203,"Fail")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$204,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$204,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -616,7 +616,7 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$203,"Pending")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$204,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -671,19 +671,19 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$203,$A12)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$204,$A12)</f>
         <v/>
       </c>
       <c r="C12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$203,$A12,'QA Checklist'!$H$5:$H$203,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$203,$A12,'QA Checklist'!$H$5:$H$203,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$204,$A12,'QA Checklist'!$H$5:$H$204,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$204,$A12,'QA Checklist'!$H$5:$H$204,"Pass")</f>
         <v/>
       </c>
       <c r="D12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$203,$A12,'QA Checklist'!$H$5:$H$203,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$203,$A12,'QA Checklist'!$H$5:$H$203,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$204,$A12,'QA Checklist'!$H$5:$H$204,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$204,$A12,'QA Checklist'!$H$5:$H$204,"Fail")</f>
         <v/>
       </c>
       <c r="E12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$203,$A12,'QA Checklist'!$H$5:$H$203,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$204,$A12,'QA Checklist'!$H$5:$H$204,"Pending")</f>
         <v/>
       </c>
       <c r="F12" s="8">
@@ -698,19 +698,19 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$203,$A13)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$204,$A13)</f>
         <v/>
       </c>
       <c r="C13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$203,$A13,'QA Checklist'!$H$5:$H$203,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$203,$A13,'QA Checklist'!$H$5:$H$203,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$204,$A13,'QA Checklist'!$H$5:$H$204,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$204,$A13,'QA Checklist'!$H$5:$H$204,"Pass")</f>
         <v/>
       </c>
       <c r="D13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$203,$A13,'QA Checklist'!$H$5:$H$203,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$203,$A13,'QA Checklist'!$H$5:$H$203,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$204,$A13,'QA Checklist'!$H$5:$H$204,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$204,$A13,'QA Checklist'!$H$5:$H$204,"Fail")</f>
         <v/>
       </c>
       <c r="E13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$203,$A13,'QA Checklist'!$H$5:$H$203,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$204,$A13,'QA Checklist'!$H$5:$H$204,"Pending")</f>
         <v/>
       </c>
       <c r="F13" s="8">
@@ -725,19 +725,19 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$203,$A14)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$204,$A14)</f>
         <v/>
       </c>
       <c r="C14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$203,$A14,'QA Checklist'!$H$5:$H$203,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$203,$A14,'QA Checklist'!$H$5:$H$203,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$204,$A14,'QA Checklist'!$H$5:$H$204,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$204,$A14,'QA Checklist'!$H$5:$H$204,"Pass")</f>
         <v/>
       </c>
       <c r="D14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$203,$A14,'QA Checklist'!$H$5:$H$203,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$203,$A14,'QA Checklist'!$H$5:$H$203,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$204,$A14,'QA Checklist'!$H$5:$H$204,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$204,$A14,'QA Checklist'!$H$5:$H$204,"Fail")</f>
         <v/>
       </c>
       <c r="E14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$203,$A14,'QA Checklist'!$H$5:$H$203,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$204,$A14,'QA Checklist'!$H$5:$H$204,"Pending")</f>
         <v/>
       </c>
       <c r="F14" s="8">
@@ -752,19 +752,19 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$203,$A15)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$204,$A15)</f>
         <v/>
       </c>
       <c r="C15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$203,$A15,'QA Checklist'!$H$5:$H$203,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$203,$A15,'QA Checklist'!$H$5:$H$203,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$204,$A15,'QA Checklist'!$H$5:$H$204,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$204,$A15,'QA Checklist'!$H$5:$H$204,"Pass")</f>
         <v/>
       </c>
       <c r="D15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$203,$A15,'QA Checklist'!$H$5:$H$203,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$203,$A15,'QA Checklist'!$H$5:$H$203,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$204,$A15,'QA Checklist'!$H$5:$H$204,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$204,$A15,'QA Checklist'!$H$5:$H$204,"Fail")</f>
         <v/>
       </c>
       <c r="E15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$203,$A15,'QA Checklist'!$H$5:$H$203,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$204,$A15,'QA Checklist'!$H$5:$H$204,"Pending")</f>
         <v/>
       </c>
       <c r="F15" s="8">
@@ -779,19 +779,19 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$203,$A16)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$204,$A16)</f>
         <v/>
       </c>
       <c r="C16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$203,$A16,'QA Checklist'!$H$5:$H$203,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$203,$A16,'QA Checklist'!$H$5:$H$203,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$204,$A16,'QA Checklist'!$H$5:$H$204,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$204,$A16,'QA Checklist'!$H$5:$H$204,"Pass")</f>
         <v/>
       </c>
       <c r="D16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$203,$A16,'QA Checklist'!$H$5:$H$203,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$203,$A16,'QA Checklist'!$H$5:$H$203,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$204,$A16,'QA Checklist'!$H$5:$H$204,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$204,$A16,'QA Checklist'!$H$5:$H$204,"Fail")</f>
         <v/>
       </c>
       <c r="E16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$203,$A16,'QA Checklist'!$H$5:$H$203,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$204,$A16,'QA Checklist'!$H$5:$H$204,"Pending")</f>
         <v/>
       </c>
       <c r="F16" s="8">
@@ -806,19 +806,19 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$203,$A17)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$204,$A17)</f>
         <v/>
       </c>
       <c r="C17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$203,$A17,'QA Checklist'!$H$5:$H$203,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$203,$A17,'QA Checklist'!$H$5:$H$203,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$204,$A17,'QA Checklist'!$H$5:$H$204,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$204,$A17,'QA Checklist'!$H$5:$H$204,"Pass")</f>
         <v/>
       </c>
       <c r="D17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$203,$A17,'QA Checklist'!$H$5:$H$203,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$203,$A17,'QA Checklist'!$H$5:$H$203,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$204,$A17,'QA Checklist'!$H$5:$H$204,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$204,$A17,'QA Checklist'!$H$5:$H$204,"Fail")</f>
         <v/>
       </c>
       <c r="E17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$203,$A17,'QA Checklist'!$H$5:$H$203,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$204,$A17,'QA Checklist'!$H$5:$H$204,"Pending")</f>
         <v/>
       </c>
       <c r="F17" s="8">
@@ -833,19 +833,19 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$203,$A18)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$204,$A18)</f>
         <v/>
       </c>
       <c r="C18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$203,$A18,'QA Checklist'!$H$5:$H$203,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$203,$A18,'QA Checklist'!$H$5:$H$203,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$204,$A18,'QA Checklist'!$H$5:$H$204,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$204,$A18,'QA Checklist'!$H$5:$H$204,"Pass")</f>
         <v/>
       </c>
       <c r="D18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$203,$A18,'QA Checklist'!$H$5:$H$203,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$203,$A18,'QA Checklist'!$H$5:$H$203,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$204,$A18,'QA Checklist'!$H$5:$H$204,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$204,$A18,'QA Checklist'!$H$5:$H$204,"Fail")</f>
         <v/>
       </c>
       <c r="E18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$203,$A18,'QA Checklist'!$H$5:$H$203,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$204,$A18,'QA Checklist'!$H$5:$H$204,"Pending")</f>
         <v/>
       </c>
       <c r="F18" s="8">
@@ -860,19 +860,19 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$203,$A19)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$204,$A19)</f>
         <v/>
       </c>
       <c r="C19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$203,$A19,'QA Checklist'!$H$5:$H$203,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$203,$A19,'QA Checklist'!$H$5:$H$203,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$204,$A19,'QA Checklist'!$H$5:$H$204,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$204,$A19,'QA Checklist'!$H$5:$H$204,"Pass")</f>
         <v/>
       </c>
       <c r="D19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$203,$A19,'QA Checklist'!$H$5:$H$203,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$203,$A19,'QA Checklist'!$H$5:$H$203,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$204,$A19,'QA Checklist'!$H$5:$H$204,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$204,$A19,'QA Checklist'!$H$5:$H$204,"Fail")</f>
         <v/>
       </c>
       <c r="E19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$203,$A19,'QA Checklist'!$H$5:$H$203,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$204,$A19,'QA Checklist'!$H$5:$H$204,"Pending")</f>
         <v/>
       </c>
       <c r="F19" s="8">
@@ -887,19 +887,19 @@
         </is>
       </c>
       <c r="B20" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$203,$A20)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$204,$A20)</f>
         <v/>
       </c>
       <c r="C20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$203,$A20,'QA Checklist'!$H$5:$H$203,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$203,$A20,'QA Checklist'!$H$5:$H$203,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$204,$A20,'QA Checklist'!$H$5:$H$204,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$204,$A20,'QA Checklist'!$H$5:$H$204,"Pass")</f>
         <v/>
       </c>
       <c r="D20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$203,$A20,'QA Checklist'!$H$5:$H$203,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$203,$A20,'QA Checklist'!$H$5:$H$203,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$204,$A20,'QA Checklist'!$H$5:$H$204,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$204,$A20,'QA Checklist'!$H$5:$H$204,"Fail")</f>
         <v/>
       </c>
       <c r="E20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$203,$A20,'QA Checklist'!$H$5:$H$203,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$204,$A20,'QA Checklist'!$H$5:$H$204,"Pending")</f>
         <v/>
       </c>
       <c r="F20" s="8">
@@ -914,19 +914,19 @@
         </is>
       </c>
       <c r="B21" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$203,$A21)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$204,$A21)</f>
         <v/>
       </c>
       <c r="C21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$203,$A21,'QA Checklist'!$H$5:$H$203,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$203,$A21,'QA Checklist'!$H$5:$H$203,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$204,$A21,'QA Checklist'!$H$5:$H$204,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$204,$A21,'QA Checklist'!$H$5:$H$204,"Pass")</f>
         <v/>
       </c>
       <c r="D21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$203,$A21,'QA Checklist'!$H$5:$H$203,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$203,$A21,'QA Checklist'!$H$5:$H$203,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$204,$A21,'QA Checklist'!$H$5:$H$204,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$204,$A21,'QA Checklist'!$H$5:$H$204,"Fail")</f>
         <v/>
       </c>
       <c r="E21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$203,$A21,'QA Checklist'!$H$5:$H$203,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$204,$A21,'QA Checklist'!$H$5:$H$204,"Pending")</f>
         <v/>
       </c>
       <c r="F21" s="8">
@@ -941,19 +941,19 @@
         </is>
       </c>
       <c r="B22" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$203,$A22)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$204,$A22)</f>
         <v/>
       </c>
       <c r="C22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$203,$A22,'QA Checklist'!$H$5:$H$203,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$203,$A22,'QA Checklist'!$H$5:$H$203,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$204,$A22,'QA Checklist'!$H$5:$H$204,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$204,$A22,'QA Checklist'!$H$5:$H$204,"Pass")</f>
         <v/>
       </c>
       <c r="D22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$203,$A22,'QA Checklist'!$H$5:$H$203,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$203,$A22,'QA Checklist'!$H$5:$H$203,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$204,$A22,'QA Checklist'!$H$5:$H$204,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$204,$A22,'QA Checklist'!$H$5:$H$204,"Fail")</f>
         <v/>
       </c>
       <c r="E22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$203,$A22,'QA Checklist'!$H$5:$H$203,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$204,$A22,'QA Checklist'!$H$5:$H$204,"Pending")</f>
         <v/>
       </c>
       <c r="F22" s="8">
@@ -1023,19 +1023,19 @@
         </is>
       </c>
       <c r="B26" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$203,$A26&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$204,$A26&amp;"*")</f>
         <v/>
       </c>
       <c r="C26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$203,$A26&amp;"*",'QA Checklist'!$H$5:$H$203,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$203,$A26&amp;"*",'QA Checklist'!$H$5:$H$203,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$204,$A26&amp;"*",'QA Checklist'!$H$5:$H$204,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$204,$A26&amp;"*",'QA Checklist'!$H$5:$H$204,"Pass")</f>
         <v/>
       </c>
       <c r="D26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$203,$A26&amp;"*",'QA Checklist'!$H$5:$H$203,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$203,$A26&amp;"*",'QA Checklist'!$H$5:$H$203,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$204,$A26&amp;"*",'QA Checklist'!$H$5:$H$204,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$204,$A26&amp;"*",'QA Checklist'!$H$5:$H$204,"Fail")</f>
         <v/>
       </c>
       <c r="E26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$203,$A26&amp;"*",'QA Checklist'!$H$5:$H$203,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$204,$A26&amp;"*",'QA Checklist'!$H$5:$H$204,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1046,19 +1046,19 @@
         </is>
       </c>
       <c r="B27" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$203,$A27&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$204,$A27&amp;"*")</f>
         <v/>
       </c>
       <c r="C27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$203,$A27&amp;"*",'QA Checklist'!$H$5:$H$203,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$203,$A27&amp;"*",'QA Checklist'!$H$5:$H$203,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$204,$A27&amp;"*",'QA Checklist'!$H$5:$H$204,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$204,$A27&amp;"*",'QA Checklist'!$H$5:$H$204,"Pass")</f>
         <v/>
       </c>
       <c r="D27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$203,$A27&amp;"*",'QA Checklist'!$H$5:$H$203,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$203,$A27&amp;"*",'QA Checklist'!$H$5:$H$203,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$204,$A27&amp;"*",'QA Checklist'!$H$5:$H$204,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$204,$A27&amp;"*",'QA Checklist'!$H$5:$H$204,"Fail")</f>
         <v/>
       </c>
       <c r="E27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$203,$A27&amp;"*",'QA Checklist'!$H$5:$H$203,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$204,$A27&amp;"*",'QA Checklist'!$H$5:$H$204,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1069,19 +1069,19 @@
         </is>
       </c>
       <c r="B28" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$203,$A28&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$204,$A28&amp;"*")</f>
         <v/>
       </c>
       <c r="C28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$203,$A28&amp;"*",'QA Checklist'!$H$5:$H$203,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$203,$A28&amp;"*",'QA Checklist'!$H$5:$H$203,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$204,$A28&amp;"*",'QA Checklist'!$H$5:$H$204,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$204,$A28&amp;"*",'QA Checklist'!$H$5:$H$204,"Pass")</f>
         <v/>
       </c>
       <c r="D28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$203,$A28&amp;"*",'QA Checklist'!$H$5:$H$203,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$203,$A28&amp;"*",'QA Checklist'!$H$5:$H$203,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$204,$A28&amp;"*",'QA Checklist'!$H$5:$H$204,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$204,$A28&amp;"*",'QA Checklist'!$H$5:$H$204,"Fail")</f>
         <v/>
       </c>
       <c r="E28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$203,$A28&amp;"*",'QA Checklist'!$H$5:$H$203,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$204,$A28&amp;"*",'QA Checklist'!$H$5:$H$204,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1096,7 +1096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I203"/>
+  <dimension ref="A1:I204"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10080,12 +10080,59 @@
         </is>
       </c>
     </row>
+    <row r="204">
+      <c r="A204" s="12" t="inlineStr">
+        <is>
+          <t>SA-78</t>
+        </is>
+      </c>
+      <c r="B204" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="C204" s="13" t="inlineStr">
+        <is>
+          <t>Tier 2 (Workflow &amp; Ergonomics)</t>
+        </is>
+      </c>
+      <c r="D204" s="13" t="inlineStr">
+        <is>
+          <t>Registered RO Appears as Same-Day Job</t>
+        </is>
+      </c>
+      <c r="E204" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="F204" s="13" t="inlineStr">
+        <is>
+          <t>On Workshop_Monitoring fill plate, model, customer and choose a Service Category; keep the Promise Date; Register RO; open Daily Intakes</t>
+        </is>
+      </c>
+      <c r="G204" s="13" t="inlineStr">
+        <is>
+          <t>No Carry-Over (C.O.) field on Workshop_Monitoring and no Service Category on Job_Order; the vehicle appears in Daily Intakes as Waiting without the Carry-Over tag, with the chosen category</t>
+        </is>
+      </c>
+      <c r="H204" s="14" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="I204" s="13" t="inlineStr">
+        <is>
+          <t>Verified by Automated Unit Tests (190 passing in tests/frontend/sla_and_logic.test.js AUT-FRONT-161) and headless Chrome 5/5 on a real registration</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:I203"/>
+  <autoFilter ref="A4:I204"/>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="H5:H203">
+  <conditionalFormatting sqref="H5:H204">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$H5="Passed"</formula>
     </cfRule>
@@ -10102,13 +10149,13 @@
       <formula>$H5="Pending"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A5:A203">
+  <conditionalFormatting sqref="A5:A204">
     <cfRule type="expression" priority="6" dxfId="3">
-      <formula>COUNTIF($A$5:$A$203,$A5)&gt;1</formula>
+      <formula>COUNTIF($A$5:$A$204,$A5)&gt;1</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H5:H203" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H5:H204" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pending,Passed,Failed"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
fix(REV-203): claim stubs assigned by the server in order, per Manila day
Claim stubs are MMDDYY + J + the customer's number for the day, first come first served. The server alone assigns them with an atomic per-day counter (claim_stub_counters), never below a number already used, using the Manila date (PHP runs on Berlin time). Stubs sent by the Studio are ignored, every vehicle entering the floor is numbered, online bookings are numbered when accepted, and stubs can no longer be edited. The Studio field is a read-only server preview that shows the assigned number after registering.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
+++ b/Hontech Documentation/HONTECH_QA_TEST_CHECKLIST.xlsx
@@ -11,7 +11,7 @@
     <sheet name="QA Checklist" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$204</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QA Checklist'!$A$4:$I$205</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'QA Checklist'!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTA('QA Checklist'!$A$5:$A$204)</f>
+        <f>COUNTA('QA Checklist'!$A$5:$A$205)</f>
         <v/>
       </c>
     </row>
@@ -594,7 +594,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$204,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$204,"Pass")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$205,"Passed")+COUNTIF('QA Checklist'!$H$5:$H$205,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$204,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$204,"Fail")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$205,"Failed")+COUNTIF('QA Checklist'!$H$5:$H$205,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -616,7 +616,7 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF('QA Checklist'!$H$5:$H$204,"Pending")</f>
+        <f>COUNTIF('QA Checklist'!$H$5:$H$205,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -671,19 +671,19 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$204,$A12)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$205,$A12)</f>
         <v/>
       </c>
       <c r="C12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$204,$A12,'QA Checklist'!$H$5:$H$204,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$204,$A12,'QA Checklist'!$H$5:$H$204,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$205,$A12,'QA Checklist'!$H$5:$H$205,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$205,$A12,'QA Checklist'!$H$5:$H$205,"Pass")</f>
         <v/>
       </c>
       <c r="D12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$204,$A12,'QA Checklist'!$H$5:$H$204,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$204,$A12,'QA Checklist'!$H$5:$H$204,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$205,$A12,'QA Checklist'!$H$5:$H$205,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$205,$A12,'QA Checklist'!$H$5:$H$205,"Fail")</f>
         <v/>
       </c>
       <c r="E12" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$204,$A12,'QA Checklist'!$H$5:$H$204,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$205,$A12,'QA Checklist'!$H$5:$H$205,"Pending")</f>
         <v/>
       </c>
       <c r="F12" s="8">
@@ -698,19 +698,19 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$204,$A13)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$205,$A13)</f>
         <v/>
       </c>
       <c r="C13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$204,$A13,'QA Checklist'!$H$5:$H$204,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$204,$A13,'QA Checklist'!$H$5:$H$204,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$205,$A13,'QA Checklist'!$H$5:$H$205,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$205,$A13,'QA Checklist'!$H$5:$H$205,"Pass")</f>
         <v/>
       </c>
       <c r="D13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$204,$A13,'QA Checklist'!$H$5:$H$204,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$204,$A13,'QA Checklist'!$H$5:$H$204,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$205,$A13,'QA Checklist'!$H$5:$H$205,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$205,$A13,'QA Checklist'!$H$5:$H$205,"Fail")</f>
         <v/>
       </c>
       <c r="E13" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$204,$A13,'QA Checklist'!$H$5:$H$204,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$205,$A13,'QA Checklist'!$H$5:$H$205,"Pending")</f>
         <v/>
       </c>
       <c r="F13" s="8">
@@ -725,19 +725,19 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$204,$A14)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$205,$A14)</f>
         <v/>
       </c>
       <c r="C14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$204,$A14,'QA Checklist'!$H$5:$H$204,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$204,$A14,'QA Checklist'!$H$5:$H$204,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$205,$A14,'QA Checklist'!$H$5:$H$205,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$205,$A14,'QA Checklist'!$H$5:$H$205,"Pass")</f>
         <v/>
       </c>
       <c r="D14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$204,$A14,'QA Checklist'!$H$5:$H$204,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$204,$A14,'QA Checklist'!$H$5:$H$204,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$205,$A14,'QA Checklist'!$H$5:$H$205,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$205,$A14,'QA Checklist'!$H$5:$H$205,"Fail")</f>
         <v/>
       </c>
       <c r="E14" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$204,$A14,'QA Checklist'!$H$5:$H$204,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$205,$A14,'QA Checklist'!$H$5:$H$205,"Pending")</f>
         <v/>
       </c>
       <c r="F14" s="8">
@@ -752,19 +752,19 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$204,$A15)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$205,$A15)</f>
         <v/>
       </c>
       <c r="C15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$204,$A15,'QA Checklist'!$H$5:$H$204,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$204,$A15,'QA Checklist'!$H$5:$H$204,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$205,$A15,'QA Checklist'!$H$5:$H$205,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$205,$A15,'QA Checklist'!$H$5:$H$205,"Pass")</f>
         <v/>
       </c>
       <c r="D15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$204,$A15,'QA Checklist'!$H$5:$H$204,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$204,$A15,'QA Checklist'!$H$5:$H$204,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$205,$A15,'QA Checklist'!$H$5:$H$205,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$205,$A15,'QA Checklist'!$H$5:$H$205,"Fail")</f>
         <v/>
       </c>
       <c r="E15" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$204,$A15,'QA Checklist'!$H$5:$H$204,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$205,$A15,'QA Checklist'!$H$5:$H$205,"Pending")</f>
         <v/>
       </c>
       <c r="F15" s="8">
@@ -779,19 +779,19 @@
         </is>
       </c>
       <c r="B16" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$204,$A16)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$205,$A16)</f>
         <v/>
       </c>
       <c r="C16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$204,$A16,'QA Checklist'!$H$5:$H$204,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$204,$A16,'QA Checklist'!$H$5:$H$204,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$205,$A16,'QA Checklist'!$H$5:$H$205,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$205,$A16,'QA Checklist'!$H$5:$H$205,"Pass")</f>
         <v/>
       </c>
       <c r="D16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$204,$A16,'QA Checklist'!$H$5:$H$204,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$204,$A16,'QA Checklist'!$H$5:$H$204,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$205,$A16,'QA Checklist'!$H$5:$H$205,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$205,$A16,'QA Checklist'!$H$5:$H$205,"Fail")</f>
         <v/>
       </c>
       <c r="E16" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$204,$A16,'QA Checklist'!$H$5:$H$204,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$205,$A16,'QA Checklist'!$H$5:$H$205,"Pending")</f>
         <v/>
       </c>
       <c r="F16" s="8">
@@ -806,19 +806,19 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$204,$A17)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$205,$A17)</f>
         <v/>
       </c>
       <c r="C17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$204,$A17,'QA Checklist'!$H$5:$H$204,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$204,$A17,'QA Checklist'!$H$5:$H$204,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$205,$A17,'QA Checklist'!$H$5:$H$205,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$205,$A17,'QA Checklist'!$H$5:$H$205,"Pass")</f>
         <v/>
       </c>
       <c r="D17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$204,$A17,'QA Checklist'!$H$5:$H$204,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$204,$A17,'QA Checklist'!$H$5:$H$204,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$205,$A17,'QA Checklist'!$H$5:$H$205,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$205,$A17,'QA Checklist'!$H$5:$H$205,"Fail")</f>
         <v/>
       </c>
       <c r="E17" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$204,$A17,'QA Checklist'!$H$5:$H$204,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$205,$A17,'QA Checklist'!$H$5:$H$205,"Pending")</f>
         <v/>
       </c>
       <c r="F17" s="8">
@@ -833,19 +833,19 @@
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$204,$A18)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$205,$A18)</f>
         <v/>
       </c>
       <c r="C18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$204,$A18,'QA Checklist'!$H$5:$H$204,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$204,$A18,'QA Checklist'!$H$5:$H$204,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$205,$A18,'QA Checklist'!$H$5:$H$205,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$205,$A18,'QA Checklist'!$H$5:$H$205,"Pass")</f>
         <v/>
       </c>
       <c r="D18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$204,$A18,'QA Checklist'!$H$5:$H$204,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$204,$A18,'QA Checklist'!$H$5:$H$204,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$205,$A18,'QA Checklist'!$H$5:$H$205,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$205,$A18,'QA Checklist'!$H$5:$H$205,"Fail")</f>
         <v/>
       </c>
       <c r="E18" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$204,$A18,'QA Checklist'!$H$5:$H$204,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$205,$A18,'QA Checklist'!$H$5:$H$205,"Pending")</f>
         <v/>
       </c>
       <c r="F18" s="8">
@@ -860,19 +860,19 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$204,$A19)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$205,$A19)</f>
         <v/>
       </c>
       <c r="C19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$204,$A19,'QA Checklist'!$H$5:$H$204,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$204,$A19,'QA Checklist'!$H$5:$H$204,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$205,$A19,'QA Checklist'!$H$5:$H$205,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$205,$A19,'QA Checklist'!$H$5:$H$205,"Pass")</f>
         <v/>
       </c>
       <c r="D19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$204,$A19,'QA Checklist'!$H$5:$H$204,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$204,$A19,'QA Checklist'!$H$5:$H$204,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$205,$A19,'QA Checklist'!$H$5:$H$205,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$205,$A19,'QA Checklist'!$H$5:$H$205,"Fail")</f>
         <v/>
       </c>
       <c r="E19" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$204,$A19,'QA Checklist'!$H$5:$H$204,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$205,$A19,'QA Checklist'!$H$5:$H$205,"Pending")</f>
         <v/>
       </c>
       <c r="F19" s="8">
@@ -887,19 +887,19 @@
         </is>
       </c>
       <c r="B20" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$204,$A20)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$205,$A20)</f>
         <v/>
       </c>
       <c r="C20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$204,$A20,'QA Checklist'!$H$5:$H$204,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$204,$A20,'QA Checklist'!$H$5:$H$204,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$205,$A20,'QA Checklist'!$H$5:$H$205,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$205,$A20,'QA Checklist'!$H$5:$H$205,"Pass")</f>
         <v/>
       </c>
       <c r="D20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$204,$A20,'QA Checklist'!$H$5:$H$204,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$204,$A20,'QA Checklist'!$H$5:$H$204,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$205,$A20,'QA Checklist'!$H$5:$H$205,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$205,$A20,'QA Checklist'!$H$5:$H$205,"Fail")</f>
         <v/>
       </c>
       <c r="E20" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$204,$A20,'QA Checklist'!$H$5:$H$204,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$205,$A20,'QA Checklist'!$H$5:$H$205,"Pending")</f>
         <v/>
       </c>
       <c r="F20" s="8">
@@ -914,19 +914,19 @@
         </is>
       </c>
       <c r="B21" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$204,$A21)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$205,$A21)</f>
         <v/>
       </c>
       <c r="C21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$204,$A21,'QA Checklist'!$H$5:$H$204,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$204,$A21,'QA Checklist'!$H$5:$H$204,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$205,$A21,'QA Checklist'!$H$5:$H$205,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$205,$A21,'QA Checklist'!$H$5:$H$205,"Pass")</f>
         <v/>
       </c>
       <c r="D21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$204,$A21,'QA Checklist'!$H$5:$H$204,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$204,$A21,'QA Checklist'!$H$5:$H$204,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$205,$A21,'QA Checklist'!$H$5:$H$205,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$205,$A21,'QA Checklist'!$H$5:$H$205,"Fail")</f>
         <v/>
       </c>
       <c r="E21" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$204,$A21,'QA Checklist'!$H$5:$H$204,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$205,$A21,'QA Checklist'!$H$5:$H$205,"Pending")</f>
         <v/>
       </c>
       <c r="F21" s="8">
@@ -941,19 +941,19 @@
         </is>
       </c>
       <c r="B22" s="5">
-        <f>COUNTIF('QA Checklist'!$B$5:$B$204,$A22)</f>
+        <f>COUNTIF('QA Checklist'!$B$5:$B$205,$A22)</f>
         <v/>
       </c>
       <c r="C22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$204,$A22,'QA Checklist'!$H$5:$H$204,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$204,$A22,'QA Checklist'!$H$5:$H$204,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$205,$A22,'QA Checklist'!$H$5:$H$205,"Passed")+COUNTIFS('QA Checklist'!$B$5:$B$205,$A22,'QA Checklist'!$H$5:$H$205,"Pass")</f>
         <v/>
       </c>
       <c r="D22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$204,$A22,'QA Checklist'!$H$5:$H$204,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$204,$A22,'QA Checklist'!$H$5:$H$204,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$205,$A22,'QA Checklist'!$H$5:$H$205,"Failed")+COUNTIFS('QA Checklist'!$B$5:$B$205,$A22,'QA Checklist'!$H$5:$H$205,"Fail")</f>
         <v/>
       </c>
       <c r="E22" s="5">
-        <f>COUNTIFS('QA Checklist'!$B$5:$B$204,$A22,'QA Checklist'!$H$5:$H$204,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$B$5:$B$205,$A22,'QA Checklist'!$H$5:$H$205,"Pending")</f>
         <v/>
       </c>
       <c r="F22" s="8">
@@ -1023,19 +1023,19 @@
         </is>
       </c>
       <c r="B26" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$204,$A26&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$205,$A26&amp;"*")</f>
         <v/>
       </c>
       <c r="C26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$204,$A26&amp;"*",'QA Checklist'!$H$5:$H$204,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$204,$A26&amp;"*",'QA Checklist'!$H$5:$H$204,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$205,$A26&amp;"*",'QA Checklist'!$H$5:$H$205,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$205,$A26&amp;"*",'QA Checklist'!$H$5:$H$205,"Pass")</f>
         <v/>
       </c>
       <c r="D26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$204,$A26&amp;"*",'QA Checklist'!$H$5:$H$204,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$204,$A26&amp;"*",'QA Checklist'!$H$5:$H$204,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$205,$A26&amp;"*",'QA Checklist'!$H$5:$H$205,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$205,$A26&amp;"*",'QA Checklist'!$H$5:$H$205,"Fail")</f>
         <v/>
       </c>
       <c r="E26" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$204,$A26&amp;"*",'QA Checklist'!$H$5:$H$204,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$205,$A26&amp;"*",'QA Checklist'!$H$5:$H$205,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1046,19 +1046,19 @@
         </is>
       </c>
       <c r="B27" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$204,$A27&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$205,$A27&amp;"*")</f>
         <v/>
       </c>
       <c r="C27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$204,$A27&amp;"*",'QA Checklist'!$H$5:$H$204,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$204,$A27&amp;"*",'QA Checklist'!$H$5:$H$204,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$205,$A27&amp;"*",'QA Checklist'!$H$5:$H$205,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$205,$A27&amp;"*",'QA Checklist'!$H$5:$H$205,"Pass")</f>
         <v/>
       </c>
       <c r="D27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$204,$A27&amp;"*",'QA Checklist'!$H$5:$H$204,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$204,$A27&amp;"*",'QA Checklist'!$H$5:$H$204,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$205,$A27&amp;"*",'QA Checklist'!$H$5:$H$205,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$205,$A27&amp;"*",'QA Checklist'!$H$5:$H$205,"Fail")</f>
         <v/>
       </c>
       <c r="E27" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$204,$A27&amp;"*",'QA Checklist'!$H$5:$H$204,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$205,$A27&amp;"*",'QA Checklist'!$H$5:$H$205,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1069,19 +1069,19 @@
         </is>
       </c>
       <c r="B28" s="5">
-        <f>COUNTIF('QA Checklist'!$C$5:$C$204,$A28&amp;"*")</f>
+        <f>COUNTIF('QA Checklist'!$C$5:$C$205,$A28&amp;"*")</f>
         <v/>
       </c>
       <c r="C28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$204,$A28&amp;"*",'QA Checklist'!$H$5:$H$204,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$204,$A28&amp;"*",'QA Checklist'!$H$5:$H$204,"Pass")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$205,$A28&amp;"*",'QA Checklist'!$H$5:$H$205,"Passed")+COUNTIFS('QA Checklist'!$C$5:$C$205,$A28&amp;"*",'QA Checklist'!$H$5:$H$205,"Pass")</f>
         <v/>
       </c>
       <c r="D28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$204,$A28&amp;"*",'QA Checklist'!$H$5:$H$204,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$204,$A28&amp;"*",'QA Checklist'!$H$5:$H$204,"Fail")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$205,$A28&amp;"*",'QA Checklist'!$H$5:$H$205,"Failed")+COUNTIFS('QA Checklist'!$C$5:$C$205,$A28&amp;"*",'QA Checklist'!$H$5:$H$205,"Fail")</f>
         <v/>
       </c>
       <c r="E28" s="5">
-        <f>COUNTIFS('QA Checklist'!$C$5:$C$204,$A28&amp;"*",'QA Checklist'!$H$5:$H$204,"Pending")</f>
+        <f>COUNTIFS('QA Checklist'!$C$5:$C$205,$A28&amp;"*",'QA Checklist'!$H$5:$H$205,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -1096,7 +1096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I204"/>
+  <dimension ref="A1:I205"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10127,12 +10127,59 @@
         </is>
       </c>
     </row>
+    <row r="205">
+      <c r="A205" s="12" t="inlineStr">
+        <is>
+          <t>SA-79</t>
+        </is>
+      </c>
+      <c r="B205" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="C205" s="13" t="inlineStr">
+        <is>
+          <t>Tier 2 (Workflow &amp; Ergonomics)</t>
+        </is>
+      </c>
+      <c r="D205" s="13" t="inlineStr">
+        <is>
+          <t>Claim Stub Order (J1, J2, J3)</t>
+        </is>
+      </c>
+      <c r="E205" s="13" t="inlineStr">
+        <is>
+          <t>Service Advisor</t>
+        </is>
+      </c>
+      <c r="F205" s="13" t="inlineStr">
+        <is>
+          <t>Register several ROs in a row from the Studio (and from two PCs at the same time); accept an online booking into the queue; try to change a stub; check the next day</t>
+        </is>
+      </c>
+      <c r="G205" s="13" t="inlineStr">
+        <is>
+          <t>Each vehicle gets the next number for the day (MMDDYYJ1, J2, J3 ...) with no duplicates or gaps, the Studio field is read-only and shows the assigned number, stubs cannot be edited, and numbering restarts at J1 on the next date</t>
+        </is>
+      </c>
+      <c r="H205" s="14" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="I205" s="13" t="inlineStr">
+        <is>
+          <t>Verified by Automated Unit Tests (191 passing in tests/frontend/sla_and_logic.test.js AUT-FRONT-162) and a live 11/11 check with six simultaneous registrations</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:I204"/>
+  <autoFilter ref="A4:I205"/>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="H5:H204">
+  <conditionalFormatting sqref="H5:H205">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$H5="Passed"</formula>
     </cfRule>
@@ -10149,13 +10196,13 @@
       <formula>$H5="Pending"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A5:A204">
+  <conditionalFormatting sqref="A5:A205">
     <cfRule type="expression" priority="6" dxfId="3">
-      <formula>COUNTIF($A$5:$A$204,$A5)&gt;1</formula>
+      <formula>COUNTIF($A$5:$A$205,$A5)&gt;1</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H5:H204" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H5:H205" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pending,Passed,Failed"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>